<commit_message>
fix(contenu): Correction de formulations différentes/coquilles dans les nomd des bibliothèques.
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tardimat\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C2FAE6E-1C02-40D0-A5B5-AF48E760366F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0AD7956-E2B8-4A87-AE47-F29B203F69B3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" tabRatio="241" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -192,9 +192,6 @@
     <t>Gestion des collections</t>
   </si>
   <si>
-    <t>Direction des collections, du traitement documentaire et des métadonnée, et Centre de conservation Lionel-Groulx</t>
-  </si>
-  <si>
     <t>514 343-6111, poste 5100</t>
   </si>
   <si>
@@ -699,9 +696,6 @@
     <t>Fatima Zahra</t>
   </si>
   <si>
-    <t>Direction des collections, du traitement documentaire et métadonnées</t>
-  </si>
-  <si>
     <t>514 343-6111, poste 1077</t>
   </si>
   <si>
@@ -984,9 +978,6 @@
     <t>julie-ouelette.jpg</t>
   </si>
   <si>
-    <t>Bibliothèques des lettres et sciences humaines | Service du prêt entre bibliothèques</t>
-  </si>
-  <si>
     <t>514 343-6111, poste 2616</t>
   </si>
   <si>
@@ -2011,13 +2002,22 @@
   </si>
   <si>
     <t>laurence-charest.jpg</t>
+  </si>
+  <si>
+    <t>Direction des collections, du traitement documentaire et des métadonnées; Centre de conservation Lionel-Groulx</t>
+  </si>
+  <si>
+    <t>Bibliothèques des lettres et sciences humaines; Bibliothèque des livres rares et collections spéciales; Service du prêt entre bibliothèques</t>
+  </si>
+  <si>
+    <t>Bibliothèques des lettres et sciences humaines; Service du prêt entre bibliothèques</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2275,7 +2275,7 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I99">
+  <sortState ref="A2:I99">
     <sortCondition ref="A1:A99"/>
   </sortState>
   <tableColumns count="9">
@@ -2294,9 +2294,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2334,9 +2334,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2369,9 +2369,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2404,9 +2421,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2581,7 +2615,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I99"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.42578125" customWidth="1"/>
     <col min="2" max="3" width="18.85546875" customWidth="1"/>
@@ -2593,36 +2627,36 @@
     <col min="9" max="9" width="75.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
+        <v>612</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>613</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>616</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>615</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>616</v>
-      </c>
-      <c r="C1" s="6" t="s">
+      <c r="E1" s="1" t="s">
+        <v>614</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>617</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>618</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>619</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>618</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>617</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>620</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>621</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>622</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>623</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="9" t="s">
         <v>8</v>
       </c>
@@ -2651,291 +2685,291 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9">
       <c r="A3" s="7" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>601</v>
       </c>
-      <c r="F3" s="7" t="s">
-        <v>440</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>602</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>603</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>604</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" s="7" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>30</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="C5" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>13</v>
       </c>
       <c r="G5" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="I5" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="I5" s="9" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>72</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>73</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>651</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>654</v>
-      </c>
-      <c r="G6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="I6" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="I6" s="7" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" s="9" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>17</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="B8" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="F8" t="s">
+        <v>183</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="I8" t="s">
         <v>577</v>
       </c>
-      <c r="F8" t="s">
-        <v>184</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>578</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>579</v>
-      </c>
-      <c r="I8" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" s="7" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="E9" s="17"/>
       <c r="F9" s="7" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>399</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="E10" s="12" t="s">
+        <v>660</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>400</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="G10" s="11" t="s">
         <v>401</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="H10" s="11" t="s">
         <v>402</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="I10" s="9" t="s">
         <v>403</v>
       </c>
-      <c r="F10" s="9" t="s">
-        <v>403</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>404</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>405</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="F11" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="G11" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="H11" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="I11" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="I11" s="9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="C12" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="D12" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="E12" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="F12" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="F12" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="G12" s="11" t="s">
+      <c r="H12" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="I12" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="I12" s="9" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13" s="9" t="s">
         <v>34</v>
       </c>
@@ -2964,12 +2998,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9">
       <c r="A14" s="9" t="s">
         <v>34</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="9" t="s">
@@ -2980,122 +3014,122 @@
         <v>13</v>
       </c>
       <c r="G14" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="H14" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="I14" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="I14" s="9" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:9">
       <c r="A15" s="7" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G15" s="7"/>
       <c r="H15" s="15" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
       <c r="A16" s="7" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>53</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="15" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="I16" s="15" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="B17" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="F17" t="s">
         <v>13</v>
       </c>
       <c r="G17" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="H17" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="I17" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" s="11" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C18" s="11"/>
       <c r="D18" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E18" s="11"/>
       <c r="F18" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="H18" s="11" t="s">
         <v>307</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="I18" s="11" t="s">
         <v>308</v>
       </c>
-      <c r="H18" s="11" t="s">
-        <v>309</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" s="7" t="s">
         <v>0</v>
       </c>
@@ -3109,7 +3143,7 @@
         <v>3</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>4</v>
@@ -3124,775 +3158,775 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9">
       <c r="A20" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="C20" s="9" t="s">
         <v>209</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>210</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>53</v>
       </c>
       <c r="E20" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="G20" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="F20" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="G20" s="9" t="s">
+      <c r="H20" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="I20" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="I20" s="9" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:9">
       <c r="A21" s="7" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
       <c r="A22" s="9" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="9" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>54</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
       <c r="A23" s="9" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="9" t="s">
         <v>17</v>
       </c>
       <c r="E23" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="G23" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="H23" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="I23" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="H23" s="9" t="s">
-        <v>280</v>
-      </c>
-      <c r="I23" s="9" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:9">
       <c r="A24" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>525</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>526</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="G24" s="9" t="s">
         <v>527</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="H24" s="9" t="s">
         <v>528</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="I24" s="9" t="s">
         <v>529</v>
       </c>
-      <c r="D24" s="9" t="s">
-        <v>402</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>307</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>530</v>
-      </c>
-      <c r="H24" s="9" t="s">
-        <v>531</v>
-      </c>
-      <c r="I24" s="9" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:9">
       <c r="A25" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>162</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>163</v>
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="E25" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="F25" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G25" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="F25" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="G25" s="7" t="s">
+      <c r="H25" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="H25" s="15" t="s">
+      <c r="I25" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="I25" s="15" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:9">
       <c r="A26" s="7" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G26" s="7"/>
       <c r="H26" s="15" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="I26" s="15" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
       <c r="A27" s="7" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="F27" s="7" t="s">
+        <v>520</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="I27" s="7" t="s">
         <v>523</v>
       </c>
-      <c r="G27" s="7" t="s">
-        <v>524</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>525</v>
-      </c>
-      <c r="I27" s="7" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:9">
       <c r="A28" s="9" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E28" s="13" t="s">
+        <v>502</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>503</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>504</v>
+      </c>
+      <c r="I28" s="9" t="s">
         <v>505</v>
       </c>
-      <c r="F28" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="G28" s="9" t="s">
-        <v>506</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>507</v>
-      </c>
-      <c r="I28" s="9" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:9">
       <c r="A29" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="B29" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="C29" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="D29" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="E29" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="F29" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G29" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="G29" s="7" t="s">
+      <c r="H29" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="H29" s="7" t="s">
+      <c r="I29" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="I29" s="7" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>443</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="E30" s="17" t="s">
         <v>444</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>445</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>446</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="E30" s="17" t="s">
-        <v>447</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
       <c r="A31" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="C31" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="D31" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E31" s="13" t="s">
         <v>236</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="E31" s="13" t="s">
-        <v>238</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>30</v>
       </c>
       <c r="G31" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="I31" s="14" t="s">
         <v>239</v>
       </c>
-      <c r="H31" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="I31" s="14" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:9">
       <c r="A32" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B32" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="C32" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="C32" s="7" t="s">
-        <v>87</v>
-      </c>
       <c r="D32" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E32" s="7"/>
       <c r="F32" s="7" t="s">
         <v>45</v>
       </c>
       <c r="G32" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="H32" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="H32" s="7" t="s">
+      <c r="I32" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="I32" s="15" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:9">
       <c r="A33" s="9" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
       <c r="A34" s="7" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
       <c r="A35" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="C35" s="7" t="s">
         <v>189</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>190</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>30</v>
       </c>
       <c r="G35" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="H35" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="H35" s="7" t="s">
+      <c r="I35" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="I35" s="7" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:9">
       <c r="A36" s="9" t="s">
+        <v>448</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>449</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="G36" s="9" t="s">
         <v>451</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="H36" s="9" t="s">
         <v>452</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="I36" s="9" t="s">
         <v>453</v>
       </c>
-      <c r="D36" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="G36" s="9" t="s">
-        <v>454</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>455</v>
-      </c>
-      <c r="I36" s="9" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:9">
       <c r="A37" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="C37" s="9" t="s">
         <v>287</v>
-      </c>
-      <c r="B37" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>289</v>
       </c>
       <c r="D37" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="F37" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="H37" s="9" t="s">
         <v>290</v>
       </c>
-      <c r="G37" s="9" t="s">
+      <c r="I37" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="H37" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="I37" s="9" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:9">
       <c r="A38" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="B38" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B38" s="9" t="s">
+      <c r="C38" s="9" t="s">
         <v>181</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>182</v>
       </c>
       <c r="D38" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E38" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="F38" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="F38" s="9" t="s">
+      <c r="G38" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="G38" s="9" t="s">
+      <c r="H38" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="H38" s="9" t="s">
+      <c r="I38" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="I38" s="9" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:9">
       <c r="A39" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B39" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>108</v>
       </c>
       <c r="C39" s="7"/>
       <c r="D39" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E39" s="7"/>
       <c r="F39" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G39" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="G39" s="7" t="s">
+      <c r="H39" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="H39" s="7" t="s">
+      <c r="I39" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="I39" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:9">
       <c r="A40" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="C40" s="7" t="s">
         <v>299</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>300</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>301</v>
       </c>
       <c r="D40" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G40" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="I40" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="H40" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="I40" s="7" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:9">
       <c r="A41" s="9" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>4</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
       <c r="A42" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B42" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="B42" s="9" t="s">
+      <c r="C42" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="C42" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="D42" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>30</v>
       </c>
       <c r="G42" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H42" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="H42" s="9" t="s">
+      <c r="I42" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="I42" s="9" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:9">
       <c r="A43" s="9" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E43" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="H43" s="9" t="s">
         <v>362</v>
       </c>
-      <c r="F43" s="9" t="s">
+      <c r="I43" s="9" t="s">
         <v>363</v>
       </c>
-      <c r="G43" s="9" t="s">
-        <v>364</v>
-      </c>
-      <c r="H43" s="9" t="s">
-        <v>365</v>
-      </c>
-      <c r="I43" s="9" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:9">
       <c r="A44" s="9" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="D44" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>30</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="I44" s="9" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
       <c r="A45" s="7" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="C45" s="15"/>
       <c r="D45" s="7" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="E45" s="17" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="G45" s="7"/>
       <c r="H45" s="7" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="I45" s="7"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9">
       <c r="A46" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B46" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="B46" s="9" t="s">
+      <c r="C46" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="C46" s="9" t="s">
-        <v>142</v>
       </c>
       <c r="D46" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>45</v>
       </c>
       <c r="G46" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="H46" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="H46" s="9" t="s">
+      <c r="I46" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="I46" s="9" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:9">
       <c r="A47" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B47" s="7" t="s">
         <v>176</v>
-      </c>
-      <c r="B47" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="C47" s="7"/>
       <c r="D47" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E47" s="7"/>
       <c r="F47" s="7" t="s">
@@ -3902,121 +3936,121 @@
         <v>5</v>
       </c>
       <c r="H47" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="I47" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="I47" s="7" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:9">
       <c r="A48" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B48" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="H48" s="7" t="s">
         <v>533</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="I48" s="7" t="s">
         <v>534</v>
       </c>
-      <c r="D48" s="7" t="s">
-        <v>535</v>
-      </c>
-      <c r="E48" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="F48" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="G48" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="H48" s="7" t="s">
-        <v>536</v>
-      </c>
-      <c r="I48" s="7" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:9">
       <c r="A49" s="9" t="s">
+        <v>384</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>386</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E49" s="13" t="s">
         <v>387</v>
       </c>
-      <c r="B49" s="9" t="s">
+      <c r="F49" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G49" s="9" t="s">
         <v>388</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="H49" s="9" t="s">
         <v>389</v>
       </c>
-      <c r="D49" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="E49" s="13" t="s">
+      <c r="I49" s="9" t="s">
         <v>390</v>
       </c>
-      <c r="F49" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="G49" s="9" t="s">
-        <v>391</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>392</v>
-      </c>
-      <c r="I49" s="9" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:9">
       <c r="A50" s="7" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C50" s="7"/>
       <c r="D50" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E50" s="7" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>30</v>
       </c>
       <c r="G50" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="H50" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="I50" s="7" t="s">
         <v>313</v>
       </c>
-      <c r="H50" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="I50" s="7" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:9">
       <c r="A51" s="7" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C51" s="7"/>
       <c r="D51" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="H51" s="7"/>
       <c r="I51" s="7"/>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9">
       <c r="A52" s="7" t="s">
         <v>41</v>
       </c>
@@ -4045,94 +4079,94 @@
         <v>48</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9">
       <c r="A53" s="9" t="s">
+        <v>485</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>486</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>487</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E53" s="9" t="s">
         <v>488</v>
-      </c>
-      <c r="B53" s="9" t="s">
-        <v>489</v>
-      </c>
-      <c r="C53" s="9" t="s">
-        <v>490</v>
-      </c>
-      <c r="D53" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="E53" s="9" t="s">
-        <v>491</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>30</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="H53" s="9" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="I53" s="9" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
       <c r="A54" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="B54" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="D54" t="s">
         <v>11</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="F54" t="s">
         <v>13</v>
       </c>
       <c r="G54" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="H54" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="I54" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9">
       <c r="A55" s="7" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="D55" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="I55" s="7" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9">
       <c r="A56" s="7" t="s">
         <v>26</v>
       </c>
@@ -4161,34 +4195,34 @@
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9">
       <c r="A57" s="9" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="9" t="s">
         <v>49</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="F57" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="H57" s="14" t="s">
+        <v>624</v>
+      </c>
+      <c r="I57" s="9" t="s">
         <v>296</v>
       </c>
-      <c r="G57" s="9" t="s">
-        <v>297</v>
-      </c>
-      <c r="H57" s="14" t="s">
-        <v>627</v>
-      </c>
-      <c r="I57" s="9" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:9">
       <c r="A58" s="9" t="s">
         <v>50</v>
       </c>
@@ -4205,222 +4239,222 @@
         <v>54</v>
       </c>
       <c r="F58" s="9" t="s">
+        <v>659</v>
+      </c>
+      <c r="G58" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="G58" s="9" t="s">
+      <c r="H58" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="H58" s="9" t="s">
+      <c r="I58" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="I58" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:9">
       <c r="A59" s="7" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="I59" s="7" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9">
       <c r="A60" s="9" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="D60" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="I60" s="9" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9">
       <c r="A61" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="C61" s="9" t="s">
         <v>265</v>
-      </c>
-      <c r="B61" s="9" t="s">
-        <v>266</v>
-      </c>
-      <c r="C61" s="9" t="s">
-        <v>267</v>
       </c>
       <c r="D61" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>30</v>
       </c>
       <c r="G61" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="H61" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="I61" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="H61" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="I61" s="9" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:9" s="4" customFormat="1">
       <c r="A62" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="C62" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="B62" s="9" t="s">
+      <c r="D62" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="C62" s="9" t="s">
+      <c r="E62" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="D62" s="9" t="s">
+      <c r="F62" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G62" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="E62" s="9" t="s">
+      <c r="H62" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="F62" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="G62" s="9" t="s">
+      <c r="I62" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="H62" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="I62" s="9" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:9">
       <c r="A63" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="E63" s="8" t="s">
         <v>367</v>
-      </c>
-      <c r="B63" s="7" t="s">
-        <v>368</v>
-      </c>
-      <c r="C63" s="7" t="s">
-        <v>369</v>
-      </c>
-      <c r="D63" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="E63" s="8" t="s">
-        <v>370</v>
       </c>
       <c r="F63" s="7" t="s">
         <v>4</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="I63" s="7" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" s="5" customFormat="1">
       <c r="A64" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="E64" s="9" t="s">
         <v>424</v>
       </c>
-      <c r="B64" s="9" t="s">
+      <c r="F64" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G64" s="9" t="s">
         <v>425</v>
       </c>
-      <c r="C64" s="9" t="s">
+      <c r="H64" s="9" t="s">
         <v>426</v>
       </c>
-      <c r="D64" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="E64" s="9" t="s">
+      <c r="I64" s="9" t="s">
         <v>427</v>
       </c>
-      <c r="F64" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="G64" s="9" t="s">
-        <v>428</v>
-      </c>
-      <c r="H64" s="9" t="s">
-        <v>429</v>
-      </c>
-      <c r="I64" s="9" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:9">
       <c r="A65" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B65" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="B65" s="7" t="s">
+      <c r="C65" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="C65" s="7" t="s">
+      <c r="D65" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="D65" s="7" t="s">
+      <c r="E65" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="E65" s="7" t="s">
+      <c r="F65" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="F65" s="7" t="s">
+      <c r="G65" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="G65" s="7" t="s">
+      <c r="H65" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="H65" s="7" t="s">
+      <c r="I65" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="I65" s="7" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:9">
       <c r="A66" s="11" t="s">
         <v>20</v>
       </c>
@@ -4432,10 +4466,10 @@
         <v>22</v>
       </c>
       <c r="E66" s="12" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="G66" s="11" t="s">
         <v>23</v>
@@ -4447,12 +4481,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9">
       <c r="A67" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C67" s="7"/>
       <c r="D67" s="7" t="s">
@@ -4460,606 +4494,606 @@
       </c>
       <c r="E67" s="7"/>
       <c r="F67" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G67" s="7"/>
       <c r="H67" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="I67" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="I67" s="7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:9">
       <c r="A68" s="7" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="C68" s="7"/>
       <c r="D68" s="7" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="E68" s="17"/>
       <c r="F68" s="7" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="G68" s="16" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H68" s="15" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="I68" s="16"/>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9">
       <c r="A69" s="7" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="D69" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="F69" s="7" t="s">
         <v>30</v>
       </c>
       <c r="G69" s="7" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="I69" s="7" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9">
       <c r="A70" s="7" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="D70" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="F70" s="7" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G70" s="7" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="H70" s="7" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="I70" s="7" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" s="4" customFormat="1">
       <c r="A71" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="C71" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="B71" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="C71" s="7" t="s">
-        <v>244</v>
       </c>
       <c r="D71" s="7" t="s">
         <v>22</v>
       </c>
       <c r="E71" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="F71" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="G71" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="H71" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="F71" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="G71" s="7" t="s">
+      <c r="I71" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="H71" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="I71" s="7" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:9">
       <c r="A72" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B72" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="B72" s="7" t="s">
+      <c r="C72" s="7" t="s">
         <v>133</v>
-      </c>
-      <c r="C72" s="7" t="s">
-        <v>134</v>
       </c>
       <c r="D72" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E72" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="F72" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="F72" s="7" t="s">
+      <c r="G72" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="G72" s="7" t="s">
+      <c r="H72" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="H72" s="7" t="s">
+      <c r="I72" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="I72" s="7" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:9">
       <c r="A73" s="16" t="s">
+        <v>255</v>
+      </c>
+      <c r="B73" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="C73" s="16" t="s">
         <v>257</v>
-      </c>
-      <c r="B73" s="16" t="s">
-        <v>258</v>
-      </c>
-      <c r="C73" s="16" t="s">
-        <v>259</v>
       </c>
       <c r="D73" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E73" s="16" t="s">
+        <v>258</v>
+      </c>
+      <c r="F73" s="16" t="s">
+        <v>259</v>
+      </c>
+      <c r="G73" s="16" t="s">
         <v>260</v>
       </c>
-      <c r="F73" s="16" t="s">
+      <c r="H73" s="16" t="s">
         <v>261</v>
       </c>
-      <c r="G73" s="16" t="s">
+      <c r="I73" s="16" t="s">
         <v>262</v>
       </c>
-      <c r="H73" s="16" t="s">
-        <v>263</v>
-      </c>
-      <c r="I73" s="16" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:9" s="4" customFormat="1">
       <c r="A74" s="9" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="C74" s="9" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="D74" s="9" t="s">
         <v>53</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F74" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="I74" s="9" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9">
       <c r="A75" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B75" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B75" s="9" t="s">
+      <c r="C75" s="9" t="s">
         <v>64</v>
-      </c>
-      <c r="C75" s="9" t="s">
-        <v>65</v>
       </c>
       <c r="D75" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E75" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="F75" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="F75" s="9" t="s">
+      <c r="G75" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G75" s="9" t="s">
+      <c r="H75" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="H75" s="9" t="s">
+      <c r="I75" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="I75" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:9">
       <c r="A76" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="B76" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="C76" s="16" t="s">
         <v>228</v>
       </c>
-      <c r="B76" s="16" t="s">
+      <c r="D76" s="16" t="s">
         <v>229</v>
       </c>
-      <c r="C76" s="16" t="s">
+      <c r="E76" s="8" t="s">
+        <v>647</v>
+      </c>
+      <c r="F76" s="16" t="s">
+        <v>651</v>
+      </c>
+      <c r="G76" s="16" t="s">
         <v>230</v>
       </c>
-      <c r="D76" s="16" t="s">
+      <c r="H76" s="16" t="s">
         <v>231</v>
       </c>
-      <c r="E76" s="8" t="s">
-        <v>650</v>
-      </c>
-      <c r="F76" s="16" t="s">
-        <v>654</v>
-      </c>
-      <c r="G76" s="16" t="s">
+      <c r="I76" s="16" t="s">
         <v>232</v>
       </c>
-      <c r="H76" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="I76" s="16" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:9">
       <c r="A77" s="9" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="B77" s="9" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>347</v>
+      </c>
+      <c r="F77" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="G77" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="H77" s="9" t="s">
         <v>349</v>
       </c>
-      <c r="E77" s="9" t="s">
+      <c r="I77" s="9" t="s">
         <v>350</v>
       </c>
-      <c r="F77" s="9" t="s">
-        <v>307</v>
-      </c>
-      <c r="G77" s="9" t="s">
-        <v>351</v>
-      </c>
-      <c r="H77" s="9" t="s">
-        <v>352</v>
-      </c>
-      <c r="I77" s="9" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:9">
       <c r="A78" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="B78" s="9" t="s">
         <v>222</v>
-      </c>
-      <c r="B78" s="9" t="s">
-        <v>223</v>
       </c>
       <c r="C78" s="9"/>
       <c r="D78" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E78" s="9"/>
       <c r="F78" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G78" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="H78" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="G78" s="9" t="s">
+      <c r="I78" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="H78" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="I78" s="9" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:9">
       <c r="A79" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="B79" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="C79" s="9" t="s">
         <v>316</v>
-      </c>
-      <c r="B79" s="9" t="s">
-        <v>317</v>
-      </c>
-      <c r="C79" s="9" t="s">
-        <v>318</v>
       </c>
       <c r="D79" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E79" s="11" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="F79" s="9" t="s">
+        <v>661</v>
+      </c>
+      <c r="G79" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="H79" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="I79" s="9" t="s">
         <v>319</v>
       </c>
-      <c r="G79" s="9" t="s">
-        <v>320</v>
-      </c>
-      <c r="H79" s="9" t="s">
-        <v>321</v>
-      </c>
-      <c r="I79" s="9" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:9">
       <c r="A80" s="9" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="C80" s="9"/>
       <c r="D80" s="9" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="E80" s="13"/>
       <c r="F80" s="9" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="G80" s="9"/>
       <c r="H80" s="9" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="I80" s="18"/>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9">
       <c r="A81" t="s">
+        <v>589</v>
+      </c>
+      <c r="B81" t="s">
+        <v>590</v>
+      </c>
+      <c r="C81" s="22" t="s">
+        <v>591</v>
+      </c>
+      <c r="D81" t="s">
+        <v>194</v>
+      </c>
+      <c r="E81" s="3" t="s">
         <v>592</v>
       </c>
-      <c r="B81" t="s">
+      <c r="F81" t="s">
+        <v>59</v>
+      </c>
+      <c r="H81" t="s">
         <v>593</v>
       </c>
-      <c r="C81" s="22" t="s">
+      <c r="I81" t="s">
         <v>594</v>
       </c>
-      <c r="D81" t="s">
-        <v>195</v>
-      </c>
-      <c r="E81" s="3" t="s">
-        <v>595</v>
-      </c>
-      <c r="F81" t="s">
-        <v>60</v>
-      </c>
-      <c r="H81" t="s">
-        <v>596</v>
-      </c>
-      <c r="I81" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:9">
       <c r="A82" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B82" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C82" s="7" t="s">
         <v>216</v>
-      </c>
-      <c r="B82" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="C82" s="7" t="s">
-        <v>217</v>
       </c>
       <c r="D82" s="7" t="s">
         <v>53</v>
       </c>
       <c r="E82" s="17" t="s">
+        <v>217</v>
+      </c>
+      <c r="F82" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G82" s="16" t="s">
         <v>218</v>
       </c>
-      <c r="F82" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G82" s="16" t="s">
+      <c r="H82" s="16" t="s">
         <v>219</v>
       </c>
-      <c r="H82" s="16" t="s">
+      <c r="I82" s="16" t="s">
         <v>220</v>
       </c>
-      <c r="I82" s="16" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:9">
       <c r="A83" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B83" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B83" s="7" t="s">
+      <c r="C83" s="7" t="s">
         <v>96</v>
-      </c>
-      <c r="C83" s="7" t="s">
-        <v>97</v>
       </c>
       <c r="D83" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E83" s="7" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="F83" s="7" t="s">
         <v>30</v>
       </c>
       <c r="G83" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="H83" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="H83" s="16" t="s">
+      <c r="I83" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="I83" s="16" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="84" spans="1:9">
       <c r="A84" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B84" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="C84" s="9" t="s">
         <v>156</v>
-      </c>
-      <c r="C84" s="9" t="s">
-        <v>157</v>
       </c>
       <c r="D84" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E84" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>30</v>
       </c>
       <c r="G84" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H84" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="H84" s="11" t="s">
+      <c r="I84" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="I84" s="11" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:9">
       <c r="A85" s="7" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="D85" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E85" s="7" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="F85" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="H85" s="16" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="I85" s="16" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9">
       <c r="A86" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="B86" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="C86" s="7" t="s">
+        <v>406</v>
+      </c>
+      <c r="D86" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="E86" s="17" t="s">
         <v>407</v>
       </c>
-      <c r="B86" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="C86" s="7" t="s">
-        <v>409</v>
-      </c>
-      <c r="D86" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="E86" s="17" t="s">
-        <v>410</v>
-      </c>
       <c r="F86" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G86" s="16"/>
       <c r="H86" s="15" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="I86" s="16" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9">
       <c r="A87" s="9" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="B87" s="9" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="C87" s="9" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="D87" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E87" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="F87" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="G87" s="11" t="s">
+        <v>375</v>
+      </c>
+      <c r="H87" s="11" t="s">
+        <v>376</v>
+      </c>
+      <c r="I87" s="11" t="s">
         <v>377</v>
       </c>
-      <c r="F87" s="9" t="s">
-        <v>296</v>
-      </c>
-      <c r="G87" s="11" t="s">
-        <v>378</v>
-      </c>
-      <c r="H87" s="11" t="s">
-        <v>379</v>
-      </c>
-      <c r="I87" s="11" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:9">
       <c r="A88" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="B88" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="C88" s="22" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="D88" t="s">
         <v>11</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F88" t="s">
         <v>30</v>
       </c>
       <c r="G88" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="H88" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="I88" s="4" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9">
+      <c r="A89" t="s">
         <v>584</v>
       </c>
-      <c r="H88" s="4" t="s">
+      <c r="B89" t="s">
         <v>585</v>
-      </c>
-      <c r="I88" s="4" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>587</v>
-      </c>
-      <c r="B89" t="s">
-        <v>588</v>
       </c>
       <c r="C89" s="19"/>
       <c r="D89" t="s">
@@ -5072,287 +5106,287 @@
         <v>13</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" s="4" customFormat="1">
       <c r="A90" s="7" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="B90" s="7" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="D90" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E90" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F90" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G90" s="16" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="H90" s="16" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="I90" s="16" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" s="4" customFormat="1">
       <c r="A91" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B91" s="7" t="s">
         <v>119</v>
-      </c>
-      <c r="B91" s="7" t="s">
-        <v>120</v>
       </c>
       <c r="C91" s="7"/>
       <c r="D91" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E91" s="17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F91" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G91" s="16"/>
       <c r="H91" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="I91" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="I91" s="16" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:9">
       <c r="A92" s="11" t="s">
+        <v>602</v>
+      </c>
+      <c r="B92" s="11" t="s">
+        <v>596</v>
+      </c>
+      <c r="C92" s="9" t="s">
+        <v>603</v>
+      </c>
+      <c r="D92" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="E92" s="11" t="s">
+        <v>604</v>
+      </c>
+      <c r="F92" s="11" t="s">
         <v>605</v>
       </c>
-      <c r="B92" s="11" t="s">
-        <v>599</v>
-      </c>
-      <c r="C92" s="9" t="s">
+      <c r="G92" s="11" t="s">
         <v>606</v>
       </c>
-      <c r="D92" s="11" t="s">
-        <v>195</v>
-      </c>
-      <c r="E92" s="11" t="s">
+      <c r="H92" s="11" t="s">
         <v>607</v>
       </c>
-      <c r="F92" s="11" t="s">
+      <c r="I92" s="11" t="s">
         <v>608</v>
       </c>
-      <c r="G92" s="11" t="s">
-        <v>609</v>
-      </c>
-      <c r="H92" s="11" t="s">
-        <v>610</v>
-      </c>
-      <c r="I92" s="11" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="93" spans="1:9">
       <c r="A93" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C93" s="23"/>
       <c r="D93" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E93" s="11"/>
       <c r="F93" s="11" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="G93" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="H93" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="H93" s="11" t="s">
+      <c r="I93" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="I93" s="11" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:9">
       <c r="A94" s="7" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C94" s="20"/>
       <c r="D94" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E94" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="F94" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G94" s="7" t="s">
+        <v>418</v>
+      </c>
+      <c r="H94" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="I94" s="7" t="s">
         <v>420</v>
       </c>
-      <c r="F94" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G94" s="7" t="s">
-        <v>421</v>
-      </c>
-      <c r="H94" s="7" t="s">
-        <v>422</v>
-      </c>
-      <c r="I94" s="7" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:9">
       <c r="A95" s="16" t="s">
+        <v>454</v>
+      </c>
+      <c r="B95" s="16" t="s">
+        <v>455</v>
+      </c>
+      <c r="C95" s="20" t="s">
+        <v>456</v>
+      </c>
+      <c r="D95" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="E95" s="16" t="s">
         <v>457</v>
       </c>
-      <c r="B95" s="16" t="s">
+      <c r="F95" s="16" t="s">
+        <v>648</v>
+      </c>
+      <c r="G95" s="16" t="s">
         <v>458</v>
       </c>
-      <c r="C95" s="20" t="s">
+      <c r="H95" s="16" t="s">
         <v>459</v>
       </c>
-      <c r="D95" s="16" t="s">
-        <v>362</v>
-      </c>
-      <c r="E95" s="16" t="s">
+      <c r="I95" s="16" t="s">
         <v>460</v>
       </c>
-      <c r="F95" s="16" t="s">
-        <v>651</v>
-      </c>
-      <c r="G95" s="16" t="s">
-        <v>461</v>
-      </c>
-      <c r="H95" s="16" t="s">
-        <v>462</v>
-      </c>
-      <c r="I95" s="16" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="96" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:9" s="5" customFormat="1">
       <c r="A96" s="9" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="B96" s="9" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C96" s="21" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="D96" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E96" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F96" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="H96" s="9" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="I96" s="9" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9">
       <c r="A97" s="7" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="B97" s="7" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="C97" s="20"/>
       <c r="D97" s="7" t="s">
         <v>53</v>
       </c>
       <c r="E97" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="F97" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="G97" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="H97" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="I97" s="7" t="s">
         <v>325</v>
       </c>
-      <c r="F97" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="G97" s="7" t="s">
-        <v>326</v>
-      </c>
-      <c r="H97" s="7" t="s">
-        <v>327</v>
-      </c>
-      <c r="I97" s="7" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:9">
       <c r="A98" s="7" t="s">
+        <v>378</v>
+      </c>
+      <c r="B98" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="C98" s="20" t="s">
+        <v>380</v>
+      </c>
+      <c r="D98" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="E98" s="17" t="s">
         <v>381</v>
       </c>
-      <c r="B98" s="7" t="s">
-        <v>382</v>
-      </c>
-      <c r="C98" s="20" t="s">
-        <v>383</v>
-      </c>
-      <c r="D98" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="E98" s="17" t="s">
-        <v>384</v>
-      </c>
       <c r="F98" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G98" s="7"/>
       <c r="H98" s="7" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I98" s="7" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9">
       <c r="A99" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C99" s="9"/>
       <c r="D99" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E99" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="E99" s="9" t="s">
+      <c r="F99" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G99" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="F99" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="G99" s="9" t="s">
+      <c r="H99" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="H99" s="9" t="s">
+      <c r="I99" s="14" t="s">
         <v>198</v>
-      </c>
-      <c r="I99" s="14" t="s">
-        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -5385,6 +5419,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f6670ae2-8190-4e72-909e-d717fe03ced5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="00db0817-461a-4a69-8eb5-8daf0756d296" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007812637FDE95774892D21861907C1625" ma:contentTypeVersion="15" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="9e26b686a71b543072340cfd27a56c29">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f6670ae2-8190-4e72-909e-d717fe03ced5" xmlns:ns3="00db0817-461a-4a69-8eb5-8daf0756d296" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8d151e41c23af60827e9e8828a6e0ebd" ns2:_="" ns3:_="">
     <xsd:import namespace="f6670ae2-8190-4e72-909e-d717fe03ced5"/>
@@ -5619,27 +5673,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="f6670ae2-8190-4e72-909e-d717fe03ced5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="00db0817-461a-4a69-8eb5-8daf0756d296"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f6670ae2-8190-4e72-909e-d717fe03ced5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="00db0817-461a-4a69-8eb5-8daf0756d296" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{141ACCEB-C60B-4854-82C0-9885432D8ACB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5656,29 +5715,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="f6670ae2-8190-4e72-909e-d717fe03ced5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="00db0817-461a-4a69-8eb5-8daf0756d296"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Liste du personnel à jour
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://udemontreal-my.sharepoint.com/personal/mathieu_nicolas_tardif_umontreal_ca/Documents/Bibliothèques/Site Web/Photos-employés-FEV-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E5DA5A0-0C4D-4454-9349-D442C5A6701D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{1E5DA5A0-0C4D-4454-9349-D442C5A6701D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE9CD409-3908-4245-8930-FBB9970F7CEB}"/>
   <bookViews>
-    <workbookView xWindow="4640" yWindow="4640" windowWidth="43200" windowHeight="23450" tabRatio="149" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19455" yWindow="4650" windowWidth="20475" windowHeight="23445" tabRatio="149" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="813">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="831">
   <si>
     <t>nom</t>
   </si>
@@ -854,9 +854,6 @@
     <t>Marc-Olivier</t>
   </si>
   <si>
-    <t>marc-olirier-croteau.jpg</t>
-  </si>
-  <si>
     <t>Psychologie, communication, journalisme</t>
   </si>
   <si>
@@ -1532,9 +1529,6 @@
     <t>Maude</t>
   </si>
   <si>
-    <t>maude-de-lethiecq-normand.jpg</t>
-  </si>
-  <si>
     <t>514-343-6111, poste 1817</t>
   </si>
   <si>
@@ -1913,9 +1907,6 @@
     <t>Ève</t>
   </si>
   <si>
-    <t>eve-paquette-gigras.jpg</t>
-  </si>
-  <si>
     <t>Gestion des données de recherche</t>
   </si>
   <si>
@@ -2487,13 +2478,76 @@
   </si>
   <si>
     <t>yan-vallee.jpg</t>
+  </si>
+  <si>
+    <t>amelie-bernard.jpg</t>
+  </si>
+  <si>
+    <t>amelie-elizabeth-levesque.jpg</t>
+  </si>
+  <si>
+    <t>anny-levesque.jpg</t>
+  </si>
+  <si>
+    <t>chantal-desrosiers.jpg</t>
+  </si>
+  <si>
+    <t>eve-paquette-bigras.jpg</t>
+  </si>
+  <si>
+    <t>jason-madooray.jpg</t>
+  </si>
+  <si>
+    <t>jeremy-prime.jpg</t>
+  </si>
+  <si>
+    <t>jessica-legault.jpg</t>
+  </si>
+  <si>
+    <t>josee-viel.jpg</t>
+  </si>
+  <si>
+    <t>judith-fafard-larose.jpg</t>
+  </si>
+  <si>
+    <t>julie-trepanier.jpg</t>
+  </si>
+  <si>
+    <t>ly-kieng-tir.jpg</t>
+  </si>
+  <si>
+    <t>magdalena-oriental.jpg</t>
+  </si>
+  <si>
+    <t>marc-olivier-croteau.jpg</t>
+  </si>
+  <si>
+    <t>marie-france-laliberte.jpg</t>
+  </si>
+  <si>
+    <t>marie-pierre-gadoua.jpg</t>
+  </si>
+  <si>
+    <t>maude-lethiecq-normand.jpg</t>
+  </si>
+  <si>
+    <t>melanie-lachapelle.jpg</t>
+  </si>
+  <si>
+    <t>nathalie-poulin.jpg</t>
+  </si>
+  <si>
+    <t>vanessa-martin.jpg</t>
+  </si>
+  <si>
+    <t>yacine-mansar.jpg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2648,7 +2702,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2686,6 +2740,8 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
@@ -2789,7 +2845,7 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J129" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:J129" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
-  <sortState ref="A2:J129">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J129">
     <sortCondition ref="A1:A129"/>
   </sortState>
   <tableColumns count="10">
@@ -2809,9 +2865,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2849,9 +2905,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2884,26 +2940,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2936,26 +2975,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3130,21 +3152,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J129"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.453125" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="38.453125" customWidth="1"/>
-    <col min="4" max="4" width="28.1796875" customWidth="1"/>
-    <col min="5" max="5" width="83.453125" customWidth="1"/>
-    <col min="6" max="6" width="75.54296875" customWidth="1"/>
-    <col min="7" max="7" width="128.7265625" customWidth="1"/>
-    <col min="8" max="8" width="31.7265625" customWidth="1"/>
-    <col min="9" max="9" width="78.7265625" customWidth="1"/>
-    <col min="10" max="10" width="20.81640625" customWidth="1"/>
+    <col min="3" max="3" width="38.42578125" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" customWidth="1"/>
+    <col min="5" max="5" width="83.42578125" customWidth="1"/>
+    <col min="6" max="6" width="75.5703125" customWidth="1"/>
+    <col min="7" max="7" width="128.7109375" customWidth="1"/>
+    <col min="8" max="8" width="31.7109375" customWidth="1"/>
+    <col min="9" max="9" width="78.7109375" customWidth="1"/>
+    <col min="10" max="10" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3176,7 +3198,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>10</v>
       </c>
@@ -3206,7 +3228,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>19</v>
       </c>
@@ -3223,7 +3245,7 @@
         <v>46</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>22</v>
@@ -3238,7 +3260,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>26</v>
       </c>
@@ -3268,7 +3290,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>35</v>
       </c>
@@ -3298,7 +3320,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>42</v>
       </c>
@@ -3318,7 +3340,7 @@
         <v>47</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>48</v>
@@ -3330,7 +3352,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>51</v>
       </c>
@@ -3360,15 +3382,15 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="B8" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
       <c r="D8" t="s">
         <v>108</v>
@@ -3377,19 +3399,19 @@
         <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
       </c>
       <c r="H8" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="I8" s="28" t="s">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>59</v>
       </c>
@@ -3418,7 +3440,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>67</v>
       </c>
@@ -3445,7 +3467,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>75</v>
       </c>
@@ -3462,10 +3484,10 @@
         <v>79</v>
       </c>
       <c r="F11" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>80</v>
@@ -3477,7 +3499,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>83</v>
       </c>
@@ -3485,7 +3507,7 @@
         <v>43</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>84</v>
@@ -3506,7 +3528,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>90</v>
       </c>
@@ -3535,7 +3557,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>99</v>
       </c>
@@ -3565,14 +3587,16 @@
         <v>105</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>106</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C15" s="8"/>
+      <c r="C15" s="8" t="s">
+        <v>810</v>
+      </c>
       <c r="D15" s="8" t="s">
         <v>108</v>
       </c>
@@ -3589,7 +3613,7 @@
       </c>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>112</v>
       </c>
@@ -3617,7 +3641,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>112</v>
       </c>
@@ -3625,7 +3649,7 @@
         <v>118</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
       <c r="D17" t="s">
         <v>108</v>
@@ -3643,7 +3667,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>122</v>
       </c>
@@ -3673,7 +3697,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>129</v>
       </c>
@@ -3702,7 +3726,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>136</v>
       </c>
@@ -3727,7 +3751,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>142</v>
       </c>
@@ -3756,7 +3780,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>151</v>
       </c>
@@ -3786,7 +3810,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>159</v>
       </c>
@@ -3816,7 +3840,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>166</v>
       </c>
@@ -3824,7 +3848,7 @@
         <v>167</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>168</v>
@@ -3833,10 +3857,10 @@
         <v>85</v>
       </c>
       <c r="F24" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="H24" s="8" t="s">
         <v>169</v>
@@ -3848,7 +3872,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>172</v>
       </c>
@@ -3856,7 +3880,7 @@
         <v>173</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>54</v>
@@ -3866,7 +3890,7 @@
         <v>174</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="H25" s="8" t="s">
         <v>175</v>
@@ -3878,7 +3902,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>178</v>
       </c>
@@ -3905,7 +3929,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>184</v>
       </c>
@@ -3913,7 +3937,7 @@
         <v>185</v>
       </c>
       <c r="C27" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="D27" t="s">
         <v>108</v>
@@ -3931,7 +3955,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>189</v>
       </c>
@@ -3939,7 +3963,7 @@
         <v>190</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>191</v>
@@ -3961,7 +3985,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>197</v>
       </c>
@@ -3969,7 +3993,7 @@
         <v>198</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>54</v>
@@ -3991,7 +4015,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>204</v>
       </c>
@@ -4021,7 +4045,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>211</v>
       </c>
@@ -4029,7 +4053,7 @@
         <v>212</v>
       </c>
       <c r="C31" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="D31" t="s">
         <v>29</v>
@@ -4041,7 +4065,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>213</v>
       </c>
@@ -4052,7 +4076,7 @@
         <v>54</v>
       </c>
       <c r="G32" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="H32" s="8" t="s">
         <v>215</v>
@@ -4064,7 +4088,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="33" spans="1:10">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>218</v>
       </c>
@@ -4083,7 +4107,7 @@
       <c r="I33" s="13"/>
       <c r="J33" s="20"/>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>221</v>
       </c>
@@ -4113,7 +4137,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>228</v>
       </c>
@@ -4142,7 +4166,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>236</v>
       </c>
@@ -4172,7 +4196,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
         <v>243</v>
       </c>
@@ -4202,7 +4226,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>250</v>
       </c>
@@ -4222,7 +4246,7 @@
         <v>255</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>256</v>
@@ -4234,7 +4258,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
         <v>259</v>
       </c>
@@ -4264,7 +4288,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>266</v>
       </c>
@@ -4272,183 +4296,185 @@
         <v>267</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>268</v>
+        <v>823</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E40" s="6"/>
       <c r="F40" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G40" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H40" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="I40" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="I40" s="6" t="s">
+      <c r="J40" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="J40" s="6" t="s">
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="41" spans="1:10">
-      <c r="A41" s="6" t="s">
+      <c r="B41" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="C41" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>275</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E41" s="6"/>
       <c r="F41" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G41" s="6" t="s">
         <v>31</v>
       </c>
       <c r="H41" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="I41" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="I41" s="6" t="s">
+      <c r="J41" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="J41" s="6" t="s">
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="8" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="42" spans="1:10">
-      <c r="A42" s="8" t="s">
+      <c r="B42" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="C42" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="D42" s="8" t="s">
         <v>282</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>283</v>
       </c>
       <c r="E42" s="6"/>
       <c r="F42" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="G42" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="H42" s="8" t="s">
         <v>285</v>
       </c>
-      <c r="G42" s="8" t="s">
-        <v>284</v>
-      </c>
-      <c r="H42" s="8" t="s">
+      <c r="I42" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="I42" s="8" t="s">
+      <c r="J42" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="J42" s="8" t="s">
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" s="8" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="43" spans="1:10">
-      <c r="A43" s="8" t="s">
+      <c r="B43" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="C43" s="8" t="s">
         <v>290</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>291</v>
       </c>
       <c r="D43" s="8" t="s">
         <v>13</v>
       </c>
       <c r="E43" s="8"/>
       <c r="F43" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="G43" s="8" t="s">
+        <v>765</v>
+      </c>
+      <c r="H43" s="8" t="s">
         <v>292</v>
       </c>
-      <c r="G43" s="8" t="s">
-        <v>768</v>
-      </c>
-      <c r="H43" s="8" t="s">
+      <c r="I43" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="I43" s="8" t="s">
+      <c r="J43" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="J43" s="8" t="s">
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" s="8" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="44" spans="1:10">
-      <c r="A44" s="8" t="s">
+      <c r="B44" s="8" t="s">
         <v>296</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="C44" s="8" t="s">
         <v>297</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>298</v>
       </c>
       <c r="D44" s="8" t="s">
         <v>13</v>
       </c>
       <c r="E44" s="8"/>
       <c r="F44" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G44" s="8" t="s">
         <v>63</v>
       </c>
       <c r="H44" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="I44" s="8" t="s">
         <v>300</v>
       </c>
-      <c r="I44" s="8" t="s">
+      <c r="J44" s="8" t="s">
         <v>301</v>
       </c>
-      <c r="J44" s="8" t="s">
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="45" spans="1:10">
-      <c r="A45" s="6" t="s">
+      <c r="B45" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="C45" s="6" t="s">
+        <v>813</v>
+      </c>
+      <c r="D45" s="6" t="s">
         <v>304</v>
-      </c>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6" t="s">
-        <v>305</v>
       </c>
       <c r="E45" s="6"/>
       <c r="F45" s="6"/>
       <c r="G45" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="H45" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="H45" s="6" t="s">
+      <c r="I45" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="I45" s="6" t="s">
+      <c r="J45" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="J45" s="6" t="s">
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="46" spans="1:10">
-      <c r="A46" t="s">
+      <c r="B46" t="s">
         <v>310</v>
       </c>
-      <c r="B46" t="s">
-        <v>311</v>
-      </c>
       <c r="C46" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
       <c r="D46" t="s">
         <v>108</v>
@@ -4457,53 +4483,55 @@
         <v>31</v>
       </c>
       <c r="H46" s="10" t="s">
+        <v>311</v>
+      </c>
+      <c r="I46" s="18" t="s">
         <v>312</v>
       </c>
-      <c r="I46" s="18" t="s">
+      <c r="J46" s="18" t="s">
         <v>313</v>
       </c>
-      <c r="J46" s="18" t="s">
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="47" spans="1:10">
-      <c r="A47" s="6" t="s">
+      <c r="B47" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="C47" s="6" t="s">
         <v>316</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>317</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E47" s="6"/>
       <c r="F47" s="6" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>63</v>
       </c>
       <c r="H47" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="I47" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="I47" s="6" t="s">
+      <c r="J47" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="J47" s="6" t="s">
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="48" spans="1:10">
-      <c r="A48" t="s">
+      <c r="B48" t="s">
         <v>322</v>
       </c>
-      <c r="B48" t="s">
-        <v>323</v>
-      </c>
-      <c r="C48" s="6"/>
+      <c r="C48" s="6" t="s">
+        <v>819</v>
+      </c>
       <c r="D48" t="s">
         <v>108</v>
       </c>
@@ -4511,24 +4539,24 @@
         <v>31</v>
       </c>
       <c r="H48" t="s">
+        <v>323</v>
+      </c>
+      <c r="I48" s="18" t="s">
         <v>324</v>
       </c>
-      <c r="I48" s="18" t="s">
+      <c r="J48" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="J48" s="18" t="s">
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" s="8" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="49" spans="1:10">
-      <c r="A49" s="8" t="s">
+      <c r="B49" s="8" t="s">
         <v>327</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="C49" s="29" t="s">
         <v>328</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>329</v>
       </c>
       <c r="D49" s="8" t="s">
         <v>168</v>
@@ -4543,60 +4571,60 @@
         <v>147</v>
       </c>
       <c r="H49" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="I49" s="8" t="s">
         <v>330</v>
       </c>
-      <c r="I49" s="8" t="s">
+      <c r="J49" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="J49" s="8" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10">
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="B50" s="8" t="s">
         <v>327</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="C50" s="29" t="s">
         <v>328</v>
       </c>
-      <c r="C50" s="6" t="s">
-        <v>329</v>
-      </c>
       <c r="D50" s="8" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>146</v>
       </c>
       <c r="F50" s="8"/>
       <c r="G50" s="8" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="H50" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="I50" s="8" t="s">
         <v>330</v>
       </c>
-      <c r="I50" s="8" t="s">
+      <c r="J50" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="J50" s="8" t="s">
+    </row>
+    <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A51" s="8" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="51" spans="1:10">
-      <c r="A51" s="8" t="s">
+      <c r="B51" s="8" t="s">
         <v>333</v>
       </c>
-      <c r="B51" s="8" t="s">
+      <c r="C51" s="8" t="s">
         <v>334</v>
-      </c>
-      <c r="C51" s="8" t="s">
-        <v>335</v>
       </c>
       <c r="D51" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F51" s="8" t="s">
         <v>47</v>
@@ -4605,21 +4633,21 @@
         <v>31</v>
       </c>
       <c r="H51" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="I51" s="8" t="s">
         <v>337</v>
       </c>
-      <c r="I51" s="8" t="s">
+      <c r="J51" s="8" t="s">
         <v>338</v>
       </c>
-      <c r="J51" s="8" t="s">
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" s="8" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="52" spans="1:10">
-      <c r="A52" s="8" t="s">
+      <c r="B52" s="8" t="s">
         <v>340</v>
-      </c>
-      <c r="B52" s="8" t="s">
-        <v>341</v>
       </c>
       <c r="C52" s="8"/>
       <c r="D52" s="8" t="s">
@@ -4627,113 +4655,115 @@
       </c>
       <c r="E52" s="8"/>
       <c r="F52" s="8" t="s">
+        <v>341</v>
+      </c>
+      <c r="G52" s="8" t="s">
         <v>342</v>
       </c>
-      <c r="G52" s="8" t="s">
+      <c r="H52" s="8" t="s">
         <v>343</v>
       </c>
-      <c r="H52" s="8" t="s">
+      <c r="I52" s="8" t="s">
         <v>344</v>
       </c>
-      <c r="I52" s="8" t="s">
+      <c r="J52" s="8" t="s">
         <v>345</v>
       </c>
-      <c r="J52" s="8" t="s">
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" s="8" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="53" spans="1:10">
-      <c r="A53" s="8" t="s">
+      <c r="B53" s="8" t="s">
         <v>347</v>
       </c>
-      <c r="B53" s="8" t="s">
+      <c r="C53" s="8" t="s">
         <v>348</v>
-      </c>
-      <c r="C53" s="8" t="s">
-        <v>349</v>
       </c>
       <c r="D53" s="8" t="s">
         <v>13</v>
       </c>
       <c r="E53" s="8"/>
       <c r="F53" s="11" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="G53" s="8" t="s">
         <v>31</v>
       </c>
       <c r="H53" s="8" t="s">
+        <v>350</v>
+      </c>
+      <c r="I53" s="8" t="s">
         <v>351</v>
       </c>
-      <c r="I53" s="8" t="s">
+      <c r="J53" s="8" t="s">
         <v>352</v>
       </c>
-      <c r="J53" s="8" t="s">
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="54" spans="1:10">
-      <c r="A54" s="6" t="s">
+      <c r="B54" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="C54" s="6" t="s">
+        <v>825</v>
+      </c>
+      <c r="D54" s="6" t="s">
         <v>355</v>
-      </c>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6" t="s">
-        <v>356</v>
       </c>
       <c r="E54" s="6"/>
       <c r="F54" s="15" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H54" s="6"/>
       <c r="I54" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="J54" s="18" t="s">
         <v>358</v>
       </c>
-      <c r="J54" s="18" t="s">
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="8" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="55" spans="1:10">
-      <c r="A55" s="8" t="s">
+      <c r="B55" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="B55" s="8" t="s">
+      <c r="C55" s="8" t="s">
         <v>361</v>
-      </c>
-      <c r="C55" s="8" t="s">
-        <v>362</v>
       </c>
       <c r="D55" s="8" t="s">
         <v>13</v>
       </c>
       <c r="E55" s="8"/>
       <c r="F55" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="G55" s="8" t="s">
         <v>363</v>
       </c>
-      <c r="G55" s="8" t="s">
+      <c r="H55" s="8" t="s">
         <v>364</v>
       </c>
-      <c r="H55" s="8" t="s">
+      <c r="I55" s="8" t="s">
         <v>365</v>
       </c>
-      <c r="I55" s="8" t="s">
+      <c r="J55" s="8" t="s">
         <v>366</v>
       </c>
-      <c r="J55" s="8" t="s">
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="56" spans="1:10">
-      <c r="A56" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="B56" s="6" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="6" t="s">
@@ -4747,48 +4777,48 @@
         <v>148</v>
       </c>
       <c r="I56" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="J56" s="6" t="s">
         <v>375</v>
       </c>
-      <c r="J56" s="6" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10">
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="B57" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="B57" s="6" t="s">
+      <c r="C57" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="C57" s="6" t="s">
+      <c r="D57" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="D57" s="6" t="s">
-        <v>371</v>
-      </c>
       <c r="E57" s="6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F57" s="6"/>
       <c r="H57" s="6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="I57" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="J57" s="16" t="s">
         <v>372</v>
       </c>
-      <c r="J57" s="16" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10">
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="B58" s="8" t="s">
         <v>377</v>
       </c>
-      <c r="B58" s="8" t="s">
+      <c r="C58" s="8" t="s">
         <v>378</v>
-      </c>
-      <c r="C58" s="8" t="s">
-        <v>379</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>29</v>
@@ -4797,51 +4827,51 @@
         <v>94</v>
       </c>
       <c r="F58" s="11" t="s">
+        <v>379</v>
+      </c>
+      <c r="H58" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="H58" s="8" t="s">
+      <c r="I58" s="8" t="s">
         <v>381</v>
       </c>
-      <c r="I58" s="8" t="s">
+      <c r="J58" s="8" t="s">
         <v>382</v>
       </c>
-      <c r="J58" s="8" t="s">
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
         <v>383</v>
       </c>
-    </row>
-    <row r="59" spans="1:10">
-      <c r="A59" s="6" t="s">
+      <c r="B59" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="B59" s="6" t="s">
-        <v>385</v>
-      </c>
       <c r="C59" s="6" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E59" s="6"/>
       <c r="F59" s="6" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G59" s="6" t="s">
         <v>31</v>
       </c>
       <c r="H59" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="I59" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="I59" s="6" t="s">
+      <c r="J59" s="16" t="s">
         <v>388</v>
       </c>
-      <c r="J59" s="16" t="s">
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
         <v>389</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10">
-      <c r="A60" s="6" t="s">
-        <v>390</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>212</v>
@@ -4852,30 +4882,30 @@
       </c>
       <c r="E60" s="6"/>
       <c r="F60" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="G60" s="6" t="s">
         <v>391</v>
       </c>
-      <c r="G60" s="6" t="s">
+      <c r="H60" s="10" t="s">
+        <v>649</v>
+      </c>
+      <c r="I60" s="16" t="s">
         <v>392</v>
       </c>
-      <c r="H60" s="10" t="s">
-        <v>652</v>
-      </c>
-      <c r="I60" s="16" t="s">
+      <c r="J60" s="22" t="s">
         <v>393</v>
       </c>
-      <c r="J60" s="22" t="s">
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="61" spans="1:10">
-      <c r="A61" s="6" t="s">
+      <c r="B61" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>396</v>
-      </c>
       <c r="C61" s="6" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>29</v>
@@ -4884,116 +4914,116 @@
         <v>94</v>
       </c>
       <c r="F61" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="G61" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="G61" s="6" t="s">
+      <c r="H61" s="6" t="s">
         <v>398</v>
-      </c>
-      <c r="H61" s="6" t="s">
-        <v>399</v>
       </c>
       <c r="I61" s="6"/>
       <c r="J61" s="6"/>
     </row>
-    <row r="62" spans="1:10">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="C62" s="6" t="s">
         <v>400</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>401</v>
       </c>
       <c r="D62" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E62" s="6"/>
       <c r="F62" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="G62" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="G62" s="6" t="s">
-        <v>364</v>
-      </c>
-      <c r="H62" s="6" t="s">
+      <c r="I62" s="6" t="s">
         <v>403</v>
       </c>
-      <c r="I62" s="6" t="s">
+      <c r="J62" s="6" t="s">
         <v>404</v>
       </c>
-      <c r="J62" s="6" t="s">
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" s="8" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="63" spans="1:10">
-      <c r="A63" s="8" t="s">
+      <c r="B63" s="8" t="s">
         <v>406</v>
       </c>
-      <c r="B63" s="8" t="s">
+      <c r="C63" s="8" t="s">
         <v>407</v>
-      </c>
-      <c r="C63" s="8" t="s">
-        <v>408</v>
       </c>
       <c r="D63" s="8" t="s">
         <v>29</v>
       </c>
       <c r="E63" s="8"/>
       <c r="F63" s="8" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="G63" s="8" t="s">
         <v>31</v>
       </c>
       <c r="H63" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="I63" s="8" t="s">
         <v>410</v>
       </c>
-      <c r="I63" s="8" t="s">
+      <c r="J63" s="8" t="s">
         <v>411</v>
       </c>
-      <c r="J63" s="8" t="s">
+    </row>
+    <row r="64" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" s="4" customFormat="1">
-      <c r="A64" t="s">
+      <c r="B64" t="s">
         <v>413</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" s="25" t="s">
         <v>414</v>
-      </c>
-      <c r="C64" s="25" t="s">
-        <v>415</v>
       </c>
       <c r="D64" t="s">
         <v>13</v>
       </c>
       <c r="E64"/>
       <c r="F64" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G64" t="s">
         <v>15</v>
       </c>
       <c r="H64" t="s">
+        <v>416</v>
+      </c>
+      <c r="I64" t="s">
         <v>417</v>
       </c>
-      <c r="I64" t="s">
+      <c r="J64" t="s">
         <v>418</v>
       </c>
-      <c r="J64" t="s">
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" s="6" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="65" spans="1:10">
-      <c r="A65" s="6" t="s">
+      <c r="B65" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="B65" s="6" t="s">
+      <c r="C65" s="6" t="s">
         <v>421</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>422</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>145</v>
@@ -5004,74 +5034,77 @@
       <c r="F65" s="7"/>
       <c r="G65" s="4"/>
       <c r="H65" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="I65" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="I65" s="6" t="s">
+      <c r="J65" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="J65" s="6" t="s">
+    </row>
+    <row r="66" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="6" t="s">
         <v>425</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" s="5" customFormat="1">
-      <c r="A66" s="6" t="s">
+      <c r="B66" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="B66" s="6" t="s">
+      <c r="C66" s="6" t="s">
         <v>427</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>428</v>
       </c>
       <c r="D66" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E66" s="6"/>
       <c r="F66" s="6" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="G66" s="6" t="s">
         <v>31</v>
       </c>
       <c r="H66" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="I66" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="I66" s="6" t="s">
+      <c r="J66" s="6" t="s">
         <v>431</v>
       </c>
-      <c r="J66" s="6" t="s">
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
         <v>432</v>
       </c>
-    </row>
-    <row r="67" spans="1:10">
-      <c r="A67" t="s">
+      <c r="B67" t="s">
         <v>433</v>
       </c>
-      <c r="B67" t="s">
-        <v>434</v>
+      <c r="C67" t="s">
+        <v>827</v>
       </c>
       <c r="D67" t="s">
         <v>54</v>
       </c>
       <c r="G67" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="H67" s="8" t="s">
+        <v>434</v>
+      </c>
+      <c r="I67" s="18" t="s">
         <v>435</v>
       </c>
-      <c r="I67" s="18" t="s">
+      <c r="J67" s="17" t="s">
         <v>436</v>
       </c>
-      <c r="J67" s="17" t="s">
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" s="8" t="s">
         <v>437</v>
       </c>
-    </row>
-    <row r="68" spans="1:10">
-      <c r="A68" s="8" t="s">
-        <v>438</v>
-      </c>
       <c r="B68" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C68" s="8"/>
       <c r="D68" s="8" t="s">
@@ -5079,28 +5112,31 @@
       </c>
       <c r="E68" s="8"/>
       <c r="F68" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="G68" s="8" t="s">
         <v>391</v>
       </c>
-      <c r="G68" s="8" t="s">
-        <v>392</v>
-      </c>
       <c r="H68" s="8" t="s">
+        <v>438</v>
+      </c>
+      <c r="I68" s="12" t="s">
+        <v>761</v>
+      </c>
+      <c r="J68" s="17" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>439</v>
-      </c>
-      <c r="I68" s="12" t="s">
-        <v>764</v>
-      </c>
-      <c r="J68" s="17" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10">
-      <c r="A69" t="s">
-        <v>440</v>
       </c>
       <c r="B69" t="s">
         <v>118</v>
       </c>
+      <c r="C69" t="s">
+        <v>824</v>
+      </c>
       <c r="D69" t="s">
         <v>108</v>
       </c>
@@ -5108,24 +5144,24 @@
         <v>31</v>
       </c>
       <c r="H69" s="21" t="s">
+        <v>440</v>
+      </c>
+      <c r="I69" s="18" t="s">
         <v>441</v>
       </c>
-      <c r="I69" s="18" t="s">
+      <c r="J69" s="18" t="s">
         <v>442</v>
       </c>
-      <c r="J69" s="18" t="s">
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" s="8" t="s">
         <v>443</v>
       </c>
-    </row>
-    <row r="70" spans="1:10">
-      <c r="A70" s="8" t="s">
+      <c r="B70" s="8" t="s">
         <v>444</v>
       </c>
-      <c r="B70" s="8" t="s">
+      <c r="C70" s="8" t="s">
         <v>445</v>
-      </c>
-      <c r="C70" s="8" t="s">
-        <v>446</v>
       </c>
       <c r="D70" s="8" t="s">
         <v>125</v>
@@ -5134,33 +5170,33 @@
         <v>85</v>
       </c>
       <c r="F70" s="8" t="s">
+        <v>446</v>
+      </c>
+      <c r="G70" s="8" t="s">
+        <v>778</v>
+      </c>
+      <c r="H70" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G70" s="8" t="s">
-        <v>781</v>
-      </c>
-      <c r="H70" s="8" t="s">
+      <c r="I70" s="8" t="s">
         <v>448</v>
       </c>
-      <c r="I70" s="8" t="s">
+      <c r="J70" s="8" t="s">
         <v>449</v>
       </c>
-      <c r="J70" s="8" t="s">
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" s="6" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="71" spans="1:10">
-      <c r="A71" s="6" t="s">
+      <c r="B71" s="6" t="s">
         <v>451</v>
       </c>
-      <c r="B71" s="6" t="s">
+      <c r="C71" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="C71" s="6" t="s">
-        <v>453</v>
-      </c>
       <c r="D71" s="6" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>146</v>
@@ -5172,56 +5208,56 @@
         <v>147</v>
       </c>
       <c r="H71" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="I71" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="I71" s="6" t="s">
+      <c r="J71" s="6" t="s">
         <v>455</v>
       </c>
-      <c r="J71" s="6" t="s">
+    </row>
+    <row r="72" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A72" s="8" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="72" spans="1:10">
-      <c r="A72" s="8" t="s">
-        <v>457</v>
-      </c>
       <c r="B72" s="8" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="D72" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E72" s="23" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F72" s="8" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="G72" s="8" t="s">
         <v>31</v>
       </c>
       <c r="H72" s="8" t="s">
+        <v>458</v>
+      </c>
+      <c r="I72" s="8" t="s">
         <v>459</v>
       </c>
-      <c r="I72" s="8" t="s">
+      <c r="J72" s="17" t="s">
         <v>460</v>
       </c>
-      <c r="J72" s="17" t="s">
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>461</v>
       </c>
-    </row>
-    <row r="73" spans="1:10">
-      <c r="A73" t="s">
+      <c r="B73" t="s">
         <v>462</v>
       </c>
-      <c r="B73" t="s">
-        <v>463</v>
-      </c>
       <c r="C73" s="6" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
       <c r="D73" t="s">
         <v>108</v>
@@ -5230,80 +5266,82 @@
         <v>31</v>
       </c>
       <c r="H73" s="21" t="s">
+        <v>463</v>
+      </c>
+      <c r="I73" s="18" t="s">
         <v>464</v>
       </c>
-      <c r="I73" s="18" t="s">
+      <c r="J73" s="18" t="s">
         <v>465</v>
       </c>
-      <c r="J73" s="18" t="s">
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A74" s="8" t="s">
         <v>466</v>
       </c>
-    </row>
-    <row r="74" spans="1:10">
-      <c r="A74" s="8" t="s">
+      <c r="B74" s="8" t="s">
         <v>467</v>
       </c>
-      <c r="B74" s="8" t="s">
+      <c r="C74" s="6" t="s">
         <v>468</v>
-      </c>
-      <c r="C74" s="6" t="s">
-        <v>469</v>
       </c>
       <c r="D74" s="8" t="s">
         <v>13</v>
       </c>
       <c r="E74" s="8"/>
       <c r="F74" s="8" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="G74" s="8" t="s">
         <v>31</v>
       </c>
       <c r="H74" s="8" t="s">
+        <v>470</v>
+      </c>
+      <c r="I74" s="8" t="s">
         <v>471</v>
       </c>
-      <c r="I74" s="8" t="s">
+      <c r="J74" s="8" t="s">
         <v>472</v>
       </c>
-      <c r="J74" s="8" t="s">
+    </row>
+    <row r="75" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>473</v>
       </c>
-    </row>
-    <row r="75" spans="1:10" s="4" customFormat="1">
-      <c r="A75" t="s">
+      <c r="B75" t="s">
         <v>474</v>
       </c>
-      <c r="B75" t="s">
-        <v>475</v>
-      </c>
-      <c r="C75" s="6"/>
+      <c r="C75" s="6" t="s">
+        <v>817</v>
+      </c>
       <c r="D75" s="8" t="s">
         <v>29</v>
       </c>
       <c r="E75" s="8"/>
       <c r="F75" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="G75" s="8" t="s">
         <v>85</v>
       </c>
       <c r="H75" t="s">
+        <v>476</v>
+      </c>
+      <c r="I75" s="18" t="s">
         <v>477</v>
       </c>
-      <c r="I75" s="18" t="s">
+      <c r="J75"/>
+    </row>
+    <row r="76" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="8" t="s">
         <v>478</v>
       </c>
-      <c r="J75"/>
-    </row>
-    <row r="76" spans="1:10" s="4" customFormat="1">
-      <c r="A76" s="8" t="s">
+      <c r="B76" s="8" t="s">
         <v>479</v>
       </c>
-      <c r="B76" s="8" t="s">
+      <c r="C76" s="6" t="s">
         <v>480</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>481</v>
       </c>
       <c r="D76" s="8" t="s">
         <v>168</v>
@@ -5315,24 +5353,24 @@
         <v>208</v>
       </c>
       <c r="H76" s="8" t="s">
+        <v>481</v>
+      </c>
+      <c r="I76" s="8" t="s">
         <v>482</v>
       </c>
-      <c r="I76" s="8" t="s">
+      <c r="J76" s="8" t="s">
         <v>483</v>
       </c>
-      <c r="J76" s="8" t="s">
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A77" s="6" t="s">
         <v>484</v>
       </c>
-    </row>
-    <row r="77" spans="1:10">
-      <c r="A77" s="6" t="s">
+      <c r="B77" s="6" t="s">
         <v>485</v>
       </c>
-      <c r="B77" s="6" t="s">
+      <c r="C77" s="6" t="s">
         <v>486</v>
-      </c>
-      <c r="C77" s="6" t="s">
-        <v>487</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>168</v>
@@ -5341,30 +5379,30 @@
         <v>146</v>
       </c>
       <c r="F77" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>763</v>
+      </c>
+      <c r="H77" s="6" t="s">
         <v>488</v>
       </c>
-      <c r="G77" s="8" t="s">
-        <v>766</v>
-      </c>
-      <c r="H77" s="6" t="s">
+      <c r="I77" s="6" t="s">
         <v>489</v>
       </c>
-      <c r="I77" s="6" t="s">
+      <c r="J77" s="6" t="s">
         <v>490</v>
       </c>
-      <c r="J77" s="6" t="s">
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A78" s="8" t="s">
         <v>491</v>
       </c>
-    </row>
-    <row r="78" spans="1:10">
-      <c r="A78" s="8" t="s">
+      <c r="B78" s="8" t="s">
         <v>492</v>
       </c>
-      <c r="B78" s="8" t="s">
-        <v>493</v>
-      </c>
       <c r="C78" s="6" t="s">
-        <v>494</v>
+        <v>826</v>
       </c>
       <c r="D78" s="8" t="s">
         <v>168</v>
@@ -5376,108 +5414,114 @@
         <v>115</v>
       </c>
       <c r="H78" s="8" t="s">
+        <v>493</v>
+      </c>
+      <c r="I78" s="8" t="s">
+        <v>494</v>
+      </c>
+      <c r="J78" s="8" t="s">
         <v>495</v>
       </c>
-      <c r="I78" s="8" t="s">
+    </row>
+    <row r="79" spans="1:10" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A79" s="6" t="s">
         <v>496</v>
       </c>
-      <c r="J78" s="8" t="s">
+      <c r="B79" s="6" t="s">
         <v>497</v>
       </c>
-    </row>
-    <row r="79" spans="1:10" s="4" customFormat="1">
-      <c r="A79" s="6" t="s">
+      <c r="C79" s="6" t="s">
         <v>498</v>
-      </c>
-      <c r="B79" s="6" t="s">
-        <v>499</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>500</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>253</v>
       </c>
       <c r="E79" s="23" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F79" s="6"/>
       <c r="G79" s="6" t="s">
         <v>155</v>
       </c>
       <c r="H79" s="6" t="s">
+        <v>499</v>
+      </c>
+      <c r="I79" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="J79" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="I79" s="6" t="s">
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A80" s="10" t="s">
         <v>502</v>
       </c>
-      <c r="J79" s="6" t="s">
+      <c r="B80" s="10" t="s">
         <v>503</v>
       </c>
-    </row>
-    <row r="80" spans="1:10">
-      <c r="A80" s="6" t="s">
+      <c r="C80" s="10" t="s">
+        <v>811</v>
+      </c>
+      <c r="D80" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E80" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="F80" t="s">
+        <v>766</v>
+      </c>
+      <c r="G80" s="10" t="s">
+        <v>777</v>
+      </c>
+      <c r="H80" s="10" t="s">
         <v>504</v>
       </c>
-      <c r="B80" s="6" t="s">
+      <c r="I80" s="10" t="s">
+        <v>505</v>
+      </c>
+      <c r="J80" s="10" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A81" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>812</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E81" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F81" s="6"/>
+      <c r="H81" s="6"/>
+      <c r="I81" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="J81" s="6" t="s">
         <v>509</v>
       </c>
-      <c r="C80" s="6"/>
-      <c r="D80" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="E80" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="F80" s="6"/>
-      <c r="H80" s="6"/>
-      <c r="I80" s="6" t="s">
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A82" s="6" t="s">
         <v>510</v>
       </c>
-      <c r="J80" s="6" t="s">
+      <c r="B82" s="6" t="s">
         <v>511</v>
       </c>
-    </row>
-    <row r="81" spans="1:10">
-      <c r="A81" s="10" t="s">
-        <v>504</v>
-      </c>
-      <c r="B81" s="10" t="s">
-        <v>505</v>
-      </c>
-      <c r="C81" s="10"/>
-      <c r="D81" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="E81" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="F81" t="s">
-        <v>769</v>
-      </c>
-      <c r="G81" s="10" t="s">
-        <v>780</v>
-      </c>
-      <c r="H81" s="10" t="s">
-        <v>506</v>
-      </c>
-      <c r="I81" s="10" t="s">
-        <v>507</v>
-      </c>
-      <c r="J81" s="10" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10">
-      <c r="A82" s="6" t="s">
+      <c r="C82" s="6" t="s">
+        <v>815</v>
+      </c>
+      <c r="D82" s="6" t="s">
         <v>512</v>
-      </c>
-      <c r="B82" s="6" t="s">
-        <v>513</v>
-      </c>
-      <c r="C82" s="6"/>
-      <c r="D82" s="6" t="s">
-        <v>514</v>
       </c>
       <c r="E82" s="6"/>
       <c r="F82" s="6"/>
@@ -5485,134 +5529,138 @@
         <v>63</v>
       </c>
       <c r="H82" s="6" t="s">
+        <v>513</v>
+      </c>
+      <c r="I82" s="16" t="s">
+        <v>514</v>
+      </c>
+      <c r="J82" s="6"/>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A83" s="6" t="s">
         <v>515</v>
       </c>
-      <c r="I82" s="16" t="s">
+      <c r="B83" s="6" t="s">
         <v>516</v>
       </c>
-      <c r="J82" s="6"/>
-    </row>
-    <row r="83" spans="1:10">
-      <c r="A83" s="6" t="s">
-        <v>517</v>
-      </c>
-      <c r="B83" s="6" t="s">
-        <v>518</v>
-      </c>
-      <c r="C83" s="6"/>
+      <c r="C83" s="6" t="s">
+        <v>830</v>
+      </c>
       <c r="D83" s="6" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="E83" s="6"/>
       <c r="F83" s="6"/>
       <c r="G83" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="H83" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="I83" s="16" t="s">
         <v>519</v>
       </c>
-      <c r="H83" s="6" t="s">
+      <c r="J83" s="6"/>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" s="6" t="s">
         <v>520</v>
       </c>
-      <c r="I83" s="16" t="s">
+      <c r="B84" s="6" t="s">
         <v>521</v>
       </c>
-      <c r="J83" s="6"/>
-    </row>
-    <row r="84" spans="1:10">
-      <c r="A84" s="6" t="s">
+      <c r="C84" s="6" t="s">
+        <v>829</v>
+      </c>
+      <c r="D84" s="6" t="s">
         <v>522</v>
-      </c>
-      <c r="B84" s="6" t="s">
-        <v>523</v>
-      </c>
-      <c r="C84" s="6"/>
-      <c r="D84" s="6" t="s">
-        <v>524</v>
       </c>
       <c r="E84" s="6"/>
       <c r="F84" s="27" t="s">
+        <v>523</v>
+      </c>
+      <c r="G84" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="H84" s="14" t="s">
+        <v>524</v>
+      </c>
+      <c r="I84" s="16" t="s">
         <v>525</v>
       </c>
-      <c r="G84" s="6" t="s">
-        <v>284</v>
-      </c>
-      <c r="H84" s="14" t="s">
+      <c r="J84" s="16" t="s">
         <v>526</v>
       </c>
-      <c r="I84" s="16" t="s">
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" s="6" t="s">
         <v>527</v>
       </c>
-      <c r="J84" s="16" t="s">
+      <c r="B85" s="6" t="s">
         <v>528</v>
       </c>
-    </row>
-    <row r="85" spans="1:10">
-      <c r="A85" s="6" t="s">
+      <c r="C85" s="6" t="s">
         <v>529</v>
-      </c>
-      <c r="B85" s="6" t="s">
-        <v>530</v>
-      </c>
-      <c r="C85" s="6" t="s">
-        <v>531</v>
       </c>
       <c r="D85" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E85" s="6"/>
       <c r="F85" s="6" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="G85" s="6" t="s">
         <v>31</v>
       </c>
       <c r="H85" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="I85" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="J85" s="6" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A86" s="6" t="s">
         <v>533</v>
       </c>
-      <c r="I85" s="6" t="s">
+      <c r="B86" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="C86" s="6" t="s">
         <v>534</v>
-      </c>
-      <c r="J85" s="6" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10">
-      <c r="A86" s="6" t="s">
-        <v>535</v>
-      </c>
-      <c r="B86" s="6" t="s">
-        <v>434</v>
-      </c>
-      <c r="C86" s="6" t="s">
-        <v>536</v>
       </c>
       <c r="D86" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E86" s="6"/>
       <c r="F86" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="G86" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="H86" s="6" t="s">
         <v>537</v>
       </c>
-      <c r="G86" s="6" t="s">
+      <c r="I86" s="6" t="s">
         <v>538</v>
       </c>
-      <c r="H86" s="6" t="s">
+      <c r="J86" s="6" t="s">
         <v>539</v>
       </c>
-      <c r="I86" s="6" t="s">
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" s="6" t="s">
         <v>540</v>
       </c>
-      <c r="J86" s="6" t="s">
+      <c r="B87" s="6" t="s">
         <v>541</v>
       </c>
-    </row>
-    <row r="87" spans="1:10">
-      <c r="A87" s="6" t="s">
+      <c r="C87" s="6" t="s">
         <v>542</v>
-      </c>
-      <c r="B87" s="6" t="s">
-        <v>543</v>
-      </c>
-      <c r="C87" s="6" t="s">
-        <v>544</v>
       </c>
       <c r="D87" s="6" t="s">
         <v>45</v>
@@ -5621,30 +5669,30 @@
         <v>85</v>
       </c>
       <c r="G87" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="H87" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="I87" s="6" t="s">
         <v>545</v>
       </c>
-      <c r="H87" s="6" t="s">
+      <c r="J87" s="6" t="s">
         <v>546</v>
       </c>
-      <c r="I87" s="6" t="s">
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" s="6" t="s">
         <v>547</v>
       </c>
-      <c r="J87" s="6" t="s">
+      <c r="B88" s="6" t="s">
         <v>548</v>
       </c>
-    </row>
-    <row r="88" spans="1:10">
-      <c r="A88" s="6" t="s">
-        <v>549</v>
-      </c>
-      <c r="B88" s="6" t="s">
-        <v>550</v>
-      </c>
       <c r="C88" s="6" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="E88" s="6"/>
       <c r="F88" s="6"/>
@@ -5652,82 +5700,82 @@
         <v>109</v>
       </c>
       <c r="H88" s="6" t="s">
+        <v>549</v>
+      </c>
+      <c r="I88" s="16" t="s">
+        <v>550</v>
+      </c>
+      <c r="J88" s="6"/>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" s="6" t="s">
         <v>551</v>
       </c>
-      <c r="I88" s="16" t="s">
+      <c r="B89" s="6" t="s">
         <v>552</v>
       </c>
-      <c r="J88" s="6"/>
-    </row>
-    <row r="89" spans="1:10">
-      <c r="A89" s="6" t="s">
+      <c r="C89" s="6" t="s">
         <v>553</v>
-      </c>
-      <c r="B89" s="6" t="s">
-        <v>554</v>
-      </c>
-      <c r="C89" s="6" t="s">
-        <v>555</v>
       </c>
       <c r="D89" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E89" s="6"/>
       <c r="F89" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="H89" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="I89" s="6" t="s">
         <v>556</v>
       </c>
-      <c r="G89" s="6" t="s">
-        <v>519</v>
-      </c>
-      <c r="H89" s="6" t="s">
+      <c r="J89" s="6" t="s">
         <v>557</v>
       </c>
-      <c r="I89" s="6" t="s">
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A90" s="14" t="s">
         <v>558</v>
       </c>
-      <c r="J89" s="6" t="s">
+      <c r="B90" s="14" t="s">
         <v>559</v>
       </c>
-    </row>
-    <row r="90" spans="1:10">
-      <c r="A90" s="14" t="s">
+      <c r="C90" s="6" t="s">
         <v>560</v>
-      </c>
-      <c r="B90" s="14" t="s">
-        <v>561</v>
-      </c>
-      <c r="C90" s="6" t="s">
-        <v>562</v>
       </c>
       <c r="D90" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E90" s="6"/>
       <c r="F90" s="14" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="G90" s="14" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H90" s="14" t="s">
+        <v>561</v>
+      </c>
+      <c r="I90" s="14" t="s">
+        <v>562</v>
+      </c>
+      <c r="J90" s="14" t="s">
         <v>563</v>
       </c>
-      <c r="I90" s="14" t="s">
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A91" s="8" t="s">
         <v>564</v>
       </c>
-      <c r="J90" s="14" t="s">
+      <c r="B91" s="8" t="s">
         <v>565</v>
       </c>
-    </row>
-    <row r="91" spans="1:10">
-      <c r="A91" s="8" t="s">
+      <c r="C91" s="6" t="s">
         <v>566</v>
-      </c>
-      <c r="B91" s="8" t="s">
-        <v>567</v>
-      </c>
-      <c r="C91" s="6" t="s">
-        <v>568</v>
       </c>
       <c r="D91" s="8" t="s">
         <v>125</v>
@@ -5740,140 +5788,142 @@
         <v>85</v>
       </c>
       <c r="H91" s="8" t="s">
+        <v>567</v>
+      </c>
+      <c r="I91" s="8" t="s">
+        <v>568</v>
+      </c>
+      <c r="J91" s="8" t="s">
         <v>569</v>
       </c>
-      <c r="I91" s="8" t="s">
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A92" s="8" t="s">
         <v>570</v>
       </c>
-      <c r="J91" s="8" t="s">
+      <c r="B92" s="8" t="s">
         <v>571</v>
       </c>
-    </row>
-    <row r="92" spans="1:10">
-      <c r="A92" s="8" t="s">
+      <c r="C92" s="6" t="s">
         <v>572</v>
-      </c>
-      <c r="B92" s="8" t="s">
-        <v>573</v>
-      </c>
-      <c r="C92" s="6" t="s">
-        <v>574</v>
       </c>
       <c r="D92" s="8" t="s">
         <v>13</v>
       </c>
       <c r="E92" s="8"/>
       <c r="F92" s="11" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="G92" s="8" t="s">
         <v>193</v>
       </c>
       <c r="H92" s="8" t="s">
+        <v>574</v>
+      </c>
+      <c r="I92" s="8" t="s">
+        <v>575</v>
+      </c>
+      <c r="J92" s="8" t="s">
         <v>576</v>
       </c>
-      <c r="I92" s="8" t="s">
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>577</v>
       </c>
-      <c r="J92" s="8" t="s">
+      <c r="B93" t="s">
         <v>578</v>
       </c>
-    </row>
-    <row r="93" spans="1:10">
-      <c r="A93" t="s">
-        <v>579</v>
-      </c>
-      <c r="B93" t="s">
-        <v>580</v>
-      </c>
       <c r="C93" s="6" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="D93" s="8" t="s">
         <v>29</v>
       </c>
       <c r="E93" s="8"/>
       <c r="F93" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="G93" s="8" t="s">
         <v>85</v>
       </c>
       <c r="H93" t="s">
+        <v>580</v>
+      </c>
+      <c r="I93" s="18" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A94" s="14" t="s">
         <v>582</v>
       </c>
-      <c r="I93" s="18" t="s">
+      <c r="B94" s="14" t="s">
         <v>583</v>
       </c>
-    </row>
-    <row r="94" spans="1:10">
-      <c r="A94" s="14" t="s">
-        <v>584</v>
-      </c>
-      <c r="B94" s="14" t="s">
-        <v>585</v>
-      </c>
       <c r="C94" s="14" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="D94" s="14" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E94" s="14" t="s">
         <v>46</v>
       </c>
       <c r="F94" s="7"/>
       <c r="G94" s="14" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="H94" s="14" t="s">
+        <v>584</v>
+      </c>
+      <c r="I94" s="14" t="s">
+        <v>585</v>
+      </c>
+      <c r="J94" s="14" t="s">
         <v>586</v>
       </c>
-      <c r="I94" s="14" t="s">
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A95" s="8" t="s">
         <v>587</v>
       </c>
-      <c r="J94" s="14" t="s">
+      <c r="B95" s="8" t="s">
         <v>588</v>
       </c>
-    </row>
-    <row r="95" spans="1:10">
-      <c r="A95" s="8" t="s">
+      <c r="C95" s="8" t="s">
+        <v>822</v>
+      </c>
+      <c r="D95" s="8" t="s">
         <v>589</v>
-      </c>
-      <c r="B95" s="8" t="s">
-        <v>590</v>
-      </c>
-      <c r="C95" s="8"/>
-      <c r="D95" s="8" t="s">
-        <v>591</v>
       </c>
       <c r="E95" s="8"/>
       <c r="F95" s="8" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="G95" s="8" t="s">
         <v>70</v>
       </c>
       <c r="H95" s="8" t="s">
+        <v>591</v>
+      </c>
+      <c r="I95" s="8" t="s">
+        <v>592</v>
+      </c>
+      <c r="J95" s="8" t="s">
         <v>593</v>
       </c>
-      <c r="I95" s="8" t="s">
+    </row>
+    <row r="96" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="8" t="s">
         <v>594</v>
       </c>
-      <c r="J95" s="8" t="s">
+      <c r="B96" s="8" t="s">
         <v>595</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" s="4" customFormat="1">
-      <c r="A96" s="8" t="s">
-        <v>596</v>
-      </c>
-      <c r="B96" s="8" t="s">
-        <v>597</v>
       </c>
       <c r="C96" s="8"/>
       <c r="D96" s="8" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E96" s="8" t="s">
         <v>85</v>
@@ -5881,82 +5931,82 @@
       <c r="F96" s="8"/>
       <c r="G96"/>
       <c r="H96" s="8" t="s">
+        <v>596</v>
+      </c>
+      <c r="I96" s="8" t="s">
+        <v>597</v>
+      </c>
+      <c r="J96" s="8" t="s">
         <v>598</v>
       </c>
-      <c r="I96" s="8" t="s">
+    </row>
+    <row r="97" spans="1:10" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A97" s="8" t="s">
         <v>599</v>
       </c>
-      <c r="J96" s="8" t="s">
+      <c r="B97" s="8" t="s">
         <v>600</v>
       </c>
-    </row>
-    <row r="97" spans="1:10" s="4" customFormat="1">
-      <c r="A97" s="8" t="s">
-        <v>601</v>
-      </c>
-      <c r="B97" s="8" t="s">
-        <v>602</v>
-      </c>
       <c r="C97" s="8" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="D97" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E97" s="23" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F97" s="10" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="G97" s="8" t="s">
         <v>31</v>
       </c>
       <c r="H97" s="8" t="s">
+        <v>602</v>
+      </c>
+      <c r="I97" s="8" t="s">
+        <v>603</v>
+      </c>
+      <c r="J97" s="17" t="s">
         <v>604</v>
       </c>
-      <c r="I97" s="8" t="s">
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A98" s="8" t="s">
         <v>605</v>
       </c>
-      <c r="J97" s="17" t="s">
+      <c r="B98" s="8" t="s">
         <v>606</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10">
-      <c r="A98" s="8" t="s">
-        <v>607</v>
-      </c>
-      <c r="B98" s="8" t="s">
-        <v>608</v>
       </c>
       <c r="C98" s="8"/>
       <c r="D98" s="8" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="E98" s="6"/>
       <c r="F98" s="27" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="G98" s="8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H98" s="8"/>
       <c r="I98" s="17" t="s">
+        <v>609</v>
+      </c>
+      <c r="J98" s="18" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>611</v>
       </c>
-      <c r="J98" s="18" t="s">
+      <c r="B99" t="s">
         <v>612</v>
       </c>
-    </row>
-    <row r="99" spans="1:10">
-      <c r="A99" t="s">
+      <c r="C99" s="30" t="s">
         <v>613</v>
-      </c>
-      <c r="B99" t="s">
-        <v>614</v>
-      </c>
-      <c r="C99" s="25" t="s">
-        <v>615</v>
       </c>
       <c r="D99" t="s">
         <v>29</v>
@@ -5965,27 +6015,27 @@
         <v>94</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="G99" t="s">
         <v>115</v>
       </c>
       <c r="I99" t="s">
+        <v>615</v>
+      </c>
+      <c r="J99" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A100" s="6" t="s">
         <v>617</v>
       </c>
-      <c r="J99" t="s">
+      <c r="B100" s="6" t="s">
         <v>618</v>
       </c>
-    </row>
-    <row r="100" spans="1:10">
-      <c r="A100" s="6" t="s">
-        <v>619</v>
-      </c>
-      <c r="B100" s="6" t="s">
-        <v>620</v>
-      </c>
       <c r="C100" s="6" t="s">
-        <v>621</v>
+        <v>814</v>
       </c>
       <c r="D100" s="6" t="s">
         <v>125</v>
@@ -5994,90 +6044,90 @@
         <v>94</v>
       </c>
       <c r="F100" s="15" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="G100" t="s">
         <v>115</v>
       </c>
       <c r="H100" s="14" t="s">
+        <v>620</v>
+      </c>
+      <c r="I100" s="14" t="s">
+        <v>621</v>
+      </c>
+      <c r="J100" s="14" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A101" s="6" t="s">
         <v>623</v>
       </c>
-      <c r="I100" s="14" t="s">
+      <c r="B101" s="6" t="s">
         <v>624</v>
       </c>
-      <c r="J100" s="14" t="s">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10">
-      <c r="A101" s="6" t="s">
-        <v>626</v>
-      </c>
-      <c r="B101" s="6" t="s">
-        <v>627</v>
-      </c>
       <c r="C101" s="6" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="D101" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E101" s="6"/>
       <c r="F101" s="6" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="G101" s="6" t="s">
         <v>31</v>
       </c>
       <c r="H101" s="14" t="s">
+        <v>626</v>
+      </c>
+      <c r="I101" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="J101" s="14" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A102" s="8" t="s">
+        <v>623</v>
+      </c>
+      <c r="B102" s="8" t="s">
         <v>629</v>
       </c>
-      <c r="I101" s="14" t="s">
+      <c r="C102" s="8" t="s">
         <v>630</v>
-      </c>
-      <c r="J101" s="14" t="s">
-        <v>631</v>
-      </c>
-    </row>
-    <row r="102" spans="1:10">
-      <c r="A102" s="8" t="s">
-        <v>626</v>
-      </c>
-      <c r="B102" s="8" t="s">
-        <v>632</v>
-      </c>
-      <c r="C102" s="8" t="s">
-        <v>633</v>
       </c>
       <c r="D102" s="8" t="s">
         <v>13</v>
       </c>
       <c r="E102" s="8"/>
       <c r="F102" s="8" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="G102" s="8" t="s">
         <v>31</v>
       </c>
       <c r="H102" s="10" t="s">
+        <v>632</v>
+      </c>
+      <c r="I102" s="10" t="s">
+        <v>633</v>
+      </c>
+      <c r="J102" s="10" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="6" t="s">
         <v>635</v>
       </c>
-      <c r="I102" s="10" t="s">
+      <c r="B103" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="C103" s="6" t="s">
         <v>636</v>
-      </c>
-      <c r="J102" s="10" t="s">
-        <v>637</v>
-      </c>
-    </row>
-    <row r="103" spans="1:10" s="5" customFormat="1">
-      <c r="A103" s="6" t="s">
-        <v>638</v>
-      </c>
-      <c r="B103" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C103" s="6" t="s">
-        <v>639</v>
       </c>
       <c r="D103" s="6" t="s">
         <v>13</v>
@@ -6090,24 +6140,24 @@
         <v>109</v>
       </c>
       <c r="H103" s="14" t="s">
+        <v>637</v>
+      </c>
+      <c r="I103" s="14" t="s">
+        <v>638</v>
+      </c>
+      <c r="J103" s="14" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="6" t="s">
         <v>640</v>
       </c>
-      <c r="I103" s="14" t="s">
+      <c r="B104" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="C104" s="6" t="s">
         <v>641</v>
-      </c>
-      <c r="J103" s="14" t="s">
-        <v>642</v>
-      </c>
-    </row>
-    <row r="104" spans="1:10" s="5" customFormat="1">
-      <c r="A104" s="6" t="s">
-        <v>643</v>
-      </c>
-      <c r="B104" s="6" t="s">
-        <v>580</v>
-      </c>
-      <c r="C104" s="6" t="s">
-        <v>644</v>
       </c>
       <c r="D104" s="6" t="s">
         <v>29</v>
@@ -6116,54 +6166,56 @@
         <v>94</v>
       </c>
       <c r="F104" s="15" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="H104" s="14"/>
       <c r="I104" s="13" t="s">
+        <v>643</v>
+      </c>
+      <c r="J104" s="14" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A105" s="8" t="s">
+        <v>645</v>
+      </c>
+      <c r="B105" s="8" t="s">
         <v>646</v>
       </c>
-      <c r="J104" s="14" t="s">
+      <c r="C105" s="8" t="s">
         <v>647</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10">
-      <c r="A105" s="8" t="s">
-        <v>648</v>
-      </c>
-      <c r="B105" s="8" t="s">
-        <v>649</v>
-      </c>
-      <c r="C105" s="8" t="s">
-        <v>650</v>
       </c>
       <c r="D105" s="8" t="s">
         <v>13</v>
       </c>
       <c r="E105" s="8"/>
       <c r="F105" s="11" t="s">
+        <v>648</v>
+      </c>
+      <c r="G105" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="H105" s="10" t="s">
+        <v>649</v>
+      </c>
+      <c r="I105" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="J105" s="10" t="s">
         <v>651</v>
       </c>
-      <c r="G105" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="H105" s="10" t="s">
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A106" s="8" t="s">
         <v>652</v>
       </c>
-      <c r="I105" s="10" t="s">
+      <c r="B106" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="J105" s="10" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10">
-      <c r="A106" s="8" t="s">
-        <v>655</v>
-      </c>
-      <c r="B106" s="8" t="s">
-        <v>656</v>
-      </c>
-      <c r="C106" s="6"/>
+      <c r="C106" s="6" t="s">
+        <v>828</v>
+      </c>
       <c r="D106" s="8" t="s">
         <v>108</v>
       </c>
@@ -6173,42 +6225,45 @@
         <v>22</v>
       </c>
       <c r="H106" s="10" t="s">
+        <v>654</v>
+      </c>
+      <c r="I106" s="17" t="s">
+        <v>655</v>
+      </c>
+      <c r="J106" s="10"/>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>656</v>
+      </c>
+      <c r="B107" t="s">
         <v>657</v>
       </c>
-      <c r="I106" s="17" t="s">
+      <c r="C107" t="s">
+        <v>816</v>
+      </c>
+      <c r="D107" t="s">
+        <v>512</v>
+      </c>
+      <c r="G107" t="s">
+        <v>765</v>
+      </c>
+      <c r="H107" s="8" t="s">
         <v>658</v>
       </c>
-      <c r="J106" s="10"/>
-    </row>
-    <row r="107" spans="1:10">
-      <c r="A107" t="s">
+      <c r="I107" s="18" t="s">
         <v>659</v>
       </c>
-      <c r="B107" t="s">
+      <c r="J107" s="17" t="s">
         <v>660</v>
       </c>
-      <c r="D107" t="s">
-        <v>514</v>
-      </c>
-      <c r="G107" t="s">
-        <v>768</v>
-      </c>
-      <c r="H107" s="8" t="s">
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>661</v>
       </c>
-      <c r="I107" s="18" t="s">
+      <c r="B108" t="s">
         <v>662</v>
-      </c>
-      <c r="J107" s="17" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="108" spans="1:10">
-      <c r="A108" t="s">
-        <v>664</v>
-      </c>
-      <c r="B108" t="s">
-        <v>665</v>
       </c>
       <c r="D108" t="s">
         <v>108</v>
@@ -6217,53 +6272,53 @@
         <v>31</v>
       </c>
       <c r="H108" t="s">
+        <v>663</v>
+      </c>
+      <c r="I108" s="18" t="s">
+        <v>664</v>
+      </c>
+      <c r="J108" s="19" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
         <v>666</v>
-      </c>
-      <c r="I108" s="18" t="s">
-        <v>667</v>
-      </c>
-      <c r="J108" s="19" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10">
-      <c r="A109" t="s">
-        <v>669</v>
       </c>
       <c r="B109" t="s">
         <v>60</v>
       </c>
       <c r="C109" s="25" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="D109" t="s">
         <v>13</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="G109" t="s">
         <v>31</v>
       </c>
       <c r="H109" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="I109" s="4" t="s">
+        <v>670</v>
+      </c>
+      <c r="J109" s="4" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A110" s="6" t="s">
         <v>672</v>
       </c>
-      <c r="I109" s="4" t="s">
+      <c r="B110" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="C110" s="6" t="s">
         <v>673</v>
-      </c>
-      <c r="J109" s="4" t="s">
-        <v>674</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10">
-      <c r="A110" s="6" t="s">
-        <v>675</v>
-      </c>
-      <c r="B110" s="6" t="s">
-        <v>522</v>
-      </c>
-      <c r="C110" s="6" t="s">
-        <v>676</v>
       </c>
       <c r="D110" s="6" t="s">
         <v>145</v>
@@ -6276,52 +6331,52 @@
         <v>139</v>
       </c>
       <c r="I110" s="14" t="s">
+        <v>674</v>
+      </c>
+      <c r="J110" s="14" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A111" s="6" t="s">
+        <v>676</v>
+      </c>
+      <c r="B111" s="6" t="s">
         <v>677</v>
       </c>
-      <c r="J110" s="14" t="s">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="111" spans="1:10">
-      <c r="A111" s="6" t="s">
-        <v>679</v>
-      </c>
-      <c r="B111" s="6" t="s">
-        <v>680</v>
-      </c>
       <c r="C111" s="6" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="D111" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E111" s="6"/>
       <c r="F111" s="15" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="G111" s="6" t="s">
         <v>193</v>
       </c>
       <c r="H111" s="14"/>
       <c r="I111" s="14" t="s">
+        <v>679</v>
+      </c>
+      <c r="J111" s="14" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>681</v>
+      </c>
+      <c r="B112" t="s">
         <v>682</v>
       </c>
-      <c r="J111" s="14" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10">
-      <c r="A112" t="s">
-        <v>684</v>
-      </c>
-      <c r="B112" t="s">
-        <v>685</v>
-      </c>
       <c r="C112" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E112" s="6"/>
       <c r="F112" s="6"/>
@@ -6329,42 +6384,42 @@
         <v>31</v>
       </c>
     </row>
-    <row r="113" spans="1:10">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" s="10" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="B113" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C113" s="8" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="D113" s="10" t="s">
         <v>29</v>
       </c>
       <c r="E113" s="10"/>
       <c r="F113" s="10" t="s">
+        <v>685</v>
+      </c>
+      <c r="G113" s="10" t="s">
+        <v>686</v>
+      </c>
+      <c r="H113" s="10" t="s">
+        <v>687</v>
+      </c>
+      <c r="I113" s="10" t="s">
         <v>688</v>
       </c>
-      <c r="G113" s="10" t="s">
+      <c r="J113" s="10" t="s">
         <v>689</v>
       </c>
-      <c r="H113" s="10" t="s">
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A114" s="10" t="s">
         <v>690</v>
       </c>
-      <c r="I113" s="10" t="s">
-        <v>691</v>
-      </c>
-      <c r="J113" s="10" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10">
-      <c r="A114" s="10" t="s">
-        <v>693</v>
-      </c>
       <c r="B114" s="10" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C114" s="10"/>
       <c r="D114" s="10" t="s">
@@ -6376,24 +6431,24 @@
       <c r="F114" s="10"/>
       <c r="G114" s="10"/>
       <c r="H114" s="10" t="s">
+        <v>691</v>
+      </c>
+      <c r="I114" s="10" t="s">
+        <v>692</v>
+      </c>
+      <c r="J114" s="10" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A115" s="6" t="s">
         <v>694</v>
       </c>
-      <c r="I114" s="10" t="s">
+      <c r="B115" s="6" t="s">
         <v>695</v>
       </c>
-      <c r="J114" s="10" t="s">
+      <c r="C115" s="6" t="s">
         <v>696</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10">
-      <c r="A115" s="6" t="s">
-        <v>697</v>
-      </c>
-      <c r="B115" s="6" t="s">
-        <v>698</v>
-      </c>
-      <c r="C115" s="6" t="s">
-        <v>699</v>
       </c>
       <c r="D115" s="6" t="s">
         <v>93</v>
@@ -6402,27 +6457,27 @@
         <v>94</v>
       </c>
       <c r="G115" s="6" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="H115" s="6" t="s">
+        <v>697</v>
+      </c>
+      <c r="I115" s="6" t="s">
+        <v>698</v>
+      </c>
+      <c r="J115" s="6" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A116" s="6" t="s">
         <v>700</v>
       </c>
-      <c r="I115" s="6" t="s">
+      <c r="B116" s="6" t="s">
         <v>701</v>
       </c>
-      <c r="J115" s="6" t="s">
-        <v>702</v>
-      </c>
-    </row>
-    <row r="116" spans="1:10">
-      <c r="A116" s="6" t="s">
-        <v>703</v>
-      </c>
-      <c r="B116" s="6" t="s">
-        <v>704</v>
-      </c>
       <c r="C116" s="26" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="D116" s="6" t="s">
         <v>108</v>
@@ -6430,55 +6485,55 @@
       <c r="E116" s="6"/>
       <c r="F116" s="6"/>
       <c r="G116" s="6" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H116" s="6"/>
       <c r="I116" s="16" t="s">
+        <v>702</v>
+      </c>
+      <c r="J116" s="6"/>
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A117" s="14" t="s">
+        <v>703</v>
+      </c>
+      <c r="B117" s="14" t="s">
+        <v>704</v>
+      </c>
+      <c r="C117" s="26" t="s">
         <v>705</v>
       </c>
-      <c r="J116" s="6"/>
-    </row>
-    <row r="117" spans="1:10">
-      <c r="A117" s="14" t="s">
+      <c r="D117" s="14" t="s">
+        <v>341</v>
+      </c>
+      <c r="E117" t="s">
         <v>706</v>
       </c>
-      <c r="B117" s="14" t="s">
+      <c r="F117" s="14" t="s">
         <v>707</v>
       </c>
-      <c r="C117" s="26" t="s">
+      <c r="G117" s="14" t="s">
+        <v>785</v>
+      </c>
+      <c r="H117" s="14" t="s">
         <v>708</v>
       </c>
-      <c r="D117" s="14" t="s">
-        <v>342</v>
-      </c>
-      <c r="E117" t="s">
+      <c r="I117" s="14" t="s">
         <v>709</v>
       </c>
-      <c r="F117" s="14" t="s">
+      <c r="J117" s="14" t="s">
         <v>710</v>
       </c>
-      <c r="G117" s="14" t="s">
-        <v>788</v>
-      </c>
-      <c r="H117" s="14" t="s">
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A118" s="8" t="s">
         <v>711</v>
       </c>
-      <c r="I117" s="14" t="s">
+      <c r="B118" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="C118" s="8" t="s">
         <v>712</v>
-      </c>
-      <c r="J117" s="14" t="s">
-        <v>713</v>
-      </c>
-    </row>
-    <row r="118" spans="1:10">
-      <c r="A118" s="8" t="s">
-        <v>714</v>
-      </c>
-      <c r="B118" s="8" t="s">
-        <v>580</v>
-      </c>
-      <c r="C118" s="8" t="s">
-        <v>715</v>
       </c>
       <c r="D118" s="8" t="s">
         <v>29</v>
@@ -6491,129 +6546,133 @@
         <v>155</v>
       </c>
       <c r="H118" s="8" t="s">
+        <v>713</v>
+      </c>
+      <c r="I118" s="8" t="s">
+        <v>714</v>
+      </c>
+      <c r="J118" s="8" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A119" s="8" t="s">
         <v>716</v>
       </c>
-      <c r="I118" s="8" t="s">
+      <c r="B119" s="8" t="s">
         <v>717</v>
       </c>
-      <c r="J118" s="8" t="s">
-        <v>718</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10">
-      <c r="A119" s="8" t="s">
-        <v>719</v>
-      </c>
-      <c r="B119" s="8" t="s">
-        <v>720</v>
-      </c>
-      <c r="C119" s="8"/>
+      <c r="C119" s="8" t="s">
+        <v>821</v>
+      </c>
       <c r="D119" s="8" t="s">
         <v>108</v>
       </c>
       <c r="E119" s="8"/>
       <c r="F119" s="8"/>
       <c r="G119" s="8" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H119" t="s">
+        <v>718</v>
+      </c>
+      <c r="I119" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="J119" s="8"/>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A120" s="6" t="s">
+        <v>720</v>
+      </c>
+      <c r="B120" s="6" t="s">
         <v>721</v>
       </c>
-      <c r="I119" s="17" t="s">
-        <v>722</v>
-      </c>
-      <c r="J119" s="8"/>
-    </row>
-    <row r="120" spans="1:10">
-      <c r="A120" s="6" t="s">
-        <v>723</v>
-      </c>
-      <c r="B120" s="6" t="s">
-        <v>724</v>
-      </c>
       <c r="C120" s="6" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="D120" s="6" t="s">
         <v>125</v>
       </c>
       <c r="E120" s="6"/>
       <c r="F120" s="15" t="s">
+        <v>722</v>
+      </c>
+      <c r="G120" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="H120" s="6" t="s">
+        <v>723</v>
+      </c>
+      <c r="I120" s="6" t="s">
+        <v>724</v>
+      </c>
+      <c r="J120" s="6" t="s">
         <v>725</v>
       </c>
-      <c r="G120" s="6" t="s">
-        <v>284</v>
-      </c>
-      <c r="H120" s="6" t="s">
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
         <v>726</v>
       </c>
-      <c r="I120" s="6" t="s">
+      <c r="B121" t="s">
+        <v>729</v>
+      </c>
+      <c r="D121" t="s">
+        <v>54</v>
+      </c>
+      <c r="F121" t="s">
+        <v>730</v>
+      </c>
+      <c r="G121" t="s">
+        <v>363</v>
+      </c>
+      <c r="H121" s="8" t="s">
+        <v>731</v>
+      </c>
+      <c r="I121" s="18" t="s">
+        <v>732</v>
+      </c>
+      <c r="J121" s="17" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A122" s="6" t="s">
+        <v>726</v>
+      </c>
+      <c r="B122" s="6" t="s">
         <v>727</v>
       </c>
-      <c r="J120" s="6" t="s">
+      <c r="C122" s="6" t="s">
+        <v>798</v>
+      </c>
+      <c r="D122" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="E122" s="6"/>
+      <c r="F122" s="6"/>
+      <c r="G122" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="H122" s="8" t="s">
+        <v>518</v>
+      </c>
+      <c r="I122" s="16" t="s">
         <v>728</v>
       </c>
-    </row>
-    <row r="121" spans="1:10">
-      <c r="A121" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="B121" s="6" t="s">
-        <v>730</v>
-      </c>
-      <c r="C121" s="6" t="s">
-        <v>801</v>
-      </c>
-      <c r="D121" s="6" t="s">
-        <v>514</v>
-      </c>
-      <c r="E121" s="6"/>
-      <c r="F121" s="6"/>
-      <c r="G121" s="6" t="s">
-        <v>519</v>
-      </c>
-      <c r="H121" s="8" t="s">
-        <v>520</v>
-      </c>
-      <c r="I121" s="16" t="s">
-        <v>731</v>
-      </c>
-      <c r="J121" s="6"/>
-    </row>
-    <row r="122" spans="1:10">
-      <c r="A122" t="s">
-        <v>729</v>
-      </c>
-      <c r="B122" t="s">
-        <v>732</v>
-      </c>
-      <c r="D122" t="s">
-        <v>54</v>
-      </c>
-      <c r="F122" t="s">
-        <v>733</v>
-      </c>
-      <c r="G122" t="s">
-        <v>364</v>
-      </c>
-      <c r="H122" s="8" t="s">
-        <v>734</v>
-      </c>
-      <c r="I122" s="18" t="s">
-        <v>735</v>
-      </c>
-      <c r="J122" s="17" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10">
+      <c r="J122" s="6"/>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="B123" t="s">
-        <v>602</v>
-      </c>
-      <c r="C123" s="6"/>
+        <v>600</v>
+      </c>
+      <c r="C123" s="6" t="s">
+        <v>820</v>
+      </c>
       <c r="D123" t="s">
         <v>168</v>
       </c>
@@ -6621,24 +6680,24 @@
         <v>46</v>
       </c>
       <c r="F123" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="G123" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="H123" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="I123" s="28" t="s">
-        <v>773</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124" s="6" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="B124" s="6" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="C124" s="6"/>
       <c r="D124" s="6" t="s">
@@ -6650,53 +6709,53 @@
         <v>63</v>
       </c>
       <c r="H124" s="6" t="s">
+        <v>736</v>
+      </c>
+      <c r="I124" s="16" t="s">
+        <v>737</v>
+      </c>
+      <c r="J124" s="6"/>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A125" s="6" t="s">
+        <v>738</v>
+      </c>
+      <c r="B125" s="6" t="s">
         <v>739</v>
       </c>
-      <c r="I124" s="16" t="s">
-        <v>740</v>
-      </c>
-      <c r="J124" s="6"/>
-    </row>
-    <row r="125" spans="1:10">
-      <c r="A125" s="6" t="s">
-        <v>741</v>
-      </c>
-      <c r="B125" s="6" t="s">
-        <v>742</v>
-      </c>
       <c r="C125" s="26" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="D125" s="6" t="s">
         <v>108</v>
       </c>
       <c r="E125" s="6"/>
       <c r="F125" s="6" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="G125" s="6" t="s">
         <v>31</v>
       </c>
       <c r="H125" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="I125" s="16" t="s">
+        <v>742</v>
+      </c>
+      <c r="J125" s="6"/>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A126" s="6" t="s">
+        <v>743</v>
+      </c>
+      <c r="B126" s="6" t="s">
         <v>744</v>
       </c>
-      <c r="I125" s="16" t="s">
-        <v>745</v>
-      </c>
-      <c r="J125" s="6"/>
-    </row>
-    <row r="126" spans="1:10">
-      <c r="A126" s="6" t="s">
-        <v>746</v>
-      </c>
-      <c r="B126" s="6" t="s">
-        <v>747</v>
-      </c>
       <c r="C126" s="6" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="D126" s="6" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="E126" s="6"/>
       <c r="F126" s="6"/>
@@ -6704,51 +6763,53 @@
         <v>63</v>
       </c>
       <c r="H126" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="I126" s="16" t="s">
+        <v>746</v>
+      </c>
+      <c r="J126" s="6"/>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A127" s="6" t="s">
+        <v>747</v>
+      </c>
+      <c r="B127" s="6" t="s">
         <v>748</v>
       </c>
-      <c r="I126" s="16" t="s">
+      <c r="C127" s="6" t="s">
         <v>749</v>
-      </c>
-      <c r="J126" s="6"/>
-    </row>
-    <row r="127" spans="1:10">
-      <c r="A127" s="6" t="s">
-        <v>750</v>
-      </c>
-      <c r="B127" s="6" t="s">
-        <v>751</v>
-      </c>
-      <c r="C127" s="6" t="s">
-        <v>752</v>
       </c>
       <c r="D127" s="6" t="s">
         <v>29</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="F127" s="15" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="G127" t="s">
         <v>115</v>
       </c>
       <c r="H127" s="6"/>
       <c r="I127" s="6" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="J127" s="6" t="s">
-        <v>756</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128" s="6" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="B128" s="6" t="s">
-        <v>742</v>
-      </c>
-      <c r="C128" s="6"/>
+        <v>739</v>
+      </c>
+      <c r="C128" s="6" t="s">
+        <v>818</v>
+      </c>
       <c r="D128" s="6" t="s">
         <v>108</v>
       </c>
@@ -6758,19 +6819,19 @@
         <v>109</v>
       </c>
       <c r="H128" s="6" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="I128" s="16" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="J128" s="6"/>
     </row>
-    <row r="129" spans="1:10">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129" s="8" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="B129" s="8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C129" s="8"/>
       <c r="D129" s="8" t="s">
@@ -6780,19 +6841,19 @@
         <v>85</v>
       </c>
       <c r="F129" s="8" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="G129" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="H129" s="8" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="I129" s="8" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="J129" s="12" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
     </row>
   </sheetData>
@@ -6818,8 +6879,8 @@
     <hyperlink ref="I125" r:id="rId19" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
     <hyperlink ref="I32" r:id="rId20" xr:uid="{7D21070C-9A14-48DF-982E-D995A034BDAD}"/>
     <hyperlink ref="J32" r:id="rId21" xr:uid="{6DBC4056-CB8A-487A-BF0C-E91ACD39E885}"/>
-    <hyperlink ref="I122" r:id="rId22" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
-    <hyperlink ref="J122" r:id="rId23" xr:uid="{86DA1E68-2F83-48AC-BB28-CC390F65E2B5}"/>
+    <hyperlink ref="I121" r:id="rId22" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
+    <hyperlink ref="J121" r:id="rId23" xr:uid="{86DA1E68-2F83-48AC-BB28-CC390F65E2B5}"/>
     <hyperlink ref="I67" r:id="rId24" xr:uid="{DCABBE8B-8789-4957-9A88-F8585AD53BBC}"/>
     <hyperlink ref="J67" r:id="rId25" xr:uid="{094149F7-E614-449F-AD70-7D3A82B2ADBF}"/>
     <hyperlink ref="I107" r:id="rId26" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
@@ -6851,7 +6912,7 @@
     <hyperlink ref="J68" r:id="rId52" xr:uid="{FC7B5D21-AD7E-44E8-B8C0-80D8AC1C6D3E}"/>
     <hyperlink ref="I75" r:id="rId53" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
     <hyperlink ref="I93" r:id="rId54" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
-    <hyperlink ref="I121" r:id="rId55" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
+    <hyperlink ref="I122" r:id="rId55" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
     <hyperlink ref="I82" r:id="rId56" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
     <hyperlink ref="I83" r:id="rId57" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
     <hyperlink ref="I88" r:id="rId58" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
@@ -6874,17 +6935,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CC83367596A4B94585FCDD3502D89912" ma:contentTypeVersion="11" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="4e4efa8c0f0f722bbfc4a6b86077b9b4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1" xmlns:ns3="9cb1c2f4-2737-4134-a1af-8acbe3d02830" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81c6aeae46cd0fb81a99420a9570330b" ns2:_="" ns3:_="">
     <xsd:import namespace="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
@@ -7079,6 +7129,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -7089,23 +7150,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="9cb1c2f4-2737-4134-a1af-8acbe3d02830"/>
-    <ds:schemaRef ds:uri="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCC2BCD-0310-4A3C-9E4B-6EFDEBA53649}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7124,6 +7168,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="9cb1c2f4-2737-4134-a1af-8acbe3d02830"/>
+    <ds:schemaRef ds:uri="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Ajout de Sarah-Julie Richard
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFAFAF59-86B9-4D32-AA0B-E473B8EB3B35}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C03D95A6-BC41-486F-9890-085BE7F0F3D4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19455" yWindow="4650" windowWidth="20475" windowHeight="23445" tabRatio="149" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="824">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1097" uniqueCount="830">
   <si>
     <t>nom</t>
   </si>
@@ -2520,6 +2520,24 @@
   </si>
   <si>
     <t>francois-constantin-d-amour.jpg</t>
+  </si>
+  <si>
+    <t>Richard</t>
+  </si>
+  <si>
+    <t>Sarah-Julie</t>
+  </si>
+  <si>
+    <t>Direction de la Bibliothèque des  lettres et sciences humaines et  Livres rares et collections Service du prêt entre bibliothèques</t>
+  </si>
+  <si>
+    <t>Direction de la Bibliothèque des  lettres et sciences humaines et  Livres rares et collections spéciales</t>
+  </si>
+  <si>
+    <t>514 343-6111, poste 3772</t>
+  </si>
+  <si>
+    <t>sarah-julie.richard@umontreal.ca</t>
   </si>
 </sst>
 </file>
@@ -2824,8 +2842,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J128" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:J128" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J129" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:J129" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
   <sortState ref="A2:J128">
     <sortCondition ref="C1:C128"/>
   </sortState>
@@ -3166,7 +3184,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J128"/>
+  <dimension ref="A1:J129"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.42578125" customWidth="1"/>
@@ -6840,10 +6858,32 @@
       <c r="E128" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G128" s="6"/>
-      <c r="H128" s="14"/>
-      <c r="I128" s="13"/>
+      <c r="G128" s="6" t="s">
+        <v>827</v>
+      </c>
+      <c r="H128" s="14" t="s">
+        <v>828</v>
+      </c>
+      <c r="I128" s="13" t="s">
+        <v>829</v>
+      </c>
       <c r="J128" s="20"/>
+    </row>
+    <row r="129" spans="1:10">
+      <c r="A129" t="s">
+        <v>824</v>
+      </c>
+      <c r="B129" t="s">
+        <v>825</v>
+      </c>
+      <c r="C129" s="6"/>
+      <c r="D129" t="s">
+        <v>108</v>
+      </c>
+      <c r="E129" s="6" t="s">
+        <v>826</v>
+      </c>
+      <c r="J129" s="20"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6914,16 +6954,37 @@
     <hyperlink ref="I5" r:id="rId65" xr:uid="{E26D4CB1-6F14-4277-AD54-18A052872B6B}"/>
     <hyperlink ref="I56" r:id="rId66" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
     <hyperlink ref="I34" r:id="rId67" xr:uid="{2E646106-878B-4504-8874-8750F3CAA7CB}"/>
+    <hyperlink ref="I128" r:id="rId68" xr:uid="{902A8808-023C-4EA1-833E-F687288B12ED}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId68"/>
+  <pageSetup orientation="portrait" r:id="rId69"/>
   <tableParts count="1">
-    <tablePart r:id="rId69"/>
+    <tablePart r:id="rId70"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CC83367596A4B94585FCDD3502D89912" ma:contentTypeVersion="11" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="4e4efa8c0f0f722bbfc4a6b86077b9b4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1" xmlns:ns3="9cb1c2f4-2737-4134-a1af-8acbe3d02830" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81c6aeae46cd0fb81a99420a9570330b" ns2:_="" ns3:_="">
     <xsd:import namespace="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
@@ -7118,41 +7179,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCC2BCD-0310-4A3C-9E4B-6EFDEBA53649}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
-    <ds:schemaRef ds:uri="9cb1c2f4-2737-4134-a1af-8acbe3d02830"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7175,9 +7205,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCC2BCD-0310-4A3C-9E4B-6EFDEBA53649}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
+    <ds:schemaRef ds:uri="9cb1c2f4-2737-4134-a1af-8acbe3d02830"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Mises à jours diverses
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84077DA4-37B3-42EF-9E1C-A05D879EA7EF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CB2AD0-A2A0-448A-9EA0-142730FB908C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19460" yWindow="4650" windowWidth="20480" windowHeight="23450" tabRatio="242" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19460" yWindow="4650" windowWidth="20480" windowHeight="23450" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="723">
   <si>
     <t>nom</t>
   </si>
@@ -1022,21 +1022,6 @@
     <t>marjorie.gauchier@umontreal.ca</t>
   </si>
   <si>
-    <t>Généreux Randall</t>
-  </si>
-  <si>
-    <t>Julia</t>
-  </si>
-  <si>
-    <t>Science politique, Démographie et sciences de la population, Études internationales, Études féministes, des genres et des sexualités</t>
-  </si>
-  <si>
-    <t>514 343-6111, poste 2623</t>
-  </si>
-  <si>
-    <t>julia.genereux.randall@umontreal.ca</t>
-  </si>
-  <si>
     <t>Gervais</t>
   </si>
   <si>
@@ -1139,9 +1124,6 @@
     <t>aminata-keita.jpg</t>
   </si>
   <si>
-    <t>Bibliothéconomie et sciences de l'information, Linguistique et traduction</t>
-  </si>
-  <si>
     <t>514 343-6111, poste 5411</t>
   </si>
   <si>
@@ -1241,9 +1223,6 @@
     <t>graham-lavender.jpg</t>
   </si>
   <si>
-    <t>Relations industrielles, Sciences économiques, Données statistiques</t>
-  </si>
-  <si>
     <t>514-343-6111, poste 2625</t>
   </si>
   <si>
@@ -1400,9 +1379,6 @@
     <t>pascal-martinolli.jpg</t>
   </si>
   <si>
-    <t>Histoire, formation</t>
-  </si>
-  <si>
     <t>514 343-6111, poste 3273</t>
   </si>
   <si>
@@ -1658,9 +1634,6 @@
     <t>david-patenaude.jpg</t>
   </si>
   <si>
-    <t>Criminologie, Travail social, Sécurité et études policières, Dépendances, Victimologie, Sexualité : enjeux de société et pratiques d'intervention</t>
-  </si>
-  <si>
     <t>514 343-6111, poste 2624</t>
   </si>
   <si>
@@ -2078,9 +2051,6 @@
     <t>myriam-boyer</t>
   </si>
   <si>
-    <t>julia-genereux-randall.jpg</t>
-  </si>
-  <si>
     <t>caroline-patenaude.jpg</t>
   </si>
   <si>
@@ -2235,6 +2205,18 @@
   </si>
   <si>
     <t>sarah-julie-richard.jpg</t>
+  </si>
+  <si>
+    <t>Bibliothéconomie et sciences de l'information, Relations industrielles</t>
+  </si>
+  <si>
+    <t>Histoire, Linguistique et traduction</t>
+  </si>
+  <si>
+    <t>Criminologie, Travail social, Démographie et sciences de la population, Sécurité et études policières, Dépendances, Victimologie, Sexualité : enjeux de société et pratiques d'intervention</t>
+  </si>
+  <si>
+    <t>Science politique, Études internationales, Études féministes - des genres et des sexualités, Sciences économiques, Données statistiques</t>
   </si>
 </sst>
 </file>
@@ -2549,16 +2531,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J130" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:J130" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="Service du prêt entre bibliothèques"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <sortState ref="A2:J129">
-    <sortCondition ref="A1:A129"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J129" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:J129" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
+  <sortState ref="A2:J128">
+    <sortCondition ref="A1:A128"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{4B04E1AF-0079-4AD2-81CA-E8A433733E21}" name="nom"/>
@@ -2899,7 +2875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J130"/>
+  <dimension ref="A1:J129"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="18.453125" customWidth="1"/>
@@ -2911,7 +2887,7 @@
     <col min="7" max="7" width="70.81640625" customWidth="1"/>
     <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="41.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="76.08984375" customWidth="1"/>
+    <col min="10" max="10" width="30.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -2946,7 +2922,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" hidden="1">
+    <row r="2" spans="1:10">
       <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
@@ -2977,7 +2953,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alexandre.amar-zifkin@umontreal.ca</v>
       </c>
     </row>
-    <row r="3" spans="1:10" hidden="1">
+    <row r="3" spans="1:10">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -2994,7 +2970,7 @@
         <v>42</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>670</v>
+        <v>661</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>21</v>
@@ -3010,7 +2986,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.angers@umontreal.ca</v>
       </c>
     </row>
-    <row r="4" spans="1:10" hidden="1">
+    <row r="4" spans="1:10">
       <c r="A4" s="5" t="s">
         <v>24</v>
       </c>
@@ -3041,7 +3017,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nadege.arsa@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="5" spans="1:10" hidden="1">
+    <row r="5" spans="1:10">
       <c r="A5" s="7" t="s">
         <v>32</v>
       </c>
@@ -3072,7 +3048,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=denis.arvisais@umontreal.ca</v>
       </c>
     </row>
-    <row r="6" spans="1:10" hidden="1">
+    <row r="6" spans="1:10">
       <c r="A6" s="5" t="s">
         <v>38</v>
       </c>
@@ -3092,7 +3068,7 @@
         <v>43</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>671</v>
+        <v>662</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>44</v>
@@ -3105,7 +3081,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.attia@umontreal.ca</v>
       </c>
     </row>
-    <row r="7" spans="1:10" hidden="1">
+    <row r="7" spans="1:10">
       <c r="A7" s="7" t="s">
         <v>46</v>
       </c>
@@ -3136,15 +3112,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=prlaval@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="8" spans="1:10" hidden="1">
+    <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>666</v>
+        <v>657</v>
       </c>
       <c r="B8" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>686</v>
+        <v>676</v>
       </c>
       <c r="D8" t="s">
         <v>96</v>
@@ -3153,23 +3129,23 @@
         <v>15</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>667</v>
+        <v>658</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
       </c>
       <c r="H8" t="s">
-        <v>668</v>
+        <v>659</v>
       </c>
       <c r="I8" s="21" t="s">
-        <v>669</v>
+        <v>660</v>
       </c>
       <c r="J8" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=eve.baribeau.marchand@umontreal.ca</v>
       </c>
     </row>
-    <row r="9" spans="1:10" hidden="1">
+    <row r="9" spans="1:10">
       <c r="A9" t="s">
         <v>53</v>
       </c>
@@ -3199,7 +3175,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.bastien@umontreal.ca</v>
       </c>
     </row>
-    <row r="10" spans="1:10" hidden="1">
+    <row r="10" spans="1:10">
       <c r="A10" s="5" t="s">
         <v>60</v>
       </c>
@@ -3227,7 +3203,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magalie.beaudoin@umontreal.ca</v>
       </c>
     </row>
-    <row r="11" spans="1:10" hidden="1">
+    <row r="11" spans="1:10">
       <c r="A11" s="7" t="s">
         <v>67</v>
       </c>
@@ -3244,10 +3220,10 @@
         <v>71</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>581</v>
+        <v>572</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>662</v>
+        <v>653</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>72</v>
@@ -3260,7 +3236,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maryna.beaulieu@umontreal.ca</v>
       </c>
     </row>
-    <row r="12" spans="1:10" hidden="1">
+    <row r="12" spans="1:10">
       <c r="A12" s="7" t="s">
         <v>74</v>
       </c>
@@ -3268,7 +3244,7 @@
         <v>39</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>679</v>
+        <v>669</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>75</v>
@@ -3290,7 +3266,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.begin-poissant@umontreal.ca</v>
       </c>
     </row>
-    <row r="13" spans="1:10" hidden="1">
+    <row r="13" spans="1:10">
       <c r="A13" s="7" t="s">
         <v>80</v>
       </c>
@@ -3320,7 +3296,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.belanger@umontreal.ca</v>
       </c>
     </row>
-    <row r="14" spans="1:10" hidden="1">
+    <row r="14" spans="1:10">
       <c r="A14" s="7" t="s">
         <v>88</v>
       </c>
@@ -3351,7 +3327,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amy.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="15" spans="1:10" hidden="1">
+    <row r="15" spans="1:10">
       <c r="A15" s="7" t="s">
         <v>94</v>
       </c>
@@ -3359,7 +3335,7 @@
         <v>95</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>696</v>
+        <v>686</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>96</v>
@@ -3380,7 +3356,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amelie.bernard@umontreal.ca</v>
       </c>
     </row>
-    <row r="16" spans="1:10" hidden="1">
+    <row r="16" spans="1:10">
       <c r="A16" t="s">
         <v>100</v>
       </c>
@@ -3388,7 +3364,7 @@
         <v>105</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>693</v>
+        <v>683</v>
       </c>
       <c r="D16" t="s">
         <v>96</v>
@@ -3407,7 +3383,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="17" spans="1:10" hidden="1">
+    <row r="17" spans="1:10">
       <c r="A17" s="5" t="s">
         <v>100</v>
       </c>
@@ -3436,7 +3412,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=hugo.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="18" spans="1:10" hidden="1">
+    <row r="18" spans="1:10">
       <c r="A18" s="5" t="s">
         <v>108</v>
       </c>
@@ -3467,7 +3443,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon.blais.longtin@umontreal.ca</v>
       </c>
     </row>
-    <row r="19" spans="1:10" hidden="1">
+    <row r="19" spans="1:10">
       <c r="A19" t="s">
         <v>114</v>
       </c>
@@ -3497,7 +3473,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tatiana.talpa@umontreal.ca</v>
       </c>
     </row>
-    <row r="20" spans="1:10" hidden="1">
+    <row r="20" spans="1:10">
       <c r="A20" s="8" t="s">
         <v>120</v>
       </c>
@@ -3523,7 +3499,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=joanna.bodnar@umontreal.ca</v>
       </c>
     </row>
-    <row r="21" spans="1:10" hidden="1">
+    <row r="21" spans="1:10">
       <c r="A21" s="5" t="s">
         <v>125</v>
       </c>
@@ -3553,7 +3529,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alain.borsi@umontreal.ca</v>
       </c>
     </row>
-    <row r="22" spans="1:10" hidden="1">
+    <row r="22" spans="1:10">
       <c r="A22" s="7" t="s">
         <v>133</v>
       </c>
@@ -3584,7 +3560,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.p.bouchard@umontreal.ca</v>
       </c>
     </row>
-    <row r="23" spans="1:10" hidden="1">
+    <row r="23" spans="1:10">
       <c r="A23" s="5" t="s">
         <v>140</v>
       </c>
@@ -3615,7 +3591,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refdroi@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="24" spans="1:10" hidden="1">
+    <row r="24" spans="1:10">
       <c r="A24" s="7" t="s">
         <v>146</v>
       </c>
@@ -3623,7 +3599,7 @@
         <v>147</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>675</v>
+        <v>666</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>148</v>
@@ -3632,10 +3608,10 @@
         <v>76</v>
       </c>
       <c r="F24" s="27" t="s">
-        <v>674</v>
+        <v>665</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>665</v>
+        <v>656</v>
       </c>
       <c r="H24" s="7" t="s">
         <v>149</v>
@@ -3648,7 +3624,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=myriam.boyer@umontreal.ca</v>
       </c>
     </row>
-    <row r="25" spans="1:10" hidden="1">
+    <row r="25" spans="1:10">
       <c r="A25" s="7" t="s">
         <v>151</v>
       </c>
@@ -3656,7 +3632,7 @@
         <v>152</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>690</v>
+        <v>680</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>49</v>
@@ -3666,7 +3642,7 @@
         <v>153</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>664</v>
+        <v>655</v>
       </c>
       <c r="H25" s="7" t="s">
         <v>154</v>
@@ -3679,7 +3655,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guylaine.brazeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="26" spans="1:10" hidden="1">
+    <row r="26" spans="1:10">
       <c r="A26" s="7" t="s">
         <v>156</v>
       </c>
@@ -3707,7 +3683,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sophie.brisebois@umontreal.ca</v>
       </c>
     </row>
-    <row r="27" spans="1:10" hidden="1">
+    <row r="27" spans="1:10">
       <c r="A27" t="s">
         <v>161</v>
       </c>
@@ -3715,7 +3691,7 @@
         <v>162</v>
       </c>
       <c r="C27" t="s">
-        <v>687</v>
+        <v>677</v>
       </c>
       <c r="D27" t="s">
         <v>96</v>
@@ -3734,7 +3710,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fanny.c.brochu@umontreal.ca</v>
       </c>
     </row>
-    <row r="28" spans="1:10" hidden="1">
+    <row r="28" spans="1:10">
       <c r="A28" s="5" t="s">
         <v>165</v>
       </c>
@@ -3742,7 +3718,7 @@
         <v>166</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>685</v>
+        <v>675</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>167</v>
@@ -3765,7 +3741,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=delphine.cado@umontreal.ca</v>
       </c>
     </row>
-    <row r="29" spans="1:10" hidden="1">
+    <row r="29" spans="1:10">
       <c r="A29" s="5" t="s">
         <v>172</v>
       </c>
@@ -3773,7 +3749,7 @@
         <v>173</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>688</v>
+        <v>678</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>49</v>
@@ -3796,7 +3772,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=siv.kham.chao@umontreal.ca</v>
       </c>
     </row>
-    <row r="30" spans="1:10" hidden="1">
+    <row r="30" spans="1:10">
       <c r="A30" s="5" t="s">
         <v>178</v>
       </c>
@@ -3827,7 +3803,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=laurence.charest@umontreal.ca</v>
       </c>
     </row>
-    <row r="31" spans="1:10" hidden="1">
+    <row r="31" spans="1:10">
       <c r="A31" t="s">
         <v>184</v>
       </c>
@@ -3835,7 +3811,7 @@
         <v>185</v>
       </c>
       <c r="C31" s="25" t="s">
-        <v>694</v>
+        <v>684</v>
       </c>
       <c r="D31" t="s">
         <v>27</v>
@@ -3851,7 +3827,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:10" hidden="1">
+    <row r="32" spans="1:10">
       <c r="A32" t="s">
         <v>186</v>
       </c>
@@ -3862,7 +3838,7 @@
         <v>49</v>
       </c>
       <c r="G32" t="s">
-        <v>652</v>
+        <v>643</v>
       </c>
       <c r="H32" s="7" t="s">
         <v>188</v>
@@ -3875,7 +3851,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=annick.charette@umontreal.ca</v>
       </c>
     </row>
-    <row r="33" spans="1:10" hidden="1">
+    <row r="33" spans="1:10">
       <c r="A33" s="5" t="s">
         <v>190</v>
       </c>
@@ -3890,20 +3866,20 @@
         <v>63</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>721</v>
+        <v>711</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>722</v>
+        <v>712</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>723</v>
+        <v>713</v>
       </c>
       <c r="J33" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
-    <row r="34" spans="1:10" hidden="1">
+    <row r="34" spans="1:10">
       <c r="A34" s="7" t="s">
         <v>193</v>
       </c>
@@ -3934,7 +3910,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah.cherrier@umontreal.ca</v>
       </c>
     </row>
-    <row r="35" spans="1:10" hidden="1">
+    <row r="35" spans="1:10">
       <c r="A35" s="5" t="s">
         <v>199</v>
       </c>
@@ -3964,7 +3940,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emir.chouchane@umontreal.ca</v>
       </c>
     </row>
-    <row r="36" spans="1:10" hidden="1">
+    <row r="36" spans="1:10">
       <c r="A36" s="7" t="s">
         <v>206</v>
       </c>
@@ -3972,7 +3948,7 @@
         <v>207</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>718</v>
+        <v>708</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>27</v>
@@ -3995,7 +3971,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=accessibilite@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="37" spans="1:10" hidden="1">
+    <row r="37" spans="1:10">
       <c r="A37" s="5" t="s">
         <v>211</v>
       </c>
@@ -4015,7 +3991,7 @@
         <v>216</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>650</v>
+        <v>641</v>
       </c>
       <c r="H37" s="5" t="s">
         <v>217</v>
@@ -4028,7 +4004,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benjamin.constantineau@umontreal.ca</v>
       </c>
     </row>
-    <row r="38" spans="1:10" hidden="1">
+    <row r="38" spans="1:10">
       <c r="A38" s="7" t="s">
         <v>219</v>
       </c>
@@ -4059,7 +4035,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon-pierre.crevier@umontreal.ca</v>
       </c>
     </row>
-    <row r="39" spans="1:10" hidden="1">
+    <row r="39" spans="1:10">
       <c r="A39" s="5" t="s">
         <v>225</v>
       </c>
@@ -4067,7 +4043,7 @@
         <v>226</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>709</v>
+        <v>699</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>13</v>
@@ -4090,7 +4066,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marc-olivier.croteau@umontreal.ca</v>
       </c>
     </row>
-    <row r="40" spans="1:10" hidden="1">
+    <row r="40" spans="1:10">
       <c r="A40" s="5" t="s">
         <v>230</v>
       </c>
@@ -4121,7 +4097,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.dalpe@umontreal.ca</v>
       </c>
     </row>
-    <row r="41" spans="1:10" hidden="1">
+    <row r="41" spans="1:10">
       <c r="A41" s="7" t="s">
         <v>236</v>
       </c>
@@ -4152,7 +4128,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=morgane.de.bellefeuille@umontreal.ca</v>
       </c>
     </row>
-    <row r="42" spans="1:10" hidden="1">
+    <row r="42" spans="1:10">
       <c r="A42" s="7" t="s">
         <v>244</v>
       </c>
@@ -4170,7 +4146,7 @@
         <v>247</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>652</v>
+        <v>643</v>
       </c>
       <c r="H42" s="7" t="s">
         <v>248</v>
@@ -4183,7 +4159,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=Indiana.delsart@umontreal.ca</v>
       </c>
     </row>
-    <row r="43" spans="1:10" hidden="1">
+    <row r="43" spans="1:10">
       <c r="A43" s="7" t="s">
         <v>250</v>
       </c>
@@ -4214,7 +4190,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=dominic.desaulniers@umontreal.ca</v>
       </c>
     </row>
-    <row r="44" spans="1:10" hidden="1">
+    <row r="44" spans="1:10">
       <c r="A44" s="5" t="s">
         <v>256</v>
       </c>
@@ -4222,7 +4198,7 @@
         <v>257</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>699</v>
+        <v>689</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>258</v>
@@ -4243,7 +4219,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.desrosiers@umontreal.ca</v>
       </c>
     </row>
-    <row r="45" spans="1:10" hidden="1">
+    <row r="45" spans="1:10">
       <c r="A45" t="s">
         <v>262</v>
       </c>
@@ -4251,7 +4227,7 @@
         <v>263</v>
       </c>
       <c r="C45" t="s">
-        <v>717</v>
+        <v>707</v>
       </c>
       <c r="D45" t="s">
         <v>96</v>
@@ -4270,7 +4246,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.dubois.mercier@umontreal.ca</v>
       </c>
     </row>
-    <row r="46" spans="1:10" hidden="1">
+    <row r="46" spans="1:10">
       <c r="A46" s="5" t="s">
         <v>266</v>
       </c>
@@ -4301,7 +4277,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jean-francois.durnin@umontreal.ca</v>
       </c>
     </row>
-    <row r="47" spans="1:10" hidden="1">
+    <row r="47" spans="1:10">
       <c r="A47" t="s">
         <v>272</v>
       </c>
@@ -4309,7 +4285,7 @@
         <v>273</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>705</v>
+        <v>695</v>
       </c>
       <c r="D47" t="s">
         <v>96</v>
@@ -4328,7 +4304,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=judith.fafard-larose@umontreal.ca</v>
       </c>
     </row>
-    <row r="48" spans="1:10" hidden="1">
+    <row r="48" spans="1:10">
       <c r="A48" s="7" t="s">
         <v>276</v>
       </c>
@@ -4361,7 +4337,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="49" spans="1:10" hidden="1">
+    <row r="49" spans="1:10">
       <c r="A49" s="7" t="s">
         <v>276</v>
       </c>
@@ -4372,14 +4348,14 @@
         <v>278</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>651</v>
+        <v>642</v>
       </c>
       <c r="E49" s="5" t="s">
         <v>129</v>
       </c>
       <c r="F49" s="7"/>
       <c r="G49" s="7" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="H49" s="7" t="s">
         <v>279</v>
@@ -4392,7 +4368,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="29" hidden="1">
+    <row r="50" spans="1:10" ht="29">
       <c r="A50" s="7" t="s">
         <v>281</v>
       </c>
@@ -4425,7 +4401,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=c.fortier@umontreal.ca</v>
       </c>
     </row>
-    <row r="51" spans="1:10" hidden="1">
+    <row r="51" spans="1:10">
       <c r="A51" s="7" t="s">
         <v>287</v>
       </c>
@@ -4454,7 +4430,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="52" spans="1:10" hidden="1">
+    <row r="52" spans="1:10">
       <c r="A52" s="7" t="s">
         <v>293</v>
       </c>
@@ -4485,7 +4461,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nino.gabrielli@umontreal.ca</v>
       </c>
     </row>
-    <row r="53" spans="1:10" hidden="1">
+    <row r="53" spans="1:10">
       <c r="A53" s="5" t="s">
         <v>299</v>
       </c>
@@ -4493,7 +4469,7 @@
         <v>300</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>711</v>
+        <v>701</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>301</v>
@@ -4514,7 +4490,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-pierre.gadoua@umontreal.ca</v>
       </c>
     </row>
-    <row r="54" spans="1:10" hidden="1">
+    <row r="54" spans="1:10">
       <c r="A54" s="7" t="s">
         <v>304</v>
       </c>
@@ -4545,7 +4521,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cynthia.gagne.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="55" spans="1:10" hidden="1">
+    <row r="55" spans="1:10">
       <c r="A55" s="5" t="s">
         <v>311</v>
       </c>
@@ -4573,7 +4549,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="56" spans="1:10" hidden="1">
+    <row r="56" spans="1:10">
       <c r="A56" s="5" t="s">
         <v>311</v>
       </c>
@@ -4599,7 +4575,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="57" spans="1:10" hidden="1">
+    <row r="57" spans="1:10">
       <c r="A57" s="7" t="s">
         <v>318</v>
       </c>
@@ -4629,191 +4605,189 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marjorie.gauchier@umontreal.ca</v>
       </c>
     </row>
-    <row r="58" spans="1:10" hidden="1">
+    <row r="58" spans="1:10">
       <c r="A58" s="5" t="s">
         <v>324</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="C58" s="5" t="s">
-        <v>676</v>
-      </c>
+        <v>185</v>
+      </c>
+      <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="E58" s="5"/>
       <c r="F58" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="G58" s="5" t="s">
         <v>326</v>
       </c>
-      <c r="G58" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H58" s="5" t="s">
+      <c r="H58" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="I58" s="13" t="s">
         <v>327</v>
       </c>
-      <c r="I58" s="5" t="s">
+      <c r="J58" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10">
+      <c r="A59" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="J58" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=julia.genereux.randall@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" hidden="1">
-      <c r="A59" s="5" t="s">
+      <c r="B59" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="B59" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="C59" s="5"/>
+      <c r="C59" s="5" t="s">
+        <v>681</v>
+      </c>
       <c r="D59" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E59" s="5"/>
+        <v>27</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>84</v>
+      </c>
       <c r="F59" s="5" t="s">
         <v>330</v>
       </c>
       <c r="G59" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="H59" s="8" t="s">
-        <v>551</v>
-      </c>
-      <c r="I59" s="13" t="s">
+      <c r="H59" s="5" t="s">
         <v>332</v>
       </c>
+      <c r="I59" s="5"/>
       <c r="J59" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" hidden="1">
+        <v/>
+      </c>
+    </row>
+    <row r="60" spans="1:10">
       <c r="A60" s="5" t="s">
         <v>333</v>
       </c>
       <c r="B60" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="C60" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="C60" s="5" t="s">
-        <v>691</v>
-      </c>
       <c r="D60" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>84</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="E60" s="5"/>
       <c r="F60" s="5" t="s">
         <v>335</v>
       </c>
       <c r="G60" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="H60" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="H60" s="5" t="s">
+      <c r="I60" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="I60" s="5"/>
       <c r="J60" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" spans="1:10" hidden="1">
-      <c r="A61" s="5" t="s">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
+      <c r="A61" s="7" t="s">
         <v>338</v>
       </c>
-      <c r="B61" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="C61" s="5" t="s">
+      <c r="B61" s="7" t="s">
         <v>339</v>
       </c>
-      <c r="D61" s="5" t="s">
+      <c r="C61" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="G61" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H61" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="I61" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="J61" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" s="3" customFormat="1">
+      <c r="A62" t="s">
+        <v>344</v>
+      </c>
+      <c r="B62" t="s">
+        <v>345</v>
+      </c>
+      <c r="C62" s="19" t="s">
+        <v>346</v>
+      </c>
+      <c r="D62" t="s">
         <v>13</v>
       </c>
-      <c r="E61" s="5"/>
-      <c r="F61" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="G61" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="H61" s="5" t="s">
-        <v>341</v>
-      </c>
-      <c r="I61" s="5" t="s">
-        <v>342</v>
-      </c>
-      <c r="J61" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" hidden="1">
-      <c r="A62" s="7" t="s">
-        <v>343</v>
-      </c>
-      <c r="B62" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C62" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="D62" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E62" s="7"/>
-      <c r="F62" s="7" t="s">
-        <v>346</v>
-      </c>
-      <c r="G62" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H62" s="7" t="s">
+      <c r="E62"/>
+      <c r="F62" s="28" t="s">
         <v>347</v>
       </c>
-      <c r="I62" s="7" t="s">
+      <c r="G62" t="s">
+        <v>15</v>
+      </c>
+      <c r="H62" t="s">
         <v>348</v>
       </c>
+      <c r="I62" t="s">
+        <v>349</v>
+      </c>
       <c r="J62" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" s="3" customFormat="1" hidden="1">
-      <c r="A63" t="s">
-        <v>349</v>
-      </c>
-      <c r="B63" t="s">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10">
+      <c r="A63" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="C63" s="19" t="s">
+      <c r="B63" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="D63" t="s">
-        <v>13</v>
-      </c>
-      <c r="E63"/>
-      <c r="F63" s="28" t="s">
+      <c r="C63" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="G63" t="s">
-        <v>15</v>
-      </c>
-      <c r="H63" t="s">
+      <c r="D63" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="E63" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F63" s="29"/>
+      <c r="G63" s="3"/>
+      <c r="H63" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="I63" t="s">
+      <c r="I63" s="5" t="s">
         <v>354</v>
       </c>
       <c r="J63" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" hidden="1">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" s="4" customFormat="1">
       <c r="A64" s="5" t="s">
         <v>355</v>
       </c>
@@ -4824,13 +4798,15 @@
         <v>357</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="E64" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F64" s="29"/>
-      <c r="G64" s="3"/>
+        <v>13</v>
+      </c>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5" t="s">
+        <v>719</v>
+      </c>
+      <c r="G64" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="H64" s="5" t="s">
         <v>358</v>
       </c>
@@ -4839,1119 +4815,1119 @@
       </c>
       <c r="J64" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" s="4" customFormat="1" hidden="1">
-      <c r="A65" s="5" t="s">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10">
+      <c r="A65" t="s">
         <v>360</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="B65" t="s">
         <v>361</v>
       </c>
-      <c r="C65" s="5" t="s">
+      <c r="C65" t="s">
+        <v>703</v>
+      </c>
+      <c r="D65" t="s">
+        <v>49</v>
+      </c>
+      <c r="G65" t="s">
+        <v>308</v>
+      </c>
+      <c r="H65" s="7" t="s">
         <v>362</v>
       </c>
-      <c r="D65" s="5" t="s">
+      <c r="I65" s="15" t="s">
+        <v>363</v>
+      </c>
+      <c r="J65" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10">
+      <c r="A66" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="B66" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="C66" s="7"/>
+      <c r="D66" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E66" s="7"/>
+      <c r="F66" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="G66" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="H66" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="I66" s="9" t="s">
+        <v>639</v>
+      </c>
+      <c r="J66" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10">
+      <c r="A67" t="s">
+        <v>366</v>
+      </c>
+      <c r="B67" t="s">
+        <v>105</v>
+      </c>
+      <c r="C67" t="s">
+        <v>700</v>
+      </c>
+      <c r="D67" t="s">
+        <v>96</v>
+      </c>
+      <c r="G67" t="s">
+        <v>29</v>
+      </c>
+      <c r="H67" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="I67" s="15" t="s">
+        <v>368</v>
+      </c>
+      <c r="J67" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10">
+      <c r="A68" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="D68" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E68" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F68" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="G68" s="7" t="s">
+        <v>655</v>
+      </c>
+      <c r="H68" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="I68" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="J68" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10">
+      <c r="A69" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G69" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="H69" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="I69" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="J69" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="29">
+      <c r="A70" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="D70" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E70" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="F70" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="G70" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H70" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="I70" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="J70" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10">
+      <c r="A71" t="s">
+        <v>384</v>
+      </c>
+      <c r="B71" t="s">
+        <v>385</v>
+      </c>
+      <c r="C71" s="5" t="s">
+        <v>650</v>
+      </c>
+      <c r="D71" t="s">
+        <v>96</v>
+      </c>
+      <c r="G71" t="s">
+        <v>29</v>
+      </c>
+      <c r="H71" s="16" t="s">
+        <v>386</v>
+      </c>
+      <c r="I71" s="15" t="s">
+        <v>387</v>
+      </c>
+      <c r="J71" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10">
+      <c r="A72" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="B72" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="D72" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E65" s="5"/>
-      <c r="F65" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="G65" s="5" t="s">
+      <c r="E72" s="7"/>
+      <c r="F72" s="7" t="s">
+        <v>722</v>
+      </c>
+      <c r="G72" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H65" s="5" t="s">
-        <v>364</v>
-      </c>
-      <c r="I65" s="5" t="s">
-        <v>365</v>
-      </c>
-      <c r="J65" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" hidden="1">
-      <c r="A66" t="s">
-        <v>366</v>
-      </c>
-      <c r="B66" t="s">
-        <v>367</v>
-      </c>
-      <c r="C66" t="s">
-        <v>713</v>
-      </c>
-      <c r="D66" t="s">
-        <v>49</v>
-      </c>
-      <c r="G66" t="s">
-        <v>308</v>
-      </c>
-      <c r="H66" s="7" t="s">
-        <v>368</v>
-      </c>
-      <c r="I66" s="15" t="s">
-        <v>369</v>
-      </c>
-      <c r="J66" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" hidden="1">
-      <c r="A67" s="7" t="s">
-        <v>370</v>
-      </c>
-      <c r="B67" s="7" t="s">
-        <v>334</v>
-      </c>
-      <c r="C67" s="7"/>
-      <c r="D67" s="7" t="s">
+      <c r="H72" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="I72" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="J72" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" s="3" customFormat="1">
+      <c r="A73" t="s">
+        <v>393</v>
+      </c>
+      <c r="B73" t="s">
+        <v>394</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>693</v>
+      </c>
+      <c r="D73" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E73" s="7"/>
+      <c r="F73" s="27" t="s">
+        <v>395</v>
+      </c>
+      <c r="G73" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="H73" t="s">
+        <v>396</v>
+      </c>
+      <c r="I73" s="15" t="s">
+        <v>397</v>
+      </c>
+      <c r="J73" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" s="3" customFormat="1">
+      <c r="A74" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="B74" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="D74" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="E74" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G74" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="H74" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="I74" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="J74" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10">
+      <c r="A75" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="B75" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="C75" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="F75" s="29" t="s">
+        <v>406</v>
+      </c>
+      <c r="G75" s="7" t="s">
+        <v>641</v>
+      </c>
+      <c r="H75" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="I75" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="J75" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10">
+      <c r="A76" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="C76" s="5" t="s">
+        <v>702</v>
+      </c>
+      <c r="D76" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="G76" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H76" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="I76" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="J76" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" s="3" customFormat="1" ht="29">
+      <c r="A77" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E77" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="F77" s="5"/>
+      <c r="G77" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="H77" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="I77" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="J77" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10">
+      <c r="A78" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>687</v>
+      </c>
+      <c r="D78" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E78" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F78" s="27" t="s">
+        <v>644</v>
+      </c>
+      <c r="G78" s="8" t="s">
+        <v>654</v>
+      </c>
+      <c r="H78" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="I78" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="J78" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10">
+      <c r="A79" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="D79" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E67" s="7"/>
-      <c r="F67" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="G67" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="H67" s="7" t="s">
-        <v>371</v>
-      </c>
-      <c r="I67" s="9" t="s">
-        <v>648</v>
-      </c>
-      <c r="J67" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" hidden="1">
-      <c r="A68" t="s">
-        <v>372</v>
-      </c>
-      <c r="B68" t="s">
-        <v>105</v>
-      </c>
-      <c r="C68" t="s">
-        <v>710</v>
-      </c>
-      <c r="D68" t="s">
-        <v>96</v>
-      </c>
-      <c r="G68" t="s">
-        <v>29</v>
-      </c>
-      <c r="H68" s="16" t="s">
-        <v>373</v>
-      </c>
-      <c r="I68" s="15" t="s">
-        <v>374</v>
-      </c>
-      <c r="J68" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" hidden="1">
-      <c r="A69" s="7" t="s">
-        <v>375</v>
-      </c>
-      <c r="B69" s="7" t="s">
-        <v>376</v>
-      </c>
-      <c r="C69" s="7" t="s">
-        <v>377</v>
-      </c>
-      <c r="D69" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E69" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F69" s="7" t="s">
-        <v>378</v>
-      </c>
-      <c r="G69" s="7" t="s">
-        <v>664</v>
-      </c>
-      <c r="H69" s="7" t="s">
-        <v>379</v>
-      </c>
-      <c r="I69" s="7" t="s">
-        <v>380</v>
-      </c>
-      <c r="J69" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" hidden="1">
-      <c r="A70" s="5" t="s">
-        <v>381</v>
-      </c>
-      <c r="B70" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C70" s="5" t="s">
-        <v>383</v>
-      </c>
-      <c r="D70" s="5" t="s">
-        <v>649</v>
-      </c>
-      <c r="E70" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="F70" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G70" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="H70" s="5" t="s">
-        <v>384</v>
-      </c>
-      <c r="I70" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="J70" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" ht="29" hidden="1">
-      <c r="A71" s="7" t="s">
-        <v>386</v>
-      </c>
-      <c r="B71" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="C71" s="7" t="s">
-        <v>658</v>
-      </c>
-      <c r="D71" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E71" s="17" t="s">
-        <v>284</v>
-      </c>
-      <c r="F71" s="7" t="s">
-        <v>387</v>
-      </c>
-      <c r="G71" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H71" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="I71" s="7" t="s">
-        <v>389</v>
-      </c>
-      <c r="J71" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" hidden="1">
-      <c r="A72" t="s">
-        <v>390</v>
-      </c>
-      <c r="B72" t="s">
-        <v>391</v>
-      </c>
-      <c r="C72" s="5" t="s">
-        <v>659</v>
-      </c>
-      <c r="D72" t="s">
-        <v>96</v>
-      </c>
-      <c r="G72" t="s">
-        <v>29</v>
-      </c>
-      <c r="H72" s="16" t="s">
-        <v>392</v>
-      </c>
-      <c r="I72" s="15" t="s">
-        <v>393</v>
-      </c>
-      <c r="J72" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" hidden="1">
-      <c r="A73" s="7" t="s">
-        <v>394</v>
-      </c>
-      <c r="B73" s="7" t="s">
-        <v>395</v>
-      </c>
-      <c r="C73" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="D73" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E73" s="7"/>
-      <c r="F73" s="7" t="s">
-        <v>397</v>
-      </c>
-      <c r="G73" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H73" s="7" t="s">
-        <v>398</v>
-      </c>
-      <c r="I73" s="7" t="s">
-        <v>399</v>
-      </c>
-      <c r="J73" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" s="3" customFormat="1" hidden="1">
-      <c r="A74" t="s">
-        <v>400</v>
-      </c>
-      <c r="B74" t="s">
-        <v>401</v>
-      </c>
-      <c r="C74" s="5" t="s">
-        <v>703</v>
-      </c>
-      <c r="D74" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E74" s="7"/>
-      <c r="F74" s="27" t="s">
-        <v>402</v>
-      </c>
-      <c r="G74" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="H74" t="s">
-        <v>403</v>
-      </c>
-      <c r="I74" s="15" t="s">
-        <v>404</v>
-      </c>
-      <c r="J74" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" s="3" customFormat="1" hidden="1">
-      <c r="A75" s="7" t="s">
-        <v>405</v>
-      </c>
-      <c r="B75" s="7" t="s">
-        <v>406</v>
-      </c>
-      <c r="C75" s="5" t="s">
-        <v>407</v>
-      </c>
-      <c r="D75" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="E75" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="G75" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="H75" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="I75" s="7" t="s">
-        <v>409</v>
-      </c>
-      <c r="J75" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" hidden="1">
-      <c r="A76" s="5" t="s">
-        <v>410</v>
-      </c>
-      <c r="B76" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="C76" s="5" t="s">
-        <v>412</v>
-      </c>
-      <c r="D76" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="E76" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="F76" s="29" t="s">
-        <v>413</v>
-      </c>
-      <c r="G76" s="7" t="s">
-        <v>650</v>
-      </c>
-      <c r="H76" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="I76" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="J76" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" hidden="1">
-      <c r="A77" s="7" t="s">
-        <v>416</v>
-      </c>
-      <c r="B77" s="7" t="s">
-        <v>417</v>
-      </c>
-      <c r="C77" s="5" t="s">
-        <v>712</v>
-      </c>
-      <c r="D77" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="E77" s="7" t="s">
+      <c r="E79" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="G77" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="H77" s="7" t="s">
-        <v>418</v>
-      </c>
-      <c r="I77" s="7" t="s">
-        <v>419</v>
-      </c>
-      <c r="J77" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" s="3" customFormat="1" ht="29" hidden="1">
-      <c r="A78" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="B78" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="C78" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="D78" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="E78" s="17" t="s">
-        <v>284</v>
-      </c>
-      <c r="F78" s="5"/>
-      <c r="G78" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="H78" s="5" t="s">
+      <c r="F79" s="5"/>
+      <c r="H79" s="5"/>
+      <c r="I79" s="5" t="s">
         <v>423</v>
       </c>
-      <c r="I78" s="5" t="s">
+      <c r="J79" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10">
+      <c r="A80" s="5" t="s">
         <v>424</v>
       </c>
-      <c r="J78" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" hidden="1">
-      <c r="A79" s="8" t="s">
+      <c r="B80" s="5" t="s">
         <v>425</v>
       </c>
-      <c r="B79" s="8" t="s">
+      <c r="C80" s="5" t="s">
+        <v>691</v>
+      </c>
+      <c r="D80" s="5" t="s">
         <v>426</v>
       </c>
-      <c r="C79" s="8" t="s">
-        <v>697</v>
-      </c>
-      <c r="D79" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E79" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F79" s="27" t="s">
-        <v>653</v>
-      </c>
-      <c r="G79" s="8" t="s">
-        <v>663</v>
-      </c>
-      <c r="H79" s="8" t="s">
+      <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H80" s="5" t="s">
         <v>427</v>
       </c>
-      <c r="I79" s="8" t="s">
+      <c r="I80" s="13" t="s">
         <v>428</v>
       </c>
-      <c r="J79" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" hidden="1">
-      <c r="A80" s="5" t="s">
-        <v>425</v>
-      </c>
-      <c r="B80" s="5" t="s">
+      <c r="J80" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10">
+      <c r="A81" s="5" t="s">
         <v>429</v>
       </c>
-      <c r="C80" s="5" t="s">
-        <v>698</v>
-      </c>
-      <c r="D80" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="E80" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F80" s="5"/>
-      <c r="H80" s="5"/>
-      <c r="I80" s="5" t="s">
+      <c r="B81" s="5" t="s">
         <v>430</v>
       </c>
-      <c r="J80" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" hidden="1">
-      <c r="A81" s="5" t="s">
-        <v>431</v>
-      </c>
-      <c r="B81" s="5" t="s">
-        <v>432</v>
-      </c>
       <c r="C81" s="5" t="s">
-        <v>701</v>
+        <v>706</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>433</v>
+        <v>426</v>
       </c>
       <c r="E81" s="5"/>
       <c r="F81" s="5"/>
       <c r="G81" s="5" t="s">
-        <v>57</v>
+        <v>431</v>
       </c>
       <c r="H81" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="I81" s="13" t="s">
+        <v>433</v>
+      </c>
+      <c r="J81" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10">
+      <c r="A82" s="5" t="s">
         <v>434</v>
       </c>
-      <c r="I81" s="13" t="s">
+      <c r="B82" s="5" t="s">
         <v>435</v>
       </c>
-      <c r="J81" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" hidden="1">
-      <c r="A82" s="5" t="s">
+      <c r="C82" s="5" t="s">
+        <v>705</v>
+      </c>
+      <c r="D82" s="5" t="s">
         <v>436</v>
       </c>
-      <c r="B82" s="5" t="s">
+      <c r="E82" s="5"/>
+      <c r="F82" s="27" t="s">
         <v>437</v>
       </c>
-      <c r="C82" s="5" t="s">
-        <v>716</v>
-      </c>
-      <c r="D82" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="E82" s="5"/>
-      <c r="F82" s="5"/>
       <c r="G82" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="H82" s="11" t="s">
         <v>438</v>
       </c>
-      <c r="H82" s="5" t="s">
+      <c r="I82" s="13" t="s">
         <v>439</v>
       </c>
-      <c r="I82" s="13" t="s">
+      <c r="J82" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10">
+      <c r="A83" s="5" t="s">
         <v>440</v>
       </c>
-      <c r="J82" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" hidden="1">
-      <c r="A83" s="5" t="s">
+      <c r="B83" s="5" t="s">
         <v>441</v>
       </c>
-      <c r="B83" s="5" t="s">
+      <c r="C83" s="5" t="s">
         <v>442</v>
       </c>
-      <c r="C83" s="5" t="s">
-        <v>715</v>
-      </c>
       <c r="D83" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E83" s="5"/>
+      <c r="F83" s="5" t="s">
+        <v>720</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H83" s="5" t="s">
         <v>443</v>
       </c>
-      <c r="E83" s="5"/>
-      <c r="F83" s="27" t="s">
+      <c r="I83" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="G83" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="H83" s="11" t="s">
+      <c r="J83" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10">
+      <c r="A84" s="5" t="s">
         <v>445</v>
       </c>
-      <c r="I83" s="13" t="s">
+      <c r="B84" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="C84" s="5" t="s">
         <v>446</v>
-      </c>
-      <c r="J83" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" hidden="1">
-      <c r="A84" s="5" t="s">
-        <v>447</v>
-      </c>
-      <c r="B84" s="5" t="s">
-        <v>448</v>
-      </c>
-      <c r="C84" s="5" t="s">
-        <v>449</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E84" s="5"/>
       <c r="F84" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="G84" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="H84" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="I84" s="5" t="s">
         <v>450</v>
       </c>
-      <c r="G84" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H84" s="5" t="s">
+      <c r="J84" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10">
+      <c r="A85" s="5" t="s">
         <v>451</v>
       </c>
-      <c r="I84" s="5" t="s">
+      <c r="B85" s="5" t="s">
         <v>452</v>
       </c>
-      <c r="J84" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" hidden="1">
-      <c r="A85" s="5" t="s">
+      <c r="C85" s="5" t="s">
         <v>453</v>
       </c>
-      <c r="B85" s="5" t="s">
-        <v>367</v>
-      </c>
-      <c r="C85" s="5" t="s">
+      <c r="D85" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E85" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="G85" s="5" t="s">
         <v>454</v>
       </c>
-      <c r="D85" s="5" t="s">
+      <c r="H85" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="I85" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="J85" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10">
+      <c r="A86" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="B86" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="C86" s="5" t="s">
+        <v>670</v>
+      </c>
+      <c r="D86" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="E86" s="5"/>
+      <c r="F86" s="5"/>
+      <c r="G86" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H86" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="I86" s="13" t="s">
+        <v>460</v>
+      </c>
+      <c r="J86" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10">
+      <c r="A87" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="D87" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E85" s="5"/>
-      <c r="F85" s="5" t="s">
-        <v>455</v>
-      </c>
-      <c r="G85" s="5" t="s">
-        <v>456</v>
-      </c>
-      <c r="H85" s="5" t="s">
-        <v>457</v>
-      </c>
-      <c r="I85" s="5" t="s">
-        <v>458</v>
-      </c>
-      <c r="J85" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" hidden="1">
-      <c r="A86" s="5" t="s">
-        <v>459</v>
-      </c>
-      <c r="B86" s="5" t="s">
-        <v>460</v>
-      </c>
-      <c r="C86" s="5" t="s">
-        <v>461</v>
-      </c>
-      <c r="D86" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E86" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="G86" s="5" t="s">
-        <v>462</v>
-      </c>
-      <c r="H86" s="5" t="s">
-        <v>463</v>
-      </c>
-      <c r="I86" s="5" t="s">
+      <c r="E87" s="5"/>
+      <c r="F87" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="J86" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" hidden="1">
-      <c r="A87" s="5" t="s">
+      <c r="G87" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H87" s="5" t="s">
         <v>465</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="I87" s="5" t="s">
         <v>466</v>
       </c>
-      <c r="C87" s="5" t="s">
-        <v>680</v>
-      </c>
-      <c r="D87" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="E87" s="5"/>
-      <c r="F87" s="5"/>
-      <c r="G87" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="H87" s="5" t="s">
+      <c r="J87" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10">
+      <c r="A88" s="11" t="s">
         <v>467</v>
       </c>
-      <c r="I87" s="13" t="s">
+      <c r="B88" s="11" t="s">
         <v>468</v>
       </c>
-      <c r="J87" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" hidden="1">
-      <c r="A88" s="5" t="s">
+      <c r="C88" s="5" t="s">
         <v>469</v>
-      </c>
-      <c r="B88" s="5" t="s">
-        <v>470</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>471</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E88" s="5"/>
-      <c r="F88" s="5" t="s">
+      <c r="F88" s="11" t="s">
+        <v>447</v>
+      </c>
+      <c r="G88" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="H88" s="11" t="s">
+        <v>470</v>
+      </c>
+      <c r="I88" s="11" t="s">
+        <v>471</v>
+      </c>
+      <c r="J88" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10">
+      <c r="A89" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="G88" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="H88" s="5" t="s">
+      <c r="B89" s="7" t="s">
         <v>473</v>
       </c>
-      <c r="I88" s="5" t="s">
+      <c r="C89" s="5" t="s">
         <v>474</v>
       </c>
-      <c r="J88" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" hidden="1">
-      <c r="A89" s="11" t="s">
+      <c r="D89" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E89" s="7"/>
+      <c r="F89" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G89" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="H89" s="7" t="s">
         <v>475</v>
       </c>
-      <c r="B89" s="11" t="s">
+      <c r="I89" s="7" t="s">
         <v>476</v>
       </c>
-      <c r="C89" s="5" t="s">
+      <c r="J89" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10">
+      <c r="A90" s="7" t="s">
         <v>477</v>
       </c>
-      <c r="D89" s="5" t="s">
+      <c r="B90" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="C90" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="D90" s="7" t="s">
         <v>13</v>
-      </c>
-      <c r="E89" s="5"/>
-      <c r="F89" s="11" t="s">
-        <v>455</v>
-      </c>
-      <c r="G89" s="11" t="s">
-        <v>456</v>
-      </c>
-      <c r="H89" s="11" t="s">
-        <v>478</v>
-      </c>
-      <c r="I89" s="11" t="s">
-        <v>479</v>
-      </c>
-      <c r="J89" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" hidden="1">
-      <c r="A90" s="7" t="s">
-        <v>480</v>
-      </c>
-      <c r="B90" s="7" t="s">
-        <v>481</v>
-      </c>
-      <c r="C90" s="5" t="s">
-        <v>482</v>
-      </c>
-      <c r="D90" s="7" t="s">
-        <v>111</v>
       </c>
       <c r="E90" s="7"/>
       <c r="F90" s="7" t="s">
-        <v>28</v>
+        <v>480</v>
       </c>
       <c r="G90" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="H90" s="7" t="s">
+        <v>481</v>
+      </c>
+      <c r="I90" s="7" t="s">
+        <v>482</v>
+      </c>
+      <c r="J90" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=assia.mourid@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10">
+      <c r="A91" t="s">
+        <v>483</v>
+      </c>
+      <c r="B91" t="s">
+        <v>484</v>
+      </c>
+      <c r="C91" s="5" t="s">
+        <v>671</v>
+      </c>
+      <c r="D91" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E91" s="7"/>
+      <c r="F91" s="27" t="s">
+        <v>485</v>
+      </c>
+      <c r="G91" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="H90" s="7" t="s">
-        <v>483</v>
-      </c>
-      <c r="I90" s="7" t="s">
-        <v>484</v>
-      </c>
-      <c r="J90" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" hidden="1">
-      <c r="A91" s="7" t="s">
-        <v>485</v>
-      </c>
-      <c r="B91" s="7" t="s">
+      <c r="H91" t="s">
         <v>486</v>
       </c>
-      <c r="C91" s="5" t="s">
+      <c r="I91" s="15" t="s">
         <v>487</v>
       </c>
-      <c r="D91" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E91" s="7"/>
-      <c r="F91" s="7" t="s">
+      <c r="J91" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10">
+      <c r="A92" s="11" t="s">
         <v>488</v>
       </c>
-      <c r="G91" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="H91" s="7" t="s">
+      <c r="B92" s="11" t="s">
         <v>489</v>
       </c>
-      <c r="I91" s="7" t="s">
+      <c r="C92" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="D92" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="E92" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F92" s="29"/>
+      <c r="G92" s="11" t="s">
+        <v>663</v>
+      </c>
+      <c r="H92" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="J91" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=assia.mourid@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" hidden="1">
-      <c r="A92" t="s">
+      <c r="I92" s="11" t="s">
         <v>491</v>
       </c>
-      <c r="B92" t="s">
+      <c r="J92" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10">
+      <c r="A93" s="7" t="s">
         <v>492</v>
       </c>
-      <c r="C92" s="5" t="s">
-        <v>681</v>
-      </c>
-      <c r="D92" s="7" t="s">
+      <c r="B93" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="C93" s="7" t="s">
+        <v>698</v>
+      </c>
+      <c r="D93" s="7" t="s">
+        <v>494</v>
+      </c>
+      <c r="E93" s="7"/>
+      <c r="F93" s="7" t="s">
+        <v>495</v>
+      </c>
+      <c r="G93" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="H93" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="I93" s="7" t="s">
+        <v>497</v>
+      </c>
+      <c r="J93" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" s="3" customFormat="1">
+      <c r="A94" s="7" t="s">
+        <v>498</v>
+      </c>
+      <c r="B94" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="C94" s="7"/>
+      <c r="D94" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="E94" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F94" s="7"/>
+      <c r="G94"/>
+      <c r="H94" s="7" t="s">
+        <v>500</v>
+      </c>
+      <c r="I94" s="7" t="s">
+        <v>501</v>
+      </c>
+      <c r="J94" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" s="3" customFormat="1">
+      <c r="A95" s="7" t="s">
+        <v>502</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>652</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E95" s="17"/>
+      <c r="F95" s="8" t="s">
+        <v>572</v>
+      </c>
+      <c r="G95" t="s">
+        <v>573</v>
+      </c>
+      <c r="H95" s="7" t="s">
+        <v>504</v>
+      </c>
+      <c r="I95" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="J95" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10">
+      <c r="A96" s="7" t="s">
+        <v>506</v>
+      </c>
+      <c r="B96" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="C96" s="7"/>
+      <c r="D96" s="7" t="s">
+        <v>508</v>
+      </c>
+      <c r="E96" s="5"/>
+      <c r="F96" s="27" t="s">
+        <v>509</v>
+      </c>
+      <c r="G96" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="H96" s="7"/>
+      <c r="I96" s="14" t="s">
+        <v>510</v>
+      </c>
+      <c r="J96" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10">
+      <c r="A97" t="s">
+        <v>511</v>
+      </c>
+      <c r="B97" t="s">
+        <v>512</v>
+      </c>
+      <c r="C97" s="23" t="s">
+        <v>513</v>
+      </c>
+      <c r="D97" t="s">
         <v>27</v>
       </c>
-      <c r="E92" s="7"/>
-      <c r="F92" s="27" t="s">
-        <v>493</v>
-      </c>
-      <c r="G92" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="H92" t="s">
-        <v>494</v>
-      </c>
-      <c r="I92" s="15" t="s">
-        <v>495</v>
-      </c>
-      <c r="J92" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" hidden="1">
-      <c r="A93" s="11" t="s">
-        <v>496</v>
-      </c>
-      <c r="B93" s="11" t="s">
-        <v>497</v>
-      </c>
-      <c r="C93" s="11" t="s">
-        <v>689</v>
-      </c>
-      <c r="D93" s="11" t="s">
-        <v>239</v>
-      </c>
-      <c r="E93" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F93" s="29"/>
-      <c r="G93" s="11" t="s">
-        <v>672</v>
-      </c>
-      <c r="H93" s="11" t="s">
-        <v>498</v>
-      </c>
-      <c r="I93" s="11" t="s">
-        <v>499</v>
-      </c>
-      <c r="J93" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" hidden="1">
-      <c r="A94" s="7" t="s">
-        <v>500</v>
-      </c>
-      <c r="B94" s="7" t="s">
-        <v>501</v>
-      </c>
-      <c r="C94" s="7" t="s">
-        <v>708</v>
-      </c>
-      <c r="D94" s="7" t="s">
-        <v>502</v>
-      </c>
-      <c r="E94" s="7"/>
-      <c r="F94" s="7" t="s">
-        <v>503</v>
-      </c>
-      <c r="G94" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="H94" s="7" t="s">
-        <v>504</v>
-      </c>
-      <c r="I94" s="7" t="s">
-        <v>505</v>
-      </c>
-      <c r="J94" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" s="3" customFormat="1" hidden="1">
-      <c r="A95" s="7" t="s">
-        <v>506</v>
-      </c>
-      <c r="B95" s="7" t="s">
-        <v>507</v>
-      </c>
-      <c r="C95" s="7"/>
-      <c r="D95" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="E95" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F95" s="7"/>
-      <c r="G95"/>
-      <c r="H95" s="7" t="s">
-        <v>508</v>
-      </c>
-      <c r="I95" s="7" t="s">
-        <v>509</v>
-      </c>
-      <c r="J95" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" s="3" customFormat="1">
-      <c r="A96" s="7" t="s">
-        <v>510</v>
-      </c>
-      <c r="B96" s="7" t="s">
-        <v>511</v>
-      </c>
-      <c r="C96" s="7" t="s">
-        <v>661</v>
-      </c>
-      <c r="D96" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E96" s="17"/>
-      <c r="F96" s="8" t="s">
-        <v>581</v>
-      </c>
-      <c r="G96" t="s">
-        <v>582</v>
-      </c>
-      <c r="H96" s="7" t="s">
-        <v>512</v>
-      </c>
-      <c r="I96" s="7" t="s">
-        <v>513</v>
-      </c>
-      <c r="J96" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" hidden="1">
-      <c r="A97" s="7" t="s">
+      <c r="E97" t="s">
+        <v>84</v>
+      </c>
+      <c r="F97" s="28" t="s">
         <v>514</v>
       </c>
-      <c r="B97" s="7" t="s">
+      <c r="G97" t="s">
+        <v>103</v>
+      </c>
+      <c r="I97" t="s">
         <v>515</v>
       </c>
-      <c r="C97" s="7"/>
-      <c r="D97" s="7" t="s">
+      <c r="J97" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10">
+      <c r="A98" s="5" t="s">
         <v>516</v>
       </c>
-      <c r="E97" s="5"/>
-      <c r="F97" s="27" t="s">
+      <c r="B98" s="5" t="s">
         <v>517</v>
       </c>
-      <c r="G97" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="H97" s="7"/>
-      <c r="I97" s="14" t="s">
+      <c r="C98" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F98" s="5" t="s">
         <v>518</v>
-      </c>
-      <c r="J97" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10" hidden="1">
-      <c r="A98" t="s">
-        <v>519</v>
-      </c>
-      <c r="B98" t="s">
-        <v>520</v>
-      </c>
-      <c r="C98" s="23" t="s">
-        <v>521</v>
-      </c>
-      <c r="D98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E98" t="s">
-        <v>84</v>
-      </c>
-      <c r="F98" s="28" t="s">
-        <v>522</v>
       </c>
       <c r="G98" t="s">
         <v>103</v>
       </c>
-      <c r="I98" t="s">
+      <c r="H98" s="11" t="s">
+        <v>519</v>
+      </c>
+      <c r="I98" s="11" t="s">
+        <v>520</v>
+      </c>
+      <c r="J98" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=eve.paquette-bigras@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10">
+      <c r="A99" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="B99" s="7" t="s">
+        <v>526</v>
+      </c>
+      <c r="C99" s="7" t="s">
+        <v>527</v>
+      </c>
+      <c r="D99" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E99" s="7"/>
+      <c r="F99" s="7" t="s">
+        <v>721</v>
+      </c>
+      <c r="G99" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H99" s="8" t="s">
+        <v>528</v>
+      </c>
+      <c r="I99" s="8" t="s">
+        <v>529</v>
+      </c>
+      <c r="J99" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10">
+      <c r="A100" s="5" t="s">
+        <v>521</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="C100" s="5" t="s">
+        <v>667</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E100" s="5"/>
+      <c r="F100" s="5" t="s">
         <v>523</v>
       </c>
-      <c r="J98" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="99" spans="1:10" hidden="1">
-      <c r="A99" s="5" t="s">
+      <c r="G100" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H100" s="11" t="s">
         <v>524</v>
       </c>
-      <c r="B99" s="5" t="s">
+      <c r="I100" s="11" t="s">
         <v>525</v>
       </c>
-      <c r="C99" s="5" t="s">
-        <v>700</v>
-      </c>
-      <c r="D99" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="E99" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F99" s="5" t="s">
-        <v>526</v>
-      </c>
-      <c r="G99" t="s">
-        <v>103</v>
-      </c>
-      <c r="H99" s="11" t="s">
-        <v>527</v>
-      </c>
-      <c r="I99" s="11" t="s">
-        <v>528</v>
-      </c>
-      <c r="J99" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=eve.paquette-bigras@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="100" spans="1:10" hidden="1">
-      <c r="A100" s="7" t="s">
-        <v>529</v>
-      </c>
-      <c r="B100" s="7" t="s">
-        <v>534</v>
-      </c>
-      <c r="C100" s="7" t="s">
-        <v>535</v>
-      </c>
-      <c r="D100" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E100" s="7"/>
-      <c r="F100" s="7" t="s">
-        <v>536</v>
-      </c>
-      <c r="G100" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H100" s="8" t="s">
-        <v>537</v>
-      </c>
-      <c r="I100" s="8" t="s">
-        <v>538</v>
-      </c>
       <c r="J100" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10" hidden="1">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" s="4" customFormat="1">
       <c r="A101" s="5" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>530</v>
+        <v>312</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>677</v>
+        <v>531</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E101" s="5"/>
       <c r="F101" s="5" t="s">
-        <v>531</v>
+        <v>143</v>
       </c>
       <c r="G101" s="5" t="s">
-        <v>29</v>
+        <v>97</v>
       </c>
       <c r="H101" s="11" t="s">
         <v>532</v>
@@ -5961,854 +5937,823 @@
       </c>
       <c r="J101" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="102" spans="1:10" s="4" customFormat="1" hidden="1">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" s="4" customFormat="1">
       <c r="A102" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E102" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F102" s="5" t="s">
+        <v>536</v>
+      </c>
+      <c r="H102" s="11"/>
+      <c r="I102" s="10" t="s">
+        <v>537</v>
+      </c>
+      <c r="J102" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10">
+      <c r="A103" s="7" t="s">
+        <v>538</v>
+      </c>
+      <c r="B103" s="7" t="s">
         <v>539</v>
       </c>
-      <c r="B102" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="C102" s="5" t="s">
+      <c r="C103" s="7" t="s">
         <v>540</v>
       </c>
-      <c r="D102" s="5" t="s">
+      <c r="D103" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E102" s="5"/>
-      <c r="F102" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="G102" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="H102" s="11" t="s">
+      <c r="E103" s="7"/>
+      <c r="F103" s="7" t="s">
         <v>541</v>
       </c>
-      <c r="I102" s="11" t="s">
+      <c r="G103" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="H103" s="8" t="s">
         <v>542</v>
       </c>
-      <c r="J102" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="103" spans="1:10" s="4" customFormat="1" hidden="1">
-      <c r="A103" s="5" t="s">
+      <c r="I103" s="8" t="s">
         <v>543</v>
       </c>
-      <c r="B103" s="5" t="s">
-        <v>492</v>
-      </c>
-      <c r="C103" s="5" t="s">
+      <c r="J103" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10">
+      <c r="A104" s="7" t="s">
         <v>544</v>
       </c>
-      <c r="D103" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E103" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F103" s="5" t="s">
+      <c r="B104" s="7" t="s">
         <v>545</v>
       </c>
-      <c r="H103" s="11"/>
-      <c r="I103" s="10" t="s">
+      <c r="C104" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="D104" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E104" s="7"/>
+      <c r="F104" s="7"/>
+      <c r="G104" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H104" s="8" t="s">
         <v>546</v>
       </c>
-      <c r="J103" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="104" spans="1:10" hidden="1">
-      <c r="A104" s="7" t="s">
+      <c r="I104" s="14" t="s">
         <v>547</v>
       </c>
-      <c r="B104" s="7" t="s">
+      <c r="J104" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10">
+      <c r="A105" t="s">
         <v>548</v>
       </c>
-      <c r="C104" s="7" t="s">
+      <c r="B105" t="s">
         <v>549</v>
       </c>
-      <c r="D104" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E104" s="7"/>
-      <c r="F104" s="7" t="s">
+      <c r="C105" t="s">
+        <v>692</v>
+      </c>
+      <c r="D105" t="s">
+        <v>426</v>
+      </c>
+      <c r="G105" t="s">
+        <v>643</v>
+      </c>
+      <c r="H105" s="7" t="s">
         <v>550</v>
       </c>
-      <c r="G104" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="H104" s="8" t="s">
+      <c r="I105" s="15" t="s">
         <v>551</v>
       </c>
-      <c r="I104" s="8" t="s">
+      <c r="J105" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10">
+      <c r="A106" t="s">
         <v>552</v>
       </c>
-      <c r="J104" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" hidden="1">
-      <c r="A105" s="7" t="s">
+      <c r="B106" t="s">
         <v>553</v>
       </c>
-      <c r="B105" s="7" t="s">
+      <c r="C106" s="25"/>
+      <c r="D106" t="s">
+        <v>96</v>
+      </c>
+      <c r="G106" t="s">
+        <v>29</v>
+      </c>
+      <c r="H106" t="s">
         <v>554</v>
       </c>
-      <c r="C105" s="5" t="s">
-        <v>714</v>
-      </c>
-      <c r="D105" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="E105" s="7"/>
-      <c r="F105" s="7"/>
-      <c r="G105" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H105" s="8" t="s">
+      <c r="I106" s="15" t="s">
         <v>555</v>
       </c>
-      <c r="I105" s="14" t="s">
-        <v>556</v>
-      </c>
-      <c r="J105" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" hidden="1">
-      <c r="A106" t="s">
-        <v>557</v>
-      </c>
-      <c r="B106" t="s">
-        <v>558</v>
-      </c>
-      <c r="C106" t="s">
-        <v>702</v>
-      </c>
-      <c r="D106" t="s">
-        <v>433</v>
-      </c>
-      <c r="G106" t="s">
-        <v>652</v>
-      </c>
-      <c r="H106" s="7" t="s">
-        <v>559</v>
-      </c>
-      <c r="I106" s="15" t="s">
-        <v>560</v>
-      </c>
       <c r="J106" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="107" spans="1:10" hidden="1">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10">
       <c r="A107" t="s">
-        <v>561</v>
+        <v>709</v>
       </c>
       <c r="B107" t="s">
-        <v>562</v>
-      </c>
-      <c r="C107" s="25"/>
+        <v>710</v>
+      </c>
+      <c r="C107" s="5" t="s">
+        <v>718</v>
+      </c>
       <c r="D107" t="s">
         <v>96</v>
       </c>
+      <c r="E107" s="5"/>
+      <c r="F107" s="8" t="s">
+        <v>572</v>
+      </c>
       <c r="G107" t="s">
-        <v>29</v>
+        <v>573</v>
       </c>
       <c r="H107" t="s">
-        <v>563</v>
-      </c>
-      <c r="I107" s="15" t="s">
-        <v>564</v>
+        <v>712</v>
+      </c>
+      <c r="I107" s="21" t="s">
+        <v>713</v>
       </c>
       <c r="J107" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
     <row r="108" spans="1:10">
       <c r="A108" t="s">
-        <v>719</v>
+        <v>556</v>
       </c>
       <c r="B108" t="s">
-        <v>720</v>
-      </c>
-      <c r="C108" s="5" t="s">
-        <v>728</v>
+        <v>54</v>
+      </c>
+      <c r="C108" s="19" t="s">
+        <v>557</v>
       </c>
       <c r="D108" t="s">
-        <v>96</v>
-      </c>
-      <c r="E108" s="5"/>
-      <c r="F108" s="8" t="s">
-        <v>581</v>
+        <v>13</v>
+      </c>
+      <c r="F108" s="28" t="s">
+        <v>558</v>
       </c>
       <c r="G108" t="s">
-        <v>582</v>
-      </c>
-      <c r="H108" t="s">
-        <v>722</v>
-      </c>
-      <c r="I108" s="21" t="s">
-        <v>723</v>
+        <v>29</v>
+      </c>
+      <c r="H108" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="I108" s="3" t="s">
+        <v>560</v>
       </c>
       <c r="J108" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10" hidden="1">
-      <c r="A109" t="s">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10">
+      <c r="A109" s="5" t="s">
+        <v>561</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="C109" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="E109" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F109" s="5"/>
+      <c r="H109" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="I109" s="11" t="s">
+        <v>563</v>
+      </c>
+      <c r="J109" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10">
+      <c r="A110" s="5" t="s">
+        <v>564</v>
+      </c>
+      <c r="B110" s="5" t="s">
         <v>565</v>
       </c>
-      <c r="B109" t="s">
-        <v>54</v>
-      </c>
-      <c r="C109" s="19" t="s">
+      <c r="C110" s="5" t="s">
+        <v>673</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E110" s="5"/>
+      <c r="F110" s="5" t="s">
         <v>566</v>
       </c>
-      <c r="D109" t="s">
-        <v>13</v>
-      </c>
-      <c r="F109" s="28" t="s">
+      <c r="G110" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="H110" s="11"/>
+      <c r="I110" s="11" t="s">
         <v>567</v>
       </c>
-      <c r="G109" t="s">
+      <c r="J110" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10">
+      <c r="A111" t="s">
+        <v>568</v>
+      </c>
+      <c r="B111" t="s">
+        <v>569</v>
+      </c>
+      <c r="C111" s="25" t="s">
+        <v>668</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="E111" s="5"/>
+      <c r="F111" s="5"/>
+      <c r="G111" t="s">
         <v>29</v>
       </c>
-      <c r="H109" s="3" t="s">
-        <v>568</v>
-      </c>
-      <c r="I109" s="3" t="s">
-        <v>569</v>
-      </c>
-      <c r="J109" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" hidden="1">
-      <c r="A110" s="5" t="s">
+      <c r="J111" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112" spans="1:10">
+      <c r="A112" s="8" t="s">
         <v>570</v>
       </c>
-      <c r="B110" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="C110" s="5" t="s">
+      <c r="B112" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C112" s="7" t="s">
         <v>571</v>
       </c>
-      <c r="D110" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="E110" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F110" s="5"/>
-      <c r="H110" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="I110" s="11" t="s">
+      <c r="D112" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E112" s="8"/>
+      <c r="F112" s="8" t="s">
         <v>572</v>
       </c>
-      <c r="J110" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="111" spans="1:10" hidden="1">
-      <c r="A111" s="5" t="s">
+      <c r="G112" s="8" t="s">
         <v>573</v>
       </c>
-      <c r="B111" s="5" t="s">
+      <c r="H112" s="8" t="s">
         <v>574</v>
       </c>
-      <c r="C111" s="5" t="s">
-        <v>683</v>
-      </c>
-      <c r="D111" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E111" s="5"/>
-      <c r="F111" s="5" t="s">
+      <c r="I112" s="8" t="s">
         <v>575</v>
       </c>
-      <c r="G111" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="H111" s="11"/>
-      <c r="I111" s="11" t="s">
-        <v>576</v>
-      </c>
-      <c r="J111" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10" hidden="1">
-      <c r="A112" t="s">
-        <v>577</v>
-      </c>
-      <c r="B112" t="s">
-        <v>578</v>
-      </c>
-      <c r="C112" s="25" t="s">
-        <v>678</v>
-      </c>
-      <c r="D112" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="E112" s="5"/>
-      <c r="F112" s="5"/>
-      <c r="G112" t="s">
-        <v>29</v>
-      </c>
       <c r="J112" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v/>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
       </c>
     </row>
     <row r="113" spans="1:10">
       <c r="A113" s="8" t="s">
+        <v>576</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="C113" s="24"/>
+      <c r="D113" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F113" s="8"/>
+      <c r="G113" s="8"/>
+      <c r="H113" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="I113" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="J113" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10">
+      <c r="A114" s="5" t="s">
         <v>579</v>
       </c>
-      <c r="B113" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C113" s="7" t="s">
+      <c r="B114" s="5" t="s">
         <v>580</v>
       </c>
-      <c r="D113" s="8" t="s">
+      <c r="C114" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="E114" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G114" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="H114" s="5" t="s">
+        <v>582</v>
+      </c>
+      <c r="I114" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="J114" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10">
+      <c r="A115" s="5" t="s">
+        <v>584</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>585</v>
+      </c>
+      <c r="C115" s="20" t="s">
+        <v>682</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="E115" s="5"/>
+      <c r="F115" s="5"/>
+      <c r="G115" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="H115" s="5"/>
+      <c r="I115" s="13" t="s">
+        <v>586</v>
+      </c>
+      <c r="J115" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10">
+      <c r="A116" s="11" t="s">
+        <v>587</v>
+      </c>
+      <c r="B116" s="11" t="s">
+        <v>588</v>
+      </c>
+      <c r="C116" s="22" t="s">
+        <v>589</v>
+      </c>
+      <c r="D116" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="E116" t="s">
+        <v>590</v>
+      </c>
+      <c r="F116" s="11" t="s">
+        <v>591</v>
+      </c>
+      <c r="G116" s="11" t="s">
+        <v>662</v>
+      </c>
+      <c r="H116" s="11" t="s">
+        <v>592</v>
+      </c>
+      <c r="I116" s="11" t="s">
+        <v>593</v>
+      </c>
+      <c r="J116" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10">
+      <c r="A117" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="B117" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="C117" s="7" t="s">
+        <v>595</v>
+      </c>
+      <c r="D117" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E113" s="8"/>
-      <c r="F113" s="8" t="s">
-        <v>581</v>
-      </c>
-      <c r="G113" s="8" t="s">
-        <v>582</v>
-      </c>
-      <c r="H113" s="8" t="s">
-        <v>583</v>
-      </c>
-      <c r="I113" s="8" t="s">
-        <v>584</v>
-      </c>
-      <c r="J113" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10" hidden="1">
-      <c r="A114" s="8" t="s">
-        <v>585</v>
-      </c>
-      <c r="B114" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="C114" s="24"/>
-      <c r="D114" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="E114" s="8" t="s">
+      <c r="E117" s="7"/>
+      <c r="F117" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="G117" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="H117" s="7" t="s">
+        <v>596</v>
+      </c>
+      <c r="I117" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="J117" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10">
+      <c r="A118" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="B118" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="C118" s="7" t="s">
+        <v>697</v>
+      </c>
+      <c r="D118" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E118" s="7"/>
+      <c r="F118" s="7"/>
+      <c r="G118" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="H118" t="s">
+        <v>600</v>
+      </c>
+      <c r="I118" s="14" t="s">
+        <v>601</v>
+      </c>
+      <c r="J118" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10">
+      <c r="A119" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="C119" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E119" s="5"/>
+      <c r="F119" s="5" t="s">
+        <v>604</v>
+      </c>
+      <c r="G119" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="H119" s="5" t="s">
+        <v>605</v>
+      </c>
+      <c r="I119" s="5" t="s">
+        <v>606</v>
+      </c>
+      <c r="J119" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10">
+      <c r="A120" s="5" t="s">
+        <v>607</v>
+      </c>
+      <c r="B120" s="5" t="s">
+        <v>608</v>
+      </c>
+      <c r="C120" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="E120" s="5"/>
+      <c r="F120" s="5"/>
+      <c r="G120" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H120" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="I120" s="13" t="s">
+        <v>609</v>
+      </c>
+      <c r="J120" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10">
+      <c r="A121" t="s">
+        <v>607</v>
+      </c>
+      <c r="B121" t="s">
+        <v>610</v>
+      </c>
+      <c r="D121" t="s">
+        <v>49</v>
+      </c>
+      <c r="F121" s="27" t="s">
+        <v>611</v>
+      </c>
+      <c r="G121" t="s">
+        <v>308</v>
+      </c>
+      <c r="H121" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="I121" s="15" t="s">
+        <v>613</v>
+      </c>
+      <c r="J121" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10">
+      <c r="A122" t="s">
+        <v>645</v>
+      </c>
+      <c r="B122" t="s">
+        <v>503</v>
+      </c>
+      <c r="C122" s="5" t="s">
+        <v>696</v>
+      </c>
+      <c r="D122" t="s">
+        <v>148</v>
+      </c>
+      <c r="E122" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F114" s="8"/>
-      <c r="G114" s="8"/>
-      <c r="H114" s="8" t="s">
-        <v>586</v>
-      </c>
-      <c r="I114" s="8" t="s">
-        <v>587</v>
-      </c>
-      <c r="J114" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" hidden="1">
-      <c r="A115" s="5" t="s">
-        <v>588</v>
-      </c>
-      <c r="B115" s="5" t="s">
-        <v>589</v>
-      </c>
-      <c r="C115" s="20" t="s">
-        <v>590</v>
-      </c>
-      <c r="D115" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="E115" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G115" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="H115" s="5" t="s">
-        <v>591</v>
-      </c>
-      <c r="I115" s="5" t="s">
-        <v>592</v>
-      </c>
-      <c r="J115" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="116" spans="1:10" hidden="1">
-      <c r="A116" s="5" t="s">
-        <v>593</v>
-      </c>
-      <c r="B116" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="C116" s="20" t="s">
-        <v>692</v>
-      </c>
-      <c r="D116" s="5" t="s">
+      <c r="F122" s="27" t="s">
+        <v>646</v>
+      </c>
+      <c r="G122" t="s">
+        <v>664</v>
+      </c>
+      <c r="H122" t="s">
+        <v>647</v>
+      </c>
+      <c r="I122" s="21" t="s">
+        <v>648</v>
+      </c>
+      <c r="J122" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10">
+      <c r="A123" s="5" t="s">
+        <v>614</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="C123" s="20"/>
+      <c r="D123" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E116" s="5"/>
-      <c r="F116" s="5"/>
-      <c r="G116" s="5" t="s">
-        <v>456</v>
-      </c>
-      <c r="H116" s="5"/>
-      <c r="I116" s="13" t="s">
-        <v>595</v>
-      </c>
-      <c r="J116" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="117" spans="1:10" hidden="1">
-      <c r="A117" s="11" t="s">
-        <v>596</v>
-      </c>
-      <c r="B117" s="11" t="s">
-        <v>597</v>
-      </c>
-      <c r="C117" s="22" t="s">
-        <v>598</v>
-      </c>
-      <c r="D117" s="11" t="s">
-        <v>289</v>
-      </c>
-      <c r="E117" t="s">
-        <v>599</v>
-      </c>
-      <c r="F117" s="11" t="s">
-        <v>600</v>
-      </c>
-      <c r="G117" s="11" t="s">
-        <v>671</v>
-      </c>
-      <c r="H117" s="11" t="s">
-        <v>601</v>
-      </c>
-      <c r="I117" s="11" t="s">
-        <v>602</v>
-      </c>
-      <c r="J117" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="118" spans="1:10" hidden="1">
-      <c r="A118" s="7" t="s">
-        <v>603</v>
-      </c>
-      <c r="B118" s="7" t="s">
-        <v>492</v>
-      </c>
-      <c r="C118" s="7" t="s">
-        <v>604</v>
-      </c>
-      <c r="D118" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E118" s="7"/>
-      <c r="F118" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="G118" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="H118" s="7" t="s">
-        <v>605</v>
-      </c>
-      <c r="I118" s="7" t="s">
-        <v>606</v>
-      </c>
-      <c r="J118" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10" hidden="1">
-      <c r="A119" s="7" t="s">
-        <v>607</v>
-      </c>
-      <c r="B119" s="7" t="s">
-        <v>608</v>
-      </c>
-      <c r="C119" s="7" t="s">
-        <v>707</v>
-      </c>
-      <c r="D119" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="E119" s="7"/>
-      <c r="F119" s="7"/>
-      <c r="G119" s="7" t="s">
-        <v>456</v>
-      </c>
-      <c r="H119" t="s">
-        <v>609</v>
-      </c>
-      <c r="I119" s="14" t="s">
-        <v>610</v>
-      </c>
-      <c r="J119" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" hidden="1">
-      <c r="A120" s="5" t="s">
-        <v>611</v>
-      </c>
-      <c r="B120" s="5" t="s">
-        <v>612</v>
-      </c>
-      <c r="C120" s="5" t="s">
-        <v>682</v>
-      </c>
-      <c r="D120" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="E120" s="5"/>
-      <c r="F120" s="5" t="s">
-        <v>613</v>
-      </c>
-      <c r="G120" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="H120" s="5" t="s">
-        <v>614</v>
-      </c>
-      <c r="I120" s="5" t="s">
-        <v>615</v>
-      </c>
-      <c r="J120" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" hidden="1">
-      <c r="A121" s="5" t="s">
+      <c r="E123" s="5"/>
+      <c r="F123" s="5"/>
+      <c r="G123" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H123" s="5" t="s">
         <v>616</v>
       </c>
-      <c r="B121" s="5" t="s">
+      <c r="I123" s="13" t="s">
         <v>617</v>
       </c>
-      <c r="C121" s="5" t="s">
-        <v>684</v>
-      </c>
-      <c r="D121" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="E121" s="5"/>
-      <c r="F121" s="5"/>
-      <c r="G121" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="H121" s="7" t="s">
-        <v>439</v>
-      </c>
-      <c r="I121" s="13" t="s">
+      <c r="J123" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10">
+      <c r="A124" s="5" t="s">
         <v>618</v>
       </c>
-      <c r="J121" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" hidden="1">
-      <c r="A122" t="s">
-        <v>616</v>
-      </c>
-      <c r="B122" t="s">
+      <c r="B124" s="5" t="s">
         <v>619</v>
       </c>
-      <c r="D122" t="s">
-        <v>49</v>
-      </c>
-      <c r="F122" s="27" t="s">
-        <v>620</v>
-      </c>
-      <c r="G122" t="s">
-        <v>308</v>
-      </c>
-      <c r="H122" s="7" t="s">
-        <v>621</v>
-      </c>
-      <c r="I122" s="15" t="s">
-        <v>622</v>
-      </c>
-      <c r="J122" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" hidden="1">
-      <c r="A123" t="s">
-        <v>654</v>
-      </c>
-      <c r="B123" t="s">
-        <v>511</v>
-      </c>
-      <c r="C123" s="5" t="s">
-        <v>706</v>
-      </c>
-      <c r="D123" t="s">
-        <v>148</v>
-      </c>
-      <c r="E123" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F123" s="27" t="s">
-        <v>655</v>
-      </c>
-      <c r="G123" t="s">
-        <v>673</v>
-      </c>
-      <c r="H123" t="s">
-        <v>656</v>
-      </c>
-      <c r="I123" s="21" t="s">
-        <v>657</v>
-      </c>
-      <c r="J123" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" hidden="1">
-      <c r="A124" s="5" t="s">
-        <v>623</v>
-      </c>
-      <c r="B124" s="5" t="s">
-        <v>624</v>
-      </c>
-      <c r="C124" s="20"/>
+      <c r="C124" s="22" t="s">
+        <v>651</v>
+      </c>
       <c r="D124" s="5" t="s">
         <v>96</v>
       </c>
       <c r="E124" s="5"/>
-      <c r="F124" s="5"/>
+      <c r="F124" s="5" t="s">
+        <v>620</v>
+      </c>
       <c r="G124" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H124" s="5" t="s">
+        <v>621</v>
+      </c>
+      <c r="I124" s="13" t="s">
+        <v>622</v>
+      </c>
+      <c r="J124" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10">
+      <c r="A125" s="5" t="s">
+        <v>623</v>
+      </c>
+      <c r="B125" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="C125" s="5" t="s">
+        <v>685</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="E125" s="5"/>
+      <c r="F125" s="5"/>
+      <c r="G125" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="H124" s="5" t="s">
+      <c r="H125" s="5" t="s">
         <v>625</v>
       </c>
-      <c r="I124" s="13" t="s">
+      <c r="I125" s="13" t="s">
         <v>626</v>
       </c>
-      <c r="J124" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="125" spans="1:10" hidden="1">
-      <c r="A125" s="5" t="s">
+      <c r="J125" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10">
+      <c r="A126" s="5" t="s">
         <v>627</v>
       </c>
-      <c r="B125" s="5" t="s">
+      <c r="B126" s="5" t="s">
         <v>628</v>
       </c>
-      <c r="C125" s="22" t="s">
-        <v>660</v>
-      </c>
-      <c r="D125" s="5" t="s">
+      <c r="C126" s="5" t="s">
+        <v>629</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E126" s="5" t="s">
+        <v>630</v>
+      </c>
+      <c r="F126" s="5" t="s">
+        <v>631</v>
+      </c>
+      <c r="G126" t="s">
+        <v>103</v>
+      </c>
+      <c r="H126" s="5"/>
+      <c r="I126" s="5" t="s">
+        <v>632</v>
+      </c>
+      <c r="J126" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-helene.vezina@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10">
+      <c r="A127" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>619</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>694</v>
+      </c>
+      <c r="D127" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E125" s="5"/>
-      <c r="F125" s="5" t="s">
-        <v>629</v>
-      </c>
-      <c r="G125" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H125" s="5" t="s">
-        <v>630</v>
-      </c>
-      <c r="I125" s="13" t="s">
-        <v>631</v>
-      </c>
-      <c r="J125" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" hidden="1">
-      <c r="A126" s="5" t="s">
-        <v>632</v>
-      </c>
-      <c r="B126" s="5" t="s">
-        <v>633</v>
-      </c>
-      <c r="C126" s="5" t="s">
-        <v>695</v>
-      </c>
-      <c r="D126" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="E126" s="5"/>
-      <c r="F126" s="5"/>
-      <c r="G126" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H126" s="5" t="s">
+      <c r="E127" s="5"/>
+      <c r="F127" s="5"/>
+      <c r="G127" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H127" s="5" t="s">
         <v>634</v>
       </c>
-      <c r="I126" s="13" t="s">
+      <c r="I127" s="13" t="s">
         <v>635</v>
       </c>
-      <c r="J126" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" hidden="1">
-      <c r="A127" s="5" t="s">
+      <c r="J127" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10">
+      <c r="A128" s="7" t="s">
         <v>636</v>
       </c>
-      <c r="B127" s="5" t="s">
+      <c r="B128" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="C128" s="7"/>
+      <c r="D128" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E128" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F128" s="7" t="s">
         <v>637</v>
       </c>
-      <c r="C127" s="5" t="s">
+      <c r="G128" t="s">
+        <v>454</v>
+      </c>
+      <c r="H128" s="7" t="s">
+        <v>475</v>
+      </c>
+      <c r="I128" s="7" t="s">
         <v>638</v>
       </c>
-      <c r="D127" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E127" s="5" t="s">
-        <v>639</v>
-      </c>
-      <c r="F127" s="5" t="s">
-        <v>640</v>
-      </c>
-      <c r="G127" t="s">
-        <v>103</v>
-      </c>
-      <c r="H127" s="5"/>
-      <c r="I127" s="5" t="s">
-        <v>641</v>
-      </c>
-      <c r="J127" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-helene.vezina@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" hidden="1">
-      <c r="A128" s="5" t="s">
-        <v>642</v>
-      </c>
-      <c r="B128" s="5" t="s">
-        <v>628</v>
-      </c>
-      <c r="C128" s="5" t="s">
-        <v>704</v>
-      </c>
-      <c r="D128" s="5" t="s">
+      <c r="J128" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10">
+      <c r="A129" t="s">
+        <v>714</v>
+      </c>
+      <c r="B129" t="s">
+        <v>615</v>
+      </c>
+      <c r="C129" s="5" t="s">
+        <v>717</v>
+      </c>
+      <c r="D129" t="s">
         <v>96</v>
       </c>
-      <c r="E128" s="5"/>
-      <c r="F128" s="5"/>
-      <c r="G128" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="H128" s="5" t="s">
-        <v>643</v>
-      </c>
-      <c r="I128" s="13" t="s">
-        <v>644</v>
-      </c>
-      <c r="J128" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" hidden="1">
-      <c r="A129" s="7" t="s">
-        <v>645</v>
-      </c>
-      <c r="B129" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="C129" s="7"/>
-      <c r="D129" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E129" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F129" s="7" t="s">
-        <v>646</v>
+      <c r="E129" s="5"/>
+      <c r="F129" s="8" t="s">
+        <v>572</v>
       </c>
       <c r="G129" t="s">
-        <v>462</v>
-      </c>
-      <c r="H129" s="7" t="s">
-        <v>483</v>
-      </c>
-      <c r="I129" s="7" t="s">
-        <v>647</v>
+        <v>573</v>
+      </c>
+      <c r="H129" t="s">
+        <v>715</v>
+      </c>
+      <c r="I129" s="21" t="s">
+        <v>716</v>
       </c>
       <c r="J129" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10">
-      <c r="A130" t="s">
-        <v>724</v>
-      </c>
-      <c r="B130" t="s">
-        <v>624</v>
-      </c>
-      <c r="C130" s="5" t="s">
-        <v>727</v>
-      </c>
-      <c r="D130" t="s">
-        <v>96</v>
-      </c>
-      <c r="E130" s="5"/>
-      <c r="F130" s="8" t="s">
-        <v>581</v>
-      </c>
-      <c r="G130" t="s">
-        <v>582</v>
-      </c>
-      <c r="H130" t="s">
-        <v>725</v>
-      </c>
-      <c r="I130" s="21" t="s">
-        <v>726</v>
-      </c>
-      <c r="J130" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
       </c>
@@ -6818,44 +6763,44 @@
     <hyperlink ref="I12" r:id="rId1" display="mailto:audrey.begin-poissant@umontreal.ca" xr:uid="{708FEBAC-F938-40E8-8D55-B34C4326210F}"/>
     <hyperlink ref="I28" r:id="rId2" display="mailto:delphine.cado@umontreal.ca" xr:uid="{0E0BF38D-BCA7-4652-84E3-BBE8A015792A}"/>
     <hyperlink ref="I17" r:id="rId3" display="mailto:hugo.bernier@umontreal.ca" xr:uid="{3F591457-DA50-462E-B1CA-F2F56ED9E3DD}"/>
-    <hyperlink ref="I67" r:id="rId4" xr:uid="{4822C834-E5A8-42FD-9734-374BFC718C85}"/>
+    <hyperlink ref="I66" r:id="rId4" xr:uid="{4822C834-E5A8-42FD-9734-374BFC718C85}"/>
     <hyperlink ref="I10" r:id="rId5" display="mailto:magalie.beaudoin@umontreal.ca" xr:uid="{2D976BF0-B68A-46E5-8412-BA8BC43FD26D}"/>
-    <hyperlink ref="I103" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
+    <hyperlink ref="I102" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
     <hyperlink ref="I4" r:id="rId7" display="mailto:nadege.arsa@bib.umontreal.ca" xr:uid="{408AF5A3-35ED-4BF5-92B9-1B21C0C475D9}"/>
     <hyperlink ref="I18" r:id="rId8" display="mailto:simon.blais.longtin@umontreal.ca" xr:uid="{EA917AC7-9087-435B-A6E7-3AE1885514AA}"/>
-    <hyperlink ref="I83" r:id="rId9" xr:uid="{8ABC26E9-CF81-491C-8A28-B209E6620D2A}"/>
-    <hyperlink ref="I125" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
+    <hyperlink ref="I82" r:id="rId9" xr:uid="{8ABC26E9-CF81-491C-8A28-B209E6620D2A}"/>
+    <hyperlink ref="I124" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
     <hyperlink ref="I32" r:id="rId11" xr:uid="{7D21070C-9A14-48DF-982E-D995A034BDAD}"/>
-    <hyperlink ref="I122" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
-    <hyperlink ref="I66" r:id="rId13" xr:uid="{DCABBE8B-8789-4957-9A88-F8585AD53BBC}"/>
-    <hyperlink ref="I106" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
+    <hyperlink ref="I121" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
+    <hyperlink ref="I65" r:id="rId13" xr:uid="{DCABBE8B-8789-4957-9A88-F8585AD53BBC}"/>
+    <hyperlink ref="I105" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
     <hyperlink ref="I45" r:id="rId15" xr:uid="{1383A46C-5C1D-4621-B4BC-67AD012D7CF5}"/>
-    <hyperlink ref="I72" r:id="rId16" xr:uid="{29D9619F-F3A7-41E8-AE0F-DEBBF802D53A}"/>
+    <hyperlink ref="I71" r:id="rId16" xr:uid="{29D9619F-F3A7-41E8-AE0F-DEBBF802D53A}"/>
     <hyperlink ref="I27" r:id="rId17" xr:uid="{9E8CD31B-437A-49A0-BA12-85176E0D9431}"/>
-    <hyperlink ref="I107" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
-    <hyperlink ref="I68" r:id="rId19" xr:uid="{3B502B79-2DDE-44A3-908B-3CB04ED1101E}"/>
+    <hyperlink ref="I106" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
+    <hyperlink ref="I67" r:id="rId19" xr:uid="{3B502B79-2DDE-44A3-908B-3CB04ED1101E}"/>
     <hyperlink ref="I16" r:id="rId20" xr:uid="{BAE0697B-7739-4A42-9702-C285F03D0F77}"/>
     <hyperlink ref="I47" r:id="rId21" xr:uid="{E1BC7B04-B072-447B-9137-59A28141883D}"/>
-    <hyperlink ref="I97" r:id="rId22" xr:uid="{BEDF45F1-312C-4FF5-B4F5-1D1C7E487C0A}"/>
-    <hyperlink ref="I59" r:id="rId23" xr:uid="{6E82D57D-36A4-4928-AD91-BE73FFC7C389}"/>
-    <hyperlink ref="I74" r:id="rId24" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
-    <hyperlink ref="I92" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
-    <hyperlink ref="I121" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
-    <hyperlink ref="I81" r:id="rId27" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
-    <hyperlink ref="I82" r:id="rId28" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
-    <hyperlink ref="I87" r:id="rId29" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
-    <hyperlink ref="I105" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
-    <hyperlink ref="I116" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
-    <hyperlink ref="I119" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
-    <hyperlink ref="I124" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
-    <hyperlink ref="I126" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
-    <hyperlink ref="I128" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
+    <hyperlink ref="I96" r:id="rId22" xr:uid="{BEDF45F1-312C-4FF5-B4F5-1D1C7E487C0A}"/>
+    <hyperlink ref="I58" r:id="rId23" xr:uid="{6E82D57D-36A4-4928-AD91-BE73FFC7C389}"/>
+    <hyperlink ref="I73" r:id="rId24" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
+    <hyperlink ref="I91" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
+    <hyperlink ref="I120" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
+    <hyperlink ref="I80" r:id="rId27" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
+    <hyperlink ref="I81" r:id="rId28" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
+    <hyperlink ref="I86" r:id="rId29" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
+    <hyperlink ref="I104" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
+    <hyperlink ref="I115" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
+    <hyperlink ref="I118" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
+    <hyperlink ref="I123" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
+    <hyperlink ref="I125" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
+    <hyperlink ref="I127" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
     <hyperlink ref="I15" r:id="rId36" xr:uid="{E26D4CB1-6F14-4277-AD54-18A052872B6B}"/>
-    <hyperlink ref="I123" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
+    <hyperlink ref="I122" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
     <hyperlink ref="I8" r:id="rId38" xr:uid="{2E646106-878B-4504-8874-8750F3CAA7CB}"/>
     <hyperlink ref="I33" r:id="rId39" xr:uid="{902A8808-023C-4EA1-833E-F687288B12ED}"/>
-    <hyperlink ref="I130" r:id="rId40" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
-    <hyperlink ref="I108" r:id="rId41" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
+    <hyperlink ref="I129" r:id="rId40" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
+    <hyperlink ref="I107" r:id="rId41" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId42"/>
@@ -7061,15 +7006,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7078,6 +7014,15 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7100,14 +7045,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7122,4 +7059,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Ajout de Taline Ekmekjian
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CB2AD0-A2A0-448A-9EA0-142730FB908C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA03163-3143-40F3-9D42-B948BFB2C5E3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19460" yWindow="4650" windowWidth="20480" windowHeight="23450" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="723">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="728">
   <si>
     <t>nom</t>
   </si>
@@ -2217,6 +2217,21 @@
   </si>
   <si>
     <t>Science politique, Études internationales, Études féministes - des genres et des sexualités, Sciences économiques, Données statistiques</t>
+  </si>
+  <si>
+    <t>Ekmekjian</t>
+  </si>
+  <si>
+    <t>Taline</t>
+  </si>
+  <si>
+    <t>Soutien aux synthèses de connaissance</t>
+  </si>
+  <si>
+    <t>514 343-6111, poste 0866</t>
+  </si>
+  <si>
+    <t>taline.ekmekjian@umontreal.ca</t>
   </si>
 </sst>
 </file>
@@ -2379,7 +2394,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2418,6 +2433,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
@@ -2531,10 +2547,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J129" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:J129" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
-  <sortState ref="A2:J128">
-    <sortCondition ref="A1:A128"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J130" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:J130" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
+  <sortState ref="A2:J129">
+    <sortCondition ref="A1:A129"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{4B04E1AF-0079-4AD2-81CA-E8A433733E21}" name="nom"/>
@@ -2875,7 +2891,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J129"/>
+  <dimension ref="A1:J130"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="18.453125" customWidth="1"/>
@@ -4278,63 +4294,61 @@
       </c>
     </row>
     <row r="47" spans="1:10">
-      <c r="A47" t="s">
+      <c r="A47" s="5" t="s">
+        <v>723</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>724</v>
+      </c>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>725</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>726</v>
+      </c>
+      <c r="I47" s="10" t="s">
+        <v>727</v>
+      </c>
+      <c r="J47" s="30" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=taline.ekmekjian@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10">
+      <c r="A48" t="s">
         <v>272</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B48" t="s">
         <v>273</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C48" s="5" t="s">
         <v>695</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D48" t="s">
         <v>96</v>
       </c>
-      <c r="G47" t="s">
+      <c r="G48" t="s">
         <v>29</v>
       </c>
-      <c r="H47" t="s">
+      <c r="H48" t="s">
         <v>274</v>
       </c>
-      <c r="I47" s="15" t="s">
+      <c r="I48" s="15" t="s">
         <v>275</v>
       </c>
-      <c r="J47" s="10" t="str">
+      <c r="J48" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=judith.fafard-larose@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10">
-      <c r="A48" s="7" t="s">
-        <v>276</v>
-      </c>
-      <c r="B48" s="7" t="s">
-        <v>277</v>
-      </c>
-      <c r="C48" s="22" t="s">
-        <v>278</v>
-      </c>
-      <c r="D48" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="F48" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="G48" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="H48" s="7" t="s">
-        <v>279</v>
-      </c>
-      <c r="I48" s="7" t="s">
-        <v>280</v>
-      </c>
-      <c r="J48" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -4348,14 +4362,16 @@
         <v>278</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>642</v>
+        <v>148</v>
       </c>
       <c r="E49" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="F49" s="7"/>
+      <c r="F49" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="G49" s="7" t="s">
-        <v>326</v>
+        <v>130</v>
       </c>
       <c r="H49" s="7" t="s">
         <v>279</v>
@@ -4368,185 +4384,188 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="29">
+    <row r="50" spans="1:10">
       <c r="A50" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C50" s="22" t="s">
+        <v>278</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="H50" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="I50" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="J50" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="29">
+      <c r="A51" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="B50" s="7" t="s">
+      <c r="B51" s="7" t="s">
         <v>282</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="C51" s="7" t="s">
         <v>283</v>
       </c>
-      <c r="D50" s="7" t="s">
+      <c r="D51" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E50" s="17" t="s">
+      <c r="E51" s="17" t="s">
         <v>284</v>
       </c>
-      <c r="F50" s="7" t="s">
+      <c r="F51" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G50" s="7" t="s">
+      <c r="G51" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H50" s="7" t="s">
+      <c r="H51" s="7" t="s">
         <v>285</v>
       </c>
-      <c r="I50" s="7" t="s">
+      <c r="I51" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="J50" s="10" t="str">
+      <c r="J51" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=c.fortier@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10">
-      <c r="A51" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="B51" s="7" t="s">
-        <v>288</v>
-      </c>
-      <c r="C51" s="7"/>
-      <c r="D51" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="E51" s="7"/>
-      <c r="F51" s="7" t="s">
-        <v>289</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>290</v>
-      </c>
-      <c r="H51" s="7" t="s">
-        <v>291</v>
-      </c>
-      <c r="I51" s="7" t="s">
-        <v>292</v>
-      </c>
-      <c r="J51" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="7" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>294</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>295</v>
-      </c>
+        <v>288</v>
+      </c>
+      <c r="C52" s="7"/>
       <c r="D52" s="7" t="s">
-        <v>13</v>
+        <v>96</v>
       </c>
       <c r="E52" s="7"/>
       <c r="F52" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="G52" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="H52" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="I52" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="J52" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10">
+      <c r="A53" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7" t="s">
         <v>296</v>
       </c>
-      <c r="G52" s="7" t="s">
+      <c r="G53" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H52" s="7" t="s">
+      <c r="H53" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="I52" s="7" t="s">
+      <c r="I53" s="7" t="s">
         <v>298</v>
       </c>
-      <c r="J52" s="10" t="str">
+      <c r="J53" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=nino.gabrielli@umontreal.ca</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
-      <c r="A53" s="5" t="s">
+    <row r="54" spans="1:10">
+      <c r="A54" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B54" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C54" s="5" t="s">
         <v>701</v>
       </c>
-      <c r="D53" s="5" t="s">
+      <c r="D54" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5" t="s">
+      <c r="E54" s="5"/>
+      <c r="F54" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="G53" s="5" t="s">
+      <c r="G54" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="H53" s="5"/>
-      <c r="I53" s="5" t="s">
+      <c r="H54" s="5"/>
+      <c r="I54" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="J53" s="10" t="str">
+      <c r="J54" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-pierre.gadoua@umontreal.ca</v>
       </c>
     </row>
-    <row r="54" spans="1:10">
-      <c r="A54" s="7" t="s">
+    <row r="55" spans="1:10">
+      <c r="A55" s="7" t="s">
         <v>304</v>
       </c>
-      <c r="B54" s="7" t="s">
+      <c r="B55" s="7" t="s">
         <v>305</v>
       </c>
-      <c r="C54" s="7" t="s">
+      <c r="C55" s="7" t="s">
         <v>306</v>
       </c>
-      <c r="D54" s="7" t="s">
+      <c r="D55" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E54" s="7"/>
-      <c r="F54" s="7" t="s">
+      <c r="E55" s="7"/>
+      <c r="F55" s="7" t="s">
         <v>307</v>
       </c>
-      <c r="G54" s="7" t="s">
+      <c r="G55" s="7" t="s">
         <v>308</v>
       </c>
-      <c r="H54" s="7" t="s">
+      <c r="H55" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="I54" s="7" t="s">
+      <c r="I55" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="J54" s="10" t="str">
+      <c r="J55" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=cynthia.gagne.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10">
-      <c r="A55" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="B55" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="C55" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="D55" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="E55" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="F55" s="5"/>
-      <c r="H55" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="I55" s="5" t="s">
-        <v>315</v>
-      </c>
-      <c r="J55" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -4554,762 +4573,761 @@
         <v>311</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>316</v>
-      </c>
-      <c r="C56" s="5"/>
+        <v>312</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="D56" s="5" t="s">
-        <v>122</v>
+        <v>314</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>129</v>
+        <v>259</v>
       </c>
       <c r="F56" s="5"/>
       <c r="H56" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="I56" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="J56" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10">
+      <c r="A57" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="F57" s="5"/>
+      <c r="H57" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="I56" s="5" t="s">
+      <c r="I57" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="J56" s="10" t="str">
+      <c r="J57" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="57" spans="1:10">
-      <c r="A57" s="7" t="s">
+    <row r="58" spans="1:10">
+      <c r="A58" s="7" t="s">
         <v>318</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="B58" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="C58" s="7" t="s">
         <v>320</v>
       </c>
-      <c r="D57" s="7" t="s">
+      <c r="D58" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E57" s="7" t="s">
+      <c r="E58" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="F57" s="7" t="s">
+      <c r="F58" s="7" t="s">
         <v>321</v>
       </c>
-      <c r="H57" s="7" t="s">
+      <c r="H58" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="I57" s="7" t="s">
+      <c r="I58" s="7" t="s">
         <v>323</v>
       </c>
-      <c r="J57" s="10" t="str">
+      <c r="J58" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=marjorie.gauchier@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10">
-      <c r="A58" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="G58" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="H58" s="8" t="s">
-        <v>542</v>
-      </c>
-      <c r="I58" s="13" t="s">
-        <v>327</v>
-      </c>
-      <c r="J58" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="5" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>681</v>
-      </c>
+        <v>185</v>
+      </c>
+      <c r="C59" s="5"/>
       <c r="D59" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E59" s="5" t="s">
-        <v>84</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="E59" s="5"/>
       <c r="F59" s="5" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="H59" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="I59" s="5"/>
+        <v>326</v>
+      </c>
+      <c r="H59" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="I59" s="13" t="s">
+        <v>327</v>
+      </c>
       <c r="J59" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v/>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="H60" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="I60" s="5"/>
+      <c r="J60" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
+      <c r="A61" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B61" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="C61" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="D60" s="5" t="s">
+      <c r="D61" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E60" s="5"/>
-      <c r="F60" s="5" t="s">
+      <c r="E61" s="5"/>
+      <c r="F61" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="G60" s="5" t="s">
+      <c r="G61" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="H60" s="5" t="s">
+      <c r="H61" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="I60" s="5" t="s">
+      <c r="I61" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="J60" s="10" t="str">
+      <c r="J61" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
       </c>
     </row>
-    <row r="61" spans="1:10">
-      <c r="A61" s="7" t="s">
+    <row r="62" spans="1:10">
+      <c r="A62" s="7" t="s">
         <v>338</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B62" s="7" t="s">
         <v>339</v>
       </c>
-      <c r="C61" s="7" t="s">
+      <c r="C62" s="7" t="s">
         <v>340</v>
       </c>
-      <c r="D61" s="7" t="s">
+      <c r="D62" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E61" s="7"/>
-      <c r="F61" s="7" t="s">
+      <c r="E62" s="7"/>
+      <c r="F62" s="7" t="s">
         <v>341</v>
       </c>
-      <c r="G61" s="7" t="s">
+      <c r="G62" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H61" s="7" t="s">
+      <c r="H62" s="7" t="s">
         <v>342</v>
       </c>
-      <c r="I61" s="7" t="s">
+      <c r="I62" s="7" t="s">
         <v>343</v>
       </c>
-      <c r="J61" s="10" t="str">
+      <c r="J62" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
       </c>
     </row>
-    <row r="62" spans="1:10" s="3" customFormat="1">
-      <c r="A62" t="s">
+    <row r="63" spans="1:10" s="3" customFormat="1">
+      <c r="A63" t="s">
         <v>344</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B63" t="s">
         <v>345</v>
       </c>
-      <c r="C62" s="19" t="s">
+      <c r="C63" s="19" t="s">
         <v>346</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D63" t="s">
         <v>13</v>
       </c>
-      <c r="E62"/>
-      <c r="F62" s="28" t="s">
+      <c r="E63"/>
+      <c r="F63" s="28" t="s">
         <v>347</v>
       </c>
-      <c r="G62" t="s">
+      <c r="G63" t="s">
         <v>15</v>
       </c>
-      <c r="H62" t="s">
+      <c r="H63" t="s">
         <v>348</v>
       </c>
-      <c r="I62" t="s">
+      <c r="I63" t="s">
         <v>349</v>
       </c>
-      <c r="J62" s="10" t="str">
+      <c r="J63" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
       </c>
     </row>
-    <row r="63" spans="1:10">
-      <c r="A63" s="5" t="s">
+    <row r="64" spans="1:10">
+      <c r="A64" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="B63" s="5" t="s">
+      <c r="B64" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="C63" s="5" t="s">
+      <c r="C64" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="D63" s="5" t="s">
+      <c r="D64" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E63" s="7" t="s">
+      <c r="E64" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="F63" s="29"/>
-      <c r="G63" s="3"/>
-      <c r="H63" s="5" t="s">
+      <c r="F64" s="29"/>
+      <c r="G64" s="3"/>
+      <c r="H64" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="I63" s="5" t="s">
+      <c r="I64" s="5" t="s">
         <v>354</v>
       </c>
-      <c r="J63" s="10" t="str">
+      <c r="J64" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
       </c>
     </row>
-    <row r="64" spans="1:10" s="4" customFormat="1">
-      <c r="A64" s="5" t="s">
+    <row r="65" spans="1:10" s="4" customFormat="1">
+      <c r="A65" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="B65" s="5" t="s">
         <v>356</v>
       </c>
-      <c r="C64" s="5" t="s">
+      <c r="C65" s="5" t="s">
         <v>357</v>
       </c>
-      <c r="D64" s="5" t="s">
+      <c r="D65" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E64" s="5"/>
-      <c r="F64" s="5" t="s">
+      <c r="E65" s="5"/>
+      <c r="F65" s="5" t="s">
         <v>719</v>
       </c>
-      <c r="G64" s="5" t="s">
+      <c r="G65" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H64" s="5" t="s">
+      <c r="H65" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="I64" s="5" t="s">
+      <c r="I65" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="J64" s="10" t="str">
+      <c r="J65" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
-      <c r="A65" t="s">
+    <row r="66" spans="1:10">
+      <c r="A66" t="s">
         <v>360</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B66" t="s">
         <v>361</v>
       </c>
-      <c r="C65" t="s">
+      <c r="C66" t="s">
         <v>703</v>
       </c>
-      <c r="D65" t="s">
+      <c r="D66" t="s">
         <v>49</v>
       </c>
-      <c r="G65" t="s">
+      <c r="G66" t="s">
         <v>308</v>
       </c>
-      <c r="H65" s="7" t="s">
+      <c r="H66" s="7" t="s">
         <v>362</v>
       </c>
-      <c r="I65" s="15" t="s">
+      <c r="I66" s="15" t="s">
         <v>363</v>
       </c>
-      <c r="J65" s="10" t="str">
+      <c r="J66" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
-      <c r="A66" s="7" t="s">
+    <row r="67" spans="1:10">
+      <c r="A67" s="7" t="s">
         <v>364</v>
       </c>
-      <c r="B66" s="7" t="s">
+      <c r="B67" s="7" t="s">
         <v>329</v>
       </c>
-      <c r="C66" s="7"/>
-      <c r="D66" s="7" t="s">
+      <c r="C67" s="7"/>
+      <c r="D67" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="E66" s="7"/>
-      <c r="F66" s="7" t="s">
+      <c r="E67" s="7"/>
+      <c r="F67" s="7" t="s">
         <v>325</v>
       </c>
-      <c r="G66" s="7" t="s">
+      <c r="G67" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="H66" s="7" t="s">
+      <c r="H67" s="7" t="s">
         <v>365</v>
       </c>
-      <c r="I66" s="9" t="s">
+      <c r="I67" s="9" t="s">
         <v>639</v>
       </c>
-      <c r="J66" s="10" t="str">
+      <c r="J67" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
       </c>
     </row>
-    <row r="67" spans="1:10">
-      <c r="A67" t="s">
+    <row r="68" spans="1:10">
+      <c r="A68" t="s">
         <v>366</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B68" t="s">
         <v>105</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C68" t="s">
         <v>700</v>
       </c>
-      <c r="D67" t="s">
+      <c r="D68" t="s">
         <v>96</v>
       </c>
-      <c r="G67" t="s">
+      <c r="G68" t="s">
         <v>29</v>
       </c>
-      <c r="H67" s="16" t="s">
+      <c r="H68" s="16" t="s">
         <v>367</v>
       </c>
-      <c r="I67" s="15" t="s">
+      <c r="I68" s="15" t="s">
         <v>368</v>
       </c>
-      <c r="J67" s="10" t="str">
+      <c r="J68" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
       </c>
     </row>
-    <row r="68" spans="1:10">
-      <c r="A68" s="7" t="s">
+    <row r="69" spans="1:10">
+      <c r="A69" s="7" t="s">
         <v>369</v>
       </c>
-      <c r="B68" s="7" t="s">
+      <c r="B69" s="7" t="s">
         <v>370</v>
       </c>
-      <c r="C68" s="7" t="s">
+      <c r="C69" s="7" t="s">
         <v>371</v>
       </c>
-      <c r="D68" s="7" t="s">
+      <c r="D69" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="E68" s="7" t="s">
+      <c r="E69" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="F68" s="7" t="s">
+      <c r="F69" s="7" t="s">
         <v>372</v>
       </c>
-      <c r="G68" s="7" t="s">
+      <c r="G69" s="7" t="s">
         <v>655</v>
       </c>
-      <c r="H68" s="7" t="s">
+      <c r="H69" s="7" t="s">
         <v>373</v>
       </c>
-      <c r="I68" s="7" t="s">
+      <c r="I69" s="7" t="s">
         <v>374</v>
       </c>
-      <c r="J68" s="10" t="str">
+      <c r="J69" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
       </c>
     </row>
-    <row r="69" spans="1:10">
-      <c r="A69" s="5" t="s">
+    <row r="70" spans="1:10">
+      <c r="A70" s="5" t="s">
         <v>375</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="B70" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="C69" s="5" t="s">
+      <c r="C70" s="5" t="s">
         <v>377</v>
       </c>
-      <c r="D69" s="5" t="s">
+      <c r="D70" s="5" t="s">
         <v>640</v>
       </c>
-      <c r="E69" s="5" t="s">
+      <c r="E70" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="F69" s="5" t="s">
+      <c r="F70" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G69" s="7" t="s">
+      <c r="G70" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="H69" s="5" t="s">
+      <c r="H70" s="5" t="s">
         <v>378</v>
       </c>
-      <c r="I69" s="5" t="s">
+      <c r="I70" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="J69" s="10" t="str">
+      <c r="J70" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="29">
-      <c r="A70" s="7" t="s">
+    <row r="71" spans="1:10" ht="29">
+      <c r="A71" s="7" t="s">
         <v>380</v>
       </c>
-      <c r="B70" s="7" t="s">
+      <c r="B71" s="7" t="s">
         <v>312</v>
       </c>
-      <c r="C70" s="7" t="s">
+      <c r="C71" s="7" t="s">
         <v>649</v>
       </c>
-      <c r="D70" s="7" t="s">
+      <c r="D71" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E70" s="17" t="s">
+      <c r="E71" s="17" t="s">
         <v>284</v>
       </c>
-      <c r="F70" s="7" t="s">
+      <c r="F71" s="7" t="s">
         <v>381</v>
       </c>
-      <c r="G70" s="7" t="s">
+      <c r="G71" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H70" s="7" t="s">
+      <c r="H71" s="7" t="s">
         <v>382</v>
       </c>
-      <c r="I70" s="7" t="s">
+      <c r="I71" s="7" t="s">
         <v>383</v>
       </c>
-      <c r="J70" s="10" t="str">
+      <c r="J71" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
       </c>
     </row>
-    <row r="71" spans="1:10">
-      <c r="A71" t="s">
+    <row r="72" spans="1:10">
+      <c r="A72" t="s">
         <v>384</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B72" t="s">
         <v>385</v>
       </c>
-      <c r="C71" s="5" t="s">
+      <c r="C72" s="5" t="s">
         <v>650</v>
       </c>
-      <c r="D71" t="s">
+      <c r="D72" t="s">
         <v>96</v>
       </c>
-      <c r="G71" t="s">
+      <c r="G72" t="s">
         <v>29</v>
       </c>
-      <c r="H71" s="16" t="s">
+      <c r="H72" s="16" t="s">
         <v>386</v>
       </c>
-      <c r="I71" s="15" t="s">
+      <c r="I72" s="15" t="s">
         <v>387</v>
       </c>
-      <c r="J71" s="10" t="str">
+      <c r="J72" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
       </c>
     </row>
-    <row r="72" spans="1:10">
-      <c r="A72" s="7" t="s">
+    <row r="73" spans="1:10">
+      <c r="A73" s="7" t="s">
         <v>388</v>
       </c>
-      <c r="B72" s="7" t="s">
+      <c r="B73" s="7" t="s">
         <v>389</v>
       </c>
-      <c r="C72" s="5" t="s">
+      <c r="C73" s="5" t="s">
         <v>390</v>
       </c>
-      <c r="D72" s="7" t="s">
+      <c r="D73" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E72" s="7"/>
-      <c r="F72" s="7" t="s">
+      <c r="E73" s="7"/>
+      <c r="F73" s="7" t="s">
         <v>722</v>
       </c>
-      <c r="G72" s="7" t="s">
+      <c r="G73" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H72" s="7" t="s">
+      <c r="H73" s="7" t="s">
         <v>391</v>
       </c>
-      <c r="I72" s="7" t="s">
+      <c r="I73" s="7" t="s">
         <v>392</v>
       </c>
-      <c r="J72" s="10" t="str">
+      <c r="J73" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
       </c>
     </row>
-    <row r="73" spans="1:10" s="3" customFormat="1">
-      <c r="A73" t="s">
+    <row r="74" spans="1:10" s="3" customFormat="1">
+      <c r="A74" t="s">
         <v>393</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B74" t="s">
         <v>394</v>
       </c>
-      <c r="C73" s="5" t="s">
+      <c r="C74" s="5" t="s">
         <v>693</v>
       </c>
-      <c r="D73" s="7" t="s">
+      <c r="D74" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E73" s="7"/>
-      <c r="F73" s="27" t="s">
+      <c r="E74" s="7"/>
+      <c r="F74" s="27" t="s">
         <v>395</v>
       </c>
-      <c r="G73" s="7" t="s">
+      <c r="G74" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="H73" t="s">
+      <c r="H74" t="s">
         <v>396</v>
       </c>
-      <c r="I73" s="15" t="s">
+      <c r="I74" s="15" t="s">
         <v>397</v>
       </c>
-      <c r="J73" s="10" t="str">
+      <c r="J74" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="74" spans="1:10" s="3" customFormat="1">
-      <c r="A74" s="7" t="s">
+    <row r="75" spans="1:10" s="3" customFormat="1">
+      <c r="A75" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="B74" s="7" t="s">
+      <c r="B75" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="C74" s="5" t="s">
+      <c r="C75" s="5" t="s">
         <v>400</v>
       </c>
-      <c r="D74" s="7" t="s">
+      <c r="D75" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="E74" s="7" t="s">
+      <c r="E75" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="G74" s="7" t="s">
+      <c r="G75" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="H74" s="7" t="s">
+      <c r="H75" s="7" t="s">
         <v>401</v>
       </c>
-      <c r="I74" s="7" t="s">
+      <c r="I75" s="7" t="s">
         <v>402</v>
       </c>
-      <c r="J74" s="10" t="str">
+      <c r="J75" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
-    <row r="75" spans="1:10">
-      <c r="A75" s="5" t="s">
+    <row r="76" spans="1:10">
+      <c r="A76" s="5" t="s">
         <v>403</v>
       </c>
-      <c r="B75" s="5" t="s">
+      <c r="B76" s="5" t="s">
         <v>404</v>
       </c>
-      <c r="C75" s="5" t="s">
+      <c r="C76" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="D75" s="5" t="s">
+      <c r="D76" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="E75" s="5" t="s">
+      <c r="E76" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="F75" s="29" t="s">
+      <c r="F76" s="29" t="s">
         <v>406</v>
       </c>
-      <c r="G75" s="7" t="s">
+      <c r="G76" s="7" t="s">
         <v>641</v>
       </c>
-      <c r="H75" s="5" t="s">
+      <c r="H76" s="5" t="s">
         <v>407</v>
       </c>
-      <c r="I75" s="5" t="s">
+      <c r="I76" s="5" t="s">
         <v>408</v>
       </c>
-      <c r="J75" s="10" t="str">
+      <c r="J76" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
       </c>
     </row>
-    <row r="76" spans="1:10">
-      <c r="A76" s="7" t="s">
+    <row r="77" spans="1:10">
+      <c r="A77" s="7" t="s">
         <v>409</v>
       </c>
-      <c r="B76" s="7" t="s">
+      <c r="B77" s="7" t="s">
         <v>410</v>
       </c>
-      <c r="C76" s="5" t="s">
+      <c r="C77" s="5" t="s">
         <v>702</v>
       </c>
-      <c r="D76" s="7" t="s">
+      <c r="D77" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="E76" s="7" t="s">
+      <c r="E77" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G76" s="7" t="s">
+      <c r="G77" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="H76" s="7" t="s">
+      <c r="H77" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="I76" s="7" t="s">
+      <c r="I77" s="7" t="s">
         <v>412</v>
       </c>
-      <c r="J76" s="10" t="str">
+      <c r="J77" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
       </c>
     </row>
-    <row r="77" spans="1:10" s="3" customFormat="1" ht="29">
-      <c r="A77" s="5" t="s">
+    <row r="78" spans="1:10" s="3" customFormat="1" ht="29">
+      <c r="A78" s="5" t="s">
         <v>413</v>
       </c>
-      <c r="B77" s="5" t="s">
+      <c r="B78" s="5" t="s">
         <v>414</v>
       </c>
-      <c r="C77" s="5" t="s">
+      <c r="C78" s="5" t="s">
         <v>415</v>
       </c>
-      <c r="D77" s="5" t="s">
+      <c r="D78" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="E77" s="17" t="s">
+      <c r="E78" s="17" t="s">
         <v>284</v>
       </c>
-      <c r="F77" s="5"/>
-      <c r="G77" s="5" t="s">
+      <c r="F78" s="5"/>
+      <c r="G78" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="H77" s="5" t="s">
+      <c r="H78" s="5" t="s">
         <v>416</v>
       </c>
-      <c r="I77" s="5" t="s">
+      <c r="I78" s="5" t="s">
         <v>417</v>
       </c>
-      <c r="J77" s="10" t="str">
+      <c r="J78" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
       </c>
     </row>
-    <row r="78" spans="1:10">
-      <c r="A78" s="8" t="s">
+    <row r="79" spans="1:10">
+      <c r="A79" s="8" t="s">
         <v>418</v>
       </c>
-      <c r="B78" s="8" t="s">
+      <c r="B79" s="8" t="s">
         <v>419</v>
       </c>
-      <c r="C78" s="8" t="s">
+      <c r="C79" s="8" t="s">
         <v>687</v>
       </c>
-      <c r="D78" s="8" t="s">
+      <c r="D79" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="E78" s="11" t="s">
+      <c r="E79" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="F78" s="27" t="s">
+      <c r="F79" s="27" t="s">
         <v>644</v>
       </c>
-      <c r="G78" s="8" t="s">
+      <c r="G79" s="8" t="s">
         <v>654</v>
       </c>
-      <c r="H78" s="8" t="s">
+      <c r="H79" s="8" t="s">
         <v>420</v>
       </c>
-      <c r="I78" s="8" t="s">
+      <c r="I79" s="8" t="s">
         <v>421</v>
       </c>
-      <c r="J78" s="10" t="str">
+      <c r="J79" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10">
-      <c r="A79" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="B79" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="C79" s="5" t="s">
-        <v>688</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="E79" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F79" s="5"/>
-      <c r="H79" s="5"/>
-      <c r="I79" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="J79" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="5" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>426</v>
-      </c>
-      <c r="E80" s="5"/>
+        <v>96</v>
+      </c>
+      <c r="E80" s="5" t="s">
+        <v>84</v>
+      </c>
       <c r="F80" s="5"/>
-      <c r="G80" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H80" s="5" t="s">
-        <v>427</v>
-      </c>
-      <c r="I80" s="13" t="s">
-        <v>428</v>
+      <c r="H80" s="5"/>
+      <c r="I80" s="5" t="s">
+        <v>423</v>
       </c>
       <c r="J80" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="5" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>706</v>
+        <v>691</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>426</v>
@@ -5317,1443 +5335,1472 @@
       <c r="E81" s="5"/>
       <c r="F81" s="5"/>
       <c r="G81" s="5" t="s">
-        <v>431</v>
+        <v>57</v>
       </c>
       <c r="H81" s="5" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="I81" s="13" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="J81" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
       </c>
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="5" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>436</v>
+        <v>426</v>
       </c>
       <c r="E82" s="5"/>
-      <c r="F82" s="27" t="s">
-        <v>437</v>
-      </c>
+      <c r="F82" s="5"/>
       <c r="G82" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="H82" s="11" t="s">
-        <v>438</v>
+        <v>431</v>
+      </c>
+      <c r="H82" s="5" t="s">
+        <v>432</v>
       </c>
       <c r="I82" s="13" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
       <c r="J82" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
       </c>
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="5" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>442</v>
+        <v>705</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>13</v>
+        <v>436</v>
       </c>
       <c r="E83" s="5"/>
-      <c r="F83" s="5" t="s">
-        <v>720</v>
+      <c r="F83" s="27" t="s">
+        <v>437</v>
       </c>
       <c r="G83" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H83" s="5" t="s">
-        <v>443</v>
-      </c>
-      <c r="I83" s="5" t="s">
-        <v>444</v>
+        <v>240</v>
+      </c>
+      <c r="H83" s="11" t="s">
+        <v>438</v>
+      </c>
+      <c r="I83" s="13" t="s">
+        <v>439</v>
       </c>
       <c r="J83" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
       </c>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="5" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>361</v>
+        <v>441</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E84" s="5"/>
       <c r="F84" s="5" t="s">
-        <v>447</v>
+        <v>720</v>
       </c>
       <c r="G84" s="5" t="s">
-        <v>448</v>
+        <v>29</v>
       </c>
       <c r="H84" s="5" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="I84" s="5" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="J84" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
       </c>
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="5" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>452</v>
+        <v>361</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>453</v>
+        <v>446</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E85" s="5" t="s">
-        <v>76</v>
+        <v>13</v>
+      </c>
+      <c r="E85" s="5"/>
+      <c r="F85" s="5" t="s">
+        <v>447</v>
       </c>
       <c r="G85" s="5" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="H85" s="5" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="I85" s="5" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="J85" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
       </c>
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="5" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>670</v>
+        <v>453</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>426</v>
-      </c>
-      <c r="E86" s="5"/>
-      <c r="F86" s="5"/>
+        <v>41</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>76</v>
+      </c>
       <c r="G86" s="5" t="s">
-        <v>97</v>
+        <v>454</v>
       </c>
       <c r="H86" s="5" t="s">
-        <v>459</v>
-      </c>
-      <c r="I86" s="13" t="s">
-        <v>460</v>
+        <v>455</v>
+      </c>
+      <c r="I86" s="5" t="s">
+        <v>456</v>
       </c>
       <c r="J86" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
       </c>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>670</v>
+      </c>
+      <c r="D87" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="E87" s="5"/>
+      <c r="F87" s="5"/>
+      <c r="G87" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H87" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="I87" s="13" t="s">
+        <v>460</v>
+      </c>
+      <c r="J87" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10">
+      <c r="A88" s="5" t="s">
         <v>461</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="B88" s="5" t="s">
         <v>462</v>
       </c>
-      <c r="C87" s="5" t="s">
+      <c r="C88" s="5" t="s">
         <v>463</v>
-      </c>
-      <c r="D87" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E87" s="5"/>
-      <c r="F87" s="5" t="s">
-        <v>464</v>
-      </c>
-      <c r="G87" s="5" t="s">
-        <v>431</v>
-      </c>
-      <c r="H87" s="5" t="s">
-        <v>465</v>
-      </c>
-      <c r="I87" s="5" t="s">
-        <v>466</v>
-      </c>
-      <c r="J87" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10">
-      <c r="A88" s="11" t="s">
-        <v>467</v>
-      </c>
-      <c r="B88" s="11" t="s">
-        <v>468</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>469</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E88" s="5"/>
-      <c r="F88" s="11" t="s">
+      <c r="F88" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="G88" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="H88" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="I88" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="J88" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10">
+      <c r="A89" s="11" t="s">
+        <v>467</v>
+      </c>
+      <c r="B89" s="11" t="s">
+        <v>468</v>
+      </c>
+      <c r="C89" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="D89" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E89" s="5"/>
+      <c r="F89" s="11" t="s">
         <v>447</v>
       </c>
-      <c r="G88" s="11" t="s">
+      <c r="G89" s="11" t="s">
         <v>448</v>
       </c>
-      <c r="H88" s="11" t="s">
+      <c r="H89" s="11" t="s">
         <v>470</v>
       </c>
-      <c r="I88" s="11" t="s">
+      <c r="I89" s="11" t="s">
         <v>471</v>
       </c>
-      <c r="J88" s="10" t="str">
+      <c r="J89" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10">
-      <c r="A89" s="7" t="s">
-        <v>472</v>
-      </c>
-      <c r="B89" s="7" t="s">
-        <v>473</v>
-      </c>
-      <c r="C89" s="5" t="s">
-        <v>474</v>
-      </c>
-      <c r="D89" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E89" s="7"/>
-      <c r="F89" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="G89" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="H89" s="7" t="s">
-        <v>475</v>
-      </c>
-      <c r="I89" s="7" t="s">
-        <v>476</v>
-      </c>
-      <c r="J89" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="7" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="B90" s="7" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="D90" s="7" t="s">
-        <v>13</v>
+        <v>111</v>
       </c>
       <c r="E90" s="7"/>
       <c r="F90" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G90" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="H90" s="7" t="s">
+        <v>475</v>
+      </c>
+      <c r="I90" s="7" t="s">
+        <v>476</v>
+      </c>
+      <c r="J90" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10">
+      <c r="A91" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="B91" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="C91" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="D91" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E91" s="7"/>
+      <c r="F91" s="7" t="s">
         <v>480</v>
       </c>
-      <c r="G90" s="7" t="s">
+      <c r="G91" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="H90" s="7" t="s">
+      <c r="H91" s="7" t="s">
         <v>481</v>
       </c>
-      <c r="I90" s="7" t="s">
+      <c r="I91" s="7" t="s">
         <v>482</v>
       </c>
-      <c r="J90" s="10" t="str">
+      <c r="J91" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=assia.mourid@umontreal.ca</v>
       </c>
     </row>
-    <row r="91" spans="1:10">
-      <c r="A91" t="s">
+    <row r="92" spans="1:10">
+      <c r="A92" t="s">
         <v>483</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B92" t="s">
         <v>484</v>
       </c>
-      <c r="C91" s="5" t="s">
+      <c r="C92" s="5" t="s">
         <v>671</v>
       </c>
-      <c r="D91" s="7" t="s">
+      <c r="D92" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E91" s="7"/>
-      <c r="F91" s="27" t="s">
+      <c r="E92" s="7"/>
+      <c r="F92" s="27" t="s">
         <v>485</v>
       </c>
-      <c r="G91" s="7" t="s">
+      <c r="G92" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="H91" t="s">
+      <c r="H92" t="s">
         <v>486</v>
       </c>
-      <c r="I91" s="15" t="s">
+      <c r="I92" s="15" t="s">
         <v>487</v>
       </c>
-      <c r="J91" s="10" t="str">
+      <c r="J92" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
       </c>
     </row>
-    <row r="92" spans="1:10">
-      <c r="A92" s="11" t="s">
+    <row r="93" spans="1:10">
+      <c r="A93" s="11" t="s">
         <v>488</v>
       </c>
-      <c r="B92" s="11" t="s">
+      <c r="B93" s="11" t="s">
         <v>489</v>
       </c>
-      <c r="C92" s="11" t="s">
+      <c r="C93" s="11" t="s">
         <v>679</v>
       </c>
-      <c r="D92" s="11" t="s">
+      <c r="D93" s="11" t="s">
         <v>239</v>
       </c>
-      <c r="E92" s="11" t="s">
+      <c r="E93" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="F92" s="29"/>
-      <c r="G92" s="11" t="s">
+      <c r="F93" s="29"/>
+      <c r="G93" s="11" t="s">
         <v>663</v>
       </c>
-      <c r="H92" s="11" t="s">
+      <c r="H93" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="I92" s="11" t="s">
+      <c r="I93" s="11" t="s">
         <v>491</v>
       </c>
-      <c r="J92" s="10" t="str">
+      <c r="J93" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="93" spans="1:10">
-      <c r="A93" s="7" t="s">
+    <row r="94" spans="1:10">
+      <c r="A94" s="7" t="s">
         <v>492</v>
       </c>
-      <c r="B93" s="7" t="s">
+      <c r="B94" s="7" t="s">
         <v>493</v>
       </c>
-      <c r="C93" s="7" t="s">
+      <c r="C94" s="7" t="s">
         <v>698</v>
       </c>
-      <c r="D93" s="7" t="s">
+      <c r="D94" s="7" t="s">
         <v>494</v>
       </c>
-      <c r="E93" s="7"/>
-      <c r="F93" s="7" t="s">
+      <c r="E94" s="7"/>
+      <c r="F94" s="7" t="s">
         <v>495</v>
       </c>
-      <c r="G93" s="7" t="s">
+      <c r="G94" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="H93" s="7" t="s">
+      <c r="H94" s="7" t="s">
         <v>496</v>
       </c>
-      <c r="I93" s="7" t="s">
+      <c r="I94" s="7" t="s">
         <v>497</v>
       </c>
-      <c r="J93" s="10" t="str">
+      <c r="J94" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" s="3" customFormat="1">
-      <c r="A94" s="7" t="s">
-        <v>498</v>
-      </c>
-      <c r="B94" s="7" t="s">
-        <v>499</v>
-      </c>
-      <c r="C94" s="7"/>
-      <c r="D94" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="E94" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F94" s="7"/>
-      <c r="G94"/>
-      <c r="H94" s="7" t="s">
-        <v>500</v>
-      </c>
-      <c r="I94" s="7" t="s">
-        <v>501</v>
-      </c>
-      <c r="J94" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
     <row r="95" spans="1:10" s="3" customFormat="1">
       <c r="A95" s="7" t="s">
+        <v>498</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="C95" s="7"/>
+      <c r="D95" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="E95" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F95" s="7"/>
+      <c r="G95"/>
+      <c r="H95" s="7" t="s">
+        <v>500</v>
+      </c>
+      <c r="I95" s="7" t="s">
+        <v>501</v>
+      </c>
+      <c r="J95" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" s="3" customFormat="1">
+      <c r="A96" s="7" t="s">
         <v>502</v>
       </c>
-      <c r="B95" s="7" t="s">
+      <c r="B96" s="7" t="s">
         <v>503</v>
       </c>
-      <c r="C95" s="7" t="s">
+      <c r="C96" s="7" t="s">
         <v>652</v>
       </c>
-      <c r="D95" s="7" t="s">
+      <c r="D96" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E95" s="17"/>
-      <c r="F95" s="8" t="s">
+      <c r="E96" s="17"/>
+      <c r="F96" s="8" t="s">
         <v>572</v>
       </c>
-      <c r="G95" t="s">
+      <c r="G96" t="s">
         <v>573</v>
       </c>
-      <c r="H95" s="7" t="s">
+      <c r="H96" s="7" t="s">
         <v>504</v>
       </c>
-      <c r="I95" s="7" t="s">
+      <c r="I96" s="7" t="s">
         <v>505</v>
       </c>
-      <c r="J95" s="10" t="str">
+      <c r="J96" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
-    <row r="96" spans="1:10">
-      <c r="A96" s="7" t="s">
+    <row r="97" spans="1:10">
+      <c r="A97" s="7" t="s">
         <v>506</v>
       </c>
-      <c r="B96" s="7" t="s">
+      <c r="B97" s="7" t="s">
         <v>507</v>
       </c>
-      <c r="C96" s="7"/>
-      <c r="D96" s="7" t="s">
+      <c r="C97" s="7"/>
+      <c r="D97" s="7" t="s">
         <v>508</v>
       </c>
-      <c r="E96" s="5"/>
-      <c r="F96" s="27" t="s">
+      <c r="E97" s="5"/>
+      <c r="F97" s="27" t="s">
         <v>509</v>
       </c>
-      <c r="G96" s="7" t="s">
+      <c r="G97" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="H96" s="7"/>
-      <c r="I96" s="14" t="s">
+      <c r="H97" s="7"/>
+      <c r="I97" s="14" t="s">
         <v>510</v>
       </c>
-      <c r="J96" s="10" t="str">
+      <c r="J97" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
       </c>
     </row>
-    <row r="97" spans="1:10">
-      <c r="A97" t="s">
+    <row r="98" spans="1:10">
+      <c r="A98" t="s">
         <v>511</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B98" t="s">
         <v>512</v>
       </c>
-      <c r="C97" s="23" t="s">
+      <c r="C98" s="23" t="s">
         <v>513</v>
       </c>
-      <c r="D97" t="s">
+      <c r="D98" t="s">
         <v>27</v>
       </c>
-      <c r="E97" t="s">
+      <c r="E98" t="s">
         <v>84</v>
       </c>
-      <c r="F97" s="28" t="s">
+      <c r="F98" s="28" t="s">
         <v>514</v>
-      </c>
-      <c r="G97" t="s">
-        <v>103</v>
-      </c>
-      <c r="I97" t="s">
-        <v>515</v>
-      </c>
-      <c r="J97" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10">
-      <c r="A98" s="5" t="s">
-        <v>516</v>
-      </c>
-      <c r="B98" s="5" t="s">
-        <v>517</v>
-      </c>
-      <c r="C98" s="5" t="s">
-        <v>690</v>
-      </c>
-      <c r="D98" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F98" s="5" t="s">
-        <v>518</v>
       </c>
       <c r="G98" t="s">
         <v>103</v>
       </c>
-      <c r="H98" s="11" t="s">
+      <c r="I98" t="s">
+        <v>515</v>
+      </c>
+      <c r="J98" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10">
+      <c r="A99" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="C99" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="D99" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E99" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F99" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="G99" t="s">
+        <v>103</v>
+      </c>
+      <c r="H99" s="11" t="s">
         <v>519</v>
       </c>
-      <c r="I98" s="11" t="s">
+      <c r="I99" s="11" t="s">
         <v>520</v>
       </c>
-      <c r="J98" s="10" t="str">
+      <c r="J99" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=eve.paquette-bigras@umontreal.ca</v>
       </c>
     </row>
-    <row r="99" spans="1:10">
-      <c r="A99" s="7" t="s">
+    <row r="100" spans="1:10">
+      <c r="A100" s="7" t="s">
         <v>521</v>
       </c>
-      <c r="B99" s="7" t="s">
+      <c r="B100" s="7" t="s">
         <v>526</v>
       </c>
-      <c r="C99" s="7" t="s">
+      <c r="C100" s="7" t="s">
         <v>527</v>
       </c>
-      <c r="D99" s="7" t="s">
+      <c r="D100" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E99" s="7"/>
-      <c r="F99" s="7" t="s">
+      <c r="E100" s="7"/>
+      <c r="F100" s="7" t="s">
         <v>721</v>
       </c>
-      <c r="G99" s="7" t="s">
+      <c r="G100" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H99" s="8" t="s">
+      <c r="H100" s="8" t="s">
         <v>528</v>
       </c>
-      <c r="I99" s="8" t="s">
+      <c r="I100" s="8" t="s">
         <v>529</v>
       </c>
-      <c r="J99" s="10" t="str">
+      <c r="J100" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="100" spans="1:10">
-      <c r="A100" s="5" t="s">
+    <row r="101" spans="1:10">
+      <c r="A101" s="5" t="s">
         <v>521</v>
       </c>
-      <c r="B100" s="5" t="s">
+      <c r="B101" s="5" t="s">
         <v>522</v>
       </c>
-      <c r="C100" s="5" t="s">
+      <c r="C101" s="5" t="s">
         <v>667</v>
-      </c>
-      <c r="D100" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E100" s="5"/>
-      <c r="F100" s="5" t="s">
-        <v>523</v>
-      </c>
-      <c r="G100" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H100" s="11" t="s">
-        <v>524</v>
-      </c>
-      <c r="I100" s="11" t="s">
-        <v>525</v>
-      </c>
-      <c r="J100" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10" s="4" customFormat="1">
-      <c r="A101" s="5" t="s">
-        <v>530</v>
-      </c>
-      <c r="B101" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="C101" s="5" t="s">
-        <v>531</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E101" s="5"/>
       <c r="F101" s="5" t="s">
-        <v>143</v>
+        <v>523</v>
       </c>
       <c r="G101" s="5" t="s">
-        <v>97</v>
+        <v>29</v>
       </c>
       <c r="H101" s="11" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
       <c r="I101" s="11" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="J101" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
       </c>
     </row>
     <row r="102" spans="1:10" s="4" customFormat="1">
       <c r="A102" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E102" s="5"/>
+      <c r="F102" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="G102" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H102" s="11" t="s">
+        <v>532</v>
+      </c>
+      <c r="I102" s="11" t="s">
+        <v>533</v>
+      </c>
+      <c r="J102" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" s="4" customFormat="1">
+      <c r="A103" s="5" t="s">
         <v>534</v>
       </c>
-      <c r="B102" s="5" t="s">
+      <c r="B103" s="5" t="s">
         <v>484</v>
       </c>
-      <c r="C102" s="5" t="s">
+      <c r="C103" s="5" t="s">
         <v>535</v>
       </c>
-      <c r="D102" s="5" t="s">
+      <c r="D103" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E102" s="5" t="s">
+      <c r="E103" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F102" s="5" t="s">
+      <c r="F103" s="5" t="s">
         <v>536</v>
       </c>
-      <c r="H102" s="11"/>
-      <c r="I102" s="10" t="s">
+      <c r="H103" s="11"/>
+      <c r="I103" s="10" t="s">
         <v>537</v>
       </c>
-      <c r="J102" s="10" t="str">
+      <c r="J103" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="103" spans="1:10">
-      <c r="A103" s="7" t="s">
-        <v>538</v>
-      </c>
-      <c r="B103" s="7" t="s">
-        <v>539</v>
-      </c>
-      <c r="C103" s="7" t="s">
-        <v>540</v>
-      </c>
-      <c r="D103" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E103" s="7"/>
-      <c r="F103" s="7" t="s">
-        <v>541</v>
-      </c>
-      <c r="G103" s="7" t="s">
-        <v>326</v>
-      </c>
-      <c r="H103" s="8" t="s">
-        <v>542</v>
-      </c>
-      <c r="I103" s="8" t="s">
-        <v>543</v>
-      </c>
-      <c r="J103" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
       </c>
     </row>
     <row r="104" spans="1:10">
       <c r="A104" s="7" t="s">
+        <v>538</v>
+      </c>
+      <c r="B104" s="7" t="s">
+        <v>539</v>
+      </c>
+      <c r="C104" s="7" t="s">
+        <v>540</v>
+      </c>
+      <c r="D104" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E104" s="7"/>
+      <c r="F104" s="7" t="s">
+        <v>541</v>
+      </c>
+      <c r="G104" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="H104" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="I104" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="J104" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10">
+      <c r="A105" s="7" t="s">
         <v>544</v>
       </c>
-      <c r="B104" s="7" t="s">
+      <c r="B105" s="7" t="s">
         <v>545</v>
       </c>
-      <c r="C104" s="5" t="s">
+      <c r="C105" s="5" t="s">
         <v>704</v>
       </c>
-      <c r="D104" s="7" t="s">
+      <c r="D105" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="E104" s="7"/>
-      <c r="F104" s="7"/>
-      <c r="G104" s="5" t="s">
+      <c r="E105" s="7"/>
+      <c r="F105" s="7"/>
+      <c r="G105" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H104" s="8" t="s">
+      <c r="H105" s="8" t="s">
         <v>546</v>
       </c>
-      <c r="I104" s="14" t="s">
+      <c r="I105" s="14" t="s">
         <v>547</v>
       </c>
-      <c r="J104" s="10" t="str">
+      <c r="J105" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10">
-      <c r="A105" t="s">
-        <v>548</v>
-      </c>
-      <c r="B105" t="s">
-        <v>549</v>
-      </c>
-      <c r="C105" t="s">
-        <v>692</v>
-      </c>
-      <c r="D105" t="s">
-        <v>426</v>
-      </c>
-      <c r="G105" t="s">
-        <v>643</v>
-      </c>
-      <c r="H105" s="7" t="s">
-        <v>550</v>
-      </c>
-      <c r="I105" s="15" t="s">
-        <v>551</v>
-      </c>
-      <c r="J105" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
     <row r="106" spans="1:10">
       <c r="A106" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="B106" t="s">
-        <v>553</v>
-      </c>
-      <c r="C106" s="25"/>
+        <v>549</v>
+      </c>
+      <c r="C106" t="s">
+        <v>692</v>
+      </c>
       <c r="D106" t="s">
-        <v>96</v>
+        <v>426</v>
       </c>
       <c r="G106" t="s">
-        <v>29</v>
-      </c>
-      <c r="H106" t="s">
-        <v>554</v>
+        <v>643</v>
+      </c>
+      <c r="H106" s="7" t="s">
+        <v>550</v>
       </c>
       <c r="I106" s="15" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="J106" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
     <row r="107" spans="1:10">
       <c r="A107" t="s">
-        <v>709</v>
+        <v>552</v>
       </c>
       <c r="B107" t="s">
-        <v>710</v>
-      </c>
-      <c r="C107" s="5" t="s">
-        <v>718</v>
-      </c>
+        <v>553</v>
+      </c>
+      <c r="C107" s="25"/>
       <c r="D107" t="s">
         <v>96</v>
       </c>
-      <c r="E107" s="5"/>
-      <c r="F107" s="8" t="s">
-        <v>572</v>
-      </c>
       <c r="G107" t="s">
-        <v>573</v>
+        <v>29</v>
       </c>
       <c r="H107" t="s">
-        <v>712</v>
-      </c>
-      <c r="I107" s="21" t="s">
-        <v>713</v>
+        <v>554</v>
+      </c>
+      <c r="I107" s="15" t="s">
+        <v>555</v>
       </c>
       <c r="J107" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
     <row r="108" spans="1:10">
       <c r="A108" t="s">
+        <v>709</v>
+      </c>
+      <c r="B108" t="s">
+        <v>710</v>
+      </c>
+      <c r="C108" s="5" t="s">
+        <v>718</v>
+      </c>
+      <c r="D108" t="s">
+        <v>96</v>
+      </c>
+      <c r="E108" s="5"/>
+      <c r="F108" s="8" t="s">
+        <v>572</v>
+      </c>
+      <c r="G108" t="s">
+        <v>573</v>
+      </c>
+      <c r="H108" t="s">
+        <v>712</v>
+      </c>
+      <c r="I108" s="21" t="s">
+        <v>713</v>
+      </c>
+      <c r="J108" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10">
+      <c r="A109" t="s">
         <v>556</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B109" t="s">
         <v>54</v>
       </c>
-      <c r="C108" s="19" t="s">
+      <c r="C109" s="19" t="s">
         <v>557</v>
       </c>
-      <c r="D108" t="s">
+      <c r="D109" t="s">
         <v>13</v>
       </c>
-      <c r="F108" s="28" t="s">
+      <c r="F109" s="28" t="s">
         <v>558</v>
       </c>
-      <c r="G108" t="s">
+      <c r="G109" t="s">
         <v>29</v>
       </c>
-      <c r="H108" s="3" t="s">
+      <c r="H109" s="3" t="s">
         <v>559</v>
       </c>
-      <c r="I108" s="3" t="s">
+      <c r="I109" s="3" t="s">
         <v>560</v>
       </c>
-      <c r="J108" s="10" t="str">
+      <c r="J109" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10">
-      <c r="A109" s="5" t="s">
-        <v>561</v>
-      </c>
-      <c r="B109" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="C109" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D109" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="E109" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F109" s="5"/>
-      <c r="H109" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="I109" s="11" t="s">
-        <v>563</v>
-      </c>
-      <c r="J109" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
       </c>
     </row>
     <row r="110" spans="1:10">
       <c r="A110" s="5" t="s">
+        <v>561</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="C110" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="E110" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F110" s="5"/>
+      <c r="H110" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="I110" s="11" t="s">
+        <v>563</v>
+      </c>
+      <c r="J110" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10">
+      <c r="A111" s="5" t="s">
         <v>564</v>
       </c>
-      <c r="B110" s="5" t="s">
+      <c r="B111" s="5" t="s">
         <v>565</v>
       </c>
-      <c r="C110" s="5" t="s">
+      <c r="C111" s="5" t="s">
         <v>673</v>
       </c>
-      <c r="D110" s="5" t="s">
+      <c r="D111" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E110" s="5"/>
-      <c r="F110" s="5" t="s">
+      <c r="E111" s="5"/>
+      <c r="F111" s="5" t="s">
         <v>566</v>
       </c>
-      <c r="G110" s="5" t="s">
+      <c r="G111" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="H110" s="11"/>
-      <c r="I110" s="11" t="s">
+      <c r="H111" s="11"/>
+      <c r="I111" s="11" t="s">
         <v>567</v>
       </c>
-      <c r="J110" s="10" t="str">
+      <c r="J111" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
       </c>
     </row>
-    <row r="111" spans="1:10">
-      <c r="A111" t="s">
+    <row r="112" spans="1:10">
+      <c r="A112" t="s">
         <v>568</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B112" t="s">
         <v>569</v>
       </c>
-      <c r="C111" s="25" t="s">
+      <c r="C112" s="25" t="s">
         <v>668</v>
       </c>
-      <c r="D111" s="5" t="s">
+      <c r="D112" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="E111" s="5"/>
-      <c r="F111" s="5"/>
-      <c r="G111" t="s">
+      <c r="E112" s="5"/>
+      <c r="F112" s="5"/>
+      <c r="G112" t="s">
         <v>29</v>
       </c>
-      <c r="J111" s="10" t="str">
+      <c r="J112" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v/>
-      </c>
-    </row>
-    <row r="112" spans="1:10">
-      <c r="A112" s="8" t="s">
-        <v>570</v>
-      </c>
-      <c r="B112" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C112" s="7" t="s">
-        <v>571</v>
-      </c>
-      <c r="D112" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="E112" s="8"/>
-      <c r="F112" s="8" t="s">
-        <v>572</v>
-      </c>
-      <c r="G112" s="8" t="s">
-        <v>573</v>
-      </c>
-      <c r="H112" s="8" t="s">
-        <v>574</v>
-      </c>
-      <c r="I112" s="8" t="s">
-        <v>575</v>
-      </c>
-      <c r="J112" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
       </c>
     </row>
     <row r="113" spans="1:10">
       <c r="A113" s="8" t="s">
+        <v>570</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C113" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="D113" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E113" s="8"/>
+      <c r="F113" s="8" t="s">
+        <v>572</v>
+      </c>
+      <c r="G113" s="8" t="s">
+        <v>573</v>
+      </c>
+      <c r="H113" s="8" t="s">
+        <v>574</v>
+      </c>
+      <c r="I113" s="8" t="s">
+        <v>575</v>
+      </c>
+      <c r="J113" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10">
+      <c r="A114" s="8" t="s">
         <v>576</v>
       </c>
-      <c r="B113" s="8" t="s">
+      <c r="B114" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="C113" s="24"/>
-      <c r="D113" s="8" t="s">
+      <c r="C114" s="24"/>
+      <c r="D114" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="E113" s="8" t="s">
+      <c r="E114" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="F113" s="8"/>
-      <c r="G113" s="8"/>
-      <c r="H113" s="8" t="s">
+      <c r="F114" s="8"/>
+      <c r="G114" s="8"/>
+      <c r="H114" s="8" t="s">
         <v>577</v>
       </c>
-      <c r="I113" s="8" t="s">
+      <c r="I114" s="8" t="s">
         <v>578</v>
       </c>
-      <c r="J113" s="10" t="str">
+      <c r="J114" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10">
-      <c r="A114" s="5" t="s">
-        <v>579</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>580</v>
-      </c>
-      <c r="C114" s="20" t="s">
-        <v>581</v>
-      </c>
-      <c r="D114" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="E114" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G114" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="H114" s="5" t="s">
-        <v>582</v>
-      </c>
-      <c r="I114" s="5" t="s">
-        <v>583</v>
-      </c>
-      <c r="J114" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
       </c>
     </row>
     <row r="115" spans="1:10">
       <c r="A115" s="5" t="s">
+        <v>579</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>580</v>
+      </c>
+      <c r="C115" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="E115" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G115" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="H115" s="5" t="s">
+        <v>582</v>
+      </c>
+      <c r="I115" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="J115" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10">
+      <c r="A116" s="5" t="s">
         <v>584</v>
       </c>
-      <c r="B115" s="5" t="s">
+      <c r="B116" s="5" t="s">
         <v>585</v>
       </c>
-      <c r="C115" s="20" t="s">
+      <c r="C116" s="20" t="s">
         <v>682</v>
       </c>
-      <c r="D115" s="5" t="s">
+      <c r="D116" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E115" s="5"/>
-      <c r="F115" s="5"/>
-      <c r="G115" s="5" t="s">
+      <c r="E116" s="5"/>
+      <c r="F116" s="5"/>
+      <c r="G116" s="5" t="s">
         <v>448</v>
       </c>
-      <c r="H115" s="5"/>
-      <c r="I115" s="13" t="s">
+      <c r="H116" s="5"/>
+      <c r="I116" s="13" t="s">
         <v>586</v>
       </c>
-      <c r="J115" s="10" t="str">
+      <c r="J116" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
       </c>
     </row>
-    <row r="116" spans="1:10">
-      <c r="A116" s="11" t="s">
+    <row r="117" spans="1:10">
+      <c r="A117" s="11" t="s">
         <v>587</v>
       </c>
-      <c r="B116" s="11" t="s">
+      <c r="B117" s="11" t="s">
         <v>588</v>
       </c>
-      <c r="C116" s="22" t="s">
+      <c r="C117" s="22" t="s">
         <v>589</v>
       </c>
-      <c r="D116" s="11" t="s">
+      <c r="D117" s="11" t="s">
         <v>289</v>
       </c>
-      <c r="E116" t="s">
+      <c r="E117" t="s">
         <v>590</v>
       </c>
-      <c r="F116" s="11" t="s">
+      <c r="F117" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="G116" s="11" t="s">
+      <c r="G117" s="11" t="s">
         <v>662</v>
       </c>
-      <c r="H116" s="11" t="s">
+      <c r="H117" s="11" t="s">
         <v>592</v>
       </c>
-      <c r="I116" s="11" t="s">
+      <c r="I117" s="11" t="s">
         <v>593</v>
       </c>
-      <c r="J116" s="10" t="str">
+      <c r="J117" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="117" spans="1:10">
-      <c r="A117" s="7" t="s">
-        <v>594</v>
-      </c>
-      <c r="B117" s="7" t="s">
-        <v>484</v>
-      </c>
-      <c r="C117" s="7" t="s">
-        <v>595</v>
-      </c>
-      <c r="D117" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E117" s="7"/>
-      <c r="F117" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="G117" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="H117" s="7" t="s">
-        <v>596</v>
-      </c>
-      <c r="I117" s="7" t="s">
-        <v>597</v>
-      </c>
-      <c r="J117" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
       </c>
     </row>
     <row r="118" spans="1:10">
       <c r="A118" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="B118" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="C118" s="7" t="s">
+        <v>595</v>
+      </c>
+      <c r="D118" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E118" s="7"/>
+      <c r="F118" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="G118" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="H118" s="7" t="s">
+        <v>596</v>
+      </c>
+      <c r="I118" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="J118" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10">
+      <c r="A119" s="7" t="s">
         <v>598</v>
       </c>
-      <c r="B118" s="7" t="s">
+      <c r="B119" s="7" t="s">
         <v>599</v>
       </c>
-      <c r="C118" s="7" t="s">
+      <c r="C119" s="7" t="s">
         <v>697</v>
       </c>
-      <c r="D118" s="7" t="s">
+      <c r="D119" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="E118" s="7"/>
-      <c r="F118" s="7"/>
-      <c r="G118" s="7" t="s">
+      <c r="E119" s="7"/>
+      <c r="F119" s="7"/>
+      <c r="G119" s="7" t="s">
         <v>448</v>
       </c>
-      <c r="H118" t="s">
+      <c r="H119" t="s">
         <v>600</v>
       </c>
-      <c r="I118" s="14" t="s">
+      <c r="I119" s="14" t="s">
         <v>601</v>
       </c>
-      <c r="J118" s="10" t="str">
+      <c r="J119" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10">
-      <c r="A119" s="5" t="s">
-        <v>602</v>
-      </c>
-      <c r="B119" s="5" t="s">
-        <v>603</v>
-      </c>
-      <c r="C119" s="5" t="s">
-        <v>672</v>
-      </c>
-      <c r="D119" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="E119" s="5"/>
-      <c r="F119" s="5" t="s">
-        <v>604</v>
-      </c>
-      <c r="G119" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="H119" s="5" t="s">
-        <v>605</v>
-      </c>
-      <c r="I119" s="5" t="s">
-        <v>606</v>
-      </c>
-      <c r="J119" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
       </c>
     </row>
     <row r="120" spans="1:10">
       <c r="A120" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="B120" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="C120" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E120" s="5"/>
+      <c r="F120" s="5" t="s">
+        <v>604</v>
+      </c>
+      <c r="G120" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="H120" s="5" t="s">
+        <v>605</v>
+      </c>
+      <c r="I120" s="5" t="s">
+        <v>606</v>
+      </c>
+      <c r="J120" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10">
+      <c r="A121" s="5" t="s">
         <v>607</v>
       </c>
-      <c r="B120" s="5" t="s">
+      <c r="B121" s="5" t="s">
         <v>608</v>
       </c>
-      <c r="C120" s="5" t="s">
+      <c r="C121" s="5" t="s">
         <v>674</v>
       </c>
-      <c r="D120" s="5" t="s">
+      <c r="D121" s="5" t="s">
         <v>426</v>
       </c>
-      <c r="E120" s="5"/>
-      <c r="F120" s="5"/>
-      <c r="G120" s="5" t="s">
+      <c r="E121" s="5"/>
+      <c r="F121" s="5"/>
+      <c r="G121" s="5" t="s">
         <v>431</v>
       </c>
-      <c r="H120" s="7" t="s">
+      <c r="H121" s="7" t="s">
         <v>432</v>
       </c>
-      <c r="I120" s="13" t="s">
+      <c r="I121" s="13" t="s">
         <v>609</v>
       </c>
-      <c r="J120" s="10" t="str">
+      <c r="J121" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10">
-      <c r="A121" t="s">
-        <v>607</v>
-      </c>
-      <c r="B121" t="s">
-        <v>610</v>
-      </c>
-      <c r="D121" t="s">
-        <v>49</v>
-      </c>
-      <c r="F121" s="27" t="s">
-        <v>611</v>
-      </c>
-      <c r="G121" t="s">
-        <v>308</v>
-      </c>
-      <c r="H121" s="7" t="s">
-        <v>612</v>
-      </c>
-      <c r="I121" s="15" t="s">
-        <v>613</v>
-      </c>
-      <c r="J121" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
       </c>
     </row>
     <row r="122" spans="1:10">
       <c r="A122" t="s">
+        <v>607</v>
+      </c>
+      <c r="B122" t="s">
+        <v>610</v>
+      </c>
+      <c r="D122" t="s">
+        <v>49</v>
+      </c>
+      <c r="F122" s="27" t="s">
+        <v>611</v>
+      </c>
+      <c r="G122" t="s">
+        <v>308</v>
+      </c>
+      <c r="H122" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="I122" s="15" t="s">
+        <v>613</v>
+      </c>
+      <c r="J122" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10">
+      <c r="A123" t="s">
         <v>645</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B123" t="s">
         <v>503</v>
       </c>
-      <c r="C122" s="5" t="s">
+      <c r="C123" s="5" t="s">
         <v>696</v>
       </c>
-      <c r="D122" t="s">
+      <c r="D123" t="s">
         <v>148</v>
       </c>
-      <c r="E122" s="5" t="s">
+      <c r="E123" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F122" s="27" t="s">
+      <c r="F123" s="27" t="s">
         <v>646</v>
       </c>
-      <c r="G122" t="s">
+      <c r="G123" t="s">
         <v>664</v>
       </c>
-      <c r="H122" t="s">
+      <c r="H123" t="s">
         <v>647</v>
       </c>
-      <c r="I122" s="21" t="s">
+      <c r="I123" s="21" t="s">
         <v>648</v>
       </c>
-      <c r="J122" s="10" t="str">
+      <c r="J123" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10">
-      <c r="A123" s="5" t="s">
-        <v>614</v>
-      </c>
-      <c r="B123" s="5" t="s">
-        <v>615</v>
-      </c>
-      <c r="C123" s="20"/>
-      <c r="D123" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="E123" s="5"/>
-      <c r="F123" s="5"/>
-      <c r="G123" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H123" s="5" t="s">
-        <v>616</v>
-      </c>
-      <c r="I123" s="13" t="s">
-        <v>617</v>
-      </c>
-      <c r="J123" s="10" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
       </c>
     </row>
     <row r="124" spans="1:10">
       <c r="A124" s="5" t="s">
-        <v>618</v>
+        <v>614</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>619</v>
-      </c>
-      <c r="C124" s="22" t="s">
-        <v>651</v>
-      </c>
+        <v>615</v>
+      </c>
+      <c r="C124" s="20"/>
       <c r="D124" s="5" t="s">
         <v>96</v>
       </c>
       <c r="E124" s="5"/>
-      <c r="F124" s="5" t="s">
-        <v>620</v>
-      </c>
+      <c r="F124" s="5"/>
       <c r="G124" s="5" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H124" s="5" t="s">
-        <v>621</v>
+        <v>616</v>
       </c>
       <c r="I124" s="13" t="s">
-        <v>622</v>
+        <v>617</v>
       </c>
       <c r="J124" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
       </c>
     </row>
     <row r="125" spans="1:10">
       <c r="A125" s="5" t="s">
-        <v>623</v>
+        <v>618</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>624</v>
-      </c>
-      <c r="C125" s="5" t="s">
-        <v>685</v>
+        <v>619</v>
+      </c>
+      <c r="C125" s="22" t="s">
+        <v>651</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>426</v>
+        <v>96</v>
       </c>
       <c r="E125" s="5"/>
-      <c r="F125" s="5"/>
+      <c r="F125" s="5" t="s">
+        <v>620</v>
+      </c>
       <c r="G125" s="5" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="H125" s="5" t="s">
-        <v>625</v>
+        <v>621</v>
       </c>
       <c r="I125" s="13" t="s">
-        <v>626</v>
+        <v>622</v>
       </c>
       <c r="J125" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
       </c>
     </row>
     <row r="126" spans="1:10">
       <c r="A126" s="5" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>629</v>
+        <v>685</v>
       </c>
       <c r="D126" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E126" s="5" t="s">
-        <v>630</v>
-      </c>
-      <c r="F126" s="5" t="s">
-        <v>631</v>
-      </c>
-      <c r="G126" t="s">
-        <v>103</v>
-      </c>
-      <c r="H126" s="5"/>
-      <c r="I126" s="5" t="s">
-        <v>632</v>
+        <v>426</v>
+      </c>
+      <c r="E126" s="5"/>
+      <c r="F126" s="5"/>
+      <c r="G126" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H126" s="5" t="s">
+        <v>625</v>
+      </c>
+      <c r="I126" s="13" t="s">
+        <v>626</v>
       </c>
       <c r="J126" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-helene.vezina@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
       </c>
     </row>
     <row r="127" spans="1:10">
       <c r="A127" s="5" t="s">
+        <v>627</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>628</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>629</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E127" s="5" t="s">
+        <v>630</v>
+      </c>
+      <c r="F127" s="5" t="s">
+        <v>631</v>
+      </c>
+      <c r="G127" t="s">
+        <v>103</v>
+      </c>
+      <c r="H127" s="5"/>
+      <c r="I127" s="5" t="s">
+        <v>632</v>
+      </c>
+      <c r="J127" s="10" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-helene.vezina@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10">
+      <c r="A128" s="5" t="s">
         <v>633</v>
       </c>
-      <c r="B127" s="5" t="s">
+      <c r="B128" s="5" t="s">
         <v>619</v>
       </c>
-      <c r="C127" s="5" t="s">
+      <c r="C128" s="5" t="s">
         <v>694</v>
       </c>
-      <c r="D127" s="5" t="s">
+      <c r="D128" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E127" s="5"/>
-      <c r="F127" s="5"/>
-      <c r="G127" s="5" t="s">
+      <c r="E128" s="5"/>
+      <c r="F128" s="5"/>
+      <c r="G128" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="H127" s="5" t="s">
+      <c r="H128" s="5" t="s">
         <v>634</v>
       </c>
-      <c r="I127" s="13" t="s">
+      <c r="I128" s="13" t="s">
         <v>635</v>
       </c>
-      <c r="J127" s="10" t="str">
+      <c r="J128" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
       </c>
     </row>
-    <row r="128" spans="1:10">
-      <c r="A128" s="7" t="s">
+    <row r="129" spans="1:10">
+      <c r="A129" s="7" t="s">
         <v>636</v>
       </c>
-      <c r="B128" s="7" t="s">
+      <c r="B129" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="C128" s="7"/>
-      <c r="D128" s="7" t="s">
+      <c r="C129" s="7"/>
+      <c r="D129" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E128" s="7" t="s">
+      <c r="E129" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="F128" s="7" t="s">
+      <c r="F129" s="7" t="s">
         <v>637</v>
       </c>
-      <c r="G128" t="s">
+      <c r="G129" t="s">
         <v>454</v>
       </c>
-      <c r="H128" s="7" t="s">
+      <c r="H129" s="7" t="s">
         <v>475</v>
       </c>
-      <c r="I128" s="7" t="s">
+      <c r="I129" s="7" t="s">
         <v>638</v>
       </c>
-      <c r="J128" s="10" t="str">
+      <c r="J129" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
       </c>
     </row>
-    <row r="129" spans="1:10">
-      <c r="A129" t="s">
+    <row r="130" spans="1:10">
+      <c r="A130" t="s">
         <v>714</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B130" t="s">
         <v>615</v>
       </c>
-      <c r="C129" s="5" t="s">
+      <c r="C130" s="5" t="s">
         <v>717</v>
       </c>
-      <c r="D129" t="s">
+      <c r="D130" t="s">
         <v>96</v>
       </c>
-      <c r="E129" s="5"/>
-      <c r="F129" s="8" t="s">
+      <c r="E130" s="5"/>
+      <c r="F130" s="8" t="s">
         <v>572</v>
       </c>
-      <c r="G129" t="s">
+      <c r="G130" t="s">
         <v>573</v>
       </c>
-      <c r="H129" t="s">
+      <c r="H130" t="s">
         <v>715</v>
       </c>
-      <c r="I129" s="21" t="s">
+      <c r="I130" s="21" t="s">
         <v>716</v>
       </c>
-      <c r="J129" s="10" t="str">
+      <c r="J130" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
       </c>
@@ -6763,49 +6810,50 @@
     <hyperlink ref="I12" r:id="rId1" display="mailto:audrey.begin-poissant@umontreal.ca" xr:uid="{708FEBAC-F938-40E8-8D55-B34C4326210F}"/>
     <hyperlink ref="I28" r:id="rId2" display="mailto:delphine.cado@umontreal.ca" xr:uid="{0E0BF38D-BCA7-4652-84E3-BBE8A015792A}"/>
     <hyperlink ref="I17" r:id="rId3" display="mailto:hugo.bernier@umontreal.ca" xr:uid="{3F591457-DA50-462E-B1CA-F2F56ED9E3DD}"/>
-    <hyperlink ref="I66" r:id="rId4" xr:uid="{4822C834-E5A8-42FD-9734-374BFC718C85}"/>
+    <hyperlink ref="I67" r:id="rId4" xr:uid="{4822C834-E5A8-42FD-9734-374BFC718C85}"/>
     <hyperlink ref="I10" r:id="rId5" display="mailto:magalie.beaudoin@umontreal.ca" xr:uid="{2D976BF0-B68A-46E5-8412-BA8BC43FD26D}"/>
-    <hyperlink ref="I102" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
+    <hyperlink ref="I103" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
     <hyperlink ref="I4" r:id="rId7" display="mailto:nadege.arsa@bib.umontreal.ca" xr:uid="{408AF5A3-35ED-4BF5-92B9-1B21C0C475D9}"/>
     <hyperlink ref="I18" r:id="rId8" display="mailto:simon.blais.longtin@umontreal.ca" xr:uid="{EA917AC7-9087-435B-A6E7-3AE1885514AA}"/>
-    <hyperlink ref="I82" r:id="rId9" xr:uid="{8ABC26E9-CF81-491C-8A28-B209E6620D2A}"/>
-    <hyperlink ref="I124" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
+    <hyperlink ref="I83" r:id="rId9" xr:uid="{8ABC26E9-CF81-491C-8A28-B209E6620D2A}"/>
+    <hyperlink ref="I125" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
     <hyperlink ref="I32" r:id="rId11" xr:uid="{7D21070C-9A14-48DF-982E-D995A034BDAD}"/>
-    <hyperlink ref="I121" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
-    <hyperlink ref="I65" r:id="rId13" xr:uid="{DCABBE8B-8789-4957-9A88-F8585AD53BBC}"/>
-    <hyperlink ref="I105" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
+    <hyperlink ref="I122" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
+    <hyperlink ref="I66" r:id="rId13" xr:uid="{DCABBE8B-8789-4957-9A88-F8585AD53BBC}"/>
+    <hyperlink ref="I106" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
     <hyperlink ref="I45" r:id="rId15" xr:uid="{1383A46C-5C1D-4621-B4BC-67AD012D7CF5}"/>
-    <hyperlink ref="I71" r:id="rId16" xr:uid="{29D9619F-F3A7-41E8-AE0F-DEBBF802D53A}"/>
+    <hyperlink ref="I72" r:id="rId16" xr:uid="{29D9619F-F3A7-41E8-AE0F-DEBBF802D53A}"/>
     <hyperlink ref="I27" r:id="rId17" xr:uid="{9E8CD31B-437A-49A0-BA12-85176E0D9431}"/>
-    <hyperlink ref="I106" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
-    <hyperlink ref="I67" r:id="rId19" xr:uid="{3B502B79-2DDE-44A3-908B-3CB04ED1101E}"/>
+    <hyperlink ref="I107" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
+    <hyperlink ref="I68" r:id="rId19" xr:uid="{3B502B79-2DDE-44A3-908B-3CB04ED1101E}"/>
     <hyperlink ref="I16" r:id="rId20" xr:uid="{BAE0697B-7739-4A42-9702-C285F03D0F77}"/>
-    <hyperlink ref="I47" r:id="rId21" xr:uid="{E1BC7B04-B072-447B-9137-59A28141883D}"/>
-    <hyperlink ref="I96" r:id="rId22" xr:uid="{BEDF45F1-312C-4FF5-B4F5-1D1C7E487C0A}"/>
-    <hyperlink ref="I58" r:id="rId23" xr:uid="{6E82D57D-36A4-4928-AD91-BE73FFC7C389}"/>
-    <hyperlink ref="I73" r:id="rId24" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
-    <hyperlink ref="I91" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
-    <hyperlink ref="I120" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
-    <hyperlink ref="I80" r:id="rId27" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
-    <hyperlink ref="I81" r:id="rId28" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
-    <hyperlink ref="I86" r:id="rId29" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
-    <hyperlink ref="I104" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
-    <hyperlink ref="I115" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
-    <hyperlink ref="I118" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
-    <hyperlink ref="I123" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
-    <hyperlink ref="I125" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
-    <hyperlink ref="I127" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
+    <hyperlink ref="I48" r:id="rId21" xr:uid="{E1BC7B04-B072-447B-9137-59A28141883D}"/>
+    <hyperlink ref="I97" r:id="rId22" xr:uid="{BEDF45F1-312C-4FF5-B4F5-1D1C7E487C0A}"/>
+    <hyperlink ref="I59" r:id="rId23" xr:uid="{6E82D57D-36A4-4928-AD91-BE73FFC7C389}"/>
+    <hyperlink ref="I74" r:id="rId24" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
+    <hyperlink ref="I92" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
+    <hyperlink ref="I121" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
+    <hyperlink ref="I81" r:id="rId27" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
+    <hyperlink ref="I82" r:id="rId28" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
+    <hyperlink ref="I87" r:id="rId29" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
+    <hyperlink ref="I105" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
+    <hyperlink ref="I116" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
+    <hyperlink ref="I119" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
+    <hyperlink ref="I124" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
+    <hyperlink ref="I126" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
+    <hyperlink ref="I128" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
     <hyperlink ref="I15" r:id="rId36" xr:uid="{E26D4CB1-6F14-4277-AD54-18A052872B6B}"/>
-    <hyperlink ref="I122" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
+    <hyperlink ref="I123" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
     <hyperlink ref="I8" r:id="rId38" xr:uid="{2E646106-878B-4504-8874-8750F3CAA7CB}"/>
     <hyperlink ref="I33" r:id="rId39" xr:uid="{902A8808-023C-4EA1-833E-F687288B12ED}"/>
-    <hyperlink ref="I129" r:id="rId40" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
-    <hyperlink ref="I107" r:id="rId41" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
+    <hyperlink ref="I130" r:id="rId40" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
+    <hyperlink ref="I108" r:id="rId41" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
+    <hyperlink ref="I47" r:id="rId42" xr:uid="{ABEB73EB-E336-4619-ADE1-0AE567E81306}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId42"/>
+  <pageSetup orientation="portrait" r:id="rId43"/>
   <tableParts count="1">
-    <tablePart r:id="rId43"/>
+    <tablePart r:id="rId44"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7006,6 +7054,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7014,15 +7071,6 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7045,6 +7093,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7059,12 +7115,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Mise à jour concernant Amy Bergeron
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA03163-3143-40F3-9D42-B948BFB2C5E3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A38366AB-A445-420B-87F8-C5E6FA28A1AD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19460" yWindow="4650" windowWidth="20480" windowHeight="23450" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="727">
   <si>
     <t>nom</t>
   </si>
@@ -298,9 +298,6 @@
   </si>
   <si>
     <t>amy-bergeron.jpg</t>
-  </si>
-  <si>
-    <t>Études médicales de premier cycle (Doctorat en médecine), gériatrie, sciences biomédicales</t>
   </si>
   <si>
     <t>514-343-6111, poste 0865</t>
@@ -2986,7 +2983,7 @@
         <v>42</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>21</v>
@@ -3084,7 +3081,7 @@
         <v>43</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>44</v>
@@ -3130,31 +3127,31 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B8" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
       </c>
       <c r="H8" t="s">
+        <v>658</v>
+      </c>
+      <c r="I8" s="21" t="s">
         <v>659</v>
-      </c>
-      <c r="I8" s="21" t="s">
-        <v>660</v>
       </c>
       <c r="J8" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3236,10 +3233,10 @@
         <v>71</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>72</v>
@@ -3260,7 +3257,7 @@
         <v>39</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>75</v>
@@ -3323,20 +3320,22 @@
         <v>90</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>128</v>
+      </c>
       <c r="F14" s="7" t="s">
-        <v>91</v>
+        <v>508</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H14" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="I14" s="8" t="s">
         <v>92</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>93</v>
       </c>
       <c r="J14" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3345,27 +3344,27 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="C15" s="7" t="s">
+        <v>685</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>95</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>686</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>96</v>
       </c>
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
       <c r="G15" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="H15" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="I15" s="14" t="s">
         <v>98</v>
-      </c>
-      <c r="I15" s="14" t="s">
-        <v>99</v>
       </c>
       <c r="J15" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3374,25 +3373,25 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="D16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G16" t="s">
         <v>29</v>
       </c>
       <c r="H16" t="s">
+        <v>105</v>
+      </c>
+      <c r="I16" s="15" t="s">
         <v>106</v>
-      </c>
-      <c r="I16" s="15" t="s">
-        <v>107</v>
       </c>
       <c r="J16" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3401,10 +3400,10 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>101</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
@@ -3414,14 +3413,14 @@
         <v>84</v>
       </c>
       <c r="F17" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="G17" t="s">
         <v>102</v>
-      </c>
-      <c r="G17" t="s">
-        <v>103</v>
       </c>
       <c r="H17" s="5"/>
       <c r="I17" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J17" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3430,29 +3429,29 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>110</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>111</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>84</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H18" s="5"/>
       <c r="I18" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J18" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3461,28 +3460,28 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
+        <v>113</v>
+      </c>
+      <c r="B19" t="s">
         <v>114</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" s="18" t="s">
         <v>115</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>116</v>
       </c>
       <c r="D19" t="s">
         <v>13</v>
       </c>
       <c r="F19" s="28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G19" t="s">
         <v>15</v>
       </c>
       <c r="H19" t="s">
+        <v>117</v>
+      </c>
+      <c r="I19" t="s">
         <v>118</v>
-      </c>
-      <c r="I19" t="s">
-        <v>119</v>
       </c>
       <c r="J19" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3491,24 +3490,24 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>120</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>121</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E20" s="8" t="s">
         <v>63</v>
       </c>
       <c r="F20" s="8"/>
       <c r="H20" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="I20" s="8" t="s">
         <v>123</v>
-      </c>
-      <c r="I20" s="8" t="s">
-        <v>124</v>
       </c>
       <c r="J20" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3517,28 +3516,28 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="G21" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="H21" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="I21" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>132</v>
       </c>
       <c r="J21" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3547,29 +3546,29 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="C22" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>135</v>
-      </c>
       <c r="D22" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="G22" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="H22" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="I22" s="7" t="s">
         <v>138</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>139</v>
       </c>
       <c r="J22" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3578,29 +3577,29 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="C23" s="5" t="s">
         <v>141</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>142</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E23" s="5"/>
       <c r="F23" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="H23" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G23" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="H23" s="5" t="s">
+      <c r="I23" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="J23" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3609,31 +3608,31 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="C24" s="7" t="s">
+        <v>665</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>147</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>666</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>148</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>76</v>
       </c>
       <c r="F24" s="27" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="H24" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="I24" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>150</v>
       </c>
       <c r="J24" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3642,29 +3641,29 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B25" s="7" t="s">
-        <v>152</v>
-      </c>
       <c r="C25" s="7" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>49</v>
       </c>
       <c r="E25" s="7"/>
       <c r="F25" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>654</v>
+      </c>
+      <c r="H25" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="G25" s="7" t="s">
-        <v>655</v>
-      </c>
-      <c r="H25" s="7" t="s">
+      <c r="I25" s="7" t="s">
         <v>154</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>155</v>
       </c>
       <c r="J25" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3673,13 +3672,13 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="C26" s="7" t="s">
         <v>157</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>158</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>70</v>
@@ -3689,10 +3688,10 @@
       </c>
       <c r="F26" s="7"/>
       <c r="H26" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="I26" s="7" t="s">
         <v>159</v>
-      </c>
-      <c r="I26" s="7" t="s">
-        <v>160</v>
       </c>
       <c r="J26" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3701,25 +3700,25 @@
     </row>
     <row r="27" spans="1:10">
       <c r="A27" t="s">
+        <v>160</v>
+      </c>
+      <c r="B27" t="s">
         <v>161</v>
       </c>
-      <c r="B27" t="s">
-        <v>162</v>
-      </c>
       <c r="C27" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="D27" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G27" t="s">
         <v>29</v>
       </c>
       <c r="H27" t="s">
+        <v>162</v>
+      </c>
+      <c r="I27" s="15" t="s">
         <v>163</v>
-      </c>
-      <c r="I27" s="15" t="s">
-        <v>164</v>
       </c>
       <c r="J27" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3728,29 +3727,29 @@
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="C28" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>166</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>675</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>167</v>
       </c>
       <c r="E28" s="5"/>
       <c r="F28" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="G28" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="G28" s="5" t="s">
+      <c r="H28" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="H28" s="5" t="s">
+      <c r="I28" s="10" t="s">
         <v>170</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>171</v>
       </c>
       <c r="J28" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3759,29 +3758,29 @@
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="B29" s="5" t="s">
-        <v>173</v>
-      </c>
       <c r="C29" s="5" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>49</v>
       </c>
       <c r="E29" s="5"/>
       <c r="F29" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G29" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="G29" s="5" t="s">
+      <c r="H29" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="H29" s="5" t="s">
+      <c r="I29" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="I29" s="5" t="s">
-        <v>177</v>
       </c>
       <c r="J29" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3790,29 +3789,29 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C30" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>180</v>
-      </c>
       <c r="D30" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>76</v>
       </c>
       <c r="F30" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="G30" t="s">
         <v>181</v>
-      </c>
-      <c r="G30" t="s">
-        <v>182</v>
       </c>
       <c r="H30" s="5"/>
       <c r="I30" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="J30" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3821,22 +3820,22 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
+        <v>183</v>
+      </c>
+      <c r="B31" t="s">
         <v>184</v>
       </c>
-      <c r="B31" t="s">
-        <v>185</v>
-      </c>
       <c r="C31" s="25" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="D31" t="s">
         <v>27</v>
       </c>
       <c r="F31" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="G31" t="s">
         <v>136</v>
-      </c>
-      <c r="G31" t="s">
-        <v>137</v>
       </c>
       <c r="J31" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3845,22 +3844,22 @@
     </row>
     <row r="32" spans="1:10">
       <c r="A32" t="s">
+        <v>185</v>
+      </c>
+      <c r="B32" t="s">
         <v>186</v>
-      </c>
-      <c r="B32" t="s">
-        <v>187</v>
       </c>
       <c r="D32" t="s">
         <v>49</v>
       </c>
       <c r="G32" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="H32" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="I32" s="15" t="s">
         <v>188</v>
-      </c>
-      <c r="I32" s="15" t="s">
-        <v>189</v>
       </c>
       <c r="J32" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3869,26 +3868,26 @@
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B33" s="5" t="s">
         <v>190</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>191</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E33" s="12" t="s">
         <v>63</v>
       </c>
       <c r="G33" s="5" t="s">
+        <v>710</v>
+      </c>
+      <c r="H33" s="11" t="s">
         <v>711</v>
       </c>
-      <c r="H33" s="11" t="s">
+      <c r="I33" s="10" t="s">
         <v>712</v>
-      </c>
-      <c r="I33" s="10" t="s">
-        <v>713</v>
       </c>
       <c r="J33" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3897,29 +3896,29 @@
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="B34" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="C34" s="7" t="s">
         <v>194</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>195</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E34" s="7"/>
       <c r="F34" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="H34" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="G34" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="H34" s="7" t="s">
+      <c r="I34" s="7" t="s">
         <v>197</v>
-      </c>
-      <c r="I34" s="7" t="s">
-        <v>198</v>
       </c>
       <c r="J34" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3928,28 +3927,28 @@
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="B35" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>202</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>84</v>
       </c>
       <c r="F35" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="H35" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="H35" s="5" t="s">
+      <c r="I35" s="5" t="s">
         <v>204</v>
-      </c>
-      <c r="I35" s="5" t="s">
-        <v>205</v>
       </c>
       <c r="J35" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3958,29 +3957,29 @@
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="B36" s="7" t="s">
-        <v>207</v>
-      </c>
       <c r="C36" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E36" s="7"/>
       <c r="F36" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G36" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H36" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="I36" s="7" t="s">
         <v>209</v>
-      </c>
-      <c r="I36" s="7" t="s">
-        <v>210</v>
       </c>
       <c r="J36" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3989,31 +3988,31 @@
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B37" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="C37" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="D37" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="E37" t="s">
         <v>214</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" s="27" t="s">
         <v>215</v>
       </c>
-      <c r="F37" s="27" t="s">
+      <c r="G37" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="H37" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="G37" s="7" t="s">
-        <v>641</v>
-      </c>
-      <c r="H37" s="5" t="s">
+      <c r="I37" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="I37" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="J37" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4022,29 +4021,29 @@
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="B38" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="C38" s="7" t="s">
         <v>220</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>221</v>
       </c>
       <c r="D38" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E38" s="7"/>
       <c r="F38" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="H38" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="G38" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="H38" s="7" t="s">
+      <c r="I38" s="7" t="s">
         <v>223</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>224</v>
       </c>
       <c r="J38" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4053,29 +4052,29 @@
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="B39" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="B39" s="5" t="s">
-        <v>226</v>
-      </c>
       <c r="C39" s="5" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E39" s="5"/>
       <c r="F39" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>57</v>
       </c>
       <c r="H39" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="I39" s="5" t="s">
         <v>228</v>
-      </c>
-      <c r="I39" s="5" t="s">
-        <v>229</v>
       </c>
       <c r="J39" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4084,29 +4083,29 @@
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="B40" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="C40" s="5" t="s">
         <v>231</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>232</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E40" s="5"/>
       <c r="F40" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H40" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="I40" s="5" t="s">
         <v>234</v>
-      </c>
-      <c r="I40" s="5" t="s">
-        <v>235</v>
       </c>
       <c r="J40" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4115,29 +4114,29 @@
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="B41" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="C41" s="26" t="s">
         <v>237</v>
       </c>
-      <c r="C41" s="26" t="s">
+      <c r="D41" s="7" t="s">
         <v>238</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>239</v>
       </c>
       <c r="E41" s="5"/>
       <c r="F41" s="27" t="s">
+        <v>240</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="H41" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="G41" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="H41" s="7" t="s">
+      <c r="I41" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="I41" s="7" t="s">
-        <v>243</v>
       </c>
       <c r="J41" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4146,29 +4145,29 @@
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="B42" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="B42" s="7" t="s">
+      <c r="C42" s="7" t="s">
         <v>245</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>246</v>
       </c>
       <c r="D42" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E42" s="7"/>
       <c r="F42" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="H42" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="G42" s="7" t="s">
-        <v>643</v>
-      </c>
-      <c r="H42" s="7" t="s">
+      <c r="I42" s="7" t="s">
         <v>248</v>
-      </c>
-      <c r="I42" s="7" t="s">
-        <v>249</v>
       </c>
       <c r="J42" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4177,29 +4176,29 @@
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="B43" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="B43" s="7" t="s">
+      <c r="C43" s="7" t="s">
         <v>251</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>252</v>
       </c>
       <c r="D43" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E43" s="7"/>
       <c r="F43" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G43" s="7" t="s">
         <v>57</v>
       </c>
       <c r="H43" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="I43" s="7" t="s">
         <v>254</v>
-      </c>
-      <c r="I43" s="7" t="s">
-        <v>255</v>
       </c>
       <c r="J43" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4208,27 +4207,27 @@
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="B44" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="C44" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="D44" s="5" t="s">
         <v>257</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>689</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>258</v>
       </c>
       <c r="E44" s="5"/>
       <c r="F44" s="5"/>
       <c r="G44" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="H44" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="H44" s="5" t="s">
+      <c r="I44" s="5" t="s">
         <v>260</v>
-      </c>
-      <c r="I44" s="5" t="s">
-        <v>261</v>
       </c>
       <c r="J44" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4237,25 +4236,25 @@
     </row>
     <row r="45" spans="1:10">
       <c r="A45" t="s">
+        <v>261</v>
+      </c>
+      <c r="B45" t="s">
         <v>262</v>
       </c>
-      <c r="B45" t="s">
-        <v>263</v>
-      </c>
       <c r="C45" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="D45" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G45" t="s">
         <v>29</v>
       </c>
       <c r="H45" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="I45" s="15" t="s">
         <v>264</v>
-      </c>
-      <c r="I45" s="15" t="s">
-        <v>265</v>
       </c>
       <c r="J45" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4264,29 +4263,29 @@
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="B46" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="C46" s="5" t="s">
         <v>267</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>268</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>57</v>
       </c>
       <c r="H46" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="I46" s="5" t="s">
         <v>270</v>
-      </c>
-      <c r="I46" s="5" t="s">
-        <v>271</v>
       </c>
       <c r="J46" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4295,29 +4294,29 @@
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="B47" s="5" t="s">
         <v>723</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>724</v>
       </c>
       <c r="C47" s="5"/>
       <c r="D47" s="5" t="s">
         <v>27</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H47" s="5" t="s">
+        <v>725</v>
+      </c>
+      <c r="I47" s="10" t="s">
         <v>726</v>
-      </c>
-      <c r="I47" s="10" t="s">
-        <v>727</v>
       </c>
       <c r="J47" s="30" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4326,25 +4325,25 @@
     </row>
     <row r="48" spans="1:10">
       <c r="A48" t="s">
+        <v>271</v>
+      </c>
+      <c r="B48" t="s">
         <v>272</v>
       </c>
-      <c r="B48" t="s">
-        <v>273</v>
-      </c>
       <c r="C48" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="D48" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G48" t="s">
         <v>29</v>
       </c>
       <c r="H48" t="s">
+        <v>273</v>
+      </c>
+      <c r="I48" s="15" t="s">
         <v>274</v>
-      </c>
-      <c r="I48" s="15" t="s">
-        <v>275</v>
       </c>
       <c r="J48" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4353,31 +4352,31 @@
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="B49" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="B49" s="7" t="s">
+      <c r="C49" s="22" t="s">
         <v>277</v>
       </c>
-      <c r="C49" s="22" t="s">
-        <v>278</v>
-      </c>
       <c r="D49" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>43</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H49" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="I49" s="7" t="s">
         <v>279</v>
-      </c>
-      <c r="I49" s="7" t="s">
-        <v>280</v>
       </c>
       <c r="J49" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4386,29 +4385,29 @@
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="B50" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="B50" s="7" t="s">
+      <c r="C50" s="22" t="s">
         <v>277</v>
       </c>
-      <c r="C50" s="22" t="s">
-        <v>278</v>
-      </c>
       <c r="D50" s="7" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F50" s="7"/>
       <c r="G50" s="7" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="H50" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="I50" s="7" t="s">
         <v>279</v>
-      </c>
-      <c r="I50" s="7" t="s">
-        <v>280</v>
       </c>
       <c r="J50" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4417,19 +4416,19 @@
     </row>
     <row r="51" spans="1:10" ht="29">
       <c r="A51" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="B51" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="B51" s="7" t="s">
+      <c r="C51" s="7" t="s">
         <v>282</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>283</v>
       </c>
       <c r="D51" s="7" t="s">
         <v>41</v>
       </c>
       <c r="E51" s="17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>43</v>
@@ -4438,10 +4437,10 @@
         <v>29</v>
       </c>
       <c r="H51" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="I51" s="7" t="s">
         <v>285</v>
-      </c>
-      <c r="I51" s="7" t="s">
-        <v>286</v>
       </c>
       <c r="J51" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4450,27 +4449,27 @@
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="B52" s="7" t="s">
         <v>287</v>
-      </c>
-      <c r="B52" s="7" t="s">
-        <v>288</v>
       </c>
       <c r="C52" s="7"/>
       <c r="D52" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E52" s="7"/>
       <c r="F52" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="G52" s="7" t="s">
         <v>289</v>
       </c>
-      <c r="G52" s="7" t="s">
+      <c r="H52" s="7" t="s">
         <v>290</v>
       </c>
-      <c r="H52" s="7" t="s">
+      <c r="I52" s="7" t="s">
         <v>291</v>
-      </c>
-      <c r="I52" s="7" t="s">
-        <v>292</v>
       </c>
       <c r="J52" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4479,29 +4478,29 @@
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="B53" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="B53" s="7" t="s">
+      <c r="C53" s="7" t="s">
         <v>294</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>295</v>
       </c>
       <c r="D53" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E53" s="7"/>
       <c r="F53" s="7" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G53" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H53" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="I53" s="7" t="s">
         <v>297</v>
-      </c>
-      <c r="I53" s="7" t="s">
-        <v>298</v>
       </c>
       <c r="J53" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4510,27 +4509,27 @@
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="B54" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="C54" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="D54" s="5" t="s">
         <v>300</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>301</v>
       </c>
       <c r="E54" s="5"/>
       <c r="F54" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H54" s="5"/>
       <c r="I54" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J54" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4539,29 +4538,29 @@
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="B55" s="7" t="s">
         <v>304</v>
       </c>
-      <c r="B55" s="7" t="s">
+      <c r="C55" s="7" t="s">
         <v>305</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>306</v>
       </c>
       <c r="D55" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E55" s="7"/>
       <c r="F55" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="G55" s="7" t="s">
         <v>307</v>
       </c>
-      <c r="G55" s="7" t="s">
+      <c r="H55" s="7" t="s">
         <v>308</v>
       </c>
-      <c r="H55" s="7" t="s">
+      <c r="I55" s="7" t="s">
         <v>309</v>
-      </c>
-      <c r="I55" s="7" t="s">
-        <v>310</v>
       </c>
       <c r="J55" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4570,26 +4569,26 @@
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="B56" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="C56" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="C56" s="5" t="s">
+      <c r="D56" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="D56" s="5" t="s">
-        <v>314</v>
-      </c>
       <c r="E56" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F56" s="5"/>
       <c r="H56" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I56" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="J56" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4598,24 +4597,24 @@
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F57" s="5"/>
       <c r="H57" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I57" s="5" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="J57" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4624,13 +4623,13 @@
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="B58" s="7" t="s">
         <v>318</v>
       </c>
-      <c r="B58" s="7" t="s">
+      <c r="C58" s="7" t="s">
         <v>319</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>320</v>
       </c>
       <c r="D58" s="7" t="s">
         <v>27</v>
@@ -4639,13 +4638,13 @@
         <v>84</v>
       </c>
       <c r="F58" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="H58" s="7" t="s">
         <v>321</v>
       </c>
-      <c r="H58" s="7" t="s">
+      <c r="I58" s="7" t="s">
         <v>322</v>
-      </c>
-      <c r="I58" s="7" t="s">
-        <v>323</v>
       </c>
       <c r="J58" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4654,10 +4653,10 @@
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C59" s="5"/>
       <c r="D59" s="5" t="s">
@@ -4665,16 +4664,16 @@
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="G59" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="G59" s="5" t="s">
+      <c r="H59" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="I59" s="13" t="s">
         <v>326</v>
-      </c>
-      <c r="H59" s="8" t="s">
-        <v>542</v>
-      </c>
-      <c r="I59" s="13" t="s">
-        <v>327</v>
       </c>
       <c r="J59" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4683,13 +4682,13 @@
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="B60" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="B60" s="5" t="s">
-        <v>329</v>
-      </c>
       <c r="C60" s="5" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>27</v>
@@ -4698,13 +4697,13 @@
         <v>84</v>
       </c>
       <c r="F60" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="G60" s="5" t="s">
         <v>330</v>
       </c>
-      <c r="G60" s="5" t="s">
+      <c r="H60" s="5" t="s">
         <v>331</v>
-      </c>
-      <c r="H60" s="5" t="s">
-        <v>332</v>
       </c>
       <c r="I60" s="5"/>
       <c r="J60" s="10" t="str">
@@ -4714,29 +4713,29 @@
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C61" s="5" t="s">
         <v>333</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>334</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E61" s="5"/>
       <c r="F61" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="G61" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="H61" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="G61" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="H61" s="5" t="s">
+      <c r="I61" s="5" t="s">
         <v>336</v>
-      </c>
-      <c r="I61" s="5" t="s">
-        <v>337</v>
       </c>
       <c r="J61" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4745,29 +4744,29 @@
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="B62" s="7" t="s">
         <v>338</v>
       </c>
-      <c r="B62" s="7" t="s">
+      <c r="C62" s="7" t="s">
         <v>339</v>
-      </c>
-      <c r="C62" s="7" t="s">
-        <v>340</v>
       </c>
       <c r="D62" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E62" s="7"/>
       <c r="F62" s="7" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G62" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H62" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="I62" s="7" t="s">
         <v>342</v>
-      </c>
-      <c r="I62" s="7" t="s">
-        <v>343</v>
       </c>
       <c r="J62" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4776,29 +4775,29 @@
     </row>
     <row r="63" spans="1:10" s="3" customFormat="1">
       <c r="A63" t="s">
+        <v>343</v>
+      </c>
+      <c r="B63" t="s">
         <v>344</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" s="19" t="s">
         <v>345</v>
-      </c>
-      <c r="C63" s="19" t="s">
-        <v>346</v>
       </c>
       <c r="D63" t="s">
         <v>13</v>
       </c>
       <c r="E63"/>
       <c r="F63" s="28" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G63" t="s">
         <v>15</v>
       </c>
       <c r="H63" t="s">
+        <v>347</v>
+      </c>
+      <c r="I63" t="s">
         <v>348</v>
-      </c>
-      <c r="I63" t="s">
-        <v>349</v>
       </c>
       <c r="J63" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4807,16 +4806,16 @@
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="B64" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="C64" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="C64" s="5" t="s">
-        <v>352</v>
-      </c>
       <c r="D64" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E64" s="7" t="s">
         <v>76</v>
@@ -4824,10 +4823,10 @@
       <c r="F64" s="29"/>
       <c r="G64" s="3"/>
       <c r="H64" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="I64" s="5" t="s">
         <v>353</v>
-      </c>
-      <c r="I64" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="J64" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4836,29 +4835,29 @@
     </row>
     <row r="65" spans="1:10" s="4" customFormat="1">
       <c r="A65" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="B65" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="C65" s="5" t="s">
         <v>356</v>
-      </c>
-      <c r="C65" s="5" t="s">
-        <v>357</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="5" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="G65" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H65" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="I65" s="5" t="s">
         <v>358</v>
-      </c>
-      <c r="I65" s="5" t="s">
-        <v>359</v>
       </c>
       <c r="J65" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4867,25 +4866,25 @@
     </row>
     <row r="66" spans="1:10">
       <c r="A66" t="s">
+        <v>359</v>
+      </c>
+      <c r="B66" t="s">
         <v>360</v>
       </c>
-      <c r="B66" t="s">
-        <v>361</v>
-      </c>
       <c r="C66" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="D66" t="s">
         <v>49</v>
       </c>
       <c r="G66" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H66" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="I66" s="15" t="s">
         <v>362</v>
-      </c>
-      <c r="I66" s="15" t="s">
-        <v>363</v>
       </c>
       <c r="J66" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4894,27 +4893,27 @@
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="7" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C67" s="7"/>
       <c r="D67" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E67" s="7"/>
       <c r="F67" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="G67" s="7" t="s">
         <v>325</v>
       </c>
-      <c r="G67" s="7" t="s">
-        <v>326</v>
-      </c>
       <c r="H67" s="7" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I67" s="9" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="J67" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4923,25 +4922,25 @@
     </row>
     <row r="68" spans="1:10">
       <c r="A68" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B68" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C68" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="D68" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G68" t="s">
         <v>29</v>
       </c>
       <c r="H68" s="16" t="s">
+        <v>366</v>
+      </c>
+      <c r="I68" s="15" t="s">
         <v>367</v>
-      </c>
-      <c r="I68" s="15" t="s">
-        <v>368</v>
       </c>
       <c r="J68" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4950,31 +4949,31 @@
     </row>
     <row r="69" spans="1:10">
       <c r="A69" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="B69" s="7" t="s">
         <v>369</v>
       </c>
-      <c r="B69" s="7" t="s">
+      <c r="C69" s="7" t="s">
         <v>370</v>
       </c>
-      <c r="C69" s="7" t="s">
-        <v>371</v>
-      </c>
       <c r="D69" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E69" s="7" t="s">
         <v>76</v>
       </c>
       <c r="F69" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="G69" s="7" t="s">
+        <v>654</v>
+      </c>
+      <c r="H69" s="7" t="s">
         <v>372</v>
       </c>
-      <c r="G69" s="7" t="s">
-        <v>655</v>
-      </c>
-      <c r="H69" s="7" t="s">
+      <c r="I69" s="7" t="s">
         <v>373</v>
-      </c>
-      <c r="I69" s="7" t="s">
-        <v>374</v>
       </c>
       <c r="J69" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4983,31 +4982,31 @@
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="B70" s="5" t="s">
         <v>375</v>
       </c>
-      <c r="B70" s="5" t="s">
+      <c r="C70" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="C70" s="5" t="s">
-        <v>377</v>
-      </c>
       <c r="D70" s="5" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F70" s="5" t="s">
         <v>43</v>
       </c>
       <c r="G70" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H70" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="I70" s="5" t="s">
         <v>378</v>
-      </c>
-      <c r="I70" s="5" t="s">
-        <v>379</v>
       </c>
       <c r="J70" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5016,31 +5015,31 @@
     </row>
     <row r="71" spans="1:10" ht="29">
       <c r="A71" s="7" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D71" s="7" t="s">
         <v>41</v>
       </c>
       <c r="E71" s="17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G71" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H71" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="I71" s="7" t="s">
         <v>382</v>
-      </c>
-      <c r="I71" s="7" t="s">
-        <v>383</v>
       </c>
       <c r="J71" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5049,25 +5048,25 @@
     </row>
     <row r="72" spans="1:10">
       <c r="A72" t="s">
+        <v>383</v>
+      </c>
+      <c r="B72" t="s">
         <v>384</v>
       </c>
-      <c r="B72" t="s">
-        <v>385</v>
-      </c>
       <c r="C72" s="5" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D72" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G72" t="s">
         <v>29</v>
       </c>
       <c r="H72" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="I72" s="15" t="s">
         <v>386</v>
-      </c>
-      <c r="I72" s="15" t="s">
-        <v>387</v>
       </c>
       <c r="J72" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5076,29 +5075,29 @@
     </row>
     <row r="73" spans="1:10">
       <c r="A73" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="B73" s="7" t="s">
         <v>388</v>
       </c>
-      <c r="B73" s="7" t="s">
+      <c r="C73" s="5" t="s">
         <v>389</v>
-      </c>
-      <c r="C73" s="5" t="s">
-        <v>390</v>
       </c>
       <c r="D73" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E73" s="7"/>
       <c r="F73" s="7" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G73" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H73" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="I73" s="7" t="s">
         <v>391</v>
-      </c>
-      <c r="I73" s="7" t="s">
-        <v>392</v>
       </c>
       <c r="J73" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5107,29 +5106,29 @@
     </row>
     <row r="74" spans="1:10" s="3" customFormat="1">
       <c r="A74" t="s">
+        <v>392</v>
+      </c>
+      <c r="B74" t="s">
         <v>393</v>
       </c>
-      <c r="B74" t="s">
-        <v>394</v>
-      </c>
       <c r="C74" s="5" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="D74" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E74" s="7"/>
       <c r="F74" s="27" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="G74" s="7" t="s">
         <v>76</v>
       </c>
       <c r="H74" t="s">
+        <v>395</v>
+      </c>
+      <c r="I74" s="15" t="s">
         <v>396</v>
-      </c>
-      <c r="I74" s="15" t="s">
-        <v>397</v>
       </c>
       <c r="J74" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5138,28 +5137,28 @@
     </row>
     <row r="75" spans="1:10" s="3" customFormat="1">
       <c r="A75" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="B75" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="B75" s="7" t="s">
+      <c r="C75" s="5" t="s">
         <v>399</v>
       </c>
-      <c r="C75" s="5" t="s">
-        <v>400</v>
-      </c>
       <c r="D75" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E75" s="7" t="s">
         <v>76</v>
       </c>
       <c r="G75" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H75" s="7" t="s">
+        <v>400</v>
+      </c>
+      <c r="I75" s="7" t="s">
         <v>401</v>
-      </c>
-      <c r="I75" s="7" t="s">
-        <v>402</v>
       </c>
       <c r="J75" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5168,31 +5167,31 @@
     </row>
     <row r="76" spans="1:10">
       <c r="A76" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="B76" s="5" t="s">
         <v>403</v>
       </c>
-      <c r="B76" s="5" t="s">
+      <c r="C76" s="5" t="s">
         <v>404</v>
       </c>
-      <c r="C76" s="5" t="s">
+      <c r="D76" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="F76" s="29" t="s">
         <v>405</v>
       </c>
-      <c r="D76" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="E76" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="F76" s="29" t="s">
+      <c r="G76" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="H76" s="5" t="s">
         <v>406</v>
       </c>
-      <c r="G76" s="7" t="s">
-        <v>641</v>
-      </c>
-      <c r="H76" s="5" t="s">
+      <c r="I76" s="5" t="s">
         <v>407</v>
-      </c>
-      <c r="I76" s="5" t="s">
-        <v>408</v>
       </c>
       <c r="J76" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5201,28 +5200,28 @@
     </row>
     <row r="77" spans="1:10">
       <c r="A77" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="B77" s="7" t="s">
         <v>409</v>
       </c>
-      <c r="B77" s="7" t="s">
-        <v>410</v>
-      </c>
       <c r="C77" s="5" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E77" s="7" t="s">
         <v>84</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H77" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="I77" s="7" t="s">
         <v>411</v>
-      </c>
-      <c r="I77" s="7" t="s">
-        <v>412</v>
       </c>
       <c r="J77" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5231,29 +5230,29 @@
     </row>
     <row r="78" spans="1:10" s="3" customFormat="1" ht="29">
       <c r="A78" s="5" t="s">
+        <v>412</v>
+      </c>
+      <c r="B78" s="5" t="s">
         <v>413</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="C78" s="5" t="s">
         <v>414</v>
       </c>
-      <c r="C78" s="5" t="s">
-        <v>415</v>
-      </c>
       <c r="D78" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E78" s="17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F78" s="5"/>
       <c r="G78" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H78" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="I78" s="5" t="s">
         <v>416</v>
-      </c>
-      <c r="I78" s="5" t="s">
-        <v>417</v>
       </c>
       <c r="J78" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5262,13 +5261,13 @@
     </row>
     <row r="79" spans="1:10">
       <c r="A79" s="8" t="s">
+        <v>417</v>
+      </c>
+      <c r="B79" s="8" t="s">
         <v>418</v>
       </c>
-      <c r="B79" s="8" t="s">
-        <v>419</v>
-      </c>
       <c r="C79" s="8" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="D79" s="8" t="s">
         <v>41</v>
@@ -5277,16 +5276,16 @@
         <v>42</v>
       </c>
       <c r="F79" s="27" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="G79" s="8" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="H79" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="I79" s="8" t="s">
         <v>420</v>
-      </c>
-      <c r="I79" s="8" t="s">
-        <v>421</v>
       </c>
       <c r="J79" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5295,16 +5294,16 @@
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="5" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E80" s="5" t="s">
         <v>84</v>
@@ -5312,7 +5311,7 @@
       <c r="F80" s="5"/>
       <c r="H80" s="5"/>
       <c r="I80" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J80" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5321,16 +5320,16 @@
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="B81" s="5" t="s">
         <v>424</v>
       </c>
-      <c r="B81" s="5" t="s">
+      <c r="C81" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="D81" s="5" t="s">
         <v>425</v>
-      </c>
-      <c r="C81" s="5" t="s">
-        <v>691</v>
-      </c>
-      <c r="D81" s="5" t="s">
-        <v>426</v>
       </c>
       <c r="E81" s="5"/>
       <c r="F81" s="5"/>
@@ -5338,10 +5337,10 @@
         <v>57</v>
       </c>
       <c r="H81" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="I81" s="13" t="s">
         <v>427</v>
-      </c>
-      <c r="I81" s="13" t="s">
-        <v>428</v>
       </c>
       <c r="J81" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5350,27 +5349,27 @@
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B82" s="5" t="s">
         <v>429</v>
       </c>
-      <c r="B82" s="5" t="s">
-        <v>430</v>
-      </c>
       <c r="C82" s="5" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E82" s="5"/>
       <c r="F82" s="5"/>
       <c r="G82" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="H82" s="5" t="s">
         <v>431</v>
       </c>
-      <c r="H82" s="5" t="s">
+      <c r="I82" s="13" t="s">
         <v>432</v>
-      </c>
-      <c r="I82" s="13" t="s">
-        <v>433</v>
       </c>
       <c r="J82" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5379,29 +5378,29 @@
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="B83" s="5" t="s">
         <v>434</v>
       </c>
-      <c r="B83" s="5" t="s">
+      <c r="C83" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="D83" s="5" t="s">
         <v>435</v>
-      </c>
-      <c r="C83" s="5" t="s">
-        <v>705</v>
-      </c>
-      <c r="D83" s="5" t="s">
-        <v>436</v>
       </c>
       <c r="E83" s="5"/>
       <c r="F83" s="27" t="s">
+        <v>436</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="H83" s="11" t="s">
         <v>437</v>
       </c>
-      <c r="G83" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="H83" s="11" t="s">
+      <c r="I83" s="13" t="s">
         <v>438</v>
-      </c>
-      <c r="I83" s="13" t="s">
-        <v>439</v>
       </c>
       <c r="J83" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5410,29 +5409,29 @@
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="B84" s="5" t="s">
         <v>440</v>
       </c>
-      <c r="B84" s="5" t="s">
+      <c r="C84" s="5" t="s">
         <v>441</v>
-      </c>
-      <c r="C84" s="5" t="s">
-        <v>442</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E84" s="5"/>
       <c r="F84" s="5" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="G84" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H84" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="I84" s="5" t="s">
         <v>443</v>
-      </c>
-      <c r="I84" s="5" t="s">
-        <v>444</v>
       </c>
       <c r="J84" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5441,29 +5440,29 @@
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="C85" s="5" t="s">
         <v>445</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="C85" s="5" t="s">
-        <v>446</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E85" s="5"/>
       <c r="F85" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="G85" s="5" t="s">
         <v>447</v>
       </c>
-      <c r="G85" s="5" t="s">
+      <c r="H85" s="5" t="s">
         <v>448</v>
       </c>
-      <c r="H85" s="5" t="s">
+      <c r="I85" s="5" t="s">
         <v>449</v>
-      </c>
-      <c r="I85" s="5" t="s">
-        <v>450</v>
       </c>
       <c r="J85" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5472,13 +5471,13 @@
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="B86" s="5" t="s">
         <v>451</v>
       </c>
-      <c r="B86" s="5" t="s">
+      <c r="C86" s="5" t="s">
         <v>452</v>
-      </c>
-      <c r="C86" s="5" t="s">
-        <v>453</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>41</v>
@@ -5487,13 +5486,13 @@
         <v>76</v>
       </c>
       <c r="G86" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="H86" s="5" t="s">
         <v>454</v>
       </c>
-      <c r="H86" s="5" t="s">
+      <c r="I86" s="5" t="s">
         <v>455</v>
-      </c>
-      <c r="I86" s="5" t="s">
-        <v>456</v>
       </c>
       <c r="J86" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5502,27 +5501,27 @@
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B87" s="5" t="s">
         <v>457</v>
       </c>
-      <c r="B87" s="5" t="s">
-        <v>458</v>
-      </c>
       <c r="C87" s="5" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E87" s="5"/>
       <c r="F87" s="5"/>
       <c r="G87" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H87" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="I87" s="13" t="s">
         <v>459</v>
-      </c>
-      <c r="I87" s="13" t="s">
-        <v>460</v>
       </c>
       <c r="J87" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5531,29 +5530,29 @@
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="B88" s="5" t="s">
         <v>461</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="C88" s="5" t="s">
         <v>462</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>463</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E88" s="5"/>
       <c r="F88" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="G88" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="H88" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="G88" s="5" t="s">
-        <v>431</v>
-      </c>
-      <c r="H88" s="5" t="s">
+      <c r="I88" s="5" t="s">
         <v>465</v>
-      </c>
-      <c r="I88" s="5" t="s">
-        <v>466</v>
       </c>
       <c r="J88" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5562,29 +5561,29 @@
     </row>
     <row r="89" spans="1:10">
       <c r="A89" s="11" t="s">
+        <v>466</v>
+      </c>
+      <c r="B89" s="11" t="s">
         <v>467</v>
       </c>
-      <c r="B89" s="11" t="s">
+      <c r="C89" s="5" t="s">
         <v>468</v>
-      </c>
-      <c r="C89" s="5" t="s">
-        <v>469</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E89" s="5"/>
       <c r="F89" s="11" t="s">
+        <v>446</v>
+      </c>
+      <c r="G89" s="11" t="s">
         <v>447</v>
       </c>
-      <c r="G89" s="11" t="s">
-        <v>448</v>
-      </c>
       <c r="H89" s="11" t="s">
+        <v>469</v>
+      </c>
+      <c r="I89" s="11" t="s">
         <v>470</v>
-      </c>
-      <c r="I89" s="11" t="s">
-        <v>471</v>
       </c>
       <c r="J89" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5593,16 +5592,16 @@
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="7" t="s">
+        <v>471</v>
+      </c>
+      <c r="B90" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="B90" s="7" t="s">
+      <c r="C90" s="5" t="s">
         <v>473</v>
       </c>
-      <c r="C90" s="5" t="s">
-        <v>474</v>
-      </c>
       <c r="D90" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E90" s="7"/>
       <c r="F90" s="7" t="s">
@@ -5612,10 +5611,10 @@
         <v>76</v>
       </c>
       <c r="H90" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="I90" s="7" t="s">
         <v>475</v>
-      </c>
-      <c r="I90" s="7" t="s">
-        <v>476</v>
       </c>
       <c r="J90" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5624,29 +5623,29 @@
     </row>
     <row r="91" spans="1:10">
       <c r="A91" s="7" t="s">
+        <v>476</v>
+      </c>
+      <c r="B91" s="7" t="s">
         <v>477</v>
       </c>
-      <c r="B91" s="7" t="s">
+      <c r="C91" s="5" t="s">
         <v>478</v>
-      </c>
-      <c r="C91" s="5" t="s">
-        <v>479</v>
       </c>
       <c r="D91" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E91" s="7"/>
       <c r="F91" s="7" t="s">
+        <v>479</v>
+      </c>
+      <c r="G91" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="H91" s="7" t="s">
         <v>480</v>
       </c>
-      <c r="G91" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="H91" s="7" t="s">
+      <c r="I91" s="7" t="s">
         <v>481</v>
-      </c>
-      <c r="I91" s="7" t="s">
-        <v>482</v>
       </c>
       <c r="J91" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5655,29 +5654,29 @@
     </row>
     <row r="92" spans="1:10">
       <c r="A92" t="s">
+        <v>482</v>
+      </c>
+      <c r="B92" t="s">
         <v>483</v>
       </c>
-      <c r="B92" t="s">
-        <v>484</v>
-      </c>
       <c r="C92" s="5" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D92" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E92" s="7"/>
       <c r="F92" s="27" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="G92" s="7" t="s">
         <v>76</v>
       </c>
       <c r="H92" t="s">
+        <v>485</v>
+      </c>
+      <c r="I92" s="15" t="s">
         <v>486</v>
-      </c>
-      <c r="I92" s="15" t="s">
-        <v>487</v>
       </c>
       <c r="J92" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5686,29 +5685,29 @@
     </row>
     <row r="93" spans="1:10">
       <c r="A93" s="11" t="s">
+        <v>487</v>
+      </c>
+      <c r="B93" s="11" t="s">
         <v>488</v>
       </c>
-      <c r="B93" s="11" t="s">
-        <v>489</v>
-      </c>
       <c r="C93" s="11" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="D93" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E93" s="11" t="s">
         <v>42</v>
       </c>
       <c r="F93" s="29"/>
       <c r="G93" s="11" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H93" s="11" t="s">
+        <v>489</v>
+      </c>
+      <c r="I93" s="11" t="s">
         <v>490</v>
-      </c>
-      <c r="I93" s="11" t="s">
-        <v>491</v>
       </c>
       <c r="J93" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5717,29 +5716,29 @@
     </row>
     <row r="94" spans="1:10">
       <c r="A94" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="B94" s="7" t="s">
         <v>492</v>
       </c>
-      <c r="B94" s="7" t="s">
+      <c r="C94" s="7" t="s">
+        <v>697</v>
+      </c>
+      <c r="D94" s="7" t="s">
         <v>493</v>
-      </c>
-      <c r="C94" s="7" t="s">
-        <v>698</v>
-      </c>
-      <c r="D94" s="7" t="s">
-        <v>494</v>
       </c>
       <c r="E94" s="7"/>
       <c r="F94" s="7" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G94" s="7" t="s">
         <v>63</v>
       </c>
       <c r="H94" s="7" t="s">
+        <v>495</v>
+      </c>
+      <c r="I94" s="7" t="s">
         <v>496</v>
-      </c>
-      <c r="I94" s="7" t="s">
-        <v>497</v>
       </c>
       <c r="J94" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5748,14 +5747,14 @@
     </row>
     <row r="95" spans="1:10" s="3" customFormat="1">
       <c r="A95" s="7" t="s">
+        <v>497</v>
+      </c>
+      <c r="B95" s="7" t="s">
         <v>498</v>
-      </c>
-      <c r="B95" s="7" t="s">
-        <v>499</v>
       </c>
       <c r="C95" s="7"/>
       <c r="D95" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E95" s="7" t="s">
         <v>76</v>
@@ -5763,10 +5762,10 @@
       <c r="F95" s="7"/>
       <c r="G95"/>
       <c r="H95" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="I95" s="7" t="s">
         <v>500</v>
-      </c>
-      <c r="I95" s="7" t="s">
-        <v>501</v>
       </c>
       <c r="J95" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5775,29 +5774,29 @@
     </row>
     <row r="96" spans="1:10" s="3" customFormat="1">
       <c r="A96" s="7" t="s">
+        <v>501</v>
+      </c>
+      <c r="B96" s="7" t="s">
         <v>502</v>
       </c>
-      <c r="B96" s="7" t="s">
-        <v>503</v>
-      </c>
       <c r="C96" s="7" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D96" s="7" t="s">
         <v>41</v>
       </c>
       <c r="E96" s="17"/>
       <c r="F96" s="8" t="s">
+        <v>571</v>
+      </c>
+      <c r="G96" t="s">
         <v>572</v>
       </c>
-      <c r="G96" t="s">
-        <v>573</v>
-      </c>
       <c r="H96" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="I96" s="7" t="s">
         <v>504</v>
-      </c>
-      <c r="I96" s="7" t="s">
-        <v>505</v>
       </c>
       <c r="J96" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5806,25 +5805,25 @@
     </row>
     <row r="97" spans="1:10">
       <c r="A97" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="B97" s="7" t="s">
         <v>506</v>
-      </c>
-      <c r="B97" s="7" t="s">
-        <v>507</v>
       </c>
       <c r="C97" s="7"/>
       <c r="D97" s="7" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="E97" s="5"/>
       <c r="F97" s="27" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="G97" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H97" s="7"/>
       <c r="I97" s="14" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="J97" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5833,13 +5832,13 @@
     </row>
     <row r="98" spans="1:10">
       <c r="A98" t="s">
+        <v>510</v>
+      </c>
+      <c r="B98" t="s">
         <v>511</v>
       </c>
-      <c r="B98" t="s">
+      <c r="C98" s="23" t="s">
         <v>512</v>
-      </c>
-      <c r="C98" s="23" t="s">
-        <v>513</v>
       </c>
       <c r="D98" t="s">
         <v>27</v>
@@ -5848,13 +5847,13 @@
         <v>84</v>
       </c>
       <c r="F98" s="28" t="s">
+        <v>513</v>
+      </c>
+      <c r="G98" t="s">
+        <v>102</v>
+      </c>
+      <c r="I98" t="s">
         <v>514</v>
-      </c>
-      <c r="G98" t="s">
-        <v>103</v>
-      </c>
-      <c r="I98" t="s">
-        <v>515</v>
       </c>
       <c r="J98" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5863,31 +5862,31 @@
     </row>
     <row r="99" spans="1:10">
       <c r="A99" s="5" t="s">
+        <v>515</v>
+      </c>
+      <c r="B99" s="5" t="s">
         <v>516</v>
       </c>
-      <c r="B99" s="5" t="s">
-        <v>517</v>
-      </c>
       <c r="C99" s="5" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="D99" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E99" s="5" t="s">
         <v>84</v>
       </c>
       <c r="F99" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="G99" t="s">
+        <v>102</v>
+      </c>
+      <c r="H99" s="11" t="s">
         <v>518</v>
       </c>
-      <c r="G99" t="s">
-        <v>103</v>
-      </c>
-      <c r="H99" s="11" t="s">
+      <c r="I99" s="11" t="s">
         <v>519</v>
-      </c>
-      <c r="I99" s="11" t="s">
-        <v>520</v>
       </c>
       <c r="J99" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5896,29 +5895,29 @@
     </row>
     <row r="100" spans="1:10">
       <c r="A100" s="7" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B100" s="7" t="s">
+        <v>525</v>
+      </c>
+      <c r="C100" s="7" t="s">
         <v>526</v>
-      </c>
-      <c r="C100" s="7" t="s">
-        <v>527</v>
       </c>
       <c r="D100" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E100" s="7"/>
       <c r="F100" s="7" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="G100" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H100" s="8" t="s">
+        <v>527</v>
+      </c>
+      <c r="I100" s="8" t="s">
         <v>528</v>
-      </c>
-      <c r="I100" s="8" t="s">
-        <v>529</v>
       </c>
       <c r="J100" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5927,29 +5926,29 @@
     </row>
     <row r="101" spans="1:10">
       <c r="A101" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="B101" s="5" t="s">
         <v>521</v>
       </c>
-      <c r="B101" s="5" t="s">
-        <v>522</v>
-      </c>
       <c r="C101" s="5" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E101" s="5"/>
       <c r="F101" s="5" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="G101" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H101" s="11" t="s">
+        <v>523</v>
+      </c>
+      <c r="I101" s="11" t="s">
         <v>524</v>
-      </c>
-      <c r="I101" s="11" t="s">
-        <v>525</v>
       </c>
       <c r="J101" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5958,29 +5957,29 @@
     </row>
     <row r="102" spans="1:10" s="4" customFormat="1">
       <c r="A102" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="C102" s="5" t="s">
         <v>530</v>
-      </c>
-      <c r="B102" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="C102" s="5" t="s">
-        <v>531</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E102" s="5"/>
       <c r="F102" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G102" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H102" s="11" t="s">
+        <v>531</v>
+      </c>
+      <c r="I102" s="11" t="s">
         <v>532</v>
-      </c>
-      <c r="I102" s="11" t="s">
-        <v>533</v>
       </c>
       <c r="J102" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5989,13 +5988,13 @@
     </row>
     <row r="103" spans="1:10" s="4" customFormat="1">
       <c r="A103" s="5" t="s">
+        <v>533</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>483</v>
+      </c>
+      <c r="C103" s="5" t="s">
         <v>534</v>
-      </c>
-      <c r="B103" s="5" t="s">
-        <v>484</v>
-      </c>
-      <c r="C103" s="5" t="s">
-        <v>535</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>27</v>
@@ -6004,11 +6003,11 @@
         <v>84</v>
       </c>
       <c r="F103" s="5" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="H103" s="11"/>
       <c r="I103" s="10" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="J103" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6017,29 +6016,29 @@
     </row>
     <row r="104" spans="1:10">
       <c r="A104" s="7" t="s">
+        <v>537</v>
+      </c>
+      <c r="B104" s="7" t="s">
         <v>538</v>
       </c>
-      <c r="B104" s="7" t="s">
+      <c r="C104" s="7" t="s">
         <v>539</v>
-      </c>
-      <c r="C104" s="7" t="s">
-        <v>540</v>
       </c>
       <c r="D104" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E104" s="7"/>
       <c r="F104" s="7" t="s">
+        <v>540</v>
+      </c>
+      <c r="G104" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="H104" s="8" t="s">
         <v>541</v>
       </c>
-      <c r="G104" s="7" t="s">
-        <v>326</v>
-      </c>
-      <c r="H104" s="8" t="s">
+      <c r="I104" s="8" t="s">
         <v>542</v>
-      </c>
-      <c r="I104" s="8" t="s">
-        <v>543</v>
       </c>
       <c r="J104" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6048,16 +6047,16 @@
     </row>
     <row r="105" spans="1:10">
       <c r="A105" s="7" t="s">
+        <v>543</v>
+      </c>
+      <c r="B105" s="7" t="s">
         <v>544</v>
       </c>
-      <c r="B105" s="7" t="s">
-        <v>545</v>
-      </c>
       <c r="C105" s="5" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="D105" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E105" s="7"/>
       <c r="F105" s="7"/>
@@ -6065,10 +6064,10 @@
         <v>21</v>
       </c>
       <c r="H105" s="8" t="s">
+        <v>545</v>
+      </c>
+      <c r="I105" s="14" t="s">
         <v>546</v>
-      </c>
-      <c r="I105" s="14" t="s">
-        <v>547</v>
       </c>
       <c r="J105" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6077,25 +6076,25 @@
     </row>
     <row r="106" spans="1:10">
       <c r="A106" t="s">
+        <v>547</v>
+      </c>
+      <c r="B106" t="s">
         <v>548</v>
       </c>
-      <c r="B106" t="s">
+      <c r="C106" t="s">
+        <v>691</v>
+      </c>
+      <c r="D106" t="s">
+        <v>425</v>
+      </c>
+      <c r="G106" t="s">
+        <v>642</v>
+      </c>
+      <c r="H106" s="7" t="s">
         <v>549</v>
       </c>
-      <c r="C106" t="s">
-        <v>692</v>
-      </c>
-      <c r="D106" t="s">
-        <v>426</v>
-      </c>
-      <c r="G106" t="s">
-        <v>643</v>
-      </c>
-      <c r="H106" s="7" t="s">
+      <c r="I106" s="15" t="s">
         <v>550</v>
-      </c>
-      <c r="I106" s="15" t="s">
-        <v>551</v>
       </c>
       <c r="J106" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6104,23 +6103,23 @@
     </row>
     <row r="107" spans="1:10">
       <c r="A107" t="s">
+        <v>551</v>
+      </c>
+      <c r="B107" t="s">
         <v>552</v>
-      </c>
-      <c r="B107" t="s">
-        <v>553</v>
       </c>
       <c r="C107" s="25"/>
       <c r="D107" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G107" t="s">
         <v>29</v>
       </c>
       <c r="H107" t="s">
+        <v>553</v>
+      </c>
+      <c r="I107" s="15" t="s">
         <v>554</v>
-      </c>
-      <c r="I107" s="15" t="s">
-        <v>555</v>
       </c>
       <c r="J107" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6129,29 +6128,29 @@
     </row>
     <row r="108" spans="1:10">
       <c r="A108" t="s">
+        <v>708</v>
+      </c>
+      <c r="B108" t="s">
         <v>709</v>
       </c>
-      <c r="B108" t="s">
-        <v>710</v>
-      </c>
       <c r="C108" s="5" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="D108" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E108" s="5"/>
       <c r="F108" s="8" t="s">
+        <v>571</v>
+      </c>
+      <c r="G108" t="s">
         <v>572</v>
       </c>
-      <c r="G108" t="s">
-        <v>573</v>
-      </c>
       <c r="H108" t="s">
+        <v>711</v>
+      </c>
+      <c r="I108" s="21" t="s">
         <v>712</v>
-      </c>
-      <c r="I108" s="21" t="s">
-        <v>713</v>
       </c>
       <c r="J108" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6160,28 +6159,28 @@
     </row>
     <row r="109" spans="1:10">
       <c r="A109" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B109" t="s">
         <v>54</v>
       </c>
       <c r="C109" s="19" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D109" t="s">
         <v>13</v>
       </c>
       <c r="F109" s="28" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="G109" t="s">
         <v>29</v>
       </c>
       <c r="H109" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="I109" s="3" t="s">
         <v>559</v>
-      </c>
-      <c r="I109" s="3" t="s">
-        <v>560</v>
       </c>
       <c r="J109" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6190,26 +6189,26 @@
     </row>
     <row r="110" spans="1:10">
       <c r="A110" s="5" t="s">
+        <v>560</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="C110" s="5" t="s">
         <v>561</v>
       </c>
-      <c r="B110" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="C110" s="5" t="s">
-        <v>562</v>
-      </c>
       <c r="D110" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>84</v>
       </c>
       <c r="F110" s="5"/>
       <c r="H110" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I110" s="11" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="J110" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6218,27 +6217,27 @@
     </row>
     <row r="111" spans="1:10">
       <c r="A111" s="5" t="s">
+        <v>563</v>
+      </c>
+      <c r="B111" s="5" t="s">
         <v>564</v>
       </c>
-      <c r="B111" s="5" t="s">
-        <v>565</v>
-      </c>
       <c r="C111" s="5" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E111" s="5"/>
       <c r="F111" s="5" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="G111" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H111" s="11"/>
       <c r="I111" s="11" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="J111" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6247,16 +6246,16 @@
     </row>
     <row r="112" spans="1:10">
       <c r="A112" t="s">
+        <v>567</v>
+      </c>
+      <c r="B112" t="s">
         <v>568</v>
       </c>
-      <c r="B112" t="s">
-        <v>569</v>
-      </c>
       <c r="C112" s="25" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="D112" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E112" s="5"/>
       <c r="F112" s="5"/>
@@ -6270,29 +6269,29 @@
     </row>
     <row r="113" spans="1:10">
       <c r="A113" s="8" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B113" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D113" s="8" t="s">
         <v>27</v>
       </c>
       <c r="E113" s="8"/>
       <c r="F113" s="8" t="s">
+        <v>571</v>
+      </c>
+      <c r="G113" s="8" t="s">
         <v>572</v>
       </c>
-      <c r="G113" s="8" t="s">
+      <c r="H113" s="8" t="s">
         <v>573</v>
       </c>
-      <c r="H113" s="8" t="s">
+      <c r="I113" s="8" t="s">
         <v>574</v>
-      </c>
-      <c r="I113" s="8" t="s">
-        <v>575</v>
       </c>
       <c r="J113" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6301,14 +6300,14 @@
     </row>
     <row r="114" spans="1:10">
       <c r="A114" s="8" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B114" s="8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C114" s="24"/>
       <c r="D114" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E114" s="8" t="s">
         <v>42</v>
@@ -6316,10 +6315,10 @@
       <c r="F114" s="8"/>
       <c r="G114" s="8"/>
       <c r="H114" s="8" t="s">
+        <v>576</v>
+      </c>
+      <c r="I114" s="8" t="s">
         <v>577</v>
-      </c>
-      <c r="I114" s="8" t="s">
-        <v>578</v>
       </c>
       <c r="J114" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6328,13 +6327,13 @@
     </row>
     <row r="115" spans="1:10">
       <c r="A115" s="5" t="s">
+        <v>578</v>
+      </c>
+      <c r="B115" s="5" t="s">
         <v>579</v>
       </c>
-      <c r="B115" s="5" t="s">
+      <c r="C115" s="20" t="s">
         <v>580</v>
-      </c>
-      <c r="C115" s="20" t="s">
-        <v>581</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>83</v>
@@ -6343,13 +6342,13 @@
         <v>84</v>
       </c>
       <c r="G115" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H115" s="5" t="s">
+        <v>581</v>
+      </c>
+      <c r="I115" s="5" t="s">
         <v>582</v>
-      </c>
-      <c r="I115" s="5" t="s">
-        <v>583</v>
       </c>
       <c r="J115" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6358,25 +6357,25 @@
     </row>
     <row r="116" spans="1:10">
       <c r="A116" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="B116" s="5" t="s">
         <v>584</v>
       </c>
-      <c r="B116" s="5" t="s">
-        <v>585</v>
-      </c>
       <c r="C116" s="20" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="D116" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E116" s="5"/>
       <c r="F116" s="5"/>
       <c r="G116" s="5" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H116" s="5"/>
       <c r="I116" s="13" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J116" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6385,31 +6384,31 @@
     </row>
     <row r="117" spans="1:10">
       <c r="A117" s="11" t="s">
+        <v>586</v>
+      </c>
+      <c r="B117" s="11" t="s">
         <v>587</v>
       </c>
-      <c r="B117" s="11" t="s">
+      <c r="C117" s="22" t="s">
         <v>588</v>
       </c>
-      <c r="C117" s="22" t="s">
+      <c r="D117" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="E117" t="s">
         <v>589</v>
       </c>
-      <c r="D117" s="11" t="s">
-        <v>289</v>
-      </c>
-      <c r="E117" t="s">
+      <c r="F117" s="11" t="s">
         <v>590</v>
       </c>
-      <c r="F117" s="11" t="s">
+      <c r="G117" s="11" t="s">
+        <v>661</v>
+      </c>
+      <c r="H117" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="G117" s="11" t="s">
-        <v>662</v>
-      </c>
-      <c r="H117" s="11" t="s">
+      <c r="I117" s="11" t="s">
         <v>592</v>
-      </c>
-      <c r="I117" s="11" t="s">
-        <v>593</v>
       </c>
       <c r="J117" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6418,29 +6417,29 @@
     </row>
     <row r="118" spans="1:10">
       <c r="A118" s="7" t="s">
+        <v>593</v>
+      </c>
+      <c r="B118" s="7" t="s">
+        <v>483</v>
+      </c>
+      <c r="C118" s="7" t="s">
         <v>594</v>
-      </c>
-      <c r="B118" s="7" t="s">
-        <v>484</v>
-      </c>
-      <c r="C118" s="7" t="s">
-        <v>595</v>
       </c>
       <c r="D118" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E118" s="7"/>
       <c r="F118" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="G118" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="G118" s="7" t="s">
-        <v>137</v>
-      </c>
       <c r="H118" s="7" t="s">
+        <v>595</v>
+      </c>
+      <c r="I118" s="7" t="s">
         <v>596</v>
-      </c>
-      <c r="I118" s="7" t="s">
-        <v>597</v>
       </c>
       <c r="J118" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6449,27 +6448,27 @@
     </row>
     <row r="119" spans="1:10">
       <c r="A119" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="B119" s="7" t="s">
         <v>598</v>
       </c>
-      <c r="B119" s="7" t="s">
-        <v>599</v>
-      </c>
       <c r="C119" s="7" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="D119" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E119" s="7"/>
       <c r="F119" s="7"/>
       <c r="G119" s="7" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H119" t="s">
+        <v>599</v>
+      </c>
+      <c r="I119" s="14" t="s">
         <v>600</v>
-      </c>
-      <c r="I119" s="14" t="s">
-        <v>601</v>
       </c>
       <c r="J119" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6478,29 +6477,29 @@
     </row>
     <row r="120" spans="1:10">
       <c r="A120" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="B120" s="5" t="s">
         <v>602</v>
       </c>
-      <c r="B120" s="5" t="s">
-        <v>603</v>
-      </c>
       <c r="C120" s="5" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="D120" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E120" s="5"/>
       <c r="F120" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="G120" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="H120" s="5" t="s">
         <v>604</v>
       </c>
-      <c r="G120" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="H120" s="5" t="s">
+      <c r="I120" s="5" t="s">
         <v>605</v>
-      </c>
-      <c r="I120" s="5" t="s">
-        <v>606</v>
       </c>
       <c r="J120" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6509,27 +6508,27 @@
     </row>
     <row r="121" spans="1:10">
       <c r="A121" s="5" t="s">
+        <v>606</v>
+      </c>
+      <c r="B121" s="5" t="s">
         <v>607</v>
       </c>
-      <c r="B121" s="5" t="s">
-        <v>608</v>
-      </c>
       <c r="C121" s="5" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D121" s="5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E121" s="5"/>
       <c r="F121" s="5"/>
       <c r="G121" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="H121" s="7" t="s">
         <v>431</v>
       </c>
-      <c r="H121" s="7" t="s">
-        <v>432</v>
-      </c>
       <c r="I121" s="13" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="J121" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6538,25 +6537,25 @@
     </row>
     <row r="122" spans="1:10">
       <c r="A122" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B122" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D122" t="s">
         <v>49</v>
       </c>
       <c r="F122" s="27" t="s">
+        <v>610</v>
+      </c>
+      <c r="G122" t="s">
+        <v>307</v>
+      </c>
+      <c r="H122" s="7" t="s">
         <v>611</v>
       </c>
-      <c r="G122" t="s">
-        <v>308</v>
-      </c>
-      <c r="H122" s="7" t="s">
+      <c r="I122" s="15" t="s">
         <v>612</v>
-      </c>
-      <c r="I122" s="15" t="s">
-        <v>613</v>
       </c>
       <c r="J122" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6565,31 +6564,31 @@
     </row>
     <row r="123" spans="1:10">
       <c r="A123" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B123" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="D123" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E123" s="5" t="s">
         <v>42</v>
       </c>
       <c r="F123" s="27" t="s">
+        <v>645</v>
+      </c>
+      <c r="G123" t="s">
+        <v>663</v>
+      </c>
+      <c r="H123" t="s">
         <v>646</v>
       </c>
-      <c r="G123" t="s">
-        <v>664</v>
-      </c>
-      <c r="H123" t="s">
+      <c r="I123" s="21" t="s">
         <v>647</v>
-      </c>
-      <c r="I123" s="21" t="s">
-        <v>648</v>
       </c>
       <c r="J123" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6598,14 +6597,14 @@
     </row>
     <row r="124" spans="1:10">
       <c r="A124" s="5" t="s">
+        <v>613</v>
+      </c>
+      <c r="B124" s="5" t="s">
         <v>614</v>
-      </c>
-      <c r="B124" s="5" t="s">
-        <v>615</v>
       </c>
       <c r="C124" s="20"/>
       <c r="D124" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E124" s="5"/>
       <c r="F124" s="5"/>
@@ -6613,10 +6612,10 @@
         <v>57</v>
       </c>
       <c r="H124" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="I124" s="13" t="s">
         <v>616</v>
-      </c>
-      <c r="I124" s="13" t="s">
-        <v>617</v>
       </c>
       <c r="J124" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6625,29 +6624,29 @@
     </row>
     <row r="125" spans="1:10">
       <c r="A125" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="B125" s="5" t="s">
         <v>618</v>
       </c>
-      <c r="B125" s="5" t="s">
-        <v>619</v>
-      </c>
       <c r="C125" s="22" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E125" s="5"/>
       <c r="F125" s="5" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="G125" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H125" s="5" t="s">
+        <v>620</v>
+      </c>
+      <c r="I125" s="13" t="s">
         <v>621</v>
-      </c>
-      <c r="I125" s="13" t="s">
-        <v>622</v>
       </c>
       <c r="J125" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6656,16 +6655,16 @@
     </row>
     <row r="126" spans="1:10">
       <c r="A126" s="5" t="s">
+        <v>622</v>
+      </c>
+      <c r="B126" s="5" t="s">
         <v>623</v>
       </c>
-      <c r="B126" s="5" t="s">
-        <v>624</v>
-      </c>
       <c r="C126" s="5" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="D126" s="5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E126" s="5"/>
       <c r="F126" s="5"/>
@@ -6673,10 +6672,10 @@
         <v>57</v>
       </c>
       <c r="H126" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="I126" s="13" t="s">
         <v>625</v>
-      </c>
-      <c r="I126" s="13" t="s">
-        <v>626</v>
       </c>
       <c r="J126" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6685,29 +6684,29 @@
     </row>
     <row r="127" spans="1:10">
       <c r="A127" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="B127" s="5" t="s">
         <v>627</v>
       </c>
-      <c r="B127" s="5" t="s">
+      <c r="C127" s="5" t="s">
         <v>628</v>
-      </c>
-      <c r="C127" s="5" t="s">
-        <v>629</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>27</v>
       </c>
       <c r="E127" s="5" t="s">
+        <v>629</v>
+      </c>
+      <c r="F127" s="5" t="s">
         <v>630</v>
       </c>
-      <c r="F127" s="5" t="s">
-        <v>631</v>
-      </c>
       <c r="G127" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H127" s="5"/>
       <c r="I127" s="5" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="J127" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6716,27 +6715,27 @@
     </row>
     <row r="128" spans="1:10">
       <c r="A128" s="5" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E128" s="5"/>
       <c r="F128" s="5"/>
       <c r="G128" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H128" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="I128" s="13" t="s">
         <v>634</v>
-      </c>
-      <c r="I128" s="13" t="s">
-        <v>635</v>
       </c>
       <c r="J128" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6745,10 +6744,10 @@
     </row>
     <row r="129" spans="1:10">
       <c r="A129" s="7" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B129" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C129" s="7"/>
       <c r="D129" s="7" t="s">
@@ -6758,16 +6757,16 @@
         <v>76</v>
       </c>
       <c r="F129" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="G129" t="s">
+        <v>453</v>
+      </c>
+      <c r="H129" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="I129" s="7" t="s">
         <v>637</v>
-      </c>
-      <c r="G129" t="s">
-        <v>454</v>
-      </c>
-      <c r="H129" s="7" t="s">
-        <v>475</v>
-      </c>
-      <c r="I129" s="7" t="s">
-        <v>638</v>
       </c>
       <c r="J129" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6776,29 +6775,29 @@
     </row>
     <row r="130" spans="1:10">
       <c r="A130" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B130" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="D130" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E130" s="5"/>
       <c r="F130" s="8" t="s">
+        <v>571</v>
+      </c>
+      <c r="G130" t="s">
         <v>572</v>
       </c>
-      <c r="G130" t="s">
-        <v>573</v>
-      </c>
       <c r="H130" t="s">
+        <v>714</v>
+      </c>
+      <c r="I130" s="21" t="s">
         <v>715</v>
-      </c>
-      <c r="I130" s="21" t="s">
-        <v>716</v>
       </c>
       <c r="J130" s="10" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7054,15 +7053,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7071,6 +7061,15 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7093,14 +7092,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7115,4 +7106,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Mise à jour des informations concernant Tara Landry
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{164F3723-9DA3-4991-ADE5-82C3F29822C0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D7C157-F2C2-4C6C-85FD-9342F1811124}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19460" yWindow="4650" windowWidth="20480" windowHeight="23450" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="733">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="732">
   <si>
     <t>nom</t>
   </si>
@@ -1965,9 +1965,6 @@
   </si>
   <si>
     <t>isabelle.lagadec@umontreal.ca</t>
-  </si>
-  <si>
-    <t>Directrice (interim)</t>
   </si>
   <si>
     <t>Bibliothèque Hubert-Reeves;Bibliothèque de kinésiologie;Bibliothèque Marguerite-d'Youville;Bibliothèque du Parc;Bibliothèque de la santé;Bibliothèque de mathématiques et informatiques</t>
@@ -2994,7 +2991,7 @@
         <v>42</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>21</v>
@@ -3092,7 +3089,7 @@
         <v>43</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>44</v>
@@ -3138,13 +3135,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B8" t="s">
         <v>516</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="D8" t="s">
         <v>95</v>
@@ -3153,16 +3150,16 @@
         <v>15</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
       </c>
       <c r="H8" t="s">
+        <v>657</v>
+      </c>
+      <c r="I8" s="20" t="s">
         <v>658</v>
-      </c>
-      <c r="I8" s="20" t="s">
-        <v>659</v>
       </c>
       <c r="J8" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3247,7 +3244,7 @@
         <v>571</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>72</v>
@@ -3268,7 +3265,7 @@
         <v>39</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>75</v>
@@ -3361,7 +3358,7 @@
         <v>94</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>95</v>
@@ -3390,7 +3387,7 @@
         <v>104</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="D16" t="s">
         <v>95</v>
@@ -3625,7 +3622,7 @@
         <v>146</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>147</v>
@@ -3634,10 +3631,10 @@
         <v>76</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>148</v>
@@ -3658,7 +3655,7 @@
         <v>151</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>49</v>
@@ -3668,7 +3665,7 @@
         <v>152</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>153</v>
@@ -3711,13 +3708,13 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
+        <v>726</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>727</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>728</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>729</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>13</v>
@@ -3726,16 +3723,16 @@
         <v>128</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="G27" t="s">
         <v>15</v>
       </c>
       <c r="H27" s="6" t="s">
+        <v>730</v>
+      </c>
+      <c r="I27" s="8" t="s">
         <v>731</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>732</v>
       </c>
       <c r="J27" s="29" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3750,7 +3747,7 @@
         <v>161</v>
       </c>
       <c r="C28" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D28" t="s">
         <v>95</v>
@@ -3777,7 +3774,7 @@
         <v>165</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>166</v>
@@ -3808,7 +3805,7 @@
         <v>172</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>49</v>
@@ -3870,7 +3867,7 @@
         <v>184</v>
       </c>
       <c r="C32" s="24" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="D32" t="s">
         <v>27</v>
@@ -3897,7 +3894,7 @@
         <v>49</v>
       </c>
       <c r="G33" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>187</v>
@@ -3925,13 +3922,13 @@
         <v>63</v>
       </c>
       <c r="G34" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="H34" s="10" t="s">
         <v>710</v>
       </c>
-      <c r="H34" s="10" t="s">
+      <c r="I34" s="9" t="s">
         <v>711</v>
-      </c>
-      <c r="I34" s="9" t="s">
-        <v>712</v>
       </c>
       <c r="J34" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4007,7 +4004,7 @@
         <v>206</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>27</v>
@@ -4050,7 +4047,7 @@
         <v>215</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="H38" s="5" t="s">
         <v>216</v>
@@ -4102,7 +4099,7 @@
         <v>225</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>13</v>
@@ -4205,7 +4202,7 @@
         <v>246</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>247</v>
@@ -4257,7 +4254,7 @@
         <v>256</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>257</v>
@@ -4286,7 +4283,7 @@
         <v>262</v>
       </c>
       <c r="C46" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="D46" t="s">
         <v>95</v>
@@ -4338,10 +4335,10 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
+        <v>721</v>
+      </c>
+      <c r="B48" s="5" t="s">
         <v>722</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>723</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5" t="s">
@@ -4351,16 +4348,16 @@
         <v>128</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G48" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H48" s="5" t="s">
+        <v>724</v>
+      </c>
+      <c r="I48" s="9" t="s">
         <v>725</v>
-      </c>
-      <c r="I48" s="9" t="s">
-        <v>726</v>
       </c>
       <c r="J48" s="29" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4375,7 +4372,7 @@
         <v>272</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="D49" t="s">
         <v>95</v>
@@ -4438,7 +4435,7 @@
         <v>277</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="E51" s="5" t="s">
         <v>128</v>
@@ -4559,7 +4556,7 @@
         <v>299</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>300</v>
@@ -4732,7 +4729,7 @@
         <v>328</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>27</v>
@@ -4892,7 +4889,7 @@
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="G66" s="5" t="s">
         <v>29</v>
@@ -4916,7 +4913,7 @@
         <v>360</v>
       </c>
       <c r="C67" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="D67" t="s">
         <v>49</v>
@@ -4972,7 +4969,7 @@
         <v>104</v>
       </c>
       <c r="C69" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="D69" t="s">
         <v>95</v>
@@ -5011,7 +5008,7 @@
         <v>371</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>372</v>
@@ -5035,7 +5032,7 @@
         <v>376</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>639</v>
+        <v>147</v>
       </c>
       <c r="E71" s="5" t="s">
         <v>128</v>
@@ -5044,7 +5041,7 @@
         <v>43</v>
       </c>
       <c r="G71" s="6" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="H71" s="5" t="s">
         <v>377</v>
@@ -5065,7 +5062,7 @@
         <v>311</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D72" s="6" t="s">
         <v>41</v>
@@ -5098,7 +5095,7 @@
         <v>384</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D73" t="s">
         <v>95</v>
@@ -5132,7 +5129,7 @@
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="6" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="G74" s="6" t="s">
         <v>29</v>
@@ -5156,7 +5153,7 @@
         <v>393</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>27</v>
@@ -5229,7 +5226,7 @@
         <v>405</v>
       </c>
       <c r="G77" s="6" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="H77" s="5" t="s">
         <v>406</v>
@@ -5250,7 +5247,7 @@
         <v>409</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="D78" s="6" t="s">
         <v>147</v>
@@ -5311,7 +5308,7 @@
         <v>418</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="D80" s="7" t="s">
         <v>41</v>
@@ -5320,10 +5317,10 @@
         <v>42</v>
       </c>
       <c r="F80" s="26" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="G80" s="7" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="H80" s="7" t="s">
         <v>419</v>
@@ -5344,7 +5341,7 @@
         <v>421</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>95</v>
@@ -5370,7 +5367,7 @@
         <v>424</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>425</v>
@@ -5399,7 +5396,7 @@
         <v>429</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>425</v>
@@ -5428,7 +5425,7 @@
         <v>434</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>435</v>
@@ -5466,7 +5463,7 @@
       </c>
       <c r="E85" s="5"/>
       <c r="F85" s="5" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="G85" s="5" t="s">
         <v>29</v>
@@ -5551,7 +5548,7 @@
         <v>457</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>425</v>
@@ -5704,7 +5701,7 @@
         <v>483</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="D93" s="6" t="s">
         <v>27</v>
@@ -5735,7 +5732,7 @@
         <v>488</v>
       </c>
       <c r="C94" s="10" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="D94" s="10" t="s">
         <v>238</v>
@@ -5745,7 +5742,7 @@
       </c>
       <c r="F94" s="28"/>
       <c r="G94" s="10" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="H94" s="10" t="s">
         <v>489</v>
@@ -5766,7 +5763,7 @@
         <v>492</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="D95" s="6" t="s">
         <v>493</v>
@@ -5824,7 +5821,7 @@
         <v>502</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D97" s="6" t="s">
         <v>41</v>
@@ -5912,7 +5909,7 @@
         <v>516</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>110</v>
@@ -5952,7 +5949,7 @@
       </c>
       <c r="E101" s="6"/>
       <c r="F101" s="6" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="G101" s="6" t="s">
         <v>29</v>
@@ -5976,7 +5973,7 @@
         <v>521</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>13</v>
@@ -6097,7 +6094,7 @@
         <v>544</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="D106" s="6" t="s">
         <v>95</v>
@@ -6126,13 +6123,13 @@
         <v>548</v>
       </c>
       <c r="C107" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="D107" t="s">
         <v>425</v>
       </c>
       <c r="G107" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="H107" s="6" t="s">
         <v>549</v>
@@ -6172,13 +6169,13 @@
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
+        <v>707</v>
+      </c>
+      <c r="B109" t="s">
         <v>708</v>
       </c>
-      <c r="B109" t="s">
-        <v>709</v>
-      </c>
       <c r="C109" s="5" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="D109" t="s">
         <v>95</v>
@@ -6191,10 +6188,10 @@
         <v>572</v>
       </c>
       <c r="H109" t="s">
+        <v>710</v>
+      </c>
+      <c r="I109" s="20" t="s">
         <v>711</v>
-      </c>
-      <c r="I109" s="20" t="s">
-        <v>712</v>
       </c>
       <c r="J109" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6267,7 +6264,7 @@
         <v>564</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>13</v>
@@ -6296,7 +6293,7 @@
         <v>568</v>
       </c>
       <c r="C113" s="24" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>257</v>
@@ -6401,13 +6398,13 @@
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B117" t="s">
         <v>614</v>
       </c>
       <c r="C117" s="19" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="D117" t="s">
         <v>95</v>
@@ -6420,10 +6417,10 @@
         <v>572</v>
       </c>
       <c r="H117" t="s">
+        <v>713</v>
+      </c>
+      <c r="I117" s="20" t="s">
         <v>714</v>
-      </c>
-      <c r="I117" s="20" t="s">
-        <v>715</v>
       </c>
       <c r="J117" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6438,7 +6435,7 @@
         <v>584</v>
       </c>
       <c r="C118" s="21" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>95</v>
@@ -6477,7 +6474,7 @@
         <v>590</v>
       </c>
       <c r="G119" s="10" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H119" s="10" t="s">
         <v>591</v>
@@ -6529,7 +6526,7 @@
         <v>598</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="D121" s="6" t="s">
         <v>95</v>
@@ -6558,7 +6555,7 @@
         <v>602</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>110</v>
@@ -6589,7 +6586,7 @@
         <v>607</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>425</v>
@@ -6639,13 +6636,13 @@
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B125" t="s">
         <v>502</v>
       </c>
       <c r="C125" s="19" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="D125" t="s">
         <v>147</v>
@@ -6654,16 +6651,16 @@
         <v>42</v>
       </c>
       <c r="F125" s="26" t="s">
+        <v>644</v>
+      </c>
+      <c r="G125" t="s">
+        <v>662</v>
+      </c>
+      <c r="H125" t="s">
         <v>645</v>
       </c>
-      <c r="G125" t="s">
-        <v>663</v>
-      </c>
-      <c r="H125" t="s">
+      <c r="I125" s="20" t="s">
         <v>646</v>
-      </c>
-      <c r="I125" s="20" t="s">
-        <v>647</v>
       </c>
       <c r="J125" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6705,7 +6702,7 @@
         <v>618</v>
       </c>
       <c r="C127" s="21" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>95</v>
@@ -6736,7 +6733,7 @@
         <v>623</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>425</v>
@@ -6796,7 +6793,7 @@
         <v>618</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="D130" s="5" t="s">
         <v>95</v>
@@ -7098,15 +7095,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7115,6 +7103,15 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7137,14 +7134,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7159,4 +7148,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Ajout de Sosthène dans le répertoire
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D7C157-F2C2-4C6C-85FD-9342F1811124}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6798BC22-21B2-4139-9A6C-461FA7869724}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19460" yWindow="4650" windowWidth="20480" windowHeight="23450" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19455" yWindow="4650" windowWidth="20475" windowHeight="23445" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="732">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="736">
   <si>
     <t>nom</t>
   </si>
@@ -1937,9 +1937,6 @@
     <t>marie-helene-vezina.jpg</t>
   </si>
   <si>
-    <t>Direction de la recherche et des initiatives numériques;</t>
-  </si>
-  <si>
     <t>Exploitation et visualisation des données</t>
   </si>
   <si>
@@ -2244,6 +2241,21 @@
   </si>
   <si>
     <t>tanya.buchet@umontreal.ca</t>
+  </si>
+  <si>
+    <t>Yamalé</t>
+  </si>
+  <si>
+    <t>Sosthène</t>
+  </si>
+  <si>
+    <t>Administrateur de systèmes</t>
+  </si>
+  <si>
+    <t>514 353-6000, poste 1617</t>
+  </si>
+  <si>
+    <t>sosthene.yamale@umontreal.ca</t>
   </si>
 </sst>
 </file>
@@ -2552,10 +2564,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J131" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:J131" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
-  <sortState ref="A2:J131">
-    <sortCondition ref="A1:A131"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J132" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:J132" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
+  <sortState ref="A2:J132">
+    <sortCondition ref="A1:A132"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{4B04E1AF-0079-4AD2-81CA-E8A433733E21}" name="nom"/>
@@ -2896,22 +2908,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J131"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J132"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.453125" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="25.90625" customWidth="1"/>
-    <col min="4" max="4" width="28.1796875" customWidth="1"/>
-    <col min="5" max="5" width="58.08984375" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" customWidth="1"/>
+    <col min="5" max="5" width="58.140625" customWidth="1"/>
     <col min="6" max="6" width="58" style="26" customWidth="1"/>
-    <col min="7" max="7" width="70.81640625" customWidth="1"/>
-    <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="41.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.1796875" customWidth="1"/>
+    <col min="7" max="7" width="70.85546875" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="86.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2943,7 +2955,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
@@ -2974,7 +2986,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alexandre.amar-zifkin@umontreal.ca</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -2991,7 +3003,7 @@
         <v>42</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>21</v>
@@ -3007,7 +3019,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.angers@umontreal.ca</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>24</v>
       </c>
@@ -3038,7 +3050,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nadege.arsa@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>32</v>
       </c>
@@ -3069,7 +3081,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=denis.arvisais@umontreal.ca</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>38</v>
       </c>
@@ -3089,7 +3101,7 @@
         <v>43</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>44</v>
@@ -3102,7 +3114,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.attia@umontreal.ca</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>46</v>
       </c>
@@ -3133,15 +3145,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=prlaval@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B8" t="s">
         <v>516</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D8" t="s">
         <v>95</v>
@@ -3150,23 +3162,23 @@
         <v>15</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
       </c>
       <c r="H8" t="s">
+        <v>656</v>
+      </c>
+      <c r="I8" s="20" t="s">
         <v>657</v>
       </c>
-      <c r="I8" s="20" t="s">
-        <v>658</v>
-      </c>
       <c r="J8" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=eve.baribeau.marchand@umontreal.ca</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>53</v>
       </c>
@@ -3196,7 +3208,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.bastien@umontreal.ca</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>60</v>
       </c>
@@ -3224,7 +3236,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magalie.beaudoin@umontreal.ca</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>67</v>
       </c>
@@ -3244,7 +3256,7 @@
         <v>571</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>72</v>
@@ -3257,7 +3269,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maryna.beaulieu@umontreal.ca</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>74</v>
       </c>
@@ -3265,7 +3277,7 @@
         <v>39</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>75</v>
@@ -3287,7 +3299,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.begin-poissant@umontreal.ca</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>80</v>
       </c>
@@ -3317,7 +3329,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.belanger@umontreal.ca</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>88</v>
       </c>
@@ -3350,7 +3362,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amy.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>93</v>
       </c>
@@ -3358,7 +3370,7 @@
         <v>94</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>95</v>
@@ -3379,7 +3391,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amelie.bernard@umontreal.ca</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>99</v>
       </c>
@@ -3387,7 +3399,7 @@
         <v>104</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D16" t="s">
         <v>95</v>
@@ -3406,7 +3418,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>99</v>
       </c>
@@ -3435,7 +3447,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=hugo.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>107</v>
       </c>
@@ -3466,7 +3478,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon.blais.longtin@umontreal.ca</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>113</v>
       </c>
@@ -3496,7 +3508,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tatiana.talpa@umontreal.ca</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>119</v>
       </c>
@@ -3522,7 +3534,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=joanna.bodnar@umontreal.ca</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>124</v>
       </c>
@@ -3552,7 +3564,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alain.borsi@umontreal.ca</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>132</v>
       </c>
@@ -3583,7 +3595,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.p.bouchard@umontreal.ca</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>139</v>
       </c>
@@ -3614,7 +3626,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refdroi@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>145</v>
       </c>
@@ -3622,7 +3634,7 @@
         <v>146</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>147</v>
@@ -3631,10 +3643,10 @@
         <v>76</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>148</v>
@@ -3647,7 +3659,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=myriam.boyer@umontreal.ca</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>150</v>
       </c>
@@ -3655,7 +3667,7 @@
         <v>151</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>49</v>
@@ -3665,7 +3677,7 @@
         <v>152</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>153</v>
@@ -3678,7 +3690,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guylaine.brazeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>155</v>
       </c>
@@ -3706,15 +3718,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sophie.brisebois@umontreal.ca</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
+        <v>725</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>726</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>727</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>728</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>13</v>
@@ -3723,23 +3735,23 @@
         <v>128</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="G27" t="s">
         <v>15</v>
       </c>
       <c r="H27" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="I27" s="8" t="s">
         <v>730</v>
       </c>
-      <c r="I27" s="8" t="s">
-        <v>731</v>
-      </c>
       <c r="J27" s="29" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=tanya.buchet@umontreal.ca</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>160</v>
       </c>
@@ -3747,7 +3759,7 @@
         <v>161</v>
       </c>
       <c r="C28" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="D28" t="s">
         <v>95</v>
@@ -3766,7 +3778,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fanny.c.brochu@umontreal.ca</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>164</v>
       </c>
@@ -3774,7 +3786,7 @@
         <v>165</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>166</v>
@@ -3797,7 +3809,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=delphine.cado@umontreal.ca</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>171</v>
       </c>
@@ -3805,7 +3817,7 @@
         <v>172</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>49</v>
@@ -3828,7 +3840,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=siv.kham.chao@umontreal.ca</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>177</v>
       </c>
@@ -3859,7 +3871,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=laurence.charest@umontreal.ca</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>183</v>
       </c>
@@ -3867,7 +3879,7 @@
         <v>184</v>
       </c>
       <c r="C32" s="24" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="D32" t="s">
         <v>27</v>
@@ -3883,7 +3895,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>185</v>
       </c>
@@ -3894,7 +3906,7 @@
         <v>49</v>
       </c>
       <c r="G33" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>187</v>
@@ -3907,7 +3919,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=annick.charette@umontreal.ca</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>189</v>
       </c>
@@ -3922,20 +3934,20 @@
         <v>63</v>
       </c>
       <c r="G34" s="5" t="s">
+        <v>708</v>
+      </c>
+      <c r="H34" s="10" t="s">
         <v>709</v>
       </c>
-      <c r="H34" s="10" t="s">
+      <c r="I34" s="9" t="s">
         <v>710</v>
       </c>
-      <c r="I34" s="9" t="s">
-        <v>711</v>
-      </c>
       <c r="J34" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>192</v>
       </c>
@@ -3966,7 +3978,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah.cherrier@umontreal.ca</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>198</v>
       </c>
@@ -3996,7 +4008,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emir.chouchane@umontreal.ca</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>205</v>
       </c>
@@ -4004,7 +4016,7 @@
         <v>206</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>27</v>
@@ -4027,7 +4039,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=accessibilite@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>210</v>
       </c>
@@ -4047,7 +4059,7 @@
         <v>215</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="H38" s="5" t="s">
         <v>216</v>
@@ -4060,7 +4072,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benjamin.constantineau@umontreal.ca</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>218</v>
       </c>
@@ -4091,7 +4103,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon-pierre.crevier@umontreal.ca</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>224</v>
       </c>
@@ -4099,7 +4111,7 @@
         <v>225</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>13</v>
@@ -4122,7 +4134,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marc-olivier.croteau@umontreal.ca</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>229</v>
       </c>
@@ -4153,7 +4165,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.dalpe@umontreal.ca</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>235</v>
       </c>
@@ -4184,7 +4196,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=morgane.de.bellefeuille@umontreal.ca</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>243</v>
       </c>
@@ -4202,7 +4214,7 @@
         <v>246</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>247</v>
@@ -4215,7 +4227,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=Indiana.delsart@umontreal.ca</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>249</v>
       </c>
@@ -4246,7 +4258,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=dominic.desaulniers@umontreal.ca</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>255</v>
       </c>
@@ -4254,7 +4266,7 @@
         <v>256</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>257</v>
@@ -4275,7 +4287,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.desrosiers@umontreal.ca</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>261</v>
       </c>
@@ -4283,7 +4295,7 @@
         <v>262</v>
       </c>
       <c r="C46" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="D46" t="s">
         <v>95</v>
@@ -4302,7 +4314,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.dubois.mercier@umontreal.ca</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>265</v>
       </c>
@@ -4333,12 +4345,12 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jean-francois.durnin@umontreal.ca</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
+        <v>720</v>
+      </c>
+      <c r="B48" s="5" t="s">
         <v>721</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>722</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5" t="s">
@@ -4348,23 +4360,23 @@
         <v>128</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G48" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H48" s="5" t="s">
+        <v>723</v>
+      </c>
+      <c r="I48" s="9" t="s">
         <v>724</v>
       </c>
-      <c r="I48" s="9" t="s">
-        <v>725</v>
-      </c>
       <c r="J48" s="29" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=taline.ekmekjian@umontreal.ca</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>271</v>
       </c>
@@ -4372,7 +4384,7 @@
         <v>272</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="D49" t="s">
         <v>95</v>
@@ -4391,7 +4403,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=judith.fafard-larose@umontreal.ca</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>275</v>
       </c>
@@ -4424,7 +4436,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>275</v>
       </c>
@@ -4435,7 +4447,7 @@
         <v>277</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="E51" s="5" t="s">
         <v>128</v>
@@ -4455,7 +4467,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>280</v>
       </c>
@@ -4488,7 +4500,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=c.fortier@umontreal.ca</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>286</v>
       </c>
@@ -4517,7 +4529,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>292</v>
       </c>
@@ -4548,7 +4560,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nino.gabrielli@umontreal.ca</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>298</v>
       </c>
@@ -4556,7 +4568,7 @@
         <v>299</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>300</v>
@@ -4577,7 +4589,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-pierre.gadoua@umontreal.ca</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>303</v>
       </c>
@@ -4608,7 +4620,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cynthia.gagne.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>310</v>
       </c>
@@ -4636,7 +4648,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
         <v>310</v>
       </c>
@@ -4662,7 +4674,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>317</v>
       </c>
@@ -4692,7 +4704,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marjorie.gauchier@umontreal.ca</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
         <v>323</v>
       </c>
@@ -4721,7 +4733,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>327</v>
       </c>
@@ -4729,7 +4741,7 @@
         <v>328</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>27</v>
@@ -4752,7 +4764,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
         <v>332</v>
       </c>
@@ -4783,7 +4795,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>337</v>
       </c>
@@ -4814,7 +4826,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
       </c>
     </row>
-    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>343</v>
       </c>
@@ -4845,7 +4857,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>349</v>
       </c>
@@ -4874,7 +4886,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
       </c>
     </row>
-    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>354</v>
       </c>
@@ -4889,7 +4901,7 @@
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="G66" s="5" t="s">
         <v>29</v>
@@ -4905,7 +4917,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>359</v>
       </c>
@@ -4913,7 +4925,7 @@
         <v>360</v>
       </c>
       <c r="C67" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="D67" t="s">
         <v>49</v>
@@ -4932,7 +4944,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>363</v>
       </c>
@@ -4954,14 +4966,14 @@
         <v>364</v>
       </c>
       <c r="I68" s="8" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="J68" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>365</v>
       </c>
@@ -4969,7 +4981,7 @@
         <v>104</v>
       </c>
       <c r="C69" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="D69" t="s">
         <v>95</v>
@@ -4988,7 +5000,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>368</v>
       </c>
@@ -5008,7 +5020,7 @@
         <v>371</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>372</v>
@@ -5021,7 +5033,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
         <v>374</v>
       </c>
@@ -5054,7 +5066,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>379</v>
       </c>
@@ -5062,7 +5074,7 @@
         <v>311</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D72" s="6" t="s">
         <v>41</v>
@@ -5087,7 +5099,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>383</v>
       </c>
@@ -5095,7 +5107,7 @@
         <v>384</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D73" t="s">
         <v>95</v>
@@ -5114,7 +5126,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>387</v>
       </c>
@@ -5129,7 +5141,7 @@
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="6" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="G74" s="6" t="s">
         <v>29</v>
@@ -5145,7 +5157,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
       </c>
     </row>
-    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>392</v>
       </c>
@@ -5153,7 +5165,7 @@
         <v>393</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>27</v>
@@ -5176,7 +5188,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>397</v>
       </c>
@@ -5206,7 +5218,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
         <v>402</v>
       </c>
@@ -5226,7 +5238,7 @@
         <v>405</v>
       </c>
       <c r="G77" s="6" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="H77" s="5" t="s">
         <v>406</v>
@@ -5239,7 +5251,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>408</v>
       </c>
@@ -5247,7 +5259,7 @@
         <v>409</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="D78" s="6" t="s">
         <v>147</v>
@@ -5269,7 +5281,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
       </c>
     </row>
-    <row r="79" spans="1:10" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
         <v>412</v>
       </c>
@@ -5300,7 +5312,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="7" t="s">
         <v>417</v>
       </c>
@@ -5308,7 +5320,7 @@
         <v>418</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="D80" s="7" t="s">
         <v>41</v>
@@ -5317,10 +5329,10 @@
         <v>42</v>
       </c>
       <c r="F80" s="26" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="G80" s="7" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="H80" s="7" t="s">
         <v>419</v>
@@ -5333,7 +5345,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
         <v>417</v>
       </c>
@@ -5341,7 +5353,7 @@
         <v>421</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>95</v>
@@ -5359,7 +5371,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
         <v>423</v>
       </c>
@@ -5367,7 +5379,7 @@
         <v>424</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>425</v>
@@ -5388,7 +5400,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
         <v>428</v>
       </c>
@@ -5396,7 +5408,7 @@
         <v>429</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>425</v>
@@ -5417,7 +5429,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
         <v>433</v>
       </c>
@@ -5425,7 +5437,7 @@
         <v>434</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>435</v>
@@ -5448,7 +5460,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
         <v>439</v>
       </c>
@@ -5463,7 +5475,7 @@
       </c>
       <c r="E85" s="5"/>
       <c r="F85" s="5" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="G85" s="5" t="s">
         <v>29</v>
@@ -5479,7 +5491,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
         <v>444</v>
       </c>
@@ -5510,7 +5522,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
         <v>450</v>
       </c>
@@ -5540,7 +5552,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
         <v>456</v>
       </c>
@@ -5548,7 +5560,7 @@
         <v>457</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>425</v>
@@ -5569,7 +5581,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
         <v>460</v>
       </c>
@@ -5600,7 +5612,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="10" t="s">
         <v>466</v>
       </c>
@@ -5631,7 +5643,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
         <v>471</v>
       </c>
@@ -5662,7 +5674,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
         <v>476</v>
       </c>
@@ -5693,7 +5705,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=assia.mourid@umontreal.ca</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>482</v>
       </c>
@@ -5701,7 +5713,7 @@
         <v>483</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="D93" s="6" t="s">
         <v>27</v>
@@ -5724,7 +5736,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="10" t="s">
         <v>487</v>
       </c>
@@ -5732,7 +5744,7 @@
         <v>488</v>
       </c>
       <c r="C94" s="10" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="D94" s="10" t="s">
         <v>238</v>
@@ -5742,7 +5754,7 @@
       </c>
       <c r="F94" s="28"/>
       <c r="G94" s="10" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="H94" s="10" t="s">
         <v>489</v>
@@ -5755,7 +5767,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
         <v>491</v>
       </c>
@@ -5763,7 +5775,7 @@
         <v>492</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="D95" s="6" t="s">
         <v>493</v>
@@ -5786,7 +5798,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
       </c>
     </row>
-    <row r="96" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
         <v>497</v>
       </c>
@@ -5813,7 +5825,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
-    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
         <v>501</v>
       </c>
@@ -5821,7 +5833,7 @@
         <v>502</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D97" s="6" t="s">
         <v>41</v>
@@ -5844,7 +5856,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
         <v>505</v>
       </c>
@@ -5871,7 +5883,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>510</v>
       </c>
@@ -5901,7 +5913,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
         <v>515</v>
       </c>
@@ -5909,7 +5921,7 @@
         <v>516</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>110</v>
@@ -5934,7 +5946,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eve.paquette-bigras@umontreal.ca</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
         <v>520</v>
       </c>
@@ -5949,7 +5961,7 @@
       </c>
       <c r="E101" s="6"/>
       <c r="F101" s="6" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="G101" s="6" t="s">
         <v>29</v>
@@ -5965,7 +5977,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
         <v>520</v>
       </c>
@@ -5973,7 +5985,7 @@
         <v>521</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>13</v>
@@ -5996,7 +6008,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
       </c>
     </row>
-    <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
         <v>529</v>
       </c>
@@ -6027,7 +6039,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
       </c>
     </row>
-    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
         <v>533</v>
       </c>
@@ -6055,7 +6067,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="6" t="s">
         <v>537</v>
       </c>
@@ -6086,7 +6098,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="6" t="s">
         <v>543</v>
       </c>
@@ -6094,7 +6106,7 @@
         <v>544</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="D106" s="6" t="s">
         <v>95</v>
@@ -6115,7 +6127,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>547</v>
       </c>
@@ -6123,13 +6135,13 @@
         <v>548</v>
       </c>
       <c r="C107" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="D107" t="s">
         <v>425</v>
       </c>
       <c r="G107" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="H107" s="6" t="s">
         <v>549</v>
@@ -6142,7 +6154,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>551</v>
       </c>
@@ -6167,15 +6179,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
+        <v>706</v>
+      </c>
+      <c r="B109" t="s">
         <v>707</v>
       </c>
-      <c r="B109" t="s">
-        <v>708</v>
-      </c>
       <c r="C109" s="5" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="D109" t="s">
         <v>95</v>
@@ -6188,17 +6200,17 @@
         <v>572</v>
       </c>
       <c r="H109" t="s">
+        <v>709</v>
+      </c>
+      <c r="I109" s="20" t="s">
         <v>710</v>
       </c>
-      <c r="I109" s="20" t="s">
-        <v>711</v>
-      </c>
       <c r="J109" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>555</v>
       </c>
@@ -6228,7 +6240,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
         <v>560</v>
       </c>
@@ -6256,7 +6268,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
         <v>563</v>
       </c>
@@ -6264,7 +6276,7 @@
         <v>564</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>13</v>
@@ -6285,7 +6297,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>567</v>
       </c>
@@ -6293,7 +6305,7 @@
         <v>568</v>
       </c>
       <c r="C113" s="24" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>257</v>
@@ -6308,7 +6320,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" s="7" t="s">
         <v>569</v>
       </c>
@@ -6339,7 +6351,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
         <v>575</v>
       </c>
@@ -6366,7 +6378,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
         <v>578</v>
       </c>
@@ -6396,15 +6408,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B117" t="s">
         <v>614</v>
       </c>
       <c r="C117" s="19" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="D117" t="s">
         <v>95</v>
@@ -6417,17 +6429,17 @@
         <v>572</v>
       </c>
       <c r="H117" t="s">
+        <v>712</v>
+      </c>
+      <c r="I117" s="20" t="s">
         <v>713</v>
       </c>
-      <c r="I117" s="20" t="s">
-        <v>714</v>
-      </c>
       <c r="J117" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
         <v>583</v>
       </c>
@@ -6435,7 +6447,7 @@
         <v>584</v>
       </c>
       <c r="C118" s="21" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>95</v>
@@ -6454,7 +6466,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
         <v>586</v>
       </c>
@@ -6474,7 +6486,7 @@
         <v>590</v>
       </c>
       <c r="G119" s="10" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="H119" s="10" t="s">
         <v>591</v>
@@ -6487,7 +6499,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" s="6" t="s">
         <v>593</v>
       </c>
@@ -6518,7 +6530,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" s="6" t="s">
         <v>597</v>
       </c>
@@ -6526,7 +6538,7 @@
         <v>598</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="D121" s="6" t="s">
         <v>95</v>
@@ -6547,7 +6559,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="s">
         <v>601</v>
       </c>
@@ -6555,7 +6567,7 @@
         <v>602</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>110</v>
@@ -6578,7 +6590,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" s="5" t="s">
         <v>606</v>
       </c>
@@ -6586,7 +6598,7 @@
         <v>607</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>425</v>
@@ -6607,7 +6619,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>606</v>
       </c>
@@ -6634,15 +6646,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B125" t="s">
         <v>502</v>
       </c>
       <c r="C125" s="19" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="D125" t="s">
         <v>147</v>
@@ -6651,23 +6663,23 @@
         <v>42</v>
       </c>
       <c r="F125" s="26" t="s">
+        <v>643</v>
+      </c>
+      <c r="G125" t="s">
+        <v>661</v>
+      </c>
+      <c r="H125" t="s">
         <v>644</v>
       </c>
-      <c r="G125" t="s">
-        <v>662</v>
-      </c>
-      <c r="H125" t="s">
+      <c r="I125" s="20" t="s">
         <v>645</v>
       </c>
-      <c r="I125" s="20" t="s">
-        <v>646</v>
-      </c>
       <c r="J125" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126" s="5" t="s">
         <v>613</v>
       </c>
@@ -6694,7 +6706,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127" s="5" t="s">
         <v>617</v>
       </c>
@@ -6702,7 +6714,7 @@
         <v>618</v>
       </c>
       <c r="C127" s="21" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D127" s="5" t="s">
         <v>95</v>
@@ -6725,7 +6737,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128" s="5" t="s">
         <v>622</v>
       </c>
@@ -6733,7 +6745,7 @@
         <v>623</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>425</v>
@@ -6754,7 +6766,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129" s="5" t="s">
         <v>626</v>
       </c>
@@ -6768,32 +6780,32 @@
         <v>27</v>
       </c>
       <c r="E129" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F129" s="5" t="s">
         <v>629</v>
-      </c>
-      <c r="F129" s="5" t="s">
-        <v>630</v>
       </c>
       <c r="G129" t="s">
         <v>102</v>
       </c>
       <c r="H129" s="5"/>
       <c r="I129" s="5" t="s">
+        <v>630</v>
+      </c>
+      <c r="J129" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-helene.vezina@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A130" s="5" t="s">
         <v>631</v>
-      </c>
-      <c r="J129" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-helene.vezina@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A130" s="5" t="s">
-        <v>632</v>
       </c>
       <c r="B130" s="5" t="s">
         <v>618</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="D130" s="5" t="s">
         <v>95</v>
@@ -6804,19 +6816,19 @@
         <v>96</v>
       </c>
       <c r="H130" s="5" t="s">
+        <v>632</v>
+      </c>
+      <c r="I130" s="12" t="s">
         <v>633</v>
       </c>
-      <c r="I130" s="12" t="s">
+      <c r="J130" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A131" s="6" t="s">
         <v>634</v>
-      </c>
-      <c r="J130" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A131" s="6" t="s">
-        <v>635</v>
       </c>
       <c r="B131" s="6" t="s">
         <v>230</v>
@@ -6829,7 +6841,7 @@
         <v>76</v>
       </c>
       <c r="F131" s="6" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="G131" t="s">
         <v>453</v>
@@ -6838,11 +6850,40 @@
         <v>474</v>
       </c>
       <c r="I131" s="6" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="J131" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A132" s="5" t="s">
+        <v>731</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>732</v>
+      </c>
+      <c r="C132" s="5"/>
+      <c r="D132" s="5" t="s">
+        <v>733</v>
+      </c>
+      <c r="E132" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F132" s="5"/>
+      <c r="G132" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H132" s="5" t="s">
+        <v>734</v>
+      </c>
+      <c r="I132" s="9" t="s">
+        <v>735</v>
+      </c>
+      <c r="J132" s="29" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=sosthene.yamale@umontreal.ca</v>
       </c>
     </row>
   </sheetData>
@@ -6890,16 +6931,37 @@
     <hyperlink ref="I109" r:id="rId41" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
     <hyperlink ref="I48" r:id="rId42" xr:uid="{ABEB73EB-E336-4619-ADE1-0AE567E81306}"/>
     <hyperlink ref="I27" r:id="rId43" xr:uid="{E819F1D0-ED89-4281-B222-20D0A6AC8A49}"/>
+    <hyperlink ref="I132" r:id="rId44" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId44"/>
+  <pageSetup orientation="portrait" r:id="rId45"/>
   <tableParts count="1">
-    <tablePart r:id="rId45"/>
+    <tablePart r:id="rId46"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CC83367596A4B94585FCDD3502D89912" ma:contentTypeVersion="11" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="4e4efa8c0f0f722bbfc4a6b86077b9b4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1" xmlns:ns3="9cb1c2f4-2737-4134-a1af-8acbe3d02830" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81c6aeae46cd0fb81a99420a9570330b" ns2:_="" ns3:_="">
     <xsd:import namespace="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
@@ -7094,41 +7156,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCC2BCD-0310-4A3C-9E4B-6EFDEBA53649}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
-    <ds:schemaRef ds:uri="9cb1c2f4-2737-4134-a1af-8acbe3d02830"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7151,9 +7182,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCC2BCD-0310-4A3C-9E4B-6EFDEBA53649}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
+    <ds:schemaRef ds:uri="9cb1c2f4-2737-4134-a1af-8acbe3d02830"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Changements concernant Thien-Huong Che-Quang
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6798BC22-21B2-4139-9A6C-461FA7869724}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0D8EDFF-109B-4264-B688-5DF9C360AE38}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19455" yWindow="4650" windowWidth="20475" windowHeight="23445" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19460" yWindow="4650" windowWidth="20480" windowHeight="23450" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="736">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="733">
   <si>
     <t>nom</t>
   </si>
@@ -1595,21 +1595,9 @@
     <t>virginie.paquet@umontreal.ca</t>
   </si>
   <si>
-    <t>Paquette-Bigras</t>
-  </si>
-  <si>
     <t>Ève</t>
   </si>
   <si>
-    <t>Gestion des données de recherche</t>
-  </si>
-  <si>
-    <t>514 343-6111, poste 17279</t>
-  </si>
-  <si>
-    <t>eve.paquette-bigras@umontreal.ca</t>
-  </si>
-  <si>
     <t>Patenaude</t>
   </si>
   <si>
@@ -2111,9 +2099,6 @@
     <t>chantal-desrosiers.jpg</t>
   </si>
   <si>
-    <t>eve-paquette-bigras.jpg</t>
-  </si>
-  <si>
     <t>jason-madooray.jpg</t>
   </si>
   <si>
@@ -2174,9 +2159,6 @@
     <t>Sarah-Julie</t>
   </si>
   <si>
-    <t>Direction de la Bibliothèque des  lettres et sciences humaines et  Livres rares et collections spéciales</t>
-  </si>
-  <si>
     <t>514 343-6111, poste 3772</t>
   </si>
   <si>
@@ -2256,6 +2238,15 @@
   </si>
   <si>
     <t>sosthene.yamale@umontreal.ca</t>
+  </si>
+  <si>
+    <t>mailto:thien-huong.che-quang@umontreal.ca</t>
+  </si>
+  <si>
+    <t>514 343-6111, poste 8735</t>
+  </si>
+  <si>
+    <t>Québec</t>
   </si>
 </sst>
 </file>
@@ -2564,10 +2555,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J132" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:J132" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
-  <sortState ref="A2:J132">
-    <sortCondition ref="A1:A132"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J131" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:J131" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
+  <sortState ref="A2:J131">
+    <sortCondition ref="A1:A131"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{4B04E1AF-0079-4AD2-81CA-E8A433733E21}" name="nom"/>
@@ -2908,22 +2899,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J132"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J131"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" customWidth="1"/>
-    <col min="4" max="4" width="28.140625" customWidth="1"/>
-    <col min="5" max="5" width="58.140625" customWidth="1"/>
+    <col min="3" max="3" width="25.81640625" customWidth="1"/>
+    <col min="4" max="4" width="28.1796875" customWidth="1"/>
+    <col min="5" max="5" width="58.1796875" customWidth="1"/>
     <col min="6" max="6" width="58" style="26" customWidth="1"/>
-    <col min="7" max="7" width="70.85546875" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="41.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="86.5703125" customWidth="1"/>
+    <col min="7" max="7" width="70.81640625" customWidth="1"/>
+    <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="86.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2955,7 +2946,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
@@ -2986,7 +2977,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alexandre.amar-zifkin@umontreal.ca</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -3003,7 +2994,7 @@
         <v>42</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>21</v>
@@ -3019,7 +3010,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.angers@umontreal.ca</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>24</v>
       </c>
@@ -3050,7 +3041,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nadege.arsa@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>32</v>
       </c>
@@ -3081,7 +3072,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=denis.arvisais@umontreal.ca</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>38</v>
       </c>
@@ -3101,7 +3092,7 @@
         <v>43</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>44</v>
@@ -3114,7 +3105,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.attia@umontreal.ca</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>46</v>
       </c>
@@ -3145,15 +3136,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=prlaval@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="B8" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="D8" t="s">
         <v>95</v>
@@ -3162,23 +3153,23 @@
         <v>15</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
       </c>
       <c r="H8" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="I8" s="20" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="J8" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=eve.baribeau.marchand@umontreal.ca</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>53</v>
       </c>
@@ -3208,7 +3199,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.bastien@umontreal.ca</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>60</v>
       </c>
@@ -3236,7 +3227,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magalie.beaudoin@umontreal.ca</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>67</v>
       </c>
@@ -3253,10 +3244,10 @@
         <v>71</v>
       </c>
       <c r="F11" s="26" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>72</v>
@@ -3269,7 +3260,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maryna.beaulieu@umontreal.ca</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
         <v>74</v>
       </c>
@@ -3277,7 +3268,7 @@
         <v>39</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>75</v>
@@ -3299,7 +3290,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.begin-poissant@umontreal.ca</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
         <v>80</v>
       </c>
@@ -3329,7 +3320,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.belanger@umontreal.ca</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
         <v>88</v>
       </c>
@@ -3362,7 +3353,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amy.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>93</v>
       </c>
@@ -3370,7 +3361,7 @@
         <v>94</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>95</v>
@@ -3391,7 +3382,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amelie.bernard@umontreal.ca</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>99</v>
       </c>
@@ -3399,7 +3390,7 @@
         <v>104</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="D16" t="s">
         <v>95</v>
@@ -3418,7 +3409,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>99</v>
       </c>
@@ -3447,7 +3438,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=hugo.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>107</v>
       </c>
@@ -3478,7 +3469,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon.blais.longtin@umontreal.ca</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>113</v>
       </c>
@@ -3508,7 +3499,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tatiana.talpa@umontreal.ca</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
         <v>119</v>
       </c>
@@ -3534,7 +3525,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=joanna.bodnar@umontreal.ca</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>124</v>
       </c>
@@ -3564,7 +3555,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alain.borsi@umontreal.ca</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
         <v>132</v>
       </c>
@@ -3595,7 +3586,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.p.bouchard@umontreal.ca</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
         <v>139</v>
       </c>
@@ -3626,7 +3617,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refdroi@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
         <v>145</v>
       </c>
@@ -3634,7 +3625,7 @@
         <v>146</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>147</v>
@@ -3643,10 +3634,10 @@
         <v>76</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>148</v>
@@ -3659,7 +3650,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=myriam.boyer@umontreal.ca</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
         <v>150</v>
       </c>
@@ -3667,7 +3658,7 @@
         <v>151</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>49</v>
@@ -3677,7 +3668,7 @@
         <v>152</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>153</v>
@@ -3690,7 +3681,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guylaine.brazeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
         <v>155</v>
       </c>
@@ -3718,15 +3709,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sophie.brisebois@umontreal.ca</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
-        <v>725</v>
+        <v>719</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>727</v>
+        <v>721</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>13</v>
@@ -3735,23 +3726,23 @@
         <v>128</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>728</v>
+        <v>722</v>
       </c>
       <c r="G27" t="s">
         <v>15</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>729</v>
+        <v>723</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>730</v>
+        <v>724</v>
       </c>
       <c r="J27" s="29" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=tanya.buchet@umontreal.ca</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>160</v>
       </c>
@@ -3759,7 +3750,7 @@
         <v>161</v>
       </c>
       <c r="C28" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="D28" t="s">
         <v>95</v>
@@ -3778,7 +3769,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fanny.c.brochu@umontreal.ca</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>164</v>
       </c>
@@ -3786,7 +3777,7 @@
         <v>165</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>166</v>
@@ -3809,7 +3800,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=delphine.cado@umontreal.ca</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>171</v>
       </c>
@@ -3817,7 +3808,7 @@
         <v>172</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>49</v>
@@ -3840,7 +3831,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=siv.kham.chao@umontreal.ca</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>177</v>
       </c>
@@ -3871,7 +3862,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=laurence.charest@umontreal.ca</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>183</v>
       </c>
@@ -3879,7 +3870,7 @@
         <v>184</v>
       </c>
       <c r="C32" s="24" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="D32" t="s">
         <v>27</v>
@@ -3895,7 +3886,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>185</v>
       </c>
@@ -3906,7 +3897,7 @@
         <v>49</v>
       </c>
       <c r="G33" t="s">
-        <v>640</v>
+        <v>636</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>187</v>
@@ -3919,7 +3910,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=annick.charette@umontreal.ca</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>189</v>
       </c>
@@ -3933,21 +3924,24 @@
       <c r="E34" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="G34" s="5" t="s">
-        <v>708</v>
+      <c r="F34" s="26" t="s">
+        <v>732</v>
+      </c>
+      <c r="G34" t="s">
+        <v>63</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>709</v>
+        <v>731</v>
       </c>
       <c r="I34" s="9" t="s">
-        <v>710</v>
+        <v>730</v>
       </c>
       <c r="J34" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mailto:thien-huong.che-quang@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
         <v>192</v>
       </c>
@@ -3978,7 +3972,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah.cherrier@umontreal.ca</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>198</v>
       </c>
@@ -4008,7 +4002,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emir.chouchane@umontreal.ca</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
         <v>205</v>
       </c>
@@ -4016,7 +4010,7 @@
         <v>206</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>27</v>
@@ -4039,7 +4033,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=accessibilite@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
         <v>210</v>
       </c>
@@ -4059,7 +4053,7 @@
         <v>215</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="H38" s="5" t="s">
         <v>216</v>
@@ -4072,7 +4066,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benjamin.constantineau@umontreal.ca</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
         <v>218</v>
       </c>
@@ -4103,7 +4097,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon-pierre.crevier@umontreal.ca</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>224</v>
       </c>
@@ -4111,7 +4105,7 @@
         <v>225</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>696</v>
+        <v>691</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>13</v>
@@ -4134,7 +4128,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marc-olivier.croteau@umontreal.ca</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
         <v>229</v>
       </c>
@@ -4165,7 +4159,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.dalpe@umontreal.ca</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
         <v>235</v>
       </c>
@@ -4196,7 +4190,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=morgane.de.bellefeuille@umontreal.ca</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
         <v>243</v>
       </c>
@@ -4214,7 +4208,7 @@
         <v>246</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>640</v>
+        <v>636</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>247</v>
@@ -4227,7 +4221,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=Indiana.delsart@umontreal.ca</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="6" t="s">
         <v>249</v>
       </c>
@@ -4258,7 +4252,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=dominic.desaulniers@umontreal.ca</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
         <v>255</v>
       </c>
@@ -4266,7 +4260,7 @@
         <v>256</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>257</v>
@@ -4287,7 +4281,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.desrosiers@umontreal.ca</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>261</v>
       </c>
@@ -4295,7 +4289,7 @@
         <v>262</v>
       </c>
       <c r="C46" t="s">
-        <v>704</v>
+        <v>699</v>
       </c>
       <c r="D46" t="s">
         <v>95</v>
@@ -4314,7 +4308,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.dubois.mercier@umontreal.ca</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
         <v>265</v>
       </c>
@@ -4345,12 +4339,12 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jean-francois.durnin@umontreal.ca</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>720</v>
+        <v>714</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>721</v>
+        <v>715</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5" t="s">
@@ -4360,23 +4354,23 @@
         <v>128</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>722</v>
+        <v>716</v>
       </c>
       <c r="G48" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>723</v>
+        <v>717</v>
       </c>
       <c r="I48" s="9" t="s">
-        <v>724</v>
+        <v>718</v>
       </c>
       <c r="J48" s="29" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=taline.ekmekjian@umontreal.ca</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>271</v>
       </c>
@@ -4384,7 +4378,7 @@
         <v>272</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>692</v>
+        <v>687</v>
       </c>
       <c r="D49" t="s">
         <v>95</v>
@@ -4403,7 +4397,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=judith.fafard-larose@umontreal.ca</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="6" t="s">
         <v>275</v>
       </c>
@@ -4436,7 +4430,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" s="6" t="s">
         <v>275</v>
       </c>
@@ -4447,7 +4441,7 @@
         <v>277</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="E51" s="5" t="s">
         <v>128</v>
@@ -4467,7 +4461,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="6" t="s">
         <v>280</v>
       </c>
@@ -4500,7 +4494,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=c.fortier@umontreal.ca</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="6" t="s">
         <v>286</v>
       </c>
@@ -4529,7 +4523,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" s="6" t="s">
         <v>292</v>
       </c>
@@ -4560,7 +4554,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nino.gabrielli@umontreal.ca</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>298</v>
       </c>
@@ -4568,7 +4562,7 @@
         <v>299</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>698</v>
+        <v>693</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>300</v>
@@ -4589,7 +4583,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-pierre.gadoua@umontreal.ca</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" s="6" t="s">
         <v>303</v>
       </c>
@@ -4620,7 +4614,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cynthia.gagne.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>310</v>
       </c>
@@ -4648,7 +4642,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>310</v>
       </c>
@@ -4674,7 +4668,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="6" t="s">
         <v>317</v>
       </c>
@@ -4704,7 +4698,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marjorie.gauchier@umontreal.ca</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
         <v>323</v>
       </c>
@@ -4723,7 +4717,7 @@
         <v>325</v>
       </c>
       <c r="H60" s="7" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="I60" s="12" t="s">
         <v>326</v>
@@ -4733,7 +4727,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>327</v>
       </c>
@@ -4741,7 +4735,7 @@
         <v>328</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>27</v>
@@ -4764,7 +4758,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>332</v>
       </c>
@@ -4795,7 +4789,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="6" t="s">
         <v>337</v>
       </c>
@@ -4826,7 +4820,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
       </c>
     </row>
-    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>343</v>
       </c>
@@ -4857,7 +4851,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
         <v>349</v>
       </c>
@@ -4886,7 +4880,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
       </c>
     </row>
-    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
         <v>354</v>
       </c>
@@ -4901,7 +4895,7 @@
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5" t="s">
-        <v>716</v>
+        <v>710</v>
       </c>
       <c r="G66" s="5" t="s">
         <v>29</v>
@@ -4917,7 +4911,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>359</v>
       </c>
@@ -4925,7 +4919,7 @@
         <v>360</v>
       </c>
       <c r="C67" t="s">
-        <v>700</v>
+        <v>695</v>
       </c>
       <c r="D67" t="s">
         <v>49</v>
@@ -4944,7 +4938,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="6" t="s">
         <v>363</v>
       </c>
@@ -4966,14 +4960,14 @@
         <v>364</v>
       </c>
       <c r="I68" s="8" t="s">
-        <v>637</v>
+        <v>633</v>
       </c>
       <c r="J68" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>365</v>
       </c>
@@ -4981,7 +4975,7 @@
         <v>104</v>
       </c>
       <c r="C69" t="s">
-        <v>697</v>
+        <v>692</v>
       </c>
       <c r="D69" t="s">
         <v>95</v>
@@ -5000,7 +4994,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" s="6" t="s">
         <v>368</v>
       </c>
@@ -5020,7 +5014,7 @@
         <v>371</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>372</v>
@@ -5033,7 +5027,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
         <v>374</v>
       </c>
@@ -5066,7 +5060,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A72" s="6" t="s">
         <v>379</v>
       </c>
@@ -5074,7 +5068,7 @@
         <v>311</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>646</v>
+        <v>642</v>
       </c>
       <c r="D72" s="6" t="s">
         <v>41</v>
@@ -5099,7 +5093,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>383</v>
       </c>
@@ -5107,7 +5101,7 @@
         <v>384</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="D73" t="s">
         <v>95</v>
@@ -5126,7 +5120,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" s="6" t="s">
         <v>387</v>
       </c>
@@ -5141,7 +5135,7 @@
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="6" t="s">
-        <v>719</v>
+        <v>713</v>
       </c>
       <c r="G74" s="6" t="s">
         <v>29</v>
@@ -5157,7 +5151,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
       </c>
     </row>
-    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>392</v>
       </c>
@@ -5165,7 +5159,7 @@
         <v>393</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>27</v>
@@ -5188,7 +5182,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A76" s="6" t="s">
         <v>397</v>
       </c>
@@ -5218,7 +5212,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
         <v>402</v>
       </c>
@@ -5238,7 +5232,7 @@
         <v>405</v>
       </c>
       <c r="G77" s="6" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="H77" s="5" t="s">
         <v>406</v>
@@ -5251,7 +5245,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" s="6" t="s">
         <v>408</v>
       </c>
@@ -5259,7 +5253,7 @@
         <v>409</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="D78" s="6" t="s">
         <v>147</v>
@@ -5281,7 +5275,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
       </c>
     </row>
-    <row r="79" spans="1:10" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
         <v>412</v>
       </c>
@@ -5312,7 +5306,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A80" s="7" t="s">
         <v>417</v>
       </c>
@@ -5320,7 +5314,7 @@
         <v>418</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="D80" s="7" t="s">
         <v>41</v>
@@ -5329,10 +5323,10 @@
         <v>42</v>
       </c>
       <c r="F80" s="26" t="s">
-        <v>641</v>
+        <v>637</v>
       </c>
       <c r="G80" s="7" t="s">
-        <v>651</v>
+        <v>647</v>
       </c>
       <c r="H80" s="7" t="s">
         <v>419</v>
@@ -5345,7 +5339,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
         <v>417</v>
       </c>
@@ -5353,7 +5347,7 @@
         <v>421</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>95</v>
@@ -5371,7 +5365,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
         <v>423</v>
       </c>
@@ -5379,7 +5373,7 @@
         <v>424</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>688</v>
+        <v>683</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>425</v>
@@ -5400,7 +5394,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
         <v>428</v>
       </c>
@@ -5408,7 +5402,7 @@
         <v>429</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>703</v>
+        <v>698</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>425</v>
@@ -5429,7 +5423,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="s">
         <v>433</v>
       </c>
@@ -5437,7 +5431,7 @@
         <v>434</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>702</v>
+        <v>697</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>435</v>
@@ -5460,7 +5454,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
         <v>439</v>
       </c>
@@ -5475,7 +5469,7 @@
       </c>
       <c r="E85" s="5"/>
       <c r="F85" s="5" t="s">
-        <v>717</v>
+        <v>711</v>
       </c>
       <c r="G85" s="5" t="s">
         <v>29</v>
@@ -5491,7 +5485,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
         <v>444</v>
       </c>
@@ -5522,7 +5516,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
         <v>450</v>
       </c>
@@ -5552,7 +5546,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
         <v>456</v>
       </c>
@@ -5560,7 +5554,7 @@
         <v>457</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>425</v>
@@ -5581,7 +5575,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
         <v>460</v>
       </c>
@@ -5612,7 +5606,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A90" s="10" t="s">
         <v>466</v>
       </c>
@@ -5643,7 +5637,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A91" s="6" t="s">
         <v>471</v>
       </c>
@@ -5674,7 +5668,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A92" s="6" t="s">
         <v>476</v>
       </c>
@@ -5705,7 +5699,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=assia.mourid@umontreal.ca</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>482</v>
       </c>
@@ -5713,7 +5707,7 @@
         <v>483</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="D93" s="6" t="s">
         <v>27</v>
@@ -5736,7 +5730,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A94" s="10" t="s">
         <v>487</v>
       </c>
@@ -5744,7 +5738,7 @@
         <v>488</v>
       </c>
       <c r="C94" s="10" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="D94" s="10" t="s">
         <v>238</v>
@@ -5754,7 +5748,7 @@
       </c>
       <c r="F94" s="28"/>
       <c r="G94" s="10" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="H94" s="10" t="s">
         <v>489</v>
@@ -5767,7 +5761,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A95" s="6" t="s">
         <v>491</v>
       </c>
@@ -5775,7 +5769,7 @@
         <v>492</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="D95" s="6" t="s">
         <v>493</v>
@@ -5798,7 +5792,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
       </c>
     </row>
-    <row r="96" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A96" s="6" t="s">
         <v>497</v>
       </c>
@@ -5825,7 +5819,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
-    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A97" s="6" t="s">
         <v>501</v>
       </c>
@@ -5833,17 +5827,17 @@
         <v>502</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>649</v>
+        <v>645</v>
       </c>
       <c r="D97" s="6" t="s">
         <v>41</v>
       </c>
       <c r="E97" s="16"/>
       <c r="F97" s="7" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="G97" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="H97" s="6" t="s">
         <v>503</v>
@@ -5856,7 +5850,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" s="6" t="s">
         <v>505</v>
       </c>
@@ -5883,7 +5877,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>510</v>
       </c>
@@ -5913,237 +5907,229 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A100" s="5" t="s">
-        <v>515</v>
-      </c>
-      <c r="B100" s="5" t="s">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A100" s="6" t="s">
         <v>516</v>
       </c>
-      <c r="C100" s="5" t="s">
-        <v>687</v>
-      </c>
-      <c r="D100" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="E100" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F100" s="5" t="s">
+      <c r="B100" s="6" t="s">
+        <v>521</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="D100" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E100" s="6"/>
+      <c r="F100" s="6" t="s">
+        <v>712</v>
+      </c>
+      <c r="G100" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H100" s="7" t="s">
+        <v>523</v>
+      </c>
+      <c r="I100" s="7" t="s">
+        <v>524</v>
+      </c>
+      <c r="J100" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A101" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B101" s="5" t="s">
         <v>517</v>
       </c>
-      <c r="G100" t="s">
-        <v>102</v>
-      </c>
-      <c r="H100" s="10" t="s">
+      <c r="C101" s="5" t="s">
+        <v>660</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E101" s="5"/>
+      <c r="F101" s="5" t="s">
         <v>518</v>
       </c>
-      <c r="I100" s="10" t="s">
+      <c r="G101" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H101" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="J100" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=eve.paquette-bigras@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A101" s="6" t="s">
+      <c r="I101" s="10" t="s">
         <v>520</v>
       </c>
-      <c r="B101" s="6" t="s">
+      <c r="J101" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A102" s="5" t="s">
         <v>525</v>
       </c>
-      <c r="C101" s="6" t="s">
+      <c r="B102" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="C102" s="5" t="s">
         <v>526</v>
-      </c>
-      <c r="D101" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E101" s="6"/>
-      <c r="F101" s="6" t="s">
-        <v>718</v>
-      </c>
-      <c r="G101" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H101" s="7" t="s">
-        <v>527</v>
-      </c>
-      <c r="I101" s="7" t="s">
-        <v>528</v>
-      </c>
-      <c r="J101" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A102" s="5" t="s">
-        <v>520</v>
-      </c>
-      <c r="B102" s="5" t="s">
-        <v>521</v>
-      </c>
-      <c r="C102" s="5" t="s">
-        <v>664</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E102" s="5"/>
       <c r="F102" s="5" t="s">
-        <v>522</v>
+        <v>142</v>
       </c>
       <c r="G102" s="5" t="s">
-        <v>29</v>
+        <v>96</v>
       </c>
       <c r="H102" s="10" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="I102" s="10" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="J102" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A103" s="5" t="s">
         <v>529</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>311</v>
+        <v>483</v>
       </c>
       <c r="C103" s="5" t="s">
         <v>530</v>
       </c>
       <c r="D103" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E103" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F103" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="H103" s="10"/>
+      <c r="I103" s="9" t="s">
+        <v>532</v>
+      </c>
+      <c r="J103" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A104" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="C104" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="D104" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E103" s="5"/>
-      <c r="F103" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="G103" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="H103" s="10" t="s">
-        <v>531</v>
-      </c>
-      <c r="I103" s="10" t="s">
-        <v>532</v>
-      </c>
-      <c r="J103" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="B104" s="5" t="s">
-        <v>483</v>
-      </c>
-      <c r="C104" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="D104" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E104" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F104" s="5" t="s">
-        <v>535</v>
-      </c>
-      <c r="H104" s="10"/>
-      <c r="I104" s="9" t="s">
+      <c r="E104" s="6"/>
+      <c r="F104" s="6" t="s">
         <v>536</v>
       </c>
+      <c r="G104" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="H104" s="7" t="s">
+        <v>537</v>
+      </c>
+      <c r="I104" s="7" t="s">
+        <v>538</v>
+      </c>
       <c r="J104" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="6" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>538</v>
-      </c>
-      <c r="C105" s="6" t="s">
-        <v>539</v>
+        <v>540</v>
+      </c>
+      <c r="C105" s="5" t="s">
+        <v>696</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="E105" s="6"/>
-      <c r="F105" s="6" t="s">
-        <v>540</v>
-      </c>
-      <c r="G105" s="6" t="s">
-        <v>325</v>
+      <c r="F105" s="6"/>
+      <c r="G105" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="H105" s="7" t="s">
         <v>541</v>
       </c>
-      <c r="I105" s="7" t="s">
+      <c r="I105" s="13" t="s">
         <v>542</v>
       </c>
       <c r="J105" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A106" s="6" t="s">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
         <v>543</v>
       </c>
-      <c r="B106" s="6" t="s">
+      <c r="B106" t="s">
         <v>544</v>
       </c>
-      <c r="C106" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="D106" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="E106" s="6"/>
-      <c r="F106" s="6"/>
-      <c r="G106" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H106" s="7" t="s">
+      <c r="C106" t="s">
+        <v>684</v>
+      </c>
+      <c r="D106" t="s">
+        <v>425</v>
+      </c>
+      <c r="G106" t="s">
+        <v>636</v>
+      </c>
+      <c r="H106" s="6" t="s">
         <v>545</v>
       </c>
-      <c r="I106" s="13" t="s">
+      <c r="I106" s="14" t="s">
         <v>546</v>
       </c>
       <c r="J106" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>547</v>
       </c>
       <c r="B107" t="s">
         <v>548</v>
       </c>
-      <c r="C107" t="s">
-        <v>689</v>
-      </c>
+      <c r="C107" s="24"/>
       <c r="D107" t="s">
-        <v>425</v>
+        <v>95</v>
       </c>
       <c r="G107" t="s">
-        <v>640</v>
-      </c>
-      <c r="H107" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H107" t="s">
         <v>549</v>
       </c>
       <c r="I107" s="14" t="s">
@@ -6151,580 +6137,584 @@
       </c>
       <c r="J107" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>551</v>
+        <v>701</v>
       </c>
       <c r="B108" t="s">
-        <v>552</v>
-      </c>
-      <c r="C108" s="24"/>
+        <v>702</v>
+      </c>
+      <c r="C108" s="5" t="s">
+        <v>709</v>
+      </c>
       <c r="D108" t="s">
         <v>95</v>
       </c>
+      <c r="E108" s="5"/>
+      <c r="F108" s="7" t="s">
+        <v>567</v>
+      </c>
       <c r="G108" t="s">
+        <v>568</v>
+      </c>
+      <c r="H108" t="s">
+        <v>703</v>
+      </c>
+      <c r="I108" s="20" t="s">
+        <v>704</v>
+      </c>
+      <c r="J108" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>551</v>
+      </c>
+      <c r="B109" t="s">
+        <v>54</v>
+      </c>
+      <c r="C109" s="18" t="s">
+        <v>552</v>
+      </c>
+      <c r="D109" t="s">
+        <v>13</v>
+      </c>
+      <c r="F109" s="27" t="s">
+        <v>553</v>
+      </c>
+      <c r="G109" t="s">
         <v>29</v>
       </c>
-      <c r="H108" t="s">
-        <v>553</v>
-      </c>
-      <c r="I108" s="14" t="s">
+      <c r="H109" s="3" t="s">
         <v>554</v>
       </c>
-      <c r="J108" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>706</v>
-      </c>
-      <c r="B109" t="s">
-        <v>707</v>
-      </c>
-      <c r="C109" s="5" t="s">
-        <v>715</v>
-      </c>
-      <c r="D109" t="s">
-        <v>95</v>
-      </c>
-      <c r="E109" s="5"/>
-      <c r="F109" s="7" t="s">
-        <v>571</v>
-      </c>
-      <c r="G109" t="s">
-        <v>572</v>
-      </c>
-      <c r="H109" t="s">
-        <v>709</v>
-      </c>
-      <c r="I109" s="20" t="s">
-        <v>710</v>
+      <c r="I109" s="3" t="s">
+        <v>555</v>
       </c>
       <c r="J109" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>555</v>
-      </c>
-      <c r="B110" t="s">
-        <v>54</v>
-      </c>
-      <c r="C110" s="18" t="s">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A110" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="D110" t="s">
+      <c r="B110" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="C110" s="5" t="s">
+        <v>557</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E110" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F110" s="5"/>
+      <c r="H110" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="I110" s="10" t="s">
+        <v>558</v>
+      </c>
+      <c r="J110" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A111" s="5" t="s">
+        <v>559</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>560</v>
+      </c>
+      <c r="C111" s="5" t="s">
+        <v>666</v>
+      </c>
+      <c r="D111" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F110" s="27" t="s">
-        <v>557</v>
-      </c>
-      <c r="G110" t="s">
-        <v>29</v>
-      </c>
-      <c r="H110" s="3" t="s">
-        <v>558</v>
-      </c>
-      <c r="I110" s="3" t="s">
-        <v>559</v>
-      </c>
-      <c r="J110" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A111" s="5" t="s">
-        <v>560</v>
-      </c>
-      <c r="B111" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="C111" s="5" t="s">
+      <c r="E111" s="5"/>
+      <c r="F111" s="5" t="s">
         <v>561</v>
       </c>
-      <c r="D111" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="E111" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F111" s="5"/>
-      <c r="H111" s="10" t="s">
-        <v>122</v>
-      </c>
+      <c r="G111" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="H111" s="10"/>
       <c r="I111" s="10" t="s">
         <v>562</v>
       </c>
       <c r="J111" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A112" s="5" t="s">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
         <v>563</v>
       </c>
-      <c r="B112" s="5" t="s">
+      <c r="B112" t="s">
         <v>564</v>
       </c>
-      <c r="C112" s="5" t="s">
-        <v>670</v>
+      <c r="C112" s="24" t="s">
+        <v>661</v>
       </c>
       <c r="D112" s="5" t="s">
-        <v>13</v>
+        <v>257</v>
       </c>
       <c r="E112" s="5"/>
-      <c r="F112" s="5" t="s">
+      <c r="F112" s="5"/>
+      <c r="G112" t="s">
+        <v>29</v>
+      </c>
+      <c r="J112" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A113" s="7" t="s">
         <v>565</v>
       </c>
-      <c r="G112" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="H112" s="10"/>
-      <c r="I112" s="10" t="s">
+      <c r="B113" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C113" s="6" t="s">
         <v>566</v>
       </c>
-      <c r="J112" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
+      <c r="D113" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E113" s="7"/>
+      <c r="F113" s="7" t="s">
         <v>567</v>
       </c>
-      <c r="B113" t="s">
+      <c r="G113" s="7" t="s">
         <v>568</v>
       </c>
-      <c r="C113" s="24" t="s">
-        <v>665</v>
-      </c>
-      <c r="D113" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="E113" s="5"/>
-      <c r="F113" s="5"/>
-      <c r="G113" t="s">
-        <v>29</v>
+      <c r="H113" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="I113" s="7" t="s">
+        <v>570</v>
       </c>
       <c r="J113" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A114" s="7" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="B114" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C114" s="6" t="s">
-        <v>570</v>
-      </c>
+        <v>256</v>
+      </c>
+      <c r="C114" s="23"/>
       <c r="D114" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E114" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F114" s="7"/>
+      <c r="G114" s="7"/>
+      <c r="H114" s="7" t="s">
+        <v>572</v>
+      </c>
+      <c r="I114" s="7" t="s">
+        <v>573</v>
+      </c>
+      <c r="J114" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A115" s="5" t="s">
+        <v>574</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>575</v>
+      </c>
+      <c r="C115" s="19" t="s">
+        <v>576</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="E115" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G115" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="H115" s="5" t="s">
+        <v>577</v>
+      </c>
+      <c r="I115" s="5" t="s">
+        <v>578</v>
+      </c>
+      <c r="J115" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>705</v>
+      </c>
+      <c r="B116" t="s">
+        <v>610</v>
+      </c>
+      <c r="C116" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="D116" t="s">
+        <v>95</v>
+      </c>
+      <c r="E116" s="5"/>
+      <c r="F116" s="7" t="s">
+        <v>567</v>
+      </c>
+      <c r="G116" t="s">
+        <v>568</v>
+      </c>
+      <c r="H116" t="s">
+        <v>706</v>
+      </c>
+      <c r="I116" s="20" t="s">
+        <v>707</v>
+      </c>
+      <c r="J116" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A117" s="5" t="s">
+        <v>579</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>580</v>
+      </c>
+      <c r="C117" s="21" t="s">
+        <v>675</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E117" s="5"/>
+      <c r="F117" s="5"/>
+      <c r="G117" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="H117" s="5"/>
+      <c r="I117" s="12" t="s">
+        <v>581</v>
+      </c>
+      <c r="J117" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A118" s="10" t="s">
+        <v>582</v>
+      </c>
+      <c r="B118" s="10" t="s">
+        <v>583</v>
+      </c>
+      <c r="C118" s="21" t="s">
+        <v>584</v>
+      </c>
+      <c r="D118" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="E118" t="s">
+        <v>585</v>
+      </c>
+      <c r="F118" s="10" t="s">
+        <v>586</v>
+      </c>
+      <c r="G118" s="10" t="s">
+        <v>655</v>
+      </c>
+      <c r="H118" s="10" t="s">
+        <v>587</v>
+      </c>
+      <c r="I118" s="10" t="s">
+        <v>588</v>
+      </c>
+      <c r="J118" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A119" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="B119" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="C119" s="6" t="s">
+        <v>590</v>
+      </c>
+      <c r="D119" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E114" s="7"/>
-      <c r="F114" s="7" t="s">
-        <v>571</v>
-      </c>
-      <c r="G114" s="7" t="s">
-        <v>572</v>
-      </c>
-      <c r="H114" s="7" t="s">
-        <v>573</v>
-      </c>
-      <c r="I114" s="7" t="s">
-        <v>574</v>
-      </c>
-      <c r="J114" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A115" s="7" t="s">
-        <v>575</v>
-      </c>
-      <c r="B115" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="C115" s="23"/>
-      <c r="D115" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="E115" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="F115" s="7"/>
-      <c r="G115" s="7"/>
-      <c r="H115" s="7" t="s">
-        <v>576</v>
-      </c>
-      <c r="I115" s="7" t="s">
-        <v>577</v>
-      </c>
-      <c r="J115" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A116" s="5" t="s">
-        <v>578</v>
-      </c>
-      <c r="B116" s="5" t="s">
-        <v>579</v>
-      </c>
-      <c r="C116" s="19" t="s">
-        <v>580</v>
-      </c>
-      <c r="D116" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="E116" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G116" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="H116" s="5" t="s">
-        <v>581</v>
-      </c>
-      <c r="I116" s="5" t="s">
-        <v>582</v>
-      </c>
-      <c r="J116" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>711</v>
-      </c>
-      <c r="B117" t="s">
-        <v>614</v>
-      </c>
-      <c r="C117" s="19" t="s">
-        <v>714</v>
-      </c>
-      <c r="D117" t="s">
-        <v>95</v>
-      </c>
-      <c r="E117" s="5"/>
-      <c r="F117" s="7" t="s">
-        <v>571</v>
-      </c>
-      <c r="G117" t="s">
-        <v>572</v>
-      </c>
-      <c r="H117" t="s">
-        <v>712</v>
-      </c>
-      <c r="I117" s="20" t="s">
-        <v>713</v>
-      </c>
-      <c r="J117" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A118" s="5" t="s">
-        <v>583</v>
-      </c>
-      <c r="B118" s="5" t="s">
-        <v>584</v>
-      </c>
-      <c r="C118" s="21" t="s">
-        <v>679</v>
-      </c>
-      <c r="D118" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="E118" s="5"/>
-      <c r="F118" s="5"/>
-      <c r="G118" s="5" t="s">
-        <v>447</v>
-      </c>
-      <c r="H118" s="5"/>
-      <c r="I118" s="12" t="s">
-        <v>585</v>
-      </c>
-      <c r="J118" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A119" s="10" t="s">
-        <v>586</v>
-      </c>
-      <c r="B119" s="10" t="s">
-        <v>587</v>
-      </c>
-      <c r="C119" s="21" t="s">
-        <v>588</v>
-      </c>
-      <c r="D119" s="10" t="s">
-        <v>288</v>
-      </c>
-      <c r="E119" t="s">
-        <v>589</v>
-      </c>
-      <c r="F119" s="10" t="s">
-        <v>590</v>
-      </c>
-      <c r="G119" s="10" t="s">
-        <v>659</v>
-      </c>
-      <c r="H119" s="10" t="s">
+      <c r="E119" s="6"/>
+      <c r="F119" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="G119" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H119" s="6" t="s">
         <v>591</v>
       </c>
-      <c r="I119" s="10" t="s">
+      <c r="I119" s="6" t="s">
         <v>592</v>
       </c>
       <c r="J119" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A120" s="6" t="s">
         <v>593</v>
       </c>
       <c r="B120" s="6" t="s">
-        <v>483</v>
+        <v>594</v>
       </c>
       <c r="C120" s="6" t="s">
-        <v>594</v>
+        <v>689</v>
       </c>
       <c r="D120" s="6" t="s">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="E120" s="6"/>
-      <c r="F120" s="6" t="s">
-        <v>135</v>
-      </c>
+      <c r="F120" s="6"/>
       <c r="G120" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="H120" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="H120" t="s">
         <v>595</v>
       </c>
-      <c r="I120" s="6" t="s">
+      <c r="I120" s="13" t="s">
         <v>596</v>
       </c>
       <c r="J120" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A121" s="6" t="s">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A121" s="5" t="s">
         <v>597</v>
       </c>
-      <c r="B121" s="6" t="s">
+      <c r="B121" s="5" t="s">
         <v>598</v>
       </c>
-      <c r="C121" s="6" t="s">
-        <v>694</v>
-      </c>
-      <c r="D121" s="6" t="s">
+      <c r="C121" s="5" t="s">
+        <v>665</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E121" s="5"/>
+      <c r="F121" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="G121" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="H121" s="5" t="s">
+        <v>600</v>
+      </c>
+      <c r="I121" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="J121" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A122" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="C122" s="5" t="s">
+        <v>667</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="E122" s="5"/>
+      <c r="F122" s="5"/>
+      <c r="G122" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="H122" s="6" t="s">
+        <v>431</v>
+      </c>
+      <c r="I122" s="12" t="s">
+        <v>604</v>
+      </c>
+      <c r="J122" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
+        <v>602</v>
+      </c>
+      <c r="B123" t="s">
+        <v>605</v>
+      </c>
+      <c r="D123" t="s">
+        <v>49</v>
+      </c>
+      <c r="F123" s="26" t="s">
+        <v>606</v>
+      </c>
+      <c r="G123" t="s">
+        <v>307</v>
+      </c>
+      <c r="H123" s="6" t="s">
+        <v>607</v>
+      </c>
+      <c r="I123" s="14" t="s">
+        <v>608</v>
+      </c>
+      <c r="J123" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
+        <v>638</v>
+      </c>
+      <c r="B124" t="s">
+        <v>502</v>
+      </c>
+      <c r="C124" s="19" t="s">
+        <v>688</v>
+      </c>
+      <c r="D124" t="s">
+        <v>147</v>
+      </c>
+      <c r="E124" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F124" s="26" t="s">
+        <v>639</v>
+      </c>
+      <c r="G124" t="s">
+        <v>657</v>
+      </c>
+      <c r="H124" t="s">
+        <v>640</v>
+      </c>
+      <c r="I124" s="20" t="s">
+        <v>641</v>
+      </c>
+      <c r="J124" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A125" s="5" t="s">
+        <v>609</v>
+      </c>
+      <c r="B125" s="5" t="s">
+        <v>610</v>
+      </c>
+      <c r="C125" s="21"/>
+      <c r="D125" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="E121" s="6"/>
-      <c r="F121" s="6"/>
-      <c r="G121" s="6" t="s">
-        <v>447</v>
-      </c>
-      <c r="H121" t="s">
-        <v>599</v>
-      </c>
-      <c r="I121" s="13" t="s">
-        <v>600</v>
-      </c>
-      <c r="J121" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A122" s="5" t="s">
-        <v>601</v>
-      </c>
-      <c r="B122" s="5" t="s">
-        <v>602</v>
-      </c>
-      <c r="C122" s="5" t="s">
-        <v>669</v>
-      </c>
-      <c r="D122" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="E122" s="5"/>
-      <c r="F122" s="5" t="s">
-        <v>603</v>
-      </c>
-      <c r="G122" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="H122" s="5" t="s">
-        <v>604</v>
-      </c>
-      <c r="I122" s="5" t="s">
-        <v>605</v>
-      </c>
-      <c r="J122" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A123" s="5" t="s">
-        <v>606</v>
-      </c>
-      <c r="B123" s="5" t="s">
-        <v>607</v>
-      </c>
-      <c r="C123" s="5" t="s">
-        <v>671</v>
-      </c>
-      <c r="D123" s="5" t="s">
-        <v>425</v>
-      </c>
-      <c r="E123" s="5"/>
-      <c r="F123" s="5"/>
-      <c r="G123" s="5" t="s">
-        <v>430</v>
-      </c>
-      <c r="H123" s="6" t="s">
-        <v>431</v>
-      </c>
-      <c r="I123" s="12" t="s">
-        <v>608</v>
-      </c>
-      <c r="J123" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>606</v>
-      </c>
-      <c r="B124" t="s">
-        <v>609</v>
-      </c>
-      <c r="D124" t="s">
-        <v>49</v>
-      </c>
-      <c r="F124" s="26" t="s">
-        <v>610</v>
-      </c>
-      <c r="G124" t="s">
-        <v>307</v>
-      </c>
-      <c r="H124" s="6" t="s">
+      <c r="E125" s="5"/>
+      <c r="F125" s="5"/>
+      <c r="G125" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H125" s="5" t="s">
         <v>611</v>
       </c>
-      <c r="I124" s="14" t="s">
+      <c r="I125" s="12" t="s">
         <v>612</v>
       </c>
-      <c r="J124" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>642</v>
-      </c>
-      <c r="B125" t="s">
-        <v>502</v>
-      </c>
-      <c r="C125" s="19" t="s">
-        <v>693</v>
-      </c>
-      <c r="D125" t="s">
-        <v>147</v>
-      </c>
-      <c r="E125" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F125" s="26" t="s">
-        <v>643</v>
-      </c>
-      <c r="G125" t="s">
-        <v>661</v>
-      </c>
-      <c r="H125" t="s">
-        <v>644</v>
-      </c>
-      <c r="I125" s="20" t="s">
-        <v>645</v>
-      </c>
       <c r="J125" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A126" s="5" t="s">
         <v>613</v>
       </c>
       <c r="B126" s="5" t="s">
         <v>614</v>
       </c>
-      <c r="C126" s="21"/>
+      <c r="C126" s="21" t="s">
+        <v>644</v>
+      </c>
       <c r="D126" s="5" t="s">
         <v>95</v>
       </c>
       <c r="E126" s="5"/>
-      <c r="F126" s="5"/>
+      <c r="F126" s="5" t="s">
+        <v>615</v>
+      </c>
       <c r="G126" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H126" s="5" t="s">
+        <v>616</v>
+      </c>
+      <c r="I126" s="12" t="s">
+        <v>617</v>
+      </c>
+      <c r="J126" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A127" s="5" t="s">
+        <v>618</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>619</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>678</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="E127" s="5"/>
+      <c r="F127" s="5"/>
+      <c r="G127" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="H126" s="5" t="s">
-        <v>615</v>
-      </c>
-      <c r="I126" s="12" t="s">
-        <v>616</v>
-      </c>
-      <c r="J126" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A127" s="5" t="s">
-        <v>617</v>
-      </c>
-      <c r="B127" s="5" t="s">
-        <v>618</v>
-      </c>
-      <c r="C127" s="21" t="s">
-        <v>648</v>
-      </c>
-      <c r="D127" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="E127" s="5"/>
-      <c r="F127" s="5" t="s">
-        <v>619</v>
-      </c>
-      <c r="G127" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="H127" s="5" t="s">
         <v>620</v>
@@ -6734,10 +6724,10 @@
       </c>
       <c r="J127" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
         <v>622</v>
       </c>
@@ -6745,143 +6735,114 @@
         <v>623</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>682</v>
+        <v>624</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>425</v>
-      </c>
-      <c r="E128" s="5"/>
-      <c r="F128" s="5"/>
-      <c r="G128" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H128" s="5" t="s">
-        <v>624</v>
-      </c>
-      <c r="I128" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E128" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F128" s="5" t="s">
         <v>625</v>
       </c>
+      <c r="G128" t="s">
+        <v>102</v>
+      </c>
+      <c r="H128" s="5"/>
+      <c r="I128" s="5" t="s">
+        <v>626</v>
+      </c>
       <c r="J128" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-helene.vezina@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>627</v>
+        <v>614</v>
       </c>
       <c r="C129" s="5" t="s">
+        <v>686</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E129" s="5"/>
+      <c r="F129" s="5"/>
+      <c r="G129" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="H129" s="5" t="s">
         <v>628</v>
       </c>
-      <c r="D129" s="5" t="s">
+      <c r="I129" s="12" t="s">
+        <v>629</v>
+      </c>
+      <c r="J129" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A130" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="B130" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="C130" s="6"/>
+      <c r="D130" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E129" s="5" t="s">
+      <c r="E130" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F130" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="G130" t="s">
+        <v>453</v>
+      </c>
+      <c r="H130" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="I130" s="6" t="s">
+        <v>632</v>
+      </c>
+      <c r="J130" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A131" s="5" t="s">
+        <v>725</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>726</v>
+      </c>
+      <c r="C131" s="5"/>
+      <c r="D131" s="5" t="s">
+        <v>727</v>
+      </c>
+      <c r="E131" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F129" s="5" t="s">
-        <v>629</v>
-      </c>
-      <c r="G129" t="s">
-        <v>102</v>
-      </c>
-      <c r="H129" s="5"/>
-      <c r="I129" s="5" t="s">
-        <v>630</v>
-      </c>
-      <c r="J129" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-helene.vezina@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A130" s="5" t="s">
-        <v>631</v>
-      </c>
-      <c r="B130" s="5" t="s">
-        <v>618</v>
-      </c>
-      <c r="C130" s="5" t="s">
-        <v>691</v>
-      </c>
-      <c r="D130" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="E130" s="5"/>
-      <c r="F130" s="5"/>
-      <c r="G130" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="H130" s="5" t="s">
-        <v>632</v>
-      </c>
-      <c r="I130" s="12" t="s">
-        <v>633</v>
-      </c>
-      <c r="J130" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A131" s="6" t="s">
-        <v>634</v>
-      </c>
-      <c r="B131" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="C131" s="6"/>
-      <c r="D131" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E131" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F131" s="6" t="s">
-        <v>635</v>
-      </c>
-      <c r="G131" t="s">
-        <v>453</v>
-      </c>
-      <c r="H131" s="6" t="s">
-        <v>474</v>
-      </c>
-      <c r="I131" s="6" t="s">
-        <v>636</v>
-      </c>
-      <c r="J131" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A132" s="5" t="s">
-        <v>731</v>
-      </c>
-      <c r="B132" s="5" t="s">
-        <v>732</v>
-      </c>
-      <c r="C132" s="5"/>
-      <c r="D132" s="5" t="s">
-        <v>733</v>
-      </c>
-      <c r="E132" s="5" t="s">
+      <c r="F131" s="5"/>
+      <c r="G131" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F132" s="5"/>
-      <c r="G132" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="H132" s="5" t="s">
-        <v>734</v>
-      </c>
-      <c r="I132" s="9" t="s">
-        <v>735</v>
-      </c>
-      <c r="J132" s="29" t="str">
+      <c r="H131" s="5" t="s">
+        <v>728</v>
+      </c>
+      <c r="I131" s="9" t="s">
+        <v>729</v>
+      </c>
+      <c r="J131" s="29" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=sosthene.yamale@umontreal.ca</v>
       </c>
@@ -6893,19 +6854,19 @@
     <hyperlink ref="I17" r:id="rId3" display="mailto:hugo.bernier@umontreal.ca" xr:uid="{3F591457-DA50-462E-B1CA-F2F56ED9E3DD}"/>
     <hyperlink ref="I68" r:id="rId4" xr:uid="{4822C834-E5A8-42FD-9734-374BFC718C85}"/>
     <hyperlink ref="I10" r:id="rId5" display="mailto:magalie.beaudoin@umontreal.ca" xr:uid="{2D976BF0-B68A-46E5-8412-BA8BC43FD26D}"/>
-    <hyperlink ref="I104" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
+    <hyperlink ref="I103" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
     <hyperlink ref="I4" r:id="rId7" display="mailto:nadege.arsa@bib.umontreal.ca" xr:uid="{408AF5A3-35ED-4BF5-92B9-1B21C0C475D9}"/>
     <hyperlink ref="I18" r:id="rId8" display="mailto:simon.blais.longtin@umontreal.ca" xr:uid="{EA917AC7-9087-435B-A6E7-3AE1885514AA}"/>
     <hyperlink ref="I84" r:id="rId9" xr:uid="{8ABC26E9-CF81-491C-8A28-B209E6620D2A}"/>
-    <hyperlink ref="I127" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
+    <hyperlink ref="I126" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
     <hyperlink ref="I33" r:id="rId11" xr:uid="{7D21070C-9A14-48DF-982E-D995A034BDAD}"/>
-    <hyperlink ref="I124" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
+    <hyperlink ref="I123" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
     <hyperlink ref="I67" r:id="rId13" xr:uid="{DCABBE8B-8789-4957-9A88-F8585AD53BBC}"/>
-    <hyperlink ref="I107" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
+    <hyperlink ref="I106" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
     <hyperlink ref="I46" r:id="rId15" xr:uid="{1383A46C-5C1D-4621-B4BC-67AD012D7CF5}"/>
     <hyperlink ref="I73" r:id="rId16" xr:uid="{29D9619F-F3A7-41E8-AE0F-DEBBF802D53A}"/>
     <hyperlink ref="I28" r:id="rId17" xr:uid="{9E8CD31B-437A-49A0-BA12-85176E0D9431}"/>
-    <hyperlink ref="I108" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
+    <hyperlink ref="I107" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
     <hyperlink ref="I69" r:id="rId19" xr:uid="{3B502B79-2DDE-44A3-908B-3CB04ED1101E}"/>
     <hyperlink ref="I16" r:id="rId20" xr:uid="{BAE0697B-7739-4A42-9702-C285F03D0F77}"/>
     <hyperlink ref="I49" r:id="rId21" xr:uid="{E1BC7B04-B072-447B-9137-59A28141883D}"/>
@@ -6913,25 +6874,25 @@
     <hyperlink ref="I60" r:id="rId23" xr:uid="{6E82D57D-36A4-4928-AD91-BE73FFC7C389}"/>
     <hyperlink ref="I75" r:id="rId24" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
     <hyperlink ref="I93" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
-    <hyperlink ref="I123" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
+    <hyperlink ref="I122" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
     <hyperlink ref="I82" r:id="rId27" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
     <hyperlink ref="I83" r:id="rId28" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
     <hyperlink ref="I88" r:id="rId29" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
-    <hyperlink ref="I106" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
-    <hyperlink ref="I118" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
-    <hyperlink ref="I121" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
-    <hyperlink ref="I126" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
-    <hyperlink ref="I128" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
-    <hyperlink ref="I130" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
+    <hyperlink ref="I105" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
+    <hyperlink ref="I117" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
+    <hyperlink ref="I120" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
+    <hyperlink ref="I125" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
+    <hyperlink ref="I127" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
+    <hyperlink ref="I129" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
     <hyperlink ref="I15" r:id="rId36" xr:uid="{E26D4CB1-6F14-4277-AD54-18A052872B6B}"/>
-    <hyperlink ref="I125" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
+    <hyperlink ref="I124" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
     <hyperlink ref="I8" r:id="rId38" xr:uid="{2E646106-878B-4504-8874-8750F3CAA7CB}"/>
     <hyperlink ref="I34" r:id="rId39" xr:uid="{902A8808-023C-4EA1-833E-F687288B12ED}"/>
-    <hyperlink ref="I117" r:id="rId40" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
-    <hyperlink ref="I109" r:id="rId41" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
+    <hyperlink ref="I116" r:id="rId40" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
+    <hyperlink ref="I108" r:id="rId41" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
     <hyperlink ref="I48" r:id="rId42" xr:uid="{ABEB73EB-E336-4619-ADE1-0AE567E81306}"/>
     <hyperlink ref="I27" r:id="rId43" xr:uid="{E819F1D0-ED89-4281-B222-20D0A6AC8A49}"/>
-    <hyperlink ref="I132" r:id="rId44" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
+    <hyperlink ref="I131" r:id="rId44" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId45"/>
@@ -6951,17 +6912,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CC83367596A4B94585FCDD3502D89912" ma:contentTypeVersion="11" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="4e4efa8c0f0f722bbfc4a6b86077b9b4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1" xmlns:ns3="9cb1c2f4-2737-4134-a1af-8acbe3d02830" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81c6aeae46cd0fb81a99420a9570330b" ns2:_="" ns3:_="">
     <xsd:import namespace="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
@@ -7156,6 +7106,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
   <ds:schemaRefs>
@@ -7165,23 +7126,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="9cb1c2f4-2737-4134-a1af-8acbe3d02830"/>
-    <ds:schemaRef ds:uri="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCC2BCD-0310-4A3C-9E4B-6EFDEBA53649}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7198,4 +7142,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="9cb1c2f4-2737-4134-a1af-8acbe3d02830"/>
+    <ds:schemaRef ds:uri="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Changements concernant David Patenaude
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0D8EDFF-109B-4264-B688-5DF9C360AE38}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D20A8ACD-3559-4BEE-930B-3010686C8BD2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19460" yWindow="4650" windowWidth="20480" windowHeight="23450" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="733">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="733">
   <si>
     <t>nom</t>
   </si>
@@ -2186,9 +2186,6 @@
     <t>Histoire, Linguistique et traduction</t>
   </si>
   <si>
-    <t>Criminologie, Travail social, Démographie et sciences de la population, Sécurité et études policières, Dépendances, Victimologie, Sexualité : enjeux de société et pratiques d'intervention</t>
-  </si>
-  <si>
     <t>Science politique, Études internationales, Études féministes - des genres et des sexualités, Sciences économiques, Données statistiques</t>
   </si>
   <si>
@@ -2247,6 +2244,9 @@
   </si>
   <si>
     <t>Québec</t>
+  </si>
+  <si>
+    <t>Criminologie, Démographie et sciences de la population, Sécurité et études policières, Dépendances, Victimologie, Sexualité : enjeux de société et pratiques d'intervention</t>
   </si>
 </sst>
 </file>
@@ -3711,13 +3711,13 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>719</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>720</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>721</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>13</v>
@@ -3726,16 +3726,16 @@
         <v>128</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="G27" t="s">
         <v>15</v>
       </c>
       <c r="H27" s="6" t="s">
+        <v>722</v>
+      </c>
+      <c r="I27" s="8" t="s">
         <v>723</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>724</v>
       </c>
       <c r="J27" s="29" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3925,16 +3925,16 @@
         <v>63</v>
       </c>
       <c r="F34" s="26" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="G34" t="s">
         <v>63</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="I34" s="9" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="J34" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4341,10 +4341,10 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
+        <v>713</v>
+      </c>
+      <c r="B48" s="5" t="s">
         <v>714</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>715</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5" t="s">
@@ -4354,16 +4354,16 @@
         <v>128</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="G48" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H48" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="I48" s="9" t="s">
         <v>717</v>
-      </c>
-      <c r="I48" s="9" t="s">
-        <v>718</v>
       </c>
       <c r="J48" s="29" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="6" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="G74" s="6" t="s">
         <v>29</v>
@@ -5920,9 +5920,11 @@
       <c r="D100" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E100" s="6"/>
+      <c r="E100" s="6" t="s">
+        <v>29</v>
+      </c>
       <c r="F100" s="6" t="s">
-        <v>712</v>
+        <v>732</v>
       </c>
       <c r="G100" s="6" t="s">
         <v>29</v>
@@ -6820,14 +6822,14 @@
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="s">
+        <v>724</v>
+      </c>
+      <c r="B131" s="5" t="s">
         <v>725</v>
-      </c>
-      <c r="B131" s="5" t="s">
-        <v>726</v>
       </c>
       <c r="C131" s="5"/>
       <c r="D131" s="5" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E131" s="5" t="s">
         <v>84</v>
@@ -6837,10 +6839,10 @@
         <v>84</v>
       </c>
       <c r="H131" s="5" t="s">
+        <v>727</v>
+      </c>
+      <c r="I131" s="9" t="s">
         <v>728</v>
-      </c>
-      <c r="I131" s="9" t="s">
-        <v>729</v>
       </c>
       <c r="J131" s="29" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>

</xml_diff>

<commit_message>
feat(repertoire-personnel): Autres changements au répertoire d'employés
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC572ED1-E944-42A0-BA08-AA44E8F9C752}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7912FB8D-84A5-4BA5-87E7-CDDFAFC0F39F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5460" yWindow="3555" windowWidth="30315" windowHeight="28125" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="770">
   <si>
     <t>nom</t>
   </si>
@@ -2331,6 +2331,33 @@
   </si>
   <si>
     <t>natalia-jabinschi.jpg</t>
+  </si>
+  <si>
+    <t>Lapalme</t>
+  </si>
+  <si>
+    <t>Marie-Josée</t>
+  </si>
+  <si>
+    <t>Technicien(ne) en muséologie</t>
+  </si>
+  <si>
+    <t>514 343-6111, poste 4585</t>
+  </si>
+  <si>
+    <t>marie-josee.lapalme@umontreal.ca</t>
+  </si>
+  <si>
+    <t>Moreau</t>
+  </si>
+  <si>
+    <t>diane-moreau.jpg</t>
+  </si>
+  <si>
+    <t>514 343-6111, poste 27731</t>
+  </si>
+  <si>
+    <t>diane.moreau@umontreal.ca</t>
   </si>
 </sst>
 </file>
@@ -2481,7 +2508,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2508,6 +2535,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
@@ -2689,10 +2717,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J143" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J143" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
-  <sortState ref="A2:J143">
-    <sortCondition ref="A1:A143"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J145" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J145" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
+  <sortState ref="A2:J145">
+    <sortCondition ref="A1:A145"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{4B04E1AF-0079-4AD2-81CA-E8A433733E21}" name="nom" dataDxfId="9"/>
@@ -3033,7 +3061,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J143"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" customWidth="1"/>
@@ -5442,350 +5470,350 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A81" s="5" t="s">
+    <row r="81" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="B81" s="18" t="s">
+        <v>762</v>
+      </c>
+      <c r="C81" s="18"/>
+      <c r="D81" s="18" t="s">
+        <v>763</v>
+      </c>
+      <c r="E81" s="18" t="s">
+        <v>668</v>
+      </c>
+      <c r="F81" s="18"/>
+      <c r="G81" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="H81" s="18" t="s">
+        <v>764</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="J81" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=marie-josee.lapalme@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A82" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="B81" s="5" t="s">
+      <c r="B82" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="C81" s="5" t="s">
+      <c r="C82" s="5" t="s">
         <v>610</v>
       </c>
-      <c r="D81" s="5" t="s">
+      <c r="D82" s="5" t="s">
         <v>710</v>
       </c>
-      <c r="E81" s="11" t="s">
+      <c r="E82" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="F81" s="5" t="s">
+      <c r="F82" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="G81" s="5" t="s">
+      <c r="G82" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H81" s="5" t="s">
+      <c r="H82" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="I81" s="5" t="s">
+      <c r="I82" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="J81" s="6" t="str">
+      <c r="J82" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+    <row r="83" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>362</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B83" t="s">
         <v>363</v>
       </c>
-      <c r="C82" s="5" t="s">
+      <c r="C83" s="5" t="s">
         <v>611</v>
       </c>
-      <c r="D82" s="5" t="s">
+      <c r="D83" s="5" t="s">
         <v>705</v>
       </c>
-      <c r="G82" t="s">
+      <c r="G83" t="s">
         <v>29</v>
       </c>
-      <c r="H82" s="13" t="s">
+      <c r="H83" s="13" t="s">
         <v>364</v>
       </c>
-      <c r="I82" s="8" t="s">
+      <c r="I83" s="8" t="s">
         <v>365</v>
       </c>
-      <c r="J82" s="6" t="str">
+      <c r="J83" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A83" s="5" t="s">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="B83" s="5" t="s">
+      <c r="B84" s="5" t="s">
         <v>367</v>
       </c>
-      <c r="C83" s="5" t="s">
+      <c r="C84" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="D83" s="5" t="s">
+      <c r="D84" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E83" s="5"/>
-      <c r="F83" s="5" t="s">
+      <c r="E84" s="5"/>
+      <c r="F84" s="5" t="s">
         <v>678</v>
       </c>
-      <c r="G83" s="5" t="s">
+      <c r="G84" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H83" s="5" t="s">
+      <c r="H84" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="I83" s="5" t="s">
+      <c r="I84" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="J83" s="6" t="str">
+      <c r="J84" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>371</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B85" t="s">
         <v>372</v>
       </c>
-      <c r="C84" s="5" t="s">
+      <c r="C85" s="5" t="s">
         <v>650</v>
       </c>
-      <c r="D84" s="5" t="s">
+      <c r="D85" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E84" s="5"/>
-      <c r="F84" t="s">
+      <c r="E85" s="5"/>
+      <c r="F85" t="s">
         <v>373</v>
       </c>
-      <c r="G84" s="5" t="s">
+      <c r="G85" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H84" t="s">
+      <c r="H85" t="s">
         <v>374</v>
       </c>
-      <c r="I84" s="8" t="s">
+      <c r="I85" s="8" t="s">
         <v>375</v>
       </c>
-      <c r="J84" s="6" t="str">
+      <c r="J85" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A85" s="5" t="s">
-        <v>376</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>377</v>
-      </c>
-      <c r="C85" s="5" t="s">
-        <v>378</v>
-      </c>
-      <c r="D85" s="5" t="s">
-        <v>710</v>
-      </c>
-      <c r="E85" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F85" s="3"/>
-      <c r="G85" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="H85" s="5" t="s">
-        <v>379</v>
-      </c>
-      <c r="I85" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="J85" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>710</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="F86" s="12" t="s">
-        <v>384</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="F86" s="3"/>
       <c r="G86" s="5" t="s">
-        <v>603</v>
+        <v>169</v>
       </c>
       <c r="H86" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="I86" s="15" t="s">
-        <v>386</v>
+        <v>379</v>
+      </c>
+      <c r="I86" s="5" t="s">
+        <v>380</v>
       </c>
       <c r="J86" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>659</v>
+        <v>383</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>710</v>
       </c>
       <c r="E87" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="F87" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G87" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="H87" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="I87" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="J87" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>659</v>
+      </c>
+      <c r="D88" s="5" t="s">
+        <v>710</v>
+      </c>
+      <c r="E88" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G87" s="5" t="s">
+      <c r="G88" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="H87" s="5" t="s">
+      <c r="H88" s="5" t="s">
         <v>389</v>
       </c>
-      <c r="I87" s="15" t="s">
+      <c r="I88" s="15" t="s">
         <v>390</v>
       </c>
-      <c r="J87" s="6" t="str">
+      <c r="J88" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A88" s="5" t="s">
+    <row r="89" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A89" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="B89" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="C88" s="5" t="s">
+      <c r="C89" s="5" t="s">
         <v>393</v>
       </c>
-      <c r="D88" s="5" t="s">
+      <c r="D89" s="5" t="s">
         <v>709</v>
       </c>
-      <c r="E88" s="11" t="s">
+      <c r="E89" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="F88" s="5"/>
-      <c r="G88" s="5" t="s">
+      <c r="F89" s="5"/>
+      <c r="G89" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="H88" s="5" t="s">
+      <c r="H89" s="5" t="s">
         <v>394</v>
       </c>
-      <c r="I88" s="5" t="s">
+      <c r="I89" s="5" t="s">
         <v>395</v>
       </c>
-      <c r="J88" s="6" t="str">
+      <c r="J89" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A89" s="3" t="s">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A90" s="3" t="s">
         <v>396</v>
       </c>
-      <c r="B89" s="3" t="s">
+      <c r="B90" s="3" t="s">
         <v>397</v>
       </c>
-      <c r="C89" s="3" t="s">
+      <c r="C90" s="3" t="s">
         <v>645</v>
       </c>
-      <c r="D89" s="5" t="s">
+      <c r="D90" s="5" t="s">
         <v>710</v>
       </c>
-      <c r="E89" s="3" t="s">
+      <c r="E90" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F89" t="s">
+      <c r="F90" t="s">
         <v>605</v>
       </c>
-      <c r="G89" s="3" t="s">
+      <c r="G90" s="3" t="s">
         <v>615</v>
       </c>
-      <c r="H89" s="3" t="s">
+      <c r="H90" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="I89" s="3" t="s">
+      <c r="I90" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="J89" s="6" t="str">
+      <c r="J90" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A90" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="B90" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="C90" s="5" t="s">
-        <v>646</v>
-      </c>
-      <c r="D90" s="5" t="s">
-        <v>708</v>
-      </c>
-      <c r="E90" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F90" s="5"/>
-      <c r="H90" s="5"/>
-      <c r="I90" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="J90" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>705</v>
-      </c>
-      <c r="E91" s="5"/>
+        <v>708</v>
+      </c>
+      <c r="E91" s="5" t="s">
+        <v>78</v>
+      </c>
       <c r="F91" s="5"/>
-      <c r="G91" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="H91" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="I91" s="8" t="s">
-        <v>405</v>
+      <c r="H91" s="5"/>
+      <c r="I91" s="5" t="s">
+        <v>401</v>
       </c>
       <c r="J91" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>663</v>
+        <v>648</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>705</v>
@@ -5793,1379 +5821,1381 @@
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
       <c r="G92" s="5" t="s">
-        <v>408</v>
+        <v>54</v>
       </c>
       <c r="H92" s="5" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="I92" s="8" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="J92" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>662</v>
-      </c>
-      <c r="D93" s="3" t="s">
-        <v>706</v>
+        <v>663</v>
+      </c>
+      <c r="D93" s="5" t="s">
+        <v>705</v>
       </c>
       <c r="E93" s="5"/>
+      <c r="F93" s="5"/>
       <c r="G93" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="H93" s="3" t="s">
-        <v>413</v>
+        <v>408</v>
+      </c>
+      <c r="H93" s="5" t="s">
+        <v>409</v>
       </c>
       <c r="I93" s="8" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="J93" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="D94" s="5" t="s">
-        <v>13</v>
+        <v>662</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>706</v>
       </c>
       <c r="E94" s="5"/>
-      <c r="F94" s="5" t="s">
-        <v>677</v>
-      </c>
       <c r="G94" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H94" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="I94" s="5" t="s">
-        <v>419</v>
+        <v>222</v>
+      </c>
+      <c r="H94" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="I94" s="8" t="s">
+        <v>414</v>
       </c>
       <c r="J94" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>339</v>
+        <v>416</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="D95" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E95" s="5"/>
       <c r="F95" s="5" t="s">
-        <v>422</v>
+        <v>677</v>
       </c>
       <c r="G95" s="5" t="s">
-        <v>423</v>
+        <v>29</v>
       </c>
       <c r="H95" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="I95" s="15" t="s">
-        <v>425</v>
+        <v>418</v>
+      </c>
+      <c r="I95" s="5" t="s">
+        <v>419</v>
       </c>
       <c r="J95" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C96" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E96" s="5"/>
+      <c r="F96" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="G96" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="H96" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="I96" s="15" t="s">
+        <v>425</v>
+      </c>
+      <c r="J96" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A97" s="5" t="s">
         <v>426</v>
       </c>
-      <c r="B96" s="5" t="s">
+      <c r="B97" s="5" t="s">
         <v>427</v>
       </c>
-      <c r="C96" s="5" t="s">
+      <c r="C97" s="5" t="s">
         <v>428</v>
       </c>
-      <c r="D96" s="5" t="s">
+      <c r="D97" s="5" t="s">
         <v>710</v>
       </c>
-      <c r="E96" s="5" t="s">
+      <c r="E97" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="G96" s="5" t="s">
+      <c r="G97" s="5" t="s">
         <v>429</v>
       </c>
-      <c r="H96" s="5" t="s">
+      <c r="H97" s="5" t="s">
         <v>430</v>
       </c>
-      <c r="I96" s="5" t="s">
+      <c r="I97" s="5" t="s">
         <v>431</v>
       </c>
-      <c r="J96" s="6" t="str">
+      <c r="J97" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="5" t="s">
-        <v>432</v>
-      </c>
-      <c r="B97" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="C97" s="5" t="s">
-        <v>630</v>
-      </c>
-      <c r="D97" s="5" t="s">
-        <v>705</v>
-      </c>
-      <c r="E97" s="5"/>
-      <c r="F97" s="5"/>
-      <c r="G97" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="H97" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="I97" s="8" t="s">
-        <v>435</v>
-      </c>
-      <c r="J97" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
       </c>
     </row>
     <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="C98" s="5" t="s">
+        <v>630</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>705</v>
+      </c>
+      <c r="E98" s="5"/>
+      <c r="F98" s="5"/>
+      <c r="G98" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H98" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="I98" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="J98" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="5" t="s">
         <v>436</v>
       </c>
-      <c r="B98" s="5" t="s">
+      <c r="B99" s="5" t="s">
         <v>437</v>
       </c>
-      <c r="C98" s="5" t="s">
+      <c r="C99" s="5" t="s">
         <v>438</v>
-      </c>
-      <c r="D98" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E98" s="5"/>
-      <c r="F98" s="5" t="s">
-        <v>439</v>
-      </c>
-      <c r="G98" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="H98" s="5" t="s">
-        <v>440</v>
-      </c>
-      <c r="I98" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="J98" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A99" s="3" t="s">
-        <v>442</v>
-      </c>
-      <c r="B99" s="3" t="s">
-        <v>443</v>
-      </c>
-      <c r="C99" s="5" t="s">
-        <v>444</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E99" s="5"/>
-      <c r="F99" s="3" t="s">
+      <c r="F99" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="G99" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="H99" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="I99" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="J99" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A100" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="C100" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E100" s="5"/>
+      <c r="F100" s="3" t="s">
         <v>422</v>
       </c>
-      <c r="G99" s="3" t="s">
+      <c r="G100" s="3" t="s">
         <v>423</v>
       </c>
-      <c r="H99" s="3" t="s">
+      <c r="H100" s="3" t="s">
         <v>445</v>
       </c>
-      <c r="I99" s="3" t="s">
+      <c r="I100" s="3" t="s">
         <v>446</v>
       </c>
-      <c r="J99" s="6" t="str">
+      <c r="J100" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A100" s="5" t="s">
-        <v>447</v>
-      </c>
-      <c r="B100" s="5" t="s">
-        <v>448</v>
-      </c>
-      <c r="C100" s="5" t="s">
-        <v>449</v>
-      </c>
-      <c r="D100" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="E100" s="5"/>
-      <c r="F100" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G100" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="H100" s="5" t="s">
-        <v>450</v>
-      </c>
-      <c r="I100" s="15" t="s">
-        <v>451</v>
-      </c>
-      <c r="J100" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="D101" s="5" t="s">
-        <v>13</v>
+        <v>103</v>
       </c>
       <c r="E101" s="5"/>
       <c r="F101" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G101" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="H101" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="I101" s="15" t="s">
+        <v>451</v>
+      </c>
+      <c r="J101" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A102" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E102" s="5"/>
+      <c r="F102" s="5" t="s">
         <v>455</v>
       </c>
-      <c r="G101" s="5" t="s">
+      <c r="G102" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="H101" s="5" t="s">
+      <c r="H102" s="5" t="s">
         <v>456</v>
       </c>
-      <c r="I101" s="5" t="s">
+      <c r="I102" s="5" t="s">
         <v>457</v>
       </c>
-      <c r="J101" s="6" t="str">
+      <c r="J102" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=assia.mourid@umontreal.ca</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A103" s="18" t="s">
+        <v>766</v>
+      </c>
+      <c r="B103" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="C103" s="18" t="s">
+        <v>767</v>
+      </c>
+      <c r="D103" s="5" t="s">
+        <v>705</v>
+      </c>
+      <c r="E103" t="s">
+        <v>67</v>
+      </c>
+      <c r="F103" s="18"/>
+      <c r="G103" t="s">
+        <v>127</v>
+      </c>
+      <c r="H103" s="18" t="s">
+        <v>768</v>
+      </c>
+      <c r="I103" s="6" t="s">
+        <v>769</v>
+      </c>
+      <c r="J103" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=diane.moreau@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
         <v>458</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B104" t="s">
         <v>459</v>
       </c>
-      <c r="C102" s="5" t="s">
+      <c r="C104" s="5" t="s">
         <v>631</v>
       </c>
-      <c r="D102" s="5" t="s">
+      <c r="D104" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E102" s="5"/>
-      <c r="F102" t="s">
+      <c r="E104" s="5"/>
+      <c r="F104" t="s">
         <v>460</v>
       </c>
-      <c r="G102" s="5" t="s">
+      <c r="G104" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H102" t="s">
+      <c r="H104" t="s">
         <v>461</v>
       </c>
-      <c r="I102" s="8" t="s">
+      <c r="I104" s="8" t="s">
         <v>462</v>
       </c>
-      <c r="J102" s="6" t="str">
+      <c r="J104" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
       </c>
     </row>
-    <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="3" t="s">
+    <row r="105" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="3" t="s">
         <v>463</v>
       </c>
-      <c r="B103" s="3" t="s">
+      <c r="B105" s="3" t="s">
         <v>464</v>
       </c>
-      <c r="C103" s="3" t="s">
+      <c r="C105" s="3" t="s">
         <v>638</v>
       </c>
-      <c r="D103" s="5" t="s">
+      <c r="D105" s="5" t="s">
         <v>711</v>
       </c>
-      <c r="E103" s="3" t="s">
+      <c r="E105" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F103" s="12"/>
-      <c r="G103" s="3" t="s">
+      <c r="F105" s="12"/>
+      <c r="G105" s="3" t="s">
         <v>623</v>
       </c>
-      <c r="H103" s="3" t="s">
+      <c r="H105" s="3" t="s">
         <v>465</v>
       </c>
-      <c r="I103" s="3" t="s">
+      <c r="I105" s="3" t="s">
         <v>466</v>
       </c>
-      <c r="J103" s="6" t="str">
+      <c r="J105" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="5" t="s">
+    <row r="106" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="B104" s="5" t="s">
+      <c r="B106" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="C104" s="5" t="s">
+      <c r="C106" s="5" t="s">
         <v>655</v>
       </c>
-      <c r="D104" s="5" t="s">
+      <c r="D106" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="E104" s="5"/>
-      <c r="F104" s="5" t="s">
+      <c r="E106" s="5"/>
+      <c r="F106" s="5" t="s">
         <v>470</v>
       </c>
-      <c r="G104" s="5" t="s">
+      <c r="G106" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="H104" s="5" t="s">
+      <c r="H106" s="5" t="s">
         <v>471</v>
       </c>
-      <c r="I104" s="15" t="s">
+      <c r="I106" s="15" t="s">
         <v>472</v>
       </c>
-      <c r="J104" s="6" t="str">
+      <c r="J106" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A105" s="5" t="s">
-        <v>473</v>
-      </c>
-      <c r="B105" s="5" t="s">
-        <v>474</v>
-      </c>
-      <c r="C105" s="5"/>
-      <c r="D105" s="3" t="s">
-        <v>706</v>
-      </c>
-      <c r="E105" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F105" s="5"/>
-      <c r="H105" s="5" t="s">
-        <v>475</v>
-      </c>
-      <c r="I105" s="5" t="s">
-        <v>476</v>
-      </c>
-      <c r="J105" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A106" s="5" t="s">
-        <v>477</v>
-      </c>
-      <c r="B106" s="5" t="s">
-        <v>478</v>
-      </c>
-      <c r="C106" s="5" t="s">
-        <v>613</v>
-      </c>
-      <c r="D106" s="5" t="s">
-        <v>710</v>
-      </c>
-      <c r="E106" s="11"/>
-      <c r="F106" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="G106" t="s">
-        <v>544</v>
-      </c>
-      <c r="H106" s="5" t="s">
-        <v>479</v>
-      </c>
-      <c r="I106" s="15" t="s">
-        <v>480</v>
-      </c>
-      <c r="J106" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
-        <v>481</v>
+        <v>473</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>482</v>
+        <v>474</v>
       </c>
       <c r="C107" s="5"/>
-      <c r="D107" s="5" t="s">
-        <v>483</v>
-      </c>
-      <c r="E107" s="5"/>
-      <c r="F107" t="s">
-        <v>484</v>
-      </c>
-      <c r="G107" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="H107" s="5"/>
-      <c r="I107" s="8" t="s">
-        <v>485</v>
+      <c r="D107" s="3" t="s">
+        <v>706</v>
+      </c>
+      <c r="E107" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F107" s="5"/>
+      <c r="H107" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="I107" s="5" t="s">
+        <v>476</v>
       </c>
       <c r="J107" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>486</v>
-      </c>
-      <c r="B108" t="s">
-        <v>487</v>
-      </c>
-      <c r="C108" s="7" t="s">
-        <v>488</v>
-      </c>
-      <c r="D108" t="s">
-        <v>27</v>
-      </c>
-      <c r="E108" t="s">
-        <v>78</v>
-      </c>
-      <c r="F108" s="5" t="s">
-        <v>489</v>
+      <c r="A108" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B108" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="C108" s="5" t="s">
+        <v>613</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>710</v>
+      </c>
+      <c r="E108" s="11"/>
+      <c r="F108" s="3" t="s">
+        <v>543</v>
       </c>
       <c r="G108" t="s">
-        <v>95</v>
-      </c>
-      <c r="I108" t="s">
-        <v>490</v>
+        <v>544</v>
+      </c>
+      <c r="H108" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="I108" s="15" t="s">
+        <v>480</v>
       </c>
       <c r="J108" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
-        <v>492</v>
+        <v>481</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>493</v>
-      </c>
-      <c r="C109" s="5" t="s">
-        <v>627</v>
-      </c>
+        <v>482</v>
+      </c>
+      <c r="C109" s="5"/>
       <c r="D109" s="5" t="s">
-        <v>13</v>
+        <v>483</v>
       </c>
       <c r="E109" s="5"/>
-      <c r="F109" s="5" t="s">
-        <v>494</v>
+      <c r="F109" t="s">
+        <v>484</v>
       </c>
       <c r="G109" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H109" s="3" t="s">
-        <v>495</v>
-      </c>
-      <c r="I109" s="3" t="s">
-        <v>496</v>
+        <v>222</v>
+      </c>
+      <c r="H109" s="5"/>
+      <c r="I109" s="8" t="s">
+        <v>485</v>
       </c>
       <c r="J109" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A110" s="5" t="s">
-        <v>492</v>
-      </c>
-      <c r="B110" s="5" t="s">
-        <v>497</v>
-      </c>
-      <c r="C110" s="5" t="s">
-        <v>498</v>
-      </c>
-      <c r="D110" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E110" s="5" t="s">
-        <v>29</v>
+      <c r="A110" t="s">
+        <v>486</v>
+      </c>
+      <c r="B110" t="s">
+        <v>487</v>
+      </c>
+      <c r="C110" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="D110" t="s">
+        <v>27</v>
+      </c>
+      <c r="E110" t="s">
+        <v>78</v>
       </c>
       <c r="F110" s="5" t="s">
-        <v>696</v>
-      </c>
-      <c r="G110" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H110" s="3" t="s">
-        <v>499</v>
-      </c>
-      <c r="I110" s="3" t="s">
-        <v>500</v>
+        <v>489</v>
+      </c>
+      <c r="G110" t="s">
+        <v>95</v>
+      </c>
+      <c r="I110" t="s">
+        <v>490</v>
       </c>
       <c r="J110" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
-        <v>501</v>
+        <v>492</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="C111" s="16" t="s">
-        <v>502</v>
+        <v>493</v>
+      </c>
+      <c r="C111" s="5" t="s">
+        <v>627</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E111" s="5"/>
       <c r="F111" s="5" t="s">
-        <v>133</v>
+        <v>494</v>
       </c>
       <c r="G111" s="5" t="s">
-        <v>89</v>
+        <v>29</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>503</v>
+        <v>495</v>
       </c>
       <c r="I111" s="3" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="J111" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
-        <v>505</v>
+        <v>492</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>459</v>
+        <v>497</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>506</v>
+        <v>498</v>
       </c>
       <c r="D112" s="5" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="F112" s="5" t="s">
-        <v>507</v>
-      </c>
-      <c r="G112" s="4"/>
-      <c r="H112" s="3"/>
-      <c r="I112" s="6" t="s">
-        <v>508</v>
+        <v>696</v>
+      </c>
+      <c r="G112" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H112" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="I112" s="3" t="s">
+        <v>500</v>
       </c>
       <c r="J112" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
-        <v>509</v>
+        <v>501</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>510</v>
-      </c>
-      <c r="C113" s="5" t="s">
-        <v>511</v>
+        <v>292</v>
+      </c>
+      <c r="C113" s="16" t="s">
+        <v>502</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E113" s="5"/>
       <c r="F113" s="5" t="s">
-        <v>512</v>
+        <v>133</v>
       </c>
       <c r="G113" s="5" t="s">
-        <v>304</v>
+        <v>89</v>
       </c>
       <c r="H113" s="3" t="s">
-        <v>513</v>
-      </c>
-      <c r="I113" s="15" t="s">
-        <v>514</v>
+        <v>503</v>
+      </c>
+      <c r="I113" s="3" t="s">
+        <v>504</v>
       </c>
       <c r="J113" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="C114" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E114" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F114" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="G114" s="4"/>
+      <c r="H114" s="3"/>
+      <c r="I114" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="J114" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A115" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>510</v>
+      </c>
+      <c r="C115" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E115" s="5"/>
+      <c r="F115" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="G115" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="H115" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="I115" s="15" t="s">
+        <v>514</v>
+      </c>
+      <c r="J115" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A116" s="5" t="s">
         <v>515</v>
       </c>
-      <c r="B114" s="5" t="s">
+      <c r="B116" s="5" t="s">
         <v>516</v>
       </c>
-      <c r="C114" s="5" t="s">
+      <c r="C116" s="5" t="s">
         <v>661</v>
       </c>
-      <c r="D114" s="5" t="s">
+      <c r="D116" s="5" t="s">
         <v>705</v>
       </c>
-      <c r="E114" s="5"/>
-      <c r="F114" s="5"/>
-      <c r="G114" s="5" t="s">
+      <c r="E116" s="5"/>
+      <c r="F116" s="5"/>
+      <c r="G116" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H114" s="3" t="s">
+      <c r="H116" s="3" t="s">
         <v>517</v>
       </c>
-      <c r="I114" s="8" t="s">
+      <c r="I116" s="8" t="s">
         <v>518</v>
       </c>
-      <c r="J114" s="6" t="str">
+      <c r="J116" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>519</v>
-      </c>
-      <c r="B115" t="s">
-        <v>520</v>
-      </c>
-      <c r="C115" t="s">
-        <v>649</v>
-      </c>
-      <c r="D115" s="5" t="s">
-        <v>705</v>
-      </c>
-      <c r="G115" t="s">
-        <v>604</v>
-      </c>
-      <c r="H115" s="5" t="s">
-        <v>521</v>
-      </c>
-      <c r="I115" s="8" t="s">
-        <v>522</v>
-      </c>
-      <c r="J115" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>738</v>
-      </c>
-      <c r="B116" t="s">
-        <v>459</v>
-      </c>
-      <c r="C116" s="14"/>
-      <c r="D116" t="s">
-        <v>755</v>
-      </c>
-      <c r="E116" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G116" t="s">
-        <v>79</v>
-      </c>
-      <c r="H116" t="s">
-        <v>310</v>
-      </c>
-      <c r="I116" s="6" t="s">
-        <v>739</v>
-      </c>
-      <c r="J116" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="B117" t="s">
-        <v>524</v>
-      </c>
-      <c r="C117" s="17"/>
+        <v>520</v>
+      </c>
+      <c r="C117" t="s">
+        <v>649</v>
+      </c>
       <c r="D117" s="5" t="s">
         <v>705</v>
       </c>
       <c r="G117" t="s">
-        <v>29</v>
-      </c>
-      <c r="H117" t="s">
-        <v>525</v>
+        <v>604</v>
+      </c>
+      <c r="H117" s="5" t="s">
+        <v>521</v>
       </c>
       <c r="I117" s="8" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="J117" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="B118" t="s">
-        <v>76</v>
-      </c>
-      <c r="C118" s="5"/>
+        <v>459</v>
+      </c>
+      <c r="C118" s="14"/>
       <c r="D118" t="s">
-        <v>726</v>
+        <v>755</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="F118" s="5"/>
-      <c r="G118" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="H118" s="5" t="s">
+      <c r="G118" t="s">
+        <v>79</v>
+      </c>
+      <c r="H118" t="s">
         <v>310</v>
       </c>
-      <c r="I118" t="s">
-        <v>720</v>
+      <c r="I118" s="6" t="s">
+        <v>739</v>
       </c>
       <c r="J118" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>666</v>
+        <v>523</v>
       </c>
       <c r="B119" t="s">
-        <v>667</v>
-      </c>
-      <c r="C119" s="16" t="s">
-        <v>675</v>
-      </c>
+        <v>524</v>
+      </c>
+      <c r="C119" s="17"/>
       <c r="D119" s="5" t="s">
         <v>705</v>
       </c>
-      <c r="E119" s="5"/>
-      <c r="F119" s="3"/>
       <c r="G119" t="s">
-        <v>544</v>
+        <v>29</v>
       </c>
       <c r="H119" t="s">
-        <v>669</v>
-      </c>
-      <c r="I119" s="6" t="s">
-        <v>670</v>
+        <v>525</v>
+      </c>
+      <c r="I119" s="8" t="s">
+        <v>526</v>
       </c>
       <c r="J119" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>527</v>
+        <v>728</v>
       </c>
       <c r="B120" t="s">
-        <v>51</v>
-      </c>
-      <c r="C120" s="7" t="s">
-        <v>528</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="C120" s="5"/>
       <c r="D120" t="s">
-        <v>13</v>
-      </c>
-      <c r="F120" s="5" t="s">
-        <v>529</v>
-      </c>
-      <c r="G120" t="s">
-        <v>29</v>
-      </c>
-      <c r="H120" s="3" t="s">
-        <v>530</v>
-      </c>
-      <c r="I120" s="3" t="s">
-        <v>531</v>
-      </c>
-      <c r="J120" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
+        <v>726</v>
+      </c>
+      <c r="E120" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F120" s="5"/>
+      <c r="G120" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="H120" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="I120" t="s">
+        <v>720</v>
+      </c>
+      <c r="J120" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
       </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
+        <v>666</v>
+      </c>
+      <c r="B121" t="s">
+        <v>667</v>
+      </c>
+      <c r="C121" s="16" t="s">
+        <v>675</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>705</v>
+      </c>
+      <c r="E121" s="5"/>
+      <c r="F121" s="3"/>
+      <c r="G121" t="s">
+        <v>544</v>
+      </c>
+      <c r="H121" t="s">
+        <v>669</v>
+      </c>
+      <c r="I121" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="J121" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>527</v>
+      </c>
+      <c r="B122" t="s">
+        <v>51</v>
+      </c>
+      <c r="C122" s="7" t="s">
+        <v>528</v>
+      </c>
+      <c r="D122" t="s">
+        <v>13</v>
+      </c>
+      <c r="F122" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="G122" t="s">
+        <v>29</v>
+      </c>
+      <c r="H122" s="3" t="s">
+        <v>530</v>
+      </c>
+      <c r="I122" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="J122" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
         <v>746</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B123" t="s">
         <v>124</v>
       </c>
-      <c r="C121" s="5"/>
-      <c r="D121" t="s">
+      <c r="C123" s="5"/>
+      <c r="D123" t="s">
         <v>755</v>
       </c>
-      <c r="E121" s="5" t="s">
+      <c r="E123" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G121" t="s">
+      <c r="G123" t="s">
         <v>79</v>
       </c>
-      <c r="H121" t="s">
+      <c r="H123" t="s">
         <v>747</v>
       </c>
-      <c r="I121" s="6" t="s">
+      <c r="I123" s="6" t="s">
         <v>748</v>
       </c>
-      <c r="J121" s="9" t="str">
+      <c r="J123" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A122" s="5" t="s">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A124" s="5" t="s">
         <v>532</v>
       </c>
-      <c r="B122" s="5" t="s">
+      <c r="B124" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="C122" s="5" t="s">
+      <c r="C124" s="5" t="s">
         <v>533</v>
       </c>
-      <c r="D122" s="5" t="s">
+      <c r="D124" s="5" t="s">
         <v>711</v>
       </c>
-      <c r="E122" s="5" t="s">
+      <c r="E124" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="F122" s="5"/>
-      <c r="H122" s="3" t="s">
+      <c r="F124" s="5"/>
+      <c r="H124" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="I122" s="15" t="s">
+      <c r="I124" s="15" t="s">
         <v>534</v>
       </c>
-      <c r="J122" s="6" t="str">
+      <c r="J124" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A123" s="5" t="s">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A125" s="5" t="s">
         <v>535</v>
       </c>
-      <c r="B123" s="5" t="s">
+      <c r="B125" s="5" t="s">
         <v>536</v>
       </c>
-      <c r="C123" s="5" t="s">
+      <c r="C125" s="5" t="s">
         <v>633</v>
       </c>
-      <c r="D123" s="5" t="s">
+      <c r="D125" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E123" s="5"/>
-      <c r="F123" s="5" t="s">
+      <c r="E125" s="5"/>
+      <c r="F125" s="5" t="s">
         <v>537</v>
       </c>
-      <c r="G123" s="5" t="s">
+      <c r="G125" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="H123" s="3"/>
-      <c r="I123" s="3" t="s">
+      <c r="H125" s="3"/>
+      <c r="I125" s="3" t="s">
         <v>538</v>
       </c>
-      <c r="J123" s="6" t="str">
+      <c r="J125" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
         <v>539</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B126" t="s">
         <v>540</v>
       </c>
-      <c r="C124" t="s">
+      <c r="C126" t="s">
         <v>628</v>
       </c>
-      <c r="D124" s="3" t="s">
-        <v>706</v>
-      </c>
-      <c r="E124" s="5"/>
-      <c r="F124" s="5"/>
-      <c r="G124" t="s">
-        <v>29</v>
-      </c>
-      <c r="J124" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A125" s="3" t="s">
-        <v>541</v>
-      </c>
-      <c r="B125" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C125" s="14" t="s">
-        <v>542</v>
-      </c>
-      <c r="D125" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E125" s="3"/>
-      <c r="F125" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="G125" s="3" t="s">
-        <v>544</v>
-      </c>
-      <c r="H125" s="3" t="s">
-        <v>545</v>
-      </c>
-      <c r="I125" s="3" t="s">
-        <v>546</v>
-      </c>
-      <c r="J125" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A126" s="3" t="s">
-        <v>547</v>
-      </c>
-      <c r="B126" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C126" s="3"/>
       <c r="D126" s="3" t="s">
         <v>706</v>
       </c>
-      <c r="E126" s="3" t="s">
+      <c r="E126" s="5"/>
+      <c r="F126" s="5"/>
+      <c r="G126" t="s">
+        <v>29</v>
+      </c>
+      <c r="J126" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A127" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C127" s="14" t="s">
+        <v>542</v>
+      </c>
+      <c r="D127" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E127" s="3"/>
+      <c r="F127" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="G127" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="H127" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="I127" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="J127" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A128" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C128" s="3"/>
+      <c r="D128" s="3" t="s">
+        <v>706</v>
+      </c>
+      <c r="E128" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F126" s="3"/>
-      <c r="G126" s="3"/>
-      <c r="H126" s="3" t="s">
+      <c r="F128" s="3"/>
+      <c r="G128" s="3"/>
+      <c r="H128" s="3" t="s">
         <v>548</v>
       </c>
-      <c r="I126" s="3" t="s">
+      <c r="I128" s="3" t="s">
         <v>549</v>
       </c>
-      <c r="J126" s="6" t="str">
+      <c r="J128" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A127" s="5" t="s">
-        <v>550</v>
-      </c>
-      <c r="B127" s="5" t="s">
-        <v>551</v>
-      </c>
-      <c r="C127" s="5" t="s">
-        <v>552</v>
-      </c>
-      <c r="D127" s="5" t="s">
-        <v>710</v>
-      </c>
-      <c r="E127" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G127" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="H127" s="5" t="s">
-        <v>553</v>
-      </c>
-      <c r="I127" s="15" t="s">
-        <v>554</v>
-      </c>
-      <c r="J127" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>671</v>
-      </c>
-      <c r="B128" t="s">
-        <v>585</v>
-      </c>
-      <c r="C128" s="5" t="s">
-        <v>674</v>
-      </c>
-      <c r="D128" s="5" t="s">
-        <v>705</v>
-      </c>
-      <c r="E128" s="5"/>
-      <c r="F128" s="3"/>
-      <c r="G128" t="s">
-        <v>544</v>
-      </c>
-      <c r="H128" t="s">
-        <v>672</v>
-      </c>
-      <c r="I128" s="6" t="s">
-        <v>673</v>
-      </c>
-      <c r="J128" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
       </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129" s="5" t="s">
-        <v>555</v>
+        <v>550</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>556</v>
+        <v>551</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>641</v>
+        <v>552</v>
       </c>
       <c r="D129" s="5" t="s">
+        <v>710</v>
+      </c>
+      <c r="E129" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G129" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="H129" s="5" t="s">
+        <v>553</v>
+      </c>
+      <c r="I129" s="15" t="s">
+        <v>554</v>
+      </c>
+      <c r="J129" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>671</v>
+      </c>
+      <c r="B130" t="s">
+        <v>585</v>
+      </c>
+      <c r="C130" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="D130" s="5" t="s">
         <v>705</v>
       </c>
-      <c r="E129" s="5"/>
-      <c r="F129" s="5"/>
-      <c r="G129" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="H129" s="5"/>
-      <c r="I129" s="8" t="s">
-        <v>557</v>
-      </c>
-      <c r="J129" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A130" s="3" t="s">
-        <v>558</v>
-      </c>
-      <c r="B130" s="3" t="s">
-        <v>559</v>
-      </c>
-      <c r="C130" s="5" t="s">
-        <v>560</v>
-      </c>
-      <c r="D130" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="E130" t="s">
-        <v>561</v>
-      </c>
-      <c r="F130" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="G130" s="3" t="s">
-        <v>622</v>
-      </c>
-      <c r="H130" s="3" t="s">
-        <v>563</v>
-      </c>
-      <c r="I130" s="15" t="s">
-        <v>564</v>
+      <c r="E130" s="5"/>
+      <c r="F130" s="3"/>
+      <c r="G130" t="s">
+        <v>544</v>
+      </c>
+      <c r="H130" t="s">
+        <v>672</v>
+      </c>
+      <c r="I130" s="6" t="s">
+        <v>673</v>
       </c>
       <c r="J130" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
       </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131" s="5" t="s">
-        <v>565</v>
+        <v>555</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>459</v>
+        <v>556</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>566</v>
+        <v>641</v>
       </c>
       <c r="D131" s="5" t="s">
-        <v>27</v>
+        <v>705</v>
       </c>
       <c r="E131" s="5"/>
-      <c r="F131" s="5" t="s">
-        <v>126</v>
-      </c>
+      <c r="F131" s="5"/>
       <c r="G131" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="H131" s="5" t="s">
-        <v>567</v>
-      </c>
-      <c r="I131" s="15" t="s">
-        <v>568</v>
+        <v>423</v>
+      </c>
+      <c r="H131" s="5"/>
+      <c r="I131" s="8" t="s">
+        <v>557</v>
       </c>
       <c r="J131" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A132" s="5" t="s">
-        <v>569</v>
-      </c>
-      <c r="B132" s="5" t="s">
-        <v>570</v>
+      <c r="A132" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>559</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>654</v>
-      </c>
-      <c r="D132" s="5" t="s">
-        <v>705</v>
-      </c>
-      <c r="E132" s="5"/>
-      <c r="F132" s="5"/>
-      <c r="G132" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="H132" t="s">
-        <v>571</v>
-      </c>
-      <c r="I132" s="8" t="s">
-        <v>572</v>
+        <v>560</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="E132" t="s">
+        <v>561</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="G132" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="H132" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="I132" s="15" t="s">
+        <v>564</v>
       </c>
       <c r="J132" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
-        <v>573</v>
+        <v>565</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>574</v>
+        <v>459</v>
       </c>
       <c r="C133" s="5" t="s">
-        <v>632</v>
+        <v>566</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>103</v>
+        <v>27</v>
       </c>
       <c r="E133" s="5"/>
       <c r="F133" s="5" t="s">
-        <v>575</v>
+        <v>126</v>
       </c>
       <c r="G133" s="5" t="s">
-        <v>222</v>
+        <v>127</v>
       </c>
       <c r="H133" s="5" t="s">
-        <v>576</v>
+        <v>567</v>
       </c>
       <c r="I133" s="15" t="s">
-        <v>577</v>
+        <v>568</v>
       </c>
       <c r="J133" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>578</v>
-      </c>
-      <c r="B134" t="s">
-        <v>581</v>
+      <c r="A134" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="B134" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="C134" s="5" t="s">
+        <v>654</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>705</v>
       </c>
-      <c r="G134" t="s">
-        <v>288</v>
-      </c>
-      <c r="H134" s="5" t="s">
-        <v>582</v>
+      <c r="E134" s="5"/>
+      <c r="F134" s="5"/>
+      <c r="G134" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="H134" t="s">
+        <v>571</v>
       </c>
       <c r="I134" s="8" t="s">
-        <v>583</v>
+        <v>572</v>
       </c>
       <c r="J134" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135" s="5" t="s">
-        <v>578</v>
+        <v>573</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>579</v>
+        <v>574</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="D135" s="5" t="s">
-        <v>705</v>
+        <v>103</v>
       </c>
       <c r="E135" s="5"/>
-      <c r="F135" s="5"/>
+      <c r="F135" s="5" t="s">
+        <v>575</v>
+      </c>
       <c r="G135" s="5" t="s">
-        <v>408</v>
+        <v>222</v>
       </c>
       <c r="H135" s="5" t="s">
-        <v>409</v>
-      </c>
-      <c r="I135" s="8" t="s">
-        <v>580</v>
+        <v>576</v>
+      </c>
+      <c r="I135" s="15" t="s">
+        <v>577</v>
       </c>
       <c r="J135" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>606</v>
+        <v>578</v>
       </c>
       <c r="B136" t="s">
-        <v>478</v>
-      </c>
-      <c r="C136" s="5" t="s">
-        <v>653</v>
+        <v>581</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>710</v>
-      </c>
-      <c r="E136" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F136" t="s">
-        <v>607</v>
+        <v>705</v>
       </c>
       <c r="G136" t="s">
-        <v>624</v>
-      </c>
-      <c r="H136" t="s">
-        <v>608</v>
-      </c>
-      <c r="I136" s="6" t="s">
-        <v>609</v>
+        <v>288</v>
+      </c>
+      <c r="H136" s="5" t="s">
+        <v>582</v>
+      </c>
+      <c r="I136" s="8" t="s">
+        <v>583</v>
       </c>
       <c r="J136" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A137" s="5" t="s">
-        <v>584</v>
+        <v>578</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>585</v>
-      </c>
-      <c r="C137" s="5"/>
+        <v>579</v>
+      </c>
+      <c r="C137" s="5" t="s">
+        <v>634</v>
+      </c>
       <c r="D137" s="5" t="s">
         <v>705</v>
       </c>
       <c r="E137" s="5"/>
       <c r="F137" s="5"/>
       <c r="G137" s="5" t="s">
-        <v>54</v>
+        <v>408</v>
       </c>
       <c r="H137" s="5" t="s">
-        <v>586</v>
+        <v>409</v>
       </c>
       <c r="I137" s="8" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
       <c r="J137" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A138" s="5" t="s">
-        <v>588</v>
-      </c>
-      <c r="B138" s="5" t="s">
-        <v>589</v>
+      <c r="A138" t="s">
+        <v>606</v>
+      </c>
+      <c r="B138" t="s">
+        <v>478</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>612</v>
+        <v>653</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>705</v>
-      </c>
-      <c r="E138" s="5"/>
-      <c r="F138" s="5"/>
-      <c r="G138" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H138" s="5" t="s">
-        <v>590</v>
-      </c>
-      <c r="I138" s="8" t="s">
-        <v>591</v>
+        <v>710</v>
+      </c>
+      <c r="E138" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F138" t="s">
+        <v>607</v>
+      </c>
+      <c r="G138" t="s">
+        <v>624</v>
+      </c>
+      <c r="H138" t="s">
+        <v>608</v>
+      </c>
+      <c r="I138" s="6" t="s">
+        <v>609</v>
       </c>
       <c r="J138" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139" s="5" t="s">
-        <v>592</v>
+        <v>584</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>593</v>
-      </c>
-      <c r="C139" s="5" t="s">
-        <v>643</v>
-      </c>
+        <v>585</v>
+      </c>
+      <c r="C139" s="5"/>
       <c r="D139" s="5" t="s">
         <v>705</v>
       </c>
@@ -7175,52 +7205,54 @@
         <v>54</v>
       </c>
       <c r="H139" s="5" t="s">
-        <v>594</v>
+        <v>586</v>
       </c>
       <c r="I139" s="8" t="s">
-        <v>595</v>
+        <v>587</v>
       </c>
       <c r="J139" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
       </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
-        <v>743</v>
-      </c>
-      <c r="B140" t="s">
-        <v>744</v>
+      <c r="A140" s="5" t="s">
+        <v>588</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>589</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>757</v>
-      </c>
-      <c r="D140" t="s">
-        <v>755</v>
-      </c>
-      <c r="E140" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G140" t="s">
-        <v>79</v>
-      </c>
-      <c r="I140" s="6" t="s">
-        <v>745</v>
-      </c>
-      <c r="J140" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
+        <v>612</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>705</v>
+      </c>
+      <c r="E140" s="5"/>
+      <c r="F140" s="5"/>
+      <c r="G140" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H140" s="5" t="s">
+        <v>590</v>
+      </c>
+      <c r="I140" s="8" t="s">
+        <v>591</v>
+      </c>
+      <c r="J140" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
       </c>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="C141" s="5" t="s">
-        <v>651</v>
+        <v>643</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>705</v>
@@ -7228,75 +7260,131 @@
       <c r="E141" s="5"/>
       <c r="F141" s="5"/>
       <c r="G141" s="5" t="s">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="H141" s="5" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="I141" s="8" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="J141" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A142" s="5" t="s">
-        <v>599</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="C142" s="5"/>
-      <c r="D142" s="5" t="s">
-        <v>27</v>
+      <c r="A142" t="s">
+        <v>743</v>
+      </c>
+      <c r="B142" t="s">
+        <v>744</v>
+      </c>
+      <c r="C142" s="5" t="s">
+        <v>757</v>
+      </c>
+      <c r="D142" t="s">
+        <v>755</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F142" s="5" t="s">
-        <v>600</v>
+        <v>78</v>
       </c>
       <c r="G142" t="s">
-        <v>429</v>
-      </c>
-      <c r="H142" s="5" t="s">
-        <v>450</v>
-      </c>
-      <c r="I142" s="15" t="s">
-        <v>601</v>
-      </c>
-      <c r="J142" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
+        <v>79</v>
+      </c>
+      <c r="I142" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="J142" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
       </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143" s="5" t="s">
-        <v>690</v>
+        <v>596</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>691</v>
-      </c>
-      <c r="C143" s="5"/>
+        <v>589</v>
+      </c>
+      <c r="C143" s="5" t="s">
+        <v>651</v>
+      </c>
       <c r="D143" s="5" t="s">
-        <v>713</v>
-      </c>
-      <c r="E143" s="5" t="s">
-        <v>78</v>
-      </c>
+        <v>705</v>
+      </c>
+      <c r="E143" s="5"/>
       <c r="F143" s="5"/>
       <c r="G143" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H143" s="5" t="s">
+        <v>597</v>
+      </c>
+      <c r="I143" s="8" t="s">
+        <v>598</v>
+      </c>
+      <c r="J143" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A144" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="B144" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="C144" s="5"/>
+      <c r="D144" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E144" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F144" s="5" t="s">
+        <v>600</v>
+      </c>
+      <c r="G144" t="s">
+        <v>429</v>
+      </c>
+      <c r="H144" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="I144" s="15" t="s">
+        <v>601</v>
+      </c>
+      <c r="J144" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A145" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="B145" s="5" t="s">
+        <v>691</v>
+      </c>
+      <c r="C145" s="5"/>
+      <c r="D145" s="5" t="s">
+        <v>713</v>
+      </c>
+      <c r="E145" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="H143" s="5" t="s">
+      <c r="F145" s="5"/>
+      <c r="G145" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="H145" s="5" t="s">
         <v>692</v>
       </c>
-      <c r="I143" s="6" t="s">
+      <c r="I145" s="6" t="s">
         <v>693</v>
       </c>
-      <c r="J143" s="9" t="str">
+      <c r="J145" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=sosthene.yamale@umontreal.ca</v>
       </c>
@@ -7309,85 +7397,87 @@
     <hyperlink ref="I18" r:id="rId3" display="mailto:hugo.bernier@umontreal.ca" xr:uid="{3F591457-DA50-462E-B1CA-F2F56ED9E3DD}"/>
     <hyperlink ref="I77" r:id="rId4" xr:uid="{4822C834-E5A8-42FD-9734-374BFC718C85}"/>
     <hyperlink ref="I11" r:id="rId5" display="mailto:magalie.beaudoin@umontreal.ca" xr:uid="{2D976BF0-B68A-46E5-8412-BA8BC43FD26D}"/>
-    <hyperlink ref="I112" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
+    <hyperlink ref="I114" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
     <hyperlink ref="I5" r:id="rId7" display="mailto:nadege.arsa@bib.umontreal.ca" xr:uid="{408AF5A3-35ED-4BF5-92B9-1B21C0C475D9}"/>
     <hyperlink ref="I21" r:id="rId8" display="mailto:simon.blais.longtin@umontreal.ca" xr:uid="{EA917AC7-9087-435B-A6E7-3AE1885514AA}"/>
-    <hyperlink ref="I93" r:id="rId9" xr:uid="{8ABC26E9-CF81-491C-8A28-B209E6620D2A}"/>
-    <hyperlink ref="I138" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
+    <hyperlink ref="I94" r:id="rId9" xr:uid="{8ABC26E9-CF81-491C-8A28-B209E6620D2A}"/>
+    <hyperlink ref="I140" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
     <hyperlink ref="I38" r:id="rId11" xr:uid="{7D21070C-9A14-48DF-982E-D995A034BDAD}"/>
-    <hyperlink ref="I134" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
+    <hyperlink ref="I136" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
     <hyperlink ref="I75" r:id="rId13" xr:uid="{DCABBE8B-8789-4957-9A88-F8585AD53BBC}"/>
-    <hyperlink ref="I115" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
+    <hyperlink ref="I117" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
     <hyperlink ref="I52" r:id="rId15" xr:uid="{1383A46C-5C1D-4621-B4BC-67AD012D7CF5}"/>
-    <hyperlink ref="I82" r:id="rId16" xr:uid="{29D9619F-F3A7-41E8-AE0F-DEBBF802D53A}"/>
+    <hyperlink ref="I83" r:id="rId16" xr:uid="{29D9619F-F3A7-41E8-AE0F-DEBBF802D53A}"/>
     <hyperlink ref="I33" r:id="rId17" xr:uid="{9E8CD31B-437A-49A0-BA12-85176E0D9431}"/>
-    <hyperlink ref="I117" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
+    <hyperlink ref="I119" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
     <hyperlink ref="I78" r:id="rId19" xr:uid="{3B502B79-2DDE-44A3-908B-3CB04ED1101E}"/>
     <hyperlink ref="I19" r:id="rId20" xr:uid="{BAE0697B-7739-4A42-9702-C285F03D0F77}"/>
     <hyperlink ref="I55" r:id="rId21" xr:uid="{E1BC7B04-B072-447B-9137-59A28141883D}"/>
-    <hyperlink ref="I107" r:id="rId22" xr:uid="{BEDF45F1-312C-4FF5-B4F5-1D1C7E487C0A}"/>
+    <hyperlink ref="I109" r:id="rId22" xr:uid="{BEDF45F1-312C-4FF5-B4F5-1D1C7E487C0A}"/>
     <hyperlink ref="I66" r:id="rId23" xr:uid="{6E82D57D-36A4-4928-AD91-BE73FFC7C389}"/>
-    <hyperlink ref="I84" r:id="rId24" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
-    <hyperlink ref="I102" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
-    <hyperlink ref="I135" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
-    <hyperlink ref="I91" r:id="rId27" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
-    <hyperlink ref="I92" r:id="rId28" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
-    <hyperlink ref="I97" r:id="rId29" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
-    <hyperlink ref="I114" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
-    <hyperlink ref="I129" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
-    <hyperlink ref="I132" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
-    <hyperlink ref="I137" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
-    <hyperlink ref="I139" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
-    <hyperlink ref="I141" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
+    <hyperlink ref="I85" r:id="rId24" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
+    <hyperlink ref="I104" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
+    <hyperlink ref="I137" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
+    <hyperlink ref="I92" r:id="rId27" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
+    <hyperlink ref="I93" r:id="rId28" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
+    <hyperlink ref="I98" r:id="rId29" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
+    <hyperlink ref="I116" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
+    <hyperlink ref="I131" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
+    <hyperlink ref="I134" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
+    <hyperlink ref="I139" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
+    <hyperlink ref="I141" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
+    <hyperlink ref="I143" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
     <hyperlink ref="I17" r:id="rId36" xr:uid="{E26D4CB1-6F14-4277-AD54-18A052872B6B}"/>
-    <hyperlink ref="I136" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
+    <hyperlink ref="I138" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
     <hyperlink ref="I9" r:id="rId38" xr:uid="{2E646106-878B-4504-8874-8750F3CAA7CB}"/>
     <hyperlink ref="I40" r:id="rId39" xr:uid="{902A8808-023C-4EA1-833E-F687288B12ED}"/>
-    <hyperlink ref="I128" r:id="rId40" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
-    <hyperlink ref="I119" r:id="rId41" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
+    <hyperlink ref="I130" r:id="rId40" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
+    <hyperlink ref="I121" r:id="rId41" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
     <hyperlink ref="I54" r:id="rId42" xr:uid="{ABEB73EB-E336-4619-ADE1-0AE567E81306}"/>
     <hyperlink ref="I32" r:id="rId43" xr:uid="{E819F1D0-ED89-4281-B222-20D0A6AC8A49}"/>
-    <hyperlink ref="I143" r:id="rId44" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
+    <hyperlink ref="I145" r:id="rId44" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
     <hyperlink ref="I20" r:id="rId45" xr:uid="{A4113BC8-FD33-4D47-854C-D964ED926E7F}"/>
     <hyperlink ref="I30" r:id="rId46" xr:uid="{7233E394-0474-4122-B129-E1E8DB3D4B70}"/>
-    <hyperlink ref="I116" r:id="rId47" xr:uid="{0924E3CD-F2EB-4646-BC88-767228D5A8FD}"/>
+    <hyperlink ref="I118" r:id="rId47" xr:uid="{0924E3CD-F2EB-4646-BC88-767228D5A8FD}"/>
     <hyperlink ref="I76" r:id="rId48" xr:uid="{FAC375AB-8F54-402B-A4F5-618AA479650B}"/>
     <hyperlink ref="I4" r:id="rId49" xr:uid="{12EFBBCC-308A-4E41-92F6-4E78BB9E9458}"/>
     <hyperlink ref="I22" r:id="rId50" xr:uid="{CAA07608-BC3B-468C-819E-F94EE0396C78}"/>
-    <hyperlink ref="I140" r:id="rId51" xr:uid="{B3DF72B2-3730-4A9C-8195-E5B8FCD87C3B}"/>
-    <hyperlink ref="I121" r:id="rId52" xr:uid="{518A2404-8625-4373-BDE5-E73718B1440B}"/>
+    <hyperlink ref="I142" r:id="rId51" xr:uid="{B3DF72B2-3730-4A9C-8195-E5B8FCD87C3B}"/>
+    <hyperlink ref="I123" r:id="rId52" xr:uid="{518A2404-8625-4373-BDE5-E73718B1440B}"/>
     <hyperlink ref="I34" r:id="rId53" xr:uid="{B383F9BF-E7F0-4AFA-A217-1F3A922E55BA}"/>
-    <hyperlink ref="I142" r:id="rId54" xr:uid="{D2BBF900-A9C8-4032-A387-C01245244DE0}"/>
+    <hyperlink ref="I144" r:id="rId54" xr:uid="{D2BBF900-A9C8-4032-A387-C01245244DE0}"/>
     <hyperlink ref="I53" r:id="rId55" xr:uid="{79C702A2-295C-4D37-BA6F-DD2C408C75BD}"/>
     <hyperlink ref="I24" r:id="rId56" xr:uid="{761F418D-12C5-4F41-8071-6031B8FBF83B}"/>
-    <hyperlink ref="I106" r:id="rId57" xr:uid="{C91A1DE6-A8FA-4481-9E51-1DB52F17F3CC}"/>
-    <hyperlink ref="I133" r:id="rId58" xr:uid="{131478F3-61ED-4B04-9E66-6F771D0E53F1}"/>
-    <hyperlink ref="I100" r:id="rId59" xr:uid="{C3534DCE-62CB-4016-B559-AE879ED29221}"/>
+    <hyperlink ref="I108" r:id="rId57" xr:uid="{C91A1DE6-A8FA-4481-9E51-1DB52F17F3CC}"/>
+    <hyperlink ref="I135" r:id="rId58" xr:uid="{131478F3-61ED-4B04-9E66-6F771D0E53F1}"/>
+    <hyperlink ref="I101" r:id="rId59" xr:uid="{C3534DCE-62CB-4016-B559-AE879ED29221}"/>
     <hyperlink ref="I73" r:id="rId60" xr:uid="{598291DC-2DD2-464C-A65A-36D0759E8852}"/>
     <hyperlink ref="I65" r:id="rId61" xr:uid="{55FAFEEC-7E6A-4254-BBB4-020FD859DB23}"/>
-    <hyperlink ref="I104" r:id="rId62" xr:uid="{E35BC25D-CA56-4FFF-B93C-72EBCAD05C3B}"/>
+    <hyperlink ref="I106" r:id="rId62" xr:uid="{E35BC25D-CA56-4FFF-B93C-72EBCAD05C3B}"/>
     <hyperlink ref="I46" r:id="rId63" xr:uid="{6B64B7D5-5396-4382-9ECB-D065E5B3F7C4}"/>
     <hyperlink ref="I58" r:id="rId64" xr:uid="{A6C3CD82-A312-40D2-B320-33ED739C6E60}"/>
-    <hyperlink ref="I86" r:id="rId65" xr:uid="{1754B384-2B8D-46A2-8C89-BDF617522295}"/>
-    <hyperlink ref="I113" r:id="rId66" xr:uid="{99B099F4-5E98-4B25-B2EB-EE4C451DC6EE}"/>
+    <hyperlink ref="I87" r:id="rId65" xr:uid="{1754B384-2B8D-46A2-8C89-BDF617522295}"/>
+    <hyperlink ref="I115" r:id="rId66" xr:uid="{99B099F4-5E98-4B25-B2EB-EE4C451DC6EE}"/>
     <hyperlink ref="I60" r:id="rId67" xr:uid="{1C080271-6DB7-4810-99C8-8FF2BA5EA430}"/>
     <hyperlink ref="I64" r:id="rId68" xr:uid="{6A0B0BD3-8872-437B-9CD4-6D8D7D98A4F9}"/>
-    <hyperlink ref="I122" r:id="rId69" xr:uid="{CE8C2C5F-3292-4BA9-A27E-19AF9661C907}"/>
+    <hyperlink ref="I124" r:id="rId69" xr:uid="{CE8C2C5F-3292-4BA9-A27E-19AF9661C907}"/>
     <hyperlink ref="I12" r:id="rId70" xr:uid="{F1246003-4D15-4FC5-9F7D-6CE88CAF21A8}"/>
-    <hyperlink ref="I131" r:id="rId71" xr:uid="{BB3A0149-0DD5-481B-8662-8134BB3FCECC}"/>
-    <hyperlink ref="I127" r:id="rId72" xr:uid="{52D55C85-F393-43A8-95EF-F57618BB179E}"/>
-    <hyperlink ref="I87" r:id="rId73" xr:uid="{CAB4CB00-83BC-4384-BF0E-208B7456F243}"/>
-    <hyperlink ref="I95" r:id="rId74" xr:uid="{4B80B43B-B062-42B6-A1CE-F4CE03CDED46}"/>
+    <hyperlink ref="I133" r:id="rId71" xr:uid="{BB3A0149-0DD5-481B-8662-8134BB3FCECC}"/>
+    <hyperlink ref="I129" r:id="rId72" xr:uid="{52D55C85-F393-43A8-95EF-F57618BB179E}"/>
+    <hyperlink ref="I88" r:id="rId73" xr:uid="{CAB4CB00-83BC-4384-BF0E-208B7456F243}"/>
+    <hyperlink ref="I96" r:id="rId74" xr:uid="{4B80B43B-B062-42B6-A1CE-F4CE03CDED46}"/>
     <hyperlink ref="I8" r:id="rId75" xr:uid="{BC76BE28-D367-49FE-95A3-98BB93483999}"/>
     <hyperlink ref="I48" r:id="rId76" xr:uid="{8598B756-3A70-45A7-ABB5-3EDBEF50BAF4}"/>
-    <hyperlink ref="I130" r:id="rId77" xr:uid="{07544A5C-3F38-40A4-9945-4E56F5EFFCF4}"/>
+    <hyperlink ref="I132" r:id="rId77" xr:uid="{07544A5C-3F38-40A4-9945-4E56F5EFFCF4}"/>
     <hyperlink ref="I28" r:id="rId78" xr:uid="{C341566A-DC48-4D81-91C1-E1CD275F4D60}"/>
     <hyperlink ref="I14" r:id="rId79" xr:uid="{FAAE6B3B-3F31-452F-868E-B6C650D083E8}"/>
+    <hyperlink ref="I81" r:id="rId80" xr:uid="{09E37274-D8A2-4A0B-832A-E187D6213477}"/>
+    <hyperlink ref="I103" r:id="rId81" xr:uid="{89D21B16-595D-4AC9-BFE9-2C29DBC329A2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId80"/>
+  <pageSetup orientation="portrait" r:id="rId82"/>
   <tableParts count="1">
-    <tablePart r:id="rId81"/>
+    <tablePart r:id="rId83"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7588,6 +7678,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7596,15 +7695,6 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7627,6 +7717,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7641,12 +7739,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Changements aux coordonnées de Julie Ouellette
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4B5ED7-8940-4F05-B457-5E7968D53BBF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B34FC95A-DAAB-4169-BD07-516977F0F067}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5460" yWindow="3555" windowWidth="30315" windowHeight="28125" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5460" yWindow="3560" windowWidth="30320" windowHeight="28130" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3047,21 +3047,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J144"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="33.85546875" customWidth="1"/>
-    <col min="4" max="4" width="45.28515625" customWidth="1"/>
-    <col min="5" max="5" width="58.140625" customWidth="1"/>
+    <col min="3" max="3" width="33.81640625" customWidth="1"/>
+    <col min="4" max="4" width="45.26953125" customWidth="1"/>
+    <col min="5" max="5" width="58.1796875" customWidth="1"/>
     <col min="6" max="6" width="58" customWidth="1"/>
-    <col min="7" max="7" width="70.85546875" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="41.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="86.5703125" customWidth="1"/>
+    <col min="7" max="7" width="70.81640625" customWidth="1"/>
+    <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="86.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3093,7 +3093,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alexandre.amar-zifkin@umontreal.ca</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.angers@umontreal.ca</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>728</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=busch.antenor.alexandre@umontreal.ca</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nadege.arsa@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
@@ -3247,7 +3247,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=denis.arvisais@umontreal.ca</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>38</v>
       </c>
@@ -3280,7 +3280,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.attia@umontreal.ca</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>45</v>
       </c>
@@ -3309,7 +3309,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=prlaval@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.bastien@umontreal.ca</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>57</v>
       </c>
@@ -3367,7 +3367,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magalie.beaudoin@umontreal.ca</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>64</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maryna.beaulieu@umontreal.ca</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>70</v>
       </c>
@@ -3430,7 +3430,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.begin-poissant@umontreal.ca</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>712</v>
       </c>
@@ -3461,7 +3461,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nima.behforouz@umontreal.ca</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>75</v>
       </c>
@@ -3491,7 +3491,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.belanger@umontreal.ca</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>82</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amy.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>87</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amelie.bernard@umontreal.ca</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>92</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=hugo.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>92</v>
       </c>
@@ -3609,7 +3609,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>693</v>
       </c>
@@ -3640,7 +3640,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cathy.bingoye@umontreal.ca</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
         <v>100</v>
       </c>
@@ -3671,7 +3671,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon.blais.longtin@umontreal.ca</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>736</v>
       </c>
@@ -3696,7 +3696,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guy.blondeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>106</v>
       </c>
@@ -3726,7 +3726,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tatiana.talpa@umontreal.ca</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>112</v>
       </c>
@@ -3752,7 +3752,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=joanna.bodnar@umontreal.ca</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>116</v>
       </c>
@@ -3782,7 +3782,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alain.borsi@umontreal.ca</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>123</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.p.bouchard@umontreal.ca</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
         <v>130</v>
       </c>
@@ -3844,7 +3844,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refdroi@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>136</v>
       </c>
@@ -3877,7 +3877,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=myriam.boyer@umontreal.ca</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
         <v>140</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guylaine.brazeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>698</v>
       </c>
@@ -3935,7 +3935,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-marie.brien.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>144</v>
       </c>
@@ -3963,7 +3963,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sophie.brisebois@umontreal.ca</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>680</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tanya.buchet@umontreal.ca</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>149</v>
       </c>
@@ -4023,7 +4023,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fanny.c.brochu@umontreal.ca</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>745</v>
       </c>
@@ -4051,7 +4051,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thierry.caballero@umontreal.ca</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>153</v>
       </c>
@@ -4082,7 +4082,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=delphine.cado@umontreal.ca</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>160</v>
       </c>
@@ -4111,7 +4111,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=siv.kham.chao@umontreal.ca</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>165</v>
       </c>
@@ -4142,7 +4142,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=laurence.charest@umontreal.ca</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>172</v>
       </c>
@@ -4166,7 +4166,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=annick.charette@umontreal.ca</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>748</v>
       </c>
@@ -4194,7 +4194,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=wassif.cheikh@umontreal.ca</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
         <v>176</v>
       </c>
@@ -4222,7 +4222,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mailto:thien-huong.che-quang@umontreal.ca</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>178</v>
       </c>
@@ -4253,7 +4253,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah.cherrier@umontreal.ca</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
         <v>184</v>
       </c>
@@ -4283,7 +4283,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emir.chouchane@umontreal.ca</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
         <v>190</v>
       </c>
@@ -4314,7 +4314,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=accessibilite@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>195</v>
       </c>
@@ -4347,7 +4347,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benjamin.constantineau@umontreal.ca</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
         <v>202</v>
       </c>
@@ -4378,7 +4378,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon-pierre.crevier@umontreal.ca</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
         <v>208</v>
       </c>
@@ -4409,7 +4409,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marc-olivier.croteau@umontreal.ca</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
         <v>213</v>
       </c>
@@ -4440,7 +4440,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.dalpe@umontreal.ca</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
         <v>219</v>
       </c>
@@ -4471,7 +4471,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=morgane.de.bellefeuille@umontreal.ca</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>226</v>
       </c>
@@ -4502,7 +4502,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=Indiana.delsart@umontreal.ca</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
         <v>232</v>
       </c>
@@ -4533,7 +4533,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=dominic.desaulniers@umontreal.ca</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>238</v>
       </c>
@@ -4562,7 +4562,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.desrosiers@umontreal.ca</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>243</v>
       </c>
@@ -4589,7 +4589,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.dubois.mercier@umontreal.ca</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>247</v>
       </c>
@@ -4620,7 +4620,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jean-francois.durnin@umontreal.ca</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>675</v>
       </c>
@@ -4651,7 +4651,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=taline.ekmekjian@umontreal.ca</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>253</v>
       </c>
@@ -4678,7 +4678,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=judith.fafard-larose@umontreal.ca</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>257</v>
       </c>
@@ -4711,7 +4711,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>262</v>
       </c>
@@ -4744,7 +4744,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=c.fortier@umontreal.ca</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>268</v>
       </c>
@@ -4771,7 +4771,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>274</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nino.gabrielli@umontreal.ca</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
         <v>280</v>
       </c>
@@ -4831,7 +4831,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-pierre.gadoua@umontreal.ca</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
         <v>284</v>
       </c>
@@ -4862,7 +4862,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cynthia.gagne.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>291</v>
       </c>
@@ -4888,7 +4888,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>291</v>
       </c>
@@ -4916,7 +4916,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
         <v>297</v>
       </c>
@@ -4946,7 +4946,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marjorie.gauchier@umontreal.ca</v>
       </c>
     </row>
-    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>727</v>
       </c>
@@ -4975,7 +4975,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=lucie.geoffroy@umontreal.ca</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
         <v>303</v>
       </c>
@@ -5002,7 +5002,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
       </c>
     </row>
-    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
         <v>306</v>
       </c>
@@ -5035,7 +5035,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.giguere.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>725</v>
       </c>
@@ -5066,7 +5066,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.hainault@umontreal.ca</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>311</v>
       </c>
@@ -5097,7 +5097,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
         <v>316</v>
       </c>
@@ -5128,7 +5128,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>322</v>
       </c>
@@ -5158,7 +5158,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>726</v>
       </c>
@@ -5189,7 +5189,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=natalia.jabinschi@umontreal.ca</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
         <v>328</v>
       </c>
@@ -5218,7 +5218,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
         <v>333</v>
       </c>
@@ -5249,7 +5249,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>338</v>
       </c>
@@ -5276,7 +5276,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
       </c>
     </row>
-    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>731</v>
       </c>
@@ -5305,7 +5305,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pierre-yves.lafleur@umontreal.ca</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
         <v>342</v>
       </c>
@@ -5332,7 +5332,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>344</v>
       </c>
@@ -5359,7 +5359,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
         <v>347</v>
       </c>
@@ -5392,7 +5392,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
       </c>
     </row>
-    <row r="79" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
         <v>353</v>
       </c>
@@ -5425,7 +5425,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
       </c>
     </row>
-    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A80" s="18" t="s">
         <v>756</v>
       </c>
@@ -5454,7 +5454,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-josee.lapalme@umontreal.ca</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
         <v>358</v>
       </c>
@@ -5487,7 +5487,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>362</v>
       </c>
@@ -5514,7 +5514,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
         <v>366</v>
       </c>
@@ -5545,7 +5545,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>371</v>
       </c>
@@ -5576,7 +5576,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
         <v>376</v>
       </c>
@@ -5607,7 +5607,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
         <v>381</v>
       </c>
@@ -5640,7 +5640,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
         <v>387</v>
       </c>
@@ -5670,7 +5670,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
         <v>391</v>
       </c>
@@ -5701,7 +5701,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
         <v>396</v>
       </c>
@@ -5734,7 +5734,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
         <v>396</v>
       </c>
@@ -5760,7 +5760,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
         <v>402</v>
       </c>
@@ -5789,7 +5789,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
         <v>406</v>
       </c>
@@ -5818,7 +5818,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
         <v>411</v>
       </c>
@@ -5846,7 +5846,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
         <v>415</v>
       </c>
@@ -5877,7 +5877,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
         <v>420</v>
       </c>
@@ -5908,7 +5908,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
         <v>426</v>
       </c>
@@ -5938,7 +5938,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
       </c>
     </row>
-    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
         <v>432</v>
       </c>
@@ -5967,7 +5967,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
       </c>
     </row>
-    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
         <v>436</v>
       </c>
@@ -5998,7 +5998,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="3" t="s">
         <v>442</v>
       </c>
@@ -6029,7 +6029,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="s">
         <v>447</v>
       </c>
@@ -6060,7 +6060,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="5" t="s">
         <v>452</v>
       </c>
@@ -6091,7 +6091,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=assia.mourid@umontreal.ca</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" s="18" t="s">
         <v>761</v>
       </c>
@@ -6122,7 +6122,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.moreau@umontreal.ca</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>458</v>
       </c>
@@ -6153,7 +6153,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
       </c>
     </row>
-    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A104" s="3" t="s">
         <v>463</v>
       </c>
@@ -6184,7 +6184,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="105" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
         <v>467</v>
       </c>
@@ -6215,7 +6215,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
         <v>473</v>
       </c>
@@ -6241,7 +6241,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
         <v>477</v>
       </c>
@@ -6254,12 +6254,12 @@
       <c r="D107" s="5" t="s">
         <v>706</v>
       </c>
-      <c r="E107" s="11"/>
-      <c r="F107" s="3" t="s">
-        <v>542</v>
-      </c>
+      <c r="E107" t="s">
+        <v>67</v>
+      </c>
+      <c r="F107" s="3"/>
       <c r="G107" t="s">
-        <v>543</v>
+        <v>29</v>
       </c>
       <c r="H107" s="5" t="s">
         <v>479</v>
@@ -6272,7 +6272,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
         <v>481</v>
       </c>
@@ -6299,7 +6299,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>486</v>
       </c>
@@ -6329,7 +6329,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
         <v>491</v>
       </c>
@@ -6360,7 +6360,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
         <v>491</v>
       </c>
@@ -6393,7 +6393,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
         <v>500</v>
       </c>
@@ -6424,7 +6424,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
         <v>504</v>
       </c>
@@ -6453,7 +6453,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="s">
         <v>508</v>
       </c>
@@ -6484,7 +6484,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A115" s="5" t="s">
         <v>514</v>
       </c>
@@ -6513,7 +6513,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>518</v>
       </c>
@@ -6540,7 +6540,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>734</v>
       </c>
@@ -6568,7 +6568,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>522</v>
       </c>
@@ -6593,7 +6593,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>724</v>
       </c>
@@ -6622,7 +6622,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>662</v>
       </c>
@@ -6651,7 +6651,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>526</v>
       </c>
@@ -6681,7 +6681,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>742</v>
       </c>
@@ -6709,7 +6709,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
         <v>531</v>
       </c>
@@ -6737,7 +6737,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A124" s="5" t="s">
         <v>534</v>
       </c>
@@ -6766,7 +6766,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>538</v>
       </c>
@@ -6789,7 +6789,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A126" s="3" t="s">
         <v>540</v>
       </c>
@@ -6820,7 +6820,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A127" s="3" t="s">
         <v>546</v>
       </c>
@@ -6847,7 +6847,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
         <v>549</v>
       </c>
@@ -6877,7 +6877,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>667</v>
       </c>
@@ -6906,7 +6906,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A130" s="5" t="s">
         <v>554</v>
       </c>
@@ -6933,7 +6933,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A131" s="3" t="s">
         <v>557</v>
       </c>
@@ -6966,7 +6966,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
         <v>564</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A133" s="5" t="s">
         <v>568</v>
       </c>
@@ -7026,7 +7026,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A134" s="5" t="s">
         <v>572</v>
       </c>
@@ -7057,7 +7057,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>577</v>
       </c>
@@ -7081,7 +7081,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A136" s="5" t="s">
         <v>577</v>
       </c>
@@ -7110,7 +7110,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>605</v>
       </c>
@@ -7143,7 +7143,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="s">
         <v>583</v>
       </c>
@@ -7170,7 +7170,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A139" s="5" t="s">
         <v>587</v>
       </c>
@@ -7199,7 +7199,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A140" s="5" t="s">
         <v>591</v>
       </c>
@@ -7228,7 +7228,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>739</v>
       </c>
@@ -7255,7 +7255,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="s">
         <v>595</v>
       </c>
@@ -7284,7 +7284,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="s">
         <v>598</v>
       </c>
@@ -7315,7 +7315,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A144" s="5" t="s">
         <v>686</v>
       </c>
@@ -7632,6 +7632,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7640,15 +7649,6 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7671,6 +7671,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7685,12 +7693,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(repertoire-personnel): Correctif de la direction d'attache
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B34FC95A-DAAB-4169-BD07-516977F0F067}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF13A67-887C-4A46-81CB-7D2A6B5C2D46}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5460" yWindow="3560" windowWidth="30320" windowHeight="28130" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5460" yWindow="3555" windowWidth="30315" windowHeight="28125" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="765">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="767">
   <si>
     <t>nom</t>
   </si>
@@ -2343,6 +2343,12 @@
   </si>
   <si>
     <t>diane.moreau@umontreal.ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direction de la Bibliothèque des  lettres et sciences humaines et Livres rares et collections spéciales; </t>
+  </si>
+  <si>
+    <t>Bibliothèque des lettres et sciences humaines et Service du prêt entre bibliothèques</t>
   </si>
 </sst>
 </file>
@@ -3047,21 +3053,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J144"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.453125" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="33.81640625" customWidth="1"/>
-    <col min="4" max="4" width="45.26953125" customWidth="1"/>
-    <col min="5" max="5" width="58.1796875" customWidth="1"/>
+    <col min="3" max="3" width="33.85546875" customWidth="1"/>
+    <col min="4" max="4" width="45.28515625" customWidth="1"/>
+    <col min="5" max="5" width="58.140625" customWidth="1"/>
     <col min="6" max="6" width="58" customWidth="1"/>
-    <col min="7" max="7" width="70.81640625" customWidth="1"/>
-    <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="41.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="86.54296875" customWidth="1"/>
+    <col min="7" max="7" width="70.85546875" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="86.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3093,7 +3099,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
@@ -3124,7 +3130,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alexandre.amar-zifkin@umontreal.ca</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -3157,7 +3163,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.angers@umontreal.ca</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>728</v>
       </c>
@@ -3185,7 +3191,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=busch.antenor.alexandre@umontreal.ca</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
@@ -3216,7 +3222,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nadege.arsa@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
@@ -3247,7 +3253,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=denis.arvisais@umontreal.ca</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>38</v>
       </c>
@@ -3280,7 +3286,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.attia@umontreal.ca</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>45</v>
       </c>
@@ -3309,7 +3315,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=prlaval@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -3339,7 +3345,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.bastien@umontreal.ca</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>57</v>
       </c>
@@ -3367,7 +3373,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magalie.beaudoin@umontreal.ca</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>64</v>
       </c>
@@ -3400,7 +3406,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maryna.beaulieu@umontreal.ca</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>70</v>
       </c>
@@ -3430,7 +3436,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.begin-poissant@umontreal.ca</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>712</v>
       </c>
@@ -3461,7 +3467,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nima.behforouz@umontreal.ca</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>75</v>
       </c>
@@ -3491,7 +3497,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.belanger@umontreal.ca</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>82</v>
       </c>
@@ -3524,7 +3530,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amy.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>87</v>
       </c>
@@ -3553,7 +3559,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amelie.bernard@umontreal.ca</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>92</v>
       </c>
@@ -3582,7 +3588,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=hugo.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>92</v>
       </c>
@@ -3609,7 +3615,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>693</v>
       </c>
@@ -3640,7 +3646,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cathy.bingoye@umontreal.ca</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>100</v>
       </c>
@@ -3671,7 +3677,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon.blais.longtin@umontreal.ca</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>736</v>
       </c>
@@ -3696,7 +3702,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guy.blondeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>106</v>
       </c>
@@ -3726,7 +3732,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tatiana.talpa@umontreal.ca</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>112</v>
       </c>
@@ -3752,7 +3758,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=joanna.bodnar@umontreal.ca</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>116</v>
       </c>
@@ -3782,7 +3788,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alain.borsi@umontreal.ca</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>123</v>
       </c>
@@ -3813,7 +3819,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.p.bouchard@umontreal.ca</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>130</v>
       </c>
@@ -3844,7 +3850,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refdroi@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>136</v>
       </c>
@@ -3877,7 +3883,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=myriam.boyer@umontreal.ca</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>140</v>
       </c>
@@ -3906,7 +3912,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guylaine.brazeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>698</v>
       </c>
@@ -3935,7 +3941,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-marie.brien.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>144</v>
       </c>
@@ -3963,7 +3969,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sophie.brisebois@umontreal.ca</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>680</v>
       </c>
@@ -3996,7 +4002,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tanya.buchet@umontreal.ca</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>149</v>
       </c>
@@ -4023,7 +4029,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fanny.c.brochu@umontreal.ca</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>745</v>
       </c>
@@ -4051,7 +4057,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thierry.caballero@umontreal.ca</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>153</v>
       </c>
@@ -4082,7 +4088,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=delphine.cado@umontreal.ca</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>160</v>
       </c>
@@ -4111,7 +4117,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=siv.kham.chao@umontreal.ca</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>165</v>
       </c>
@@ -4142,7 +4148,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=laurence.charest@umontreal.ca</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>172</v>
       </c>
@@ -4166,7 +4172,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=annick.charette@umontreal.ca</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>748</v>
       </c>
@@ -4194,7 +4200,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=wassif.cheikh@umontreal.ca</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>176</v>
       </c>
@@ -4222,7 +4228,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mailto:thien-huong.che-quang@umontreal.ca</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>178</v>
       </c>
@@ -4253,7 +4259,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah.cherrier@umontreal.ca</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>184</v>
       </c>
@@ -4283,7 +4289,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emir.chouchane@umontreal.ca</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>190</v>
       </c>
@@ -4314,7 +4320,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=accessibilite@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>195</v>
       </c>
@@ -4347,7 +4353,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benjamin.constantineau@umontreal.ca</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>202</v>
       </c>
@@ -4378,7 +4384,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon-pierre.crevier@umontreal.ca</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>208</v>
       </c>
@@ -4409,7 +4415,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marc-olivier.croteau@umontreal.ca</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>213</v>
       </c>
@@ -4440,7 +4446,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.dalpe@umontreal.ca</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>219</v>
       </c>
@@ -4471,7 +4477,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=morgane.de.bellefeuille@umontreal.ca</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>226</v>
       </c>
@@ -4502,7 +4508,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=Indiana.delsart@umontreal.ca</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>232</v>
       </c>
@@ -4533,7 +4539,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=dominic.desaulniers@umontreal.ca</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>238</v>
       </c>
@@ -4562,7 +4568,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.desrosiers@umontreal.ca</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>243</v>
       </c>
@@ -4589,7 +4595,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.dubois.mercier@umontreal.ca</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>247</v>
       </c>
@@ -4620,7 +4626,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jean-francois.durnin@umontreal.ca</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>675</v>
       </c>
@@ -4651,7 +4657,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=taline.ekmekjian@umontreal.ca</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>253</v>
       </c>
@@ -4678,7 +4684,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=judith.fafard-larose@umontreal.ca</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>257</v>
       </c>
@@ -4711,7 +4717,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>262</v>
       </c>
@@ -4744,7 +4750,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=c.fortier@umontreal.ca</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>268</v>
       </c>
@@ -4771,7 +4777,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
         <v>274</v>
       </c>
@@ -4802,7 +4808,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nino.gabrielli@umontreal.ca</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
         <v>280</v>
       </c>
@@ -4831,7 +4837,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-pierre.gadoua@umontreal.ca</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
         <v>284</v>
       </c>
@@ -4862,7 +4868,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cynthia.gagne.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>291</v>
       </c>
@@ -4888,7 +4894,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
         <v>291</v>
       </c>
@@ -4916,7 +4922,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>297</v>
       </c>
@@ -4946,7 +4952,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marjorie.gauchier@umontreal.ca</v>
       </c>
     </row>
-    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>727</v>
       </c>
@@ -4975,7 +4981,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=lucie.geoffroy@umontreal.ca</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>303</v>
       </c>
@@ -5002,7 +5008,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
       </c>
     </row>
-    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>306</v>
       </c>
@@ -5035,7 +5041,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.giguere.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>725</v>
       </c>
@@ -5066,7 +5072,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.hainault@umontreal.ca</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
         <v>311</v>
       </c>
@@ -5097,7 +5103,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>316</v>
       </c>
@@ -5128,7 +5134,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>322</v>
       </c>
@@ -5158,7 +5164,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>726</v>
       </c>
@@ -5189,7 +5195,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=natalia.jabinschi@umontreal.ca</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>328</v>
       </c>
@@ -5218,7 +5224,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
         <v>333</v>
       </c>
@@ -5249,7 +5255,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>338</v>
       </c>
@@ -5276,7 +5282,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
       </c>
     </row>
-    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>731</v>
       </c>
@@ -5305,7 +5311,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pierre-yves.lafleur@umontreal.ca</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
         <v>342</v>
       </c>
@@ -5332,7 +5338,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>344</v>
       </c>
@@ -5359,7 +5365,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
         <v>347</v>
       </c>
@@ -5392,7 +5398,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
       </c>
     </row>
-    <row r="79" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
         <v>353</v>
       </c>
@@ -5425,7 +5431,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
       </c>
     </row>
-    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="18" t="s">
         <v>756</v>
       </c>
@@ -5454,7 +5460,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-josee.lapalme@umontreal.ca</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
         <v>358</v>
       </c>
@@ -5487,7 +5493,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>362</v>
       </c>
@@ -5514,7 +5520,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
         <v>366</v>
       </c>
@@ -5545,7 +5551,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>371</v>
       </c>
@@ -5576,7 +5582,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
         <v>376</v>
       </c>
@@ -5607,7 +5613,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
         <v>381</v>
       </c>
@@ -5640,7 +5646,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
         <v>387</v>
       </c>
@@ -5670,7 +5676,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
         <v>391</v>
       </c>
@@ -5701,7 +5707,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>396</v>
       </c>
@@ -5734,7 +5740,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
         <v>396</v>
       </c>
@@ -5760,7 +5766,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
         <v>402</v>
       </c>
@@ -5789,7 +5795,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
         <v>406</v>
       </c>
@@ -5818,7 +5824,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
         <v>411</v>
       </c>
@@ -5846,7 +5852,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
         <v>415</v>
       </c>
@@ -5877,7 +5883,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
         <v>420</v>
       </c>
@@ -5908,7 +5914,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
         <v>426</v>
       </c>
@@ -5938,7 +5944,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
       </c>
     </row>
-    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
         <v>432</v>
       </c>
@@ -5967,7 +5973,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
       </c>
     </row>
-    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
         <v>436</v>
       </c>
@@ -5998,7 +6004,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
         <v>442</v>
       </c>
@@ -6029,7 +6035,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
         <v>447</v>
       </c>
@@ -6060,7 +6066,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
         <v>452</v>
       </c>
@@ -6091,7 +6097,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=assia.mourid@umontreal.ca</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="18" t="s">
         <v>761</v>
       </c>
@@ -6122,7 +6128,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.moreau@umontreal.ca</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>458</v>
       </c>
@@ -6153,7 +6159,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
       </c>
     </row>
-    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
         <v>463</v>
       </c>
@@ -6184,7 +6190,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="105" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
         <v>467</v>
       </c>
@@ -6215,7 +6221,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
         <v>473</v>
       </c>
@@ -6241,7 +6247,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
         <v>477</v>
       </c>
@@ -6255,11 +6261,11 @@
         <v>706</v>
       </c>
       <c r="E107" t="s">
-        <v>67</v>
+        <v>765</v>
       </c>
       <c r="F107" s="3"/>
       <c r="G107" t="s">
-        <v>29</v>
+        <v>766</v>
       </c>
       <c r="H107" s="5" t="s">
         <v>479</v>
@@ -6272,7 +6278,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
         <v>481</v>
       </c>
@@ -6299,7 +6305,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>486</v>
       </c>
@@ -6329,7 +6335,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
         <v>491</v>
       </c>
@@ -6360,7 +6366,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
         <v>491</v>
       </c>
@@ -6393,7 +6399,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
         <v>500</v>
       </c>
@@ -6424,7 +6430,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
         <v>504</v>
       </c>
@@ -6453,7 +6459,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
         <v>508</v>
       </c>
@@ -6484,7 +6490,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115" s="5" t="s">
         <v>514</v>
       </c>
@@ -6513,7 +6519,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>518</v>
       </c>
@@ -6540,7 +6546,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>734</v>
       </c>
@@ -6568,7 +6574,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>522</v>
       </c>
@@ -6593,7 +6599,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>724</v>
       </c>
@@ -6622,7 +6628,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>662</v>
       </c>
@@ -6651,7 +6657,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>526</v>
       </c>
@@ -6681,7 +6687,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>742</v>
       </c>
@@ -6709,7 +6715,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" s="5" t="s">
         <v>531</v>
       </c>
@@ -6737,7 +6743,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124" s="5" t="s">
         <v>534</v>
       </c>
@@ -6766,7 +6772,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>538</v>
       </c>
@@ -6789,7 +6795,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
         <v>540</v>
       </c>
@@ -6820,7 +6826,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
         <v>546</v>
       </c>
@@ -6847,7 +6853,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128" s="5" t="s">
         <v>549</v>
       </c>
@@ -6877,7 +6883,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>667</v>
       </c>
@@ -6906,7 +6912,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130" s="5" t="s">
         <v>554</v>
       </c>
@@ -6933,7 +6939,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
         <v>557</v>
       </c>
@@ -6966,7 +6972,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132" s="5" t="s">
         <v>564</v>
       </c>
@@ -6997,7 +7003,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
         <v>568</v>
       </c>
@@ -7026,7 +7032,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A134" s="5" t="s">
         <v>572</v>
       </c>
@@ -7057,7 +7063,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>577</v>
       </c>
@@ -7081,7 +7087,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136" s="5" t="s">
         <v>577</v>
       </c>
@@ -7110,7 +7116,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>605</v>
       </c>
@@ -7143,7 +7149,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138" s="5" t="s">
         <v>583</v>
       </c>
@@ -7170,7 +7176,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139" s="5" t="s">
         <v>587</v>
       </c>
@@ -7199,7 +7205,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A140" s="5" t="s">
         <v>591</v>
       </c>
@@ -7228,7 +7234,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>739</v>
       </c>
@@ -7255,7 +7261,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142" s="5" t="s">
         <v>595</v>
       </c>
@@ -7284,7 +7290,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143" s="5" t="s">
         <v>598</v>
       </c>
@@ -7315,7 +7321,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A144" s="5" t="s">
         <v>686</v>
       </c>
@@ -7632,15 +7638,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7649,6 +7646,15 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7671,14 +7677,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7693,4 +7691,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Retrait d'Assia Mourid
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF13A67-887C-4A46-81CB-7D2A6B5C2D46}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6D1527A-C78C-4EFF-9C36-9451491784A8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5460" yWindow="3555" windowWidth="30315" windowHeight="28125" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="767">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="761">
   <si>
     <t>nom</t>
   </si>
@@ -1404,24 +1404,6 @@
   </si>
   <si>
     <t>justine.menard.1@umontreal.ca</t>
-  </si>
-  <si>
-    <t>Mourid</t>
-  </si>
-  <si>
-    <t>Assia</t>
-  </si>
-  <si>
-    <t>assia-mourid.jpg</t>
-  </si>
-  <si>
-    <t>Sciences infirmières, gérontologie</t>
-  </si>
-  <si>
-    <t>514 343-6111, poste 1846</t>
-  </si>
-  <si>
-    <t>assia.mourid@umontreal.ca</t>
   </si>
   <si>
     <t>Murray-Samuel</t>
@@ -2708,10 +2690,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J144" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J144" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
-  <sortState ref="A2:J144">
-    <sortCondition ref="A1:A144"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J143" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J143" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
+  <sortState ref="A2:J143">
+    <sortCondition ref="A1:A143"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{4B04E1AF-0079-4AD2-81CA-E8A433733E21}" name="nom" dataDxfId="9"/>
@@ -3052,7 +3034,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J144"/>
+  <dimension ref="A1:J143"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" customWidth="1"/>
@@ -3147,7 +3129,7 @@
         <v>41</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>617</v>
+        <v>611</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>21</v>
@@ -3165,14 +3147,14 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>728</v>
+        <v>722</v>
       </c>
       <c r="B4" t="s">
-        <v>729</v>
+        <v>723</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" t="s">
-        <v>751</v>
+        <v>745</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>78</v>
@@ -3184,7 +3166,7 @@
         <v>310</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>730</v>
+        <v>724</v>
       </c>
       <c r="J4" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3264,7 +3246,7 @@
         <v>40</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>41</v>
@@ -3273,7 +3255,7 @@
         <v>42</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>618</v>
+        <v>612</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>43</v>
@@ -3297,7 +3279,7 @@
         <v>47</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
@@ -3384,16 +3366,16 @@
         <v>66</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>707</v>
+        <v>701</v>
       </c>
       <c r="E11" t="s">
         <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>613</v>
+        <v>607</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>68</v>
@@ -3414,10 +3396,10 @@
         <v>39</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>625</v>
+        <v>619</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>719</v>
+        <v>713</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>71</v>
@@ -3438,13 +3420,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>712</v>
+        <v>706</v>
       </c>
       <c r="B13" t="s">
-        <v>711</v>
+        <v>705</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>754</v>
+        <v>748</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>27</v>
@@ -3460,7 +3442,7 @@
         <v>310</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>713</v>
+        <v>707</v>
       </c>
       <c r="J13" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3478,7 +3460,7 @@
         <v>77</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>78</v>
@@ -3514,7 +3496,7 @@
         <v>119</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>15</v>
@@ -3538,10 +3520,10 @@
         <v>88</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>640</v>
+        <v>634</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
@@ -3596,10 +3578,10 @@
         <v>97</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>638</v>
+        <v>632</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="G18" t="s">
         <v>29</v>
@@ -3617,13 +3599,13 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>693</v>
+        <v>687</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>694</v>
+        <v>688</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>695</v>
+        <v>689</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>27</v>
@@ -3632,14 +3614,14 @@
         <v>78</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>696</v>
+        <v>690</v>
       </c>
       <c r="G19" t="s">
         <v>78</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="6" t="s">
-        <v>697</v>
+        <v>691</v>
       </c>
       <c r="J19" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3679,14 +3661,14 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>736</v>
+        <v>730</v>
       </c>
       <c r="B21" t="s">
-        <v>737</v>
+        <v>731</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" t="s">
-        <v>751</v>
+        <v>745</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>78</v>
@@ -3695,7 +3677,7 @@
         <v>79</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>738</v>
+        <v>732</v>
       </c>
       <c r="J21" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3741,7 +3723,7 @@
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="3" t="s">
-        <v>702</v>
+        <v>696</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>60</v>
@@ -3769,7 +3751,7 @@
         <v>118</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>707</v>
+        <v>701</v>
       </c>
       <c r="E24" t="s">
         <v>119</v>
@@ -3858,19 +3840,19 @@
         <v>137</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>622</v>
+        <v>616</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>71</v>
       </c>
       <c r="F27" t="s">
-        <v>621</v>
+        <v>615</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>616</v>
+        <v>610</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>138</v>
@@ -3891,15 +3873,15 @@
         <v>141</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>635</v>
+        <v>629</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E28" s="5"/>
       <c r="F28" s="5"/>
       <c r="G28" s="5" t="s">
-        <v>615</v>
+        <v>609</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>142</v>
@@ -3914,27 +3896,27 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>698</v>
+        <v>692</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>664</v>
+        <v>658</v>
       </c>
       <c r="F29" s="5"/>
       <c r="G29" t="s">
         <v>29</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>699</v>
+        <v>693</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>700</v>
+        <v>694</v>
       </c>
       <c r="J29" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3952,7 +3934,7 @@
         <v>146</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>707</v>
+        <v>701</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>60</v>
@@ -3971,13 +3953,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>680</v>
+        <v>674</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>13</v>
@@ -3986,16 +3968,16 @@
         <v>119</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>683</v>
+        <v>677</v>
       </c>
       <c r="G31" t="s">
         <v>15</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>684</v>
+        <v>678</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>685</v>
+        <v>679</v>
       </c>
       <c r="J31" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4010,10 +3992,10 @@
         <v>150</v>
       </c>
       <c r="C32" t="s">
-        <v>632</v>
+        <v>626</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
@@ -4031,14 +4013,14 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>745</v>
+        <v>739</v>
       </c>
       <c r="B33" t="s">
-        <v>746</v>
+        <v>740</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" t="s">
-        <v>751</v>
+        <v>745</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>78</v>
@@ -4047,10 +4029,10 @@
         <v>79</v>
       </c>
       <c r="H33" t="s">
-        <v>743</v>
+        <v>737</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>747</v>
+        <v>741</v>
       </c>
       <c r="J33" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4065,7 +4047,7 @@
         <v>154</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>631</v>
+        <v>625</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>155</v>
@@ -4096,10 +4078,10 @@
         <v>161</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>633</v>
+        <v>627</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E35" s="5"/>
       <c r="F35" s="5"/>
@@ -4156,10 +4138,10 @@
         <v>173</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="G37" t="s">
-        <v>603</v>
+        <v>597</v>
       </c>
       <c r="H37" s="5" t="s">
         <v>174</v>
@@ -4174,14 +4156,14 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>748</v>
+        <v>742</v>
       </c>
       <c r="B38" t="s">
-        <v>749</v>
+        <v>743</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" t="s">
-        <v>751</v>
+        <v>745</v>
       </c>
       <c r="E38" s="5" t="s">
         <v>78</v>
@@ -4190,10 +4172,10 @@
         <v>79</v>
       </c>
       <c r="H38" t="s">
-        <v>743</v>
+        <v>737</v>
       </c>
       <c r="I38" t="s">
-        <v>750</v>
+        <v>744</v>
       </c>
       <c r="J38" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4209,7 +4191,7 @@
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>703</v>
+        <v>697</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>60</v>
@@ -4218,10 +4200,10 @@
         <v>60</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>691</v>
+        <v>685</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>690</v>
+        <v>684</v>
       </c>
       <c r="J39" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4270,7 +4252,7 @@
         <v>186</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>708</v>
+        <v>702</v>
       </c>
       <c r="E41" s="5" t="s">
         <v>78</v>
@@ -4297,7 +4279,7 @@
         <v>191</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>661</v>
+        <v>655</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>27</v>
@@ -4331,7 +4313,7 @@
         <v>197</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E43" t="s">
         <v>198</v>
@@ -4340,7 +4322,7 @@
         <v>199</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>602</v>
+        <v>596</v>
       </c>
       <c r="H43" s="5" t="s">
         <v>200</v>
@@ -4392,7 +4374,7 @@
         <v>209</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>652</v>
+        <v>646</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>13</v>
@@ -4457,7 +4439,7 @@
         <v>221</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>707</v>
+        <v>701</v>
       </c>
       <c r="E47" s="5"/>
       <c r="F47" t="s">
@@ -4495,7 +4477,7 @@
         <v>229</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>603</v>
+        <v>597</v>
       </c>
       <c r="H48" s="5" t="s">
         <v>230</v>
@@ -4547,10 +4529,10 @@
         <v>239</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>643</v>
+        <v>637</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>702</v>
+        <v>696</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
@@ -4576,10 +4558,10 @@
         <v>244</v>
       </c>
       <c r="C51" t="s">
-        <v>660</v>
+        <v>654</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="G51" t="s">
         <v>29</v>
@@ -4628,10 +4610,10 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>675</v>
+        <v>669</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>676</v>
+        <v>670</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
@@ -4641,16 +4623,16 @@
         <v>119</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>677</v>
+        <v>671</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>678</v>
+        <v>672</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>679</v>
+        <v>673</v>
       </c>
       <c r="J53" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4665,10 +4647,10 @@
         <v>254</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="G54" t="s">
         <v>29</v>
@@ -4695,7 +4677,7 @@
         <v>259</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E55" s="5" t="s">
         <v>119</v>
@@ -4728,7 +4710,7 @@
         <v>264</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E56" s="11" t="s">
         <v>265</v>
@@ -4759,7 +4741,7 @@
       </c>
       <c r="C57" s="16"/>
       <c r="D57" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E57" s="5"/>
       <c r="F57" s="5"/>
@@ -4816,10 +4798,10 @@
         <v>281</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>654</v>
+        <v>648</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>708</v>
+        <v>702</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5" t="s">
@@ -4877,7 +4859,7 @@
       </c>
       <c r="C61" s="5"/>
       <c r="D61" s="3" t="s">
-        <v>702</v>
+        <v>696</v>
       </c>
       <c r="E61" s="5" t="s">
         <v>119</v>
@@ -4905,7 +4887,7 @@
         <v>293</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>710</v>
+        <v>704</v>
       </c>
       <c r="E62" s="5" t="s">
         <v>240</v>
@@ -4954,10 +4936,10 @@
     </row>
     <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>727</v>
+        <v>721</v>
       </c>
       <c r="B64" t="s">
-        <v>720</v>
+        <v>714</v>
       </c>
       <c r="C64" s="5"/>
       <c r="D64" s="5" t="s">
@@ -4974,7 +4956,7 @@
         <v>310</v>
       </c>
       <c r="I64" s="15" t="s">
-        <v>714</v>
+        <v>708</v>
       </c>
       <c r="J64" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4990,7 +4972,7 @@
       </c>
       <c r="C65" s="5"/>
       <c r="D65" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
@@ -4998,7 +4980,7 @@
         <v>304</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="I65" s="8" t="s">
         <v>305</v>
@@ -5016,7 +4998,7 @@
         <v>307</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>636</v>
+        <v>630</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>27</v>
@@ -5034,7 +5016,7 @@
         <v>310</v>
       </c>
       <c r="I66" s="5" t="s">
-        <v>715</v>
+        <v>709</v>
       </c>
       <c r="J66" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5043,16 +5025,16 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>725</v>
+        <v>719</v>
       </c>
       <c r="B67" t="s">
         <v>292</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>753</v>
+        <v>747</v>
       </c>
       <c r="D67" t="s">
-        <v>719</v>
+        <v>713</v>
       </c>
       <c r="E67" s="5" t="s">
         <v>78</v>
@@ -5065,7 +5047,7 @@
         <v>310</v>
       </c>
       <c r="I67" t="s">
-        <v>717</v>
+        <v>711</v>
       </c>
       <c r="J67" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5166,16 +5148,16 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="B71" t="s">
-        <v>721</v>
+        <v>715</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>755</v>
+        <v>749</v>
       </c>
       <c r="D71" t="s">
-        <v>723</v>
+        <v>717</v>
       </c>
       <c r="E71" s="5" t="s">
         <v>78</v>
@@ -5188,7 +5170,7 @@
         <v>310</v>
       </c>
       <c r="I71" t="s">
-        <v>718</v>
+        <v>712</v>
       </c>
       <c r="J71" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5206,7 +5188,7 @@
         <v>330</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>707</v>
+        <v>701</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>71</v>
@@ -5239,7 +5221,7 @@
       </c>
       <c r="E73" s="5"/>
       <c r="F73" s="5" t="s">
-        <v>672</v>
+        <v>666</v>
       </c>
       <c r="G73" s="5" t="s">
         <v>29</v>
@@ -5263,10 +5245,10 @@
         <v>339</v>
       </c>
       <c r="C74" t="s">
-        <v>656</v>
+        <v>650</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="G74" t="s">
         <v>288</v>
@@ -5284,14 +5266,14 @@
     </row>
     <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>731</v>
+        <v>725</v>
       </c>
       <c r="B75" t="s">
-        <v>732</v>
+        <v>726</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" t="s">
-        <v>751</v>
+        <v>745</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>78</v>
@@ -5304,7 +5286,7 @@
         <v>310</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>733</v>
+        <v>727</v>
       </c>
       <c r="J75" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5320,7 +5302,7 @@
       </c>
       <c r="C76" s="5"/>
       <c r="D76" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E76" s="5"/>
       <c r="F76" s="5"/>
@@ -5331,7 +5313,7 @@
         <v>343</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>601</v>
+        <v>595</v>
       </c>
       <c r="J76" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5346,10 +5328,10 @@
         <v>97</v>
       </c>
       <c r="C77" t="s">
-        <v>653</v>
+        <v>647</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="G77" t="s">
         <v>29</v>
@@ -5385,7 +5367,7 @@
         <v>350</v>
       </c>
       <c r="G78" s="5" t="s">
-        <v>615</v>
+        <v>609</v>
       </c>
       <c r="H78" s="5" t="s">
         <v>351</v>
@@ -5409,7 +5391,7 @@
         <v>355</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E79" s="5" t="s">
         <v>119</v>
@@ -5433,27 +5415,27 @@
     </row>
     <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="18" t="s">
-        <v>756</v>
+        <v>750</v>
       </c>
       <c r="B80" s="18" t="s">
-        <v>757</v>
+        <v>751</v>
       </c>
       <c r="C80" s="18"/>
       <c r="D80" s="18" t="s">
-        <v>758</v>
+        <v>752</v>
       </c>
       <c r="E80" s="18" t="s">
-        <v>664</v>
+        <v>658</v>
       </c>
       <c r="F80" s="18"/>
       <c r="G80" s="18" t="s">
         <v>127</v>
       </c>
       <c r="H80" s="18" t="s">
-        <v>759</v>
+        <v>753</v>
       </c>
       <c r="I80" s="6" t="s">
-        <v>760</v>
+        <v>754</v>
       </c>
       <c r="J80" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5468,10 +5450,10 @@
         <v>292</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>609</v>
+        <v>603</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E81" s="11" t="s">
         <v>265</v>
@@ -5501,10 +5483,10 @@
         <v>363</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="G82" t="s">
         <v>29</v>
@@ -5535,7 +5517,7 @@
       </c>
       <c r="E83" s="5"/>
       <c r="F83" s="5" t="s">
-        <v>674</v>
+        <v>668</v>
       </c>
       <c r="G83" s="5" t="s">
         <v>29</v>
@@ -5559,7 +5541,7 @@
         <v>372</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>27</v>
@@ -5593,7 +5575,7 @@
         <v>378</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E85" s="5" t="s">
         <v>71</v>
@@ -5624,7 +5606,7 @@
         <v>383</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E86" s="5" t="s">
         <v>119</v>
@@ -5633,7 +5615,7 @@
         <v>384</v>
       </c>
       <c r="G86" s="5" t="s">
-        <v>602</v>
+        <v>596</v>
       </c>
       <c r="H86" s="5" t="s">
         <v>385</v>
@@ -5654,10 +5636,10 @@
         <v>388</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>655</v>
+        <v>649</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>78</v>
@@ -5687,7 +5669,7 @@
         <v>393</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>705</v>
+        <v>699</v>
       </c>
       <c r="E88" s="11" t="s">
         <v>265</v>
@@ -5715,19 +5697,19 @@
         <v>397</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>641</v>
+        <v>635</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>41</v>
       </c>
       <c r="F89" t="s">
-        <v>604</v>
+        <v>598</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>614</v>
+        <v>608</v>
       </c>
       <c r="H89" s="3" t="s">
         <v>398</v>
@@ -5748,10 +5730,10 @@
         <v>400</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>642</v>
+        <v>636</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>704</v>
+        <v>698</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>78</v>
@@ -5774,10 +5756,10 @@
         <v>403</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>644</v>
+        <v>638</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E91" s="5"/>
       <c r="F91" s="5"/>
@@ -5803,10 +5785,10 @@
         <v>407</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>659</v>
+        <v>653</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
@@ -5832,10 +5814,10 @@
         <v>412</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>658</v>
+        <v>652</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>702</v>
+        <v>696</v>
       </c>
       <c r="E93" s="5"/>
       <c r="G93" s="5" t="s">
@@ -5867,7 +5849,7 @@
       </c>
       <c r="E94" s="5"/>
       <c r="F94" s="5" t="s">
-        <v>673</v>
+        <v>667</v>
       </c>
       <c r="G94" s="5" t="s">
         <v>29</v>
@@ -5925,7 +5907,7 @@
         <v>428</v>
       </c>
       <c r="D96" s="5" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="E96" s="5" t="s">
         <v>71</v>
@@ -5952,10 +5934,10 @@
         <v>433</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>626</v>
+        <v>620</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E97" s="5"/>
       <c r="F97" s="5"/>
@@ -6067,396 +6049,396 @@
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A101" s="5" t="s">
+      <c r="A101" s="18" t="s">
+        <v>755</v>
+      </c>
+      <c r="B101" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="C101" s="18" t="s">
+        <v>756</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="E101" t="s">
+        <v>67</v>
+      </c>
+      <c r="F101" s="18"/>
+      <c r="G101" t="s">
+        <v>127</v>
+      </c>
+      <c r="H101" s="18" t="s">
+        <v>757</v>
+      </c>
+      <c r="I101" s="6" t="s">
+        <v>758</v>
+      </c>
+      <c r="J101" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=diane.moreau@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>452</v>
       </c>
-      <c r="B101" s="5" t="s">
+      <c r="B102" t="s">
         <v>453</v>
       </c>
-      <c r="C101" s="5" t="s">
+      <c r="C102" s="5" t="s">
+        <v>621</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E102" s="5"/>
+      <c r="F102" t="s">
         <v>454</v>
       </c>
-      <c r="D101" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E101" s="5"/>
-      <c r="F101" s="5" t="s">
+      <c r="G102" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="H102" t="s">
         <v>455</v>
       </c>
-      <c r="G101" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="H101" s="5" t="s">
+      <c r="I102" s="8" t="s">
         <v>456</v>
       </c>
-      <c r="I101" s="5" t="s">
+      <c r="J102" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="J101" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=assia.mourid@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A102" s="18" t="s">
-        <v>761</v>
-      </c>
-      <c r="B102" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="C102" s="18" t="s">
-        <v>762</v>
-      </c>
-      <c r="D102" s="5" t="s">
+      <c r="B103" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="D103" s="5" t="s">
         <v>701</v>
       </c>
-      <c r="E102" t="s">
-        <v>67</v>
-      </c>
-      <c r="F102" s="18"/>
-      <c r="G102" t="s">
-        <v>127</v>
-      </c>
-      <c r="H102" s="18" t="s">
-        <v>763</v>
-      </c>
-      <c r="I102" s="6" t="s">
-        <v>764</v>
-      </c>
-      <c r="J102" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=diane.moreau@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>458</v>
-      </c>
-      <c r="B103" t="s">
+      <c r="E103" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F103" s="12"/>
+      <c r="G103" s="3" t="s">
+        <v>613</v>
+      </c>
+      <c r="H103" s="3" t="s">
         <v>459</v>
       </c>
-      <c r="C103" s="5" t="s">
-        <v>627</v>
-      </c>
-      <c r="D103" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E103" s="5"/>
-      <c r="F103" t="s">
+      <c r="I103" s="3" t="s">
         <v>460</v>
       </c>
-      <c r="G103" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="H103" t="s">
+      <c r="J103" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="5" t="s">
         <v>461</v>
       </c>
-      <c r="I103" s="8" t="s">
+      <c r="B104" s="5" t="s">
         <v>462</v>
       </c>
-      <c r="J103" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="3" t="s">
+      <c r="C104" s="5" t="s">
+        <v>645</v>
+      </c>
+      <c r="D104" s="5" t="s">
         <v>463</v>
       </c>
-      <c r="B104" s="3" t="s">
+      <c r="E104" s="5"/>
+      <c r="F104" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="C104" s="3" t="s">
-        <v>634</v>
-      </c>
-      <c r="D104" s="5" t="s">
-        <v>707</v>
-      </c>
-      <c r="E104" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F104" s="12"/>
-      <c r="G104" s="3" t="s">
-        <v>619</v>
-      </c>
-      <c r="H104" s="3" t="s">
+      <c r="G104" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="H104" s="5" t="s">
         <v>465</v>
       </c>
-      <c r="I104" s="3" t="s">
+      <c r="I104" s="15" t="s">
         <v>466</v>
       </c>
       <c r="J104" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
         <v>467</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="C105" s="5" t="s">
-        <v>651</v>
-      </c>
-      <c r="D105" s="5" t="s">
+      <c r="C105" s="5"/>
+      <c r="D105" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="E105" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F105" s="5"/>
+      <c r="H105" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="E105" s="5"/>
-      <c r="F105" s="5" t="s">
+      <c r="I105" s="5" t="s">
         <v>470</v>
       </c>
-      <c r="G105" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="H105" s="5" t="s">
-        <v>471</v>
-      </c>
-      <c r="I105" s="15" t="s">
-        <v>472</v>
-      </c>
       <c r="J105" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="C106" s="5" t="s">
+        <v>606</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="E106" t="s">
+        <v>759</v>
+      </c>
+      <c r="F106" s="3"/>
+      <c r="G106" t="s">
+        <v>760</v>
+      </c>
+      <c r="H106" s="5" t="s">
         <v>473</v>
       </c>
-      <c r="B106" s="5" t="s">
+      <c r="I106" s="15" t="s">
         <v>474</v>
       </c>
-      <c r="C106" s="5"/>
-      <c r="D106" s="3" t="s">
-        <v>702</v>
-      </c>
-      <c r="E106" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F106" s="5"/>
-      <c r="H106" s="5" t="s">
-        <v>475</v>
-      </c>
-      <c r="I106" s="5" t="s">
-        <v>476</v>
-      </c>
       <c r="J106" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="C107" s="5"/>
+      <c r="D107" s="5" t="s">
         <v>477</v>
       </c>
-      <c r="B107" s="5" t="s">
+      <c r="E107" s="5"/>
+      <c r="F107" t="s">
         <v>478</v>
       </c>
-      <c r="C107" s="5" t="s">
-        <v>612</v>
-      </c>
-      <c r="D107" s="5" t="s">
-        <v>706</v>
-      </c>
-      <c r="E107" t="s">
-        <v>765</v>
-      </c>
-      <c r="F107" s="3"/>
-      <c r="G107" t="s">
-        <v>766</v>
-      </c>
-      <c r="H107" s="5" t="s">
+      <c r="G107" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H107" s="5"/>
+      <c r="I107" s="8" t="s">
         <v>479</v>
       </c>
-      <c r="I107" s="15" t="s">
+      <c r="J107" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>480</v>
       </c>
-      <c r="J107" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A108" s="5" t="s">
+      <c r="B108" t="s">
         <v>481</v>
       </c>
-      <c r="B108" s="5" t="s">
+      <c r="C108" s="7" t="s">
         <v>482</v>
       </c>
-      <c r="C108" s="5"/>
-      <c r="D108" s="5" t="s">
+      <c r="D108" t="s">
+        <v>27</v>
+      </c>
+      <c r="E108" t="s">
+        <v>78</v>
+      </c>
+      <c r="F108" s="5" t="s">
         <v>483</v>
       </c>
-      <c r="E108" s="5"/>
-      <c r="F108" t="s">
+      <c r="G108" t="s">
+        <v>95</v>
+      </c>
+      <c r="I108" t="s">
         <v>484</v>
       </c>
-      <c r="G108" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="H108" s="5"/>
-      <c r="I108" s="8" t="s">
+      <c r="J108" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A109" s="5" t="s">
         <v>485</v>
       </c>
-      <c r="J108" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+      <c r="B109" s="5" t="s">
         <v>486</v>
       </c>
-      <c r="B109" t="s">
+      <c r="C109" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E109" s="5"/>
+      <c r="F109" s="5" t="s">
         <v>487</v>
       </c>
-      <c r="C109" s="7" t="s">
+      <c r="G109" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H109" s="3" t="s">
         <v>488</v>
       </c>
-      <c r="D109" t="s">
-        <v>27</v>
-      </c>
-      <c r="E109" t="s">
-        <v>78</v>
-      </c>
-      <c r="F109" s="5" t="s">
+      <c r="I109" s="3" t="s">
         <v>489</v>
       </c>
-      <c r="G109" t="s">
-        <v>95</v>
-      </c>
-      <c r="I109" t="s">
-        <v>490</v>
-      </c>
       <c r="J109" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="C110" s="5" t="s">
         <v>491</v>
-      </c>
-      <c r="B110" s="5" t="s">
-        <v>492</v>
-      </c>
-      <c r="C110" s="5" t="s">
-        <v>623</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E110" s="5"/>
+      <c r="E110" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="F110" s="5" t="s">
-        <v>493</v>
+        <v>686</v>
       </c>
       <c r="G110" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H110" s="3" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="I110" s="3" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="J110" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>496</v>
-      </c>
-      <c r="C111" s="5" t="s">
-        <v>497</v>
+        <v>292</v>
+      </c>
+      <c r="C111" s="16" t="s">
+        <v>495</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E111" s="5" t="s">
-        <v>29</v>
-      </c>
+      <c r="E111" s="5"/>
       <c r="F111" s="5" t="s">
-        <v>692</v>
+        <v>133</v>
       </c>
       <c r="G111" s="5" t="s">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="I111" s="3" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="J111" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="C112" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D112" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E112" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F112" s="5" t="s">
         <v>500</v>
       </c>
-      <c r="B112" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="C112" s="16" t="s">
+      <c r="G112" s="4"/>
+      <c r="H112" s="3"/>
+      <c r="I112" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="D112" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E112" s="5"/>
-      <c r="F112" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="G112" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="H112" s="3" t="s">
-        <v>502</v>
-      </c>
-      <c r="I112" s="3" t="s">
-        <v>503</v>
-      </c>
       <c r="J112" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="C113" s="5" t="s">
         <v>504</v>
       </c>
-      <c r="B113" s="5" t="s">
-        <v>459</v>
-      </c>
-      <c r="C113" s="5" t="s">
+      <c r="D113" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E113" s="5"/>
+      <c r="F113" s="5" t="s">
         <v>505</v>
       </c>
-      <c r="D113" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E113" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F113" s="5" t="s">
+      <c r="G113" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="H113" s="3" t="s">
         <v>506</v>
       </c>
-      <c r="G113" s="4"/>
-      <c r="H113" s="3"/>
-      <c r="I113" s="6" t="s">
+      <c r="I113" s="15" t="s">
         <v>507</v>
       </c>
       <c r="J113" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.25">
@@ -6467,332 +6449,332 @@
         <v>509</v>
       </c>
       <c r="C114" s="5" t="s">
+        <v>651</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="E114" s="5"/>
+      <c r="F114" s="5"/>
+      <c r="G114" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H114" s="3" t="s">
         <v>510</v>
       </c>
-      <c r="D114" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E114" s="5"/>
-      <c r="F114" s="5" t="s">
+      <c r="I114" s="8" t="s">
         <v>511</v>
       </c>
-      <c r="G114" s="5" t="s">
-        <v>304</v>
-      </c>
-      <c r="H114" s="3" t="s">
+      <c r="J114" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
         <v>512</v>
       </c>
-      <c r="I114" s="15" t="s">
+      <c r="B115" t="s">
         <v>513</v>
       </c>
-      <c r="J114" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A115" s="5" t="s">
+      <c r="C115" t="s">
+        <v>639</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="G115" t="s">
+        <v>597</v>
+      </c>
+      <c r="H115" s="5" t="s">
         <v>514</v>
       </c>
-      <c r="B115" s="5" t="s">
+      <c r="I115" s="8" t="s">
         <v>515</v>
       </c>
-      <c r="C115" s="5" t="s">
-        <v>657</v>
-      </c>
-      <c r="D115" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="E115" s="5"/>
-      <c r="F115" s="5"/>
-      <c r="G115" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H115" s="3" t="s">
-        <v>516</v>
-      </c>
-      <c r="I115" s="8" t="s">
-        <v>517</v>
-      </c>
       <c r="J115" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>518</v>
+        <v>728</v>
       </c>
       <c r="B116" t="s">
-        <v>519</v>
-      </c>
-      <c r="C116" t="s">
-        <v>645</v>
-      </c>
-      <c r="D116" s="5" t="s">
-        <v>701</v>
+        <v>453</v>
+      </c>
+      <c r="C116" s="14"/>
+      <c r="D116" t="s">
+        <v>745</v>
+      </c>
+      <c r="E116" s="5" t="s">
+        <v>78</v>
       </c>
       <c r="G116" t="s">
-        <v>603</v>
-      </c>
-      <c r="H116" s="5" t="s">
-        <v>520</v>
-      </c>
-      <c r="I116" s="8" t="s">
-        <v>521</v>
-      </c>
-      <c r="J116" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
+        <v>79</v>
+      </c>
+      <c r="H116" t="s">
+        <v>310</v>
+      </c>
+      <c r="I116" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="J116" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>734</v>
+        <v>516</v>
       </c>
       <c r="B117" t="s">
-        <v>459</v>
-      </c>
-      <c r="C117" s="14"/>
-      <c r="D117" t="s">
-        <v>751</v>
-      </c>
-      <c r="E117" s="5" t="s">
-        <v>78</v>
+        <v>517</v>
+      </c>
+      <c r="C117" s="17"/>
+      <c r="D117" s="5" t="s">
+        <v>695</v>
       </c>
       <c r="G117" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="H117" t="s">
-        <v>310</v>
-      </c>
-      <c r="I117" s="6" t="s">
-        <v>735</v>
-      </c>
-      <c r="J117" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
+        <v>518</v>
+      </c>
+      <c r="I117" s="8" t="s">
+        <v>519</v>
+      </c>
+      <c r="J117" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>522</v>
+        <v>718</v>
       </c>
       <c r="B118" t="s">
-        <v>523</v>
-      </c>
-      <c r="C118" s="17"/>
-      <c r="D118" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="G118" t="s">
-        <v>29</v>
-      </c>
-      <c r="H118" t="s">
-        <v>524</v>
-      </c>
-      <c r="I118" s="8" t="s">
-        <v>525</v>
-      </c>
-      <c r="J118" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
+        <v>76</v>
+      </c>
+      <c r="C118" s="5"/>
+      <c r="D118" t="s">
+        <v>716</v>
+      </c>
+      <c r="E118" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F118" s="5"/>
+      <c r="G118" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="H118" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="I118" t="s">
+        <v>710</v>
+      </c>
+      <c r="J118" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>724</v>
+        <v>656</v>
       </c>
       <c r="B119" t="s">
-        <v>76</v>
-      </c>
-      <c r="C119" s="5"/>
-      <c r="D119" t="s">
-        <v>722</v>
-      </c>
-      <c r="E119" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F119" s="5"/>
-      <c r="G119" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="H119" s="5" t="s">
-        <v>310</v>
-      </c>
-      <c r="I119" t="s">
-        <v>716</v>
-      </c>
-      <c r="J119" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
+        <v>657</v>
+      </c>
+      <c r="C119" s="16" t="s">
+        <v>665</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="E119" s="5"/>
+      <c r="F119" s="3"/>
+      <c r="G119" t="s">
+        <v>537</v>
+      </c>
+      <c r="H119" t="s">
+        <v>659</v>
+      </c>
+      <c r="I119" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="J119" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>662</v>
+        <v>520</v>
       </c>
       <c r="B120" t="s">
-        <v>663</v>
-      </c>
-      <c r="C120" s="16" t="s">
-        <v>671</v>
-      </c>
-      <c r="D120" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="E120" s="5"/>
-      <c r="F120" s="3"/>
+        <v>51</v>
+      </c>
+      <c r="C120" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="D120" t="s">
+        <v>13</v>
+      </c>
+      <c r="F120" s="5" t="s">
+        <v>522</v>
+      </c>
       <c r="G120" t="s">
-        <v>543</v>
-      </c>
-      <c r="H120" t="s">
-        <v>665</v>
-      </c>
-      <c r="I120" s="6" t="s">
-        <v>666</v>
+        <v>29</v>
+      </c>
+      <c r="H120" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="I120" s="3" t="s">
+        <v>524</v>
       </c>
       <c r="J120" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
       </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
+        <v>736</v>
+      </c>
+      <c r="B121" t="s">
+        <v>124</v>
+      </c>
+      <c r="C121" s="5"/>
+      <c r="D121" t="s">
+        <v>745</v>
+      </c>
+      <c r="E121" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G121" t="s">
+        <v>79</v>
+      </c>
+      <c r="H121" t="s">
+        <v>737</v>
+      </c>
+      <c r="I121" s="6" t="s">
+        <v>738</v>
+      </c>
+      <c r="J121" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A122" s="5" t="s">
+        <v>525</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="C122" s="5" t="s">
         <v>526</v>
       </c>
-      <c r="B121" t="s">
-        <v>51</v>
-      </c>
-      <c r="C121" s="7" t="s">
-        <v>527</v>
-      </c>
-      <c r="D121" t="s">
-        <v>13</v>
-      </c>
-      <c r="F121" s="5" t="s">
-        <v>528</v>
-      </c>
-      <c r="G121" t="s">
-        <v>29</v>
-      </c>
-      <c r="H121" s="3" t="s">
-        <v>529</v>
-      </c>
-      <c r="I121" s="3" t="s">
-        <v>530</v>
-      </c>
-      <c r="J121" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>742</v>
-      </c>
-      <c r="B122" t="s">
-        <v>124</v>
-      </c>
-      <c r="C122" s="5"/>
-      <c r="D122" t="s">
-        <v>751</v>
+      <c r="D122" s="5" t="s">
+        <v>701</v>
       </c>
       <c r="E122" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G122" t="s">
-        <v>79</v>
-      </c>
-      <c r="H122" t="s">
-        <v>743</v>
-      </c>
-      <c r="I122" s="6" t="s">
-        <v>744</v>
-      </c>
-      <c r="J122" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
+      <c r="F122" s="5"/>
+      <c r="H122" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I122" s="15" t="s">
+        <v>527</v>
+      </c>
+      <c r="J122" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="C123" s="5" t="s">
+        <v>623</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E123" s="5"/>
+      <c r="F123" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="G123" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="H123" s="3"/>
+      <c r="I123" s="3" t="s">
         <v>531</v>
       </c>
-      <c r="B123" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="C123" s="5" t="s">
+      <c r="J123" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
         <v>532</v>
       </c>
-      <c r="D123" s="5" t="s">
-        <v>707</v>
-      </c>
-      <c r="E123" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F123" s="5"/>
-      <c r="H123" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="I123" s="15" t="s">
+      <c r="B124" t="s">
         <v>533</v>
       </c>
-      <c r="J123" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A124" s="5" t="s">
+      <c r="C124" t="s">
+        <v>618</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="E124" s="5"/>
+      <c r="F124" s="5"/>
+      <c r="G124" t="s">
+        <v>29</v>
+      </c>
+      <c r="J124" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A125" s="3" t="s">
         <v>534</v>
       </c>
-      <c r="B124" s="5" t="s">
+      <c r="B125" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C125" s="14" t="s">
         <v>535</v>
       </c>
-      <c r="C124" s="5" t="s">
-        <v>629</v>
-      </c>
-      <c r="D124" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E124" s="5"/>
-      <c r="F124" s="5" t="s">
+      <c r="D125" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E125" s="3"/>
+      <c r="F125" s="3" t="s">
         <v>536</v>
       </c>
-      <c r="G124" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="H124" s="3"/>
-      <c r="I124" s="3" t="s">
+      <c r="G125" s="3" t="s">
         <v>537</v>
       </c>
-      <c r="J124" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
+      <c r="H125" s="3" t="s">
         <v>538</v>
       </c>
-      <c r="B125" t="s">
+      <c r="I125" s="3" t="s">
         <v>539</v>
       </c>
-      <c r="C125" t="s">
-        <v>624</v>
-      </c>
-      <c r="D125" s="3" t="s">
-        <v>702</v>
-      </c>
-      <c r="E125" s="5"/>
-      <c r="F125" s="5"/>
-      <c r="G125" t="s">
-        <v>29</v>
-      </c>
       <c r="J125" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v/>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
       </c>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.25">
@@ -6800,552 +6782,521 @@
         <v>540</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C126" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="C126" s="3"/>
+      <c r="D126" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="E126" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F126" s="3"/>
+      <c r="G126" s="3"/>
+      <c r="H126" s="3" t="s">
         <v>541</v>
       </c>
-      <c r="D126" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E126" s="3"/>
-      <c r="F126" s="3" t="s">
+      <c r="I126" s="3" t="s">
         <v>542</v>
       </c>
-      <c r="G126" s="3" t="s">
+      <c r="J126" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A127" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="H126" s="3" t="s">
+      <c r="B127" s="5" t="s">
         <v>544</v>
       </c>
-      <c r="I126" s="3" t="s">
+      <c r="C127" s="5" t="s">
         <v>545</v>
       </c>
-      <c r="J126" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A127" s="3" t="s">
+      <c r="D127" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="E127" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G127" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="H127" s="5" t="s">
         <v>546</v>
       </c>
-      <c r="B127" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C127" s="3"/>
-      <c r="D127" s="3" t="s">
-        <v>702</v>
-      </c>
-      <c r="E127" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F127" s="3"/>
-      <c r="G127" s="3"/>
-      <c r="H127" s="3" t="s">
+      <c r="I127" s="15" t="s">
         <v>547</v>
       </c>
-      <c r="I127" s="3" t="s">
+      <c r="J127" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>661</v>
+      </c>
+      <c r="B128" t="s">
+        <v>578</v>
+      </c>
+      <c r="C128" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="E128" s="5"/>
+      <c r="F128" s="3"/>
+      <c r="G128" t="s">
+        <v>537</v>
+      </c>
+      <c r="H128" t="s">
+        <v>662</v>
+      </c>
+      <c r="I128" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="J128" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A129" s="5" t="s">
         <v>548</v>
       </c>
-      <c r="J127" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A128" s="5" t="s">
+      <c r="B129" s="5" t="s">
         <v>549</v>
       </c>
-      <c r="B128" s="5" t="s">
+      <c r="C129" s="5" t="s">
+        <v>631</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="E129" s="5"/>
+      <c r="F129" s="5"/>
+      <c r="G129" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="H129" s="5"/>
+      <c r="I129" s="8" t="s">
         <v>550</v>
       </c>
-      <c r="C128" s="5" t="s">
+      <c r="J129" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A130" s="3" t="s">
         <v>551</v>
       </c>
-      <c r="D128" s="5" t="s">
-        <v>706</v>
-      </c>
-      <c r="E128" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G128" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="H128" s="5" t="s">
+      <c r="B130" s="3" t="s">
         <v>552</v>
       </c>
-      <c r="I128" s="15" t="s">
+      <c r="C130" s="5" t="s">
         <v>553</v>
       </c>
-      <c r="J128" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
-        <v>667</v>
-      </c>
-      <c r="B129" t="s">
-        <v>584</v>
-      </c>
-      <c r="C129" s="5" t="s">
-        <v>670</v>
-      </c>
-      <c r="D129" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="E129" s="5"/>
-      <c r="F129" s="3"/>
-      <c r="G129" t="s">
-        <v>543</v>
-      </c>
-      <c r="H129" t="s">
-        <v>668</v>
-      </c>
-      <c r="I129" s="6" t="s">
-        <v>669</v>
-      </c>
-      <c r="J129" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A130" s="5" t="s">
+      <c r="D130" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="E130" t="s">
         <v>554</v>
       </c>
-      <c r="B130" s="5" t="s">
+      <c r="F130" s="3" t="s">
         <v>555</v>
       </c>
-      <c r="C130" s="5" t="s">
-        <v>637</v>
-      </c>
-      <c r="D130" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="E130" s="5"/>
-      <c r="F130" s="5"/>
-      <c r="G130" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="H130" s="5"/>
-      <c r="I130" s="8" t="s">
+      <c r="G130" s="3" t="s">
+        <v>612</v>
+      </c>
+      <c r="H130" s="3" t="s">
         <v>556</v>
       </c>
+      <c r="I130" s="15" t="s">
+        <v>557</v>
+      </c>
       <c r="J130" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
       </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A131" s="3" t="s">
-        <v>557</v>
-      </c>
-      <c r="B131" s="3" t="s">
+      <c r="A131" s="5" t="s">
         <v>558</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>453</v>
       </c>
       <c r="C131" s="5" t="s">
         <v>559</v>
       </c>
-      <c r="D131" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="E131" t="s">
+      <c r="D131" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E131" s="5"/>
+      <c r="F131" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="G131" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="H131" s="5" t="s">
         <v>560</v>
       </c>
-      <c r="F131" s="3" t="s">
+      <c r="I131" s="15" t="s">
         <v>561</v>
       </c>
-      <c r="G131" s="3" t="s">
-        <v>618</v>
-      </c>
-      <c r="H131" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="I131" s="15" t="s">
-        <v>563</v>
-      </c>
       <c r="J131" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>563</v>
+      </c>
+      <c r="C132" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="E132" s="5"/>
+      <c r="F132" s="5"/>
+      <c r="G132" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="H132" t="s">
         <v>564</v>
       </c>
-      <c r="B132" s="5" t="s">
-        <v>459</v>
-      </c>
-      <c r="C132" s="5" t="s">
+      <c r="I132" s="8" t="s">
         <v>565</v>
       </c>
-      <c r="D132" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E132" s="5"/>
-      <c r="F132" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="G132" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="H132" s="5" t="s">
-        <v>566</v>
-      </c>
-      <c r="I132" s="15" t="s">
-        <v>567</v>
-      </c>
       <c r="J132" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
+        <v>566</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>567</v>
+      </c>
+      <c r="C133" s="5" t="s">
+        <v>622</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E133" s="5"/>
+      <c r="F133" s="5" t="s">
         <v>568</v>
       </c>
-      <c r="B133" s="5" t="s">
+      <c r="G133" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H133" s="5" t="s">
         <v>569</v>
       </c>
-      <c r="C133" s="5" t="s">
-        <v>650</v>
-      </c>
-      <c r="D133" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="E133" s="5"/>
-      <c r="F133" s="5"/>
-      <c r="G133" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="H133" t="s">
+      <c r="I133" s="15" t="s">
         <v>570</v>
       </c>
-      <c r="I133" s="8" t="s">
+      <c r="J133" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
         <v>571</v>
       </c>
-      <c r="J133" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A134" s="5" t="s">
-        <v>572</v>
-      </c>
-      <c r="B134" s="5" t="s">
-        <v>573</v>
-      </c>
-      <c r="C134" s="5" t="s">
-        <v>628</v>
+      <c r="B134" t="s">
+        <v>574</v>
       </c>
       <c r="D134" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="E134" s="5"/>
-      <c r="F134" s="5" t="s">
-        <v>574</v>
-      </c>
-      <c r="G134" s="5" t="s">
-        <v>222</v>
+        <v>695</v>
+      </c>
+      <c r="G134" t="s">
+        <v>288</v>
       </c>
       <c r="H134" s="5" t="s">
         <v>575</v>
       </c>
-      <c r="I134" s="15" t="s">
+      <c r="I134" s="8" t="s">
         <v>576</v>
       </c>
       <c r="J134" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
+      <c r="A135" s="5" t="s">
+        <v>571</v>
+      </c>
+      <c r="B135" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="C135" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="E135" s="5"/>
+      <c r="F135" s="5"/>
+      <c r="G135" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="H135" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="I135" s="8" t="s">
+        <v>573</v>
+      </c>
+      <c r="J135" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>599</v>
+      </c>
+      <c r="B136" t="s">
+        <v>472</v>
+      </c>
+      <c r="C136" s="5" t="s">
+        <v>643</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="E136" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F136" t="s">
+        <v>600</v>
+      </c>
+      <c r="G136" t="s">
+        <v>614</v>
+      </c>
+      <c r="H136" t="s">
+        <v>601</v>
+      </c>
+      <c r="I136" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="J136" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A137" s="5" t="s">
         <v>577</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B137" s="5" t="s">
+        <v>578</v>
+      </c>
+      <c r="C137" s="5"/>
+      <c r="D137" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="E137" s="5"/>
+      <c r="F137" s="5"/>
+      <c r="G137" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H137" s="5" t="s">
+        <v>579</v>
+      </c>
+      <c r="I137" s="8" t="s">
         <v>580</v>
       </c>
-      <c r="D135" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="G135" t="s">
-        <v>288</v>
-      </c>
-      <c r="H135" s="5" t="s">
-        <v>581</v>
-      </c>
-      <c r="I135" s="8" t="s">
-        <v>582</v>
-      </c>
-      <c r="J135" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A136" s="5" t="s">
-        <v>577</v>
-      </c>
-      <c r="B136" s="5" t="s">
-        <v>578</v>
-      </c>
-      <c r="C136" s="5" t="s">
-        <v>630</v>
-      </c>
-      <c r="D136" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="E136" s="5"/>
-      <c r="F136" s="5"/>
-      <c r="G136" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="H136" s="5" t="s">
-        <v>409</v>
-      </c>
-      <c r="I136" s="8" t="s">
-        <v>579</v>
-      </c>
-      <c r="J136" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>605</v>
-      </c>
-      <c r="B137" t="s">
-        <v>478</v>
-      </c>
-      <c r="C137" s="5" t="s">
-        <v>649</v>
-      </c>
-      <c r="D137" s="5" t="s">
-        <v>706</v>
-      </c>
-      <c r="E137" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F137" t="s">
-        <v>606</v>
-      </c>
-      <c r="G137" t="s">
-        <v>620</v>
-      </c>
-      <c r="H137" t="s">
-        <v>607</v>
-      </c>
-      <c r="I137" s="6" t="s">
-        <v>608</v>
-      </c>
       <c r="J137" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138" s="5" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>584</v>
-      </c>
-      <c r="C138" s="5"/>
+        <v>582</v>
+      </c>
+      <c r="C138" s="5" t="s">
+        <v>605</v>
+      </c>
       <c r="D138" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
       <c r="G138" s="5" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="H138" s="5" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="I138" s="8" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="J138" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139" s="5" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>611</v>
+        <v>633</v>
       </c>
       <c r="D139" s="5" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="E139" s="5"/>
       <c r="F139" s="5"/>
       <c r="G139" s="5" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="H139" s="5" t="s">
+        <v>587</v>
+      </c>
+      <c r="I139" s="8" t="s">
+        <v>588</v>
+      </c>
+      <c r="J139" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>733</v>
+      </c>
+      <c r="B140" t="s">
+        <v>734</v>
+      </c>
+      <c r="C140" s="5" t="s">
+        <v>746</v>
+      </c>
+      <c r="D140" t="s">
+        <v>745</v>
+      </c>
+      <c r="E140" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G140" t="s">
+        <v>79</v>
+      </c>
+      <c r="I140" s="6" t="s">
+        <v>735</v>
+      </c>
+      <c r="J140" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A141" s="5" t="s">
         <v>589</v>
       </c>
-      <c r="I139" s="8" t="s">
+      <c r="B141" s="5" t="s">
+        <v>582</v>
+      </c>
+      <c r="C141" s="5" t="s">
+        <v>641</v>
+      </c>
+      <c r="D141" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="E141" s="5"/>
+      <c r="F141" s="5"/>
+      <c r="G141" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H141" s="5" t="s">
         <v>590</v>
       </c>
-      <c r="J139" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A140" s="5" t="s">
+      <c r="I141" s="8" t="s">
         <v>591</v>
       </c>
-      <c r="B140" s="5" t="s">
-        <v>592</v>
-      </c>
-      <c r="C140" s="5" t="s">
-        <v>639</v>
-      </c>
-      <c r="D140" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="E140" s="5"/>
-      <c r="F140" s="5"/>
-      <c r="G140" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="H140" s="5" t="s">
-        <v>593</v>
-      </c>
-      <c r="I140" s="8" t="s">
-        <v>594</v>
-      </c>
-      <c r="J140" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
-        <v>739</v>
-      </c>
-      <c r="B141" t="s">
-        <v>740</v>
-      </c>
-      <c r="C141" s="5" t="s">
-        <v>752</v>
-      </c>
-      <c r="D141" t="s">
-        <v>751</v>
-      </c>
-      <c r="E141" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G141" t="s">
-        <v>79</v>
-      </c>
-      <c r="I141" s="6" t="s">
-        <v>741</v>
-      </c>
-      <c r="J141" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
+      <c r="J141" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142" s="5" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>588</v>
-      </c>
-      <c r="C142" s="5" t="s">
-        <v>647</v>
-      </c>
+        <v>214</v>
+      </c>
+      <c r="C142" s="5"/>
       <c r="D142" s="5" t="s">
-        <v>701</v>
-      </c>
-      <c r="E142" s="5"/>
-      <c r="F142" s="5"/>
-      <c r="G142" s="5" t="s">
-        <v>89</v>
+        <v>27</v>
+      </c>
+      <c r="E142" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F142" s="5" t="s">
+        <v>593</v>
+      </c>
+      <c r="G142" t="s">
+        <v>429</v>
       </c>
       <c r="H142" s="5" t="s">
-        <v>596</v>
-      </c>
-      <c r="I142" s="8" t="s">
-        <v>597</v>
+        <v>450</v>
+      </c>
+      <c r="I142" s="15" t="s">
+        <v>594</v>
       </c>
       <c r="J142" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
       </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143" s="5" t="s">
-        <v>598</v>
+        <v>680</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>214</v>
+        <v>681</v>
       </c>
       <c r="C143" s="5"/>
       <c r="D143" s="5" t="s">
-        <v>27</v>
+        <v>703</v>
       </c>
       <c r="E143" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F143" s="5" t="s">
-        <v>599</v>
-      </c>
-      <c r="G143" t="s">
-        <v>429</v>
+        <v>78</v>
+      </c>
+      <c r="F143" s="5"/>
+      <c r="G143" s="5" t="s">
+        <v>78</v>
       </c>
       <c r="H143" s="5" t="s">
-        <v>450</v>
-      </c>
-      <c r="I143" s="15" t="s">
-        <v>600</v>
-      </c>
-      <c r="J143" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A144" s="5" t="s">
-        <v>686</v>
-      </c>
-      <c r="B144" s="5" t="s">
-        <v>687</v>
-      </c>
-      <c r="C144" s="5"/>
-      <c r="D144" s="5" t="s">
-        <v>709</v>
-      </c>
-      <c r="E144" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F144" s="5"/>
-      <c r="G144" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="H144" s="5" t="s">
-        <v>688</v>
-      </c>
-      <c r="I144" s="6" t="s">
-        <v>689</v>
-      </c>
-      <c r="J144" s="9" t="str">
+        <v>682</v>
+      </c>
+      <c r="I143" s="6" t="s">
+        <v>683</v>
+      </c>
+      <c r="J143" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=sosthene.yamale@umontreal.ca</v>
       </c>
@@ -7358,81 +7309,81 @@
     <hyperlink ref="I17" r:id="rId3" display="mailto:hugo.bernier@umontreal.ca" xr:uid="{3F591457-DA50-462E-B1CA-F2F56ED9E3DD}"/>
     <hyperlink ref="I76" r:id="rId4" xr:uid="{4822C834-E5A8-42FD-9734-374BFC718C85}"/>
     <hyperlink ref="I10" r:id="rId5" display="mailto:magalie.beaudoin@umontreal.ca" xr:uid="{2D976BF0-B68A-46E5-8412-BA8BC43FD26D}"/>
-    <hyperlink ref="I113" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
+    <hyperlink ref="I112" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
     <hyperlink ref="I5" r:id="rId7" display="mailto:nadege.arsa@bib.umontreal.ca" xr:uid="{408AF5A3-35ED-4BF5-92B9-1B21C0C475D9}"/>
     <hyperlink ref="I20" r:id="rId8" display="mailto:simon.blais.longtin@umontreal.ca" xr:uid="{EA917AC7-9087-435B-A6E7-3AE1885514AA}"/>
     <hyperlink ref="I93" r:id="rId9" xr:uid="{8ABC26E9-CF81-491C-8A28-B209E6620D2A}"/>
-    <hyperlink ref="I139" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
+    <hyperlink ref="I138" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
     <hyperlink ref="I37" r:id="rId11" xr:uid="{7D21070C-9A14-48DF-982E-D995A034BDAD}"/>
-    <hyperlink ref="I135" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
+    <hyperlink ref="I134" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
     <hyperlink ref="I74" r:id="rId13" xr:uid="{DCABBE8B-8789-4957-9A88-F8585AD53BBC}"/>
-    <hyperlink ref="I116" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
+    <hyperlink ref="I115" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
     <hyperlink ref="I51" r:id="rId15" xr:uid="{1383A46C-5C1D-4621-B4BC-67AD012D7CF5}"/>
     <hyperlink ref="I82" r:id="rId16" xr:uid="{29D9619F-F3A7-41E8-AE0F-DEBBF802D53A}"/>
     <hyperlink ref="I32" r:id="rId17" xr:uid="{9E8CD31B-437A-49A0-BA12-85176E0D9431}"/>
-    <hyperlink ref="I118" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
+    <hyperlink ref="I117" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
     <hyperlink ref="I77" r:id="rId19" xr:uid="{3B502B79-2DDE-44A3-908B-3CB04ED1101E}"/>
     <hyperlink ref="I18" r:id="rId20" xr:uid="{BAE0697B-7739-4A42-9702-C285F03D0F77}"/>
     <hyperlink ref="I54" r:id="rId21" xr:uid="{E1BC7B04-B072-447B-9137-59A28141883D}"/>
-    <hyperlink ref="I108" r:id="rId22" xr:uid="{BEDF45F1-312C-4FF5-B4F5-1D1C7E487C0A}"/>
+    <hyperlink ref="I107" r:id="rId22" xr:uid="{BEDF45F1-312C-4FF5-B4F5-1D1C7E487C0A}"/>
     <hyperlink ref="I65" r:id="rId23" xr:uid="{6E82D57D-36A4-4928-AD91-BE73FFC7C389}"/>
     <hyperlink ref="I84" r:id="rId24" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
-    <hyperlink ref="I103" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
-    <hyperlink ref="I136" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
+    <hyperlink ref="I102" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
+    <hyperlink ref="I135" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
     <hyperlink ref="I91" r:id="rId27" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
     <hyperlink ref="I92" r:id="rId28" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
     <hyperlink ref="I97" r:id="rId29" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
-    <hyperlink ref="I115" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
-    <hyperlink ref="I130" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
-    <hyperlink ref="I133" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
-    <hyperlink ref="I138" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
-    <hyperlink ref="I140" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
-    <hyperlink ref="I142" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
+    <hyperlink ref="I114" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
+    <hyperlink ref="I129" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
+    <hyperlink ref="I132" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
+    <hyperlink ref="I137" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
+    <hyperlink ref="I139" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
+    <hyperlink ref="I141" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
     <hyperlink ref="I16" r:id="rId36" xr:uid="{E26D4CB1-6F14-4277-AD54-18A052872B6B}"/>
-    <hyperlink ref="I137" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
+    <hyperlink ref="I136" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
     <hyperlink ref="I39" r:id="rId38" xr:uid="{902A8808-023C-4EA1-833E-F687288B12ED}"/>
-    <hyperlink ref="I129" r:id="rId39" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
-    <hyperlink ref="I120" r:id="rId40" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
+    <hyperlink ref="I128" r:id="rId39" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
+    <hyperlink ref="I119" r:id="rId40" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
     <hyperlink ref="I53" r:id="rId41" xr:uid="{ABEB73EB-E336-4619-ADE1-0AE567E81306}"/>
     <hyperlink ref="I31" r:id="rId42" xr:uid="{E819F1D0-ED89-4281-B222-20D0A6AC8A49}"/>
-    <hyperlink ref="I144" r:id="rId43" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
+    <hyperlink ref="I143" r:id="rId43" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
     <hyperlink ref="I19" r:id="rId44" xr:uid="{A4113BC8-FD33-4D47-854C-D964ED926E7F}"/>
     <hyperlink ref="I29" r:id="rId45" xr:uid="{7233E394-0474-4122-B129-E1E8DB3D4B70}"/>
-    <hyperlink ref="I117" r:id="rId46" xr:uid="{0924E3CD-F2EB-4646-BC88-767228D5A8FD}"/>
+    <hyperlink ref="I116" r:id="rId46" xr:uid="{0924E3CD-F2EB-4646-BC88-767228D5A8FD}"/>
     <hyperlink ref="I75" r:id="rId47" xr:uid="{FAC375AB-8F54-402B-A4F5-618AA479650B}"/>
     <hyperlink ref="I4" r:id="rId48" xr:uid="{12EFBBCC-308A-4E41-92F6-4E78BB9E9458}"/>
     <hyperlink ref="I21" r:id="rId49" xr:uid="{CAA07608-BC3B-468C-819E-F94EE0396C78}"/>
-    <hyperlink ref="I141" r:id="rId50" xr:uid="{B3DF72B2-3730-4A9C-8195-E5B8FCD87C3B}"/>
-    <hyperlink ref="I122" r:id="rId51" xr:uid="{518A2404-8625-4373-BDE5-E73718B1440B}"/>
+    <hyperlink ref="I140" r:id="rId50" xr:uid="{B3DF72B2-3730-4A9C-8195-E5B8FCD87C3B}"/>
+    <hyperlink ref="I121" r:id="rId51" xr:uid="{518A2404-8625-4373-BDE5-E73718B1440B}"/>
     <hyperlink ref="I33" r:id="rId52" xr:uid="{B383F9BF-E7F0-4AFA-A217-1F3A922E55BA}"/>
-    <hyperlink ref="I143" r:id="rId53" xr:uid="{D2BBF900-A9C8-4032-A387-C01245244DE0}"/>
+    <hyperlink ref="I142" r:id="rId53" xr:uid="{D2BBF900-A9C8-4032-A387-C01245244DE0}"/>
     <hyperlink ref="I52" r:id="rId54" xr:uid="{79C702A2-295C-4D37-BA6F-DD2C408C75BD}"/>
     <hyperlink ref="I23" r:id="rId55" xr:uid="{761F418D-12C5-4F41-8071-6031B8FBF83B}"/>
-    <hyperlink ref="I107" r:id="rId56" xr:uid="{C91A1DE6-A8FA-4481-9E51-1DB52F17F3CC}"/>
-    <hyperlink ref="I134" r:id="rId57" xr:uid="{131478F3-61ED-4B04-9E66-6F771D0E53F1}"/>
+    <hyperlink ref="I106" r:id="rId56" xr:uid="{C91A1DE6-A8FA-4481-9E51-1DB52F17F3CC}"/>
+    <hyperlink ref="I133" r:id="rId57" xr:uid="{131478F3-61ED-4B04-9E66-6F771D0E53F1}"/>
     <hyperlink ref="I100" r:id="rId58" xr:uid="{C3534DCE-62CB-4016-B559-AE879ED29221}"/>
     <hyperlink ref="I72" r:id="rId59" xr:uid="{598291DC-2DD2-464C-A65A-36D0759E8852}"/>
     <hyperlink ref="I64" r:id="rId60" xr:uid="{55FAFEEC-7E6A-4254-BBB4-020FD859DB23}"/>
-    <hyperlink ref="I105" r:id="rId61" xr:uid="{E35BC25D-CA56-4FFF-B93C-72EBCAD05C3B}"/>
+    <hyperlink ref="I104" r:id="rId61" xr:uid="{E35BC25D-CA56-4FFF-B93C-72EBCAD05C3B}"/>
     <hyperlink ref="I45" r:id="rId62" xr:uid="{6B64B7D5-5396-4382-9ECB-D065E5B3F7C4}"/>
     <hyperlink ref="I57" r:id="rId63" xr:uid="{A6C3CD82-A312-40D2-B320-33ED739C6E60}"/>
     <hyperlink ref="I86" r:id="rId64" xr:uid="{1754B384-2B8D-46A2-8C89-BDF617522295}"/>
-    <hyperlink ref="I114" r:id="rId65" xr:uid="{99B099F4-5E98-4B25-B2EB-EE4C451DC6EE}"/>
+    <hyperlink ref="I113" r:id="rId65" xr:uid="{99B099F4-5E98-4B25-B2EB-EE4C451DC6EE}"/>
     <hyperlink ref="I59" r:id="rId66" xr:uid="{1C080271-6DB7-4810-99C8-8FF2BA5EA430}"/>
     <hyperlink ref="I63" r:id="rId67" xr:uid="{6A0B0BD3-8872-437B-9CD4-6D8D7D98A4F9}"/>
-    <hyperlink ref="I123" r:id="rId68" xr:uid="{CE8C2C5F-3292-4BA9-A27E-19AF9661C907}"/>
+    <hyperlink ref="I122" r:id="rId68" xr:uid="{CE8C2C5F-3292-4BA9-A27E-19AF9661C907}"/>
     <hyperlink ref="I11" r:id="rId69" xr:uid="{F1246003-4D15-4FC5-9F7D-6CE88CAF21A8}"/>
-    <hyperlink ref="I132" r:id="rId70" xr:uid="{BB3A0149-0DD5-481B-8662-8134BB3FCECC}"/>
-    <hyperlink ref="I128" r:id="rId71" xr:uid="{52D55C85-F393-43A8-95EF-F57618BB179E}"/>
+    <hyperlink ref="I131" r:id="rId70" xr:uid="{BB3A0149-0DD5-481B-8662-8134BB3FCECC}"/>
+    <hyperlink ref="I127" r:id="rId71" xr:uid="{52D55C85-F393-43A8-95EF-F57618BB179E}"/>
     <hyperlink ref="I87" r:id="rId72" xr:uid="{CAB4CB00-83BC-4384-BF0E-208B7456F243}"/>
     <hyperlink ref="I95" r:id="rId73" xr:uid="{4B80B43B-B062-42B6-A1CE-F4CE03CDED46}"/>
     <hyperlink ref="I8" r:id="rId74" xr:uid="{BC76BE28-D367-49FE-95A3-98BB93483999}"/>
     <hyperlink ref="I47" r:id="rId75" xr:uid="{8598B756-3A70-45A7-ABB5-3EDBEF50BAF4}"/>
-    <hyperlink ref="I131" r:id="rId76" xr:uid="{07544A5C-3F38-40A4-9945-4E56F5EFFCF4}"/>
+    <hyperlink ref="I130" r:id="rId76" xr:uid="{07544A5C-3F38-40A4-9945-4E56F5EFFCF4}"/>
     <hyperlink ref="I27" r:id="rId77" xr:uid="{C341566A-DC48-4D81-91C1-E1CD275F4D60}"/>
     <hyperlink ref="I13" r:id="rId78" xr:uid="{FAAE6B3B-3F31-452F-868E-B6C650D083E8}"/>
     <hyperlink ref="I80" r:id="rId79" xr:uid="{09E37274-D8A2-4A0B-832A-E187D6213477}"/>
-    <hyperlink ref="I102" r:id="rId80" xr:uid="{89D21B16-595D-4AC9-BFE9-2C29DBC329A2}"/>
+    <hyperlink ref="I101" r:id="rId80" xr:uid="{89D21B16-595D-4AC9-BFE9-2C29DBC329A2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId81"/>

</xml_diff>

<commit_message>
feat(repertoire-personnel): Changements divers au répertoire
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6D1527A-C78C-4EFF-9C36-9451491784A8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59054CF3-272E-4C5B-9FF4-F69B35BD050B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5460" yWindow="3555" windowWidth="30315" windowHeight="28125" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5460" yWindow="3560" windowWidth="30320" windowHeight="28130" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="762">
   <si>
     <t>nom</t>
   </si>
@@ -2331,6 +2331,9 @@
   </si>
   <si>
     <t>Bibliothèque des lettres et sciences humaines et Service du prêt entre bibliothèques</t>
+  </si>
+  <si>
+    <t>514 343-6111, poste 2744</t>
   </si>
 </sst>
 </file>
@@ -3035,21 +3038,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J143"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="33.85546875" customWidth="1"/>
-    <col min="4" max="4" width="45.28515625" customWidth="1"/>
-    <col min="5" max="5" width="58.140625" customWidth="1"/>
+    <col min="3" max="3" width="33.81640625" customWidth="1"/>
+    <col min="4" max="4" width="45.26953125" customWidth="1"/>
+    <col min="5" max="5" width="58.1796875" customWidth="1"/>
     <col min="6" max="6" width="58" customWidth="1"/>
-    <col min="7" max="7" width="70.85546875" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="41.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="86.5703125" customWidth="1"/>
+    <col min="7" max="7" width="70.81640625" customWidth="1"/>
+    <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="86.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3081,7 +3084,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
@@ -3112,7 +3115,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alexandre.amar-zifkin@umontreal.ca</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -3145,7 +3148,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.angers@umontreal.ca</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>722</v>
       </c>
@@ -3173,7 +3176,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=busch.antenor.alexandre@umontreal.ca</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
@@ -3204,7 +3207,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nadege.arsa@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
@@ -3235,7 +3238,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=denis.arvisais@umontreal.ca</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>38</v>
       </c>
@@ -3268,7 +3271,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.attia@umontreal.ca</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>45</v>
       </c>
@@ -3281,7 +3284,9 @@
       <c r="D8" s="5" t="s">
         <v>695</v>
       </c>
-      <c r="E8" s="5"/>
+      <c r="E8" s="5" t="s">
+        <v>41</v>
+      </c>
       <c r="F8" s="5"/>
       <c r="G8" s="5" t="s">
         <v>21</v>
@@ -3297,7 +3302,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=prlaval@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -3327,7 +3332,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.bastien@umontreal.ca</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>57</v>
       </c>
@@ -3355,7 +3360,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magalie.beaudoin@umontreal.ca</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>64</v>
       </c>
@@ -3388,7 +3393,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maryna.beaulieu@umontreal.ca</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>70</v>
       </c>
@@ -3418,7 +3423,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.begin-poissant@umontreal.ca</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>706</v>
       </c>
@@ -3449,7 +3454,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nima.behforouz@umontreal.ca</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>75</v>
       </c>
@@ -3479,7 +3484,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.belanger@umontreal.ca</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>82</v>
       </c>
@@ -3512,7 +3517,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amy.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>87</v>
       </c>
@@ -3541,7 +3546,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amelie.bernard@umontreal.ca</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>92</v>
       </c>
@@ -3570,7 +3575,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=hugo.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>92</v>
       </c>
@@ -3597,7 +3602,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>687</v>
       </c>
@@ -3628,7 +3633,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cathy.bingoye@umontreal.ca</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
         <v>100</v>
       </c>
@@ -3659,7 +3664,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon.blais.longtin@umontreal.ca</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>730</v>
       </c>
@@ -3684,7 +3689,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guy.blondeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>106</v>
       </c>
@@ -3714,7 +3719,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tatiana.talpa@umontreal.ca</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>112</v>
       </c>
@@ -3740,7 +3745,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=joanna.bodnar@umontreal.ca</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>116</v>
       </c>
@@ -3770,7 +3775,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alain.borsi@umontreal.ca</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>123</v>
       </c>
@@ -3801,7 +3806,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.p.bouchard@umontreal.ca</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
         <v>130</v>
       </c>
@@ -3832,7 +3837,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refdroi@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>136</v>
       </c>
@@ -3865,7 +3870,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=myriam.boyer@umontreal.ca</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
         <v>140</v>
       </c>
@@ -3894,7 +3899,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guylaine.brazeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>692</v>
       </c>
@@ -3923,7 +3928,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-marie.brien.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>144</v>
       </c>
@@ -3951,7 +3956,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sophie.brisebois@umontreal.ca</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>674</v>
       </c>
@@ -3984,7 +3989,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tanya.buchet@umontreal.ca</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>149</v>
       </c>
@@ -4011,7 +4016,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fanny.c.brochu@umontreal.ca</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>739</v>
       </c>
@@ -4039,7 +4044,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thierry.caballero@umontreal.ca</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>153</v>
       </c>
@@ -4070,7 +4075,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=delphine.cado@umontreal.ca</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>160</v>
       </c>
@@ -4099,7 +4104,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=siv.kham.chao@umontreal.ca</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>165</v>
       </c>
@@ -4130,7 +4135,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=laurence.charest@umontreal.ca</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>172</v>
       </c>
@@ -4154,7 +4159,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=annick.charette@umontreal.ca</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>742</v>
       </c>
@@ -4182,7 +4187,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=wassif.cheikh@umontreal.ca</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
         <v>176</v>
       </c>
@@ -4210,7 +4215,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mailto:thien-huong.che-quang@umontreal.ca</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>178</v>
       </c>
@@ -4241,7 +4246,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah.cherrier@umontreal.ca</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
         <v>184</v>
       </c>
@@ -4271,7 +4276,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emir.chouchane@umontreal.ca</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
         <v>190</v>
       </c>
@@ -4302,7 +4307,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=accessibilite@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>195</v>
       </c>
@@ -4335,7 +4340,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benjamin.constantineau@umontreal.ca</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
         <v>202</v>
       </c>
@@ -4366,7 +4371,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon-pierre.crevier@umontreal.ca</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
         <v>208</v>
       </c>
@@ -4397,7 +4402,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marc-olivier.croteau@umontreal.ca</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
         <v>213</v>
       </c>
@@ -4428,7 +4433,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.dalpe@umontreal.ca</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
         <v>219</v>
       </c>
@@ -4459,7 +4464,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=morgane.de.bellefeuille@umontreal.ca</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>226</v>
       </c>
@@ -4490,7 +4495,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=Indiana.delsart@umontreal.ca</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
         <v>232</v>
       </c>
@@ -4521,7 +4526,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=dominic.desaulniers@umontreal.ca</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>238</v>
       </c>
@@ -4550,7 +4555,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.desrosiers@umontreal.ca</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>243</v>
       </c>
@@ -4577,7 +4582,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.dubois.mercier@umontreal.ca</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>247</v>
       </c>
@@ -4608,7 +4613,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jean-francois.durnin@umontreal.ca</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>669</v>
       </c>
@@ -4639,7 +4644,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=taline.ekmekjian@umontreal.ca</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>253</v>
       </c>
@@ -4666,7 +4671,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=judith.fafard-larose@umontreal.ca</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>257</v>
       </c>
@@ -4699,7 +4704,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>262</v>
       </c>
@@ -4732,7 +4737,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=c.fortier@umontreal.ca</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>268</v>
       </c>
@@ -4759,7 +4764,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>274</v>
       </c>
@@ -4790,7 +4795,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nino.gabrielli@umontreal.ca</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
         <v>280</v>
       </c>
@@ -4819,7 +4824,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-pierre.gadoua@umontreal.ca</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
         <v>284</v>
       </c>
@@ -4850,7 +4855,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cynthia.gagne.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>291</v>
       </c>
@@ -4876,7 +4881,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>291</v>
       </c>
@@ -4904,7 +4909,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
         <v>297</v>
       </c>
@@ -4934,7 +4939,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marjorie.gauchier@umontreal.ca</v>
       </c>
     </row>
-    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>721</v>
       </c>
@@ -4963,7 +4968,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=lucie.geoffroy@umontreal.ca</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
         <v>303</v>
       </c>
@@ -4990,7 +4995,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
       </c>
     </row>
-    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
         <v>306</v>
       </c>
@@ -5023,7 +5028,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.giguere.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>719</v>
       </c>
@@ -5054,7 +5059,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.hainault@umontreal.ca</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>311</v>
       </c>
@@ -5085,7 +5090,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
         <v>316</v>
       </c>
@@ -5116,7 +5121,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>322</v>
       </c>
@@ -5146,7 +5151,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>720</v>
       </c>
@@ -5177,7 +5182,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=natalia.jabinschi@umontreal.ca</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
         <v>328</v>
       </c>
@@ -5206,7 +5211,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
         <v>333</v>
       </c>
@@ -5237,7 +5242,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>338</v>
       </c>
@@ -5264,7 +5269,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
       </c>
     </row>
-    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>725</v>
       </c>
@@ -5293,7 +5298,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pierre-yves.lafleur@umontreal.ca</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
         <v>342</v>
       </c>
@@ -5320,7 +5325,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>344</v>
       </c>
@@ -5347,7 +5352,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
         <v>347</v>
       </c>
@@ -5380,7 +5385,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
       </c>
     </row>
-    <row r="79" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
         <v>353</v>
       </c>
@@ -5413,7 +5418,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
       </c>
     </row>
-    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A80" s="18" t="s">
         <v>750</v>
       </c>
@@ -5442,7 +5447,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-josee.lapalme@umontreal.ca</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
         <v>358</v>
       </c>
@@ -5475,7 +5480,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>362</v>
       </c>
@@ -5502,7 +5507,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
         <v>366</v>
       </c>
@@ -5533,7 +5538,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>371</v>
       </c>
@@ -5564,7 +5569,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
         <v>376</v>
       </c>
@@ -5595,7 +5600,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
         <v>381</v>
       </c>
@@ -5628,7 +5633,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
         <v>387</v>
       </c>
@@ -5658,7 +5663,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
         <v>391</v>
       </c>
@@ -5689,7 +5694,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
         <v>396</v>
       </c>
@@ -5722,7 +5727,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
         <v>396</v>
       </c>
@@ -5748,7 +5753,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
         <v>402</v>
       </c>
@@ -5777,7 +5782,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
         <v>406</v>
       </c>
@@ -5806,7 +5811,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
         <v>411</v>
       </c>
@@ -5834,7 +5839,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
         <v>415</v>
       </c>
@@ -5865,7 +5870,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
         <v>420</v>
       </c>
@@ -5896,7 +5901,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
         <v>426</v>
       </c>
@@ -5926,7 +5931,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
       </c>
     </row>
-    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
         <v>432</v>
       </c>
@@ -5955,7 +5960,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
       </c>
     </row>
-    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
         <v>436</v>
       </c>
@@ -5986,7 +5991,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="3" t="s">
         <v>442</v>
       </c>
@@ -6017,7 +6022,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="s">
         <v>447</v>
       </c>
@@ -6048,7 +6053,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="18" t="s">
         <v>755</v>
       </c>
@@ -6079,7 +6084,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.moreau@umontreal.ca</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>452</v>
       </c>
@@ -6110,7 +6115,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
       </c>
     </row>
-    <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A103" s="3" t="s">
         <v>457</v>
       </c>
@@ -6141,7 +6146,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A104" s="5" t="s">
         <v>461</v>
       </c>
@@ -6172,7 +6177,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
         <v>467</v>
       </c>
@@ -6198,7 +6203,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
         <v>471</v>
       </c>
@@ -6229,7 +6234,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
         <v>475</v>
       </c>
@@ -6256,7 +6261,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>480</v>
       </c>
@@ -6286,7 +6291,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
         <v>485</v>
       </c>
@@ -6317,7 +6322,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
         <v>485</v>
       </c>
@@ -6350,7 +6355,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
         <v>494</v>
       </c>
@@ -6381,7 +6386,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
         <v>498</v>
       </c>
@@ -6410,7 +6415,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
         <v>502</v>
       </c>
@@ -6441,7 +6446,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="s">
         <v>508</v>
       </c>
@@ -6470,7 +6475,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>512</v>
       </c>
@@ -6497,7 +6502,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>728</v>
       </c>
@@ -6525,7 +6530,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>516</v>
       </c>
@@ -6550,7 +6555,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>718</v>
       </c>
@@ -6579,7 +6584,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>656</v>
       </c>
@@ -6608,7 +6613,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>520</v>
       </c>
@@ -6638,7 +6643,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>736</v>
       </c>
@@ -6666,7 +6671,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
         <v>525</v>
       </c>
@@ -6694,7 +6699,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
         <v>528</v>
       </c>
@@ -6723,7 +6728,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>532</v>
       </c>
@@ -6746,7 +6751,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A125" s="3" t="s">
         <v>534</v>
       </c>
@@ -6777,7 +6782,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A126" s="3" t="s">
         <v>540</v>
       </c>
@@ -6804,7 +6809,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A127" s="5" t="s">
         <v>543</v>
       </c>
@@ -6834,7 +6839,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>661</v>
       </c>
@@ -6863,7 +6868,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="s">
         <v>548</v>
       </c>
@@ -6876,12 +6881,16 @@
       <c r="D129" s="5" t="s">
         <v>695</v>
       </c>
-      <c r="E129" s="5"/>
+      <c r="E129" s="5" t="s">
+        <v>41</v>
+      </c>
       <c r="F129" s="5"/>
       <c r="G129" s="5" t="s">
         <v>423</v>
       </c>
-      <c r="H129" s="5"/>
+      <c r="H129" s="5" t="s">
+        <v>761</v>
+      </c>
       <c r="I129" s="8" t="s">
         <v>550</v>
       </c>
@@ -6890,7 +6899,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A130" s="3" t="s">
         <v>551</v>
       </c>
@@ -6923,7 +6932,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="s">
         <v>558</v>
       </c>
@@ -6954,7 +6963,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
         <v>562</v>
       </c>
@@ -6967,7 +6976,9 @@
       <c r="D132" s="5" t="s">
         <v>695</v>
       </c>
-      <c r="E132" s="5"/>
+      <c r="E132" s="5" t="s">
+        <v>41</v>
+      </c>
       <c r="F132" s="5"/>
       <c r="G132" s="5" t="s">
         <v>423</v>
@@ -6983,7 +6994,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A133" s="5" t="s">
         <v>566</v>
       </c>
@@ -7014,7 +7025,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>571</v>
       </c>
@@ -7038,7 +7049,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A135" s="5" t="s">
         <v>571</v>
       </c>
@@ -7067,7 +7078,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>599</v>
       </c>
@@ -7100,7 +7111,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="s">
         <v>577</v>
       </c>
@@ -7127,7 +7138,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="s">
         <v>581</v>
       </c>
@@ -7156,7 +7167,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A139" s="5" t="s">
         <v>585</v>
       </c>
@@ -7185,7 +7196,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>733</v>
       </c>
@@ -7212,7 +7223,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A141" s="5" t="s">
         <v>589</v>
       </c>
@@ -7241,7 +7252,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="s">
         <v>592</v>
       </c>
@@ -7272,7 +7283,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="s">
         <v>680</v>
       </c>
@@ -7589,6 +7600,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7597,15 +7617,6 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7628,6 +7639,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7642,12 +7661,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): MAJ Delphine Cado
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59054CF3-272E-4C5B-9FF4-F69B35BD050B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8F96EF2-FB3B-4D10-B60C-66209B778A6A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5460" yWindow="3560" windowWidth="30320" windowHeight="28130" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="762">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="762">
   <si>
     <t>nom</t>
   </si>
@@ -495,32 +495,6 @@
     <t>BIbliothécaire</t>
   </si>
   <si>
-    <r>
-      <t>Référence et offre pédagogique de première ligne,</t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>sciences infirmières premier cycle</t>
-    </r>
-  </si>
-  <si>
     <t>Bibliothèque Marguerite-d'Youville</t>
   </si>
   <si>
@@ -2334,13 +2308,16 @@
   </si>
   <si>
     <t>514 343-6111, poste 2744</t>
+  </si>
+  <si>
+    <t>Sciences infirmières et gérontologie</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2385,14 +2362,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <strike/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -2499,11 +2468,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -3132,7 +3101,7 @@
         <v>41</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>21</v>
@@ -3150,14 +3119,14 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>721</v>
+      </c>
+      <c r="B4" t="s">
         <v>722</v>
-      </c>
-      <c r="B4" t="s">
-        <v>723</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>78</v>
@@ -3166,10 +3135,10 @@
         <v>79</v>
       </c>
       <c r="H4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="J4" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3249,7 +3218,7 @@
         <v>40</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>41</v>
@@ -3258,7 +3227,7 @@
         <v>42</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>43</v>
@@ -3282,7 +3251,7 @@
         <v>47</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>41</v>
@@ -3371,16 +3340,16 @@
         <v>66</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E11" t="s">
         <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>68</v>
@@ -3401,10 +3370,10 @@
         <v>39</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>71</v>
@@ -3425,13 +3394,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B13" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>27</v>
@@ -3441,13 +3410,13 @@
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="H13" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="H13" s="5" t="s">
-        <v>310</v>
-      </c>
       <c r="I13" s="15" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="J13" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3465,7 +3434,7 @@
         <v>77</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>78</v>
@@ -3501,7 +3470,7 @@
         <v>119</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>15</v>
@@ -3525,10 +3494,10 @@
         <v>88</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
@@ -3583,10 +3552,10 @@
         <v>97</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="G18" t="s">
         <v>29</v>
@@ -3604,13 +3573,13 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
+        <v>686</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>687</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>688</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>689</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>27</v>
@@ -3619,14 +3588,14 @@
         <v>78</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="G19" t="s">
         <v>78</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="6" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="J19" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3666,14 +3635,14 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
+        <v>729</v>
+      </c>
+      <c r="B21" t="s">
         <v>730</v>
-      </c>
-      <c r="B21" t="s">
-        <v>731</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>78</v>
@@ -3682,7 +3651,7 @@
         <v>79</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="J21" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3728,7 +3697,7 @@
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>60</v>
@@ -3756,7 +3725,7 @@
         <v>118</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E24" t="s">
         <v>119</v>
@@ -3845,19 +3814,19 @@
         <v>137</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>71</v>
       </c>
       <c r="F27" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>138</v>
@@ -3878,15 +3847,15 @@
         <v>141</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E28" s="5"/>
       <c r="F28" s="5"/>
       <c r="G28" s="5" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>142</v>
@@ -3901,27 +3870,27 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F29" s="5"/>
       <c r="G29" t="s">
         <v>29</v>
       </c>
       <c r="H29" s="5" t="s">
+        <v>692</v>
+      </c>
+      <c r="I29" s="6" t="s">
         <v>693</v>
-      </c>
-      <c r="I29" s="6" t="s">
-        <v>694</v>
       </c>
       <c r="J29" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3939,7 +3908,7 @@
         <v>146</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>60</v>
@@ -3958,13 +3927,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
+        <v>673</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>674</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>675</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>676</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>13</v>
@@ -3973,16 +3942,16 @@
         <v>119</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="G31" t="s">
         <v>15</v>
       </c>
       <c r="H31" s="5" t="s">
+        <v>677</v>
+      </c>
+      <c r="I31" s="6" t="s">
         <v>678</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>679</v>
       </c>
       <c r="J31" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3997,10 +3966,10 @@
         <v>150</v>
       </c>
       <c r="C32" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
@@ -4018,14 +3987,14 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>738</v>
+      </c>
+      <c r="B33" t="s">
         <v>739</v>
-      </c>
-      <c r="B33" t="s">
-        <v>740</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>78</v>
@@ -4034,10 +4003,10 @@
         <v>79</v>
       </c>
       <c r="H33" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="J33" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4052,23 +4021,25 @@
         <v>154</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="F34" t="s">
+        <v>761</v>
+      </c>
+      <c r="G34" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="G34" s="5" t="s">
+      <c r="H34" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="H34" s="5" t="s">
+      <c r="I34" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="I34" s="6" t="s">
-        <v>159</v>
       </c>
       <c r="J34" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4077,27 +4048,27 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B35" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>161</v>
-      </c>
       <c r="C35" s="5" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E35" s="5"/>
       <c r="F35" s="5"/>
       <c r="G35" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="H35" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="H35" s="5" t="s">
+      <c r="I35" s="5" t="s">
         <v>163</v>
-      </c>
-      <c r="I35" s="5" t="s">
-        <v>164</v>
       </c>
       <c r="J35" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4106,13 +4077,13 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="C36" s="5" t="s">
         <v>166</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>167</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>155</v>
@@ -4121,14 +4092,14 @@
         <v>71</v>
       </c>
       <c r="F36" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="G36" t="s">
         <v>168</v>
-      </c>
-      <c r="G36" t="s">
-        <v>169</v>
       </c>
       <c r="H36" s="5"/>
       <c r="I36" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J36" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4137,22 +4108,22 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
+        <v>171</v>
+      </c>
+      <c r="B37" t="s">
         <v>172</v>
       </c>
-      <c r="B37" t="s">
+      <c r="D37" s="5" t="s">
+        <v>694</v>
+      </c>
+      <c r="G37" t="s">
+        <v>596</v>
+      </c>
+      <c r="H37" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>695</v>
-      </c>
-      <c r="G37" t="s">
-        <v>597</v>
-      </c>
-      <c r="H37" s="5" t="s">
+      <c r="I37" s="8" t="s">
         <v>174</v>
-      </c>
-      <c r="I37" s="8" t="s">
-        <v>175</v>
       </c>
       <c r="J37" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4161,14 +4132,14 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
+        <v>741</v>
+      </c>
+      <c r="B38" t="s">
         <v>742</v>
-      </c>
-      <c r="B38" t="s">
-        <v>743</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E38" s="5" t="s">
         <v>78</v>
@@ -4177,10 +4148,10 @@
         <v>79</v>
       </c>
       <c r="H38" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="I38" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="J38" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4189,14 +4160,14 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="B39" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>177</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>60</v>
@@ -4205,10 +4176,10 @@
         <v>60</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="J39" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4217,29 +4188,29 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B40" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="C40" s="16" t="s">
         <v>179</v>
-      </c>
-      <c r="C40" s="16" t="s">
-        <v>180</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E40" s="5"/>
       <c r="F40" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="H40" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="G40" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="H40" s="5" t="s">
+      <c r="I40" s="5" t="s">
         <v>182</v>
-      </c>
-      <c r="I40" s="5" t="s">
-        <v>183</v>
       </c>
       <c r="J40" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4248,28 +4219,28 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B41" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="C41" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="C41" s="5" t="s">
-        <v>186</v>
-      </c>
       <c r="D41" s="5" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="E41" s="5" t="s">
         <v>78</v>
       </c>
       <c r="F41" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="H41" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="H41" s="5" t="s">
+      <c r="I41" s="5" t="s">
         <v>188</v>
-      </c>
-      <c r="I41" s="5" t="s">
-        <v>189</v>
       </c>
       <c r="J41" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4278,29 +4249,29 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B42" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="B42" s="5" t="s">
-        <v>191</v>
-      </c>
       <c r="C42" s="5" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>27</v>
       </c>
       <c r="E42" s="5"/>
       <c r="F42" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H42" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="I42" s="5" t="s">
         <v>193</v>
-      </c>
-      <c r="I42" s="5" t="s">
-        <v>194</v>
       </c>
       <c r="J42" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4309,31 +4280,31 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B43" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="C43" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="D43" s="5" t="s">
+        <v>699</v>
+      </c>
+      <c r="E43" t="s">
         <v>197</v>
       </c>
-      <c r="D43" s="5" t="s">
-        <v>700</v>
-      </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
         <v>198</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" s="5" t="s">
+        <v>595</v>
+      </c>
+      <c r="H43" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="G43" s="5" t="s">
-        <v>596</v>
-      </c>
-      <c r="H43" s="5" t="s">
+      <c r="I43" s="5" t="s">
         <v>200</v>
-      </c>
-      <c r="I43" s="5" t="s">
-        <v>201</v>
       </c>
       <c r="J43" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4342,29 +4313,29 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B44" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="C44" s="5" t="s">
         <v>203</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>204</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E44" s="5"/>
       <c r="F44" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="H44" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="G44" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="H44" s="5" t="s">
+      <c r="I44" s="5" t="s">
         <v>206</v>
-      </c>
-      <c r="I44" s="5" t="s">
-        <v>207</v>
       </c>
       <c r="J44" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4373,29 +4344,29 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="B45" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="B45" s="5" t="s">
-        <v>209</v>
-      </c>
       <c r="C45" s="5" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>54</v>
       </c>
       <c r="H45" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="I45" s="15" t="s">
         <v>211</v>
-      </c>
-      <c r="I45" s="15" t="s">
-        <v>212</v>
       </c>
       <c r="J45" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4404,29 +4375,29 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="B46" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="C46" s="5" t="s">
         <v>214</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>215</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H46" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="I46" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="I46" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="J46" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4435,29 +4406,29 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="B47" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="C47" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="C47" s="5" t="s">
-        <v>221</v>
-      </c>
       <c r="D47" s="5" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E47" s="5"/>
       <c r="F47" t="s">
+        <v>222</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="H47" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="G47" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="H47" s="5" t="s">
+      <c r="I47" s="15" t="s">
         <v>224</v>
-      </c>
-      <c r="I47" s="15" t="s">
-        <v>225</v>
       </c>
       <c r="J47" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4466,29 +4437,29 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="B48" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="C48" s="5" t="s">
         <v>227</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>228</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E48" s="5"/>
       <c r="F48" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>596</v>
+      </c>
+      <c r="H48" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="G48" s="5" t="s">
-        <v>597</v>
-      </c>
-      <c r="H48" s="5" t="s">
+      <c r="I48" s="5" t="s">
         <v>230</v>
-      </c>
-      <c r="I48" s="5" t="s">
-        <v>231</v>
       </c>
       <c r="J48" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4497,29 +4468,29 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="B49" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="C49" s="5" t="s">
         <v>233</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>234</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E49" s="5"/>
       <c r="F49" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G49" s="5" t="s">
         <v>54</v>
       </c>
       <c r="H49" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="I49" s="5" t="s">
         <v>236</v>
-      </c>
-      <c r="I49" s="5" t="s">
-        <v>237</v>
       </c>
       <c r="J49" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4528,27 +4499,27 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="B50" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="B50" s="5" t="s">
-        <v>239</v>
-      </c>
       <c r="C50" s="5" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
       <c r="G50" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="H50" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="H50" s="5" t="s">
+      <c r="I50" s="5" t="s">
         <v>241</v>
-      </c>
-      <c r="I50" s="5" t="s">
-        <v>242</v>
       </c>
       <c r="J50" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4557,25 +4528,25 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
+        <v>242</v>
+      </c>
+      <c r="B51" t="s">
         <v>243</v>
       </c>
-      <c r="B51" t="s">
-        <v>244</v>
-      </c>
       <c r="C51" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="G51" t="s">
         <v>29</v>
       </c>
       <c r="H51" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="I51" s="8" t="s">
         <v>245</v>
-      </c>
-      <c r="I51" s="8" t="s">
-        <v>246</v>
       </c>
       <c r="J51" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4584,29 +4555,29 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B52" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="C52" s="5" t="s">
         <v>248</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>249</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E52" s="5"/>
       <c r="F52" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G52" s="5" t="s">
         <v>54</v>
       </c>
       <c r="H52" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="I52" s="15" t="s">
         <v>251</v>
-      </c>
-      <c r="I52" s="15" t="s">
-        <v>252</v>
       </c>
       <c r="J52" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4615,10 +4586,10 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="B53" s="5" t="s">
         <v>669</v>
-      </c>
-      <c r="B53" s="5" t="s">
-        <v>670</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
@@ -4628,16 +4599,16 @@
         <v>119</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H53" s="5" t="s">
+        <v>671</v>
+      </c>
+      <c r="I53" s="6" t="s">
         <v>672</v>
-      </c>
-      <c r="I53" s="6" t="s">
-        <v>673</v>
       </c>
       <c r="J53" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4646,25 +4617,25 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
+        <v>252</v>
+      </c>
+      <c r="B54" t="s">
         <v>253</v>
       </c>
-      <c r="B54" t="s">
-        <v>254</v>
-      </c>
       <c r="C54" s="5" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="G54" t="s">
         <v>29</v>
       </c>
       <c r="H54" t="s">
+        <v>254</v>
+      </c>
+      <c r="I54" s="8" t="s">
         <v>255</v>
-      </c>
-      <c r="I54" s="8" t="s">
-        <v>256</v>
       </c>
       <c r="J54" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4673,16 +4644,16 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="B55" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="C55" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="C55" s="5" t="s">
-        <v>259</v>
-      </c>
       <c r="D55" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E55" s="5" t="s">
         <v>119</v>
@@ -4694,10 +4665,10 @@
         <v>120</v>
       </c>
       <c r="H55" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="I55" s="5" t="s">
         <v>260</v>
-      </c>
-      <c r="I55" s="5" t="s">
-        <v>261</v>
       </c>
       <c r="J55" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4706,19 +4677,19 @@
     </row>
     <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="B56" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="C56" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="C56" s="5" t="s">
+      <c r="D56" s="5" t="s">
+        <v>699</v>
+      </c>
+      <c r="E56" s="11" t="s">
         <v>264</v>
-      </c>
-      <c r="D56" s="5" t="s">
-        <v>700</v>
-      </c>
-      <c r="E56" s="11" t="s">
-        <v>265</v>
       </c>
       <c r="F56" s="5" t="s">
         <v>42</v>
@@ -4727,10 +4698,10 @@
         <v>29</v>
       </c>
       <c r="H56" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="I56" s="5" t="s">
         <v>266</v>
-      </c>
-      <c r="I56" s="5" t="s">
-        <v>267</v>
       </c>
       <c r="J56" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4739,25 +4710,25 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="B57" s="5" t="s">
         <v>268</v>
-      </c>
-      <c r="B57" s="5" t="s">
-        <v>269</v>
       </c>
       <c r="C57" s="16"/>
       <c r="D57" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E57" s="5"/>
       <c r="F57" s="5"/>
       <c r="G57" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="H57" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="H57" s="5" t="s">
+      <c r="I57" s="15" t="s">
         <v>272</v>
-      </c>
-      <c r="I57" s="15" t="s">
-        <v>273</v>
       </c>
       <c r="J57" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4766,29 +4737,29 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="B58" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="C58" s="5" t="s">
         <v>275</v>
-      </c>
-      <c r="C58" s="5" t="s">
-        <v>276</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E58" s="5"/>
       <c r="F58" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G58" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H58" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="I58" s="5" t="s">
         <v>278</v>
-      </c>
-      <c r="I58" s="5" t="s">
-        <v>279</v>
       </c>
       <c r="J58" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4797,27 +4768,27 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="B59" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="B59" s="5" t="s">
-        <v>281</v>
-      </c>
       <c r="C59" s="5" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H59" s="5"/>
       <c r="I59" s="15" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J59" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4826,29 +4797,29 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="B60" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="C60" s="5" t="s">
         <v>285</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>286</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E60" s="5"/>
       <c r="F60" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="G60" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="G60" s="5" t="s">
+      <c r="H60" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="H60" s="5" t="s">
+      <c r="I60" s="5" t="s">
         <v>289</v>
-      </c>
-      <c r="I60" s="5" t="s">
-        <v>290</v>
       </c>
       <c r="J60" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4857,14 +4828,14 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C61" s="5"/>
       <c r="D61" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E61" s="5" t="s">
         <v>119</v>
@@ -4874,7 +4845,7 @@
         <v>121</v>
       </c>
       <c r="I61" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J61" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4883,26 +4854,26 @@
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="B62" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="C62" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="C62" s="5" t="s">
-        <v>293</v>
-      </c>
       <c r="D62" s="5" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F62" s="5"/>
       <c r="H62" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I62" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J62" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4911,13 +4882,13 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="B63" s="5" t="s">
         <v>297</v>
       </c>
-      <c r="B63" s="5" t="s">
+      <c r="C63" s="5" t="s">
         <v>298</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>299</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>27</v>
@@ -4926,13 +4897,13 @@
         <v>78</v>
       </c>
       <c r="F63" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="H63" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="H63" s="5" t="s">
+      <c r="I63" s="15" t="s">
         <v>301</v>
-      </c>
-      <c r="I63" s="15" t="s">
-        <v>302</v>
       </c>
       <c r="J63" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4941,10 +4912,10 @@
     </row>
     <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="B64" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="C64" s="5"/>
       <c r="D64" s="5" t="s">
@@ -4955,13 +4926,13 @@
       </c>
       <c r="F64" s="5"/>
       <c r="G64" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="H64" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="H64" s="5" t="s">
-        <v>310</v>
-      </c>
       <c r="I64" s="15" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="J64" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4970,25 +4941,25 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C65" s="5"/>
       <c r="D65" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
       <c r="G65" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="I65" s="8" t="s">
         <v>304</v>
-      </c>
-      <c r="H65" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="I65" s="8" t="s">
-        <v>305</v>
       </c>
       <c r="J65" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4997,13 +4968,13 @@
     </row>
     <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="B66" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="B66" s="5" t="s">
-        <v>307</v>
-      </c>
       <c r="C66" s="5" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>27</v>
@@ -5012,16 +4983,16 @@
         <v>78</v>
       </c>
       <c r="F66" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="G66" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="G66" s="5" t="s">
+      <c r="H66" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="H66" s="5" t="s">
-        <v>310</v>
-      </c>
       <c r="I66" s="5" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="J66" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5030,29 +5001,29 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="B67" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="D67" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="E67" s="5" t="s">
         <v>78</v>
       </c>
       <c r="F67" s="5"/>
       <c r="G67" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="H67" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="H67" s="5" t="s">
-        <v>310</v>
-      </c>
       <c r="I67" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="J67" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5061,29 +5032,29 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="C68" s="5" t="s">
         <v>311</v>
-      </c>
-      <c r="B68" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="C68" s="5" t="s">
-        <v>312</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E68" s="5"/>
       <c r="F68" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="H68" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="G68" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="H68" s="5" t="s">
+      <c r="I68" s="5" t="s">
         <v>314</v>
-      </c>
-      <c r="I68" s="5" t="s">
-        <v>315</v>
       </c>
       <c r="J68" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5092,29 +5063,29 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="B69" s="5" t="s">
         <v>316</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="C69" s="5" t="s">
         <v>317</v>
-      </c>
-      <c r="C69" s="5" t="s">
-        <v>318</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>27</v>
       </c>
       <c r="E69" s="5"/>
       <c r="F69" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G69" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H69" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="I69" s="5" t="s">
         <v>320</v>
-      </c>
-      <c r="I69" s="5" t="s">
-        <v>321</v>
       </c>
       <c r="J69" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5123,28 +5094,28 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
+        <v>321</v>
+      </c>
+      <c r="B70" t="s">
         <v>322</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" s="7" t="s">
         <v>323</v>
-      </c>
-      <c r="C70" s="7" t="s">
-        <v>324</v>
       </c>
       <c r="D70" t="s">
         <v>13</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="G70" t="s">
         <v>15</v>
       </c>
       <c r="H70" t="s">
+        <v>325</v>
+      </c>
+      <c r="I70" t="s">
         <v>326</v>
-      </c>
-      <c r="I70" t="s">
-        <v>327</v>
       </c>
       <c r="J70" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5153,29 +5124,29 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B71" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="D71" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="E71" s="5" t="s">
         <v>78</v>
       </c>
       <c r="F71" s="5"/>
       <c r="G71" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="H71" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="H71" s="5" t="s">
-        <v>310</v>
-      </c>
       <c r="I71" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="J71" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5184,16 +5155,16 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="B72" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="B72" s="5" t="s">
+      <c r="C72" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="C72" s="5" t="s">
-        <v>330</v>
-      </c>
       <c r="D72" s="5" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>71</v>
@@ -5201,10 +5172,10 @@
       <c r="F72" s="12"/>
       <c r="G72" s="3"/>
       <c r="H72" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="I72" s="15" t="s">
         <v>331</v>
-      </c>
-      <c r="I72" s="15" t="s">
-        <v>332</v>
       </c>
       <c r="J72" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5213,29 +5184,29 @@
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="B73" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="B73" s="5" t="s">
+      <c r="C73" s="5" t="s">
         <v>334</v>
-      </c>
-      <c r="C73" s="5" t="s">
-        <v>335</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E73" s="5"/>
       <c r="F73" s="5" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G73" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H73" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="I73" s="5" t="s">
         <v>336</v>
-      </c>
-      <c r="I73" s="5" t="s">
-        <v>337</v>
       </c>
       <c r="J73" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5244,25 +5215,25 @@
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
+        <v>337</v>
+      </c>
+      <c r="B74" t="s">
         <v>338</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C74" t="s">
+        <v>649</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>694</v>
+      </c>
+      <c r="G74" t="s">
+        <v>287</v>
+      </c>
+      <c r="H74" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="C74" t="s">
-        <v>650</v>
-      </c>
-      <c r="D74" s="5" t="s">
-        <v>695</v>
-      </c>
-      <c r="G74" t="s">
-        <v>288</v>
-      </c>
-      <c r="H74" s="5" t="s">
+      <c r="I74" s="8" t="s">
         <v>340</v>
-      </c>
-      <c r="I74" s="8" t="s">
-        <v>341</v>
       </c>
       <c r="J74" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5271,14 +5242,14 @@
     </row>
     <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
+        <v>724</v>
+      </c>
+      <c r="B75" t="s">
         <v>725</v>
-      </c>
-      <c r="B75" t="s">
-        <v>726</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>78</v>
@@ -5288,10 +5259,10 @@
         <v>79</v>
       </c>
       <c r="H75" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="J75" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5300,25 +5271,25 @@
     </row>
     <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C76" s="5"/>
       <c r="D76" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E76" s="5"/>
       <c r="F76" s="5"/>
       <c r="G76" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H76" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="J76" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5327,25 +5298,25 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B77" t="s">
         <v>97</v>
       </c>
       <c r="C77" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="G77" t="s">
         <v>29</v>
       </c>
       <c r="H77" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="I77" s="8" t="s">
         <v>345</v>
-      </c>
-      <c r="I77" s="8" t="s">
-        <v>346</v>
       </c>
       <c r="J77" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5354,13 +5325,13 @@
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="B78" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="C78" s="5" t="s">
         <v>348</v>
-      </c>
-      <c r="C78" s="5" t="s">
-        <v>349</v>
       </c>
       <c r="D78" s="5" t="s">
         <v>103</v>
@@ -5369,16 +5340,16 @@
         <v>71</v>
       </c>
       <c r="F78" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="G78" s="5" t="s">
+        <v>608</v>
+      </c>
+      <c r="H78" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="G78" s="5" t="s">
-        <v>609</v>
-      </c>
-      <c r="H78" s="5" t="s">
+      <c r="I78" s="5" t="s">
         <v>351</v>
-      </c>
-      <c r="I78" s="5" t="s">
-        <v>352</v>
       </c>
       <c r="J78" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5387,16 +5358,16 @@
     </row>
     <row r="79" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="B79" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="B79" s="5" t="s">
+      <c r="C79" s="5" t="s">
         <v>354</v>
       </c>
-      <c r="C79" s="5" t="s">
-        <v>355</v>
-      </c>
       <c r="D79" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E79" s="5" t="s">
         <v>119</v>
@@ -5408,10 +5379,10 @@
         <v>15</v>
       </c>
       <c r="H79" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="I79" s="5" t="s">
         <v>356</v>
-      </c>
-      <c r="I79" s="5" t="s">
-        <v>357</v>
       </c>
       <c r="J79" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5420,27 +5391,27 @@
     </row>
     <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A80" s="18" t="s">
+        <v>749</v>
+      </c>
+      <c r="B80" s="18" t="s">
         <v>750</v>
-      </c>
-      <c r="B80" s="18" t="s">
-        <v>751</v>
       </c>
       <c r="C80" s="18"/>
       <c r="D80" s="18" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="E80" s="18" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F80" s="18"/>
       <c r="G80" s="18" t="s">
         <v>127</v>
       </c>
       <c r="H80" s="18" t="s">
+        <v>752</v>
+      </c>
+      <c r="I80" s="6" t="s">
         <v>753</v>
-      </c>
-      <c r="I80" s="6" t="s">
-        <v>754</v>
       </c>
       <c r="J80" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5449,31 +5420,31 @@
     </row>
     <row r="81" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="B81" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="C81" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>699</v>
+      </c>
+      <c r="E81" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="F81" s="5" t="s">
         <v>358</v>
-      </c>
-      <c r="B81" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="C81" s="5" t="s">
-        <v>603</v>
-      </c>
-      <c r="D81" s="5" t="s">
-        <v>700</v>
-      </c>
-      <c r="E81" s="11" t="s">
-        <v>265</v>
-      </c>
-      <c r="F81" s="5" t="s">
-        <v>359</v>
       </c>
       <c r="G81" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H81" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="I81" s="5" t="s">
         <v>360</v>
-      </c>
-      <c r="I81" s="5" t="s">
-        <v>361</v>
       </c>
       <c r="J81" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5482,25 +5453,25 @@
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
+        <v>361</v>
+      </c>
+      <c r="B82" t="s">
         <v>362</v>
       </c>
-      <c r="B82" t="s">
-        <v>363</v>
-      </c>
       <c r="C82" s="5" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="G82" t="s">
         <v>29</v>
       </c>
       <c r="H82" s="13" t="s">
+        <v>363</v>
+      </c>
+      <c r="I82" s="8" t="s">
         <v>364</v>
-      </c>
-      <c r="I82" s="8" t="s">
-        <v>365</v>
       </c>
       <c r="J82" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5509,29 +5480,29 @@
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="B83" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="B83" s="5" t="s">
+      <c r="C83" s="5" t="s">
         <v>367</v>
-      </c>
-      <c r="C83" s="5" t="s">
-        <v>368</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E83" s="5"/>
       <c r="F83" s="5" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="G83" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H83" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="I83" s="5" t="s">
         <v>369</v>
-      </c>
-      <c r="I83" s="5" t="s">
-        <v>370</v>
       </c>
       <c r="J83" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5540,29 +5511,29 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
+        <v>370</v>
+      </c>
+      <c r="B84" t="s">
         <v>371</v>
       </c>
-      <c r="B84" t="s">
-        <v>372</v>
-      </c>
       <c r="C84" s="5" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>27</v>
       </c>
       <c r="E84" s="5"/>
       <c r="F84" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G84" s="5" t="s">
         <v>71</v>
       </c>
       <c r="H84" t="s">
+        <v>373</v>
+      </c>
+      <c r="I84" s="8" t="s">
         <v>374</v>
-      </c>
-      <c r="I84" s="8" t="s">
-        <v>375</v>
       </c>
       <c r="J84" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5571,29 +5542,29 @@
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="B85" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="B85" s="5" t="s">
+      <c r="C85" s="5" t="s">
         <v>377</v>
       </c>
-      <c r="C85" s="5" t="s">
-        <v>378</v>
-      </c>
       <c r="D85" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E85" s="5" t="s">
         <v>71</v>
       </c>
       <c r="F85" s="3"/>
       <c r="G85" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H85" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="I85" s="5" t="s">
         <v>379</v>
-      </c>
-      <c r="I85" s="5" t="s">
-        <v>380</v>
       </c>
       <c r="J85" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5602,31 +5573,31 @@
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="B86" s="5" t="s">
         <v>381</v>
       </c>
-      <c r="B86" s="5" t="s">
+      <c r="C86" s="5" t="s">
         <v>382</v>
       </c>
-      <c r="C86" s="5" t="s">
-        <v>383</v>
-      </c>
       <c r="D86" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E86" s="5" t="s">
         <v>119</v>
       </c>
       <c r="F86" s="12" t="s">
+        <v>383</v>
+      </c>
+      <c r="G86" s="5" t="s">
+        <v>595</v>
+      </c>
+      <c r="H86" s="5" t="s">
         <v>384</v>
       </c>
-      <c r="G86" s="5" t="s">
-        <v>596</v>
-      </c>
-      <c r="H86" s="5" t="s">
+      <c r="I86" s="15" t="s">
         <v>385</v>
-      </c>
-      <c r="I86" s="15" t="s">
-        <v>386</v>
       </c>
       <c r="J86" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5635,16 +5606,16 @@
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="B87" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="B87" s="5" t="s">
-        <v>388</v>
-      </c>
       <c r="C87" s="5" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>78</v>
@@ -5653,10 +5624,10 @@
         <v>95</v>
       </c>
       <c r="H87" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="I87" s="15" t="s">
         <v>389</v>
-      </c>
-      <c r="I87" s="15" t="s">
-        <v>390</v>
       </c>
       <c r="J87" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5665,29 +5636,29 @@
     </row>
     <row r="88" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="B88" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="C88" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="C88" s="5" t="s">
-        <v>393</v>
-      </c>
       <c r="D88" s="5" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="E88" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F88" s="5"/>
       <c r="G88" s="5" t="s">
         <v>127</v>
       </c>
       <c r="H88" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="I88" s="5" t="s">
         <v>394</v>
-      </c>
-      <c r="I88" s="5" t="s">
-        <v>395</v>
       </c>
       <c r="J88" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5696,31 +5667,31 @@
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="B89" s="3" t="s">
         <v>396</v>
       </c>
-      <c r="B89" s="3" t="s">
-        <v>397</v>
-      </c>
       <c r="C89" s="3" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>41</v>
       </c>
       <c r="F89" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H89" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="I89" s="3" t="s">
         <v>398</v>
-      </c>
-      <c r="I89" s="3" t="s">
-        <v>399</v>
       </c>
       <c r="J89" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5729,16 +5700,16 @@
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>78</v>
@@ -5746,7 +5717,7 @@
       <c r="F90" s="5"/>
       <c r="H90" s="5"/>
       <c r="I90" s="5" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="J90" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5755,16 +5726,16 @@
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="B91" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="B91" s="5" t="s">
-        <v>403</v>
-      </c>
       <c r="C91" s="5" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E91" s="5"/>
       <c r="F91" s="5"/>
@@ -5772,10 +5743,10 @@
         <v>54</v>
       </c>
       <c r="H91" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="I91" s="8" t="s">
         <v>404</v>
-      </c>
-      <c r="I91" s="8" t="s">
-        <v>405</v>
       </c>
       <c r="J91" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5784,27 +5755,27 @@
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="B92" s="5" t="s">
         <v>406</v>
       </c>
-      <c r="B92" s="5" t="s">
-        <v>407</v>
-      </c>
       <c r="C92" s="5" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
       <c r="G92" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="H92" s="5" t="s">
         <v>408</v>
       </c>
-      <c r="H92" s="5" t="s">
+      <c r="I92" s="8" t="s">
         <v>409</v>
-      </c>
-      <c r="I92" s="8" t="s">
-        <v>410</v>
       </c>
       <c r="J92" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5813,26 +5784,26 @@
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="B93" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="B93" s="5" t="s">
-        <v>412</v>
-      </c>
       <c r="C93" s="5" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E93" s="5"/>
       <c r="G93" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H93" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="I93" s="8" t="s">
         <v>413</v>
-      </c>
-      <c r="I93" s="8" t="s">
-        <v>414</v>
       </c>
       <c r="J93" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5841,29 +5812,29 @@
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="B94" s="5" t="s">
         <v>415</v>
       </c>
-      <c r="B94" s="5" t="s">
+      <c r="C94" s="5" t="s">
         <v>416</v>
-      </c>
-      <c r="C94" s="5" t="s">
-        <v>417</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E94" s="5"/>
       <c r="F94" s="5" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="G94" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H94" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="I94" s="5" t="s">
         <v>418</v>
-      </c>
-      <c r="I94" s="5" t="s">
-        <v>419</v>
       </c>
       <c r="J94" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5872,29 +5843,29 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="C95" s="5" t="s">
         <v>420</v>
-      </c>
-      <c r="B95" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="C95" s="5" t="s">
-        <v>421</v>
       </c>
       <c r="D95" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E95" s="5"/>
       <c r="F95" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="G95" s="5" t="s">
         <v>422</v>
       </c>
-      <c r="G95" s="5" t="s">
+      <c r="H95" s="5" t="s">
         <v>423</v>
       </c>
-      <c r="H95" s="5" t="s">
+      <c r="I95" s="15" t="s">
         <v>424</v>
-      </c>
-      <c r="I95" s="15" t="s">
-        <v>425</v>
       </c>
       <c r="J95" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5903,28 +5874,28 @@
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="B96" s="5" t="s">
         <v>426</v>
       </c>
-      <c r="B96" s="5" t="s">
+      <c r="C96" s="5" t="s">
         <v>427</v>
       </c>
-      <c r="C96" s="5" t="s">
-        <v>428</v>
-      </c>
       <c r="D96" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E96" s="5" t="s">
         <v>71</v>
       </c>
       <c r="G96" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="H96" s="5" t="s">
         <v>429</v>
       </c>
-      <c r="H96" s="5" t="s">
+      <c r="I96" s="5" t="s">
         <v>430</v>
-      </c>
-      <c r="I96" s="5" t="s">
-        <v>431</v>
       </c>
       <c r="J96" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5933,16 +5904,16 @@
     </row>
     <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B97" s="5" t="s">
         <v>432</v>
       </c>
-      <c r="B97" s="5" t="s">
-        <v>433</v>
-      </c>
       <c r="C97" s="5" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E97" s="5"/>
       <c r="F97" s="5"/>
@@ -5950,10 +5921,10 @@
         <v>89</v>
       </c>
       <c r="H97" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="I97" s="8" t="s">
         <v>434</v>
-      </c>
-      <c r="I97" s="8" t="s">
-        <v>435</v>
       </c>
       <c r="J97" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5962,29 +5933,29 @@
     </row>
     <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="B98" s="5" t="s">
         <v>436</v>
       </c>
-      <c r="B98" s="5" t="s">
+      <c r="C98" s="5" t="s">
         <v>437</v>
-      </c>
-      <c r="C98" s="5" t="s">
-        <v>438</v>
       </c>
       <c r="D98" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E98" s="5"/>
       <c r="F98" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="G98" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="H98" s="5" t="s">
         <v>439</v>
       </c>
-      <c r="G98" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="H98" s="5" t="s">
+      <c r="I98" s="5" t="s">
         <v>440</v>
-      </c>
-      <c r="I98" s="5" t="s">
-        <v>441</v>
       </c>
       <c r="J98" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5993,29 +5964,29 @@
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="B99" s="3" t="s">
         <v>442</v>
       </c>
-      <c r="B99" s="3" t="s">
+      <c r="C99" s="5" t="s">
         <v>443</v>
-      </c>
-      <c r="C99" s="5" t="s">
-        <v>444</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E99" s="5"/>
       <c r="F99" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="G99" s="3" t="s">
         <v>422</v>
       </c>
-      <c r="G99" s="3" t="s">
-        <v>423</v>
-      </c>
       <c r="H99" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="I99" s="3" t="s">
         <v>445</v>
-      </c>
-      <c r="I99" s="3" t="s">
-        <v>446</v>
       </c>
       <c r="J99" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6024,13 +5995,13 @@
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="B100" s="5" t="s">
         <v>447</v>
       </c>
-      <c r="B100" s="5" t="s">
+      <c r="C100" s="5" t="s">
         <v>448</v>
-      </c>
-      <c r="C100" s="5" t="s">
-        <v>449</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>103</v>
@@ -6043,10 +6014,10 @@
         <v>71</v>
       </c>
       <c r="H100" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="I100" s="15" t="s">
         <v>450</v>
-      </c>
-      <c r="I100" s="15" t="s">
-        <v>451</v>
       </c>
       <c r="J100" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6055,16 +6026,16 @@
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="18" t="s">
+        <v>754</v>
+      </c>
+      <c r="B101" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="C101" s="18" t="s">
         <v>755</v>
       </c>
-      <c r="B101" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="C101" s="18" t="s">
-        <v>756</v>
-      </c>
       <c r="D101" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E101" t="s">
         <v>67</v>
@@ -6074,10 +6045,10 @@
         <v>127</v>
       </c>
       <c r="H101" s="18" t="s">
+        <v>756</v>
+      </c>
+      <c r="I101" s="6" t="s">
         <v>757</v>
-      </c>
-      <c r="I101" s="6" t="s">
-        <v>758</v>
       </c>
       <c r="J101" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6086,29 +6057,29 @@
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
+        <v>451</v>
+      </c>
+      <c r="B102" t="s">
         <v>452</v>
       </c>
-      <c r="B102" t="s">
-        <v>453</v>
-      </c>
       <c r="C102" s="5" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>27</v>
       </c>
       <c r="E102" s="5"/>
       <c r="F102" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="G102" s="5" t="s">
         <v>71</v>
       </c>
       <c r="H102" t="s">
+        <v>454</v>
+      </c>
+      <c r="I102" s="8" t="s">
         <v>455</v>
-      </c>
-      <c r="I102" s="8" t="s">
-        <v>456</v>
       </c>
       <c r="J102" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6117,29 +6088,29 @@
     </row>
     <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A103" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="B103" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="B103" s="3" t="s">
-        <v>458</v>
-      </c>
       <c r="C103" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D103" s="5" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E103" s="3" t="s">
         <v>41</v>
       </c>
       <c r="F103" s="12"/>
       <c r="G103" s="3" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="H103" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="I103" s="3" t="s">
         <v>459</v>
-      </c>
-      <c r="I103" s="3" t="s">
-        <v>460</v>
       </c>
       <c r="J103" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6148,29 +6119,29 @@
     </row>
     <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A104" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="B104" s="5" t="s">
         <v>461</v>
       </c>
-      <c r="B104" s="5" t="s">
+      <c r="C104" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="D104" s="5" t="s">
         <v>462</v>
-      </c>
-      <c r="C104" s="5" t="s">
-        <v>645</v>
-      </c>
-      <c r="D104" s="5" t="s">
-        <v>463</v>
       </c>
       <c r="E104" s="5"/>
       <c r="F104" s="5" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G104" s="5" t="s">
         <v>60</v>
       </c>
       <c r="H104" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="I104" s="15" t="s">
         <v>465</v>
-      </c>
-      <c r="I104" s="15" t="s">
-        <v>466</v>
       </c>
       <c r="J104" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6179,24 +6150,24 @@
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B105" s="5" t="s">
         <v>467</v>
-      </c>
-      <c r="B105" s="5" t="s">
-        <v>468</v>
       </c>
       <c r="C105" s="5"/>
       <c r="D105" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E105" s="5" t="s">
         <v>71</v>
       </c>
       <c r="F105" s="5"/>
       <c r="H105" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="I105" s="5" t="s">
         <v>469</v>
-      </c>
-      <c r="I105" s="5" t="s">
-        <v>470</v>
       </c>
       <c r="J105" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6205,29 +6176,29 @@
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="B106" s="5" t="s">
         <v>471</v>
       </c>
-      <c r="B106" s="5" t="s">
-        <v>472</v>
-      </c>
       <c r="C106" s="5" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D106" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E106" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="F106" s="3"/>
       <c r="G106" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="H106" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="I106" s="15" t="s">
         <v>473</v>
-      </c>
-      <c r="I106" s="15" t="s">
-        <v>474</v>
       </c>
       <c r="J106" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6236,25 +6207,25 @@
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="B107" s="5" t="s">
         <v>475</v>
-      </c>
-      <c r="B107" s="5" t="s">
-        <v>476</v>
       </c>
       <c r="C107" s="5"/>
       <c r="D107" s="5" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="E107" s="5"/>
       <c r="F107" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="G107" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H107" s="5"/>
       <c r="I107" s="8" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="J107" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6263,13 +6234,13 @@
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
+        <v>479</v>
+      </c>
+      <c r="B108" t="s">
         <v>480</v>
       </c>
-      <c r="B108" t="s">
+      <c r="C108" s="7" t="s">
         <v>481</v>
-      </c>
-      <c r="C108" s="7" t="s">
-        <v>482</v>
       </c>
       <c r="D108" t="s">
         <v>27</v>
@@ -6278,13 +6249,13 @@
         <v>78</v>
       </c>
       <c r="F108" s="5" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="G108" t="s">
         <v>95</v>
       </c>
       <c r="I108" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="J108" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6293,29 +6264,29 @@
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="B109" s="5" t="s">
         <v>485</v>
       </c>
-      <c r="B109" s="5" t="s">
-        <v>486</v>
-      </c>
       <c r="C109" s="5" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E109" s="5"/>
       <c r="F109" s="5" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="G109" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H109" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="I109" s="3" t="s">
         <v>488</v>
-      </c>
-      <c r="I109" s="3" t="s">
-        <v>489</v>
       </c>
       <c r="J109" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6324,13 +6295,13 @@
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B110" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="C110" s="5" t="s">
         <v>490</v>
-      </c>
-      <c r="C110" s="5" t="s">
-        <v>491</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>13</v>
@@ -6339,16 +6310,16 @@
         <v>29</v>
       </c>
       <c r="F110" s="5" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="G110" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H110" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="I110" s="3" t="s">
         <v>492</v>
-      </c>
-      <c r="I110" s="3" t="s">
-        <v>493</v>
       </c>
       <c r="J110" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6357,13 +6328,13 @@
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
+        <v>493</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="C111" s="16" t="s">
         <v>494</v>
-      </c>
-      <c r="B111" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="C111" s="16" t="s">
-        <v>495</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>13</v>
@@ -6376,10 +6347,10 @@
         <v>89</v>
       </c>
       <c r="H111" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="I111" s="3" t="s">
         <v>496</v>
-      </c>
-      <c r="I111" s="3" t="s">
-        <v>497</v>
       </c>
       <c r="J111" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6388,13 +6359,13 @@
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="C112" s="5" t="s">
         <v>498</v>
-      </c>
-      <c r="B112" s="5" t="s">
-        <v>453</v>
-      </c>
-      <c r="C112" s="5" t="s">
-        <v>499</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>27</v>
@@ -6403,12 +6374,12 @@
         <v>78</v>
       </c>
       <c r="F112" s="5" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="G112" s="4"/>
       <c r="H112" s="3"/>
       <c r="I112" s="6" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="J112" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6417,29 +6388,29 @@
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="B113" s="5" t="s">
         <v>502</v>
       </c>
-      <c r="B113" s="5" t="s">
+      <c r="C113" s="5" t="s">
         <v>503</v>
-      </c>
-      <c r="C113" s="5" t="s">
-        <v>504</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E113" s="5"/>
       <c r="F113" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="G113" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="H113" s="3" t="s">
         <v>505</v>
       </c>
-      <c r="G113" s="5" t="s">
-        <v>304</v>
-      </c>
-      <c r="H113" s="3" t="s">
+      <c r="I113" s="15" t="s">
         <v>506</v>
-      </c>
-      <c r="I113" s="15" t="s">
-        <v>507</v>
       </c>
       <c r="J113" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6448,16 +6419,16 @@
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B114" s="5" t="s">
         <v>508</v>
       </c>
-      <c r="B114" s="5" t="s">
-        <v>509</v>
-      </c>
       <c r="C114" s="5" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D114" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E114" s="5"/>
       <c r="F114" s="5"/>
@@ -6465,10 +6436,10 @@
         <v>21</v>
       </c>
       <c r="H114" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="I114" s="8" t="s">
         <v>510</v>
-      </c>
-      <c r="I114" s="8" t="s">
-        <v>511</v>
       </c>
       <c r="J114" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6477,25 +6448,25 @@
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
+        <v>511</v>
+      </c>
+      <c r="B115" t="s">
         <v>512</v>
       </c>
-      <c r="B115" t="s">
+      <c r="C115" t="s">
+        <v>638</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>694</v>
+      </c>
+      <c r="G115" t="s">
+        <v>596</v>
+      </c>
+      <c r="H115" s="5" t="s">
         <v>513</v>
       </c>
-      <c r="C115" t="s">
-        <v>639</v>
-      </c>
-      <c r="D115" s="5" t="s">
-        <v>695</v>
-      </c>
-      <c r="G115" t="s">
-        <v>597</v>
-      </c>
-      <c r="H115" s="5" t="s">
+      <c r="I115" s="8" t="s">
         <v>514</v>
-      </c>
-      <c r="I115" s="8" t="s">
-        <v>515</v>
       </c>
       <c r="J115" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6504,14 +6475,14 @@
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="B116" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C116" s="14"/>
       <c r="D116" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E116" s="5" t="s">
         <v>78</v>
@@ -6520,10 +6491,10 @@
         <v>79</v>
       </c>
       <c r="H116" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I116" s="6" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="J116" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6532,23 +6503,23 @@
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
+        <v>515</v>
+      </c>
+      <c r="B117" t="s">
         <v>516</v>
-      </c>
-      <c r="B117" t="s">
-        <v>517</v>
       </c>
       <c r="C117" s="17"/>
       <c r="D117" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="G117" t="s">
         <v>29</v>
       </c>
       <c r="H117" t="s">
+        <v>517</v>
+      </c>
+      <c r="I117" s="8" t="s">
         <v>518</v>
-      </c>
-      <c r="I117" s="8" t="s">
-        <v>519</v>
       </c>
       <c r="J117" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6557,27 +6528,27 @@
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B118" t="s">
         <v>76</v>
       </c>
       <c r="C118" s="5"/>
       <c r="D118" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>78</v>
       </c>
       <c r="F118" s="5"/>
       <c r="G118" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="H118" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="H118" s="5" t="s">
-        <v>310</v>
-      </c>
       <c r="I118" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="J118" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6586,27 +6557,27 @@
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
+        <v>655</v>
+      </c>
+      <c r="B119" t="s">
         <v>656</v>
       </c>
-      <c r="B119" t="s">
-        <v>657</v>
-      </c>
       <c r="C119" s="16" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="D119" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E119" s="5"/>
       <c r="F119" s="3"/>
       <c r="G119" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="H119" t="s">
+        <v>658</v>
+      </c>
+      <c r="I119" s="6" t="s">
         <v>659</v>
-      </c>
-      <c r="I119" s="6" t="s">
-        <v>660</v>
       </c>
       <c r="J119" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6615,28 +6586,28 @@
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B120" t="s">
         <v>51</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="D120" t="s">
         <v>13</v>
       </c>
       <c r="F120" s="5" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="G120" t="s">
         <v>29</v>
       </c>
       <c r="H120" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="I120" s="3" t="s">
         <v>523</v>
-      </c>
-      <c r="I120" s="3" t="s">
-        <v>524</v>
       </c>
       <c r="J120" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6645,14 +6616,14 @@
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="B121" t="s">
         <v>124</v>
       </c>
       <c r="C121" s="5"/>
       <c r="D121" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E121" s="5" t="s">
         <v>78</v>
@@ -6661,10 +6632,10 @@
         <v>79</v>
       </c>
       <c r="H121" t="s">
+        <v>736</v>
+      </c>
+      <c r="I121" s="6" t="s">
         <v>737</v>
-      </c>
-      <c r="I121" s="6" t="s">
-        <v>738</v>
       </c>
       <c r="J121" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6673,16 +6644,16 @@
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="C122" s="5" t="s">
         <v>525</v>
       </c>
-      <c r="B122" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="C122" s="5" t="s">
-        <v>526</v>
-      </c>
       <c r="D122" s="5" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E122" s="5" t="s">
         <v>78</v>
@@ -6692,7 +6663,7 @@
         <v>114</v>
       </c>
       <c r="I122" s="15" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="J122" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6701,27 +6672,27 @@
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="B123" s="5" t="s">
         <v>528</v>
       </c>
-      <c r="B123" s="5" t="s">
-        <v>529</v>
-      </c>
       <c r="C123" s="5" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E123" s="5"/>
       <c r="F123" s="5" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="G123" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H123" s="3"/>
       <c r="I123" s="3" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="J123" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6730,16 +6701,16 @@
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
+        <v>531</v>
+      </c>
+      <c r="B124" t="s">
         <v>532</v>
       </c>
-      <c r="B124" t="s">
-        <v>533</v>
-      </c>
       <c r="C124" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E124" s="5"/>
       <c r="F124" s="5"/>
@@ -6753,29 +6724,29 @@
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A125" s="3" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B125" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C125" s="14" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>27</v>
       </c>
       <c r="E125" s="3"/>
       <c r="F125" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="G125" s="3" t="s">
         <v>536</v>
       </c>
-      <c r="G125" s="3" t="s">
+      <c r="H125" s="3" t="s">
         <v>537</v>
       </c>
-      <c r="H125" s="3" t="s">
+      <c r="I125" s="3" t="s">
         <v>538</v>
-      </c>
-      <c r="I125" s="3" t="s">
-        <v>539</v>
       </c>
       <c r="J125" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6784,14 +6755,14 @@
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A126" s="3" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C126" s="3"/>
       <c r="D126" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E126" s="3" t="s">
         <v>41</v>
@@ -6799,10 +6770,10 @@
       <c r="F126" s="3"/>
       <c r="G126" s="3"/>
       <c r="H126" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="I126" s="3" t="s">
         <v>541</v>
-      </c>
-      <c r="I126" s="3" t="s">
-        <v>542</v>
       </c>
       <c r="J126" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6811,28 +6782,28 @@
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A127" s="5" t="s">
+        <v>542</v>
+      </c>
+      <c r="B127" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="B127" s="5" t="s">
+      <c r="C127" s="5" t="s">
         <v>544</v>
       </c>
-      <c r="C127" s="5" t="s">
-        <v>545</v>
-      </c>
       <c r="D127" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E127" s="5" t="s">
         <v>78</v>
       </c>
       <c r="G127" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H127" s="5" t="s">
+        <v>545</v>
+      </c>
+      <c r="I127" s="15" t="s">
         <v>546</v>
-      </c>
-      <c r="I127" s="15" t="s">
-        <v>547</v>
       </c>
       <c r="J127" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6841,27 +6812,27 @@
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B128" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E128" s="5"/>
       <c r="F128" s="3"/>
       <c r="G128" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="H128" t="s">
+        <v>661</v>
+      </c>
+      <c r="I128" s="6" t="s">
         <v>662</v>
-      </c>
-      <c r="I128" s="6" t="s">
-        <v>663</v>
       </c>
       <c r="J128" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6870,29 +6841,29 @@
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B129" s="5" t="s">
         <v>548</v>
       </c>
-      <c r="B129" s="5" t="s">
-        <v>549</v>
-      </c>
       <c r="C129" s="5" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D129" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E129" s="5" t="s">
         <v>41</v>
       </c>
       <c r="F129" s="5"/>
       <c r="G129" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="H129" s="5" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="I129" s="8" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="J129" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6901,31 +6872,31 @@
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A130" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="B130" s="3" t="s">
         <v>551</v>
       </c>
-      <c r="B130" s="3" t="s">
+      <c r="C130" s="5" t="s">
         <v>552</v>
       </c>
-      <c r="C130" s="5" t="s">
+      <c r="D130" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="E130" t="s">
         <v>553</v>
       </c>
-      <c r="D130" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="E130" t="s">
+      <c r="F130" s="3" t="s">
         <v>554</v>
       </c>
-      <c r="F130" s="3" t="s">
+      <c r="G130" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="H130" s="3" t="s">
         <v>555</v>
       </c>
-      <c r="G130" s="3" t="s">
-        <v>612</v>
-      </c>
-      <c r="H130" s="3" t="s">
+      <c r="I130" s="15" t="s">
         <v>556</v>
-      </c>
-      <c r="I130" s="15" t="s">
-        <v>557</v>
       </c>
       <c r="J130" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6934,13 +6905,13 @@
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="s">
+        <v>557</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="C131" s="5" t="s">
         <v>558</v>
-      </c>
-      <c r="B131" s="5" t="s">
-        <v>453</v>
-      </c>
-      <c r="C131" s="5" t="s">
-        <v>559</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>27</v>
@@ -6953,10 +6924,10 @@
         <v>127</v>
       </c>
       <c r="H131" s="5" t="s">
+        <v>559</v>
+      </c>
+      <c r="I131" s="15" t="s">
         <v>560</v>
-      </c>
-      <c r="I131" s="15" t="s">
-        <v>561</v>
       </c>
       <c r="J131" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6965,29 +6936,29 @@
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
+        <v>561</v>
+      </c>
+      <c r="B132" s="5" t="s">
         <v>562</v>
       </c>
-      <c r="B132" s="5" t="s">
-        <v>563</v>
-      </c>
       <c r="C132" s="5" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D132" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E132" s="5" t="s">
         <v>41</v>
       </c>
       <c r="F132" s="5"/>
       <c r="G132" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="H132" t="s">
+        <v>563</v>
+      </c>
+      <c r="I132" s="8" t="s">
         <v>564</v>
-      </c>
-      <c r="I132" s="8" t="s">
-        <v>565</v>
       </c>
       <c r="J132" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6996,29 +6967,29 @@
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A133" s="5" t="s">
+        <v>565</v>
+      </c>
+      <c r="B133" s="5" t="s">
         <v>566</v>
       </c>
-      <c r="B133" s="5" t="s">
-        <v>567</v>
-      </c>
       <c r="C133" s="5" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>103</v>
       </c>
       <c r="E133" s="5"/>
       <c r="F133" s="5" t="s">
+        <v>567</v>
+      </c>
+      <c r="G133" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="H133" s="5" t="s">
         <v>568</v>
       </c>
-      <c r="G133" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="H133" s="5" t="s">
+      <c r="I133" s="15" t="s">
         <v>569</v>
-      </c>
-      <c r="I133" s="15" t="s">
-        <v>570</v>
       </c>
       <c r="J133" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7027,22 +6998,22 @@
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B134" t="s">
+        <v>573</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>694</v>
+      </c>
+      <c r="G134" t="s">
+        <v>287</v>
+      </c>
+      <c r="H134" s="5" t="s">
         <v>574</v>
       </c>
-      <c r="D134" s="5" t="s">
-        <v>695</v>
-      </c>
-      <c r="G134" t="s">
-        <v>288</v>
-      </c>
-      <c r="H134" s="5" t="s">
+      <c r="I134" s="8" t="s">
         <v>575</v>
-      </c>
-      <c r="I134" s="8" t="s">
-        <v>576</v>
       </c>
       <c r="J134" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7051,27 +7022,27 @@
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A135" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="B135" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="B135" s="5" t="s">
-        <v>572</v>
-      </c>
       <c r="C135" s="5" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D135" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E135" s="5"/>
       <c r="F135" s="5"/>
       <c r="G135" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="H135" s="5" t="s">
         <v>408</v>
       </c>
-      <c r="H135" s="5" t="s">
-        <v>409</v>
-      </c>
       <c r="I135" s="8" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="J135" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7080,31 +7051,31 @@
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B136" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>41</v>
       </c>
       <c r="F136" t="s">
+        <v>599</v>
+      </c>
+      <c r="G136" t="s">
+        <v>613</v>
+      </c>
+      <c r="H136" t="s">
         <v>600</v>
       </c>
-      <c r="G136" t="s">
-        <v>614</v>
-      </c>
-      <c r="H136" t="s">
+      <c r="I136" s="6" t="s">
         <v>601</v>
-      </c>
-      <c r="I136" s="6" t="s">
-        <v>602</v>
       </c>
       <c r="J136" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7113,14 +7084,14 @@
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="B137" s="5" t="s">
         <v>577</v>
-      </c>
-      <c r="B137" s="5" t="s">
-        <v>578</v>
       </c>
       <c r="C137" s="5"/>
       <c r="D137" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E137" s="5"/>
       <c r="F137" s="5"/>
@@ -7128,10 +7099,10 @@
         <v>54</v>
       </c>
       <c r="H137" s="5" t="s">
+        <v>578</v>
+      </c>
+      <c r="I137" s="8" t="s">
         <v>579</v>
-      </c>
-      <c r="I137" s="8" t="s">
-        <v>580</v>
       </c>
       <c r="J137" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7140,16 +7111,16 @@
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="s">
+        <v>580</v>
+      </c>
+      <c r="B138" s="5" t="s">
         <v>581</v>
       </c>
-      <c r="B138" s="5" t="s">
-        <v>582</v>
-      </c>
       <c r="C138" s="5" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
@@ -7157,10 +7128,10 @@
         <v>29</v>
       </c>
       <c r="H138" s="5" t="s">
+        <v>582</v>
+      </c>
+      <c r="I138" s="8" t="s">
         <v>583</v>
-      </c>
-      <c r="I138" s="8" t="s">
-        <v>584</v>
       </c>
       <c r="J138" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7169,16 +7140,16 @@
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A139" s="5" t="s">
+        <v>584</v>
+      </c>
+      <c r="B139" s="5" t="s">
         <v>585</v>
       </c>
-      <c r="B139" s="5" t="s">
-        <v>586</v>
-      </c>
       <c r="C139" s="5" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D139" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E139" s="5"/>
       <c r="F139" s="5"/>
@@ -7186,10 +7157,10 @@
         <v>54</v>
       </c>
       <c r="H139" s="5" t="s">
+        <v>586</v>
+      </c>
+      <c r="I139" s="8" t="s">
         <v>587</v>
-      </c>
-      <c r="I139" s="8" t="s">
-        <v>588</v>
       </c>
       <c r="J139" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7198,16 +7169,16 @@
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
+        <v>732</v>
+      </c>
+      <c r="B140" t="s">
         <v>733</v>
       </c>
-      <c r="B140" t="s">
-        <v>734</v>
-      </c>
       <c r="C140" s="5" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="D140" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>78</v>
@@ -7216,7 +7187,7 @@
         <v>79</v>
       </c>
       <c r="I140" s="6" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="J140" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7225,16 +7196,16 @@
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A141" s="5" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="C141" s="5" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D141" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E141" s="5"/>
       <c r="F141" s="5"/>
@@ -7242,10 +7213,10 @@
         <v>89</v>
       </c>
       <c r="H141" s="5" t="s">
+        <v>589</v>
+      </c>
+      <c r="I141" s="8" t="s">
         <v>590</v>
-      </c>
-      <c r="I141" s="8" t="s">
-        <v>591</v>
       </c>
       <c r="J141" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7254,10 +7225,10 @@
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C142" s="5"/>
       <c r="D142" s="5" t="s">
@@ -7267,16 +7238,16 @@
         <v>71</v>
       </c>
       <c r="F142" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="G142" t="s">
+        <v>428</v>
+      </c>
+      <c r="H142" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="I142" s="15" t="s">
         <v>593</v>
-      </c>
-      <c r="G142" t="s">
-        <v>429</v>
-      </c>
-      <c r="H142" s="5" t="s">
-        <v>450</v>
-      </c>
-      <c r="I142" s="15" t="s">
-        <v>594</v>
       </c>
       <c r="J142" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7285,14 +7256,14 @@
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="s">
+        <v>679</v>
+      </c>
+      <c r="B143" s="5" t="s">
         <v>680</v>
-      </c>
-      <c r="B143" s="5" t="s">
-        <v>681</v>
       </c>
       <c r="C143" s="5"/>
       <c r="D143" s="5" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="E143" s="5" t="s">
         <v>78</v>
@@ -7302,18 +7273,18 @@
         <v>78</v>
       </c>
       <c r="H143" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="I143" s="6" t="s">
         <v>682</v>
       </c>
-      <c r="I143" s="6" t="s">
-        <v>683</v>
-      </c>
       <c r="J143" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=sosthene.yamale@umontreal.ca</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="10" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="I12" r:id="rId1" display="mailto:audrey.begin-poissant@umontreal.ca" xr:uid="{708FEBAC-F938-40E8-8D55-B34C4326210F}"/>
     <hyperlink ref="I34" r:id="rId2" display="mailto:delphine.cado@umontreal.ca" xr:uid="{0E0BF38D-BCA7-4652-84E3-BBE8A015792A}"/>
@@ -7600,15 +7571,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7617,6 +7579,15 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7639,14 +7610,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7661,4 +7624,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Changements au répertoire du personnel.
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8F96EF2-FB3B-4D10-B60C-66209B778A6A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFC44DD4-D07C-4339-AA44-69472959CE76}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5460" yWindow="3560" windowWidth="30320" windowHeight="28130" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="762">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="758">
   <si>
     <t>nom</t>
   </si>
@@ -1464,21 +1464,6 @@
     <t>francois-xavier.panaccio@umontreal.ca</t>
   </si>
   <si>
-    <t>Paquet</t>
-  </si>
-  <si>
-    <t>Virginie</t>
-  </si>
-  <si>
-    <t>virginie-paquet.jpg</t>
-  </si>
-  <si>
-    <t>Impact de la recherche</t>
-  </si>
-  <si>
-    <t>virginie.paquet@umontreal.ca</t>
-  </si>
-  <si>
     <t>Patenaude</t>
   </si>
   <si>
@@ -2311,6 +2296,9 @@
   </si>
   <si>
     <t>Sciences infirmières et gérontologie</t>
+  </si>
+  <si>
+    <t>anne-marie-brien.jpg</t>
   </si>
 </sst>
 </file>
@@ -2662,10 +2650,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J143" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J143" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
-  <sortState ref="A2:J143">
-    <sortCondition ref="A1:A143"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J142" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J142" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
+  <sortState ref="A2:J142">
+    <sortCondition ref="A1:A142"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{4B04E1AF-0079-4AD2-81CA-E8A433733E21}" name="nom" dataDxfId="9"/>
@@ -3006,7 +2994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J143"/>
+  <dimension ref="A1:J142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.453125" customWidth="1"/>
@@ -3101,7 +3089,7 @@
         <v>41</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>610</v>
+        <v>605</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>21</v>
@@ -3119,14 +3107,14 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>721</v>
+        <v>716</v>
       </c>
       <c r="B4" t="s">
-        <v>722</v>
+        <v>717</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>78</v>
@@ -3138,7 +3126,7 @@
         <v>309</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>723</v>
+        <v>718</v>
       </c>
       <c r="J4" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3218,7 +3206,7 @@
         <v>40</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>41</v>
@@ -3227,7 +3215,7 @@
         <v>42</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>611</v>
+        <v>606</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>43</v>
@@ -3251,7 +3239,7 @@
         <v>47</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>41</v>
@@ -3340,16 +3328,16 @@
         <v>66</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>700</v>
+        <v>695</v>
       </c>
       <c r="E11" t="s">
         <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>535</v>
+        <v>530</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>606</v>
+        <v>601</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>68</v>
@@ -3370,10 +3358,10 @@
         <v>39</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>618</v>
+        <v>613</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>71</v>
@@ -3394,13 +3382,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="B13" t="s">
-        <v>704</v>
+        <v>699</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>747</v>
+        <v>742</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>27</v>
@@ -3416,7 +3404,7 @@
         <v>309</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
       <c r="J13" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3434,7 +3422,7 @@
         <v>77</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>78</v>
@@ -3494,10 +3482,10 @@
         <v>88</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>633</v>
+        <v>628</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
@@ -3552,10 +3540,10 @@
         <v>97</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="G18" t="s">
         <v>29</v>
@@ -3573,13 +3561,13 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>686</v>
+        <v>681</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>687</v>
+        <v>682</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>688</v>
+        <v>683</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>27</v>
@@ -3588,14 +3576,14 @@
         <v>78</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>689</v>
+        <v>684</v>
       </c>
       <c r="G19" t="s">
         <v>78</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="6" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="J19" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3635,14 +3623,14 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>729</v>
+        <v>724</v>
       </c>
       <c r="B21" t="s">
-        <v>730</v>
+        <v>725</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>78</v>
@@ -3651,7 +3639,7 @@
         <v>79</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="J21" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3697,7 +3685,7 @@
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="3" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>60</v>
@@ -3725,7 +3713,7 @@
         <v>118</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>700</v>
+        <v>695</v>
       </c>
       <c r="E24" t="s">
         <v>119</v>
@@ -3814,19 +3802,19 @@
         <v>137</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>615</v>
+        <v>610</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>71</v>
       </c>
       <c r="F27" t="s">
-        <v>614</v>
+        <v>609</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>609</v>
+        <v>604</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>138</v>
@@ -3847,15 +3835,15 @@
         <v>141</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E28" s="5"/>
       <c r="F28" s="5"/>
       <c r="G28" s="5" t="s">
-        <v>608</v>
+        <v>603</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>142</v>
@@ -3870,27 +3858,27 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>691</v>
+        <v>686</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="C29" s="5"/>
+      <c r="C29" s="5" t="s">
+        <v>757</v>
+      </c>
       <c r="D29" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>657</v>
-      </c>
+        <v>689</v>
+      </c>
+      <c r="E29" s="5"/>
       <c r="F29" s="5"/>
       <c r="G29" t="s">
         <v>29</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>692</v>
+        <v>687</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>693</v>
+        <v>688</v>
       </c>
       <c r="J29" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3908,7 +3896,7 @@
         <v>146</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>700</v>
+        <v>695</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>60</v>
@@ -3927,13 +3915,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
-        <v>673</v>
+        <v>668</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>674</v>
+        <v>669</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>675</v>
+        <v>670</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>13</v>
@@ -3942,16 +3930,16 @@
         <v>119</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>676</v>
+        <v>671</v>
       </c>
       <c r="G31" t="s">
         <v>15</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>678</v>
+        <v>673</v>
       </c>
       <c r="J31" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3966,10 +3954,10 @@
         <v>150</v>
       </c>
       <c r="C32" t="s">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
@@ -3987,14 +3975,14 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>738</v>
+        <v>733</v>
       </c>
       <c r="B33" t="s">
-        <v>739</v>
+        <v>734</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>78</v>
@@ -4003,10 +3991,10 @@
         <v>79</v>
       </c>
       <c r="H33" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="J33" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4021,7 +4009,7 @@
         <v>154</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>13</v>
@@ -4030,7 +4018,7 @@
         <v>119</v>
       </c>
       <c r="F34" t="s">
-        <v>761</v>
+        <v>756</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>156</v>
@@ -4054,10 +4042,10 @@
         <v>160</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>626</v>
+        <v>621</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E35" s="5"/>
       <c r="F35" s="5"/>
@@ -4114,10 +4102,10 @@
         <v>172</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="G37" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="H37" s="5" t="s">
         <v>173</v>
@@ -4132,14 +4120,14 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>741</v>
+        <v>736</v>
       </c>
       <c r="B38" t="s">
-        <v>742</v>
+        <v>737</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="E38" s="5" t="s">
         <v>78</v>
@@ -4148,10 +4136,10 @@
         <v>79</v>
       </c>
       <c r="H38" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="I38" t="s">
-        <v>743</v>
+        <v>738</v>
       </c>
       <c r="J38" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4167,7 +4155,7 @@
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>696</v>
+        <v>691</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>60</v>
@@ -4176,10 +4164,10 @@
         <v>60</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>684</v>
+        <v>679</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>683</v>
+        <v>678</v>
       </c>
       <c r="J39" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4228,7 +4216,7 @@
         <v>185</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>701</v>
+        <v>696</v>
       </c>
       <c r="E41" s="5" t="s">
         <v>78</v>
@@ -4255,7 +4243,7 @@
         <v>190</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>654</v>
+        <v>649</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>27</v>
@@ -4289,7 +4277,7 @@
         <v>196</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E43" t="s">
         <v>197</v>
@@ -4298,7 +4286,7 @@
         <v>198</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>595</v>
+        <v>590</v>
       </c>
       <c r="H43" s="5" t="s">
         <v>199</v>
@@ -4350,7 +4338,7 @@
         <v>208</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>645</v>
+        <v>640</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>13</v>
@@ -4415,7 +4403,7 @@
         <v>220</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>700</v>
+        <v>695</v>
       </c>
       <c r="E47" s="5"/>
       <c r="F47" t="s">
@@ -4453,7 +4441,7 @@
         <v>228</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="H48" s="5" t="s">
         <v>229</v>
@@ -4505,10 +4493,10 @@
         <v>238</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>636</v>
+        <v>631</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
@@ -4534,10 +4522,10 @@
         <v>243</v>
       </c>
       <c r="C51" t="s">
-        <v>653</v>
+        <v>648</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="G51" t="s">
         <v>29</v>
@@ -4586,10 +4574,10 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>668</v>
+        <v>663</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>669</v>
+        <v>664</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
@@ -4599,16 +4587,16 @@
         <v>119</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>670</v>
+        <v>665</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>671</v>
+        <v>666</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>672</v>
+        <v>667</v>
       </c>
       <c r="J53" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4623,10 +4611,10 @@
         <v>253</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>641</v>
+        <v>636</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="G54" t="s">
         <v>29</v>
@@ -4653,7 +4641,7 @@
         <v>258</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E55" s="5" t="s">
         <v>119</v>
@@ -4686,7 +4674,7 @@
         <v>263</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E56" s="11" t="s">
         <v>264</v>
@@ -4717,7 +4705,7 @@
       </c>
       <c r="C57" s="16"/>
       <c r="D57" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E57" s="5"/>
       <c r="F57" s="5"/>
@@ -4774,10 +4762,10 @@
         <v>280</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>647</v>
+        <v>642</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>701</v>
+        <v>696</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5" t="s">
@@ -4835,7 +4823,7 @@
       </c>
       <c r="C61" s="5"/>
       <c r="D61" s="3" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="E61" s="5" t="s">
         <v>119</v>
@@ -4863,7 +4851,7 @@
         <v>292</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>703</v>
+        <v>698</v>
       </c>
       <c r="E62" s="5" t="s">
         <v>239</v>
@@ -4912,10 +4900,10 @@
     </row>
     <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>720</v>
+        <v>715</v>
       </c>
       <c r="B64" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
       <c r="C64" s="5"/>
       <c r="D64" s="5" t="s">
@@ -4932,7 +4920,7 @@
         <v>309</v>
       </c>
       <c r="I64" s="15" t="s">
-        <v>707</v>
+        <v>702</v>
       </c>
       <c r="J64" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4948,7 +4936,7 @@
       </c>
       <c r="C65" s="5"/>
       <c r="D65" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
@@ -4956,7 +4944,7 @@
         <v>303</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="I65" s="8" t="s">
         <v>304</v>
@@ -4974,7 +4962,7 @@
         <v>306</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>629</v>
+        <v>624</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>27</v>
@@ -4992,7 +4980,7 @@
         <v>309</v>
       </c>
       <c r="I66" s="5" t="s">
-        <v>708</v>
+        <v>703</v>
       </c>
       <c r="J66" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5001,16 +4989,16 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>718</v>
+        <v>713</v>
       </c>
       <c r="B67" t="s">
         <v>291</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>746</v>
+        <v>741</v>
       </c>
       <c r="D67" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
       <c r="E67" s="5" t="s">
         <v>78</v>
@@ -5023,7 +5011,7 @@
         <v>309</v>
       </c>
       <c r="I67" t="s">
-        <v>710</v>
+        <v>705</v>
       </c>
       <c r="J67" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5124,16 +5112,16 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
       <c r="B71" t="s">
-        <v>714</v>
+        <v>709</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>748</v>
+        <v>743</v>
       </c>
       <c r="D71" t="s">
-        <v>716</v>
+        <v>711</v>
       </c>
       <c r="E71" s="5" t="s">
         <v>78</v>
@@ -5146,7 +5134,7 @@
         <v>309</v>
       </c>
       <c r="I71" t="s">
-        <v>711</v>
+        <v>706</v>
       </c>
       <c r="J71" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5164,7 +5152,7 @@
         <v>329</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>700</v>
+        <v>695</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>71</v>
@@ -5197,7 +5185,7 @@
       </c>
       <c r="E73" s="5"/>
       <c r="F73" s="5" t="s">
-        <v>665</v>
+        <v>660</v>
       </c>
       <c r="G73" s="5" t="s">
         <v>29</v>
@@ -5221,10 +5209,10 @@
         <v>338</v>
       </c>
       <c r="C74" t="s">
-        <v>649</v>
+        <v>644</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="G74" t="s">
         <v>287</v>
@@ -5242,14 +5230,14 @@
     </row>
     <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="B75" t="s">
-        <v>725</v>
+        <v>720</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>78</v>
@@ -5262,7 +5250,7 @@
         <v>309</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>726</v>
+        <v>721</v>
       </c>
       <c r="J75" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5278,7 +5266,7 @@
       </c>
       <c r="C76" s="5"/>
       <c r="D76" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E76" s="5"/>
       <c r="F76" s="5"/>
@@ -5289,7 +5277,7 @@
         <v>342</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>594</v>
+        <v>589</v>
       </c>
       <c r="J76" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5304,10 +5292,10 @@
         <v>97</v>
       </c>
       <c r="C77" t="s">
-        <v>646</v>
+        <v>641</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="G77" t="s">
         <v>29</v>
@@ -5343,7 +5331,7 @@
         <v>349</v>
       </c>
       <c r="G78" s="5" t="s">
-        <v>608</v>
+        <v>603</v>
       </c>
       <c r="H78" s="5" t="s">
         <v>350</v>
@@ -5367,7 +5355,7 @@
         <v>354</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E79" s="5" t="s">
         <v>119</v>
@@ -5391,27 +5379,27 @@
     </row>
     <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A80" s="18" t="s">
-        <v>749</v>
+        <v>744</v>
       </c>
       <c r="B80" s="18" t="s">
-        <v>750</v>
+        <v>745</v>
       </c>
       <c r="C80" s="18"/>
       <c r="D80" s="18" t="s">
-        <v>751</v>
+        <v>746</v>
       </c>
       <c r="E80" s="18" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="F80" s="18"/>
       <c r="G80" s="18" t="s">
         <v>127</v>
       </c>
       <c r="H80" s="18" t="s">
-        <v>752</v>
+        <v>747</v>
       </c>
       <c r="I80" s="6" t="s">
-        <v>753</v>
+        <v>748</v>
       </c>
       <c r="J80" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5426,10 +5414,10 @@
         <v>291</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E81" s="11" t="s">
         <v>264</v>
@@ -5459,10 +5447,10 @@
         <v>362</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>603</v>
+        <v>598</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="G82" t="s">
         <v>29</v>
@@ -5493,7 +5481,7 @@
       </c>
       <c r="E83" s="5"/>
       <c r="F83" s="5" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="G83" s="5" t="s">
         <v>29</v>
@@ -5517,7 +5505,7 @@
         <v>371</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>639</v>
+        <v>634</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>27</v>
@@ -5551,7 +5539,7 @@
         <v>377</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E85" s="5" t="s">
         <v>71</v>
@@ -5582,7 +5570,7 @@
         <v>382</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E86" s="5" t="s">
         <v>119</v>
@@ -5591,7 +5579,7 @@
         <v>383</v>
       </c>
       <c r="G86" s="5" t="s">
-        <v>595</v>
+        <v>590</v>
       </c>
       <c r="H86" s="5" t="s">
         <v>384</v>
@@ -5612,10 +5600,10 @@
         <v>387</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>78</v>
@@ -5645,7 +5633,7 @@
         <v>392</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>698</v>
+        <v>693</v>
       </c>
       <c r="E88" s="11" t="s">
         <v>264</v>
@@ -5673,19 +5661,19 @@
         <v>396</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>41</v>
       </c>
       <c r="F89" t="s">
-        <v>597</v>
+        <v>592</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>607</v>
+        <v>602</v>
       </c>
       <c r="H89" s="3" t="s">
         <v>397</v>
@@ -5706,10 +5694,10 @@
         <v>399</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>635</v>
+        <v>630</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>697</v>
+        <v>692</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>78</v>
@@ -5732,10 +5720,10 @@
         <v>402</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>637</v>
+        <v>632</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E91" s="5"/>
       <c r="F91" s="5"/>
@@ -5761,10 +5749,10 @@
         <v>406</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>652</v>
+        <v>647</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
@@ -5790,10 +5778,10 @@
         <v>411</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>651</v>
+        <v>646</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="E93" s="5"/>
       <c r="G93" s="5" t="s">
@@ -5825,7 +5813,7 @@
       </c>
       <c r="E94" s="5"/>
       <c r="F94" s="5" t="s">
-        <v>666</v>
+        <v>661</v>
       </c>
       <c r="G94" s="5" t="s">
         <v>29</v>
@@ -5883,7 +5871,7 @@
         <v>427</v>
       </c>
       <c r="D96" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E96" s="5" t="s">
         <v>71</v>
@@ -5910,10 +5898,10 @@
         <v>432</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>619</v>
+        <v>614</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E97" s="5"/>
       <c r="F97" s="5"/>
@@ -6026,16 +6014,16 @@
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="18" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="B101" s="18" t="s">
         <v>294</v>
       </c>
       <c r="C101" s="18" t="s">
-        <v>755</v>
+        <v>750</v>
       </c>
       <c r="D101" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E101" t="s">
         <v>67</v>
@@ -6045,10 +6033,10 @@
         <v>127</v>
       </c>
       <c r="H101" s="18" t="s">
-        <v>756</v>
+        <v>751</v>
       </c>
       <c r="I101" s="6" t="s">
-        <v>757</v>
+        <v>752</v>
       </c>
       <c r="J101" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6063,7 +6051,7 @@
         <v>452</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>620</v>
+        <v>615</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>27</v>
@@ -6094,17 +6082,17 @@
         <v>457</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>627</v>
+        <v>622</v>
       </c>
       <c r="D103" s="5" t="s">
-        <v>700</v>
+        <v>695</v>
       </c>
       <c r="E103" s="3" t="s">
         <v>41</v>
       </c>
       <c r="F103" s="12"/>
       <c r="G103" s="3" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="H103" s="3" t="s">
         <v>458</v>
@@ -6125,7 +6113,7 @@
         <v>461</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>644</v>
+        <v>639</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>462</v>
@@ -6157,7 +6145,7 @@
       </c>
       <c r="C105" s="5"/>
       <c r="D105" s="3" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="E105" s="5" t="s">
         <v>71</v>
@@ -6182,17 +6170,17 @@
         <v>471</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>605</v>
+        <v>600</v>
       </c>
       <c r="D106" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="E106" t="s">
-        <v>758</v>
+        <v>753</v>
       </c>
       <c r="F106" s="3"/>
       <c r="G106" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="H106" s="5" t="s">
         <v>472</v>
@@ -6233,1052 +6221,1022 @@
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A108" t="s">
+      <c r="A108" s="5" t="s">
         <v>479</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="5" t="s">
         <v>480</v>
       </c>
-      <c r="C108" s="7" t="s">
+      <c r="C108" s="5" t="s">
+        <v>611</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E108" s="5"/>
+      <c r="F108" s="5" t="s">
         <v>481</v>
       </c>
-      <c r="D108" t="s">
-        <v>27</v>
-      </c>
-      <c r="E108" t="s">
-        <v>78</v>
-      </c>
-      <c r="F108" s="5" t="s">
+      <c r="G108" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H108" s="3" t="s">
         <v>482</v>
       </c>
-      <c r="G108" t="s">
-        <v>95</v>
-      </c>
-      <c r="I108" t="s">
+      <c r="I108" s="3" t="s">
         <v>483</v>
       </c>
       <c r="J108" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=virginie.paquet@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B109" s="5" t="s">
         <v>484</v>
       </c>
-      <c r="B109" s="5" t="s">
+      <c r="C109" s="5" t="s">
         <v>485</v>
-      </c>
-      <c r="C109" s="5" t="s">
-        <v>616</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E109" s="5"/>
+      <c r="E109" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="F109" s="5" t="s">
-        <v>486</v>
+        <v>680</v>
       </c>
       <c r="G109" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H109" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="I109" s="3" t="s">
         <v>487</v>
       </c>
-      <c r="I109" s="3" t="s">
-        <v>488</v>
-      </c>
       <c r="J109" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="B110" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="C110" s="16" t="s">
         <v>489</v>
-      </c>
-      <c r="C110" s="5" t="s">
-        <v>490</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E110" s="5" t="s">
-        <v>29</v>
-      </c>
+      <c r="E110" s="5"/>
       <c r="F110" s="5" t="s">
-        <v>685</v>
+        <v>133</v>
       </c>
       <c r="G110" s="5" t="s">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="H110" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="I110" s="3" t="s">
         <v>491</v>
       </c>
-      <c r="I110" s="3" t="s">
-        <v>492</v>
-      </c>
       <c r="J110" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="C111" s="5" t="s">
         <v>493</v>
       </c>
-      <c r="B111" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="C111" s="16" t="s">
+      <c r="D111" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E111" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F111" s="5" t="s">
         <v>494</v>
       </c>
-      <c r="D111" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E111" s="5"/>
-      <c r="F111" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="G111" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="H111" s="3" t="s">
+      <c r="G111" s="4"/>
+      <c r="H111" s="3"/>
+      <c r="I111" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="I111" s="3" t="s">
-        <v>496</v>
-      </c>
       <c r="J111" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="B112" s="5" t="s">
         <v>497</v>
-      </c>
-      <c r="B112" s="5" t="s">
-        <v>452</v>
       </c>
       <c r="C112" s="5" t="s">
         <v>498</v>
       </c>
       <c r="D112" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E112" s="5" t="s">
-        <v>78</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="E112" s="5"/>
       <c r="F112" s="5" t="s">
         <v>499</v>
       </c>
-      <c r="G112" s="4"/>
-      <c r="H112" s="3"/>
-      <c r="I112" s="6" t="s">
+      <c r="G112" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="H112" s="3" t="s">
         <v>500</v>
       </c>
+      <c r="I112" s="15" t="s">
+        <v>501</v>
+      </c>
       <c r="J112" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>503</v>
+        <v>645</v>
       </c>
       <c r="D113" s="5" t="s">
-        <v>13</v>
+        <v>689</v>
       </c>
       <c r="E113" s="5"/>
-      <c r="F113" s="5" t="s">
+      <c r="F113" s="5"/>
+      <c r="G113" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H113" s="3" t="s">
         <v>504</v>
       </c>
-      <c r="G113" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="H113" s="3" t="s">
+      <c r="I113" s="8" t="s">
         <v>505</v>
       </c>
-      <c r="I113" s="15" t="s">
+      <c r="J113" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
         <v>506</v>
       </c>
-      <c r="J113" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A114" s="5" t="s">
+      <c r="B114" t="s">
         <v>507</v>
       </c>
-      <c r="B114" s="5" t="s">
+      <c r="C114" t="s">
+        <v>633</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="G114" t="s">
+        <v>591</v>
+      </c>
+      <c r="H114" s="5" t="s">
         <v>508</v>
       </c>
-      <c r="C114" s="5" t="s">
-        <v>650</v>
-      </c>
-      <c r="D114" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="E114" s="5"/>
-      <c r="F114" s="5"/>
-      <c r="G114" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H114" s="3" t="s">
+      <c r="I114" s="8" t="s">
         <v>509</v>
       </c>
-      <c r="I114" s="8" t="s">
-        <v>510</v>
-      </c>
       <c r="J114" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>511</v>
+        <v>722</v>
       </c>
       <c r="B115" t="s">
-        <v>512</v>
-      </c>
-      <c r="C115" t="s">
-        <v>638</v>
-      </c>
-      <c r="D115" s="5" t="s">
-        <v>694</v>
+        <v>452</v>
+      </c>
+      <c r="C115" s="14"/>
+      <c r="D115" t="s">
+        <v>739</v>
+      </c>
+      <c r="E115" s="5" t="s">
+        <v>78</v>
       </c>
       <c r="G115" t="s">
-        <v>596</v>
-      </c>
-      <c r="H115" s="5" t="s">
-        <v>513</v>
-      </c>
-      <c r="I115" s="8" t="s">
-        <v>514</v>
-      </c>
-      <c r="J115" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
+        <v>79</v>
+      </c>
+      <c r="H115" t="s">
+        <v>309</v>
+      </c>
+      <c r="I115" s="6" t="s">
+        <v>723</v>
+      </c>
+      <c r="J115" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>727</v>
+        <v>510</v>
       </c>
       <c r="B116" t="s">
-        <v>452</v>
-      </c>
-      <c r="C116" s="14"/>
-      <c r="D116" t="s">
-        <v>744</v>
-      </c>
-      <c r="E116" s="5" t="s">
-        <v>78</v>
+        <v>511</v>
+      </c>
+      <c r="C116" s="17"/>
+      <c r="D116" s="5" t="s">
+        <v>689</v>
       </c>
       <c r="G116" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="H116" t="s">
-        <v>309</v>
-      </c>
-      <c r="I116" s="6" t="s">
-        <v>728</v>
-      </c>
-      <c r="J116" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
+        <v>512</v>
+      </c>
+      <c r="I116" s="8" t="s">
+        <v>513</v>
+      </c>
+      <c r="J116" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>515</v>
+        <v>712</v>
       </c>
       <c r="B117" t="s">
-        <v>516</v>
-      </c>
-      <c r="C117" s="17"/>
-      <c r="D117" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="G117" t="s">
-        <v>29</v>
-      </c>
-      <c r="H117" t="s">
-        <v>517</v>
-      </c>
-      <c r="I117" s="8" t="s">
-        <v>518</v>
-      </c>
-      <c r="J117" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
+        <v>76</v>
+      </c>
+      <c r="C117" s="5"/>
+      <c r="D117" t="s">
+        <v>710</v>
+      </c>
+      <c r="E117" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F117" s="5"/>
+      <c r="G117" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="H117" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="I117" t="s">
+        <v>704</v>
+      </c>
+      <c r="J117" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>717</v>
+        <v>650</v>
       </c>
       <c r="B118" t="s">
-        <v>76</v>
-      </c>
-      <c r="C118" s="5"/>
-      <c r="D118" t="s">
-        <v>715</v>
-      </c>
-      <c r="E118" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F118" s="5"/>
-      <c r="G118" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="H118" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="I118" t="s">
-        <v>709</v>
-      </c>
-      <c r="J118" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
+        <v>651</v>
+      </c>
+      <c r="C118" s="16" t="s">
+        <v>659</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="E118" s="5"/>
+      <c r="F118" s="3"/>
+      <c r="G118" t="s">
+        <v>531</v>
+      </c>
+      <c r="H118" t="s">
+        <v>653</v>
+      </c>
+      <c r="I118" s="6" t="s">
+        <v>654</v>
+      </c>
+      <c r="J118" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>655</v>
+        <v>514</v>
       </c>
       <c r="B119" t="s">
-        <v>656</v>
-      </c>
-      <c r="C119" s="16" t="s">
-        <v>664</v>
-      </c>
-      <c r="D119" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="E119" s="5"/>
-      <c r="F119" s="3"/>
+        <v>51</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="D119" t="s">
+        <v>13</v>
+      </c>
+      <c r="F119" s="5" t="s">
+        <v>516</v>
+      </c>
       <c r="G119" t="s">
-        <v>536</v>
-      </c>
-      <c r="H119" t="s">
-        <v>658</v>
-      </c>
-      <c r="I119" s="6" t="s">
-        <v>659</v>
+        <v>29</v>
+      </c>
+      <c r="H119" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="I119" s="3" t="s">
+        <v>518</v>
       </c>
       <c r="J119" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
+        <v>730</v>
+      </c>
+      <c r="B120" t="s">
+        <v>124</v>
+      </c>
+      <c r="C120" s="5"/>
+      <c r="D120" t="s">
+        <v>739</v>
+      </c>
+      <c r="E120" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G120" t="s">
+        <v>79</v>
+      </c>
+      <c r="H120" t="s">
+        <v>731</v>
+      </c>
+      <c r="I120" s="6" t="s">
+        <v>732</v>
+      </c>
+      <c r="J120" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A121" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="B120" t="s">
-        <v>51</v>
-      </c>
-      <c r="C120" s="7" t="s">
+      <c r="B121" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="C121" s="5" t="s">
         <v>520</v>
       </c>
-      <c r="D120" t="s">
-        <v>13</v>
-      </c>
-      <c r="F120" s="5" t="s">
-        <v>521</v>
-      </c>
-      <c r="G120" t="s">
-        <v>29</v>
-      </c>
-      <c r="H120" s="3" t="s">
-        <v>522</v>
-      </c>
-      <c r="I120" s="3" t="s">
-        <v>523</v>
-      </c>
-      <c r="J120" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A121" t="s">
-        <v>735</v>
-      </c>
-      <c r="B121" t="s">
-        <v>124</v>
-      </c>
-      <c r="C121" s="5"/>
-      <c r="D121" t="s">
-        <v>744</v>
+      <c r="D121" s="5" t="s">
+        <v>695</v>
       </c>
       <c r="E121" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G121" t="s">
-        <v>79</v>
-      </c>
-      <c r="H121" t="s">
-        <v>736</v>
-      </c>
-      <c r="I121" s="6" t="s">
-        <v>737</v>
-      </c>
-      <c r="J121" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
+      <c r="F121" s="5"/>
+      <c r="H121" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I121" s="15" t="s">
+        <v>521</v>
+      </c>
+      <c r="J121" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
       </c>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="C122" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E122" s="5"/>
+      <c r="F122" s="5" t="s">
         <v>524</v>
       </c>
-      <c r="B122" s="5" t="s">
-        <v>410</v>
-      </c>
-      <c r="C122" s="5" t="s">
+      <c r="G122" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="H122" s="3"/>
+      <c r="I122" s="3" t="s">
         <v>525</v>
       </c>
-      <c r="D122" s="5" t="s">
-        <v>700</v>
-      </c>
-      <c r="E122" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F122" s="5"/>
-      <c r="H122" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="I122" s="15" t="s">
+      <c r="J122" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
         <v>526</v>
       </c>
-      <c r="J122" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A123" s="5" t="s">
+      <c r="B123" t="s">
         <v>527</v>
       </c>
-      <c r="B123" s="5" t="s">
+      <c r="C123" t="s">
+        <v>612</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="E123" s="5"/>
+      <c r="F123" s="5"/>
+      <c r="G123" t="s">
+        <v>29</v>
+      </c>
+      <c r="J123" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A124" s="3" t="s">
         <v>528</v>
       </c>
-      <c r="C123" s="5" t="s">
-        <v>622</v>
-      </c>
-      <c r="D123" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E123" s="5"/>
-      <c r="F123" s="5" t="s">
+      <c r="B124" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C124" s="14" t="s">
         <v>529</v>
       </c>
-      <c r="G123" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="H123" s="3"/>
-      <c r="I123" s="3" t="s">
+      <c r="D124" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E124" s="3"/>
+      <c r="F124" s="3" t="s">
         <v>530</v>
       </c>
-      <c r="J123" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A124" t="s">
+      <c r="G124" s="3" t="s">
         <v>531</v>
       </c>
-      <c r="B124" t="s">
+      <c r="H124" s="3" t="s">
         <v>532</v>
       </c>
-      <c r="C124" t="s">
-        <v>617</v>
-      </c>
-      <c r="D124" s="3" t="s">
-        <v>695</v>
-      </c>
-      <c r="E124" s="5"/>
-      <c r="F124" s="5"/>
-      <c r="G124" t="s">
-        <v>29</v>
+      <c r="I124" s="3" t="s">
+        <v>533</v>
       </c>
       <c r="J124" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v/>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
       </c>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A125" s="3" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C125" s="14" t="s">
-        <v>534</v>
-      </c>
+        <v>238</v>
+      </c>
+      <c r="C125" s="3"/>
       <c r="D125" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="E125" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F125" s="3"/>
+      <c r="G125" s="3"/>
+      <c r="H125" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="I125" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="J125" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A126" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="B126" s="5" t="s">
+        <v>538</v>
+      </c>
+      <c r="C126" s="5" t="s">
+        <v>539</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>694</v>
+      </c>
+      <c r="E126" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G126" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="H126" s="5" t="s">
+        <v>540</v>
+      </c>
+      <c r="I126" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="J126" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
+        <v>655</v>
+      </c>
+      <c r="B127" t="s">
+        <v>572</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="E127" s="5"/>
+      <c r="F127" s="3"/>
+      <c r="G127" t="s">
+        <v>531</v>
+      </c>
+      <c r="H127" t="s">
+        <v>656</v>
+      </c>
+      <c r="I127" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="J127" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A128" s="5" t="s">
+        <v>542</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="C128" s="5" t="s">
+        <v>625</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="E128" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F128" s="5"/>
+      <c r="G128" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="H128" s="5" t="s">
+        <v>755</v>
+      </c>
+      <c r="I128" s="8" t="s">
+        <v>544</v>
+      </c>
+      <c r="J128" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A129" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="C129" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="E129" t="s">
+        <v>548</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="G129" s="3" t="s">
+        <v>606</v>
+      </c>
+      <c r="H129" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="I129" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="J129" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A130" s="5" t="s">
+        <v>552</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="C130" s="5" t="s">
+        <v>553</v>
+      </c>
+      <c r="D130" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E125" s="3"/>
-      <c r="F125" s="3" t="s">
-        <v>535</v>
-      </c>
-      <c r="G125" s="3" t="s">
-        <v>536</v>
-      </c>
-      <c r="H125" s="3" t="s">
-        <v>537</v>
-      </c>
-      <c r="I125" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="J125" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A126" s="3" t="s">
-        <v>539</v>
-      </c>
-      <c r="B126" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="C126" s="3"/>
-      <c r="D126" s="3" t="s">
-        <v>695</v>
-      </c>
-      <c r="E126" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F126" s="3"/>
-      <c r="G126" s="3"/>
-      <c r="H126" s="3" t="s">
-        <v>540</v>
-      </c>
-      <c r="I126" s="3" t="s">
-        <v>541</v>
-      </c>
-      <c r="J126" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A127" s="5" t="s">
-        <v>542</v>
-      </c>
-      <c r="B127" s="5" t="s">
-        <v>543</v>
-      </c>
-      <c r="C127" s="5" t="s">
-        <v>544</v>
-      </c>
-      <c r="D127" s="5" t="s">
-        <v>699</v>
-      </c>
-      <c r="E127" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G127" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="H127" s="5" t="s">
-        <v>545</v>
-      </c>
-      <c r="I127" s="15" t="s">
-        <v>546</v>
-      </c>
-      <c r="J127" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A128" t="s">
-        <v>660</v>
-      </c>
-      <c r="B128" t="s">
-        <v>577</v>
-      </c>
-      <c r="C128" s="5" t="s">
-        <v>663</v>
-      </c>
-      <c r="D128" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="E128" s="5"/>
-      <c r="F128" s="3"/>
-      <c r="G128" t="s">
-        <v>536</v>
-      </c>
-      <c r="H128" t="s">
-        <v>661</v>
-      </c>
-      <c r="I128" s="6" t="s">
-        <v>662</v>
-      </c>
-      <c r="J128" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A129" s="5" t="s">
-        <v>547</v>
-      </c>
-      <c r="B129" s="5" t="s">
-        <v>548</v>
-      </c>
-      <c r="C129" s="5" t="s">
-        <v>630</v>
-      </c>
-      <c r="D129" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="E129" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F129" s="5"/>
-      <c r="G129" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="H129" s="5" t="s">
-        <v>760</v>
-      </c>
-      <c r="I129" s="8" t="s">
-        <v>549</v>
-      </c>
-      <c r="J129" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A130" s="3" t="s">
-        <v>550</v>
-      </c>
-      <c r="B130" s="3" t="s">
-        <v>551</v>
-      </c>
-      <c r="C130" s="5" t="s">
-        <v>552</v>
-      </c>
-      <c r="D130" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="E130" t="s">
-        <v>553</v>
-      </c>
-      <c r="F130" s="3" t="s">
+      <c r="E130" s="5"/>
+      <c r="F130" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="G130" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="H130" s="5" t="s">
         <v>554</v>
       </c>
-      <c r="G130" s="3" t="s">
-        <v>611</v>
-      </c>
-      <c r="H130" s="3" t="s">
+      <c r="I130" s="15" t="s">
         <v>555</v>
       </c>
-      <c r="I130" s="15" t="s">
-        <v>556</v>
-      </c>
       <c r="J130" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
       </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="B131" s="5" t="s">
         <v>557</v>
       </c>
-      <c r="B131" s="5" t="s">
-        <v>452</v>
-      </c>
       <c r="C131" s="5" t="s">
+        <v>638</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F131" s="5"/>
+      <c r="G131" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="H131" t="s">
         <v>558</v>
       </c>
-      <c r="D131" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E131" s="5"/>
-      <c r="F131" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="G131" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="H131" s="5" t="s">
+      <c r="I131" s="8" t="s">
         <v>559</v>
       </c>
-      <c r="I131" s="15" t="s">
-        <v>560</v>
-      </c>
       <c r="J131" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
+        <v>560</v>
+      </c>
+      <c r="B132" s="5" t="s">
         <v>561</v>
       </c>
-      <c r="B132" s="5" t="s">
+      <c r="C132" s="5" t="s">
+        <v>616</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E132" s="5"/>
+      <c r="F132" s="5" t="s">
         <v>562</v>
       </c>
-      <c r="C132" s="5" t="s">
-        <v>643</v>
-      </c>
-      <c r="D132" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="E132" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F132" s="5"/>
       <c r="G132" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="H132" t="s">
+        <v>221</v>
+      </c>
+      <c r="H132" s="5" t="s">
         <v>563</v>
       </c>
-      <c r="I132" s="8" t="s">
+      <c r="I132" s="15" t="s">
         <v>564</v>
       </c>
       <c r="J132" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A133" s="5" t="s">
+      <c r="A133" t="s">
         <v>565</v>
       </c>
-      <c r="B133" s="5" t="s">
+      <c r="B133" t="s">
+        <v>568</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="G133" t="s">
+        <v>287</v>
+      </c>
+      <c r="H133" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="I133" s="8" t="s">
+        <v>570</v>
+      </c>
+      <c r="J133" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A134" s="5" t="s">
+        <v>565</v>
+      </c>
+      <c r="B134" s="5" t="s">
         <v>566</v>
       </c>
-      <c r="C133" s="5" t="s">
-        <v>621</v>
-      </c>
-      <c r="D133" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="E133" s="5"/>
-      <c r="F133" s="5" t="s">
+      <c r="C134" s="5" t="s">
+        <v>618</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="E134" s="5"/>
+      <c r="F134" s="5"/>
+      <c r="G134" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="H134" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="I134" s="8" t="s">
         <v>567</v>
       </c>
-      <c r="G133" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="H133" s="5" t="s">
-        <v>568</v>
-      </c>
-      <c r="I133" s="15" t="s">
-        <v>569</v>
-      </c>
-      <c r="J133" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A134" t="s">
-        <v>570</v>
-      </c>
-      <c r="B134" t="s">
-        <v>573</v>
-      </c>
-      <c r="D134" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="G134" t="s">
-        <v>287</v>
-      </c>
-      <c r="H134" s="5" t="s">
-        <v>574</v>
-      </c>
-      <c r="I134" s="8" t="s">
-        <v>575</v>
-      </c>
       <c r="J134" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A135" s="5" t="s">
-        <v>570</v>
-      </c>
-      <c r="B135" s="5" t="s">
-        <v>571</v>
+      <c r="A135" t="s">
+        <v>593</v>
+      </c>
+      <c r="B135" t="s">
+        <v>471</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>623</v>
+        <v>637</v>
       </c>
       <c r="D135" s="5" t="s">
         <v>694</v>
       </c>
-      <c r="E135" s="5"/>
-      <c r="F135" s="5"/>
-      <c r="G135" s="5" t="s">
-        <v>407</v>
-      </c>
-      <c r="H135" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="I135" s="8" t="s">
+      <c r="E135" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F135" t="s">
+        <v>594</v>
+      </c>
+      <c r="G135" t="s">
+        <v>608</v>
+      </c>
+      <c r="H135" t="s">
+        <v>595</v>
+      </c>
+      <c r="I135" s="6" t="s">
+        <v>596</v>
+      </c>
+      <c r="J135" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A136" s="5" t="s">
+        <v>571</v>
+      </c>
+      <c r="B136" s="5" t="s">
         <v>572</v>
       </c>
-      <c r="J135" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A136" t="s">
-        <v>598</v>
-      </c>
-      <c r="B136" t="s">
-        <v>471</v>
-      </c>
-      <c r="C136" s="5" t="s">
-        <v>642</v>
-      </c>
+      <c r="C136" s="5"/>
       <c r="D136" s="5" t="s">
-        <v>699</v>
-      </c>
-      <c r="E136" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F136" t="s">
-        <v>599</v>
-      </c>
-      <c r="G136" t="s">
-        <v>613</v>
-      </c>
-      <c r="H136" t="s">
-        <v>600</v>
-      </c>
-      <c r="I136" s="6" t="s">
-        <v>601</v>
+        <v>689</v>
+      </c>
+      <c r="E136" s="5"/>
+      <c r="F136" s="5"/>
+      <c r="G136" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H136" s="5" t="s">
+        <v>573</v>
+      </c>
+      <c r="I136" s="8" t="s">
+        <v>574</v>
       </c>
       <c r="J136" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="s">
+        <v>575</v>
+      </c>
+      <c r="B137" s="5" t="s">
         <v>576</v>
       </c>
-      <c r="B137" s="5" t="s">
-        <v>577</v>
-      </c>
-      <c r="C137" s="5"/>
+      <c r="C137" s="5" t="s">
+        <v>599</v>
+      </c>
       <c r="D137" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E137" s="5"/>
       <c r="F137" s="5"/>
       <c r="G137" s="5" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="H137" s="5" t="s">
+        <v>577</v>
+      </c>
+      <c r="I137" s="8" t="s">
         <v>578</v>
       </c>
-      <c r="I137" s="8" t="s">
-        <v>579</v>
-      </c>
       <c r="J137" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="s">
+        <v>579</v>
+      </c>
+      <c r="B138" s="5" t="s">
         <v>580</v>
       </c>
-      <c r="B138" s="5" t="s">
-        <v>581</v>
-      </c>
       <c r="C138" s="5" t="s">
-        <v>604</v>
+        <v>627</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
       <c r="G138" s="5" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="H138" s="5" t="s">
+        <v>581</v>
+      </c>
+      <c r="I138" s="8" t="s">
         <v>582</v>
       </c>
-      <c r="I138" s="8" t="s">
+      <c r="J138" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
+        <v>727</v>
+      </c>
+      <c r="B139" t="s">
+        <v>728</v>
+      </c>
+      <c r="C139" s="5" t="s">
+        <v>740</v>
+      </c>
+      <c r="D139" t="s">
+        <v>739</v>
+      </c>
+      <c r="E139" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G139" t="s">
+        <v>79</v>
+      </c>
+      <c r="I139" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="J139" s="9" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A140" s="5" t="s">
         <v>583</v>
       </c>
-      <c r="J138" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A139" s="5" t="s">
+      <c r="B140" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="C140" s="5" t="s">
+        <v>635</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="E140" s="5"/>
+      <c r="F140" s="5"/>
+      <c r="G140" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H140" s="5" t="s">
         <v>584</v>
       </c>
-      <c r="B139" s="5" t="s">
+      <c r="I140" s="8" t="s">
         <v>585</v>
       </c>
-      <c r="C139" s="5" t="s">
-        <v>632</v>
-      </c>
-      <c r="D139" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="E139" s="5"/>
-      <c r="F139" s="5"/>
-      <c r="G139" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="H139" s="5" t="s">
-        <v>586</v>
-      </c>
-      <c r="I139" s="8" t="s">
-        <v>587</v>
-      </c>
-      <c r="J139" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A140" t="s">
-        <v>732</v>
-      </c>
-      <c r="B140" t="s">
-        <v>733</v>
-      </c>
-      <c r="C140" s="5" t="s">
-        <v>745</v>
-      </c>
-      <c r="D140" t="s">
-        <v>744</v>
-      </c>
-      <c r="E140" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G140" t="s">
-        <v>79</v>
-      </c>
-      <c r="I140" s="6" t="s">
-        <v>734</v>
-      </c>
-      <c r="J140" s="9" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
+      <c r="J140" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
       </c>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A141" s="5" t="s">
+        <v>586</v>
+      </c>
+      <c r="B141" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="C141" s="5"/>
+      <c r="D141" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E141" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F141" s="5" t="s">
+        <v>587</v>
+      </c>
+      <c r="G141" t="s">
+        <v>428</v>
+      </c>
+      <c r="H141" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="I141" s="15" t="s">
         <v>588</v>
       </c>
-      <c r="B141" s="5" t="s">
-        <v>581</v>
-      </c>
-      <c r="C141" s="5" t="s">
-        <v>640</v>
-      </c>
-      <c r="D141" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="E141" s="5"/>
-      <c r="F141" s="5"/>
-      <c r="G141" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="H141" s="5" t="s">
-        <v>589</v>
-      </c>
-      <c r="I141" s="8" t="s">
-        <v>590</v>
-      </c>
       <c r="J141" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="s">
-        <v>591</v>
+        <v>674</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>213</v>
+        <v>675</v>
       </c>
       <c r="C142" s="5"/>
       <c r="D142" s="5" t="s">
-        <v>27</v>
+        <v>697</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F142" s="5" t="s">
-        <v>592</v>
-      </c>
-      <c r="G142" t="s">
-        <v>428</v>
+        <v>78</v>
+      </c>
+      <c r="F142" s="5"/>
+      <c r="G142" s="5" t="s">
+        <v>78</v>
       </c>
       <c r="H142" s="5" t="s">
-        <v>449</v>
-      </c>
-      <c r="I142" s="15" t="s">
-        <v>593</v>
-      </c>
-      <c r="J142" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A143" s="5" t="s">
-        <v>679</v>
-      </c>
-      <c r="B143" s="5" t="s">
-        <v>680</v>
-      </c>
-      <c r="C143" s="5"/>
-      <c r="D143" s="5" t="s">
-        <v>702</v>
-      </c>
-      <c r="E143" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F143" s="5"/>
-      <c r="G143" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="H143" s="5" t="s">
-        <v>681</v>
-      </c>
-      <c r="I143" s="6" t="s">
-        <v>682</v>
-      </c>
-      <c r="J143" s="9" t="str">
+        <v>676</v>
+      </c>
+      <c r="I142" s="6" t="s">
+        <v>677</v>
+      </c>
+      <c r="J142" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=sosthene.yamale@umontreal.ca</v>
       </c>
@@ -7291,19 +7249,19 @@
     <hyperlink ref="I17" r:id="rId3" display="mailto:hugo.bernier@umontreal.ca" xr:uid="{3F591457-DA50-462E-B1CA-F2F56ED9E3DD}"/>
     <hyperlink ref="I76" r:id="rId4" xr:uid="{4822C834-E5A8-42FD-9734-374BFC718C85}"/>
     <hyperlink ref="I10" r:id="rId5" display="mailto:magalie.beaudoin@umontreal.ca" xr:uid="{2D976BF0-B68A-46E5-8412-BA8BC43FD26D}"/>
-    <hyperlink ref="I112" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
+    <hyperlink ref="I111" r:id="rId6" display="mailto:mathieu.pigeon@umontreal.ca" xr:uid="{F73DFC6E-4D6D-42F3-84C0-454956AEC7E8}"/>
     <hyperlink ref="I5" r:id="rId7" display="mailto:nadege.arsa@bib.umontreal.ca" xr:uid="{408AF5A3-35ED-4BF5-92B9-1B21C0C475D9}"/>
     <hyperlink ref="I20" r:id="rId8" display="mailto:simon.blais.longtin@umontreal.ca" xr:uid="{EA917AC7-9087-435B-A6E7-3AE1885514AA}"/>
     <hyperlink ref="I93" r:id="rId9" xr:uid="{8ABC26E9-CF81-491C-8A28-B209E6620D2A}"/>
-    <hyperlink ref="I138" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
+    <hyperlink ref="I137" r:id="rId10" xr:uid="{B455CC78-8572-42C6-950F-67FBEC488BBE}"/>
     <hyperlink ref="I37" r:id="rId11" xr:uid="{7D21070C-9A14-48DF-982E-D995A034BDAD}"/>
-    <hyperlink ref="I134" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
+    <hyperlink ref="I133" r:id="rId12" xr:uid="{0C92A93F-14B9-4EBD-9C0E-42EDAA49F3AB}"/>
     <hyperlink ref="I74" r:id="rId13" xr:uid="{DCABBE8B-8789-4957-9A88-F8585AD53BBC}"/>
-    <hyperlink ref="I115" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
+    <hyperlink ref="I114" r:id="rId14" xr:uid="{C37D08E3-EE29-4008-958D-7BCCC40EBCA4}"/>
     <hyperlink ref="I51" r:id="rId15" xr:uid="{1383A46C-5C1D-4621-B4BC-67AD012D7CF5}"/>
     <hyperlink ref="I82" r:id="rId16" xr:uid="{29D9619F-F3A7-41E8-AE0F-DEBBF802D53A}"/>
     <hyperlink ref="I32" r:id="rId17" xr:uid="{9E8CD31B-437A-49A0-BA12-85176E0D9431}"/>
-    <hyperlink ref="I117" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
+    <hyperlink ref="I116" r:id="rId18" xr:uid="{D112D4D2-EACF-41EC-8833-0BCADA67F58D}"/>
     <hyperlink ref="I77" r:id="rId19" xr:uid="{3B502B79-2DDE-44A3-908B-3CB04ED1101E}"/>
     <hyperlink ref="I18" r:id="rId20" xr:uid="{BAE0697B-7739-4A42-9702-C285F03D0F77}"/>
     <hyperlink ref="I54" r:id="rId21" xr:uid="{E1BC7B04-B072-447B-9137-59A28141883D}"/>
@@ -7311,61 +7269,61 @@
     <hyperlink ref="I65" r:id="rId23" xr:uid="{6E82D57D-36A4-4928-AD91-BE73FFC7C389}"/>
     <hyperlink ref="I84" r:id="rId24" xr:uid="{278FDD6D-245D-42BB-9DC6-1D47D17CC5FD}"/>
     <hyperlink ref="I102" r:id="rId25" xr:uid="{5BCD15FE-E90C-4C6C-864A-F66215BE8839}"/>
-    <hyperlink ref="I135" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
+    <hyperlink ref="I134" r:id="rId26" xr:uid="{FDD0DDC4-7A67-4339-BDFC-3AA7CBFB9040}"/>
     <hyperlink ref="I91" r:id="rId27" xr:uid="{6C259D22-E49F-4548-B971-5B79C0A1D1A3}"/>
     <hyperlink ref="I92" r:id="rId28" xr:uid="{7328D0A7-0B9F-4556-BBCF-C84267E93A32}"/>
     <hyperlink ref="I97" r:id="rId29" xr:uid="{7F7A355D-E6B8-443A-AF2B-0A53F4B15B21}"/>
-    <hyperlink ref="I114" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
-    <hyperlink ref="I129" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
-    <hyperlink ref="I132" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
-    <hyperlink ref="I137" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
-    <hyperlink ref="I139" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
-    <hyperlink ref="I141" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
+    <hyperlink ref="I113" r:id="rId30" xr:uid="{3078ED0B-307C-47F2-B4E5-65F31B4FF7CB}"/>
+    <hyperlink ref="I128" r:id="rId31" xr:uid="{1A3BB298-F78B-474C-A8E7-739C762F9819}"/>
+    <hyperlink ref="I131" r:id="rId32" xr:uid="{9037CA9B-E8A7-4F4D-8F0A-7DD7E74AD41B}"/>
+    <hyperlink ref="I136" r:id="rId33" xr:uid="{B083C43A-D8A2-4E8E-9E8A-BDC13AA93D54}"/>
+    <hyperlink ref="I138" r:id="rId34" xr:uid="{A0852ED6-2CA4-4FFA-94EF-8EB908CD7BEB}"/>
+    <hyperlink ref="I140" r:id="rId35" xr:uid="{00BAEA16-152E-416E-A034-87CB2800061D}"/>
     <hyperlink ref="I16" r:id="rId36" xr:uid="{E26D4CB1-6F14-4277-AD54-18A052872B6B}"/>
-    <hyperlink ref="I136" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
+    <hyperlink ref="I135" r:id="rId37" xr:uid="{37C73F8E-25A1-477F-AA74-E9785B7E918A}"/>
     <hyperlink ref="I39" r:id="rId38" xr:uid="{902A8808-023C-4EA1-833E-F687288B12ED}"/>
-    <hyperlink ref="I128" r:id="rId39" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
-    <hyperlink ref="I119" r:id="rId40" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
+    <hyperlink ref="I127" r:id="rId39" xr:uid="{0F562F25-AF6E-412E-962D-4CACCF0BD4F0}"/>
+    <hyperlink ref="I118" r:id="rId40" xr:uid="{349E580E-212A-42D9-8F7B-BDF3DFB61650}"/>
     <hyperlink ref="I53" r:id="rId41" xr:uid="{ABEB73EB-E336-4619-ADE1-0AE567E81306}"/>
     <hyperlink ref="I31" r:id="rId42" xr:uid="{E819F1D0-ED89-4281-B222-20D0A6AC8A49}"/>
-    <hyperlink ref="I143" r:id="rId43" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
+    <hyperlink ref="I142" r:id="rId43" xr:uid="{EDD92A66-A56B-419B-967E-B8D761D72C58}"/>
     <hyperlink ref="I19" r:id="rId44" xr:uid="{A4113BC8-FD33-4D47-854C-D964ED926E7F}"/>
-    <hyperlink ref="I29" r:id="rId45" xr:uid="{7233E394-0474-4122-B129-E1E8DB3D4B70}"/>
-    <hyperlink ref="I116" r:id="rId46" xr:uid="{0924E3CD-F2EB-4646-BC88-767228D5A8FD}"/>
-    <hyperlink ref="I75" r:id="rId47" xr:uid="{FAC375AB-8F54-402B-A4F5-618AA479650B}"/>
-    <hyperlink ref="I4" r:id="rId48" xr:uid="{12EFBBCC-308A-4E41-92F6-4E78BB9E9458}"/>
-    <hyperlink ref="I21" r:id="rId49" xr:uid="{CAA07608-BC3B-468C-819E-F94EE0396C78}"/>
-    <hyperlink ref="I140" r:id="rId50" xr:uid="{B3DF72B2-3730-4A9C-8195-E5B8FCD87C3B}"/>
-    <hyperlink ref="I121" r:id="rId51" xr:uid="{518A2404-8625-4373-BDE5-E73718B1440B}"/>
-    <hyperlink ref="I33" r:id="rId52" xr:uid="{B383F9BF-E7F0-4AFA-A217-1F3A922E55BA}"/>
-    <hyperlink ref="I142" r:id="rId53" xr:uid="{D2BBF900-A9C8-4032-A387-C01245244DE0}"/>
-    <hyperlink ref="I52" r:id="rId54" xr:uid="{79C702A2-295C-4D37-BA6F-DD2C408C75BD}"/>
-    <hyperlink ref="I23" r:id="rId55" xr:uid="{761F418D-12C5-4F41-8071-6031B8FBF83B}"/>
-    <hyperlink ref="I106" r:id="rId56" xr:uid="{C91A1DE6-A8FA-4481-9E51-1DB52F17F3CC}"/>
-    <hyperlink ref="I133" r:id="rId57" xr:uid="{131478F3-61ED-4B04-9E66-6F771D0E53F1}"/>
-    <hyperlink ref="I100" r:id="rId58" xr:uid="{C3534DCE-62CB-4016-B559-AE879ED29221}"/>
-    <hyperlink ref="I72" r:id="rId59" xr:uid="{598291DC-2DD2-464C-A65A-36D0759E8852}"/>
-    <hyperlink ref="I64" r:id="rId60" xr:uid="{55FAFEEC-7E6A-4254-BBB4-020FD859DB23}"/>
-    <hyperlink ref="I104" r:id="rId61" xr:uid="{E35BC25D-CA56-4FFF-B93C-72EBCAD05C3B}"/>
-    <hyperlink ref="I45" r:id="rId62" xr:uid="{6B64B7D5-5396-4382-9ECB-D065E5B3F7C4}"/>
-    <hyperlink ref="I57" r:id="rId63" xr:uid="{A6C3CD82-A312-40D2-B320-33ED739C6E60}"/>
-    <hyperlink ref="I86" r:id="rId64" xr:uid="{1754B384-2B8D-46A2-8C89-BDF617522295}"/>
-    <hyperlink ref="I113" r:id="rId65" xr:uid="{99B099F4-5E98-4B25-B2EB-EE4C451DC6EE}"/>
-    <hyperlink ref="I59" r:id="rId66" xr:uid="{1C080271-6DB7-4810-99C8-8FF2BA5EA430}"/>
-    <hyperlink ref="I63" r:id="rId67" xr:uid="{6A0B0BD3-8872-437B-9CD4-6D8D7D98A4F9}"/>
-    <hyperlink ref="I122" r:id="rId68" xr:uid="{CE8C2C5F-3292-4BA9-A27E-19AF9661C907}"/>
-    <hyperlink ref="I11" r:id="rId69" xr:uid="{F1246003-4D15-4FC5-9F7D-6CE88CAF21A8}"/>
-    <hyperlink ref="I131" r:id="rId70" xr:uid="{BB3A0149-0DD5-481B-8662-8134BB3FCECC}"/>
-    <hyperlink ref="I127" r:id="rId71" xr:uid="{52D55C85-F393-43A8-95EF-F57618BB179E}"/>
-    <hyperlink ref="I87" r:id="rId72" xr:uid="{CAB4CB00-83BC-4384-BF0E-208B7456F243}"/>
-    <hyperlink ref="I95" r:id="rId73" xr:uid="{4B80B43B-B062-42B6-A1CE-F4CE03CDED46}"/>
-    <hyperlink ref="I8" r:id="rId74" xr:uid="{BC76BE28-D367-49FE-95A3-98BB93483999}"/>
-    <hyperlink ref="I47" r:id="rId75" xr:uid="{8598B756-3A70-45A7-ABB5-3EDBEF50BAF4}"/>
-    <hyperlink ref="I130" r:id="rId76" xr:uid="{07544A5C-3F38-40A4-9945-4E56F5EFFCF4}"/>
-    <hyperlink ref="I27" r:id="rId77" xr:uid="{C341566A-DC48-4D81-91C1-E1CD275F4D60}"/>
-    <hyperlink ref="I13" r:id="rId78" xr:uid="{FAAE6B3B-3F31-452F-868E-B6C650D083E8}"/>
-    <hyperlink ref="I80" r:id="rId79" xr:uid="{09E37274-D8A2-4A0B-832A-E187D6213477}"/>
-    <hyperlink ref="I101" r:id="rId80" xr:uid="{89D21B16-595D-4AC9-BFE9-2C29DBC329A2}"/>
+    <hyperlink ref="I115" r:id="rId45" xr:uid="{0924E3CD-F2EB-4646-BC88-767228D5A8FD}"/>
+    <hyperlink ref="I75" r:id="rId46" xr:uid="{FAC375AB-8F54-402B-A4F5-618AA479650B}"/>
+    <hyperlink ref="I4" r:id="rId47" xr:uid="{12EFBBCC-308A-4E41-92F6-4E78BB9E9458}"/>
+    <hyperlink ref="I21" r:id="rId48" xr:uid="{CAA07608-BC3B-468C-819E-F94EE0396C78}"/>
+    <hyperlink ref="I139" r:id="rId49" xr:uid="{B3DF72B2-3730-4A9C-8195-E5B8FCD87C3B}"/>
+    <hyperlink ref="I120" r:id="rId50" xr:uid="{518A2404-8625-4373-BDE5-E73718B1440B}"/>
+    <hyperlink ref="I33" r:id="rId51" xr:uid="{B383F9BF-E7F0-4AFA-A217-1F3A922E55BA}"/>
+    <hyperlink ref="I141" r:id="rId52" xr:uid="{D2BBF900-A9C8-4032-A387-C01245244DE0}"/>
+    <hyperlink ref="I52" r:id="rId53" xr:uid="{79C702A2-295C-4D37-BA6F-DD2C408C75BD}"/>
+    <hyperlink ref="I23" r:id="rId54" xr:uid="{761F418D-12C5-4F41-8071-6031B8FBF83B}"/>
+    <hyperlink ref="I106" r:id="rId55" xr:uid="{C91A1DE6-A8FA-4481-9E51-1DB52F17F3CC}"/>
+    <hyperlink ref="I132" r:id="rId56" xr:uid="{131478F3-61ED-4B04-9E66-6F771D0E53F1}"/>
+    <hyperlink ref="I100" r:id="rId57" xr:uid="{C3534DCE-62CB-4016-B559-AE879ED29221}"/>
+    <hyperlink ref="I72" r:id="rId58" xr:uid="{598291DC-2DD2-464C-A65A-36D0759E8852}"/>
+    <hyperlink ref="I64" r:id="rId59" xr:uid="{55FAFEEC-7E6A-4254-BBB4-020FD859DB23}"/>
+    <hyperlink ref="I104" r:id="rId60" xr:uid="{E35BC25D-CA56-4FFF-B93C-72EBCAD05C3B}"/>
+    <hyperlink ref="I45" r:id="rId61" xr:uid="{6B64B7D5-5396-4382-9ECB-D065E5B3F7C4}"/>
+    <hyperlink ref="I57" r:id="rId62" xr:uid="{A6C3CD82-A312-40D2-B320-33ED739C6E60}"/>
+    <hyperlink ref="I86" r:id="rId63" xr:uid="{1754B384-2B8D-46A2-8C89-BDF617522295}"/>
+    <hyperlink ref="I112" r:id="rId64" xr:uid="{99B099F4-5E98-4B25-B2EB-EE4C451DC6EE}"/>
+    <hyperlink ref="I59" r:id="rId65" xr:uid="{1C080271-6DB7-4810-99C8-8FF2BA5EA430}"/>
+    <hyperlink ref="I63" r:id="rId66" xr:uid="{6A0B0BD3-8872-437B-9CD4-6D8D7D98A4F9}"/>
+    <hyperlink ref="I121" r:id="rId67" xr:uid="{CE8C2C5F-3292-4BA9-A27E-19AF9661C907}"/>
+    <hyperlink ref="I11" r:id="rId68" xr:uid="{F1246003-4D15-4FC5-9F7D-6CE88CAF21A8}"/>
+    <hyperlink ref="I130" r:id="rId69" xr:uid="{BB3A0149-0DD5-481B-8662-8134BB3FCECC}"/>
+    <hyperlink ref="I126" r:id="rId70" xr:uid="{52D55C85-F393-43A8-95EF-F57618BB179E}"/>
+    <hyperlink ref="I87" r:id="rId71" xr:uid="{CAB4CB00-83BC-4384-BF0E-208B7456F243}"/>
+    <hyperlink ref="I95" r:id="rId72" xr:uid="{4B80B43B-B062-42B6-A1CE-F4CE03CDED46}"/>
+    <hyperlink ref="I8" r:id="rId73" xr:uid="{BC76BE28-D367-49FE-95A3-98BB93483999}"/>
+    <hyperlink ref="I47" r:id="rId74" xr:uid="{8598B756-3A70-45A7-ABB5-3EDBEF50BAF4}"/>
+    <hyperlink ref="I129" r:id="rId75" xr:uid="{07544A5C-3F38-40A4-9945-4E56F5EFFCF4}"/>
+    <hyperlink ref="I27" r:id="rId76" xr:uid="{C341566A-DC48-4D81-91C1-E1CD275F4D60}"/>
+    <hyperlink ref="I13" r:id="rId77" xr:uid="{FAAE6B3B-3F31-452F-868E-B6C650D083E8}"/>
+    <hyperlink ref="I80" r:id="rId78" xr:uid="{09E37274-D8A2-4A0B-832A-E187D6213477}"/>
+    <hyperlink ref="I101" r:id="rId79" xr:uid="{89D21B16-595D-4AC9-BFE9-2C29DBC329A2}"/>
+    <hyperlink ref="I29" r:id="rId80" xr:uid="{7233E394-0474-4122-B129-E1E8DB3D4B70}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId81"/>
@@ -7571,6 +7529,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7579,15 +7546,6 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7610,6 +7568,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7624,12 +7590,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Répertoire TCTDM prise 2
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tardimat\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59AAF8D1-9BC2-49D9-B5E4-389D3C3CC4B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F053A0F2-0008-446D-823D-89DCBEE08142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="31920" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="759">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="758">
   <si>
     <t>nom</t>
   </si>
@@ -1830,9 +1830,6 @@
   </si>
   <si>
     <t>Bibliothèque de droit;Bibliothèque de musique</t>
-  </si>
-  <si>
-    <t>Centre de conservation Lionel-Groulx;Centre de conservation Marcel-Laurin</t>
   </si>
   <si>
     <t>Référence et offre pédagogique de première ligne, psychoéducation, psychologie, sciences de l'éducation, sciences infirmières, travail social – premier cycle</t>
@@ -3065,7 +3062,7 @@
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>21</v>
@@ -3083,14 +3080,14 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>709</v>
+      </c>
+      <c r="B4" t="s">
         <v>710</v>
-      </c>
-      <c r="B4" t="s">
-        <v>711</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>77</v>
@@ -3102,7 +3099,7 @@
         <v>307</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="J4" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3182,7 +3179,7 @@
         <v>40</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>544</v>
@@ -3191,7 +3188,7 @@
         <v>41</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>42</v>
@@ -3215,7 +3212,7 @@
         <v>46</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
@@ -3302,7 +3299,7 @@
         <v>65</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E11" t="s">
         <v>66</v>
@@ -3332,10 +3329,10 @@
         <v>39</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>70</v>
@@ -3344,7 +3341,7 @@
         <v>71</v>
       </c>
       <c r="G12" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>72</v>
@@ -3359,13 +3356,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B13" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>27</v>
@@ -3381,7 +3378,7 @@
         <v>307</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="J13" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3399,7 +3396,7 @@
         <v>76</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>77</v>
@@ -3459,10 +3456,10 @@
         <v>87</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
@@ -3517,10 +3514,10 @@
         <v>96</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G18" t="s">
         <v>29</v>
@@ -3538,13 +3535,13 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>676</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>677</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>27</v>
@@ -3553,14 +3550,14 @@
         <v>77</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="G19" t="s">
         <v>77</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="6" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="J19" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3600,14 +3597,14 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>717</v>
+      </c>
+      <c r="B21" t="s">
         <v>718</v>
-      </c>
-      <c r="B21" t="s">
-        <v>719</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>77</v>
@@ -3616,7 +3613,7 @@
         <v>78</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="J21" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3662,7 +3659,7 @@
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="3" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>59</v>
@@ -3690,7 +3687,7 @@
         <v>117</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E24" t="s">
         <v>118</v>
@@ -3779,19 +3776,19 @@
         <v>136</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>70</v>
       </c>
       <c r="F27" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>137</v>
@@ -3812,15 +3809,19 @@
         <v>140</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>683</v>
-      </c>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
+        <v>682</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>347</v>
+      </c>
       <c r="G28" s="5" t="s">
-        <v>598</v>
+        <v>753</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>141</v>
@@ -3835,16 +3836,16 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>345</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E29" s="5"/>
       <c r="F29" s="5"/>
@@ -3852,10 +3853,10 @@
         <v>29</v>
       </c>
       <c r="H29" s="5" t="s">
+        <v>680</v>
+      </c>
+      <c r="I29" s="6" t="s">
         <v>681</v>
-      </c>
-      <c r="I29" s="6" t="s">
-        <v>682</v>
       </c>
       <c r="J29" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3873,7 +3874,7 @@
         <v>145</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>59</v>
@@ -3892,13 +3893,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
+        <v>661</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>662</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>663</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>664</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>13</v>
@@ -3907,16 +3908,16 @@
         <v>118</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="G31" t="s">
         <v>15</v>
       </c>
       <c r="H31" s="5" t="s">
+        <v>665</v>
+      </c>
+      <c r="I31" s="6" t="s">
         <v>666</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>667</v>
       </c>
       <c r="J31" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3931,10 +3932,10 @@
         <v>149</v>
       </c>
       <c r="C32" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G32" t="s">
         <v>29</v>
@@ -3952,14 +3953,14 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>726</v>
+      </c>
+      <c r="B33" t="s">
         <v>727</v>
-      </c>
-      <c r="B33" t="s">
-        <v>728</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>77</v>
@@ -3968,10 +3969,10 @@
         <v>78</v>
       </c>
       <c r="H33" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="J33" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3986,7 +3987,7 @@
         <v>153</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>13</v>
@@ -3995,7 +3996,7 @@
         <v>118</v>
       </c>
       <c r="F34" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>155</v>
@@ -4019,10 +4020,10 @@
         <v>159</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E35" s="5"/>
       <c r="F35" s="5"/>
@@ -4079,7 +4080,7 @@
         <v>171</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G37" t="s">
         <v>586</v>
@@ -4097,14 +4098,14 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>729</v>
+      </c>
+      <c r="B38" t="s">
         <v>730</v>
-      </c>
-      <c r="B38" t="s">
-        <v>731</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E38" s="5" t="s">
         <v>77</v>
@@ -4113,10 +4114,10 @@
         <v>78</v>
       </c>
       <c r="H38" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="I38" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="J38" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4132,7 +4133,7 @@
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>59</v>
@@ -4141,10 +4142,10 @@
         <v>59</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="J39" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4193,7 +4194,7 @@
         <v>184</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="E41" s="5" t="s">
         <v>77</v>
@@ -4220,7 +4221,7 @@
         <v>189</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>27</v>
@@ -4254,7 +4255,7 @@
         <v>195</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E43" t="s">
         <v>196</v>
@@ -4315,14 +4316,14 @@
         <v>207</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="5" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>53</v>
@@ -4380,7 +4381,7 @@
         <v>218</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E47" s="5"/>
       <c r="F47" t="s">
@@ -4470,10 +4471,10 @@
         <v>236</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
@@ -4499,10 +4500,10 @@
         <v>241</v>
       </c>
       <c r="C51" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G51" t="s">
         <v>29</v>
@@ -4551,10 +4552,10 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
+        <v>656</v>
+      </c>
+      <c r="B53" s="5" t="s">
         <v>657</v>
-      </c>
-      <c r="B53" s="5" t="s">
-        <v>658</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
@@ -4564,16 +4565,16 @@
         <v>118</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H53" s="5" t="s">
+        <v>659</v>
+      </c>
+      <c r="I53" s="6" t="s">
         <v>660</v>
-      </c>
-      <c r="I53" s="6" t="s">
-        <v>661</v>
       </c>
       <c r="J53" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4588,10 +4589,10 @@
         <v>251</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G54" t="s">
         <v>29</v>
@@ -4618,7 +4619,7 @@
         <v>256</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E55" s="5" t="s">
         <v>118</v>
@@ -4651,7 +4652,7 @@
         <v>261</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E56" s="11" t="s">
         <v>262</v>
@@ -4682,7 +4683,7 @@
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E57" s="5"/>
       <c r="F57" s="5"/>
@@ -4739,10 +4740,10 @@
         <v>278</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5" t="s">
@@ -4800,7 +4801,7 @@
       </c>
       <c r="C61" s="5"/>
       <c r="D61" s="3" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E61" s="5" t="s">
         <v>118</v>
@@ -4828,7 +4829,7 @@
         <v>290</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="E62" s="5" t="s">
         <v>237</v>
@@ -4877,10 +4878,10 @@
     </row>
     <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="B64" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C64" s="5"/>
       <c r="D64" s="5" t="s">
@@ -4897,7 +4898,7 @@
         <v>307</v>
       </c>
       <c r="I64" s="15" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="J64" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4913,7 +4914,7 @@
       </c>
       <c r="C65" s="5"/>
       <c r="D65" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
@@ -4939,7 +4940,7 @@
         <v>304</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>27</v>
@@ -4957,7 +4958,7 @@
         <v>307</v>
       </c>
       <c r="I66" s="5" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="J66" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -4966,16 +4967,16 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="B67" t="s">
         <v>289</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="D67" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E67" s="5" t="s">
         <v>77</v>
@@ -4988,7 +4989,7 @@
         <v>307</v>
       </c>
       <c r="I67" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="J67" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5089,16 +5090,16 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B71" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="D71" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="E71" s="5" t="s">
         <v>77</v>
@@ -5111,7 +5112,7 @@
         <v>307</v>
       </c>
       <c r="I71" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="J71" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5129,7 +5130,7 @@
         <v>327</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>70</v>
@@ -5162,7 +5163,7 @@
       </c>
       <c r="E73" s="5"/>
       <c r="F73" s="5" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="G73" s="5" t="s">
         <v>29</v>
@@ -5186,10 +5187,10 @@
         <v>336</v>
       </c>
       <c r="C74" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G74" t="s">
         <v>285</v>
@@ -5207,14 +5208,14 @@
     </row>
     <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>712</v>
+      </c>
+      <c r="B75" t="s">
         <v>713</v>
-      </c>
-      <c r="B75" t="s">
-        <v>714</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>77</v>
@@ -5227,7 +5228,7 @@
         <v>307</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="J75" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5243,7 +5244,7 @@
       </c>
       <c r="C76" s="5"/>
       <c r="D76" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E76" s="5"/>
       <c r="F76" s="5"/>
@@ -5269,10 +5270,10 @@
         <v>96</v>
       </c>
       <c r="C77" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G77" t="s">
         <v>29</v>
@@ -5308,7 +5309,7 @@
         <v>347</v>
       </c>
       <c r="G78" s="5" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="H78" s="5" t="s">
         <v>348</v>
@@ -5332,7 +5333,7 @@
         <v>352</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E79" s="5" t="s">
         <v>118</v>
@@ -5356,27 +5357,27 @@
     </row>
     <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
+        <v>737</v>
+      </c>
+      <c r="B80" s="5" t="s">
         <v>738</v>
-      </c>
-      <c r="B80" s="5" t="s">
-        <v>739</v>
       </c>
       <c r="C80" s="5"/>
       <c r="D80" s="5" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="F80" s="5"/>
       <c r="G80" s="5" t="s">
         <v>126</v>
       </c>
       <c r="H80" s="5" t="s">
+        <v>740</v>
+      </c>
+      <c r="I80" s="6" t="s">
         <v>741</v>
-      </c>
-      <c r="I80" s="6" t="s">
-        <v>742</v>
       </c>
       <c r="J80" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -5394,7 +5395,7 @@
         <v>592</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E81" s="11" t="s">
         <v>262</v>
@@ -5427,7 +5428,7 @@
         <v>593</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G82" t="s">
         <v>29</v>
@@ -5458,7 +5459,7 @@
       </c>
       <c r="E83" s="5"/>
       <c r="F83" s="5" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="G83" s="5" t="s">
         <v>29</v>
@@ -5482,7 +5483,7 @@
         <v>369</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>27</v>
@@ -5491,7 +5492,7 @@
         <v>70</v>
       </c>
       <c r="F84" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G84" s="5" t="s">
         <v>425</v>
@@ -5518,7 +5519,7 @@
         <v>374</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E85" s="5" t="s">
         <v>70</v>
@@ -5549,7 +5550,7 @@
         <v>379</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E86" s="5" t="s">
         <v>118</v>
@@ -5579,10 +5580,10 @@
         <v>384</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>77</v>
@@ -5612,7 +5613,7 @@
         <v>389</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E88" s="11" t="s">
         <v>262</v>
@@ -5640,10 +5641,10 @@
         <v>393</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>544</v>
@@ -5673,10 +5674,10 @@
         <v>396</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>77</v>
@@ -5699,10 +5700,10 @@
         <v>399</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E91" s="5"/>
       <c r="F91" s="5"/>
@@ -5728,10 +5729,10 @@
         <v>403</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
@@ -5757,10 +5758,10 @@
         <v>408</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E93" s="5"/>
       <c r="G93" s="5" t="s">
@@ -5792,7 +5793,7 @@
       </c>
       <c r="E94" s="5"/>
       <c r="F94" s="5" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="G94" s="5" t="s">
         <v>29</v>
@@ -5850,7 +5851,7 @@
         <v>424</v>
       </c>
       <c r="D96" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E96" s="5" t="s">
         <v>70</v>
@@ -5877,10 +5878,10 @@
         <v>429</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E97" s="5"/>
       <c r="F97" s="5"/>
@@ -5977,10 +5978,10 @@
         <v>70</v>
       </c>
       <c r="F100" s="5" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="G100" s="5" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="H100" s="5" t="s">
         <v>446</v>
@@ -5995,16 +5996,16 @@
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>292</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="D101" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E101" t="s">
         <v>66</v>
@@ -6014,10 +6015,10 @@
         <v>126</v>
       </c>
       <c r="H101" s="5" t="s">
+        <v>744</v>
+      </c>
+      <c r="I101" s="6" t="s">
         <v>745</v>
-      </c>
-      <c r="I101" s="6" t="s">
-        <v>746</v>
       </c>
       <c r="J101" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6032,7 +6033,7 @@
         <v>449</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>27</v>
@@ -6041,7 +6042,7 @@
         <v>70</v>
       </c>
       <c r="F102" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="G102" s="5" t="s">
         <v>425</v>
@@ -6065,17 +6066,17 @@
         <v>453</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D103" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E103" s="3" t="s">
         <v>544</v>
       </c>
       <c r="F103" s="12"/>
       <c r="G103" s="3" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="H103" s="3" t="s">
         <v>454</v>
@@ -6096,7 +6097,7 @@
         <v>457</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>458</v>
@@ -6128,7 +6129,7 @@
       </c>
       <c r="C105" s="5"/>
       <c r="D105" s="3" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E105" s="5" t="s">
         <v>70</v>
@@ -6156,14 +6157,14 @@
         <v>595</v>
       </c>
       <c r="D106" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E106" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="F106" s="3"/>
       <c r="G106" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="H106" s="5" t="s">
         <v>468</v>
@@ -6211,7 +6212,7 @@
         <v>476</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D108" s="5" t="s">
         <v>13</v>
@@ -6251,7 +6252,7 @@
         <v>29</v>
       </c>
       <c r="F109" s="5" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="G109" s="5" t="s">
         <v>29</v>
@@ -6366,10 +6367,10 @@
         <v>499</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D113" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E113" s="5"/>
       <c r="F113" s="5"/>
@@ -6395,10 +6396,10 @@
         <v>503</v>
       </c>
       <c r="C114" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D114" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G114" t="s">
         <v>586</v>
@@ -6416,14 +6417,14 @@
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B115" t="s">
         <v>449</v>
       </c>
       <c r="C115" s="14"/>
       <c r="D115" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E115" s="5" t="s">
         <v>77</v>
@@ -6435,7 +6436,7 @@
         <v>307</v>
       </c>
       <c r="I115" s="6" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="J115" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6451,7 +6452,7 @@
       </c>
       <c r="C116" s="16"/>
       <c r="D116" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G116" t="s">
         <v>29</v>
@@ -6469,14 +6470,14 @@
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B117" t="s">
         <v>75</v>
       </c>
       <c r="C117" s="5"/>
       <c r="D117" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E117" s="5" t="s">
         <v>77</v>
@@ -6489,7 +6490,7 @@
         <v>307</v>
       </c>
       <c r="I117" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="J117" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6498,16 +6499,16 @@
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
+        <v>643</v>
+      </c>
+      <c r="B118" t="s">
         <v>644</v>
       </c>
-      <c r="B118" t="s">
-        <v>645</v>
-      </c>
       <c r="C118" s="5" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D118" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E118" s="5"/>
       <c r="F118" s="3"/>
@@ -6515,10 +6516,10 @@
         <v>527</v>
       </c>
       <c r="H118" t="s">
+        <v>646</v>
+      </c>
+      <c r="I118" s="6" t="s">
         <v>647</v>
-      </c>
-      <c r="I118" s="6" t="s">
-        <v>648</v>
       </c>
       <c r="J118" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6557,14 +6558,14 @@
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B120" t="s">
         <v>123</v>
       </c>
       <c r="C120" s="5"/>
       <c r="D120" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E120" s="5" t="s">
         <v>77</v>
@@ -6573,10 +6574,10 @@
         <v>78</v>
       </c>
       <c r="H120" t="s">
+        <v>724</v>
+      </c>
+      <c r="I120" s="6" t="s">
         <v>725</v>
-      </c>
-      <c r="I120" s="6" t="s">
-        <v>726</v>
       </c>
       <c r="J120" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6594,7 +6595,7 @@
         <v>516</v>
       </c>
       <c r="D121" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E121" s="5" t="s">
         <v>77</v>
@@ -6619,7 +6620,7 @@
         <v>519</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>13</v>
@@ -6648,10 +6649,10 @@
         <v>523</v>
       </c>
       <c r="C123" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E123" s="5"/>
       <c r="F123" s="5"/>
@@ -6703,7 +6704,7 @@
       </c>
       <c r="C125" s="3"/>
       <c r="D125" s="3" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E125" s="3" t="s">
         <v>544</v>
@@ -6732,7 +6733,7 @@
         <v>535</v>
       </c>
       <c r="D126" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E126" s="5" t="s">
         <v>77</v>
@@ -6753,16 +6754,16 @@
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B127" t="s">
         <v>568</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D127" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E127" s="5"/>
       <c r="F127" s="3"/>
@@ -6770,10 +6771,10 @@
         <v>527</v>
       </c>
       <c r="H127" t="s">
+        <v>649</v>
+      </c>
+      <c r="I127" s="6" t="s">
         <v>650</v>
-      </c>
-      <c r="I127" s="6" t="s">
-        <v>651</v>
       </c>
       <c r="J127" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -6788,10 +6789,10 @@
         <v>539</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E128" s="5"/>
       <c r="F128" s="5"/>
@@ -6799,7 +6800,7 @@
         <v>419</v>
       </c>
       <c r="H128" s="5" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="I128" s="8" t="s">
         <v>540</v>
@@ -6829,7 +6830,7 @@
         <v>545</v>
       </c>
       <c r="G129" s="3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H129" s="3" t="s">
         <v>546</v>
@@ -6881,10 +6882,10 @@
         <v>553</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D131" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E131" s="5"/>
       <c r="F131" s="5"/>
@@ -6910,7 +6911,7 @@
         <v>557</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D132" s="5" t="s">
         <v>102</v>
@@ -6941,7 +6942,7 @@
         <v>564</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G133" t="s">
         <v>285</v>
@@ -6965,10 +6966,10 @@
         <v>562</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D134" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E134" s="5"/>
       <c r="F134" s="5"/>
@@ -6994,10 +6995,10 @@
         <v>467</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D135" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E135" s="5" t="s">
         <v>544</v>
@@ -7006,7 +7007,7 @@
         <v>589</v>
       </c>
       <c r="G135" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="H135" t="s">
         <v>590</v>
@@ -7028,7 +7029,7 @@
       </c>
       <c r="C136" s="5"/>
       <c r="D136" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E136" s="5"/>
       <c r="F136" s="5"/>
@@ -7057,7 +7058,7 @@
         <v>594</v>
       </c>
       <c r="D137" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E137" s="5"/>
       <c r="F137" s="5"/>
@@ -7083,10 +7084,10 @@
         <v>576</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
@@ -7106,16 +7107,16 @@
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
+        <v>720</v>
+      </c>
+      <c r="B139" t="s">
         <v>721</v>
       </c>
-      <c r="B139" t="s">
-        <v>722</v>
-      </c>
       <c r="C139" s="5" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="D139" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E139" s="5" t="s">
         <v>77</v>
@@ -7124,7 +7125,7 @@
         <v>78</v>
       </c>
       <c r="I139" s="6" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="J139" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7139,10 +7140,10 @@
         <v>572</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D140" s="5" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E140" s="5"/>
       <c r="F140" s="5"/>
@@ -7175,7 +7176,7 @@
         <v>70</v>
       </c>
       <c r="F141" s="5" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="G141" t="s">
         <v>425</v>
@@ -7193,14 +7194,14 @@
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142" s="5" t="s">
+        <v>667</v>
+      </c>
+      <c r="B142" s="5" t="s">
         <v>668</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>669</v>
       </c>
       <c r="C142" s="5"/>
       <c r="D142" s="5" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="E142" s="5" t="s">
         <v>77</v>
@@ -7210,10 +7211,10 @@
         <v>77</v>
       </c>
       <c r="H142" s="5" t="s">
+        <v>669</v>
+      </c>
+      <c r="I142" s="6" t="s">
         <v>670</v>
-      </c>
-      <c r="I142" s="6" t="s">
-        <v>671</v>
       </c>
       <c r="J142" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7313,15 +7314,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7330,6 +7322,15 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7528,14 +7529,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7548,6 +7541,14 @@
     <ds:schemaRef ds:uri="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
fix(repertoire-personnel): Correction d'un problème de régression concernant Julie Ouellette
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F536F2-F289-4455-BD5C-233B88CE0983}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E023120D-A5E0-401E-AEBF-0E1F4FE82CBD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5460" yWindow="3555" windowWidth="30315" windowHeight="28125" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5460" yWindow="3560" windowWidth="30320" windowHeight="28130" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2286,9 +2286,6 @@
     <t xml:space="preserve">Direction de la Bibliothèque des  lettres et sciences humaines et Livres rares et collections spéciales; </t>
   </si>
   <si>
-    <t>Bibliothèque des lettres et sciences humaines et Service du prêt entre bibliothèques</t>
-  </si>
-  <si>
     <t>514 343-6111, poste 2744</t>
   </si>
   <si>
@@ -2299,6 +2296,9 @@
   </si>
   <si>
     <t>Communication, journalisme et travail social</t>
+  </si>
+  <si>
+    <t>Bibliothèque des lettres et sciences humaines; Service du prêt entre bibliothèques</t>
   </si>
 </sst>
 </file>
@@ -2653,7 +2653,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J142" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A1:J142" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
   <sortState ref="A2:J142">
-    <sortCondition ref="A1:A142"/>
+    <sortCondition ref="A2:A142"/>
+    <sortCondition ref="B2:B142"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{4B04E1AF-0079-4AD2-81CA-E8A433733E21}" name="nom" dataDxfId="9"/>
@@ -2995,21 +2996,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J142"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="33.85546875" customWidth="1"/>
-    <col min="4" max="4" width="45.28515625" customWidth="1"/>
-    <col min="5" max="5" width="58.140625" customWidth="1"/>
+    <col min="3" max="3" width="33.81640625" customWidth="1"/>
+    <col min="4" max="4" width="45.26953125" customWidth="1"/>
+    <col min="5" max="5" width="58.1796875" customWidth="1"/>
     <col min="6" max="6" width="58" customWidth="1"/>
-    <col min="7" max="7" width="70.85546875" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="41.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="86.5703125" customWidth="1"/>
+    <col min="7" max="7" width="70.81640625" customWidth="1"/>
+    <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="86.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3041,7 +3042,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
@@ -3072,7 +3073,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alexandre.amar-zifkin@umontreal.ca</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -3105,7 +3106,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.angers@umontreal.ca</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>715</v>
       </c>
@@ -3133,7 +3134,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=busch.antenor.alexandre@umontreal.ca</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
@@ -3164,7 +3165,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nadege.arsa@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
@@ -3195,7 +3196,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=denis.arvisais@umontreal.ca</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>38</v>
       </c>
@@ -3228,7 +3229,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.attia@umontreal.ca</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>45</v>
       </c>
@@ -3259,7 +3260,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=prlaval@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -3289,7 +3290,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.bastien@umontreal.ca</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>57</v>
       </c>
@@ -3317,7 +3318,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magalie.beaudoin@umontreal.ca</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>64</v>
       </c>
@@ -3350,7 +3351,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maryna.beaulieu@umontreal.ca</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>70</v>
       </c>
@@ -3380,7 +3381,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.begin-poissant@umontreal.ca</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>699</v>
       </c>
@@ -3411,7 +3412,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nima.behforouz@umontreal.ca</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>75</v>
       </c>
@@ -3441,7 +3442,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.belanger@umontreal.ca</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>82</v>
       </c>
@@ -3474,7 +3475,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amy.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>87</v>
       </c>
@@ -3503,7 +3504,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amelie.bernard@umontreal.ca</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>92</v>
       </c>
@@ -3532,7 +3533,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=hugo.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>92</v>
       </c>
@@ -3559,7 +3560,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>680</v>
       </c>
@@ -3590,7 +3591,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cathy.bingoye@umontreal.ca</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
         <v>100</v>
       </c>
@@ -3621,7 +3622,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon.blais.longtin@umontreal.ca</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>723</v>
       </c>
@@ -3646,7 +3647,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guy.blondeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>106</v>
       </c>
@@ -3676,7 +3677,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tatiana.talpa@umontreal.ca</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>112</v>
       </c>
@@ -3702,7 +3703,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=joanna.bodnar@umontreal.ca</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>116</v>
       </c>
@@ -3732,7 +3733,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alain.borsi@umontreal.ca</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>123</v>
       </c>
@@ -3763,7 +3764,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.p.bouchard@umontreal.ca</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
         <v>130</v>
       </c>
@@ -3794,7 +3795,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refdroi@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>136</v>
       </c>
@@ -3827,7 +3828,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=myriam.boyer@umontreal.ca</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
         <v>140</v>
       </c>
@@ -3856,7 +3857,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guylaine.brazeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>685</v>
       </c>
@@ -3864,7 +3865,7 @@
         <v>346</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>688</v>
@@ -3885,7 +3886,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-marie.brien.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>144</v>
       </c>
@@ -3913,7 +3914,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sophie.brisebois@umontreal.ca</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>667</v>
       </c>
@@ -3946,7 +3947,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tanya.buchet@umontreal.ca</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>149</v>
       </c>
@@ -3973,7 +3974,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fanny.c.brochu@umontreal.ca</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>732</v>
       </c>
@@ -4001,7 +4002,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thierry.caballero@umontreal.ca</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>153</v>
       </c>
@@ -4018,7 +4019,7 @@
         <v>119</v>
       </c>
       <c r="F34" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>156</v>
@@ -4034,7 +4035,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=delphine.cado@umontreal.ca</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>159</v>
       </c>
@@ -4063,7 +4064,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=siv.kham.chao@umontreal.ca</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>164</v>
       </c>
@@ -4094,7 +4095,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=laurence.charest@umontreal.ca</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>171</v>
       </c>
@@ -4118,7 +4119,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=annick.charette@umontreal.ca</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>735</v>
       </c>
@@ -4146,7 +4147,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=wassif.cheikh@umontreal.ca</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
         <v>175</v>
       </c>
@@ -4174,7 +4175,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mailto:thien-huong.che-quang@umontreal.ca</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>177</v>
       </c>
@@ -4205,7 +4206,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah.cherrier@umontreal.ca</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
         <v>183</v>
       </c>
@@ -4235,7 +4236,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emir.chouchane@umontreal.ca</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
         <v>189</v>
       </c>
@@ -4266,7 +4267,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=accessibilite@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>194</v>
       </c>
@@ -4299,7 +4300,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benjamin.constantineau@umontreal.ca</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
         <v>201</v>
       </c>
@@ -4330,7 +4331,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon-pierre.crevier@umontreal.ca</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
         <v>207</v>
       </c>
@@ -4345,7 +4346,7 @@
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="5" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>54</v>
@@ -4361,7 +4362,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marc-olivier.croteau@umontreal.ca</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
         <v>211</v>
       </c>
@@ -4392,7 +4393,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.dalpe@umontreal.ca</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
         <v>217</v>
       </c>
@@ -4423,7 +4424,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=morgane.de.bellefeuille@umontreal.ca</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>224</v>
       </c>
@@ -4454,7 +4455,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=Indiana.delsart@umontreal.ca</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
         <v>230</v>
       </c>
@@ -4485,7 +4486,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=dominic.desaulniers@umontreal.ca</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>236</v>
       </c>
@@ -4514,7 +4515,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.desrosiers@umontreal.ca</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>241</v>
       </c>
@@ -4541,7 +4542,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.dubois.mercier@umontreal.ca</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>245</v>
       </c>
@@ -4572,7 +4573,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jean-francois.durnin@umontreal.ca</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>662</v>
       </c>
@@ -4603,7 +4604,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=taline.ekmekjian@umontreal.ca</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>251</v>
       </c>
@@ -4630,7 +4631,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=judith.fafard-larose@umontreal.ca</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>255</v>
       </c>
@@ -4663,7 +4664,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>260</v>
       </c>
@@ -4696,7 +4697,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=c.fortier@umontreal.ca</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>266</v>
       </c>
@@ -4723,7 +4724,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>272</v>
       </c>
@@ -4754,7 +4755,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nino.gabrielli@umontreal.ca</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
         <v>278</v>
       </c>
@@ -4783,7 +4784,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-pierre.gadoua@umontreal.ca</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
         <v>282</v>
       </c>
@@ -4814,7 +4815,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cynthia.gagne.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>289</v>
       </c>
@@ -4840,7 +4841,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>289</v>
       </c>
@@ -4868,7 +4869,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
         <v>295</v>
       </c>
@@ -4898,7 +4899,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marjorie.gauchier@umontreal.ca</v>
       </c>
     </row>
-    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>714</v>
       </c>
@@ -4927,7 +4928,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=lucie.geoffroy@umontreal.ca</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
         <v>301</v>
       </c>
@@ -4954,7 +4955,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
       </c>
     </row>
-    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
         <v>304</v>
       </c>
@@ -4987,7 +4988,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.giguere.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>712</v>
       </c>
@@ -5018,7 +5019,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.hainault@umontreal.ca</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>309</v>
       </c>
@@ -5049,7 +5050,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
         <v>314</v>
       </c>
@@ -5080,7 +5081,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>320</v>
       </c>
@@ -5110,7 +5111,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>713</v>
       </c>
@@ -5141,7 +5142,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=natalia.jabinschi@umontreal.ca</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
         <v>326</v>
       </c>
@@ -5170,7 +5171,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
         <v>331</v>
       </c>
@@ -5201,7 +5202,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>336</v>
       </c>
@@ -5228,7 +5229,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
       </c>
     </row>
-    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>718</v>
       </c>
@@ -5257,7 +5258,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pierre-yves.lafleur@umontreal.ca</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
         <v>340</v>
       </c>
@@ -5284,7 +5285,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>342</v>
       </c>
@@ -5311,7 +5312,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
         <v>345</v>
       </c>
@@ -5344,7 +5345,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
       </c>
     </row>
-    <row r="79" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
         <v>351</v>
       </c>
@@ -5377,7 +5378,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
       </c>
     </row>
-    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A80" s="18" t="s">
         <v>743</v>
       </c>
@@ -5406,7 +5407,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-josee.lapalme@umontreal.ca</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
         <v>356</v>
       </c>
@@ -5439,7 +5440,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>360</v>
       </c>
@@ -5466,7 +5467,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
         <v>364</v>
       </c>
@@ -5497,7 +5498,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>369</v>
       </c>
@@ -5528,7 +5529,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
         <v>374</v>
       </c>
@@ -5559,7 +5560,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
         <v>379</v>
       </c>
@@ -5592,7 +5593,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
         <v>385</v>
       </c>
@@ -5622,7 +5623,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
         <v>389</v>
       </c>
@@ -5653,7 +5654,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
         <v>394</v>
       </c>
@@ -5686,7 +5687,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
         <v>394</v>
       </c>
@@ -5712,7 +5713,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
         <v>400</v>
       </c>
@@ -5741,7 +5742,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
         <v>404</v>
       </c>
@@ -5770,7 +5771,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
         <v>409</v>
       </c>
@@ -5798,7 +5799,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
         <v>413</v>
       </c>
@@ -5829,7 +5830,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
         <v>418</v>
       </c>
@@ -5860,7 +5861,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
         <v>424</v>
       </c>
@@ -5890,7 +5891,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
       </c>
     </row>
-    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
         <v>430</v>
       </c>
@@ -5919,7 +5920,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
       </c>
     </row>
-    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
         <v>434</v>
       </c>
@@ -5950,7 +5951,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="3" t="s">
         <v>440</v>
       </c>
@@ -5981,7 +5982,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="s">
         <v>445</v>
       </c>
@@ -6012,7 +6013,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="18" t="s">
         <v>748</v>
       </c>
@@ -6043,7 +6044,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.moreau@umontreal.ca</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>450</v>
       </c>
@@ -6074,7 +6075,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
       </c>
     </row>
-    <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A103" s="3" t="s">
         <v>455</v>
       </c>
@@ -6105,7 +6106,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A104" s="5" t="s">
         <v>459</v>
       </c>
@@ -6136,7 +6137,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
         <v>465</v>
       </c>
@@ -6162,7 +6163,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
         <v>469</v>
       </c>
@@ -6180,7 +6181,7 @@
       </c>
       <c r="F106" s="3"/>
       <c r="G106" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="H106" s="5" t="s">
         <v>471</v>
@@ -6193,7 +6194,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=julie.ouellette@umontreal.ca</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
         <v>473</v>
       </c>
@@ -6220,7 +6221,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
         <v>478</v>
       </c>
@@ -6251,7 +6252,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
         <v>478</v>
       </c>
@@ -6284,7 +6285,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
         <v>487</v>
       </c>
@@ -6315,7 +6316,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
         <v>491</v>
       </c>
@@ -6344,7 +6345,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
         <v>495</v>
       </c>
@@ -6375,7 +6376,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
         <v>501</v>
       </c>
@@ -6404,7 +6405,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>505</v>
       </c>
@@ -6431,7 +6432,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>721</v>
       </c>
@@ -6459,7 +6460,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>509</v>
       </c>
@@ -6484,7 +6485,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>711</v>
       </c>
@@ -6513,7 +6514,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>649</v>
       </c>
@@ -6542,7 +6543,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>513</v>
       </c>
@@ -6572,7 +6573,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>729</v>
       </c>
@@ -6600,7 +6601,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A121" s="5" t="s">
         <v>518</v>
       </c>
@@ -6628,7 +6629,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
         <v>521</v>
       </c>
@@ -6657,7 +6658,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>525</v>
       </c>
@@ -6680,7 +6681,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A124" s="3" t="s">
         <v>527</v>
       </c>
@@ -6711,7 +6712,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A125" s="3" t="s">
         <v>533</v>
       </c>
@@ -6738,7 +6739,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A126" s="5" t="s">
         <v>536</v>
       </c>
@@ -6768,7 +6769,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>654</v>
       </c>
@@ -6797,7 +6798,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
         <v>541</v>
       </c>
@@ -6818,7 +6819,7 @@
         <v>421</v>
       </c>
       <c r="H128" s="5" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="I128" s="8" t="s">
         <v>543</v>
@@ -6828,7 +6829,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A129" s="3" t="s">
         <v>544</v>
       </c>
@@ -6861,7 +6862,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A130" s="5" t="s">
         <v>551</v>
       </c>
@@ -6892,7 +6893,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="s">
         <v>555</v>
       </c>
@@ -6923,7 +6924,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
         <v>559</v>
       </c>
@@ -6954,7 +6955,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>564</v>
       </c>
@@ -6978,7 +6979,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A134" s="5" t="s">
         <v>564</v>
       </c>
@@ -7007,7 +7008,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>592</v>
       </c>
@@ -7040,7 +7041,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A136" s="5" t="s">
         <v>570</v>
       </c>
@@ -7067,7 +7068,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="s">
         <v>574</v>
       </c>
@@ -7096,7 +7097,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="s">
         <v>578</v>
       </c>
@@ -7125,7 +7126,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>726</v>
       </c>
@@ -7152,7 +7153,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A140" s="5" t="s">
         <v>582</v>
       </c>
@@ -7181,7 +7182,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A141" s="5" t="s">
         <v>585</v>
       </c>
@@ -7212,7 +7213,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="s">
         <v>673</v>
       </c>
@@ -7529,6 +7530,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1">
@@ -7537,15 +7547,6 @@
     <TaxCatchAll xmlns="9cb1c2f4-2737-4134-a1af-8acbe3d02830" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7568,6 +7569,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7582,12 +7591,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(repertoire-personnel): Correction d'une régression concernant Julie Ouellette
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B171802-AAEA-499A-BCE5-62494C54E740}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{421D5A94-17B4-4C36-84BB-FB59B6C0C11B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="31920" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2268,9 +2268,6 @@
     <t xml:space="preserve">Direction de la Bibliothèque des  lettres et sciences humaines et Livres rares et collections spéciales; </t>
   </si>
   <si>
-    <t>Bibliothèque des lettres et sciences humaines et Service du prêt entre bibliothèques</t>
-  </si>
-  <si>
     <t>514 343-6111, poste 2744</t>
   </si>
   <si>
@@ -2308,6 +2305,9 @@
   </si>
   <si>
     <t>billie.bergeron@umontreal.ca</t>
+  </si>
+  <si>
+    <t>Bibliothèque des lettres et sciences humaines; Service du prêt entre bibliothèques</t>
   </si>
 </sst>
 </file>
@@ -3376,7 +3376,7 @@
         <v>71</v>
       </c>
       <c r="G12" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>72</v>
@@ -3455,7 +3455,7 @@
         <v>81</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="17" t="s">
@@ -3469,10 +3469,10 @@
         <v>285</v>
       </c>
       <c r="H15" s="19" t="s">
+        <v>758</v>
+      </c>
+      <c r="I15" s="6" t="s">
         <v>759</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>760</v>
       </c>
       <c r="J15" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -3852,7 +3852,7 @@
         <v>602</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>137</v>
@@ -3885,7 +3885,7 @@
         <v>347</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="H29" s="5" t="s">
         <v>141</v>
@@ -3906,7 +3906,7 @@
         <v>345</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>682</v>
@@ -4060,7 +4060,7 @@
         <v>118</v>
       </c>
       <c r="F35" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>155</v>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>53</v>
@@ -5373,7 +5373,7 @@
         <v>347</v>
       </c>
       <c r="G79" s="5" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="H79" s="5" t="s">
         <v>348</v>
@@ -5556,7 +5556,7 @@
         <v>70</v>
       </c>
       <c r="F85" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="G85" s="5" t="s">
         <v>425</v>
@@ -6042,10 +6042,10 @@
         <v>70</v>
       </c>
       <c r="F101" s="5" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G101" s="5" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="H101" s="5" t="s">
         <v>446</v>
@@ -6106,7 +6106,7 @@
         <v>70</v>
       </c>
       <c r="F103" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="G103" s="5" t="s">
         <v>425</v>
@@ -6228,7 +6228,7 @@
       </c>
       <c r="F107" s="3"/>
       <c r="G107" t="s">
-        <v>747</v>
+        <v>760</v>
       </c>
       <c r="H107" s="5" t="s">
         <v>468</v>
@@ -6864,7 +6864,7 @@
         <v>419</v>
       </c>
       <c r="H129" s="5" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="I129" s="8" t="s">
         <v>540</v>
@@ -7240,7 +7240,7 @@
         <v>70</v>
       </c>
       <c r="F142" s="5" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="G142" t="s">
         <v>425</v>
@@ -7390,6 +7390,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CC83367596A4B94585FCDD3502D89912" ma:contentTypeVersion="11" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="4e4efa8c0f0f722bbfc4a6b86077b9b4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1" xmlns:ns3="9cb1c2f4-2737-4134-a1af-8acbe3d02830" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81c6aeae46cd0fb81a99420a9570330b" ns2:_="" ns3:_="">
     <xsd:import namespace="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
@@ -7584,15 +7593,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
@@ -7611,6 +7611,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCC2BCD-0310-4A3C-9E4B-6EFDEBA53649}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7627,12 +7635,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(repertoire-personnel): Changements concernant François-Xavier Panaccio
</commit_message>
<xml_diff>
--- a/content/personnel/liste-personnel.xlsx
+++ b/content/personnel/liste-personnel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projets\coquille-web\content\personnel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{421D5A94-17B4-4C36-84BB-FB59B6C0C11B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA8F971-2809-4A4B-9D37-65390BE8D030}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="31920" tabRatio="130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="764">
   <si>
     <t>nom</t>
   </si>
@@ -1443,9 +1443,6 @@
     <t>François-Xavier</t>
   </si>
   <si>
-    <t>Technopédagoque</t>
-  </si>
-  <si>
     <t xml:space="preserve">Offre pédagogique en bibliothèque </t>
   </si>
   <si>
@@ -2308,6 +2305,18 @@
   </si>
   <si>
     <t>Bibliothèque des lettres et sciences humaines; Service du prêt entre bibliothèques</t>
+  </si>
+  <si>
+    <t>Technopédagogue</t>
+  </si>
+  <si>
+    <t>Direction des bibliothèques sociétés et création</t>
+  </si>
+  <si>
+    <t>Bibliothèque d'aménagement; Bibliothèque de droit; Bibliothèque Thérèse-Gouin-Décarie; Bibliothèque du Campus de Laval; Bibliothèque de musique</t>
+  </si>
+  <si>
+    <t>514 910-2720</t>
   </si>
 </sst>
 </file>
@@ -2661,7 +2670,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}" name="Tableau1" displayName="Tableau1" ref="A1:J143" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J143" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}"/>
+  <autoFilter ref="A1:J143" xr:uid="{4A0AF7E1-A614-44BF-8C48-5C26377DC552}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Panaccio"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState ref="A2:J143">
     <sortCondition ref="A1:A143"/>
   </sortState>
@@ -3051,7 +3066,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
@@ -3082,7 +3097,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alexandre.amar-zifkin@umontreal.ca</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -3097,7 +3112,7 @@
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>21</v>
@@ -3113,16 +3128,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.angers@umontreal.ca</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>708</v>
+      </c>
+      <c r="B4" t="s">
         <v>709</v>
-      </c>
-      <c r="B4" t="s">
-        <v>710</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>77</v>
@@ -3134,14 +3149,14 @@
         <v>307</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="J4" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=busch.antenor.alexandre@umontreal.ca</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
@@ -3172,7 +3187,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nadege.arsa@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
@@ -3203,7 +3218,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=denis.arvisais@umontreal.ca</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>38</v>
       </c>
@@ -3214,16 +3229,16 @@
         <v>40</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>41</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>42</v>
@@ -3236,7 +3251,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.attia@umontreal.ca</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>44</v>
       </c>
@@ -3247,7 +3262,7 @@
         <v>46</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
@@ -3265,7 +3280,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=prlaval@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>49</v>
       </c>
@@ -3295,7 +3310,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.bastien@umontreal.ca</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>56</v>
       </c>
@@ -3323,7 +3338,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magalie.beaudoin@umontreal.ca</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>63</v>
       </c>
@@ -3334,16 +3349,16 @@
         <v>65</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E11" t="s">
         <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>67</v>
@@ -3356,7 +3371,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maryna.beaulieu@umontreal.ca</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>69</v>
       </c>
@@ -3364,10 +3379,10 @@
         <v>39</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>70</v>
@@ -3376,7 +3391,7 @@
         <v>71</v>
       </c>
       <c r="G12" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>72</v>
@@ -3389,15 +3404,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=audrey.begin-poissant@umontreal.ca</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B13" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>27</v>
@@ -3413,14 +3428,14 @@
         <v>307</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="J13" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=nima.behforouz@umontreal.ca</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>74</v>
       </c>
@@ -3431,7 +3446,7 @@
         <v>76</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>77</v>
@@ -3450,16 +3465,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.belanger@umontreal.ca</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="17" t="s">
         <v>81</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="17" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="E15" s="17" t="s">
         <v>118</v>
@@ -3469,17 +3484,17 @@
         <v>285</v>
       </c>
       <c r="H15" s="19" t="s">
+        <v>757</v>
+      </c>
+      <c r="I15" s="6" t="s">
         <v>758</v>
       </c>
-      <c r="I15" s="6" t="s">
-        <v>759</v>
-      </c>
       <c r="J15" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=billie.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>81</v>
       </c>
@@ -3496,7 +3511,7 @@
         <v>118</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>15</v>
@@ -3512,7 +3527,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amy.bergeron@umontreal.ca</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>86</v>
       </c>
@@ -3520,10 +3535,10 @@
         <v>87</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
@@ -3541,7 +3556,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=amelie.bernard@umontreal.ca</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>91</v>
       </c>
@@ -3570,7 +3585,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=hugo.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>91</v>
       </c>
@@ -3578,10 +3593,10 @@
         <v>96</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G19" t="s">
         <v>29</v>
@@ -3597,15 +3612,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.bernier@umontreal.ca</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
+        <v>673</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>674</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>675</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>676</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>27</v>
@@ -3614,21 +3629,21 @@
         <v>77</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="G20" t="s">
         <v>77</v>
       </c>
       <c r="H20" s="5"/>
       <c r="I20" s="6" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="J20" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=cathy.bingoye@umontreal.ca</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>99</v>
       </c>
@@ -3659,16 +3674,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon.blais.longtin@umontreal.ca</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
+        <v>716</v>
+      </c>
+      <c r="B22" t="s">
         <v>717</v>
-      </c>
-      <c r="B22" t="s">
-        <v>718</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>77</v>
@@ -3677,14 +3692,14 @@
         <v>78</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="J22" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=guy.blondeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>105</v>
       </c>
@@ -3714,7 +3729,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tatiana.talpa@umontreal.ca</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>111</v>
       </c>
@@ -3723,7 +3738,7 @@
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>59</v>
@@ -3740,7 +3755,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=joanna.bodnar@umontreal.ca</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>115</v>
       </c>
@@ -3751,7 +3766,7 @@
         <v>117</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E25" t="s">
         <v>118</v>
@@ -3770,7 +3785,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alain.borsi@umontreal.ca</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
         <v>122</v>
       </c>
@@ -3801,7 +3816,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.p.bouchard@umontreal.ca</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>129</v>
       </c>
@@ -3832,7 +3847,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=refdroi@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
         <v>135</v>
       </c>
@@ -3840,19 +3855,19 @@
         <v>136</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>70</v>
       </c>
       <c r="F28" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>137</v>
@@ -3865,7 +3880,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=myriam.boyer@umontreal.ca</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>139</v>
       </c>
@@ -3873,10 +3888,10 @@
         <v>140</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>70</v>
@@ -3885,7 +3900,7 @@
         <v>347</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="H29" s="5" t="s">
         <v>141</v>
@@ -3898,18 +3913,18 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=guylaine.brazeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>345</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E30" s="5"/>
       <c r="F30" s="5"/>
@@ -3917,17 +3932,17 @@
         <v>29</v>
       </c>
       <c r="H30" s="5" t="s">
+        <v>679</v>
+      </c>
+      <c r="I30" s="6" t="s">
         <v>680</v>
       </c>
-      <c r="I30" s="6" t="s">
-        <v>681</v>
-      </c>
       <c r="J30" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-marie.brien.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>143</v>
       </c>
@@ -3938,7 +3953,7 @@
         <v>145</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>59</v>
@@ -3955,15 +3970,15 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sophie.brisebois@umontreal.ca</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
+        <v>660</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>661</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="C32" s="5" t="s">
         <v>662</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>663</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>13</v>
@@ -3972,23 +3987,23 @@
         <v>118</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="G32" t="s">
         <v>15</v>
       </c>
       <c r="H32" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="I32" s="6" t="s">
         <v>665</v>
       </c>
-      <c r="I32" s="6" t="s">
-        <v>666</v>
-      </c>
       <c r="J32" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=tanya.buchet@umontreal.ca</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>148</v>
       </c>
@@ -3996,10 +4011,10 @@
         <v>149</v>
       </c>
       <c r="C33" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G33" t="s">
         <v>29</v>
@@ -4015,16 +4030,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fanny.c.brochu@umontreal.ca</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
+        <v>725</v>
+      </c>
+      <c r="B34" t="s">
         <v>726</v>
-      </c>
-      <c r="B34" t="s">
-        <v>727</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>77</v>
@@ -4033,17 +4048,17 @@
         <v>78</v>
       </c>
       <c r="H34" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="J34" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=thierry.caballero@umontreal.ca</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>152</v>
       </c>
@@ -4051,7 +4066,7 @@
         <v>153</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>13</v>
@@ -4060,7 +4075,7 @@
         <v>118</v>
       </c>
       <c r="F35" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>155</v>
@@ -4076,7 +4091,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=delphine.cado@umontreal.ca</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>158</v>
       </c>
@@ -4084,10 +4099,10 @@
         <v>159</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E36" s="5"/>
       <c r="F36" s="5"/>
@@ -4105,7 +4120,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=siv.kham.chao@umontreal.ca</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
         <v>163</v>
       </c>
@@ -4136,7 +4151,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=laurence.charest@umontreal.ca</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>170</v>
       </c>
@@ -4144,10 +4159,10 @@
         <v>171</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G38" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="H38" s="5" t="s">
         <v>172</v>
@@ -4160,16 +4175,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=annick.charette@umontreal.ca</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
+        <v>728</v>
+      </c>
+      <c r="B39" t="s">
         <v>729</v>
-      </c>
-      <c r="B39" t="s">
-        <v>730</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E39" s="5" t="s">
         <v>77</v>
@@ -4178,17 +4193,17 @@
         <v>78</v>
       </c>
       <c r="H39" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="I39" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="J39" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=wassif.cheikh@umontreal.ca</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>174</v>
       </c>
@@ -4197,7 +4212,7 @@
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E40" s="10" t="s">
         <v>59</v>
@@ -4206,17 +4221,17 @@
         <v>59</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="J40" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=mailto:thien-huong.che-quang@umontreal.ca</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
         <v>176</v>
       </c>
@@ -4247,7 +4262,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah.cherrier@umontreal.ca</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
         <v>182</v>
       </c>
@@ -4258,7 +4273,7 @@
         <v>184</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E42" s="5" t="s">
         <v>77</v>
@@ -4277,7 +4292,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emir.chouchane@umontreal.ca</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>188</v>
       </c>
@@ -4285,7 +4300,7 @@
         <v>189</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>27</v>
@@ -4308,7 +4323,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=accessibilite@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
         <v>193</v>
       </c>
@@ -4319,7 +4334,7 @@
         <v>195</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E44" t="s">
         <v>196</v>
@@ -4328,7 +4343,7 @@
         <v>197</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="H44" s="5" t="s">
         <v>198</v>
@@ -4341,7 +4356,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benjamin.constantineau@umontreal.ca</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
         <v>200</v>
       </c>
@@ -4372,7 +4387,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=simon-pierre.crevier@umontreal.ca</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
         <v>206</v>
       </c>
@@ -4380,14 +4395,14 @@
         <v>207</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>53</v>
@@ -4403,7 +4418,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marc-olivier.croteau@umontreal.ca</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
         <v>210</v>
       </c>
@@ -4434,7 +4449,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.dalpe@umontreal.ca</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>216</v>
       </c>
@@ -4445,7 +4460,7 @@
         <v>218</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E48" s="5"/>
       <c r="F48" t="s">
@@ -4465,7 +4480,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=morgane.de.bellefeuille@umontreal.ca</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
         <v>223</v>
       </c>
@@ -4483,7 +4498,7 @@
         <v>226</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="H49" s="5" t="s">
         <v>227</v>
@@ -4496,7 +4511,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=Indiana.delsart@umontreal.ca</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>229</v>
       </c>
@@ -4527,7 +4542,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=dominic.desaulniers@umontreal.ca</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>235</v>
       </c>
@@ -4535,10 +4550,10 @@
         <v>236</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>
@@ -4556,7 +4571,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.desrosiers@umontreal.ca</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>240</v>
       </c>
@@ -4564,10 +4579,10 @@
         <v>241</v>
       </c>
       <c r="C52" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G52" t="s">
         <v>29</v>
@@ -4583,7 +4598,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.dubois.mercier@umontreal.ca</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>244</v>
       </c>
@@ -4614,12 +4629,12 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jean-francois.durnin@umontreal.ca</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="B54" s="5" t="s">
         <v>656</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>657</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5" t="s">
@@ -4629,23 +4644,23 @@
         <v>118</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="G54" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H54" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="I54" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="I54" s="6" t="s">
-        <v>660</v>
-      </c>
       <c r="J54" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=taline.ekmekjian@umontreal.ca</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>250</v>
       </c>
@@ -4653,10 +4668,10 @@
         <v>251</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G55" t="s">
         <v>29</v>
@@ -4672,7 +4687,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=judith.fafard-larose@umontreal.ca</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>254</v>
       </c>
@@ -4683,7 +4698,7 @@
         <v>256</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E56" s="5" t="s">
         <v>118</v>
@@ -4705,7 +4720,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=sylvie.fontaine.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>259</v>
       </c>
@@ -4716,7 +4731,7 @@
         <v>261</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E57" s="11" t="s">
         <v>262</v>
@@ -4738,7 +4753,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=c.fortier@umontreal.ca</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>265</v>
       </c>
@@ -4747,7 +4762,7 @@
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E58" s="5"/>
       <c r="F58" s="5"/>
@@ -4765,7 +4780,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=7077duParc@bib.umontreal.ca</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
         <v>271</v>
       </c>
@@ -4796,7 +4811,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=nino.gabrielli@umontreal.ca</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
         <v>277</v>
       </c>
@@ -4804,10 +4819,10 @@
         <v>278</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E60" s="5"/>
       <c r="F60" s="5" t="s">
@@ -4825,7 +4840,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-pierre.gadoua@umontreal.ca</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>281</v>
       </c>
@@ -4856,7 +4871,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=cynthia.gagne.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>288</v>
       </c>
@@ -4865,7 +4880,7 @@
       </c>
       <c r="C62" s="5"/>
       <c r="D62" s="3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E62" s="5" t="s">
         <v>118</v>
@@ -4882,7 +4897,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
         <v>288</v>
       </c>
@@ -4893,7 +4908,7 @@
         <v>290</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="E63" s="5" t="s">
         <v>237</v>
@@ -4910,7 +4925,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.gagnon@umontreal.ca</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="s">
         <v>294</v>
       </c>
@@ -4940,12 +4955,12 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marjorie.gauchier@umontreal.ca</v>
       </c>
     </row>
-    <row r="65" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B65" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C65" s="5"/>
       <c r="D65" s="5" t="s">
@@ -4962,14 +4977,14 @@
         <v>307</v>
       </c>
       <c r="I65" s="15" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="J65" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=lucie.geoffroy@umontreal.ca</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
         <v>300</v>
       </c>
@@ -4978,7 +4993,7 @@
       </c>
       <c r="C66" s="5"/>
       <c r="D66" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
@@ -4986,7 +5001,7 @@
         <v>301</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="I66" s="8" t="s">
         <v>302</v>
@@ -4996,7 +5011,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=noemie.gervais@umontreal.ca</v>
       </c>
     </row>
-    <row r="67" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="5" t="s">
         <v>303</v>
       </c>
@@ -5004,7 +5019,7 @@
         <v>304</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>27</v>
@@ -5022,25 +5037,25 @@
         <v>307</v>
       </c>
       <c r="I67" s="5" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="J67" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.giguere.4@umontreal.ca</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B68" t="s">
         <v>289</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="D68" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E68" s="5" t="s">
         <v>77</v>
@@ -5053,14 +5068,14 @@
         <v>307</v>
       </c>
       <c r="I68" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="J68" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.hainault@umontreal.ca</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
         <v>308</v>
       </c>
@@ -5091,7 +5106,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne.hakier@umontreal.ca</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
         <v>313</v>
       </c>
@@ -5122,7 +5137,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=rose.carine.henriquez@umontreal.ca</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>319</v>
       </c>
@@ -5152,18 +5167,18 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=thien.sa.hoang@umontreal.ca</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="B72" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D72" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>77</v>
@@ -5176,14 +5191,14 @@
         <v>307</v>
       </c>
       <c r="I72" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="J72" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=natalia.jabinschi@umontreal.ca</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
         <v>325</v>
       </c>
@@ -5194,7 +5209,7 @@
         <v>327</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>70</v>
@@ -5212,7 +5227,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=khalid.jouamaa@umontreal.ca</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
         <v>330</v>
       </c>
@@ -5227,7 +5242,7 @@
       </c>
       <c r="E74" s="5"/>
       <c r="F74" s="5" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="G74" s="5" t="s">
         <v>29</v>
@@ -5243,7 +5258,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=aminata.keita@umontreal.ca</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>335</v>
       </c>
@@ -5251,10 +5266,10 @@
         <v>336</v>
       </c>
       <c r="C75" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G75" t="s">
         <v>285</v>
@@ -5270,16 +5285,16 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.lachapelle@umontreal.ca</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
+        <v>711</v>
+      </c>
+      <c r="B76" t="s">
         <v>712</v>
-      </c>
-      <c r="B76" t="s">
-        <v>713</v>
       </c>
       <c r="C76" s="5"/>
       <c r="D76" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E76" s="5" t="s">
         <v>77</v>
@@ -5292,14 +5307,14 @@
         <v>307</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="J76" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=pierre-yves.lafleur@umontreal.ca</v>
       </c>
     </row>
-    <row r="77" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
         <v>339</v>
       </c>
@@ -5308,7 +5323,7 @@
       </c>
       <c r="C77" s="5"/>
       <c r="D77" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E77" s="5"/>
       <c r="F77" s="5"/>
@@ -5319,14 +5334,14 @@
         <v>340</v>
       </c>
       <c r="I77" s="6" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="J77" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=isabelle.lagadec@umontreal.ca</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>341</v>
       </c>
@@ -5334,10 +5349,10 @@
         <v>96</v>
       </c>
       <c r="C78" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G78" t="s">
         <v>29</v>
@@ -5353,7 +5368,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-france.laliberte@umontreal.ca</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
         <v>344</v>
       </c>
@@ -5373,7 +5388,7 @@
         <v>347</v>
       </c>
       <c r="G79" s="5" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="H79" s="5" t="s">
         <v>348</v>
@@ -5386,7 +5401,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=am.lalonde@umontreal.ca</v>
       </c>
     </row>
-    <row r="80" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
         <v>350</v>
       </c>
@@ -5397,7 +5412,7 @@
         <v>352</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E80" s="5" t="s">
         <v>118</v>
@@ -5419,36 +5434,36 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=tara.landry@umontreal.ca</v>
       </c>
     </row>
-    <row r="81" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
+        <v>736</v>
+      </c>
+      <c r="B81" s="5" t="s">
         <v>737</v>
-      </c>
-      <c r="B81" s="5" t="s">
-        <v>738</v>
       </c>
       <c r="C81" s="5"/>
       <c r="D81" s="5" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F81" s="5"/>
       <c r="G81" s="5" t="s">
         <v>126</v>
       </c>
       <c r="H81" s="5" t="s">
+        <v>739</v>
+      </c>
+      <c r="I81" s="6" t="s">
         <v>740</v>
       </c>
-      <c r="I81" s="6" t="s">
-        <v>741</v>
-      </c>
       <c r="J81" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=marie-josee.lapalme@umontreal.ca</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
         <v>355</v>
       </c>
@@ -5456,10 +5471,10 @@
         <v>289</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E82" s="11" t="s">
         <v>262</v>
@@ -5481,7 +5496,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.lariviere-roberge@umontreal.ca</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>359</v>
       </c>
@@ -5489,10 +5504,10 @@
         <v>360</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G83" t="s">
         <v>29</v>
@@ -5508,7 +5523,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=alex-sandrine.lavallee-masse@umontreal.ca</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="s">
         <v>363</v>
       </c>
@@ -5523,7 +5538,7 @@
       </c>
       <c r="E84" s="5"/>
       <c r="F84" s="5" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="G84" s="5" t="s">
         <v>29</v>
@@ -5539,7 +5554,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=graham.lavender@umontreal.ca</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>368</v>
       </c>
@@ -5547,7 +5562,7 @@
         <v>369</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>27</v>
@@ -5556,7 +5571,7 @@
         <v>70</v>
       </c>
       <c r="F85" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="G85" s="5" t="s">
         <v>425</v>
@@ -5572,7 +5587,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jessica.legault.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
         <v>372</v>
       </c>
@@ -5583,7 +5598,7 @@
         <v>374</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E86" s="5" t="s">
         <v>70</v>
@@ -5603,7 +5618,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=genevieve.lemarier@umontreal.ca</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
         <v>377</v>
       </c>
@@ -5614,7 +5629,7 @@
         <v>379</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>118</v>
@@ -5623,7 +5638,7 @@
         <v>380</v>
       </c>
       <c r="G87" s="5" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="H87" s="5" t="s">
         <v>381</v>
@@ -5636,7 +5651,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mariane.leonard@umontreal.ca</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
         <v>383</v>
       </c>
@@ -5644,10 +5659,10 @@
         <v>384</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E88" s="5" t="s">
         <v>77</v>
@@ -5666,7 +5681,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=maude.lethiecq-normand@umontreal.ca</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
         <v>387</v>
       </c>
@@ -5677,7 +5692,7 @@
         <v>389</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="E89" s="11" t="s">
         <v>262</v>
@@ -5697,7 +5712,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=danny.letourneau@umontreal.ca</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="3" t="s">
         <v>392</v>
       </c>
@@ -5705,19 +5720,19 @@
         <v>393</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F90" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="H90" s="3" t="s">
         <v>394</v>
@@ -5730,7 +5745,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ae.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
         <v>392</v>
       </c>
@@ -5738,10 +5753,10 @@
         <v>396</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="E91" s="5" t="s">
         <v>77</v>
@@ -5756,7 +5771,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=anny.levesque@umontreal.ca</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
         <v>398</v>
       </c>
@@ -5764,10 +5779,10 @@
         <v>399</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
@@ -5785,7 +5800,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=jason.madooray@umontreal.ca</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
         <v>402</v>
       </c>
@@ -5793,10 +5808,10 @@
         <v>403</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D93" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E93" s="5"/>
       <c r="F93" s="5"/>
@@ -5814,7 +5829,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=yacine.mansar@umontreal.ca</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
         <v>407</v>
       </c>
@@ -5822,10 +5837,10 @@
         <v>408</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E94" s="5"/>
       <c r="G94" s="5" t="s">
@@ -5842,7 +5857,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=vanessa.martin.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
         <v>411</v>
       </c>
@@ -5857,7 +5872,7 @@
       </c>
       <c r="E95" s="5"/>
       <c r="F95" s="5" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="G95" s="5" t="s">
         <v>29</v>
@@ -5873,7 +5888,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=pascal.martinolli@umontreal.ca</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
         <v>416</v>
       </c>
@@ -5904,7 +5919,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=melanie.masse.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
         <v>422</v>
       </c>
@@ -5915,7 +5930,7 @@
         <v>424</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E97" s="5" t="s">
         <v>70</v>
@@ -5934,7 +5949,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=gabrielle.mathieu-dupuis@umontreal.ca</v>
       </c>
     </row>
-    <row r="98" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
         <v>428</v>
       </c>
@@ -5942,10 +5957,10 @@
         <v>429</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D98" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E98" s="5"/>
       <c r="F98" s="5"/>
@@ -5963,7 +5978,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=benoit.mayrand@umontreal.ca</v>
       </c>
     </row>
-    <row r="99" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="5" t="s">
         <v>432</v>
       </c>
@@ -5994,7 +6009,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=christiane.melancon@umontreal.ca</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="3" t="s">
         <v>438</v>
       </c>
@@ -6025,7 +6040,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=ginette-denyse.melancon.bolduc@umontreal.ca</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="5" t="s">
         <v>443</v>
       </c>
@@ -6042,10 +6057,10 @@
         <v>70</v>
       </c>
       <c r="F101" s="5" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="G101" s="5" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="H101" s="5" t="s">
         <v>446</v>
@@ -6058,18 +6073,18 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=justine.menard.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="5" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>292</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="D102" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E102" t="s">
         <v>66</v>
@@ -6079,17 +6094,17 @@
         <v>126</v>
       </c>
       <c r="H102" s="5" t="s">
+        <v>743</v>
+      </c>
+      <c r="I102" s="6" t="s">
         <v>744</v>
       </c>
-      <c r="I102" s="6" t="s">
-        <v>745</v>
-      </c>
       <c r="J102" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=diane.moreau@umontreal.ca</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>448</v>
       </c>
@@ -6097,7 +6112,7 @@
         <v>449</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>27</v>
@@ -6106,7 +6121,7 @@
         <v>70</v>
       </c>
       <c r="F103" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G103" s="5" t="s">
         <v>425</v>
@@ -6122,7 +6137,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.murray-samuel@umontreal.ca</v>
       </c>
     </row>
-    <row r="104" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="3" t="s">
         <v>452</v>
       </c>
@@ -6130,17 +6145,17 @@
         <v>453</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D104" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F104" s="12"/>
       <c r="G104" s="3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="H104" s="3" t="s">
         <v>454</v>
@@ -6153,7 +6168,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=france.nadeau@umontreal.ca</v>
       </c>
     </row>
-    <row r="105" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
         <v>456</v>
       </c>
@@ -6161,7 +6176,7 @@
         <v>457</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>458</v>
@@ -6184,7 +6199,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=magdalena.oriental@umontreal.ca</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
         <v>462</v>
       </c>
@@ -6193,7 +6208,7 @@
       </c>
       <c r="C106" s="5"/>
       <c r="D106" s="3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E106" s="5" t="s">
         <v>70</v>
@@ -6210,7 +6225,7 @@
         <v>https://teams.microsoft.com/l/chat/0/0?users=fatima.zahra.ouadrhiri@umontreal.ca</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
         <v>466</v>
       </c>
@@ -6218,17 +6233,17 @@
         <v>467</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="D107" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E107" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="F107" s="3"/>
       <c r="G107" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="H107" s="5" t="s">
         <v>468</v>
@@ -6250,64 +6265,68 @@
       </c>
       <c r="C108" s="5"/>
       <c r="D108" s="5" t="s">
+        <v>760</v>
+      </c>
+      <c r="E108" s="5" t="s">
+        <v>761</v>
+      </c>
+      <c r="F108" t="s">
         <v>472</v>
       </c>
-      <c r="E108" s="5"/>
-      <c r="F108" t="s">
+      <c r="G108" s="5" t="s">
+        <v>762</v>
+      </c>
+      <c r="H108" s="5" t="s">
+        <v>763</v>
+      </c>
+      <c r="I108" s="8" t="s">
         <v>473</v>
       </c>
-      <c r="G108" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="H108" s="5"/>
-      <c r="I108" s="8" t="s">
+      <c r="J108" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A109" s="5" t="s">
         <v>474</v>
       </c>
-      <c r="J108" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=francois-xavier.panaccio@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A109" s="5" t="s">
+      <c r="B109" s="5" t="s">
         <v>475</v>
       </c>
-      <c r="B109" s="5" t="s">
-        <v>476</v>
-      </c>
       <c r="C109" s="5" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E109" s="5"/>
       <c r="F109" s="5" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G109" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H109" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="I109" s="3" t="s">
         <v>478</v>
       </c>
-      <c r="I109" s="3" t="s">
+      <c r="J109" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A110" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="B110" s="5" t="s">
         <v>479</v>
       </c>
-      <c r="J109" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=caroline.patenaude@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A110" s="5" t="s">
-        <v>475</v>
-      </c>
-      <c r="B110" s="5" t="s">
+      <c r="C110" s="5" t="s">
         <v>480</v>
-      </c>
-      <c r="C110" s="5" t="s">
-        <v>481</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>13</v>
@@ -6316,31 +6335,31 @@
         <v>29</v>
       </c>
       <c r="F110" s="5" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="G110" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H110" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="I110" s="3" t="s">
         <v>482</v>
       </c>
-      <c r="I110" s="3" t="s">
+      <c r="J110" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A111" s="5" t="s">
         <v>483</v>
-      </c>
-      <c r="J110" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=david.patenaude.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A111" s="5" t="s">
-        <v>484</v>
       </c>
       <c r="B111" s="5" t="s">
         <v>289</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>13</v>
@@ -6353,25 +6372,25 @@
         <v>88</v>
       </c>
       <c r="H111" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="I111" s="3" t="s">
         <v>486</v>
       </c>
-      <c r="I111" s="3" t="s">
+      <c r="J111" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A112" s="5" t="s">
         <v>487</v>
-      </c>
-      <c r="J111" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=stephanie.pham-dang@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A112" s="5" t="s">
-        <v>488</v>
       </c>
       <c r="B112" s="5" t="s">
         <v>449</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>27</v>
@@ -6380,61 +6399,61 @@
         <v>77</v>
       </c>
       <c r="F112" s="5" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="G112" s="4"/>
       <c r="H112" s="3"/>
       <c r="I112" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="J112" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A113" s="5" t="s">
         <v>491</v>
       </c>
-      <c r="J112" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.pigeon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A113" s="5" t="s">
+      <c r="B113" s="5" t="s">
         <v>492</v>
       </c>
-      <c r="B113" s="5" t="s">
+      <c r="C113" s="5" t="s">
         <v>493</v>
-      </c>
-      <c r="C113" s="5" t="s">
-        <v>494</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E113" s="5"/>
       <c r="F113" s="5" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G113" s="5" t="s">
         <v>301</v>
       </c>
       <c r="H113" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="I113" s="15" t="s">
         <v>496</v>
       </c>
-      <c r="I113" s="15" t="s">
+      <c r="J113" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A114" s="5" t="s">
         <v>497</v>
       </c>
-      <c r="J113" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=refmede@bib.umontreal.ca</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A114" s="5" t="s">
+      <c r="B114" s="5" t="s">
         <v>498</v>
       </c>
-      <c r="B114" s="5" t="s">
-        <v>499</v>
-      </c>
       <c r="C114" s="5" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D114" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E114" s="5"/>
       <c r="F114" s="5"/>
@@ -6442,53 +6461,53 @@
         <v>21</v>
       </c>
       <c r="H114" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="I114" s="8" t="s">
         <v>500</v>
       </c>
-      <c r="I114" s="8" t="s">
+      <c r="J114" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
         <v>501</v>
       </c>
-      <c r="J114" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nathalie.poulin.4@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A115" t="s">
+      <c r="B115" t="s">
         <v>502</v>
       </c>
-      <c r="B115" t="s">
+      <c r="C115" t="s">
+        <v>625</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="G115" t="s">
+        <v>585</v>
+      </c>
+      <c r="H115" s="5" t="s">
         <v>503</v>
       </c>
-      <c r="C115" t="s">
-        <v>626</v>
-      </c>
-      <c r="D115" s="5" t="s">
-        <v>682</v>
-      </c>
-      <c r="G115" t="s">
-        <v>586</v>
-      </c>
-      <c r="H115" s="5" t="s">
+      <c r="I115" s="8" t="s">
         <v>504</v>
       </c>
-      <c r="I115" s="8" t="s">
-        <v>505</v>
-      </c>
       <c r="J115" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=jeremy.prime@umontreal.ca</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B116" t="s">
         <v>449</v>
       </c>
       <c r="C116" s="14"/>
       <c r="D116" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E116" s="5" t="s">
         <v>77</v>
@@ -6500,48 +6519,48 @@
         <v>307</v>
       </c>
       <c r="I116" s="6" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="J116" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.proulx@umontreal.ca</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
+        <v>505</v>
+      </c>
+      <c r="B117" t="s">
         <v>506</v>
-      </c>
-      <c r="B117" t="s">
-        <v>507</v>
       </c>
       <c r="C117" s="16"/>
       <c r="D117" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G117" t="s">
         <v>29</v>
       </c>
       <c r="H117" t="s">
+        <v>507</v>
+      </c>
+      <c r="I117" s="8" t="s">
         <v>508</v>
       </c>
-      <c r="I117" s="8" t="s">
-        <v>509</v>
-      </c>
       <c r="J117" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=clotilde.rajalu@umontreal.ca</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="B118" t="s">
         <v>75</v>
       </c>
       <c r="C118" s="5"/>
       <c r="D118" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>77</v>
@@ -6554,82 +6573,82 @@
         <v>307</v>
       </c>
       <c r="I118" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="J118" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=christian.remillard@umontreal.ca</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
+        <v>642</v>
+      </c>
+      <c r="B119" t="s">
         <v>643</v>
       </c>
-      <c r="B119" t="s">
-        <v>644</v>
-      </c>
       <c r="C119" s="5" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D119" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E119" s="5"/>
       <c r="F119" s="3"/>
       <c r="G119" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H119" t="s">
+        <v>645</v>
+      </c>
+      <c r="I119" s="6" t="s">
         <v>646</v>
       </c>
-      <c r="I119" s="6" t="s">
-        <v>647</v>
-      </c>
       <c r="J119" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=sarah-julie.richard@umontreal.ca</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B120" t="s">
         <v>50</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="D120" t="s">
         <v>13</v>
       </c>
       <c r="F120" s="5" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G120" t="s">
         <v>29</v>
       </c>
       <c r="H120" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="I120" s="3" t="s">
         <v>513</v>
       </c>
-      <c r="I120" s="3" t="s">
-        <v>514</v>
-      </c>
       <c r="J120" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=valerie.rioux.3@umontreal.ca</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B121" t="s">
         <v>123</v>
       </c>
       <c r="C121" s="5"/>
       <c r="D121" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E121" s="5" t="s">
         <v>77</v>
@@ -6638,28 +6657,28 @@
         <v>78</v>
       </c>
       <c r="H121" t="s">
+        <v>723</v>
+      </c>
+      <c r="I121" s="6" t="s">
         <v>724</v>
       </c>
-      <c r="I121" s="6" t="s">
-        <v>725</v>
-      </c>
       <c r="J121" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=eric.romano@umontreal.ca</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B122" s="5" t="s">
         <v>407</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D122" s="5" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E122" s="5" t="s">
         <v>77</v>
@@ -6669,54 +6688,54 @@
         <v>113</v>
       </c>
       <c r="I122" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="J122" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A123" s="5" t="s">
         <v>517</v>
       </c>
-      <c r="J122" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.sevigny@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A123" s="5" t="s">
+      <c r="B123" s="5" t="s">
         <v>518</v>
       </c>
-      <c r="B123" s="5" t="s">
-        <v>519</v>
-      </c>
       <c r="C123" s="5" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E123" s="5"/>
       <c r="F123" s="5" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="G123" s="5" t="s">
         <v>155</v>
       </c>
       <c r="H123" s="3"/>
       <c r="I123" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="J123" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
         <v>521</v>
       </c>
-      <c r="J123" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chloe.sinotte@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A124" t="s">
+      <c r="B124" t="s">
         <v>522</v>
       </c>
-      <c r="B124" t="s">
-        <v>523</v>
-      </c>
       <c r="C124" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E124" s="5"/>
       <c r="F124" s="5"/>
@@ -6728,76 +6747,76 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="3" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B125" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C125" s="14" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>27</v>
       </c>
       <c r="E125" s="3"/>
       <c r="F125" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="G125" s="3" t="s">
         <v>526</v>
       </c>
-      <c r="G125" s="3" t="s">
+      <c r="H125" s="3" t="s">
         <v>527</v>
       </c>
-      <c r="H125" s="3" t="s">
+      <c r="I125" s="3" t="s">
         <v>528</v>
       </c>
-      <c r="I125" s="3" t="s">
+      <c r="J125" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A126" s="3" t="s">
         <v>529</v>
-      </c>
-      <c r="J125" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=viviane.st-arnaud@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A126" s="3" t="s">
-        <v>530</v>
       </c>
       <c r="B126" s="3" t="s">
         <v>236</v>
       </c>
       <c r="C126" s="3"/>
       <c r="D126" s="3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F126" s="3"/>
       <c r="G126" s="3"/>
       <c r="H126" s="3" t="s">
+        <v>530</v>
+      </c>
+      <c r="I126" s="3" t="s">
         <v>531</v>
       </c>
-      <c r="I126" s="3" t="s">
+      <c r="J126" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A127" s="5" t="s">
         <v>532</v>
       </c>
-      <c r="J126" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=chantal.taillon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A127" s="5" t="s">
+      <c r="B127" s="5" t="s">
         <v>533</v>
       </c>
-      <c r="B127" s="5" t="s">
+      <c r="C127" s="5" t="s">
         <v>534</v>
       </c>
-      <c r="C127" s="5" t="s">
-        <v>535</v>
-      </c>
       <c r="D127" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E127" s="5" t="s">
         <v>77</v>
@@ -6806,57 +6825,57 @@
         <v>306</v>
       </c>
       <c r="H127" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="I127" s="15" t="s">
         <v>536</v>
       </c>
-      <c r="I127" s="15" t="s">
-        <v>537</v>
-      </c>
       <c r="J127" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=mathieu.nicolas.tardif@umontreal.ca</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B128" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E128" s="5"/>
       <c r="F128" s="3"/>
       <c r="G128" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H128" t="s">
+        <v>648</v>
+      </c>
+      <c r="I128" s="6" t="s">
         <v>649</v>
       </c>
-      <c r="I128" s="6" t="s">
-        <v>650</v>
-      </c>
       <c r="J128" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.theberge.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="B129" s="5" t="s">
         <v>538</v>
       </c>
-      <c r="B129" s="5" t="s">
-        <v>539</v>
-      </c>
       <c r="C129" s="5" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D129" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E129" s="5"/>
       <c r="F129" s="5"/>
@@ -6864,58 +6883,58 @@
         <v>419</v>
       </c>
       <c r="H129" s="5" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="I129" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="J129" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A130" s="3" t="s">
         <v>540</v>
       </c>
-      <c r="J129" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=karine.theriault-dube@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A130" s="3" t="s">
+      <c r="B130" s="3" t="s">
         <v>541</v>
       </c>
-      <c r="B130" s="3" t="s">
+      <c r="C130" s="5" t="s">
         <v>542</v>
-      </c>
-      <c r="C130" s="5" t="s">
-        <v>543</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>267</v>
       </c>
       <c r="E130" t="s">
+        <v>543</v>
+      </c>
+      <c r="F130" s="3" t="s">
         <v>544</v>
       </c>
-      <c r="F130" s="3" t="s">
+      <c r="G130" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="H130" s="3" t="s">
         <v>545</v>
       </c>
-      <c r="G130" s="3" t="s">
-        <v>599</v>
-      </c>
-      <c r="H130" s="3" t="s">
+      <c r="I130" s="15" t="s">
         <v>546</v>
       </c>
-      <c r="I130" s="15" t="s">
+      <c r="J130" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A131" s="5" t="s">
         <v>547</v>
-      </c>
-      <c r="J130" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=mylene.therrien@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A131" s="5" t="s">
-        <v>548</v>
       </c>
       <c r="B131" s="5" t="s">
         <v>449</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>27</v>
@@ -6928,28 +6947,28 @@
         <v>126</v>
       </c>
       <c r="H131" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="I131" s="15" t="s">
         <v>550</v>
       </c>
-      <c r="I131" s="15" t="s">
+      <c r="J131" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A132" s="5" t="s">
         <v>551</v>
       </c>
-      <c r="J131" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=m.thomas@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A132" s="5" t="s">
+      <c r="B132" s="5" t="s">
         <v>552</v>
       </c>
-      <c r="B132" s="5" t="s">
-        <v>553</v>
-      </c>
       <c r="C132" s="5" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D132" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E132" s="5"/>
       <c r="F132" s="5"/>
@@ -6957,83 +6976,83 @@
         <v>419</v>
       </c>
       <c r="H132" t="s">
+        <v>553</v>
+      </c>
+      <c r="I132" s="8" t="s">
         <v>554</v>
       </c>
-      <c r="I132" s="8" t="s">
+      <c r="J132" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A133" s="5" t="s">
         <v>555</v>
       </c>
-      <c r="J132" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=ly.kieng.tir@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A133" s="5" t="s">
+      <c r="B133" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="B133" s="5" t="s">
-        <v>557</v>
-      </c>
       <c r="C133" s="5" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E133" s="5"/>
       <c r="F133" s="5" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="G133" s="5" t="s">
         <v>219</v>
       </c>
       <c r="H133" s="5" t="s">
+        <v>558</v>
+      </c>
+      <c r="I133" s="15" t="s">
         <v>559</v>
       </c>
-      <c r="I133" s="15" t="s">
+      <c r="J133" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
         <v>560</v>
       </c>
-      <c r="J133" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=juliette.tirard-collet@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A134" t="s">
-        <v>561</v>
-      </c>
       <c r="B134" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="D134" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="G134" t="s">
         <v>285</v>
       </c>
       <c r="H134" s="5" t="s">
+        <v>564</v>
+      </c>
+      <c r="I134" s="8" t="s">
         <v>565</v>
       </c>
-      <c r="I134" s="8" t="s">
-        <v>566</v>
-      </c>
       <c r="J134" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=anne-julie.tremblay.2@umontreal.ca</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="5" t="s">
+        <v>560</v>
+      </c>
+      <c r="B135" s="5" t="s">
         <v>561</v>
       </c>
-      <c r="B135" s="5" t="s">
-        <v>562</v>
-      </c>
       <c r="C135" s="5" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D135" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E135" s="5"/>
       <c r="F135" s="5"/>
@@ -7044,56 +7063,56 @@
         <v>405</v>
       </c>
       <c r="I135" s="8" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="J135" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=frederic.tremblay.1@umontreal.ca</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B136" t="s">
         <v>467</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E136" s="5" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F136" t="s">
+        <v>588</v>
+      </c>
+      <c r="G136" t="s">
+        <v>600</v>
+      </c>
+      <c r="H136" t="s">
         <v>589</v>
       </c>
-      <c r="G136" t="s">
-        <v>601</v>
-      </c>
-      <c r="H136" t="s">
+      <c r="I136" s="6" t="s">
         <v>590</v>
       </c>
-      <c r="I136" s="6" t="s">
-        <v>591</v>
-      </c>
       <c r="J136" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=j.trepanier@umontreal.ca</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="s">
+        <v>566</v>
+      </c>
+      <c r="B137" s="5" t="s">
         <v>567</v>
-      </c>
-      <c r="B137" s="5" t="s">
-        <v>568</v>
       </c>
       <c r="C137" s="5"/>
       <c r="D137" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E137" s="5"/>
       <c r="F137" s="5"/>
@@ -7101,28 +7120,28 @@
         <v>53</v>
       </c>
       <c r="H137" s="5" t="s">
+        <v>568</v>
+      </c>
+      <c r="I137" s="8" t="s">
         <v>569</v>
       </c>
-      <c r="I137" s="8" t="s">
+      <c r="J137" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A138" s="5" t="s">
         <v>570</v>
       </c>
-      <c r="J137" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=nancy.turgeon@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A138" s="5" t="s">
+      <c r="B138" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="B138" s="5" t="s">
-        <v>572</v>
-      </c>
       <c r="C138" s="5" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
@@ -7130,28 +7149,28 @@
         <v>29</v>
       </c>
       <c r="H138" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="I138" s="8" t="s">
         <v>573</v>
       </c>
-      <c r="I138" s="8" t="s">
+      <c r="J138" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A139" s="5" t="s">
         <v>574</v>
       </c>
-      <c r="J138" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.vachon.1@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A139" s="5" t="s">
+      <c r="B139" s="5" t="s">
         <v>575</v>
       </c>
-      <c r="B139" s="5" t="s">
-        <v>576</v>
-      </c>
       <c r="C139" s="5" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D139" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E139" s="5"/>
       <c r="F139" s="5"/>
@@ -7159,28 +7178,28 @@
         <v>53</v>
       </c>
       <c r="H139" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="I139" s="8" t="s">
         <v>577</v>
       </c>
-      <c r="I139" s="8" t="s">
-        <v>578</v>
-      </c>
       <c r="J139" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=yan.vallee@umontreal.ca</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
+        <v>719</v>
+      </c>
+      <c r="B140" t="s">
         <v>720</v>
       </c>
-      <c r="B140" t="s">
-        <v>721</v>
-      </c>
       <c r="C140" s="5" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="D140" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>77</v>
@@ -7189,25 +7208,25 @@
         <v>78</v>
       </c>
       <c r="I140" s="6" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J140" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=guillaume.viart@umontreal.ca</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="5" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="C141" s="5" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D141" s="5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E141" s="5"/>
       <c r="F141" s="5"/>
@@ -7215,19 +7234,19 @@
         <v>88</v>
       </c>
       <c r="H141" s="5" t="s">
+        <v>579</v>
+      </c>
+      <c r="I141" s="8" t="s">
         <v>580</v>
       </c>
-      <c r="I141" s="8" t="s">
+      <c r="J141" s="6" t="str">
+        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
+        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A142" s="5" t="s">
         <v>581</v>
-      </c>
-      <c r="J141" s="6" t="str">
-        <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
-        <v>https://teams.microsoft.com/l/chat/0/0?users=josee.viel@umontreal.ca</v>
-      </c>
-    </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A142" s="5" t="s">
-        <v>582</v>
       </c>
       <c r="B142" s="5" t="s">
         <v>211</v>
@@ -7240,7 +7259,7 @@
         <v>70</v>
       </c>
       <c r="F142" s="5" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="G142" t="s">
         <v>425</v>
@@ -7249,23 +7268,23 @@
         <v>446</v>
       </c>
       <c r="I142" s="15" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="J142" s="6" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
         <v>https://teams.microsoft.com/l/chat/0/0?users=emilie.walsh@umontreal.ca</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="s">
+        <v>666</v>
+      </c>
+      <c r="B143" s="5" t="s">
         <v>667</v>
-      </c>
-      <c r="B143" s="5" t="s">
-        <v>668</v>
       </c>
       <c r="C143" s="5"/>
       <c r="D143" s="5" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="E143" s="5" t="s">
         <v>77</v>
@@ -7275,10 +7294,10 @@
         <v>77</v>
       </c>
       <c r="H143" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="I143" s="6" t="s">
         <v>669</v>
-      </c>
-      <c r="I143" s="6" t="s">
-        <v>670</v>
       </c>
       <c r="J143" s="9" t="str">
         <f>IF(ISBLANK(Tableau1[[#This Row],[courriel]]), "", HYPERLINK(_xlfn.CONCAT("https://teams.microsoft.com/l/chat/0/0?users=",Tableau1[[#This Row],[courriel]])))</f>
@@ -7390,15 +7409,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CC83367596A4B94585FCDD3502D89912" ma:contentTypeVersion="11" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="4e4efa8c0f0f722bbfc4a6b86077b9b4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1" xmlns:ns3="9cb1c2f4-2737-4134-a1af-8acbe3d02830" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81c6aeae46cd0fb81a99420a9570330b" ns2:_="" ns3:_="">
     <xsd:import namespace="7c5d7804-4d0b-4e60-9ce8-4dcaa1999ed1"/>
@@ -7593,6 +7603,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBEF5B7A-066E-4CFA-AECB-2B495BA6263D}">
   <ds:schemaRefs>
@@ -7611,14 +7630,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCC2BCD-0310-4A3C-9E4B-6EFDEBA53649}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7635,4 +7646,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3747C807-31DC-4949-A88C-18B7D05A7D8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>